<commit_message>
chore: update latest_deduped.xlsx [2026-02-20 15:44 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Americold (COLD) Soars 15.7% on Upbeat 2026 Outlook, CFO Appointment - Bitget</t>
+          <t>B&amp;M £20 'sleek' laundry basket nearly half price of B&amp;Q £39 'elegant' option - Essex Live</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Americold (COLD) Soars 15.7% on Upbeat 2026 Outlook, CFO Appointment - Bitget</t>
+          <t>B&amp;M £20 'sleek' laundry basket nearly half price of B&amp;Q £39 'elegant' option - Essex Live</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:43:10 GMT</t>
+          <t>Fri, 20 Feb 2026 11:56:22 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE9yTzNwcEpmdGlfWDVVcHkwTHZ5bnRIYzJ1VHZNR0ZxbTdNY1oyQkp2cUdVZU1BM2daSS1ab0s4MnlCOUVyWHRmTjV2YTJZMkhzY2FsUjVMZldCcUVXanlTcEtOd9IBY0FVX3lxTE9yTzNwcEpmdGlfWDVVcHkwTHZ5bnRIYzJ1VHZNR0ZxbTdNY1oyQkp2cUdVZU1BM2daSS1ab0s4MnlCOUVyWHRmTjV2YTJZMkhzY2FsUjVMZldCcUVXanlTcEtOdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPWHpaMVB3R3B0VjN2ME80Q1pfZC1UcUEwQjQzVjVLeE1VYklFMkUwLXFkaEpFbkxtX29OYW5YOFRjRzByODFfMHJfdUNORlVQUDNwWm1yQWtROE5ZR3ViRTZJZkR1Ri1rbDBsT1RqQ1hxbEhrbDJ0bzBHeGtEa1dmWXA5dmRSakk?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46073.44664351852</v>
+        <v>46073.49747685185</v>
       </c>
     </row>
     <row r="3">
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B&amp;M £20 'sleek' laundry basket nearly half price of B&amp;Q £39 'elegant' option - Kent Live</t>
+          <t>Americold (COLD) Soars 15.7% on Upbeat 2026 Outlook, CFO Appointment - Bitget</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B&amp;M £20 'sleek' laundry basket nearly half price of B&amp;Q £39 'elegant' option - Kent Live</t>
+          <t>Americold (COLD) Soars 15.7% on Upbeat 2026 Outlook, CFO Appointment - Bitget</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 08:42:46 GMT</t>
+          <t>Fri, 20 Feb 2026 10:43:10 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxOaDd0aV9pS21ndUtZdXRlY0tVcXUtMTM0Q09pRnI0VDA5U1dRX1hvRHNpWVVaektzajJyNHRKTFktMDhBQ3pMS01yZV9qbXlqdzFuMm5RMHVNdGpTSUVjQ3RkRjhjQlk4WWlEQkVFNzVEWEY2SEY1WW5CRXgwekpKa3liSmFSUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE9yTzNwcEpmdGlfWDVVcHkwTHZ5bnRIYzJ1VHZNR0ZxbTdNY1oyQkp2cUdVZU1BM2daSS1ab0s4MnlCOUVyWHRmTjV2YTJZMkhzY2FsUjVMZldCcUVXanlTcEtOd9IBY0FVX3lxTE9yTzNwcEpmdGlfWDVVcHkwTHZ5bnRIYzJ1VHZNR0ZxbTdNY1oyQkp2cUdVZU1BM2daSS1ab0s4MnlCOUVyWHRmTjV2YTJZMkhzY2FsUjVMZldCcUVXanlTcEtOdw?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46073.3630324074</v>
+        <v>46073.44664351852</v>
       </c>
     </row>
     <row r="4">
@@ -645,32 +645,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>Politie opgeroepen voor schietpartij in Sint-Jans-Molenbeek - Nieuwsblad</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>Police called for shooting in Sint-Jans-Molenbeek - Nieuwsblad</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 06:12:26 GMT</t>
+          <t>Fri, 20 Feb 2026 15:28:55 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQOGNjVDdzNXFXVEZHMEFmaGdnaVZTN1UzZ0txV1BGYzc1dm5CLTg2dmEtSEdYSVBlN3drRUVGSmJrNmg4QWxkdUd3by0wN0ZIRVNJd3c2cDJqenFCTnNyWTJyZnlEUVZ4MWFaU3p5LUJXNzNRWEhBVEVjUTQ1U2o2aGJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOZ05fQW93OTZLWm51TDhlYXQ3WURtbDRNY1JXdjBQYWlQazRmZXF4SGtKUzBFbmRvQ2Z5c3E4S3d4TG54S3VyZ3FJZ0JBdVJIaXd6Y0kxY3BtV21tUjdmeW90X3hHcVhpcGZaMGl5VGhzdFFDRm82SnZSdUw2cy11QXpUYnB6Zl9mWkxsdHpJTVNHdGluMHRYUnd0bFRFRTR4ZnF6NjZkcHNValU3UEFSZVMyU0c?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46073.25863425926</v>
+        <v>46073.64508101852</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fallen tree blocks railway line and causes delays - AOL.com</t>
+          <t>"Overwinning voor alle overlevenden": familie Epstein-slachtoffer Virginia Giuffre reageert op arrestatie Andrew - VRT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Fallen tree blocks railway line and causes delays - AOL.com</t>
+          <t>"Victory for all survivors": Epstein victim Virginia Giuffre's family responds to Andrew's arrest - VRT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 23:53:37 GMT</t>
+          <t>Fri, 20 Feb 2026 11:01:01 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxOelJRdGRTOC1PMjNCNERYenB5Ml9OSjJMOHNDcXQ2dWd6U3NZeWxHMlJKb1NUT3JmN3dFVTl0QlVMMldxTGFJcWxObm5UN2ZfRVUySmxfQURXNktUNi1BN1FKSmxQZUkwVDZlSlV4bEwxZmF3cEdQcW0yTEF4cEFaaQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNMFBjUkoxZldtaEhqbmpmc0oyWlEteF95WWFIX1RmcEtqVi1mTXhsbmpBMVlNZUFaamo0N0NEbTRKZjMxdXFaeEk4Q2pCOWVsM2tOc21oTU5hejB2SkJHeGlBZnY5d2M3WURCWU4yTVFPcTRYcE02al9HSXVsRjhabWhpc1FOb0RmUUU2SWVudmg2NkFseVJjRzJ0a2RleFF5LThtQnU3MGwxazRwOXZB?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,21 +735,21 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46072.99556712963</v>
+        <v>46073.45903935185</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Gewonde bij steekpartij vlak bij bekend café - Nieuwsblad</t>
+          <t>Scooterrijder gooit zwaar vuurwerk onder de auto van Frans Theunisz: ‘Geen idee uit welke hoek dit komt’ - De Limburger</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Injured in stabbing near well-known café - Nieuwsblad</t>
+          <t>Scooter rider throws heavy fireworks under Frans Theunisz's car: 'No idea where this came from' - De Limburger</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 17:58:00 GMT</t>
+          <t>Fri, 20 Feb 2026 12:07:28 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPekJQa2h4emRrRV9zbml6c0dmZDVfRHd3eWlnSDVqR1dqemlhalphOTQ3WGo1aVNzN19sN1JuNWFyalM0ajh5QTlIR1N4Nmt5QUZhQnpSdXcyVXI3WUV6VWVyTjVYZjljZHlBNkdrZHU4eXVLS2xUWUs3MXN3ek5hbmdYdi1ISXY1aml1czNWNVhCTVdXdVRiNFh2SlFOU2pveU1JazRCTE1RWWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxPVTRGc1VJNk9UQlZVenZuamd1aG1CakdYQVZrb1FjUzJLazRiUFNtTFdtVjUwT0tlZnQzWUlZQnBVRUdabkE1WEpXb1pldzhjbV9JTGlmMzJ3ZHczYTFZNnJIUGJWVUIxOW9xOFJIaFNxQUFtNm9FbjZXeFRVLXgxUlMzSHRkNlBacnY2cUF0b3c3NFNwSjF4RFF4SWhLWE96VGtjTExYbUFvcEJHTzlvSzU4Yi1UWDVnUTd4aE0xZk9lSnVJd3hFZldkV3pBRnZkZTI5SjNaWjRWYTFzT1VpaFh0ZWZHSXV0MGE4QUNXQQ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46072.74861111111</v>
+        <v>46073.50518518518</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ivan Ollevier in Londen: "Veel Britten verwachtten dat arrestatie eraan zat te komen" - VRT</t>
+          <t>Importverbod op Russische olie per schip vertraagd - Nieuwsblad Transport</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ivan Ollevier in London: "Many Britons expected that arrest was coming" - VRT</t>
+          <t>Import ban on Russian oil by ship delayed - Nieuwsblad Transport</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 18:18:09 GMT</t>
+          <t>Fri, 20 Feb 2026 11:18:17 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNMVRWWmRPaThXYXFqR3dTUHFVLTY3b1J4S180WGxmcDN5dmZrOF9DQ1A3dWNqNWw3X1FGZFBWUGRNLTE2NDR2Wmx3VTBnZTd0VGl4VmJWU0VUYlpiUXV6dGc2MkJUVEZnN3pYRDUzaXdNemRkeHc1cnNhN2xtSzVJczluZG4yYV91UWp1MVQxZW5Zdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNZTVMSVdIUDhqZUVobFVoZ1pLdUJiVGlSRjhBSGcxSmdWWDJwZGdxOFdNeGpMZW1TVGllc1RfV2YyUnZaRzdyMEVDMkpaUW9GT1pvTkFpZUJwQ0JZVzRpS1pNdUJtd291dmMyMGZtTjNjLURzM0tkY2dfTEZ6YVFHbXBiZzY4WXk1V3dubF8zcTRYX0Vpbnkw?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46072.76260416667</v>
+        <v>46073.47103009259</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Scooterrijder gooit zwaar vuurwerk onder de auto van Frans Theunisz: ‘Geen idee uit welke hoek dit komt’ - De Limburger</t>
+          <t>Explosie bij bedrijfspand in Helmond: harde knal en veel schade - AD.nl</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Scooter rider throws heavy fireworks under Frans Theunisz's car: 'No idea where this came from' - De Limburger</t>
+          <t>Explosion at business premises in Helmond: loud bang and a lot of damage - AD.nl</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:07:28 GMT</t>
+          <t>Fri, 20 Feb 2026 09:42:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxPVTRGc1VJNk9UQlZVenZuamd1aG1CakdYQVZrb1FjUzJLazRiUFNtTFdtVjUwT0tlZnQzWUlZQnBVRUdabkE1WEpXb1pldzhjbV9JTGlmMzJ3ZHczYTFZNnJIUGJWVUIxOW9xOFJIaFNxQUFtNm9FbjZXeFRVLXgxUlMzSHRkNlBacnY2cUF0b3c3NFNwSjF4RFF4SWhLWE96VGtjTExYbUFvcEJHTzlvSzU4Yi1UWDVnUTd4aE0xZk9lSnVJd3hFZldkV3pBRnZkZTI5SjNaWjRWYTFzT1VpaFh0ZWZHSXV0MGE4QUNXQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQdEN1aWVLUmtRb0wzcjNGWVhGT1pWQjU5eC1qX0dRUHhWTUV0dHAxaUlQb1ZEZ3AwSDFOSkJHUHdJQW9hR0lleFZ5QXY1b1JnOFFCQ1Rud0FNRjhFVUQxajJtSkNONHNvazlkeHNBbEpVM2VFbXgyYlhyZWc2Y2J5dWg4YTVlWDJBRUIwNnQzcTlrQmViYlIyb0I5Y180R2s?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,38 +914,38 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46073.50518518518</v>
+        <v>46073.40416666667</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Minstens 12 doden bij explosie in vuurwerkwinkel in China - MSN</t>
+          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>At least 12 dead in explosion at fireworks store in China - MSN</t>
+          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 22:39:40 GMT</t>
+          <t>Fri, 20 Feb 2026 10:04:47 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQbzlENDYzcVNBVmlsa05GdXVQUkdISGVjODBBZVZYOGlLRzBhWDNDVFdwcjhHd1dZb0dnQ1RhSGhDckRGYW83Qld5UVFWdnNpYS1HREFUX01YOTM3SzlPbGVHeEZOc2VOdmthcTB0eDZ0OWVmNWxEdUVqYnJHemxpRUs4UTBWMVFLbEhlWjFqZEhUeVRGQTJmWkJ1WWdLdTZ6N0dBRWdKZ0pFdWtf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOcVV3cGgtM0t5Nm5XbTFJbGR2N0Q1RHRhVmJ3VnJFTGhiUVN5bFJpWUUyNUxVLVEwVjF1elZ4WXdIVUVVWXVmcm1nelZXYV9FcEVBS3ZPeU92aDlmRko2eWI3WjZqRWxUeTlteVVvVDM3Y2ZlbkJWT2QtWFJNQ0paNUJDOTh2b1JaZVdOSVdsVndLbXVUNU0tTlBTUUdKUFF5TVdF?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46072.94421296296</v>
+        <v>46073.41998842593</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Persoon verschanst zich in woning in Schaarbeek: politie pakt verdachte op - HLN</t>
+          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Person is hiding in a home in Schaerbeek: police arrest suspect - HLN</t>
+          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 18:08:22 GMT</t>
+          <t>Fri, 20 Feb 2026 12:57:47 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOcng1R3ZFQTVKU2FzcHBkVzRTNHpwaFNuQ2U4TFE4VEtscDFQc1ctbVU4X3AtQkp3eGtzd19fWWJCRVR3Y2VTY2U4UHlvTnhMWXl2dUxFWEoxRS1LVXkyYXIxdGtWdTJPemRGZjQ0ZFV1aFd2XzdlRWt1ejRhYXdSaHRBeUNwWURmUEQtdUc3TENKbFh6LWdidHNQVGZFTzQ1VEdVVDd6b0hRTUxUUGdv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQNkdQYmNiZjFHS0pDdmR0MEJkMkQxcGZRUlJZVzJPeEJBY1VoZWNabWN3NFdZM25Qb01iaWVVSVNyUlZUUXc3QmdPN2RvWFFkdlhDZU1rRjdRUF9kRV8xTy0xOE03SmhHUmdyLWdyclJaQXBEYUFlNl95eXR5Vy1WUmFHaHVDSlpNVUdwUnlSUWtKbl8xMU5wLWs5Q2V0bUhCdVBhaHBMR21JdlowUTNNVU4wNzh1Wk5ORjIw?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46072.75581018518</v>
+        <v>46073.54012731482</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bedrijfsgebouw loopt schade op door explosie in Helmond - De Gelderlander</t>
+          <t>Un Belge détenu en France pour agression sexuelle sur un garçon de 13 ans extradé vers la Belgique - 7sur7.be</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Business building sustains damage due to explosion in Helmond - De Gelderlander</t>
+          <t>Belgian detained in France for sexual assault on 13-year-old boy extradited to Belgium - 7sur7.be</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:20:44 GMT</t>
+          <t>Fri, 20 Feb 2026 15:35:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOT2dpbThDbnlQOVM3S19zalFPTWs4ZmItZ2dHTGtCOXZaeEhhTmYxMk9zem5fZ3gwcnZJVjQ5OTNBOXpiUXFSd05uMC1hZTF0STdHWFZOdGN4V1VudExMX2ZPOVVaUGVfYmhIU2tNWUZPandtRVNJUnNqSXBVMHlMVWdhZ0FkaTl6Ti00a21CUVYxbGswWldvdGh3eG5zMWdrVVdsOFJB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNWF9veDBvVHRlMy1ESVJ4MTFVUTJzSm5FeXB4RUExV01BaE9PaEdjMElYRE5wb2NlVFJsclV1U1A0R3BjN0pqb1NWeDI5T0IyNWFqV0VUZDhtZjZRSFMySXdoSDdHZEluMXA0bWp2MXZCVFkxUDc2Y2l4UWxRZDZybmU3YjRXdXN0MTNkTkxGQ3hweXJDV1JhdUhpM3lQNldib1RuajFPMjRualdMSlpRMC1DWWxQYkFFNU5CYXpNbzZrdnRCam1fN0U3ZEFzdGo2a2VhTjZrWEZNZw?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46073.55606481482</v>
+        <v>46073.64930555555</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Koning Charles ontwijkt vragen over arrestatie Andrew - HLN</t>
+          <t>Des adolescents forcés à monter en voiture et dépouillés en périphérie bruxelloise : le véhicule retrouvé à Molenbeek - BruxellesToday</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>King Charles avoids questions about Andrew's arrest - HLN</t>
+          <t>Teenagers forced into a car and robbed on the outskirts of Brussels: the vehicle found in Molenbeek - BruxellesToday</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 18:36:42 GMT</t>
+          <t>Fri, 20 Feb 2026 11:18:00 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQNTJOZjRXWWdoUzdYRXpacjZ1ZE1lUHJnelBqZEpYUl9kQmZYYWlNa2NQR0pOTlRFX2JSVmh6dXRWcVQ5cnNuOHhDMzI1OXBaRnFSN3dhTDZwQnB6UTZJSjBrOC1Od3JyQ3NOMGZlSHFBUnZVU254QnJ4bnZnYUgyTDRaTGVIYWpEV2hsUUhlSmlSZkNNMDFWdFVuOWZoZ3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNa1czMENlV0VNOUxwc3VuaXpucVNSdy1DYnM2WjZZNm9KN2MwVG1pWnBIRUVJc0ZJbThrVzVQVlBLejl0RDZ1RmZDVzdtcTBBYV9MQ2JPdFV2RElUbVpqQ2xCSmkyMjRMcGNQUHZtUl9HWWVMcDJtRTZSNnJFSHVGUWRMbG9QZnE5Nm4wWXBxNnpkZzlmODhmanNkUXZfM2Qw?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46072.77548611111</v>
+        <v>46073.47083333333</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Weer woning in straat Amstenrade vernield door explosie vanwege mogelijk zwaar vuurwerk - De Limburger</t>
+          <t>#FrigoVide : les associations dénoncent l’explosion de la précarité alimentaire - tvcom.be</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Another house in Amstenrade street destroyed by explosion due to possible heavy fireworks - De Limburger</t>
+          <t>#FrigoVide: associations denounce the explosion of food insecurity - tvcom.be</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 14:58:20 GMT</t>
+          <t>Fri, 20 Feb 2026 15:39:26 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNUkc4SnVsNnRhaF9CSXlkbVU4MTBhaEhNSXUtbGVRNkpKdzluUmZ3UlY1NUhHV2JFVk9qOW13bFdDS2JlU01ha1c2RHJPZ1g1NGsyazE4RmFMQlJoN0tnbmJuei13U2JoSVZObl9kc1pQQ3VlVVBrM1JTMVNtaVJQOUtJRURkVkRLWG13MDhCRVZOOTdmelFIMFBKek5WZlBJMXp1bTJfcG1LQXdOZUEwXzNSU2tBcUtmS05VMTl1cHJ4Q01rTGpXNHB0dE9ySDNqOFpKRUM1YlQzaUhWVVBIWE9kZ3dRWUgtcXNV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUWpKRFpFYlQ5ZTd6NFJfQXZlRnZhMVo0ZlFDMExaQkRldUEweDFNSWd2eFdBMDB1TGlzYk93MFRQR0ZJWVZsQ19yak04UmZlZFMwWDMyUllJUVB5d2R1WTJQT3dQS2NOMTN4TC1DeTMwM3FxWEFuQ09aeE5STWpiSGpUZmVtbzJILWx2aWFaZ3UtejV0cnRRUXRMdVFsYUJ1dGNuSWV3LVZyODg?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46072.62384259259</v>
+        <v>46073.65238425926</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>‘Grey’s Anatomy’-acteur Eric Dane (53) overleden na strijd tegen spierziekte ALS - HLN</t>
+          <t>Un député québécois agressé à Bruxelles: “Triste que les villes européennes en soient rendues là” - 7sur7.be</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>'Grey's Anatomy' actor Eric Dane (53) died after battling ALS - HLN</t>
+          <t>A Quebec MP attacked in Brussels: “Sad that European cities have reached this point” - 7sur7.be</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 05:57:55 GMT</t>
+          <t>Fri, 20 Feb 2026 12:56:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPM3FIUGRDWFBxcmtkTDRCWXVnZHhZVm55TzJsZDV2ZjJLZll1Y2VCcGEwRW9oRzlLb3dpc0xfSVZTNzFNUTUyS3dXX2R0QjFXaG9jX0xEY3duUVNuUHdrbkF5bzhPVHdqMmZkQ2o2QkVEWmlKalkwYnBDSlJSaUUwamhVUjlxT3ZLUmtuc3c4MHJuLUFMNkc2YzAyQkx3d0h2WmlRTGZ3Y0tDbUJuRjFmQ0JvVDU2UEd4czZucQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPeDFBWkdGenBYUkpaZXpzNVB4RzZJemNrTFlwbnpiUzRta0VpcjJUdGhhd0NuMWJjb25ZTFZBZGZhQ2c1VTQzNDVoVzhQYW84Z2k1cFY4R1FGWEpSSkxxQzdXQ2xaWU1Yajh0aG15TEtpLUpMVHRHUXdUd2d4eTZrWHdOZXpNNjJVMHFhV0t4ckdrR2dvOEJFY1RXR044d2ZYODhRYkpOUEJSQWxsTDdQejVaUkwxZFQ1aDNzUkNDaTBsczY1bUREbDNEQmpHMlFEUUZvRlpB?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46073.24855324074</v>
+        <v>46073.53888888889</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cannabisdealer betrapt aan station van Londerzeel... met joint in de hand - HLN</t>
+          <t>Un cycliste perd la vie après avoir été percuté par un camion à Kuurne - 7sur7.be</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cannabis dealer caught at Londerzeel station... with joint in hand - HLN</t>
+          <t>Cyclist dies after being hit by truck in Kuurne - 7sur7.be</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 17:54:40 GMT</t>
+          <t>Fri, 20 Feb 2026 14:16:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOeGdFdXhGZlYta2llNndpTkRTUmF4VUNNcWpRLV82dmYtWjdvMV85M3hMNTFxY3pTU0swd29ESVdkdTltajNLMjIwZC1JUWpBcW5zenpVbUxBZmJQRk16SEt3clVZMXdqaWlqX3BEemVsNWxlVGs0RXc4UnVRUm5WTmpRMG1IZmd1Nm5ZYi1GMDRzenBqdlNWcTNJcUlNakdoQ3dxaVZuT01uLTM0bkJJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPRFNoR2lJX2FBOEFZcnlvN1NYTFgxemZoTG5KWVJETkdmb3kyY2FuUUlGQktvMXAtUlMyWGNHZWZ6RDc4WHY0REhVMTlHdnpzWHpMdUY3VmUyZUNibXVDTnl3S3ZscVZxQjhKTGpvWHFSNDlEUUIwM19lVk5hVm1BY2RMSHlhbFZDTVNoZDFjQ1hqZ3hnYlNSbU1vMjVWNlVnQ2ZoRGxWTlpZOUdYemV4SkhJQXI?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46072.7462962963</v>
+        <v>46073.59444444445</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Intense video shows Alabama women attacked in Brussels - WVTM</t>
+          <t>TC Hasselt - Sept ans de prison pour des violences sexuelles sur ses deux belles-petites-filles - DHnet</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Intense video shows Alabama women attacked in Brussels - WVTM</t>
+          <t>TC Hasselt - Seven years in prison for sexual violence against his two step-granddaughters - DHnet</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 08:23:37 GMT</t>
+          <t>Fri, 20 Feb 2026 09:55:00 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNQ25NMlNoVkhHQUVlcGduTDFmcXh4ZzNfNWRnS2Rwc3phS2VFenl6d1BlWGFwdWgydXNuRElmbDFMMkRkVTNiVFpZT05TVGtaMnBhVjZlT0FKZDdxanczNmNVSFBQbFYzVER4VXl4VDBIWGgxX3N1UG12WG41U0Rydm56MFZFSnBwTll4SnZpbndqUGpiWU85bVh1bmlmMExWLUU4alh2VU5xS1k5MFMzZlk3TFA0XzBmNzJIbnAwQnE2REp4cV9Ya0oxQXNBRTdxekNnTmJFY3hMQlZqY2NTNGVFR3ZaNjNnbjN3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQaHF5Vnl2YUlleldpV0kzTDJZZEtSM2ZJT3pOaWw0aVFxUFpiTGxJaXQ4ajlNSFlibDllVUpHeWhCcnY1WE9DbEdsMzhWb1VXTVJ0MkVBTFZ1NVpONXczUjd2ellXSlRGRWsySFNjdmt4Q1VTU1NPcWVfOG81WEtJcjhlUjFBcDVXSWl5alNXbHlCSjFMeVZUNFZiNFNJamZCS2pVLUt6UVppblVVUjhLeUFfbV9CSUY3OUVrQllHcFRrZDlmVEI4UEpXZWhoYzcxbURqZVR0RnBuenVnb2xhbmVYX2k5QXRnVXRUaUotYjBjWTItZzBxQmNxM3NjRUdaLUE?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46073.3497337963</v>
+        <v>46073.41319444445</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Stabbing near Jeanneke Pis in central Brussels - The Brussels Times</t>
+          <t>French PM says government intends to criminalize calls for any country’s destruction - The Times of Israel</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Stabbing near Jeanneke Pis in central Brussels - The Brussels Times</t>
+          <t>French PM says government intends to criminalize calls for any country’s destruction - The Times of Israel</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 02:45:42 GMT</t>
+          <t>Fri, 20 Feb 2026 09:57:21 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQaVM3ckRmSC1GMW1STGVuMHJnVV9PWVRDb0JmNFo4ZVN3cVBYdjZLc3dVd0VXY0h2SGQwN2ZUSmhPcGFuWHhaV25OT3RvS1lWaFE5ejNvVjVXemdMSUtQdXBlSHFsYVpMcHpDS3hOUU1PME5YUzBVYW1kTmt2Q0FDUjZmZ2JIek1YSFNReA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPdHVVcjRxOUM5a2JxNUlFUjNPdG5iTTc2UDk1cFU1c1ZCd1ltODY4blN2UTdXcGYwN3ZSWXZyV3pFMXZTZWlRemlhTmVib2EtMmhlVHd2RGdNaWlvMmQ2clpBWUYyakE2R09aR1F6Mnk1MHNqV0FsVjlUWmZyWkJuVG03NmstTmIzVmxfQlZkdnNVZmR3N0JabFR3Z1ptOEtRQ1ROQ3huWlZuOHZFV21NeFRyWkVhMmxvOUVhTzdFZ2xJN0xYU0piZA?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1400,47 +1400,47 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46073.11506944444</v>
+        <v>46073.41482638889</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>‘We are a player, not just a payer’: EU Commission defends attendance at Trump’s Peace Board - EUobserver</t>
+          <t>Hundreds of Belgians locked up in foreign prisons - The Brussels Times</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>‘We are a player, not just a payer’: EU Commission defends attendance at Trump’s Peace Board - EUobserver</t>
+          <t>Hundreds of Belgians locked up in foreign prisons - The Brussels Times</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 15:40:11 GMT</t>
+          <t>Fri, 20 Feb 2026 12:13:13 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNUmF0NnVwYVV0V3JJZ3J6elJiMFBjTmo2OTl0dF9WTTBGWFdJSURIci1lT0ZWQWJCNTNKc3p0cl9yYmh1SThPOXBfWi1GMm54MllqbF9JU1VXcVhjOXg2WnVvY20wSi1sNEFNblREYkNZcndFTXN2QnA4cmZVWFdJZ2FGaE5ubnVMWlUwQUczS2xyZTFWalJ0d08waVhaZWpoaVNRUG1NVnR6WGVhQkdWN2ZxZDZKNTBRbVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOM1dqd09VU1RVSjFaYnlfVzlYRmUzc0lWZXN0TVRmZDdOdmJzaTE5TmRxQ1VncHpGM3BJSFItLTVTSktKNDRjdFJEMVVsNHBtbUo1R1J3eFJhdnRhR05RMHk5MExTdGNENnROZ1g2NXREUFZjNU1pWFBEUE9zS3dlckYzSFdSbVhqa3lDTUNFZw?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1455,47 +1455,47 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46072.65290509259</v>
+        <v>46073.50917824074</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
+          <t>Wertheim: 48 junge Beamte zu Polizeiobermeistern ernannt - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
+          <t>Wertheim: 48 young officers appointed police chiefs - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:04:47 GMT</t>
+          <t>Fri, 20 Feb 2026 11:00:00 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOcVV3cGgtM0t5Nm5XbTFJbGR2N0Q1RHRhVmJ3VnJFTGhiUVN5bFJpWUUyNUxVLVEwVjF1elZ4WXdIVUVVWXVmcm1nelZXYV9FcEVBS3ZPeU92aDlmRko2eWI3WjZqRWxUeTlteVVvVDM3Y2ZlbkJWT2QtWFJNQ0paNUJDOTh2b1JaZVdOSVdsVndLbXVUNU0tTlBTUUdKUFF5TVdF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOVmx1X1F5RFNnSlRmakZ1d2dxcmtYcnJQWFdSeVlKWVBCMzE0Y3d6b1VSVTRPN1l5LWZPa2NGX25Gb0ktUEVxaEFnYkpHc1pTTHl3WTkxMHhrRlVnazRPcE9JcE1OaExlRHhEZ2ZRYkN4TWRSakg5VFdodHAwV0pRSHI2TlRLU1dXZjNXVDVEVDNULXI3amZuX0FLVEFCTWVDX05VTG16bE1WYWtkRVBoVXFkbUxmYjdzSlhTMEhsRzBKTDBFTGc?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46073.41998842593</v>
+        <v>46073.45833333334</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:57:47 GMT</t>
+          <t>Fri, 20 Feb 2026 12:52:05 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQNkdQYmNiZjFHS0pDdmR0MEJkMkQxcGZRUlJZVzJPeEJBY1VoZWNabWN3NFdZM25Qb01iaWVVSVNyUlZUUXc3QmdPN2RvWFFkdlhDZU1rRjdRUF9kRV8xTy0xOE03SmhHUmdyLWdyclJaQXBEYUFlNl95eXR5Vy1WUmFHaHVDSlpNVUdwUnlSUWtKbl8xMU5wLWs5Q2V0bUhCdVBhaHBMR21JdlowUTNNVU4wNzh1Wk5ORjIw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46073.54012731482</v>
+        <v>46073.53616898148</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Quick smoking break leads to prison sentence for Brussels dealer - The Brussels Times</t>
+          <t>​Ochsenfurt: E-Scooter-Fahrer mit fast drei Promille erwischt - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Quick smoking break leads to prison sentence for Brussels dealer - The Brussels Times</t>
+          <t>​Ochsenfurt: E-scooter driver caught with almost three per mille - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 02:37:30 GMT</t>
+          <t>Fri, 20 Feb 2026 15:15:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQcS13NHhuQndIMkFmd2t2azQwaHZfT1ljUXkzUFhuOTFwTXl2bGRXQVlvRUx3NzFuQTNrdFV0RE9IQnRjakI4NU9hSnBmQjBwd3FZWGx2RkF1LXZNUjgwSjZWOU1leE5uWHV3LW9DbFlLUXR2RlZDV1gtbDNxSlVmZHRSeW14VkpCWU1XRHIzVE1sQzZneldHNG9vLUFnMlM2TEp5b0RDaEViYldYamJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPcmhQcUtxRGRzSmpkbEpwdmYwR2NzTWI5eXRDSzg2Sm1Cd3FuYXFaTmtvMzdWLWFRU1FXcVhDWXF2ZGcxT0ZETzFGeHZoWDdIY29zNjUwNndnLVp5M202cDRsNnFiRVpUQkRMZlJUN0VZeFpXZmt6N2FfWkdkQ0dSZ1Q5NmtmZXNYVnBUT3RQRExkMmZjQlc4TA?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46073.109375</v>
+        <v>46073.63541666666</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Belgium in Brief: Good things come in threes - The Brussels Times</t>
+          <t>Randersacker: Telefontrickbetrüger mit Arzt-Masche erfolgreich - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Belgium in Brief: Good things come in threes - The Brussels Times</t>
+          <t>Randersacker: Telephone scammer with doctor scam successful - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 18:31:58 GMT</t>
+          <t>Fri, 20 Feb 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNMXhkVFo3LWFhMGtMY3VpclJMTEtvanZXUXljWThjcGw1N3d2WWRRckxhaTFZazlwOXFfQkFUUUk0aXhRU0VrZGQtVEZnLU5HTWdFYnZ0QlVQQk9YTVZFb0lET1ltamRiRk45U3J5Q0hsdTNtZGxxYW1IbW9HT3R1QWNYRk41aWF5TXNuQm03RzJmZ0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPMGh3SXFhTUFXXzVCVUQxa1UxSmNGSEhOZ1N6c2VOM0xabHk4a3I4QkwyQWNzaUl2V3VCc2VzZUNmTTFnX1J6TFhRR04zUXlMRDVJc0REZmFRLWZOV0hzMDNzbGtHd1RUYXE0dXVLbkdxOEJNR0dzLXJxOGR0eFpxeTlzdURxRHE2RmtQX0R0VDlOWXNJV0loNjd2cHRMZEVV?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46072.77219907408</v>
+        <v>46073.58333333334</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Des adolescents forcés à monter en voiture et dépouillés en périphérie bruxelloise : le véhicule retrouvé à Molenbeek - BruxellesToday</t>
+          <t>Einbruch in Laufacher Fachgeschäft: Zeugen gesucht | Foto: Silas Stein - main-echo.de</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Teenagers forced into a car and robbed on the outskirts of Brussels: the vehicle found in Molenbeek - BruxellesToday</t>
+          <t>Burglary in Laufach specialist store: Witnesses wanted | Photo: Silas Stein - main-echo.de</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:18:00 GMT</t>
+          <t>Fri, 20 Feb 2026 10:31:21 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNa1czMENlV0VNOUxwc3VuaXpucVNSdy1DYnM2WjZZNm9KN2MwVG1pWnBIRUVJc0ZJbThrVzVQVlBLejl0RDZ1RmZDVzdtcTBBYV9MQ2JPdFV2RElUbVpqQ2xCSmkyMjRMcGNQUHZtUl9HWWVMcDJtRTZSNnJFSHVGUWRMbG9QZnE5Nm4wWXBxNnpkZzlmODhmanNkUXZfM2Qw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNWmtnWnFmSm5hNWthTXJnQXFTSHA1aFdfNkZmQlFPQ0xPenNWMG1PMnpIbEVYblFlN0djMXBIOXZKVWtoRXFadkNrbE9zQnV3YnJ4RENiV1BDeHJkQUt3VkVGdmwxN0FqOTAteDY1ZlZKcVZkTV9OT2xQUTdWOERNU09RZ2lQelo3VkNsUGNfRXdtb1ZPOHFleGtLaDBzZF83TWpWbGQ2NlMxQQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46073.47083333333</v>
+        <v>46073.4384375</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Un député québécois agressé à Bruxelles: “Triste que les villes européennes en soient rendues là” - 7sur7.be</t>
+          <t>Mobile Blitzer in Aschaffenburg aktuell am Freitag: Hier nimmt die Polizei am 20.02.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A Quebec MP attacked in Brussels: “Sad that European cities have reached this point” - 7sur7.be</t>
+          <t>Mobile speed cameras in Aschaffenburg currently on Friday: Here the police are targeting speeders on February 20th, 2026 - News.de</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:56:00 GMT</t>
+          <t>Fri, 20 Feb 2026 13:15:45 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPeDFBWkdGenBYUkpaZXpzNVB4RzZJemNrTFlwbnpiUzRta0VpcjJUdGhhd0NuMWJjb25ZTFZBZGZhQ2c1VTQzNDVoVzhQYW84Z2k1cFY4R1FGWEpSSkxxQzdXQ2xaWU1Yajh0aG15TEtpLUpMVHRHUXdUd2d4eTZrWHdOZXpNNjJVMHFhV0t4ckdrR2dvOEJFY1RXR044d2ZYODhRYkpOUEJSQWxsTDdQejVaUkwxZFQ1aDNzUkNDaTBsczY1bUREbDNEQmpHMlFEUUZvRlpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQNkVuMENSQnJIdUE5ZUpFWWJRNHZVeEVXcHFMQVRwQ1hub2V0Q1VmdDZtS2hsSDQ1d2JiUjhrTW11bHZjWXcxQ0tfNmZpRUdYVHY3OTlzblhSMUVKNmU3THJFdXhNTTd1SGczbjdwbmJDWjNOLS1femx5UjJpUmR5NzNsN3EwWGI2Q3Frb2RESlNBcF9wcVM0WnN0QUdYQ2o2YXJQTDQ5ekJ5bEtFYjlxZlBkOGVUby1lbzFqbXJqMjNVdU5oMEZNZFRYNG5NY0txbFNrUTdNOWJmX1ZibzRtZkN1UC0wVzI2V0hua0pFcllSbFAtSVRn0gH8AUFVX3lxTE90amswVGNHQ01Odnl5TkpmNkQzd2laX3VMSXJjaXQzU3JRcGlfbnJfUi10LWlSM1JjM29KSWIyanFZWnNtcHN3Xy1KOHFIdWRRN2EwUERsWHVrZTZKaWc1bENIdHpGb1Ztb1pKNGNkeVZnQ2lnTi0tRWZlVERwNW5aWGhLOFVPMG8xWmF0OXYtd1QwLVJjaTdWU3hqRkIzV0pRSWk5eW5KelRnbE5IM1cwQ1hDQTBNWko3bS1kdkdPR3V1N09IVEpKRHNTNnhNUFdZUlBCM01oSlFIMlNBMG1SbzRxM1hIVjh5ZG9fNlJGdkU3TU41WXEwUG13SA?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46073.53888888889</v>
+        <v>46073.55260416667</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Un cycliste perd la vie après avoir été percuté par un camion à Kuurne - 7sur7.be</t>
+          <t>Polizei-News Bamberg / Schweinfurt / Würzburg, 20.02.26: Zollamt Schweinfurt intensiviert Kampf gegen Schwarzarbeit 2025 - News.de</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Cyclist dies after being hit by truck in Kuurne - 7sur7.be</t>
+          <t>Police News Bamberg / Schweinfurt / Würzburg, February 20, 2026: Schweinfurt Customs Office intensifies the fight against undeclared work 2025 - News.de</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 14:16:00 GMT</t>
+          <t>Fri, 20 Feb 2026 09:54:02 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPRFNoR2lJX2FBOEFZcnlvN1NYTFgxemZoTG5KWVJETkdmb3kyY2FuUUlGQktvMXAtUlMyWGNHZWZ6RDc4WHY0REhVMTlHdnpzWHpMdUY3VmUyZUNibXVDTnl3S3ZscVZxQjhKTGpvWHFSNDlEUUIwM19lVk5hVm1BY2RMSHlhbFZDTVNoZDFjQ1hqZ3hnYlNSbU1vMjVWNlVnQ2ZoRGxWTlpZOUdYemV4SkhJQXI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPT0gzcXJvcDBRa3pZM3AxVzlTeldTSVU5aGVZSmMwclE3STQ1RTE3c2RXNW9abjg1QXY3ZTQ1UWs1ZVUxX0o1R1BITEdWYmVncXd5aXB0MnlrcG5YT29DS1JTQ3pnb2dBMEZ2RU1kUTV6THlBeXlUejJjTlV1cXpZS01YRUU2a0ZEWmtTdUJRQTQ5eFh3THEtU0RnOEdaV2dleUltLXpSaHRtZUxRdlFV0gG0AUFVX3lxTFB1WmM1eFdVSHVJTVVXN1F4dTRsRkpaaTVWTFZxVWVwMG1JdENPelhXVndjX01Gb3p1NndvblN5WjJPTWdUMG52eFcxOWxDenRSWnBvb0tCUllITTJyNmZDR2t0S2lqbnVnZ2dBMkhIRnBOLXNpbmZ2bnJ2b25IOEtoSmROUDlfajRpLW11Z01lTzUzS3VGZS1oTHZybmxBYkFXdmszQXdtRzJ0Z05lOHozNGFuSQ?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46073.59444444445</v>
+        <v>46073.41252314814</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>La cause de l’interruption du tram 55 à Evere jeudi après-midi est connue - 7sur7.be</t>
+          <t>Polizeimeldung Bamberg, 20.02.2026: Einbrecher entkommen mit Tresor - News.de</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>The cause of the interruption of tram 55 in Evere on Thursday afternoon is known - 7sur7.be</t>
+          <t>Police report Bamberg, February 20, 2026: Burglars escape with a safe - News.de</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:22:00 GMT</t>
+          <t>Fri, 20 Feb 2026 11:35:02 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQODZkcFNoajdpWVBDeFEwdHFtVThXYU9nVkVpMU5qUUYxdFk4WHZWcDNkSWVXN0RnMndHVm5WOXBkX1FldnFkQTZ6UlNwSUFfZVhZRG5sb08zS1ZWTzZHcEJZVVd0NVAtV3NSQmRZb3F2RVV4dU14WTZYTzlNQ2x0WmxZdGFxcG1fdkQzUVVLMTZUYUczRkUtR2ZzT2oxcFFxTGZ2bHAxVE1aS0NzUjN4bDl1MHhMWVU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQTDRVeGxRTzBmZ200OEl2d2huS2VhcFZvTWxucWc0VVhaQkJzak96dW51NEt3V2g3SC1INEZmWXdjbDBVbVRqeDl0NDBqYzJZSHV6Vllwa1NXbC1YRGRLWkpmbWFKdFBHSW5WWVFLQW1vb3hfeWIyY2R1bm5EUllUTkRtLW5iQ3phV3pNSjF0S3dyYS1XZzZkOTd6NG9UWFY1c3Qw0gGoAUFVX3lxTFBlLXFyeU1ONEpmNEV5bFpuQUV6V0lhazdlY21XUFpZaUpVUVFEUVBGbjItWEJaX3ZxWVZpSW1UczJCak9DNkxiMW9NTFhZeXhDUmR0R3M5WGFJbjQtUjN5TldKbkdZOVIyVTVKcUZJd2VHdjdBektOT2ltZ1VwREZDSmFqWVdKeXVBbEhZcGRZYXAzTjhDOW5wX1o2d05SU3RwOTdCSTk4Xw?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46073.39027777778</v>
+        <v>46073.48266203704</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Nids-de-poule et bus déviés dans le quartier de Scheut: "Les habitants se sentent abandonnés" - BruxellesToday</t>
+          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Potholes and diverted buses in the Scheut district: “Residents feel abandoned” - BruxellesToday</t>
+          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 06:00:00 GMT</t>
+          <t>Fri, 20 Feb 2026 15:22:25 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPTEVpNW1QSHZMVU9VOGs2ZGRXM2hrd2NTZFBkUU5VazQyMDRBaVVoa2ZVbTNIWjJxSjF6TEdxQlpuN1Rwa2FvYlcxS3gwOGl2R0NFeEMwOEk2V1V1Mndka1RnQTBvbHFTTW1fSk9WckRnamYzaVRNUGVIdUxObHhHeVhGdnhTcmZpYmdNSW1SVGQxbC1oRjBsNUlWZ2lWUGlnSFF0QXpR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNb01GazY5VElxMXdSWmg3MnpPcFFIYy1pM1FzTFV6enF3SG81MzhFS0xPNzlDUzZCcm5aMXF6NzdEanlKRnpFbHBuNVJqSGN4MU1sUGIzYTZUWldieTF5UHhrQVdQbmZaT0pOOV9QYTZBbTFvdlc2dlVSaER0QVFGQ1Rpc2N3Tlh2WDFIUlZTM1VXYko5YVZZVk5jZlJMb1ExYWVpUnNhamRqUTdPUUIxaUJNNFpONXNU?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46073.25</v>
+        <v>46073.64056712963</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>"Leoni a été tué par l'ex-compagnon de sa petite amie" - BruxellesToday</t>
+          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>“Leoni was killed by his girlfriend’s ex-companion” – BruxellesToday</t>
+          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 16:30:00 GMT</t>
+          <t>Fri, 20 Feb 2026 10:02:00 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNUl9lWXRPcThEaXE4eGdmb0JKcTNjdWtNQnhoRXRpa2UxN25NWmx2emJrUWVxS29YazdjYmFSak9lTnNCQktuSDVnenloQjhXWXhkZ1FCRS1TNklyYzBFSUtCLWFudHVYY1A0d2wxN3B4eUstclh6dmtLNjlTdV8wRHpjMjBjNVU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPdkVfYlpLQ2ViMnBuUy1hUUtTYUhZbFhiUlNHeUJ2cEkzT3QtWEdBcHRDS2tnZ0dWSVBSZ2tGRnUtYjBHbnB5eVN1Z2gzWUtlZVNTZXR3UFZiZDBsQ1NaRWJlNEcyNHlUbWhiNDNlMjMtMjJkaHZKVWtOVGJ2OG9mZm1qWmVRWkFQaGRSaXlnSGM4NzhuSlkwcWplaTF2dXVHMGZjVHZzSWxtdW9ZWmtnNkpVQTVHZjlaMVRSQ0FKR0lWT01zcVROVi1nQnl1NV9NR2p3ZkI2X05Ua1k?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46072.6875</v>
+        <v>46073.41805555556</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mort de Quentin: deux premiers suspects mis en examen pour “homicide volontaire” - 7sur7.be</t>
+          <t>Autobahn gesperrt: Getränkelaster rutscht in die Leitplanke – Unfall auf A93 - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Death of Quentin: first two suspects indicted for “intentional homicide” - 7sur7.be</t>
+          <t>Motorway closed: drinks truck slides into the guardrail - accident on A93 - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 20:22:04 GMT</t>
+          <t>Fri, 20 Feb 2026 10:46:49 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQMnJzSmVWNHNSSEp0OW56bElpQ0p4SkVyQWJrOG83OHNXWnVLZUNjZlJ2SUZyQU5SVmNBVHhTNXNjZ1ZmUnpvMy0tX0VuVllaREJrMHJlaWxZOWRNTWI4eFBLOVFXYVY1eGpZYjRfQjhwZkItODJsT2dTWUE1OS1VMGNwZXctaDNXNU5tQm5ia1IzdXlDcDJsZHhMODl4SjY4VHdSN3JjdUg1WVFuZnVMR2pTc0piLUp3QVZ4MkFn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQb2RxcW1rQ0l1LWN0UnJ6c2RNXzdPdGJwbW9IWjlSN3czX1NaRE9LSGIyZ0JuRi1aWTFrVFBHTEdmaFdUZXZ3T3NRcmI3dHp3WkF6NGYxeUtjLS1XUlZROW5jcG0tS1lCdEFGZl9ibi1VLUFoSjFnS3pmc3E3VDdkS2JBNWRUX3hhU05qcThTM29hWTFXLW5temVmR0w0QzBsbWZKeFJtZnZlUjE2YVNPVXpMVWZWNlN4MHFFY0h1Z0lkX2VvVnhuNHBxTnV1dWxKR0NBZDcyQjVyRFVMM3NDRw?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46072.8486574074</v>
+        <v>46073.44917824074</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>"Pas de fascisme ici": 150 personnes se sont ressemblé à Saint-Josse contre l'extrême droite - BruxellesToday</t>
+          <t>Bayern: Polizei- und Feuerwehrmeldungen am 20.02.2026 - Newsflash24</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>“No fascism here”: 150 people united in Saint-Josse against the far right - BruxellesToday</t>
+          <t>Bavaria: Police and fire brigade reports on February 20, 2026 - Newsflash24</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 19:52:00 GMT</t>
+          <t>Fri, 20 Feb 2026 08:46:00 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxPbnZjS1BSa1hQS3VXNVlYM21WMm1SUlF0cHNPM2VlUFNmUE1XRkZQV1Y1WUF5YWlIQ1NGakJ1Q0dEZGswVEJNYUJJTUFFNUZiNDloTTVLbEUzM0Njem95bUZFRWZxUUE3aGFPR05GdDZ6eWE1QWpITnB5eTFXb2c1MUgtTWhNei1aMjRCbTNPZ3VoNE1BOXJxS09vOWxEd2tROVpRUFlCelh0WXVNS1Y4ekd0TVJaUjZJNTdnWXhWVjlpV1RCTW1mT0gzaWFIQms?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQNmd1b2lTdTQwQ003YVZEc0RlQTFpRHBkcVUzNnU4OWlkOXpHbXRwZF9QUTEtU0FvWVoxQW40SUgxRzVIenoyLUdES3cyX2llYnBvOE1qRVByeDRXWTRTN2syT1IzbFJZSndCZlJManFkbjhVc3ByVV9BcVM1Y3dlUjlFdW02d0hOVW9nZnZPQnJZdXpTaU9r?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46072.82777777778</v>
+        <v>46073.36527777778</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Meer dan 100 kandidaten melden zich na één dag voor 50 vacatures cipier in Hasselt en Tongeren - VRT</t>
+          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>More than 100 candidates register after one day for 50 prisoner vacancies in Hasselt and Tongeren - VRT</t>
+          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 06:53:49 GMT</t>
+          <t>Fri, 20 Feb 2026 11:30:00 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiQ0FVX3lxTE5wNGJWQTM2TURGa0hLSm90STVhUU9DRkRWMVMyNzQ0SU5yLWN4RUhOUFQ5YUZReHJQZEFlZm5pbVc3U0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPQmRWY0VOQzRiY3U1amZfOUIwSVplbGFjTkpXUGxfQ25IWjQtWlMyN1gwcmMtVm1LSnNBMzFGYnJaYklsMG1RdG15R2JBVWFXcHF3R1NGUmZGcHpUSGFnb0RhdUZVXzBCMlJKbWs1ODJ6WHY0Si1rMkRXZmVUaFZZU2lCZnNzUnhWdmQyaXkySmJ5R0l6QlBqV04wMTMtVHJKZW5oN05PT3RtZktCNWVyS2pYYUh0UGZ3RVE?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46073.28737268518</v>
+        <v>46073.47916666666</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Village Las Rozas La Roca (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Veertiger opgepakt voor geweld tegen twee agenten in politiezone Lanaken-Maasmechelen - MSN</t>
+          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Forties arrested for violence against two officers in Lanaken-Maasmechelen police zone - MSN</t>
+          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 22:53:01 GMT</t>
+          <t>Fri, 20 Feb 2026 09:18:53 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNYkFBeFJzakhhYjY4blpLa0g5S19oMjZlTEh3SW1SbXotc1R5N3BwdzBLQW0zcDZVLW9UNnhGZjVuRzJyajAyQmpUTlI2WmRFSDRQY1RNbnRyektRWUNNM0NIbzM5QlFpdTRTSmlXZWdXMDNOQmZSN1dpZXRtWXhHUjVYU0lqeFZ3bXF3NjhPdjFNbmdua3FNaW9lSjJMYmFjYmpCSjE2R05sLWhmNXYtMUE2a2JDMXZ0Q3d1WjREdWFGSG9FcjlhT2prQXZLQ3dlcFlLOEx5SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPekk2OFAwVk0tWG5ua3NUdkQzQXV0T1B1WHpraDZIckNOeWZ6dHpkMjRQc3JKb1pkSV9WMkltZkdzanVQV0VtNmRqRTBBNXI0TWNWRjY0SlpuUV9uTHFuaFctbEJ6cWRKYm1kc3hjejhTV1pXMU9hOV9GMVpYcERnc1VwWGRkakNqNl8tcENveENHeGFaZHZZWVZUalA1WHMtWXkwNGpaTGxUbTNwWXow?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,52 +2220,52 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46072.95348379629</v>
+        <v>46073.38811342593</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Politie in Genk rolt internationale oldtimerbende op: 11 diefstallen van Porsches en Mercedes tot 150.000 euro - MSN</t>
+          <t>Kildare woman who went on theft spree avoids jail - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Police in Genk round up international classic car gang: 11 thefts of Porsches and Mercedes up to 150,000 euros - MSN</t>
+          <t>Kildare woman who went on theft spree avoids jail - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 23:08:39 GMT</t>
+          <t>Fri, 20 Feb 2026 13:09:31 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxORWZKSzN2M2JUcFJKd1JPRFh5VUFjeEhxQkdPSjVfN0VkTnBsZGhlYTNFcG11bXVhN1FkM0JURDZ4UHhpWFRkb1FnSDFxaVhjQ3NYUGxXWnRqdmR5U3RROUdMVllxdE01d1g4YmdpX19ydjdRUndEUmhlLVcyQnZlNGtBSGVZaE9zQkVNY2ZyVEg1NjF2R2wweEcyQ0ZvZl82VmJScFE5SjZyR1A0bVR5SHowakF3a2lMRHQ5REdXSVZORU9CRF9jWnZXdjNOMlQ1U3lrU05pU1JLajVaUHZnMnBLdjYyRXRSZW13RXVjWmY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQclVHcWtrOEZBRVkwWmc1Zzc2VzRtYlJrek1hSnVnYzRUTjR6ejRJeGdhbnNtTXFGd2drdWctcFg1R01MOG5fY3ZBd2RMOUFSY2U0NktsQ0tnS2dMUE5OY1NyTmpLaTlGeHR4UExkdWNqMEZoLTZGbWEzcXVfSjl1YmVJazFiNEN3VVoxMC1DNXpGS1RQamhpZE5tM1N1T3BoY0RUakV2bXk?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46072.96434027778</v>
+        <v>46073.54827546296</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>TC Hasselt - Sept ans de prison pour des violences sexuelles sur ses deux belles-petites-filles - DHnet</t>
+          <t>LATEST: Approval for new 50-bed care facility for Kildare - Kildare Now</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>TC Hasselt - Seven years in prison for sexual violence against his two step-granddaughters - DHnet</t>
+          <t>LATEST: Approval for new 50-bed care facility for Kildare - Kildare Now</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:55:00 GMT</t>
+          <t>Fri, 20 Feb 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxQaHF5Vnl2YUlleldpV0kzTDJZZEtSM2ZJT3pOaWw0aVFxUFpiTGxJaXQ4ajlNSFlibDllVUpHeWhCcnY1WE9DbEdsMzhWb1VXTVJ0MkVBTFZ1NVpONXczUjd2ellXSlRGRWsySFNjdmt4Q1VTU1NPcWVfOG81WEtJcjhlUjFBcDVXSWl5alNXbHlCSjFMeVZUNFZiNFNJamZCS2pVLUt6UVppblVVUjhLeUFfbV9CSUY3OUVrQllHcFRrZDlmVEI4UEpXZWhoYzcxbURqZVR0RnBuenVnb2xhbmVYX2k5QXRnVXRUaUotYjBjWTItZzBxQmNxM3NjRUdaLUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPbExsSFlvZXFyanNuUkpoQzRGbDgtOHpleTd5Z05LVmdXSDM1SzJ2bFhLMG92RWZld1MzNEh3LUxIUEE0VEtWaGdLbVNDeExYa295cExfOWtRal85cGhKQi1XRWNnT00wS20zRTBaOHNuZmlBSGd5ZktrcmhwRHJOcXRJMEk1OU82WG9vektZU3JCcGpaR19OWnFSQmxlMUF0X1BsTmJQWjI4U290WmtDRjJR?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46073.41319444445</v>
+        <v>46073.58333333334</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Wertheim: 48 junge Beamte zu Polizeiobermeistern ernannt - Fränkische Nachrichten</t>
+          <t>TEAM NEWS: Dublin LGFA Senior Panel is Announced for Kildare Clash - dublingaa.ie</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Wertheim: 48 young officers appointed police chiefs - Fränkische Nachrichten</t>
+          <t>TEAM NEWS: Dublin LGFA Senior Panel is Announced for Kildare Clash - dublingaa.ie</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:00:00 GMT</t>
+          <t>Fri, 20 Feb 2026 12:05:44 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOVmx1X1F5RFNnSlRmakZ1d2dxcmtYcnJQWFdSeVlKWVBCMzE0Y3d6b1VSVTRPN1l5LWZPa2NGX25Gb0ktUEVxaEFnYkpHc1pTTHl3WTkxMHhrRlVnazRPcE9JcE1OaExlRHhEZ2ZRYkN4TWRSakg5VFdodHAwV0pRSHI2TlRLU1dXZjNXVDVEVDNULXI3amZuX0FLVEFCTWVDX05VTG16bE1WYWtkRVBoVXFkbUxmYjdzSlhTMEhsRzBKTDBFTGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNMTd1bndiQlVXcTAtUjV3aHZ0ZE9McEV3VGp2Z0wwMF94b2Q5Z21uaWRTZFZXQzJOZVVOMjFJTkhmYzE2OVRqQmpwSXAtbDVRVG41bGRFVnlmU252TVdNTjlPa3NSdDdwaXFjMnFUU05RVXIxem9pQ1pkWlJzNUhFMjd3azNIdTlfeDVtTG1uRlRfYnU4SWZneWRGbw?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46073.45833333334</v>
+        <v>46073.50398148148</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Würzburg: Mann greift Polizei an – Drei Beamte verletzt - inFranken.de</t>
+          <t>A new spin on Irish mythology: Kildare-based author to launch his debut children's fantasy book - Kildare Now</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Würzburg: Man attacks police – three officers injured - inFranken.de</t>
+          <t>A new spin on Irish mythology: Kildare-based author to launch his debut children's fantasy book - Kildare Now</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 19:44:00 GMT</t>
+          <t>Fri, 20 Feb 2026 11:05:00 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNUGNPS3lGb25GUm81THN3MUpqdmFYQUdDSmdyNXZhR2pMSFJTanpoNjhhVzJ0eVRCejZ5ZWxqTHduUEJINmZfa2JrS1h2T0VSeS1EaTlwd0UwYWVIYkstR3NqaDN6RTBidTR6YkppOEczbzFwWGdmenF4M0FyanQ5WXFsdldWTmNBZHNyLTVSV09nR1didmNzaE5qNFJ3a04zUjdyZHEzUkRWWlBJR0MwWU93a9IBswFBVV95cUxNUGNPS3lGb25GUm81THN3MUpqdmFYQUdDSmdyNXZhR2pMSFJTanpoNjhhVzJ0eVRCejZ5ZWxqTHduUEJINmZfa2JrS1h2T0VSeS1EaTlwd0UwYWVIYkstR3NqaDN6RTBidTR6YkppOEczbzFwWGdmenF4M0FyanQ5WXFsdldWTmNBZHNyLTVSV09nR1didmNzaE5qNFJ3a04zUjdyZHEzUkRWWlBJR0MwWU93aw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNNlQ4bXZjaGp1VG5KNjUxSFhzZFhVZXV2NDEzR3BqX3lVUS10NW9oYWx4bjRNYndyczhudXJ3NFhjWkNhcTlQOXNwQjBUMl96NGZqaGo3eUdqM3hxQlBBbDN3bTNhQVBlX0pTSnRhTUhSMVFVX2NEYmlDS3FzQ3hqTTBvQjBiTWpvblNva3YyTWthXy1NVDVOWnF3dTRtUlF6RlowNlpEOUVwOVZSR1dDdWo0SkpYcUpQeTBlM2VHbDNGQlp4OWZXVmYzVGNLOEVMQklTV2NyNkdVV1l1S1k1aUg2ZS0?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46072.82222222222</v>
+        <v>46073.46180555555</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Telefonbetrug in Würzburg: Warnung vor falschen Ärzten – Schutz-Tipps - inFranken.de</t>
+          <t>Kildare student represents county on Gaisce Youth Ambassador Panel - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Telephone fraud in Würzburg: Warning about fake doctors – protection tips - inFranken.de</t>
+          <t>Kildare student represents county on Gaisce Youth Ambassador Panel - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 19:37:00 GMT</t>
+          <t>Fri, 20 Feb 2026 14:01:22 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPcjg3N21MakkzZHJTNldnLUhBbHhHdm9lT1EybVdaTlZUbzJrZ3pxS3ZzV3YxbWd5TjZLWTdpcG1CSU9pV0djTXNaVDhKVVRfYmJDOVJhNzViY1dlNmM4Sy02cHRqbWdpOFppTlpqZHphNEtBWUh6VzFGeHM4cUlncGExelJVanp4M19LYm5VdGNuNkhCdEhlN0ozSnlhV0RfRTc2d3h1U253Z3NjUll0MmJuTG5lNDZ6RzVSYk55Mm1sVEoxUkdR0gHHAUFVX3lxTE9yODc3bUxqSTNkclM2V2ctSEFseEd2b2VPUTJtV1pOVlRvMmtnenFLdnNXdjFtZ3lONktZN2lwbUJJT2lXR2NNc1pUOEpVVF9iYkM5UmE3NWJjV2U2YzhLLTZwdGptZ2k4WmlOWmpkemE0S0FZSHpXMUZ4czhxSWdwYTF6UlVqengzX0tiblV0Y242SEJ0SGU3SjNKeWFXRF9FNzZ3eHVTbndnc2NSWXQyYm5MbmU0NnpHNVJiTnkybWxUSjFSR1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOd3lPbGJWMkdJdVdaR0FHU253VUQyYWtkMnV6UFVWWTB3QVpPN0hReV9LZ1NRWFpwRGZMWFRMN2JHdDNYTXBhM0JIVm14MmxqOTAwanMxb3gybkd5emd4XzBUSmdGQWFVZjItZXE4REg4Umd5bE9rOGxnd1Y1c0FlQXRselBoRkxkZGgzMUl5WGpxdUxRb3o3NkhqejI0UFAzU0xyR3liblJFUGw5MEh1WmxhU2d5OE9feHJvUFYzdw?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46072.81736111111</v>
+        <v>46073.58428240741</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Great news for Kildare house hunters! 24 new properties get green light - Kildare Now</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Great news for Kildare house hunters! 24 new properties get green light - Kildare Now</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:52:05 GMT</t>
+          <t>Fri, 20 Feb 2026 10:26:00 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOWHlfdkVaZnhqWkFoXzBNaURZcG5MX3cxamJNTzkwOThlQ2lmSEx2VzBVQVp6YWZjN19YX2lyY3Z1YTBNbWhMUWlLRUwtZjlJbGFGaG9iakFHdU5KVG9zZ3JjUDM3VVoyelhVVEo1Nm9ycThXQUk1bkdjR3oxSzI4d3BnUXlyc0RaQnlPN2lrZDFkRENwR3pYenZQNmMtMFdraldPb3liWmN2S3VrU2RlbGhQbDlJUndaaGhXckt2M3FLYWx1?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46073.53616898148</v>
+        <v>46073.43472222222</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Rund 110 wetterbedingte Einsätze in Unterfranken - aschaffenburg.news</t>
+          <t>Bus stop between Newbridge and Naas is ‘a mud bath’, Kildare County Council is told - Kildare Now</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Around 110 weather-related missions in Lower Franconia - aschaffenburg.news</t>
+          <t>Bus stop between Newbridge and Naas is ‘a mud bath’, Kildare County Council is told - Kildare Now</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 22:01:01 GMT</t>
+          <t>Fri, 20 Feb 2026 09:35:00 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQUmFOa1RCM0dXaGFGaW1oTkw3RUNvbEZfQXJiT2oxNFVXdlJxaEoxaFczeXZ1NWo3MlAxNW9YenhGWWlHblJBRmFIa0Rpc2t0M0hhNEpVYVoxS1hEOGw1S25faGpUZTVwblV4VkZTaVVubjJRMTNTSmVQX3U3VXdvNnJ5bWtOc0tmRjNnakpyQ1o3YnJtQnpZRzVB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxON2daWDdiY3FuQWdJcUNjRFJHQ1FlZ3luX0o5OGJaNDlfSlFRSVZVVi1yTVh6bVJXMUxPOENXMDZ5OWZUcmN0cjVPTjhKTEYwSjVfTHl6Y1ZPZVpLU2w2WmxxRHZ1RGw3LXF4Q2U5Tkx4QWdTX1ptY0VNRTZsd21KSWNWNHh6VkpDOVBXMlhIRDBRMmhmVFhFdmtKYlhpQzQzZV9yQ2U3ejhIaUQwWnppLVUxX3RCekdHRnc2NWx6QUpOOW9wbVltMFJVdkIwX1NSN2c?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46072.91737268519</v>
+        <v>46073.39930555555</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Würzburg : Vandalismus und Schäden in Berner Straße &amp; Elefantengasse - inFranken.de</t>
+          <t>Kildare Death Notices for today: Friday, February 20 2026 - Kildare Now</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Würzburg: Vandalism and damage in Berner Straße &amp; Elephantgasse - inFranken.de</t>
+          <t>Kildare Death Notices for today: Friday, February 20 2026 - Kildare Now</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Thu, 19 Feb 2026 19:43:00 GMT</t>
+          <t>Fri, 20 Feb 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOUk1vb2x5dllGS2djUHRoNmFrWWVQMnJQUzYzeFZvNERKY2ZyUklwbFlYV09SUHdoN2xJaEhySEF1SU9WZ3E1SEN5cEl3RVh6TE5EbHBraW1PTzZEMk9uLTRZTjdpXzRMR1RDZEx3clYxa2F2S01RSkdxbkpNTFgyemRxTFBDSXJTSXM1X0ZPVks2THUwcl9xTUx4SlQ3djM4enhoaUkxdDNVVDZ2WkxqLW40TER5WXNiZVJVZmpsVWlDOGs2NVHSAcYBQVVfeXFMTlJNb29seXZZRktnY1B0aDZha1llUDJyUFM2M3hWbzRESmNmclJJcGxZWFdPUlB3aDdsSWhIckhBdUlPVmdxNUhDeXBJd0VYekxORGxwa2ltT082RDJPbi00WU43aV80TEdUQ2RMd3JWMWthdktNUUpHcW5KTUxYMnpkcUxQQ0lyU0lzNV9GT1ZLNkx1MHJfcU1MeEpUN3YzOHp4aGlJMXQzVVQ2dlpMai1uNExEeVlzYmVSVWZqbFVpQzhrNjVR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNSTFFSkdXdUJsYWtmMHloQ1QyOUNQc3R2UngtM1VQZElxOWVzYm9BeGg4WTF2dkxIdGRKUWVUc25hdUZob3dOX25wSUxhcHJVM0ZsekVQRHBITjBxeHhpV2hRNXcyYkprRzJ6MUlpaUJ1SjhSUUgydmJoazg2MUhxRDFpcWdLZGhLNk1iZXpFb1N2R3R4eE9zMFVnbFpLSnRFNVJWc01tQ1kzX2s?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46072.82152777778</v>
+        <v>46073.41666666666</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Polizei-News Bamberg / Schweinfurt / Würzburg, 20.02.26: Zollamt Schweinfurt intensiviert Kampf gegen Schwarzarbeit 2025 - News.de</t>
+          <t>‘Unprecedented’ demand for jewellery helps retail sales surge in January - Bicester Advertiser</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Police News Bamberg / Schweinfurt / Würzburg, February 20, 2026: Schweinfurt Customs Office intensifies the fight against undeclared work 2025 - News.de</t>
+          <t>‘Unprecedented’ demand for jewellery helps retail sales surge in January - Bicester Advertiser</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:54:02 GMT</t>
+          <t>Fri, 20 Feb 2026 13:31:56 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPT0gzcXJvcDBRa3pZM3AxVzlTeldTSVU5aGVZSmMwclE3STQ1RTE3c2RXNW9abjg1QXY3ZTQ1UWs1ZVUxX0o1R1BITEdWYmVncXd5aXB0MnlrcG5YT29DS1JTQ3pnb2dBMEZ2RU1kUTV6THlBeXlUejJjTlV1cXpZS01YRUU2a0ZEWmtTdUJRQTQ5eFh3THEtU0RnOEdaV2dleUltLXpSaHRtZUxRdlFV0gG0AUFVX3lxTFB1WmM1eFdVSHVJTVVXN1F4dTRsRkpaaTVWTFZxVWVwMG1JdENPelhXVndjX01Gb3p1NndvblN5WjJPTWdUMG52eFcxOWxDenRSWnBvb0tCUllITTJyNmZDR2t0S2lqbnVnZ2dBMkhIRnBOLXNpbmZ2bnJ2b25IOEtoSmROUDlfajRpLW11Z01lTzUzS3VGZS1oTHZybmxBYkFXdmszQXdtRzJ0Z05lOHozNGFuSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPV2w4cTNCTFlMZlA5R3d4VklDNDVJVUJGWFVKSHlDVHVHYV9HQTRwLXd2SUFvckladTMwbzFlUHl0Y3g5M1FzM2NrLUxEWHg2TlNqRGZ0UXJic01oNTJrTWJ2OTliaHZZcnpta2haVkdIMkFMc1h2Z3FsTjRHekU2aUJ5S3A0VmlkOE9ia3BJdHZqRG5CbmR6MUt5ZVc0MzZrYk1vc3pkRzdGcVB4QmhjWGR5c3pTX2VsU09LNTJiOA?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46073.41252314814</v>
+        <v>46073.56384259259</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Aschaffenburg aktuell am Freitag: Hier nimmt die Polizei am 20.02.2026 Raser ins Visier - News.de</t>
+          <t>Riverbank Arts Centre and Kildare Jazz Festival announce Hayley Kavanagh as the 2026 Emerging Act - Kildare Now</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Aschaffenburg currently on Friday: Here the police are targeting speeders on February 20th, 2026 - News.de</t>
+          <t>Riverbank Arts Centre and Kildare Jazz Festival announce Hayley Kavanagh as the 2026 Emerging Act - Kildare Now</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:15:45 GMT</t>
+          <t>Fri, 20 Feb 2026 13:30:00 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQNkVuMENSQnJIdUE5ZUpFWWJRNHZVeEVXcHFMQVRwQ1hub2V0Q1VmdDZtS2hsSDQ1d2JiUjhrTW11bHZjWXcxQ0tfNmZpRUdYVHY3OTlzblhSMUVKNmU3THJFdXhNTTd1SGczbjdwbmJDWjNOLS1femx5UjJpUmR5NzNsN3EwWGI2Q3Frb2RESlNBcF9wcVM0WnN0QUdYQ2o2YXJQTDQ5ekJ5bEtFYjlxZlBkOGVUby1lbzFqbXJqMjNVdU5oMEZNZFRYNG5NY0txbFNrUTdNOWJmX1ZibzRtZkN1UC0wVzI2V0hua0pFcllSbFAtSVRn0gH8AUFVX3lxTE90amswVGNHQ01Odnl5TkpmNkQzd2laX3VMSXJjaXQzU3JRcGlfbnJfUi10LWlSM1JjM29KSWIyanFZWnNtcHN3Xy1KOHFIdWRRN2EwUERsWHVrZTZKaWc1bENIdHpGb1Ztb1pKNGNkeVZnQ2lnTi0tRWZlVERwNW5aWGhLOFVPMG8xWmF0OXYtd1QwLVJjaTdWU3hqRkIzV0pRSWk5eW5KelRnbE5IM1cwQ1hDQTBNWko3bS1kdkdPR3V1N09IVEpKRHNTNnhNUFdZUlBCM01oSlFIMlNBMG1SbzRxM1hIVjh5ZG9fNlJGdkU3TU41WXEwUG13SA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxNT0xWZElNc1lMTS02WWIwU21RemFTUmpsYVEtSTdTc3NZdW1NQzdVTExzNzlWMExCU1dlajluQzZjZmItdlA4TlJ2T3JRSnZ4MXp1YW5VOTNTSnBTblJja3IyLURGV2pYY0RDdkRZX1QteFVJRHdZNDFuVHZVcmdzcmhKcUhhcTE1TzFtYk9aRGw0azZNMmdFZE9xRldYajFXVG1FN3NZSTVvYkV5c0ttMk9rOHVZS2o4Nk9PSkJvVjR1alE3dW1NZUItZW1aZW9INEJXdTg2bE0zcTFVc0k0a1Q0OTRIdWla?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46073.55260416667</v>
+        <v>46073.5625</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Polizeimeldung Bamberg, 20.02.2026: Einbrecher entkommen mit Tresor - News.de</t>
+          <t>Cautious optimism expressed over Kildare bridge project - Kildare Now</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Police report Bamberg, February 20, 2026: Burglars escape with a safe - News.de</t>
+          <t>Cautious optimism expressed over Kildare bridge project - Kildare Now</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:35:02 GMT</t>
+          <t>Fri, 20 Feb 2026 15:05:00 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQTDRVeGxRTzBmZ200OEl2d2huS2VhcFZvTWxucWc0VVhaQkJzak96dW51NEt3V2g3SC1INEZmWXdjbDBVbVRqeDl0NDBqYzJZSHV6Vllwa1NXbC1YRGRLWkpmbWFKdFBHSW5WWVFLQW1vb3hfeWIyY2R1bm5EUllUTkRtLW5iQ3phV3pNSjF0S3dyYS1XZzZkOTd6NG9UWFY1c3Qw0gGoAUFVX3lxTFBlLXFyeU1ONEpmNEV5bFpuQUV6V0lhazdlY21XUFpZaUpVUVFEUVBGbjItWEJaX3ZxWVZpSW1UczJCak9DNkxiMW9NTFhZeXhDUmR0R3M5WGFJbjQtUjN5TldKbkdZOVIyVTVKcUZJd2VHdjdBektOT2ltZ1VwREZDSmFqWVdKeXVBbEhZcGRZYXAzTjhDOW5wX1o2d05SU3RwOTdCSTk4Xw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPVjJER2xhQ2VUa1owNjFaMWRKVnpFcnVoZ0N3UjVlcHhIWlJ3N0VyelU0WDZlNkdLMVlQX3ZvVkpiTnhELTBodGk5Sk9wQzR6eGxtQ3QtSVVXZlg0NGhqdkhSQlVaWU9laktQQ2JRNTl1RVRwQnlJX0lJS1QzQ2IwcmpSQ0h5UmVKR1Q4MGJYY19aRW5ZSHRGdGU0dDQ4a1J5RDhiOFZFMk5MOVF1QnFnRw?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,52 +2825,52 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46073.48266203704</v>
+        <v>46073.62847222222</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
+          <t>Sadness as long-standing Athy business to close - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
+          <t>Sadness as long-standing Athy business to close - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:02:00 GMT</t>
+          <t>Fri, 20 Feb 2026 14:24:33 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPdkVfYlpLQ2ViMnBuUy1hUUtTYUhZbFhiUlNHeUJ2cEkzT3QtWEdBcHRDS2tnZ0dWSVBSZ2tGRnUtYjBHbnB5eVN1Z2gzWUtlZVNTZXR3UFZiZDBsQ1NaRWJlNEcyNHlUbWhiNDNlMjMtMjJkaHZKVWtOVGJ2OG9mZm1qWmVRWkFQaGRSaXlnSGM4NzhuSlkwcWplaTF2dXVHMGZjVHZzSWxtdW9ZWmtnNkpVQTVHZjlaMVRSQ0FKR0lWT01zcVROVi1nQnl1NV9NR2p3ZkI2X05Ua1k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNVEN3ZVJBblhZYjJSVUlOUEl0cG91WGxRMGt1X2FtUEdEWXJfZkctREVMWHYxOF9Kd3pBMkNiTzA0NGlTNi1obnY1N3BQTjRieUxhMTRhSDNLTDVBWjNxdHpwUTZBQy15dTI0QTJ4eGh0alJ4Q05TZFplYkVnWTAwZGZCQkowbEo3ZnFReHdIR0Z1Unc2VDZnTld2V2VnQ2FHZ1VtRkVB?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2894,38 +2894,38 @@
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46073.41805555556</v>
+        <v>46073.60038194444</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Autobahn gesperrt: Getränkelaster rutscht in die Leitplanke – Unfall auf A93 - Augsburger Allgemeine</t>
+          <t>Plans granted for residential development in Athy, Kildare - Ireland Live</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Motorway closed: drinks truck slides into the guardrail - accident on A93 - Augsburger Allgemeine</t>
+          <t>Plans granted for residential development in Athy, Kildare - Ireland Live</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:46:49 GMT</t>
+          <t>Fri, 20 Feb 2026 12:33:30 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQb2RxcW1rQ0l1LWN0UnJ6c2RNXzdPdGJwbW9IWjlSN3czX1NaRE9LSGIyZ0JuRi1aWTFrVFBHTEdmaFdUZXZ3T3NRcmI3dHp3WkF6NGYxeUtjLS1XUlZROW5jcG0tS1lCdEFGZl9ibi1VLUFoSjFnS3pmc3E3VDdkS2JBNWRUX3hhU05qcThTM29hWTFXLW5temVmR0w0QzBsbWZKeFJtZnZlUjE2YVNPVXpMVWZWNlN4MHFFY0h1Z0lkX2VvVnhuNHBxTnV1dWxKR0NBZDcyQjVyRFVMM3NDRw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPNVpadk9wS3hjS2dUTmp0dmJ2T0JLTlhiLUhybFk1X2RSS3FMU29ZZFc0VUNaODNRQVZqYjhYRVRtSDdycWFZNXMyUkI2X1c5ZEUzNGRkWjA1RWdReDZzQnA1U04tRGo4U3pLMkdEWFZlOXV4S1lYclNYRkMxTHdiY0NGeng3RmRaVGF2TlY3Z0tXaWpwUVhLRDVTOUZiREgxY1gwTnJBUlF3ZDNTSmNZTVdzSnBSdw?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46073.44917824074</v>
+        <v>46073.52326388889</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bayern: Polizei- und Feuerwehrmeldungen am 20.02.2026 - Newsflash24</t>
+          <t>Home from home for Byrne’s first pro fight - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Bavaria: Police and fire brigade reports on February 20, 2026 - Newsflash24</t>
+          <t>Home from home for Byrne’s first pro fight - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 08:46:00 GMT</t>
+          <t>Fri, 20 Feb 2026 11:51:12 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQNmd1b2lTdTQwQ003YVZEc0RlQTFpRHBkcVUzNnU4OWlkOXpHbXRwZF9QUTEtU0FvWVoxQW40SUgxRzVIenoyLUdES3cyX2llYnBvOE1qRVByeDRXWTRTN2syT1IzbFJZSndCZlJManFkbjhVc3ByVV9BcVM1Y3dlUjlFdW02d0hOVW9nZnZPQnJZdXpTaU9r?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOcFllajRWcUNjNkZLTjVZdGNSR21TR2VvYk5ISUlza3JlNEVsRGxmcWVOVm9nR3piZjVmc0djMS0yM0V4YTJjUmJKSEdHWEZqWTRrbm1EM21EWG0zRkY2QlI3bmZpcjRXdXBFQTEwenhuUi03aDFScmI3THRHcnpFM1BTNmhtTnJxMlpWaGltdXZna3h0cGJiVnE4X0ZQUQ?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46073.36527777778</v>
+        <v>46073.49388888889</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
+          <t>TII urged to discuss controversial Kildare cycleway project with councillors - Kildare Now</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
+          <t>TII urged to discuss controversial Kildare cycleway project with councillors - Kildare Now</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:30:00 GMT</t>
+          <t>Fri, 20 Feb 2026 13:05:00 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPQmRWY0VOQzRiY3U1amZfOUIwSVplbGFjTkpXUGxfQ25IWjQtWlMyN1gwcmMtVm1LSnNBMzFGYnJaYklsMG1RdG15R2JBVWFXcHF3R1NGUmZGcHpUSGFnb0RhdUZVXzBCMlJKbWs1ODJ6WHY0Si1rMkRXZmVUaFZZU2lCZnNzUnhWdmQyaXkySmJ5R0l6QlBqV04wMTMtVHJKZW5oN05PT3RtZktCNWVyS2pYYUh0UGZ3RVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOdzVpNUNBTVJnOUtlQ2NGUVBYaWxiXzZSeHZRbmptX3l2dFVacHBMYk8weldFcEFCaEVLTnlDamgzTkw2a1RwalJ2SkdnbGpJeW92Zy16UXByV1lWSXBhQ0Z6eG5ya18tNDYwblkwa0hVS1ZxYjBqX00tNjBNUnpCdDQ0VDVxbXhVWW91U05WRElHdFpySmY5SE53VnFGWm83RlNSY2pQNjlxYlBLMXJ3TWlRSm5BM3FoNHJZLWlLMXhBTTV1?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3059,1052 +3059,7 @@
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46073.47916666666</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>News: New Audi RS 5 PHEV: Up to 639PS/825Nm, 8-speed gearbox, quattro AWD - CarSifu</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>News: New Audi RS 5 PHEV: Up to 639PS/825Nm, 8-speed gearbox, quattro AWD - CarSifu</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 08:33:41 GMT</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQdkNzSEZZZ1BNdE4xZm9KZjM0blhjdnZscWtHN25CWkQ2eS1QWjBrRjllMHNXNG5Ba3BFQmRPZ2hFUm1uNmE1aHJTck9QQ1NYX255YTBPUVU1QllZTlZoaC1Ed1Q2NGlEbVM2T2ZCUVNoUTZad3dqN3NZZHBCNWpwcFFxZkxqT3ZEZEZCamxnX2lDYnN5S3ZUQg?oc=5</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K49" s="1" t="n">
-        <v>46073.35672453704</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 09:18:53 GMT</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPekk2OFAwVk0tWG5ua3NUdkQzQXV0T1B1WHpraDZIckNOeWZ6dHpkMjRQc3JKb1pkSV9WMkltZkdzanVQV0VtNmRqRTBBNXI0TWNWRjY0SlpuUV9uTHFuaFctbEJ6cWRKYm1kc3hjejhTV1pXMU9hOV9GMVpYcERnc1VwWGRkakNqNl8tcENveENHeGFaZHZZWVZUalA1WHMtWXkwNGpaTGxUbTNwWXow?oc=5</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K50" s="1" t="n">
-        <v>46073.38811342593</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Kildare woman who went on theft spree avoids jail - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Kildare woman who went on theft spree avoids jail - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 13:09:31 GMT</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQclVHcWtrOEZBRVkwWmc1Zzc2VzRtYlJrek1hSnVnYzRUTjR6ejRJeGdhbnNtTXFGd2drdWctcFg1R01MOG5fY3ZBd2RMOUFSY2U0NktsQ0tnS2dMUE5OY1NyTmpLaTlGeHR4UExkdWNqMEZoLTZGbWEzcXVfSjl1YmVJazFiNEN3VVoxMC1DNXpGS1RQamhpZE5tM1N1T3BoY0RUakV2bXk?oc=5</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K51" s="1" t="n">
-        <v>46073.54827546296</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>LATEST: Approval for new 50-bed care facility for Kildare - Kildare Now</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>LATEST: Approval for new 50-bed care facility for Kildare - Kildare Now</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 14:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPbExsSFlvZXFyanNuUkpoQzRGbDgtOHpleTd5Z05LVmdXSDM1SzJ2bFhLMG92RWZld1MzNEh3LUxIUEE0VEtWaGdLbVNDeExYa295cExfOWtRal85cGhKQi1XRWNnT00wS20zRTBaOHNuZmlBSGd5ZktrcmhwRHJOcXRJMEk1OU82WG9vektZU3JCcGpaR19OWnFSQmxlMUF0X1BsTmJQWjI4U290WmtDRjJR?oc=5</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K52" s="1" t="n">
-        <v>46073.58333333334</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>TEAM NEWS: Dublin LGFA Senior Panel is Announced for Kildare Clash - dublingaa.ie</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>TEAM NEWS: Dublin LGFA Senior Panel is Announced for Kildare Clash - dublingaa.ie</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 12:05:44 GMT</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNMTd1bndiQlVXcTAtUjV3aHZ0ZE9McEV3VGp2Z0wwMF94b2Q5Z21uaWRTZFZXQzJOZVVOMjFJTkhmYzE2OVRqQmpwSXAtbDVRVG41bGRFVnlmU252TVdNTjlPa3NSdDdwaXFjMnFUU05RVXIxem9pQ1pkWlJzNUhFMjd3azNIdTlfeDVtTG1uRlRfYnU4SWZneWRGbw?oc=5</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K53" s="1" t="n">
-        <v>46073.50398148148</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>News - Kildare County Council</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>News - Kildare County Council</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 15:54:20 GMT</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQaWJJUkp1R0JtbUJsUmZNTncxLUR1V1ZLZ3pJV2JlWklJcEcyTDM1Ry1jNFZKc1BOVkk1YjNxQkZwLXp6SG1IYWIzalMzSHo4NExpbWNfOXNPNDktUmN2Q0o3TlhxUU1DdUM0WW1hc1dYTmFtenhvMlh6M0dpeUVWV2lOc1ZpUUFUTTR2cWJ1U2dVUWxFb0dfWWcyNG83UzNBYTZLbGtjdVJYSDg?oc=5</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K54" s="1" t="n">
-        <v>46072.66273148148</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Kildare student represents county on Gaisce Youth Ambassador Panel - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Kildare student represents county on Gaisce Youth Ambassador Panel - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 14:01:22 GMT</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOd3lPbGJWMkdJdVdaR0FHU253VUQyYWtkMnV6UFVWWTB3QVpPN0hReV9LZ1NRWFpwRGZMWFRMN2JHdDNYTXBhM0JIVm14MmxqOTAwanMxb3gybkd5emd4XzBUSmdGQWFVZjItZXE4REg4Umd5bE9rOGxnd1Y1c0FlQXRselBoRkxkZGgzMUl5WGpxdUxRb3o3NkhqejI0UFAzU0xyR3liblJFUGw5MEh1WmxhU2d5OE9feHJvUFYzdw?oc=5</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K55" s="1" t="n">
-        <v>46073.58428240741</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Great news for Kildare house hunters! 24 new properties get green light - Kildare Now</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Great news for Kildare house hunters! 24 new properties get green light - Kildare Now</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 10:26:00 GMT</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOWHlfdkVaZnhqWkFoXzBNaURZcG5MX3cxamJNTzkwOThlQ2lmSEx2VzBVQVp6YWZjN19YX2lyY3Z1YTBNbWhMUWlLRUwtZjlJbGFGaG9iakFHdU5KVG9zZ3JjUDM3VVoyelhVVEo1Nm9ycThXQUk1bkdjR3oxSzI4d3BnUXlyc0RaQnlPN2lrZDFkRENwR3pYenZQNmMtMFdraldPb3liWmN2S3VrU2RlbGhQbDlJUndaaGhXckt2M3FLYWx1?oc=5</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K56" s="1" t="n">
-        <v>46073.43472222222</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Kildare gardai investigating theft of vehicle in Kildare town - Leinster Leader</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Kildare gardai investigating theft of vehicle in Kildare town - Leinster Leader</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 17:32:37 GMT</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPcVF4c1pZdklyZnNtdnF1VHpwX0JhTnFIWHpubVFmR1AzaWhLSHFoRHItZmJ1aUtzNUtoa0dCOE54N2tLdmxhSEZidjBnZnlIYTJyYVpoNlVkcXlCUjhqMEcwN0JYR1o3bDF3RENDUlByWXV2MnN4ZDYzY1JrS2hnRDEyc2tqRk1xd0tUQXA2d1loT1ZLQTlCLTk0OG8wa1FtM2pmN2c0R0lCZTJGMDBtaHliTDEya1Z1V3UxSQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K57" s="1" t="n">
-        <v>46072.7309837963</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Bus stop between Newbridge and Naas is ‘a mud bath’, Kildare County Council is told - Kildare Now</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Bus stop between Newbridge and Naas is ‘a mud bath’, Kildare County Council is told - Kildare Now</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 09:35:00 GMT</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxON2daWDdiY3FuQWdJcUNjRFJHQ1FlZ3luX0o5OGJaNDlfSlFRSVZVVi1yTVh6bVJXMUxPOENXMDZ5OWZUcmN0cjVPTjhKTEYwSjVfTHl6Y1ZPZVpLU2w2WmxxRHZ1RGw3LXF4Q2U5Tkx4QWdTX1ptY0VNRTZsd21KSWNWNHh6VkpDOVBXMlhIRDBRMmhmVFhFdmtKYlhpQzQzZV9yQ2U3ejhIaUQwWnppLVUxX3RCekdHRnc2NWx6QUpOOW9wbVltMFJVdkIwX1NSN2c?oc=5</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K58" s="1" t="n">
-        <v>46073.39930555555</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Motorist arrested in Kildare after driving 116kph in 60kph zone - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Motorist arrested in Kildare after driving 116kph in 60kph zone - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 17:29:40 GMT</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOSnhrWm1Vczk1d3dsVnFhUDR1U2IzWlNDZXhvTjJrT2wtYUY0eGlFelYyTi14NzdJcEJIQnpyUUlWeGljbDRkWXVNd3JpQTJWNzRqSVlRSnhENXpnRXMzUmlsZlgwdVJfZ0ZDcmNETTdwWTZON2R3Vl9FVzBWbEduaXNsQThlWVZaQ1VxRG8zd0h2UXVRV2R4dGJiblhQLXNtZ2EwVG1TOVlWTmRpVWl0d0ZRZDR4MWJUbVRn?oc=5</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K59" s="1" t="n">
-        <v>46072.72893518519</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Kildare Death Notices for today: Friday, February 20 2026 - Kildare Now</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Kildare Death Notices for today: Friday, February 20 2026 - Kildare Now</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 10:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNSTFFSkdXdUJsYWtmMHloQ1QyOUNQc3R2UngtM1VQZElxOWVzYm9BeGg4WTF2dkxIdGRKUWVUc25hdUZob3dOX25wSUxhcHJVM0ZsekVQRHBITjBxeHhpV2hRNXcyYkprRzJ6MUlpaUJ1SjhSUUgydmJoazg2MUhxRDFpcWdLZGhLNk1iZXpFb1N2R3R4eE9zMFVnbFpLSnRFNVJWc01tQ1kzX2s?oc=5</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K60" s="1" t="n">
-        <v>46073.41666666666</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Blow for Kildare as Beirne to miss Cavan showdown - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Blow for Kildare as Beirne to miss Cavan showdown - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 22:19:01 GMT</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPeVJlaVhUZXNzd0s0NzNFVld6MTgwZVdidlRXejFOVnRIRFdhVjY0Tk5MVjZTVkk0bGU3LWhsWlZXMDZSZk9DRXVKR1pyRlc3bVBvQ0lzcWowbkxwajdxN2FHdldNOG9BQm16TGdJejUzT3lPRERJZER3V1FnbWpxT3dNMnMyTExGNlhpZ1ZLNnBpdFYtN05xcjBjM0JtaHVSYUs0YzVLQ0g?oc=5</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K61" s="1" t="n">
-        <v>46072.92987268518</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Sport - Kildare Now</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Sport - Kildare Now</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 18:06:00 GMT</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE9TR2hPdDFDS2RUU2E4WFEzYXBZQVpkd2lvQ1NlVllWMkQwd3MwSXdQUnhsVmhJUjI1b3k5RjBwUmNZRDZkSXUyNHNSd3Q3Nkl1YmR0U2RTVQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K62" s="1" t="n">
-        <v>46072.75416666667</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Kildare country star back on stage after heart attack - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Kildare country star back on stage after heart attack - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 20:14:36 GMT</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPS0QxNG0wV3o4dzJ2SnVuc3JKYTd2SU9fVTdyUmpkZTh0b3FpZEFtR1FfbnYwZUw3SFBJTWNmWktiWUk3XzNFRnBoVl9jd1ZfUjZUUFFKZFNUb1gtSGtYODR6OWlWZHZKYzdBS3g1ZnFGRUNRYWRsOE1nMUpqaEZQYXdkT19Tc01DaTh5MlFTdktTRFpGSHBiQmx2ZnI5SGhJdmJ1Qi1EXzJ1dnFYWUE?oc=5</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K63" s="1" t="n">
-        <v>46072.84347222222</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>LATEST: "Buried car" among lines of inquiry at Deirdre Jacob search on Kildare border - Kildare Now</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>LATEST: "Buried car" among lines of inquiry at Deirdre Jacob search on Kildare border - Kildare Now</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 16:59:00 GMT</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNZlkyRFh3M1YySzZIMjNRY2QzeGN5WHpXUVFKcmR0V3htQXpjcXdsaEQ1UExyQTBKVm5abHB6Q19Vck1LWU1XeE1fdTZqdnNuYWZRSkRYU1pkWEJsUXJrS2w0cWJybGEwOWhZdi00VGU3YWFtOU92OHJXM1FvR3JveTQ4c0RodzdTZGtqSEVnX3JuNjc3THJZclBlYTUyN3ZQT09qYjJxeHJnd3NJZUlXRmE5VHhOMWppMWtsOHJ5NExabi1WQTFnTlRUZw?oc=5</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K64" s="1" t="n">
-        <v>46072.70763888889</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Minister visits lauds battery storage centre near Kildare/Offaly border - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Minister visits lauds battery storage centre near Kildare/Offaly border - kildare-nationalist.ie</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 16:08:53 GMT</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNTno0TXZzdnlTZHczNUQ5Skk5cUYtVFNoalg1dGw5Z1ZfeTYyZXFHYV8zTjFBYkg4ZmFKRElQUmU2OHNSSVJqUmg0eVJTYnVWRnVsSVZKVjNPUEZUQjZ0VG1KQnB2SDZ6MDNnTUJWMGdkN0dhZ2ZtRk1NSmVxbVpkQkdCOENhalAxem1BY0FuOC1ScWlIbHRNVGlwVmdyYkdtNjdNQll3Y0Z5Z2JWdnFXRFlyNmRHUXZMU1NwUmdrWTdmZjdMeEE?oc=5</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K65" s="1" t="n">
-        <v>46072.67283564815</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare (fallback)</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Stagecoach Announces Bicester Bus Service Improvements From 22 February - Oxfordshire Guardian</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Stagecoach Announces Bicester Bus Service Improvements From 22 February - Oxfordshire Guardian</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 18:06:47 GMT</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPVWlOajUzaFJTVWZuUnl2UmRkZ1VsdDMzUzl4YUFJeHFCWUZMcUJjM0RuR0JnVWRNYWppZXp0R25pUmJTd0hYVlQ5LXFoQmlZcS1OZnFLWHBWcWpJaGJESUlmb0o2aHNVekFrR2ZJWkRfVGkwRS1ESjZzbzFRX1RZTy1rRFY0NFhSYzY2VkJyRW12SF9ZMWo0TjZ1d1dNRDdzSEduSm1lU24yQQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K66" s="1" t="n">
-        <v>46072.75471064815</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Sparatoria Rogoredo, si rafforza ipotesi omicidio volontario per agente - Sky TG24</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Rogoredo shooting, hypothesis of voluntary homicide by officer strengthened - Sky TG24</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Thu, 19 Feb 2026 20:02:21 GMT</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOc0NHMVh3emlvNnh4S1NKOUk5Q0RJaGcxM2FoUVcxRXRHbTVOcWt6cUhsYTFfRFlTT250azZMdnpuV2IxNnZueEt6NS16SWN6VmN4eS04NXg3QlZxU3dlX0hwanhhMDJLeDNubXRoMHN2d0FRdWIzLTFqbU9GRTlIYXdQN2pMaWVtMzRseVFR?oc=5</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K67" s="1" t="n">
-        <v>46072.83496527778</v>
+        <v>46073.54513888889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-21 14:27 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M £20 'sleek' laundry basket nearly half price of B&amp;Q £39 'elegant' option - Essex Live</t>
+          <t>Steinhoff's Business Report: Adapting to Market Challenges - Studocu</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M £20 'sleek' laundry basket nearly half price of B&amp;Q £39 'elegant' option - Essex Live</t>
+          <t>Steinhoff's Business Report: Adapting to Market Challenges - Studocu</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:56:22 GMT</t>
+          <t>Fri, 20 Feb 2026 20:16:22 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPWHpaMVB3R3B0VjN2ME80Q1pfZC1UcUEwQjQzVjVLeE1VYklFMkUwLXFkaEpFbkxtX29OYW5YOFRjRzByODFfMHJfdUNORlVQUDNwWm1yQWtROE5ZR3ViRTZJZkR1Ri1rbDBsT1RqQ1hxbEhrbDJ0bzBHeGtEa1dmWXA5dmRSakk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOczUwYXFCX3dNZk9ZLUpWQjN0b2hTaDA1V0QwWjFIV2RmdUpmV1gzbmdJU1Q2OE9xNGduSDFpbEFQcG81bklHZGVXRTR4Mk5oUnRNRVlXM2VWSjFNZmUxRElUYVI0U3ZraTFBd05BX3BKMDZLaXl6aFBpSFVXWHFvVHpVdUY4ektSbkpsQkZManl4dXFJSFRIbXpPU1gxNjRQbF9mUHlDbEVoZzVtcUJ0cHZMejVITTZjN2F0RnFENWptMUJRajBOa3hxTE5lbFJPQW9GeHRXUTFPS2J6WUJVX2tBWXNOYS1xSGJ6N0VZb2lmc3NPVlNj?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46073.49747685185</v>
+        <v>46073.84469907408</v>
       </c>
     </row>
     <row r="3">
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Americold (COLD) Soars 15.7% on Upbeat 2026 Outlook, CFO Appointment - Bitget</t>
+          <t>GUNPOINT ROBBERY: Rs 12 Cr Gold Looted After Employees Tied Up in Assam’s Barpeta Road - NorthEast India24</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Americold (COLD) Soars 15.7% on Upbeat 2026 Outlook, CFO Appointment - Bitget</t>
+          <t>GUNPOINT ROBBERY: Rs 12 Cr Gold Looted After Employees Tied Up in Assam’s Barpeta Road - NorthEast India24</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:43:10 GMT</t>
+          <t>Fri, 20 Feb 2026 15:46:38 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiY0FVX3lxTE9yTzNwcEpmdGlfWDVVcHkwTHZ5bnRIYzJ1VHZNR0ZxbTdNY1oyQkp2cUdVZU1BM2daSS1ab0s4MnlCOUVyWHRmTjV2YTJZMkhzY2FsUjVMZldCcUVXanlTcEtOd9IBY0FVX3lxTE9yTzNwcEpmdGlfWDVVcHkwTHZ5bnRIYzJ1VHZNR0ZxbTdNY1oyQkp2cUdVZU1BM2daSS1ab0s4MnlCOUVyWHRmTjV2YTJZMkhzY2FsUjVMZldCcUVXanlTcEtOdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNZEE3cFZDZTF0aWNaOUc5WTFMUzRHcVUzNXJEbE1GdFE0S1hkUndPTnpGU19KNzdGZUZRWXpIOU1nclRkNDNGQ2VUVUpoQ1hjWmlibVdKeXIzQzljdnBzY1pHcWlWaVRVVHJLdHd3eHNOeHIzT0NTMG9KVjV0OUZaMGh0UmxLelVjWDhxN29CWWtfN0wzbjVfUFBKNlNLOERiSkw0UDVDdldVWjg5eUg1ZVI1Uks?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46073.44664351852</v>
+        <v>46073.65738425926</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Steinhoff's Business Report: Adapting to Market Challenges - Studocu</t>
+          <t>Prue Leith didn't want to 'overstay her welcome on GBBO - RTE.ie</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Steinhoff's Business Report: Adapting to Market Challenges - Studocu</t>
+          <t>Prue Leith didn't want to 'overstay her welcome on GBBO - RTE.ie</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 20:16:22 GMT</t>
+          <t>Sat, 21 Feb 2026 11:58:59 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOczUwYXFCX3dNZk9ZLUpWQjN0b2hTaDA1V0QwWjFIV2RmdUpmV1gzbmdJU1Q2OE9xNGduSDFpbEFQcG81bklHZGVXRTR4Mk5oUnRNRVlXM2VWSjFNZmUxRElUYVI0U3ZraTFBd05BX3BKMDZLaXl6aFBpSFVXWHFvVHpVdUY4ektSbkpsQkZManl4dXFJSFRIbXpPU1gxNjRQbF9mUHlDbEVoZzVtcUJ0cHZMejVITTZjN2F0RnFENWptMUJRajBOa3hxTE5lbFJPQW9GeHRXUTFPS2J6WUJVX2tBWXNOYS1xSGJ6N0VZb2lmc3NPVlNj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQa1JzWFZ1SzF3Y0U2dUI5aGtLeDRyTmZuVVMxMDRYQlZlcGYzX3puUHR1cnV0dDNqRWFJUDlxUXN3MDNnNVNtbVFyZUg3VU1iLTFHV09fb0NPWXpYU0NtYlhjTXpHZTEzMktSdGVYbHV1bXhWSEpOOElOSDlDeXhSeTRqNUo3M2E0c1ZTTUN2dHVmNUhVZXdxLTB3cEFhUjhFZ2VKaHo2WF8?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46073.84469907408</v>
+        <v>46074.49929398148</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GUNPOINT ROBBERY: Rs 12 Cr Gold Looted After Employees Tied Up in Assam’s Barpeta Road - NorthEast India24</t>
+          <t>The Best Hotels, Restaurants and Shops to Visit in the Cotswolds — the Hamptons of London - The Hollywood Reporter</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GUNPOINT ROBBERY: Rs 12 Cr Gold Looted After Employees Tied Up in Assam’s Barpeta Road - NorthEast India24</t>
+          <t>The Best Hotels, Restaurants and Shops to Visit in the Cotswolds — the Hamptons of London - The Hollywood Reporter</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:46:38 GMT</t>
+          <t>Sat, 21 Feb 2026 02:13:23 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNZEE3cFZDZTF0aWNaOUc5WTFMUzRHcVUzNXJEbE1GdFE0S1hkUndPTnpGU19KNzdGZUZRWXpIOU1nclRkNDNGQ2VUVUpoQ1hjWmlibVdKeXIzQzljdnBzY1pHcWlWaVRVVHJLdHd3eHNOeHIzT0NTMG9KVjV0OUZaMGh0UmxLelVjWDhxN29CWWtfN0wzbjVfUFBKNlNLOERiSkw0UDVDdldVWjg5eUg1ZVI1Uks?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNMVBPdmNZZ3ByY0FYNVpyck1fS0NKT3pmN19mTTBjMGFOcy1adlpnZmVRYWVtU05kYndYMkpvNk9SOEluanVEZTYxRnNaeFVyQy1DemtLNGtKTFRSYVdYZ1VJdUx0NlBUVXY1UWtpSllTSE9QVUVYMWppLUlyZ0hTdzZ0UGFjOHRsZXBZSk5ReDM5UktWVHJGaWl0SjdxbS1Kc21qeU42azAzSVV1d1NEQTR4TVZKbDk3bzJBZllFX2c?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46073.65738425926</v>
+        <v>46074.09262731481</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The Best Hotels, Restaurants and Shops to Visit in the Cotswolds — the Hamptons of London - The Hollywood Reporter</t>
+          <t>Brusselse regering betaalt 56 miljoen euro aan achterstallige renovatiepremies uit - HLN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The Best Hotels, Restaurants and Shops to Visit in the Cotswolds — the Hamptons of London - The Hollywood Reporter</t>
+          <t>Brussels government pays out 56 million euros in overdue renovation premiums - HLN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 02:13:23 GMT</t>
+          <t>Sat, 21 Feb 2026 12:58:54 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNMVBPdmNZZ3ByY0FYNVpyck1fS0NKT3pmN19mTTBjMGFOcy1adlpnZmVRYWVtU05kYndYMkpvNk9SOEluanVEZTYxRnNaeFVyQy1DemtLNGtKTFRSYVdYZ1VJdUx0NlBUVXY1UWtpSllTSE9QVUVYMWppLUlyZ0hTdzZ0UGFjOHRsZXBZSk5ReDM5UktWVHJGaWl0SjdxbS1Kc21qeU42azAzSVV1d1NEQTR4TVZKbDk3bzJBZllFX2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPSFk5bUllMUo4QnlLY1dmdWFrUWZUNW8yWUJJblVZSThHbWQ0OHR0bXdBTEIwU1V0WGd5YWZpZ2JhR0d1djBTVVRuLVZiRlpXaTYwOUtwbE16U3NkRkJUMVh4ZC00dTY4bjl0c1I5MHpFaFY0cF9pbERDa3FZQnFYOFBYbDRwT1NXM0VlWlVOWmtqRng4bTllU21iNFVqblNKQXNXNzFZTHV4R3pUY0xaemdBUzVqUDZzZU1zSA?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46074.09262731481</v>
+        <v>46074.54090277778</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>New survey names Doncaster as UK shoplifting hot spot - Doncaster Free Press</t>
+          <t>Je ging er winkelen omdat het zo goedkoop was, maar je wou er niet gezien worden: 50 jaar Aldi in België - Nieuwsblad</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>New survey names Doncaster as UK shoplifting hot spot - Doncaster Free Press</t>
+          <t>You went shopping there because it was so cheap, but you didn't want to be seen there: 50 years of Aldi in Belgium - Nieuwsblad</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:06:00 GMT</t>
+          <t>Sat, 21 Feb 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOa2ZMT1lMellVa1p4RDRyR0xhZnVzVjN2cE5RSjU4emY1ZzdyUVRoZDJJc0xkb2Z0MTFhZXpPdi1mS0hIN0prdTNoa2ZIcWpPVEljY1h4VWJyUVduUjk0ai13OW9iNEwteGptQVQ0V1hGRjV5eC0zMnAtMHFUbGxCeEw0MWxjLUJCczFFMklXaHp0M2pBZnI4ZWw5QjBRbFBjNXIyMVM2VlZaSm5MVUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOR21rUTU0a2VRWXRQLW5kOTFYOHM2RVlzNEdGc3hLazJrT3dISGVqN09VbnY1cXQyUE8xS1pOY2dOMDhVNmY2clB1SE94NTNSdS1KdjdMQmwxMlp4STdKWGVEQWk3NUhQc3BUM2V0VC1ha1NTOExWQURITVRzRWZMSjdtM0p4Y2U2dFhsakNuaFNyQm1GYVhCcnkzMUoyMzNDZXptd1k1M183dTQ3MmkwRkhURHZVV1N3RlNzWFZjVlVKaHEyeEFmdkdENnVCcWVsMUxxLVlSZnpPVVFhYTNoLXdOLTN3X0I4THc?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,21 +790,21 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46073.4625</v>
+        <v>46074.41666666666</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Politie opgeroepen voor schietpartij in Sint-Jans-Molenbeek - Nieuwsblad</t>
+          <t>Cokeconflict tussen Bolle Jos en zijn oude rechterhand: ‘Heb zware materiaal daar, die overleven dit niet’ - pzc.nl</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Police called for shooting in Sint-Jans-Molenbeek - Nieuwsblad</t>
+          <t>Coke conflict between Bolle Jos and his old right hand: 'I have heavy equipment there, they won't survive this' - pzc.nl</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:28:55 GMT</t>
+          <t>Sat, 21 Feb 2026 06:22:00 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOZ05fQW93OTZLWm51TDhlYXQ3WURtbDRNY1JXdjBQYWlQazRmZXF4SGtKUzBFbmRvQ2Z5c3E4S3d4TG54S3VyZ3FJZ0JBdVJIaXd6Y0kxY3BtV21tUjdmeW90X3hHcVhpcGZaMGl5VGhzdFFDRm82SnZSdUw2cy11QXpUYnB6Zl9mWkxsdHpJTVNHdGluMHRYUnd0bFRFRTR4ZnF6NjZkcHNValU3UEFSZVMyU0c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNR2tLcDk0Ul9Genp6eDlwdE9nb0ZOaVRTa3VLMUZWTHJhdllHZVVReVJ4NEZCemVpQzVUUEoyT3p1aGxXR3pVbzY1eWNkeGNVSFNqaXVsQ0lKQnQyS2hEX0VseGJ4TUtIeEtyaUc1WEE5NTQtMk5uWDJlOXV1VDdrcW1WaXQyZ2pVc3g0UC16Sld4T1U4UUwzRlhFSWY2bUNZX1dwY3p5aGZIWXJVUzVXbk1QVlNtdmVfSEZ1em1UQUtQMFJFdjc1QUk4bkNqVEhWQ2ZxUHdONndkQQ?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46073.64508101852</v>
+        <v>46074.26527777778</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cokeconflict tussen Bolle Jos en zijn oude rechterhand: ‘Heb zware materiaal daar, die overleven dit niet’ - AD.nl</t>
+          <t>DC The Aces ongeslagen kampioen in tweede divisie: “Meer stress dan bij het voetbal” - HLN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Coke conflict between Bolle Jos and his old right hand: 'I have heavy equipment there, they won't survive this' - AD.nl</t>
+          <t>DC The Aces undefeated champions in the second division: “More stress than in football” - HLN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 06:22:00 GMT</t>
+          <t>Sat, 21 Feb 2026 11:38:30 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxNYjA1ZTJNUHhLM1QwVXg2V2czM21tOFZFUGR3V0Y5bW9mQldYMEZCZHJfV2pXd0g0OUliTW9xcVU3cmVHN1g2Q2dieWVJd2tubG5HZEFxeUhONWwxYWgtX3R4R1loSmI3TXhPYmJBbV9FZzVGS2ZyVzZOZHQ0VDZWS1FTNUlGUm5YaXdjaUVGS01Tb09jWlplN1BtaVluN0dFVzh1bFkzZllXX0pfRzFOeHJCRmFBS19YckFPaEF2VFpPWjQ0bWN5VERUbTBNS0NhbHhmSFZuYTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNSlZMSWFxNVI1NzNPMEYzYkIyY2hZVTBiLW96NV9aVXFfMDE1cy1GN3Y3UDVvaGN5ejFmc1lKeE5pcFJTS3M1UlNqd3JqSHJ1QkN6NnFJRHdWMnFVRk8yLWxEbEo4bXNQWVlLOU9RR0FiWldvaW80NUFOWTdYVkVaa0t3UVFKcHdaTUZtNEJNbnRFcjM0dGpydGdidE5vRWVwOXA4X0Z6Zk1TUEJpRTBXOXBlMnB1OGc1emc?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46074.26527777778</v>
+        <v>46074.48506944445</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Scooterrijder gooit zwaar vuurwerk onder de auto van Frans Theunisz: ‘Geen idee uit welke hoek dit komt’ - De Limburger</t>
+          <t>Drie twintigers de cel in voor vuurwerkbommen in Roermond, maar waarom ze het deden blijft een mysterie - De Limburger</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Scooter rider throws heavy fireworks under Frans Theunisz's car: 'No idea where this came from' - De Limburger</t>
+          <t>Three people in their twenties jailed for fireworks bombs in Roermond, but why they did it remains a mystery - De Limburger</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:07:28 GMT</t>
+          <t>Sat, 21 Feb 2026 13:51:36 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxPVTRGc1VJNk9UQlZVenZuamd1aG1CakdYQVZrb1FjUzJLazRiUFNtTFdtVjUwT0tlZnQzWUlZQnBVRUdabkE1WEpXb1pldzhjbV9JTGlmMzJ3ZHczYTFZNnJIUGJWVUIxOW9xOFJIaFNxQUFtNm9FbjZXeFRVLXgxUlMzSHRkNlBacnY2cUF0b3c3NFNwSjF4RFF4SWhLWE96VGtjTExYbUFvcEJHTzlvSzU4Yi1UWDVnUTd4aE0xZk9lSnVJd3hFZldkV3pBRnZkZTI5SjNaWjRWYTFzT1VpaFh0ZWZHSXV0MGE4QUNXQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxNRkQxU1RjNC1RNUlmb2NVZmM2QXVtSzQtQmtTLXQ1WWktd19BbzNJaXhyQVV5YzhCZzRLSGVpWE5QeVY4NU40ZjJQVnJGRENRVERraFF6UXRHVUtmNENaaEtPS3VVWEgzSVVaZWlRZDBNbDJhRk5UWGNXS0d5S2p3RnNodERvN2hZLU9CVHExZVZPS1dYbDdORUdrRjZIU3FyTFMxcjNKSjRiM2FZQy1GRnRNa1ZUUExNaG92Wkd5LUVBbGRCUU9zcUdBejI5NWt0UFhGaHdvUmdGMHpuS2oxMlJPVUdqLUhwVlkzejhR?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46073.50518518518</v>
+        <v>46074.5775</v>
       </c>
     </row>
     <row r="11">
@@ -985,22 +985,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Gheysens schiet uit krammen: bom ontploft bij Antwerp - VoetbalNieuws.be</t>
+          <t>Politie opgeroepen voor schietpartij in Sint-Jans-Molenbeek - Nieuwsblad</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Gheysens shoots out of jams: bomb explodes near Antwerp - VoetbalNieuws.be</t>
+          <t>Police called for shooting in Sint-Jans-Molenbeek - Nieuwsblad</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 16:41:00 GMT</t>
+          <t>Fri, 20 Feb 2026 15:28:55 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPdkR3UDd5RHNTR1VOVWVBdl9lV3ZLTVpnYThkWFcwWFVtQmFrVzhFcUhCZDN0dnhTTWtPcHV2UjdOY2ZFZnZRVjd6MGxEdE90dnBaSWg4MDlkZENVeEVUT2lsZUNRMDZUTVZnM2Q3ZTdIZ0tsYmtEV1J1OEttbWN3OVR3ZU1fOUhRdlhiVERWZmZsSUoxeVFBTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOZ05fQW93OTZLWm51TDhlYXQ3WURtbDRNY1JXdjBQYWlQazRmZXF4SGtKUzBFbmRvQ2Z5c3E4S3d4TG54S3VyZ3FJZ0JBdVJIaXd6Y0kxY3BtV21tUjdmeW90X3hHcVhpcGZaMGl5VGhzdFFDRm82SnZSdUw2cy11QXpUYnB6Zl9mWkxsdHpJTVNHdGluMHRYUnd0bFRFRTR4ZnF6NjZkcHNValU3UEFSZVMyU0c?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46073.69513888889</v>
+        <v>46073.64508101852</v>
       </c>
     </row>
     <row r="12">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Importverbod op Russische olie per schip vertraagd - Nieuwsblad Transport</t>
+          <t>Gheysens schiet uit krammen: bom ontploft bij Antwerp - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Import ban on Russian oil by ship delayed - Nieuwsblad Transport</t>
+          <t>Gheysens shoots out of jams: bomb explodes near Antwerp - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:18:17 GMT</t>
+          <t>Fri, 20 Feb 2026 16:41:00 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNZTVMSVdIUDhqZUVobFVoZ1pLdUJiVGlSRjhBSGcxSmdWWDJwZGdxOFdNeGpMZW1TVGllc1RfV2YyUnZaRzdyMEVDMkpaUW9GT1pvTkFpZUJwQ0JZVzRpS1pNdUJtd291dmMyMGZtTjNjLURzM0tkY2dfTEZ6YVFHbXBiZzY4WXk1V3dubF8zcTRYX0Vpbnkw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPdkR3UDd5RHNTR1VOVWVBdl9lV3ZLTVpnYThkWFcwWFVtQmFrVzhFcUhCZDN0dnhTTWtPcHV2UjdOY2ZFZnZRVjd6MGxEdE90dnBaSWg4MDlkZENVeEVUT2lsZUNRMDZUTVZnM2Q3ZTdIZ0tsYmtEV1J1OEttbWN3OVR3ZU1fOUhRdlhiVERWZmZsSUoxeVFBTQ?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46073.47103009259</v>
+        <v>46073.69513888889</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>OpenAI overwoog Canadese politie te waarschuwen over latere schoolschutter maar greep toen niet in - Nieuwsblad</t>
+          <t>In Gronsveld betrapte dronken automobilist reed al 30 jaar zonder rijbewijs - De Limburger</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>OpenAI considered alerting Canadian police about later school shooter but did not intervene - Nieuwsblad</t>
+          <t>Drunken driver caught in Gronsveld had been driving without a driver's license for 30 years - De Limburger</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 05:05:33 GMT</t>
+          <t>Sat, 21 Feb 2026 12:11:02 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxOeGxqcjFnVEVUeUFyRUFVWkhOb2Z3RE1OcExMR2tXeG9yNXJYVERveGpwSmZTNjBqRmdoVGFBZGR0YWtIenFuaWtZUC1qYzc2WHhMdjM1RXlFRDU1NUNRaldpd256TEN5YmVacmFPSlNXTThoenBadG5qUEZaakJ0cnZycmwzRXpBeTJxYzYtOFJHUF9sOXhENmFLRGM2cjFjTXJSLU9yVVUxa2ZlcEI3OWpvSzZhMHhlbWtWRkw3dmNtUmdCNzItaTVKTW5TUkZ4V3VjT2lBeXduajkwbE1WWk1sMHQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQTUk5V1RQcnhZOGE5R1hFUWVwd2lyMG8zaDRxQVJReE9KbjJTUzNxVFhiX3ZlT0VITDNESGptVmdRUEtEaTNUSERWM0c4YjBPUU5jV2NUOF9RUnJ6N0RCTkI5VUFkZ3RqU1Fjcmd6b1o0bnk4WDRJTDZpS25uUDR2TC1xTy04QnRrZ3FheHFxNWV1em55ejhZMWJBNjhQTHk1T1RvR2tvV29WMlprUGZ4NUJlbTVRSnRXSXlxejhLb1JKMnB6X052RkZHSXg2dW91WWczYWhVeU5CVGNQNnNjazY4RQ?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46074.2121875</v>
+        <v>46074.50766203704</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Shots fired near metro station in Molenbeek - The Brussels Times</t>
+          <t>'NO WAR MONEY UNTIL RUSSIAN…’ EU Powerhouse Stuns Brussels, Freezes Billions Meant For Ukraine - The Times of India</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Shots fired near metro station in Molenbeek - The Brussels Times</t>
+          <t>'NO WAR MONEY UNTIL RUSSIAN…’ EU Powerhouse Stuns Brussels, Freezes Billions Meant For Ukraine - The Times of India</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 01:07:30 GMT</t>
+          <t>Sat, 21 Feb 2026 11:35:33 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxPV0o2UTVpdFBzMTU3TFJPNjFCRGVickVXbG5EUW5haVlrWkJHLXNGcXpjSUJnek8wTkIxWVpFZ1gxcXRvM2doRHBBTFJOY2FSWGRwZFVCWnFzTHBiMk1BQVdVR0dkYVpQaTlBVEdmc042MW4wUTNVNnJEZ0JKdHc4MzFkM3dHTTVp?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxOczE3elRoMGczeW9qZjdTLWxlTzhYajVyemdsNXQzVS1UdEMydFg0NW84WFREcEtfU2xHWUlmM3JPMlhmQmZiTHVvV3J1Z3VZWjczOTh5SGpOSUFlS3FhVzhGYjBfcHdCLWFCbm03QVhoNVB4RFRQOF9YaWMtSnhFZGt6ZHVhbk5VbWtnXzBIMnFaeVRpRkJPbmRQTG1PSndFSWdGeG9nRjgzYzRtelRrVUhxSjFLdUlSUl9yS2tHVmE4TXN1REF4UU5xRHBHS0pEd2xmRzM1VlVoRC11cDRlN3RMR0NkMmZFeDVoYmxlQ0lGOXpSWW1ETUhuSk9oNHd10gGGAkFVX3lxTFBNVk40bFlKX3gwak4wMDhJYUZ2TXJURkJTUmRwdzljXzV3dnB5NFdubTlGdjR6X1hETl9oN0NBTXV3eWVGaDNweklUekVTUzI5amVlN3dyT0F0VUk1STF6Q3RsLXo4a0RtckpGY1lZT1dhVlp5ZF9YQTFzaGNvV2tYQnlWMlcybVpPNFh3dHV4dUVka3M4Q1ZEaTlWV2cyeENhTDF1d0ZRQzkxS2hSNmNxNmY2VXpfTFNxQjhjaWsyeEREVDFnaVhuTU85OUZkckhIR0M1UVFCdGtGRHAwVTJUT2pTWE9xSmdrSkJUR0NjbTVES2RxV3VXOFd4NlVyZThBNmpKcVE?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46074.046875</v>
+        <v>46074.48302083334</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
+          <t>Yet Another Brussels Shooting: Gunfire Near Metro Station - The European Conservative</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
+          <t>Yet Another Brussels Shooting: Gunfire Near Metro Station - The European Conservative</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 22:07:18 GMT</t>
+          <t>Sat, 21 Feb 2026 13:36:40 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOcVV3cGgtM0t5Nm5XbTFJbGR2N0Q1RHRhVmJ3VnJFTGhiUVN5bFJpWUUyNUxVLVEwVjF1elZ4WXdIVUVVWXVmcm1nelZXYV9FcEVBS3ZPeU92aDlmRko2eWI3WjZqRWxUeTlteVVvVDM3Y2ZlbkJWT2QtWFJNQ0paNUJDOTh2b1JaZVdOSVdsVndLbXVUNU0tTlBTUUdKUFF5TVdF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPd25WaVVWZVRqMFFwU194S2gtVEpWUVJPbU5CLXFKVmR4QnJjcXczMzJHOGFzYjZGQlRfalgwTG1GV0lHcTZla3JWbHd5QmlNQmJCOWVIZFN0a0s2RTVQZkFrMkdMbjBqQWt5eDk2RnNjUUhBVkgtRm1Gd1RpUUdFZGlsWVpiOEd6cEY0SFNwb3lDVW1PWXp0M0wwLWd5RFlxNXVEY0R1R00ySHFkM0RocA?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46073.92173611111</v>
+        <v>46074.56712962963</v>
       </c>
     </row>
     <row r="17">
@@ -1315,22 +1315,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Germany, partners prepare to send Ukraine additional PAC-3 interceptors - The New Voice of Ukraine</t>
+          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Germany, partners prepare to send Ukraine additional PAC-3 interceptors - The New Voice of Ukraine</t>
+          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 19:06:00 GMT</t>
+          <t>Sat, 21 Feb 2026 09:34:18 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPa2d1RGR3b2xkU3UxYzRoWmNmTGpOTWpaajBwUDQ3UlFrdFVVckhYZ1JncEgyLTB1bXU4MjA0STF6TFE0VmZ2ZDhycG03d250VVdtTWJJQlFHcWJpN1ktTDJKWlJEWWVtZWRrSHBfNGtEMC0zdW05c0diTUxrVjBUcjB3WHA1TDY1S2hCSExJX3Jma19YRi16ctIBlAFBVV95cUxQLTZEZTJzSzNuc3dqcHJGbDZYVnNYWWxSdG1QLXB3TV94ZkxBSWdFaVdzYlUzYXUwOWItYmhsSXJ4RmtqS3dEdXFSQU1PaEFLRkxLV2I5N0IyRGQyVUVLQi0wUW4zUU5OX29nV3k3NHdSNGVma3o1TXBsTjFuV2V1ckdmUkRqR2dCNDdYejViSExpdzM4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNZlBCeEZXakZ5VVBhQWpxMEpCVzFtTm9CYlZ2emxsaXhUci1GUXRybGp0T2ZKRDJNYmFXYjFNZDRSS3NTLXBrRnVfS3RLRndzcFNTUU9rVGFmM3ZnV3hFbGNUN0JMVHRjSnpqWkVSWDFrS2pQa1JjeFZzN3luS2pqS1U3REhERHQ3dV9WUGVZeWl6Q014Sk5EenVfaGY?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46073.79583333333</v>
+        <v>46074.39881944445</v>
       </c>
     </row>
     <row r="18">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Several Belgian teenagers abducted and robbed at knifepoint in stolen car - The Brussels Times</t>
+          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Several Belgian teenagers abducted and robbed at knifepoint in stolen car - The Brussels Times</t>
+          <t>Turkey arrests European activists probing prison conditions - The Straits Times</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:14:33 GMT</t>
+          <t>Fri, 20 Feb 2026 22:07:18 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPNkJQRzUtRTNwSkt5RmdyUEZaUV9jOXhLTERWY2xUOXBZTlBQWDZjY0tTY2lOS1oyTFlKWEU4aFdjaXl1aVdDckxTVGRUWVdIaXJjN2NiQzlJU2xXenZlenY5UWtESllJNF9JSmNKRENMc0RvdzJVSHVzWFF3WVFiUVgtWFQ1MnR5cGktanRmRnhtVE1HcnFwV0htWERTZjMtTmI3cWp4aTg0ckxYVTNvWg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOcVV3cGgtM0t5Nm5XbTFJbGR2N0Q1RHRhVmJ3VnJFTGhiUVN5bFJpWUUyNUxVLVEwVjF1elZ4WXdIVUVVWXVmcm1nelZXYV9FcEVBS3ZPeU92aDlmRko2eWI3WjZqRWxUeTlteVVvVDM3Y2ZlbkJWT2QtWFJNQ0paNUJDOTh2b1JaZVdOSVdsVndLbXVUNU0tTlBTUUdKUFF5TVdF?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46073.51010416666</v>
+        <v>46073.92173611111</v>
       </c>
     </row>
     <row r="19">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
+          <t>Germany, partners prepare to send Ukraine additional PAC-3 interceptors - The New Voice of Ukraine</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>The student who was injured in the "Gjuta" hotel, the fiancée of a police officer, the lawyer, BLOWS the bomb: She lied to the boy about her age and origin! - Vox News Albania</t>
+          <t>Germany, partners prepare to send Ukraine additional PAC-3 interceptors - The New Voice of Ukraine</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:57:47 GMT</t>
+          <t>Fri, 20 Feb 2026 19:06:00 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQNkdQYmNiZjFHS0pDdmR0MEJkMkQxcGZRUlJZVzJPeEJBY1VoZWNabWN3NFdZM25Qb01iaWVVSVNyUlZUUXc3QmdPN2RvWFFkdlhDZU1rRjdRUF9kRV8xTy0xOE03SmhHUmdyLWdyclJaQXBEYUFlNl95eXR5Vy1WUmFHaHVDSlpNVUdwUnlSUWtKbl8xMU5wLWs5Q2V0bUhCdVBhaHBMR21JdlowUTNNVU4wNzh1Wk5ORjIw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPa2d1RGR3b2xkU3UxYzRoWmNmTGpOTWpaajBwUDQ3UlFrdFVVckhYZ1JncEgyLTB1bXU4MjA0STF6TFE0VmZ2ZDhycG03d250VVdtTWJJQlFHcWJpN1ktTDJKWlJEWWVtZWRrSHBfNGtEMC0zdW05c0diTUxrVjBUcjB3WHA1TDY1S2hCSExJX3Jma19YRi16ctIBlAFBVV95cUxQLTZEZTJzSzNuc3dqcHJGbDZYVnNYWWxSdG1QLXB3TV94ZkxBSWdFaVdzYlUzYXUwOWItYmhsSXJ4RmtqS3dEdXFSQU1PaEFLRkxLV2I5N0IyRGQyVUVLQi0wUW4zUU5OX29nV3k3NHdSNGVma3o1TXBsTjFuV2V1ckdmUkRqR2dCNDdYejViSExpdzM4?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46073.54012731482</v>
+        <v>46073.79583333333</v>
       </c>
     </row>
     <row r="20">
@@ -1480,22 +1480,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fusillade à proximité de la station Étangs Noirs - BruxellesToday</t>
+          <t>Plainte pour atteinte à l’intégrité sexuelle d’une stagiaire contre Marc Uyttendaele : des étudian... - L-Post</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Shooting near Étangs Noirs station - BruxellesToday</t>
+          <t>Complaint for violation of the sexual integrity of an intern against Marc Uyttendaele: students... - L-Post</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:34:29 GMT</t>
+          <t>Sat, 21 Feb 2026 00:04:19 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxObV9GWTNXT0pnV2VZLW5zUGFTUDZ5UjEwaXlFZ2N6V2g4a2tLMjVyUGdXeXZRWmFwVURCYTJ1bnR2bnZVcEZTRHVmMmtoR2ZSaDFjcGVPWnRSLVFkQUpPTU82ZGx4MTBBWFR6elU3MTV6RXhyazI0ckdFXzJyQlNJS0RVOEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxQeWRLOThYc195ZlAzSGNFX2ppSHVCQzMwRE0xUXBtaTRFa0xOR2M0M1EtOUpwdTFTLUtWeFgyMEt6eXpvNERHeGpubUpIaUZTTG9jSlZ1NEl0bTNSbnI0OHhBS0xoaTM2b201VW15ajFMSUZSRUl2Nmg1UlJwcHZobTY0U3JELTJwVmUxZW9MaTh0RHBKTDBJVlAzajdoTUJfQXYxR19hVHloa2ozbE9QZnUzbm1LUUtrUUFwMWNnRU1oaHpoaTl3X3F0cmtnQ2lRV05pT01SdVBtemt1UHJFT3FGeUpyamwwcXhoMy0tb9IB7wFBVV95cUxQeWRLOThYc195ZlAzSGNFX2ppSHVCQzMwRE0xUXBtaTRFa0xOR2M0M1EtOUpwdTFTLUtWeFgyMEt6eXpvNERHeGpubUpIaUZTTG9jSlZ1NEl0bTNSbnI0OHhBS0xoaTM2b201VW15ajFMSUZSRUl2Nmg1UlJwcHZobTY0U3JELTJwVmUxZW9MaTh0RHBKTDBJVlAzajdoTUJfQXYxR19hVHloa2ozbE9QZnUzbm1LUUtrUUFwMWNnRU1oaHpoaTl3X3F0cmtnQ2lRV05pT01SdVBtemt1UHJFT3FGeUpyamwwcXhoMy0tbw?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46073.64894675926</v>
+        <v>46074.00299768519</v>
       </c>
     </row>
     <row r="21">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Un Belge détenu en France pour agression sexuelle sur un garçon de 13 ans extradé vers la Belgique - 7sur7.be</t>
+          <t>Une jeune cycliste de 16 ans perd la vie après avoir été percutée par un camion à Kuurne - 7sur7.be</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Belgian detained in France for sexual assault on 13-year-old boy extradited to Belgium - 7sur7.be</t>
+          <t>A 16-year-old cyclist dies after being hit by a truck in Kuurne - 7sur7.be</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:35:00 GMT</t>
+          <t>Fri, 20 Feb 2026 20:35:12 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNWF9veDBvVHRlMy1ESVJ4MTFVUTJzSm5FeXB4RUExV01BaE9PaEdjMElYRE5wb2NlVFJsclV1U1A0R3BjN0pqb1NWeDI5T0IyNWFqV0VUZDhtZjZRSFMySXdoSDdHZEluMXA0bWp2MXZCVFkxUDc2Y2l4UWxRZDZybmU3YjRXdXN0MTNkTkxGQ3hweXJDV1JhdUhpM3lQNldib1RuajFPMjRualdMSlpRMC1DWWxQYkFFNU5CYXpNbzZrdnRCam1fN0U3ZEFzdGo2a2VhTjZrWEZNZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPQlphMVNkODZVRkcxX3FhN2dZVTI1bkprRE9ET290QnJBWWtWeWFpMUFvMnFseG91UkpXY1NNSktGNHlRN2l4R2RoTnN3Sk14Rm5YTlE5a0U3MkN0MW84aVdteXJkclRPS1NuR1hDMGR2clppQkRsQ3RDcllyTjFiRFo1Ry1LOGxhZ0lMNDg2TzZCRlI5M0dMYWxSM2JLSkhzUTVqWEpGZjdkcGFZRmwtSUk0WnpubjkyY0RKZXJkNGh0UXhFenZKSENJX0Y?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46073.64930555555</v>
+        <v>46073.85777777778</v>
       </c>
     </row>
     <row r="22">
@@ -1590,22 +1590,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Plainte pour atteinte à l’intégrité sexuelle d’une stagiaire contre Marc Uyttendaele : des étudian... - L-Post</t>
+          <t>Nouvelle stratégie de la Croix-Rouge de Flandre : « En cas de catastrophe majeure, il faudra pouvoir se débrouiller plus longtemps seul - De Standaard</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Complaint for violation of the sexual integrity of an intern against Marc Uyttendaele: students... - L-Post</t>
+          <t>New strategy of the Flanders Red Cross: “In the event of a major disaster, we will need to be able to manage alone for longer - De Standaard</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 00:04:19 GMT</t>
+          <t>Fri, 20 Feb 2026 23:42:16 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxQeWRLOThYc195ZlAzSGNFX2ppSHVCQzMwRE0xUXBtaTRFa0xOR2M0M1EtOUpwdTFTLUtWeFgyMEt6eXpvNERHeGpubUpIaUZTTG9jSlZ1NEl0bTNSbnI0OHhBS0xoaTM2b201VW15ajFMSUZSRUl2Nmg1UlJwcHZobTY0U3JELTJwVmUxZW9MaTh0RHBKTDBJVlAzajdoTUJfQXYxR19hVHloa2ozbE9QZnUzbm1LUUtrUUFwMWNnRU1oaHpoaTl3X3F0cmtnQ2lRV05pT01SdVBtemt1UHJFT3FGeUpyamwwcXhoMy0tb9IB7wFBVV95cUxQeWRLOThYc195ZlAzSGNFX2ppSHVCQzMwRE0xUXBtaTRFa0xOR2M0M1EtOUpwdTFTLUtWeFgyMEt6eXpvNERHeGpubUpIaUZTTG9jSlZ1NEl0bTNSbnI0OHhBS0xoaTM2b201VW15ajFMSUZSRUl2Nmg1UlJwcHZobTY0U3JELTJwVmUxZW9MaTh0RHBKTDBJVlAzajdoTUJfQXYxR19hVHloa2ozbE9QZnUzbm1LUUtrUUFwMWNnRU1oaHpoaTl3X3F0cmtnQ2lRV05pT01SdVBtemt1UHJFT3FGeUpyamwwcXhoMy0tbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPTjhOa3haWkhPQ1ZxbTVXWUJ5N2dwVXRlTy1aXzhmcllfbnBCREM3bE43eHNRRFZnYlE1UkxBMUJnVzFhbjVHaXNoZmlERnFydWpySmM2MVJKX3Bnd2R1ZTNpSFBhbjRNSFA2TFRZNWZxYzRnYzNpM1lnZzhBRVExUTJHTW81bVQ5bk1mNFVxY2FYY0RsTEZRV3FjZDNxeGhqekU1X1hLUnZhcXZKaGlOeHpRZ2lJOG5uaFRuXy1yWVZlY2Z4aU9aei1LNTJmbU5EV2R1bjhQWEJ1dlNtRXN2b0puNF8xTVRtYkRtWHQza0J1Ykx4N3JoQ1N2TWNPWHg3TEhEcFB6SQ?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46074.00299768519</v>
+        <v>46073.98768518519</v>
       </c>
     </row>
     <row r="23">
@@ -1645,22 +1645,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Nouvelle stratégie de la Croix-Rouge de Flandre : « En cas de catastrophe majeure, il faudra pouvoir se débrouiller plus longtemps seul - De Standaard</t>
+          <t>#FrigoVide : les associations dénoncent l’explosion de la précarité alimentaire - tvcom.be</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>New strategy of the Flanders Red Cross: “In the event of a major disaster, we will need to be able to manage alone for longer - De Standaard</t>
+          <t>#FrigoVide: associations denounce the explosion of food insecurity - tvcom.be</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 23:42:16 GMT</t>
+          <t>Fri, 20 Feb 2026 15:39:26 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPTjhOa3haWkhPQ1ZxbTVXWUJ5N2dwVXRlTy1aXzhmcllfbnBCREM3bE43eHNRRFZnYlE1UkxBMUJnVzFhbjVHaXNoZmlERnFydWpySmM2MVJKX3Bnd2R1ZTNpSFBhbjRNSFA2TFRZNWZxYzRnYzNpM1lnZzhBRVExUTJHTW81bVQ5bk1mNFVxY2FYY0RsTEZRV3FjZDNxeGhqekU1X1hLUnZhcXZKaGlOeHpRZ2lJOG5uaFRuXy1yWVZlY2Z4aU9aei1LNTJmbU5EV2R1bjhQWEJ1dlNtRXN2b0puNF8xTVRtYkRtWHQza0J1Ykx4N3JoQ1N2TWNPWHg3TEhEcFB6SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUWpKRFpFYlQ5ZTd6NFJfQXZlRnZhMVo0ZlFDMExaQkRldUEweDFNSWd2eFdBMDB1TGlzYk93MFRQR0ZJWVZsQ19yak04UmZlZFMwWDMyUllJUVB5d2R1WTJQT3dQS2NOMTN4TC1DeTMwM3FxWEFuQ09aeE5STWpiSGpUZmVtbzJILWx2aWFaZ3UtejV0cnRRUXRMdVFsYUJ1dGNuSWV3LVZyODg?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46073.98768518519</v>
+        <v>46073.65238425926</v>
       </c>
     </row>
     <row r="24">
@@ -1700,22 +1700,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>#FrigoVide : les associations dénoncent l’explosion de la précarité alimentaire - tvcom.be</t>
+          <t>Un Belge détenu en France pour agression sexuelle sur un garçon de 13 ans extradé vers la Belgique - 7sur7.be</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>#FrigoVide: associations denounce the explosion of food insecurity - tvcom.be</t>
+          <t>Belgian detained in France for sexual assault on 13-year-old boy extradited to Belgium - 7sur7.be</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:39:26 GMT</t>
+          <t>Fri, 20 Feb 2026 15:42:42 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUWpKRFpFYlQ5ZTd6NFJfQXZlRnZhMVo0ZlFDMExaQkRldUEweDFNSWd2eFdBMDB1TGlzYk93MFRQR0ZJWVZsQ19yak04UmZlZFMwWDMyUllJUVB5d2R1WTJQT3dQS2NOMTN4TC1DeTMwM3FxWEFuQ09aeE5STWpiSGpUZmVtbzJILWx2aWFaZ3UtejV0cnRRUXRMdVFsYUJ1dGNuSWV3LVZyODg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNWF9veDBvVHRlMy1ESVJ4MTFVUTJzSm5FeXB4RUExV01BaE9PaEdjMElYRE5wb2NlVFJsclV1U1A0R3BjN0pqb1NWeDI5T0IyNWFqV0VUZDhtZjZRSFMySXdoSDdHZEluMXA0bWp2MXZCVFkxUDc2Y2l4UWxRZDZybmU3YjRXdXN0MTNkTkxGQ3hweXJDV1JhdUhpM3lQNldib1RuajFPMjRualdMSlpRMC1DWWxQYkFFNU5CYXpNbzZrdnRCam1fN0U3ZEFzdGo2a2VhTjZrWEZNZw?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46073.65238425926</v>
+        <v>46073.65465277778</v>
       </c>
     </row>
     <row r="25">
@@ -1755,22 +1755,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Un député québécois agressé à Bruxelles: “Triste que les villes européennes en soient rendues là” - 7sur7.be</t>
+          <t>Accident entre une moto et un camion place Madou: deux personnes hospitalisées - BruxellesToday</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A Quebec MP attacked in Brussels: “Sad that European cities have reached this point” - 7sur7.be</t>
+          <t>Accident between a motorcycle and a truck at Madou Square: two people hospitalized - BruxellesToday</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:56:00 GMT</t>
+          <t>Fri, 20 Feb 2026 17:01:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPeDFBWkdGenBYUkpaZXpzNVB4RzZJemNrTFlwbnpiUzRta0VpcjJUdGhhd0NuMWJjb25ZTFZBZGZhQ2c1VTQzNDVoVzhQYW84Z2k1cFY4R1FGWEpSSkxxQzdXQ2xaWU1Yajh0aG15TEtpLUpMVHRHUXdUd2d4eTZrWHdOZXpNNjJVMHFhV0t4ckdrR2dvOEJFY1RXR044d2ZYODhRYkpOUEJSQWxsTDdQejVaUkwxZFQ1aDNzUkNDaTBsczY1bUREbDNEQmpHMlFEUUZvRlpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOZVFQQzlPaFFsSjBwaVBickxVRmdtd0ZjZ3ZnbmtiT3U0cEgxblVZWmNFN2hfMnByT1pvQUItNEVtZ0dlMkMxRlFFX0dkdEUzM0lWdGtLX0VMQmNNczdtMGZoTnNvZ0RpQWdWNm9TREo2YU9fcVlocGpNeXFGM1ZHX1FvS0hhVVk?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46073.53888888889</v>
+        <v>46073.70902777778</v>
       </c>
     </row>
     <row r="26">
@@ -1810,22 +1810,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Accident entre une moto et un camion place Madou: deux personnes hospitalisées - BruxellesToday</t>
+          <t>Des coups de feu tirés dans le quartier des Étangs Noirs à Molenbeek - 7sur7.be</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Accident between a motorcycle and a truck at Madou Square: two people hospitalized - BruxellesToday</t>
+          <t>Shots fired in the Étangs Noirs district of Molenbeek - 7sur7.be</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 17:01:00 GMT</t>
+          <t>Fri, 20 Feb 2026 15:40:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOZVFQQzlPaFFsSjBwaVBickxVRmdtd0ZjZ3ZnbmtiT3U0cEgxblVZWmNFN2hfMnByT1pvQUItNEVtZ0dlMkMxRlFFX0dkdEUzM0lWdGtLX0VMQmNNczdtMGZoTnNvZ0RpQWdWNm9TREo2YU9fcVlocGpNeXFGM1ZHX1FvS0hhVVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOZ3pqenJJLWhNLWpnMUM1VnNYd1dWQXdJbkdnY2JxSDU3MXhJZHBUY3FSMktYaUQ1NzRXbzUxS0swUmpab1hXSWJuRVRMVG95N3FQUmdvRzJpMUJsNDZIXzdvNVJ2UlJ1ekloRjBqcDF3QTRhZEMzeHJlWXZ3NG9jeWF6RHRfNWtrc0ZOUmxIMFg4ZmN4TmdjdjZsYVo0MEtINTNNRjktalZ3NkJjU1Jydll3?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46073.70902777778</v>
+        <v>46073.65277777778</v>
       </c>
     </row>
     <row r="27">
@@ -1865,22 +1865,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Des adolescents embarqués en voiture puis dépouillés à Braine-l’Alleud et à Waterloo - 7sur7.be</t>
+          <t>Alertes à la bombe: la tour Montparnasse et Sciences Po Paris évacués - 7sur7.be</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Teenagers taken by car then robbed in Braine-l’Alleud and Waterloo - 7sur7.be</t>
+          <t>Bomb threats: the Montparnasse tower and Sciences Po Paris evacuated - 7sur7.be</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:18:00 GMT</t>
+          <t>Fri, 20 Feb 2026 19:30:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQdWZrakJRZHh6c1h0RzJHaWtoU0NCYkdmZlNsWWdlaEgxQTJ2ZUxfVUczU2c5MkxwNkM2NF9YY3pRek1NRUw4R0JCZlRWc0FORWxKdWh1dm1RRl9HbUVPMFVpbjZYZklhZVdtejVScnFWYjlKX05xTThIQWpUelRLZVp5cU1TR3Uzc3R1aGNzTWJVV3VDYXI1S2ZESG96bFN4Wkg5UEMzaTNkcXNNWmwwQVcxT0VnWlMySW04OU5DODFYYVNmZFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQVzBXYjBsbHhQa09jeElaeEVUR2JYdFlza1NFUzIzeVpLT1JnbzNRaDRZaG1WYUxNemg2eE5BVzNYZi1CZWZGcGlWMEgyUjRuTk5QOE9XX2x4bnN3dFlHUThIMklYUWg0c2EwVG9xNkxWdmwxN3RNOWNvb1RMeHB6UHpBRWVnTkU5QVJtYmtuaXE1V1I5enVHWFN2czNDaHhyRFBVTXZES1lmY0lNOG5zWVN3?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46073.47083333333</v>
+        <v>46073.8125</v>
       </c>
     </row>
     <row r="28">
@@ -1965,32 +1965,32 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Verdachte gevat na crash bij politieachtervolging in Hasselt-Kortessem - MSN</t>
+          <t>"Samedi 21 février, l’extrême droite marche dans les rues de Lyon, et nous continuerons à résister" - Politis.fr</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Suspect caught after crash during police chase in Hasselt-Kortessem - MSN</t>
+          <t>“Saturday February 21, the far right marches in the streets of Lyon, and we will continue to resist” - Politis.fr</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:17:18 GMT</t>
+          <t>Fri, 20 Feb 2026 14:49:09 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gJBVV95cUxNV0VnTkp1dmVVT3pBOTNwdnU3dVhCUy14UTF4TXBPamttNjJfc212eWF6N1NMX2hlTS10Ullqckd6SjJUVlhkVV9yWTl3cW90U0UyYmtiSkJMM0xYcndpRElhbTZxTk9rNVhRSVRSZDNPQW5iaGw2YjhXSDVLWmpMaldWYWdrQWtxZ05SRmM0Y0JLNFJEclFObjFDTVN4SEk0UGgxX1NNUWRtdTNLZEdPWGxKVWpfaDVMZmVDSmVRVkZ4cnE5c3VEVGR3UThMVVFGZFpjdS03OENTdjM3Snd1TFFVY1R6ZTBHa29OaGllVlpJaWdNQWU5ck5lSWFmRW5seVo1cUhVTGxPVnNNcWtGNVdxbXhmNHlNNjc3cGxPV21reTZIeGQtWGl4SGlMRHFDRjVyTnZTOEgzS3kxSDFLbDJLWm1MX2NZYnZmdXpBaERsTDBTZncyaTR3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPUEpJREtJZFcwTlZpcWRJNk9jLXR6aUU4aVBiejZ0cmwzX2NNcmF2M0V5S29uVHExMXI1RGZvUmRIWVZNZDlsY2tRTTBNNnNKU1EzX3FkdjBDOGJDaHRlSVJaeVRKTDRETVVaME5rRExuUE12N2lDdDR0ZEdGN3ZoaEtEWUQyek43b0xsU05XaU0xQVFlTFl6QkszRHVNcnh6em9fLU9DR1NVRjFWUnNSN1RIZFhPV2p3Mlk1NGI0OUs3Q2NNcFJ1QURCd1M4RmN5?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2010,42 +2010,42 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46073.38701388889</v>
+        <v>46073.61746527778</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TC Hasselt - Sept ans de prison pour des violences sexuelles sur ses deux belles-petites-filles - La Libre.be</t>
+          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>TC Hasselt - Seven years in prison for sexual violence against his two step-granddaughters - La Libre.be</t>
+          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:55:00 GMT</t>
+          <t>Sat, 21 Feb 2026 11:03:22 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOclBuU1RUenlOSXdkOXhpbFZkYndoLXF4aFAtUzFidUtabDlLemJ4bklOLTFMcWRKVk50VnRCaHZxOURvLTl1TTNuSm5CZFQxOHJfNFpqdVYybzRuR2RRS3QwbGVJdHhRWkZxWDhvancybUctWUdpTGNmZkpjclJSa1E5S1haTW93SWUxYURpS3plQ2wtTGxXaEc4d0RTQ3dfRFhOM296SGtMc0s1NU1HM19yeXRZYk5ic1RJOUQxdXRSQUVoY2dseGU3UGlaMlZaRkwwOG4wWmVxQi1fdm1Fa0lBWm51ek9XTnBvUUE3QmJhU1Bnc2pxLXdWX2lhcFpoNk5HVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8waEpNdEZmMmtDMFhIVzRBZ0QteWtGc0JMUjRFT2hzUXNGa25Pa2FPNzRHSWtUZVVvcGNORnNvYjFVZ2dIeVBMNEs4dTBvdVhmYUt0UWx6T0RQR2daak9ZR2p2SFpZU3lRS2dNaXJ0M0pSMGM3bmcyeEJvT1Y?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46073.41319444445</v>
+        <v>46074.4606712963</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>"Samedi 21 février, l’extrême droite marche dans les rues de Lyon, et nous continuerons à résister" - Politis.fr</t>
+          <t>​Lkr. Würzburg: Nach Einbrüchen in Kürnach und Gerbrunn – Zeugen gesucht - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>“Saturday February 21, the far right marches in the streets of Lyon, and we will continue to resist” - Politis.fr</t>
+          <t>​Lkr. Würzburg: Witnesses wanted after break-ins in Kürnach and Gerbrunn - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 14:49:09 GMT</t>
+          <t>Fri, 20 Feb 2026 15:00:00 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPUEpJREtJZFcwTlZpcWRJNk9jLXR6aUU4aVBiejZ0cmwzX2NNcmF2M0V5S29uVHExMXI1RGZvUmRIWVZNZDlsY2tRTTBNNnNKU1EzX3FkdjBDOGJDaHRlSVJaeVRKTDRETVVaME5rRExuUE12N2lDdDR0ZEdGN3ZoaEtEWUQyek43b0xsU05XaU0xQVFlTFl6QkszRHVNcnh6em9fLU9DR1NVRjFWUnNSN1RIZFhPV2p3Mlk1NGI0OUs3Q2NNcFJ1QURCd1M4RmN5?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQV2FjWFB5LVFqM0tJZm9pMkpqcThoaFFTWmt5V1JwUTYtT2RqejFFdF9XZTZOZmFubERuZEZBMGJKbWxFMHVNdDdWRVNBbDhBNXYydEZMRjZ4VGRtV0MtVWZBQzhhQnAyTkc1NzlpOUlORGptMFRkaVFwNjZ3RDJtTmNQbnI0eWsxSHhTdnNmTVh4eWxhTWo0a0FUcjUwOTBZZ0xjVm1FNks0YU0?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46073.61746527778</v>
+        <v>46073.625</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Jeugd Patro Eisden Maasmechelen vs RFC Liege Livescore,... - SportyTV</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Youth Patro Eisden Maasmechelen vs RFC Liege Livescore,... - SportyTV</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 10:06:22 GMT</t>
+          <t>Sat, 21 Feb 2026 11:43:11 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxObldNLU5POXlqSFY5bzV5TGJ3Qy1qbEE0SlYxUk41YlZsNW9yOHhGMW9XdjE4aDZpVXd6bjNoV3lSMTFIUFBqSjdyWXdhb3Byd2RFZU9Vb2lJbklsRWRaQ1paampuV0doRmZieHZPU2hnSmFIeVJzajU3YjNqSVpXcXJiTWxqbWwxV2tlcll4SUIweGdmc3FjaGI1R0s?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46073.42108796296</v>
+        <v>46074.48832175926</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>French PM says government intends to criminalize calls for any country’s destruction - The Times of Israel</t>
+          <t>​Ochsenfurt: E-Scooter-Fahrer mit fast drei Promille erwischt - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>French PM says government intends to criminalize calls for any country’s destruction - The Times of Israel</t>
+          <t>​Ochsenfurt: E-scooter driver caught with almost three per mille - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:57:21 GMT</t>
+          <t>Fri, 20 Feb 2026 15:15:00 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPdHVVcjRxOUM5a2JxNUlFUjNPdG5iTTc2UDk1cFU1c1ZCd1ltODY4blN2UTdXcGYwN3ZSWXZyV3pFMXZTZWlRemlhTmVib2EtMmhlVHd2RGdNaWlvMmQ2clpBWUYyakE2R09aR1F6Mnk1MHNqV0FsVjlUWmZyWkJuVG03NmstTmIzVmxfQlZkdnNVZmR3N0JabFR3Z1ptOEtRQ1ROQ3huWlZuOHZFV21NeFRyWkVhMmxvOUVhTzdFZ2xJN0xYU0piZA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxONmFITnUybVNkanBFVkpVbU55VktuTUJRYzJacnlFdXA2X1ZvakdvMlo5RGxkZ2E0aDl4R2xsbVAwdUhPY2Jfclg2S0dIYU1OV0lWZkJSZ25iMVQ5ck5UX19lZlByeHlZSjVSY09VLTJYWHFObmZXbEtNVmlFUWRUZ0lxQ0FUMzVhWDRNbXl6RmRfVkNtMnZWb2tDSGg?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,52 +2220,52 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46073.41482638889</v>
+        <v>46073.63541666666</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Hundreds of Belgians locked up in foreign prisons - The Brussels Times</t>
+          <t>Bad Neustadt: Person von Güterzug erfasst – Bahnstrecke war stundenlang gesperrt - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Hundreds of Belgians locked up in foreign prisons - The Brussels Times</t>
+          <t>Bad Neustadt: Person hit by freight train - railway line was closed for hours - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 12:13:14 GMT</t>
+          <t>Fri, 20 Feb 2026 16:30:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOM1dqd09VU1RVSjFaYnlfVzlYRmUzc0lWZXN0TVRmZDdOdmJzaTE5TmRxQ1VncHpGM3BJSFItLTVTSktKNDRjdFJEMVVsNHBtbUo1R1J3eFJhdnRhR05RMHk5MExTdGNENnROZ1g2NXREUFZjNU1pWFBEUE9zS3dlckYzSFdSbVhqa3lDTUNFZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNZ1BkcFp4Smw0OVB5M1hrbk5nWmp3ZHdWUWVMMGEzSjN1MjNUSDR2djNsd19kS0o3NTJtblg5Umw4R1lFOWYxRE83bGlHd3hjRU1XNlh3Q1pESndBNFdnTmV1T2VsM0xJcm1Ub0Z6cUNCTGdMVkh0blNhNk5fcjlNalk1aW5INmtPM3A2QUdnUG1seGoyMzVDX2JHLXEyY3hTd1pJQlZVWU9IMWkwMU4xb1pQZzJOQ1hSNHc?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46073.50918981482</v>
+        <v>46073.6875</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 16:35:57 GMT</t>
+          <t>Fri, 20 Feb 2026 15:22:25 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8waEpNdEZmMmtDMFhIVzRBZ0QteWtGc0JMUjRFT2hzUXNGa25Pa2FPNzRHSWtUZVVvcGNORnNvYjFVZ2dIeVBMNEs4dTBvdVhmYUt0UWx6T0RQR2daak9ZR2p2SFpZU3lRS2dNaXJ0M0pSMGM3bmcyeEJvT1Y?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNb01GazY5VElxMXdSWmg3MnpPcFFIYy1pM1FzTFV6enF3SG81MzhFS0xPNzlDUzZCcm5aMXF6NzdEanlKRnpFbHBuNVJqSGN4MU1sUGIzYTZUWldieTF5UHhrQVdQbmZaT0pOOV9QYTZBbTFvdlc2dlVSaER0QVFGQ1Rpc2N3Tlh2WDFIUlZTM1VXYko5YVZZVk5jZlJMb1ExYWVpUnNhamRqUTdPUUIxaUJNNFpONXNU?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2344,38 +2344,38 @@
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46073.69163194444</v>
+        <v>46073.64056712963</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Wertheim: 48 junge Beamte zu Polizeiobermeistern ernannt - Fränkische Nachrichten</t>
+          <t>Meet the Palm Beach billionaire who paid $2 million for a private White House visit with Trump - AOL.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Wertheim: 48 young officers appointed police chiefs - Fränkische Nachrichten</t>
+          <t>Meet the Palm Beach billionaire who paid $2 million for a private White House visit with Trump - AOL.com</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:00:00 GMT</t>
+          <t>Fri, 20 Feb 2026 14:50:03 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOVmx1X1F5RFNnSlRmakZ1d2dxcmtYcnJQWFdSeVlKWVBCMzE0Y3d6b1VSVTRPN1l5LWZPa2NGX25Gb0ktUEVxaEFnYkpHc1pTTHl3WTkxMHhrRlVnazRPcE9JcE1OaExlRHhEZ2ZRYkN4TWRSakg5VFdodHAwV0pRSHI2TlRLU1dXZjNXVDVEVDNULXI3amZuX0FLVEFCTWVDX05VTG16bE1WYWtkRVBoVXFkbUxmYjdzSlhTMEhsRzBKTDBFTGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQdDllcG81Ym1TUUc2aFJtMjliUGh4QjF1cFNFLWtpcnRHLS02XzE0NzYwWTNwZWNiZ29SVUpjdmhPSEFfeFNZVFRUem9wOG05S3RQR1ZVVmNoZXZXdzBWTXRoY0ZPUFFWWUM2dFJSUW1tWmVNeTJMQkw5VlZFakFGT3pR?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46073.45833333334</v>
+        <v>46073.61809027778</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>​Lkr. Würzburg: Nach Einbrüchen in Kürnach und Gerbrunn – Zeugen gesucht - Charivari Würzburg</t>
+          <t>Serie von Pkw-Aufbrüchen in Ingolstadt: Die Polizei hofft auf Zeugen-Hinweise - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>​Lkr. Würzburg: Witnesses wanted after break-ins in Kürnach and Gerbrunn - Charivari Würzburg</t>
+          <t>Series of car break-ins in Ingolstadt: The police are hoping for information from witnesses - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:00:00 GMT</t>
+          <t>Sat, 21 Feb 2026 13:06:00 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQV2FjWFB5LVFqM0tJZm9pMkpqcThoaFFTWmt5V1JwUTYtT2RqejFFdF9XZTZOZmFubERuZEZBMGJKbWxFMHVNdDdWRVNBbDhBNXYydEZMRjZ4VGRtV0MtVWZBQzhhQnAyTkc1NzlpOUlORGptMFRkaVFwNjZ3RDJtTmNQbnI0eWsxSHhTdnNmTVh4eWxhTWo0a0FUcjUwOTBZZ0xjVm1FNks0YU0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE00R0p0QnpCVEpWcXV3TlJkOUsyb1dEUDRGM1VVU0JUUVRhZHF5YnZBbjczX2FORHVxRERzSjBUNzVaUW40QTM2V0VfTmV0cWt5N0s2c3hWd2g0S2trV3lJRDExeW5ORHhPUVE?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2454,38 +2454,38 @@
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46073.625</v>
+        <v>46074.54583333333</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>​Ochsenfurt: E-Scooter-Fahrer mit fast drei Promille erwischt - Charivari Würzburg</t>
+          <t>Verkehrskontrolle endet mit Hausdurchsuchung - RegionalReporter</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>​Ochsenfurt: E-scooter driver caught with almost three per mille - Charivari Würzburg</t>
+          <t>Traffic stop ends with house search - RegionalReporter</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:15:00 GMT</t>
+          <t>Sat, 21 Feb 2026 08:36:45 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxONmFITnUybVNkanBFVkpVbU55VktuTUJRYzJacnlFdXA2X1ZvakdvMlo5RGxkZ2E0aDl4R2xsbVAwdUhPY2Jfclg2S0dIYU1OV0lWZkJSZ25iMVQ5ck5UX19lZlByeHlZSjVSY09VLTJYWHFObmZXbEtNVmlFUWRUZ0lxQ0FUMzVhWDRNbXl6RmRfVkNtMnZWb2tDSGg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOZTZ4YW9vQXJUMWc5N3VZV3E0QWdnd2NhOUZRcFZXcjM4c2w1NnVRWE11LWk1dmU0NThiaVBaS0ttYjRibG9YOHlIUFAyeXZfc09WdThvalllUG9yZG1KVDFHR3ZZVGlZZkdnTEVvOUd6SjUzZ2E3S1BtZXA1RF9QT1lJSVlyb2RoZzRXNnN5Z1pVTDZRVk9KWEJLb2hNa09WVUE?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2509,38 +2509,38 @@
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46073.63541666666</v>
+        <v>46074.35885416667</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Bad Neustadt: Person von Güterzug erfasst – Bahnstrecke war stundenlang gesperrt - Charivari Würzburg</t>
+          <t>Studentenparty in Ingolstadt endet blutig - RegionalReporter</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Bad Neustadt: Person hit by freight train - railway line was closed for hours - Charivari Würzburg</t>
+          <t>Student party in Ingolstadt ends bloody - RegionalReporter</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 16:30:00 GMT</t>
+          <t>Sat, 21 Feb 2026 08:32:05 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNZ1BkcFp4Smw0OVB5M1hrbk5nWmp3ZHdWUWVMMGEzSjN1MjNUSDR2djNsd19kS0o3NTJtblg5Umw4R1lFOWYxRE83bGlHd3hjRU1XNlh3Q1pESndBNFdnTmV1T2VsM0xJcm1Ub0Z6cUNCTGdMVkh0blNhNk5fcjlNalk1aW5INmtPM3A2QUdnUG1seGoyMzVDX2JHLXEyY3hTd1pJQlZVWU9IMWkwMU4xb1pQZzJOQ1hSNHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNekFGTXBBUWExY0VBZ3MxMGVSMVpGektSMWpvdU1DQXRMV0U5VTAwbUFwMTNUUUtXNzJfV25rWXpTRE9wQTBoYjZiX1lhcnhETFVnUFp5WDFZaC1maEtiMFBtNEU5azBkakRTU2hDbGVHalFfRTlOaEhGOGJMODEzM1Q3RWJIeVFOLUQ5Yi1IVUtqaTMtbFpkTzk4RzR3WVdGWlE?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2564,38 +2564,38 @@
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46073.6875</v>
+        <v>46074.35561342593</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Aschaffenburg aktuell am Freitag: Hier nimmt die Polizei am 20.02.2026 Raser ins Visier - News.de</t>
+          <t>Studenten-Party in Ingolstadt eskaliert: Schlägerei fordert zwei Verletzte - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Aschaffenburg currently on Friday: Here the police are targeting speeders on February 20th, 2026 - News.de</t>
+          <t>Student party in Ingolstadt escalates: Brawl leaves two injured - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:15:00 GMT</t>
+          <t>Sat, 21 Feb 2026 11:50:22 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQNkVuMENSQnJIdUE5ZUpFWWJRNHZVeEVXcHFMQVRwQ1hub2V0Q1VmdDZtS2hsSDQ1d2JiUjhrTW11bHZjWXcxQ0tfNmZpRUdYVHY3OTlzblhSMUVKNmU3THJFdXhNTTd1SGczbjdwbmJDWjNOLS1femx5UjJpUmR5NzNsN3EwWGI2Q3Frb2RESlNBcF9wcVM0WnN0QUdYQ2o2YXJQTDQ5ekJ5bEtFYjlxZlBkOGVUby1lbzFqbXJqMjNVdU5oMEZNZFRYNG5NY0txbFNrUTdNOWJmX1ZibzRtZkN1UC0wVzI2V0hua0pFcllSbFAtSVRn0gH8AUFVX3lxTE90amswVGNHQ01Odnl5TkpmNkQzd2laX3VMSXJjaXQzU3JRcGlfbnJfUi10LWlSM1JjM29KSWIyanFZWnNtcHN3Xy1KOHFIdWRRN2EwUERsWHVrZTZKaWc1bENIdHpGb1Ztb1pKNGNkeVZnQ2lnTi0tRWZlVERwNW5aWGhLOFVPMG8xWmF0OXYtd1QwLVJjaTdWU3hqRkIzV0pRSWk5eW5KelRnbE5IM1cwQ1hDQTBNWko3bS1kdkdPR3V1N09IVEpKRHNTNnhNUFdZUlBCM01oSlFIMlNBMG1SbzRxM1hIVjh5ZG9fNlJGdkU3TU41WXEwUG13SA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE9tcFJnQUMzR01xVm9seU9EU0dPQVFlODV5UGI3anJnME93UHNxQnNXME5mVktrdnVNUEpzLUo2ajhhNzJNb2JjMnBpWmdYUUYtaElTSFY4Nl9mcHNranlpSXQ3cTVHdXVPT3p3Z1lyNkFvbHc1SEZSbzFzcw?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2619,38 +2619,38 @@
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46073.55208333334</v>
+        <v>46074.49331018519</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Polizei-News Bamberg / Schweinfurt / Würzburg, 20.02.26: Zollamt Schweinfurt intensiviert Kampf gegen Schwarzarbeit 2025 - News.de</t>
+          <t>Why the Audi A6 e-tron makes me thankful for wing mirrors - evo.co.uk</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Police News Bamberg / Schweinfurt / Würzburg, February 20, 2026: Schweinfurt Customs Office intensifies the fight against undeclared work 2025 - News.de</t>
+          <t>Why the Audi A6 e-tron makes me thankful for wing mirrors - evo.co.uk</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 09:54:02 GMT</t>
+          <t>Fri, 20 Feb 2026 17:59:48 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPT0gzcXJvcDBRa3pZM3AxVzlTeldTSVU5aGVZSmMwclE3STQ1RTE3c2RXNW9abjg1QXY3ZTQ1UWs1ZVUxX0o1R1BITEdWYmVncXd5aXB0MnlrcG5YT29DS1JTQ3pnb2dBMEZ2RU1kUTV6THlBeXlUejJjTlV1cXpZS01YRUU2a0ZEWmtTdUJRQTQ5eFh3THEtU0RnOEdaV2dleUltLXpSaHRtZUxRdlFV0gG0AUFVX3lxTFB1WmM1eFdVSHVJTVVXN1F4dTRsRkpaaTVWTFZxVWVwMG1JdENPelhXVndjX01Gb3p1NndvblN5WjJPTWdUMG52eFcxOWxDenRSWnBvb0tCUllITTJyNmZDR2t0S2lqbnVnZ2dBMkhIRnBOLXNpbmZ2bnJ2b25IOEtoSmROUDlfajRpLW11Z01lTzUzS3VGZS1oTHZybmxBYkFXdmszQXdtRzJ0Z05lOHozNGFuSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQZDhCYURsaFYtb081ZzlCQ1ZyQzdnRHB3OGU1OEozWVVlTmMwbEVSanFlc0IteFlwdkVQa1hSU3FFVlVlNnAyd2RDZ2I2eW5PT2FPUTNiaWNuSTFaVXlUSEkwWXVETXJPSTc1Z2g0ckFoZ0lKRjd6QUlmeXQ2cjBKQVVheXRDTnl3cEJNOFpxYXVxMHZ5bmIyVXNpeTVRcTM3ZGJEMlZPSEJSUQ?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46073.41252314814</v>
+        <v>46073.74986111111</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Demo-Termine heute, 20.02.2026: Wo gibt's am Freitag Demos gegen AfD, Menschenhass und Rechtsruck? - News.de</t>
+          <t>See The Guests At An Exclusive Preview Of Kildare Village’s The Edit - The Gloss Magazine</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Demo dates today, February 20th, 2026: Where will there be demos against AfD, misanthropy and the shift to the right on Friday? - News.de</t>
+          <t>See The Guests At An Exclusive Preview Of Kildare Village’s The Edit - The Gloss Magazine</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 13:25:00 GMT</t>
+          <t>Fri, 20 Feb 2026 17:55:26 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxNWTdIQ1g4R3pnTEZCSHU0dFZnX3M2OURENy1obTNCUDBjQWFQa0VZTFZ5RWJoRFl5ajY0RGktdXBvOTZZbXo5QU4ya25BVlhKVjJHV1ZEM3pfR0dfc2NPRDAwMTJtcUt3cTlUZWlUZ3FvZEV1bUNaUERVeWxjWW5rMzFqSnY3LWVoa0ZyUFdJa09UamZlVUs3RHQ0c0JvemxJYzZWajBpNk1MSGVqNlYzY19rbi1YSGdFQ3ozMW9oNE5GbVBsOTRkNzUzeTRranhOY0w3RldDZGZNZHF1NUdyMFpiM3pvUWQ4S0JnSXpiTDhnbVVER2RWak1jNWZWY215TG5r0gGIAkFVX3lxTE1QblRoS0tQdEFtdVNHdzQ3YUIyb1pVOEFmeTk4NDRVb3RDNTVhYW1rVmN3RmlZd0NYeFpaVTR1VDhFakNuYWpLY0VzLURIM2VMUlI2aWNtS1VzUjRVZFkxV1IyQl9vNm1LdjdqWnVQZE0zOElnc082VDE1Vzd2UUhHcThnRm1sMzNyLXpyRTh4REdFWEptVTF1dmdFMVhKb2RUTGsxclR1WVhiYkY0dWV2ekhuTERlUkhUaExhOXNuQXNXWlVhRUNLVlUteWZpOE1mb3lpSXVHa01VY0lWeW9XSHA3UlV0b2RJRWlFVXJhU2o0QndFdlhUdGk4VWhZLWFGWXk2Z1hKNg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOMkxfOWp5U1FDTThlcGN2UV9HUUV3SXp4NlppbE52Ym0ydGpNMTc3b2d5RnZmLVVfQUpiYVRIM1A3b1RWNGsxTUJGelRNeWNBZU9MU1ZDdmZaVzVkeFJ3Rk9zeDNSY09pbkd0QnFVaFFJSXdYVWw4NVQ5M0lqMkwweG9YNkF6RDJtcFdudG5EQXhYUQ?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46073.55902777778</v>
+        <v>46073.7468287037</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City France English</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Paris" OR "Île-de-France") AND "France" AND ("bomb threat" OR "suspicious package" OR "shooting" OR "stabbing" OR "terror attack" OR "police operation" OR evacuation) AND -Texas AND -"Paris, Texas" AND -film AND -movie AND -football AND -transfer</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Polizeimeldung Bamberg, 20.02.2026: Einbrecher entkommen mit Tresor - News.de</t>
+          <t>Bomb threat in Paris as major landmarks evacuated by police - The Mirror</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Police report Bamberg, February 20, 2026: Burglars escape with a safe - News.de</t>
+          <t>Bomb threat in Paris as major landmarks evacuated by police - The Mirror</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 11:35:02 GMT</t>
+          <t>Fri, 20 Feb 2026 21:57:21 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQTDRVeGxRTzBmZ200OEl2d2huS2VhcFZvTWxucWc0VVhaQkJzak96dW51NEt3V2g3SC1INEZmWXdjbDBVbVRqeDl0NDBqYzJZSHV6Vllwa1NXbC1YRGRLWkpmbWFKdFBHSW5WWVFLQW1vb3hfeWIyY2R1bm5EUllUTkRtLW5iQ3phV3pNSjF0S3dyYS1XZzZkOTd6NG9UWFY1c3Qw0gGoAUFVX3lxTFBlLXFyeU1ONEpmNEV5bFpuQUV6V0lhazdlY21XUFpZaUpVUVFEUVBGbjItWEJaX3ZxWVZpSW1UczJCak9DNkxiMW9NTFhZeXhDUmR0R3M5WGFJbjQtUjN5TldKbkdZOVIyVTVKcUZJd2VHdjdBektOT2ltZ1VwREZDSmFqWVdKeXVBbEhZcGRZYXAzTjhDOW5wX1o2d05SU3RwOTdCSTk4Xw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxORmk1NjhhUjlMSTNZOVJJb2luVGwwXzlNZVNhUFFMOU55VUs2cllsellWdENXUjNuSHBCRVZlY2p6X1paTVg4LVlHWlNzbnMzWllhWlJ0Sm1mSnNmQVZlZXdSdUdrdHBjWTVpMVI3cmp4LTZrQlQ1dUdhcFQ4NDlITmF1SnBfcm1nUkN30gGQAUFVX3lxTE13b1hBY3Bsb3luazcwcTIwWTRnM2lIN3VKX1RzZFNEbk8xVExIVWhyYXNqcS1EbjZoWUZhQ1JHREtyc2pLdnZkNGVORG1FbnNVMmtvUFFqS3lpd0pJdWFGc2p5QURxengwUUFsa29kVWpsbFdjc2VFbFNlMlpSNExNeVNmNGp3Y2h4a2NpazBaVA?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>FR:en</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46073.48266203704</v>
+        <v>46073.91482638889</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City France French</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Paris" OR "Île-de-France") AND ("alerte à la bombe" OR "colis suspect" OR "menace à la bombe" OR fusillade OR "attentat" OR "attaque au couteau" OR "opération de police" OR évacuation) AND -immobilier AND -"prix immobilier" AND -foot AND -transfert AND -Texas</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
+          <t>INFO BFMTV. Tour Montparnasse et Sciences Po évacués après un signalement: levée de doute terminée, aucun engin explosif trouvé - BFM</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Business of Healthcare Summit welcomes another packed house - Florida State University News</t>
+          <t>INFO BFMTV. Tour Montparnasse and Sciences Po evacuated after a report: doubt cleared, no explosive device found - BFM</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fri, 20 Feb 2026 15:22:25 GMT</t>
+          <t>Fri, 20 Feb 2026 19:22:16 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNb01GazY5VElxMXdSWmg3MnpPcFFIYy1pM1FzTFV6enF3SG81MzhFS0xPNzlDUzZCcm5aMXF6NzdEanlKRnpFbHBuNVJqSGN4MU1sUGIzYTZUWldieTF5UHhrQVdQbmZaT0pOOV9QYTZBbTFvdlc2dlVSaER0QVFGQ1Rpc2N3Tlh2WDFIUlZTM1VXYko5YVZZVk5jZlJMb1ExYWVpUnNhamRqUTdPUUIxaUJNNFpONXNU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxNRDdZR2stLV9SN1dDaG9yTlUyN3VzUEpVa2VpVnc5ZXQtX1FoR0tVWDlpXzlhSW5xd1FDcVNBSzBPdGtwLWpnQ0RTRy1TcTUyRGFNbG5nM2RrSkdPZVU1Y0pKUFlsbG81SVdqaWZyaWdfVXlOVUxUNnhMN1VUbGtWX1lwTWM5ZmUyNXdHOVFlUy1DVFpQa3lvVW1mcTh3b0hYX3E5R0wtTW44N1M1bHhpX1V1MGFPVnd6bzZwdUVudjJmVGNhSjZ3NE1fQk94RTh1RG5DOXdseVZtb3hhbGNwckZXTlZBYXBfeGlsUlZhTHpvR3NyWXhJZW9acEZIaWtBa2psbTJSSG1sWkNS?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,681 +2825,21 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>FR:fr</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46073.64056712963</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Village Wertheim (fallback)</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>University of Florida expands study abroad with Antarctic expedition - Gainesville Sun</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 10:02:00 GMT</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPdkVfYlpLQ2ViMnBuUy1hUUtTYUhZbFhiUlNHeUJ2cEkzT3QtWEdBcHRDS2tnZ0dWSVBSZ2tGRnUtYjBHbnB5eVN1Z2gzWUtlZVNTZXR3UFZiZDBsQ1NaRWJlNEcyNHlUbWhiNDNlMjMtMjJkaHZKVWtOVGJ2OG9mZm1qWmVRWkFQaGRSaXlnSGM4NzhuSlkwcWplaTF2dXVHMGZjVHZzSWxtdW9ZWmtnNkpVQTVHZjlaMVRSQ0FKR0lWT01zcVROVi1nQnl1NV9NR2p3ZkI2X05Ua1k?oc=5</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K45" s="1" t="n">
-        <v>46073.41805555556</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Autobahn gesperrt: Getränkelaster rutscht in die Leitplanke – Unfall auf A93 - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Motorway closed: drinks truck slides into the guardrail - accident on A93 - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 10:46:49 GMT</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQb2RxcW1rQ0l1LWN0UnJ6c2RNXzdPdGJwbW9IWjlSN3czX1NaRE9LSGIyZ0JuRi1aWTFrVFBHTEdmaFdUZXZ3T3NRcmI3dHp3WkF6NGYxeUtjLS1XUlZROW5jcG0tS1lCdEFGZl9ibi1VLUFoSjFnS3pmc3E3VDdkS2JBNWRUX3hhU05qcThTM29hWTFXLW5temVmR0w0QzBsbWZKeFJtZnZlUjE2YVNPVXpMVWZWNlN4MHFFY0h1Z0lkX2VvVnhuNHBxTnV1dWxKR0NBZDcyQjVyRFVMM3NDRw?oc=5</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K46" s="1" t="n">
-        <v>46073.44917824074</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Vollsperrung der A93 bei Wolnzach nach Sattelzug-Unfall mit Ladungs-Verlust - Pfaffenhofen Today</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Complete closure of the A93 near Wolnzach after a tractor-trailer accident with loss of load - Pfaffenhofen Today</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 12:23:00 GMT</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBmdXlwZFk1ckJ3R05ia2YwTVNwcm9xTzY4VTBpREN3REYxMUwzMzZ0SkFOeWpHQ25yR25mNWs5M2xvSzBXcV9uTHdLLUUwcmdieFJLS1JoMHBkbjdfTUN0N2tjV2tUU3c?oc=5</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K47" s="1" t="n">
-        <v>46073.51597222222</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Why the Audi A6 e-tron makes me thankful for wing mirrors - evo.co.uk</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Why the Audi A6 e-tron makes me thankful for wing mirrors - evo.co.uk</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 17:59:48 GMT</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQZDhCYURsaFYtb081ZzlCQ1ZyQzdnRHB3OGU1OEozWVVlTmMwbEVSanFlc0IteFlwdkVQa1hSU3FFVlVlNnAyd2RDZ2I2eW5PT2FPUTNiaWNuSTFaVXlUSEkwWXVETXJPSTc1Z2g0ckFoZ0lKRjd6QUlmeXQ2cjBKQVVheXRDTnl3cEJNOFpxYXVxMHZ5bmIyVXNpeTVRcTM3ZGJEMlZPSEJSUQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K48" s="1" t="n">
-        <v>46073.74986111111</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>New attendance record! Remaining regular season games sold out - EHC Red Bull München</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 11:30:00 GMT</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPQmRWY0VOQzRiY3U1amZfOUIwSVplbGFjTkpXUGxfQ25IWjQtWlMyN1gwcmMtVm1LSnNBMzFGYnJaYklsMG1RdG15R2JBVWFXcHF3R1NGUmZGcHpUSGFnb0RhdUZVXzBCMlJKbWs1ODJ6WHY0Si1rMkRXZmVUaFZZU2lCZnNzUnhWdmQyaXkySmJ5R0l6QlBqV04wMTMtVHJKZW5oN05PT3RtZktCNWVyS2pYYUh0UGZ3RVE?oc=5</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K49" s="1" t="n">
-        <v>46073.47916666666</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>FC Ingolstadt 04 vs. TSV Havelse - Boxscore - Live Score - February 21, 2026 - FOX Sports</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>FC Ingolstadt 04 vs. TSV Havelse - Boxscore - Live Score - February 21, 2026 - FOX Sports</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 11:37:50 GMT</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPT3BDbXZudFp6N2FtcVBuSWpWQmhTTVNWRkNlbk9mVlRSLUYwTW8zTkJ0ekZRcDUtYlNMMWI3bERueTNIRms3YTA5LUhNX25DaGlxZDc1eTkxZjFLLV96bmdtb0g5bDU2NVc3c3lOQWdRYWcya3BEalJKQ0hKSnFBY0cwdkRBc1MyanNfSTBLaDVhTklTSVpiMms2RzNydDl2bXZ0LUVld0lMemZCQ29nbnZtUW4?oc=5</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K50" s="1" t="n">
-        <v>46073.48460648148</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>News: New Audi RS 5 PHEV: Up to 639PS/825Nm, 8-speed gearbox, quattro AWD - CarSifu</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>News: New Audi RS 5 PHEV: Up to 639PS/825Nm, 8-speed gearbox, quattro AWD - CarSifu</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 09:08:29 GMT</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOd3M4d3l4OHplRHNoNW1EYzBiVzkwNHRMcFh6RWRKRWFEUktLWXJQbzVab3dKSVFZSTYyMDVMZE0xenFEWUNWU201Tk85bXJudnlKOUdVaTlXS1puRmhybzVZa3BJcWpJN3NxNEFSUjhBZFFvcVNDYU03Z3pJMk15RTE1MURBLWUyYUwwQWVzdGtrS0tWX093?oc=5</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K51" s="1" t="n">
-        <v>46073.38089120371</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Surprising results: why more parents in Madrid are opting for gadget bans, making unexpected choices for the sake of family harmony - russpain.com</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 09:18:53 GMT</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPekk2OFAwVk0tWG5ua3NUdkQzQXV0T1B1WHpraDZIckNOeWZ6dHpkMjRQc3JKb1pkSV9WMkltZkdzanVQV0VtNmRqRTBBNXI0TWNWRjY0SlpuUV9uTHFuaFctbEJ6cWRKYm1kc3hjejhTV1pXMU9hOV9GMVpYcERnc1VwWGRkakNqNl8tcENveENHeGFaZHZZWVZUalA1WHMtWXkwNGpaTGxUbTNwWXow?oc=5</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K52" s="1" t="n">
-        <v>46073.38811342593</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>See The Guests At An Exclusive Preview Of Kildare Village’s The Edit - The Gloss Magazine</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>See The Guests At An Exclusive Preview Of Kildare Village’s The Edit - The Gloss Magazine</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 17:55:26 GMT</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOMkxfOWp5U1FDTThlcGN2UV9HUUV3SXp4NlppbE52Ym0ydGpNMTc3b2d5RnZmLVVfQUpiYVRIM1A3b1RWNGsxTUJGelRNeWNBZU9MU1ZDdmZaVzVkeFJ3Rk9zeDNSY09pbkd0QnFVaFFJSXdYVWw4NVQ5M0lqMkwweG9YNkF6RDJtcFdudG5EQXhYUQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K53" s="1" t="n">
-        <v>46073.7468287037</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>High Level City France English</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>("Paris" OR "Île-de-France") AND "France" AND ("bomb threat" OR "suspicious package" OR "shooting" OR "stabbing" OR "terror attack" OR "police operation" OR evacuation) AND -Texas AND -"Paris, Texas" AND -film AND -movie AND -football AND -transfer</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Bomb threat in Paris as major landmarks evacuated by police - The Mirror</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Bomb threat in Paris as major landmarks evacuated by police - The Mirror</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 21:57:21 GMT</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxORmk1NjhhUjlMSTNZOVJJb2luVGwwXzlNZVNhUFFMOU55VUs2cllsellWdENXUjNuSHBCRVZlY2p6X1paTVg4LVlHWlNzbnMzWllhWlJ0Sm1mSnNmQVZlZXdSdUdrdHBjWTVpMVI3cmp4LTZrQlQ1dUdhcFQ4NDlITmF1SnBfcm1nUkN30gGQAUFVX3lxTE13b1hBY3Bsb3luazcwcTIwWTRnM2lIN3VKX1RzZFNEbk8xVExIVWhyYXNqcS1EbjZoWUZhQ1JHREtyc2pLdnZkNGVORG1FbnNVMmtvUFFqS3lpd0pJdWFGc2p5QURxengwUUFsa29kVWpsbFdjc2VFbFNlMlpSNExNeVNmNGp3Y2h4a2NpazBaVA?oc=5</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>FR:en</t>
-        </is>
-      </c>
-      <c r="K54" s="1" t="n">
-        <v>46073.91482638889</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>High Level City France French</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>("Paris" OR "Île-de-France") AND ("alerte à la bombe" OR "colis suspect" OR "menace à la bombe" OR fusillade OR "attentat" OR "attaque au couteau" OR "opération de police" OR évacuation) AND -immobilier AND -"prix immobilier" AND -foot AND -transfert AND -Texas</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>INFO BFMTV. Tour Montparnasse et Sciences Po évacués après un signalement: levée de doute terminée, aucun engin explosif trouvé - BFM</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>INFO BFMTV. Tour Montparnasse and Sciences Po evacuated after a report: doubt cleared, no explosive device found - BFM</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 19:22:16 GMT</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxNRDdZR2stLV9SN1dDaG9yTlUyN3VzUEpVa2VpVnc5ZXQtX1FoR0tVWDlpXzlhSW5xd1FDcVNBSzBPdGtwLWpnQ0RTRy1TcTUyRGFNbG5nM2RrSkdPZVU1Y0pKUFlsbG81SVdqaWZyaWdfVXlOVUxUNnhMN1VUbGtWX1lwTWM5ZmUyNXdHOVFlUy1DVFpQa3lvVW1mcTh3b0hYX3E5R0wtTW44N1M1bHhpX1V1MGFPVnd6bzZwdUVudjJmVGNhSjZ3NE1fQk94RTh1RG5DOXdseVZtb3hhbGNwckZXTlZBYXBfeGlsUlZhTHpvR3NyWXhJZW9acEZIaWtBa2psbTJSSG1sWkNS?oc=5</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>fr</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>FR:fr</t>
-        </is>
-      </c>
-      <c r="K55" s="1" t="n">
         <v>46073.80712962963</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>High Level City France French</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>("Paris" OR "Île-de-France") AND ("alerte à la bombe" OR "colis suspect" OR "menace à la bombe" OR fusillade OR "attentat" OR "attaque au couteau" OR "opération de police" OR évacuation) AND -immobilier AND -"prix immobilier" AND -foot AND -transfert AND -Texas</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Alertes à la bombe à Paris, Sciences Po et la tour Montparnasse évacués - 20 Minutes</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Bomb alerts in Paris, Sciences Po and the Montparnasse tower evacuated - 20 Minutes</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Fri, 20 Feb 2026 20:17:00 GMT</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOcVFrb1pIOGJKdlU1OGIzRHd5dnJsZXY0NVBWbE55RmJ1QU1uS0NqYy1ESXBpdER6OUtZZ0JQVVdUdm04SzEtaENGN0RaWExiV2FHSGpuVUlVOGtmTzRXcGpKTlVUSjdSMXN3aXMyUGk1OUp4Z2NwZWtRbnlrRTdjM256NDhNNDRZXy1Lbk0wOHAzTnlLOTZhTXBnd1N0VDE1cVJRUmhPZTN3Vi1kdlRjWU5HZjZBU2R1dzlkZmxlMFBxMHRzWEpQekV3Tm8xQQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>fr</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>FR:fr</t>
-        </is>
-      </c>
-      <c r="K56" s="1" t="n">
-        <v>46073.84513888889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-22 14:27 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Prue Leith didn't want to 'overstay her welcome on GBBO - RTE.ie</t>
+          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Prue Leith didn't want to 'overstay her welcome on GBBO - RTE.ie</t>
+          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 11:58:59 GMT</t>
+          <t>Sat, 21 Feb 2026 22:32:35 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQa1JzWFZ1SzF3Y0U2dUI5aGtLeDRyTmZuVVMxMDRYQlZlcGYzX3puUHR1cnV0dDNqRWFJUDlxUXN3MDNnNVNtbVFyZUg3VU1iLTFHV09fb0NPWXpYU0NtYlhjTXpHZTEzMktSdGVYbHV1bXhWSEpOOElOSDlDeXhSeTRqNUo3M2E0c1ZTTUN2dHVmNUhVZXdxLTB3cEFhUjhFZ2VKaHo2WF8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQOGNjVDdzNXFXVEZHMEFmaGdnaVZTN1UzZ0txV1BGYzc1dm5CLTg2dmEtSEdYSVBlN3drRUVGSmJrNmg4QWxkdUd3by0wN0ZIRVNJd3c2cDJqenFCTnNyWTJyZnlEUVZ4MWFaU3p5LUJXNzNRWEhBVEVjUTQ1U2o2aGJn?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46074.49929398148</v>
+        <v>46074.93929398148</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>Schoten gelost in centrum Brussel, verdachten op de vlucht - BRUZZ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>Shots fired in the center of Brussels, suspects on the run - BRUZZ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 22:32:35 GMT</t>
+          <t>Sun, 22 Feb 2026 07:37:20 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQOGNjVDdzNXFXVEZHMEFmaGdnaVZTN1UzZ0txV1BGYzc1dm5CLTg2dmEtSEdYSVBlN3drRUVGSmJrNmg4QWxkdUd3by0wN0ZIRVNJd3c2cDJqenFCTnNyWTJyZnlEUVZ4MWFaU3p5LUJXNzNRWEhBVEVjUTQ1U2o2aGJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPWmo4U0ZjR3FRZk92dVJHZnhpUDBLY0hsMGc5SWhZblV0T0tfMllRNHEtLTZmZW1fZEg1dGE3NXFobHd1QjRMeUkxcW14YWM3R2JCa1E5RVg5SzZBenFmWi1pVkgtLVE0MXZ0dHdLVWZGZHc1cmxzQW0wY1hkRnFhU3NfMmpWb1B5N1VQWTJ1UndNcFRPbUx0Q0JOOFI0d0tQam4wNldB?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,21 +570,21 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46074.93929398148</v>
+        <v>46075.31759259259</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Opnieuw schoten gelost in Brussel: geen gewonden, verdachten op de vlucht - HLN</t>
+          <t>Explosief ontploft onder auto van volkszanger Frans Theunisz terwijl hij in Lanaken op het podium staat - HBVL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>More shots fired in Brussels: no injuries, suspects on the run - HLN</t>
+          <t>Explosive exploded under the car of folk singer Frans Theunisz while he was on stage in Lanaken - HBVL</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 03:29:49 GMT</t>
+          <t>Sun, 22 Feb 2026 14:24:32 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQanRHTmNGcXViYjdJMlFTTndRMW1Icnd2R2JmVVdzeHc0TF8zTm0yZlNsSlN1cWFac05oMllLNF9HQXBaUTFLdHpyRFQxWUQyRXQweTlMX0FBckNCakd4VUhvNTd3cDV3ekdUeUJ1bzRQLVBrUURqYk1OMmpHRGRQZlNYVlZ3dXdCRWFzNTBTQ2FIWWNtYnhkQ0s4b3FnZnZMRFNRVFpKZXBxMmQ2?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQSWlUQ2V3U012MWRWY0JOTGp0dlFiTVpoblhvUUk0NWJzdEt6aHJhcV94RElKX29NbG1xbmpLSlE1bXdxeW1RUFZCb0NLWExKNTJjU3R1WXBOclJNS2k5MktaOUVsOW9MTFpmVFNWSS1SbE9HQkQ3d2lFSWhLdnpPRC1oOEZqY0ZNMG1QSjR0a0tHLVFlemtYaUhpdERYN19NOEV5MEJ6S002bVZ2VjRnNnhvaklaMEJzSjVxc2JQUS1zMlRpMDc2Yml1LTVyYS00ZkJFazlQZFNhVVNta3FMbzYxU21WcWc4X2N2ZkdNYTM0dw?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46075.14570601852</v>
+        <v>46075.60037037037</v>
       </c>
     </row>
     <row r="5">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Goed nieuws voor Ronald, Zoë, Cillian en honderden Brusselaars: regering maakt 56 miljoen euro vrij voor achterstallige renovatiepremies - HLN</t>
+          <t>Ruben Van Gucht in shock: 'Bekentenis slaat in als een bom' - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Good news for Ronald, Zoë, Cillian and hundreds of Brussels residents: government releases 56 million euros for overdue renovation premiums - HLN</t>
+          <t>Ruben Van Gucht in shock: 'Confession hits like a bomb' - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 14:08:39 GMT</t>
+          <t>Sun, 22 Feb 2026 13:46:40 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxOeHNyNFpRc3ROUlVCWW8yNHo5OElBRWZwUnJyZUl3ekdWMWpMWkdYZ1pndFJJUkd5SzBlbWJ6c1MyN0xuQm1vQk9TdmoxMTExRUVhMm5nMmpjaFY4OEZIbGJQYWMzTXkwMWZUTEJTR3FwOFJyNU0zRjlmMU5ZQ2pzUWpkMGV6V3VLWnh2RWZNUlhQQWVwQS1nWjNjX1BhNkQyWDhqVGVJbTZVaDJva0dXQWVFU1dWTTRFNkVnUmZPMHhCSVVnQ1N4N0hTNlFSRFBQXzZaZ1hPVlF6bDNTTG91WmVNTUxYTHA5WC0zYUZWWWxETXVFdjIzM0RVTG9UVjly?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQNTBkNjR2dWVMcWRqcEp5MmM0eHZSenlEOWVsejhsOXM2aDZsdHhKMlI5Vm16NHJreWM0MlA3WmQ3LW5WUTNxMVg0bS04dFFtYUdpbHNfT256QWhHM1kzVDQzS0ZtVjdQLTZlWjJvaTR3WjNDQWRzNEhyNzgxV3c5U0FpaUYxXy10alJUOFNCYk5GTWlTTlVVZkw5VFluM1lBVkE?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46074.58934027778</v>
+        <v>46075.57407407407</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ongeval met letsel op Wilhelminalaan in Valkenburg - AD.nl</t>
+          <t>In lijstje met Obama Center: BBC tipt Kanal-Centre Pompidou in Brussel bij “zes meest veelbelovende museumopeningen ter wereld” - HLN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Accident with injuries on Wilhelminalaan in Valkenburg - AD.nl</t>
+          <t>In list with Obama Center: BBC recommends Kanal-Centre Pompidou in Brussels among “six most promising museum openings in the world” - HLN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 17:57:00 GMT</t>
+          <t>Sun, 22 Feb 2026 09:03:57 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQanpMRjRySTZPcTQydFUxQjVXUzhuTXJBT0VxWHh3REpmNFlDY2M4MVh5aV9HQUpoSGRuQ19NMTRXVGIxMXU1c0xCbWZ1VmdpUG01LVR5Znp0NmFtMW9GcUlpODNrSEFVbW55WEZpTG90ekpSb1BhRmJzWGZLLXNNc0YwUDZNNHNJUGdmWV9fdDVBVkt2LVBZdmJMcjJyazZBMUs1dzJET1FWYjdNb1VGMXJR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxPS18wMUl6RndXdjExZGZvZUx6N2IzQ3VKYXZvajZodkdJSi1wSnZLZ3VGcm1YM3NCSUF2bnhGenViTElvZDdLUjNwdnpWTGpXcWphdTlzakZtOE91UERQbmo5NDVUOFJLYkszc0s4eVVqaTFIYTlaVzJSWmlTSUtkTU9objhONDF0ckY0bk5GcW1haVVSVXljS2JLQWg5U3d0d1BLRi1FaTVaSzk0eDRaZHBlY3lPZDhUTzJMUDgxUlVvNFc4bVFEZVc3QWl0b2lBZndrNDNwdWZuWmlh?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,38 +914,38 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46074.74791666667</v>
+        <v>46075.37774305556</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>American citizen killed by an immigration agent in Texas last year, records show - NBC 5 Dallas-Fort Worth</t>
+          <t>Ongeval met letsel op Wilhelminalaan in Valkenburg - AD.nl</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>American citizen killed by an immigration agent in Texas last year, records show - NBC 5 Dallas-Fort Worth</t>
+          <t>Accident with injuries on Wilhelminalaan in Valkenburg - AD.nl</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 18:07:53 GMT</t>
+          <t>Sat, 21 Feb 2026 17:57:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPQW54SkdIdzdMaXZsemJzZE1qTXRnV2c4cGdxSWFHdHRJOTROcGVjTlhWVzNBamJWNURMTHpWT00tVzQ2STNXb2JWTEZzbGlrVDdCWUVkMWxKSU1LTmwtdDRHaHUxMG9QMk9jUkMxV1REVlNvaDVvUUUwaVlmX3lRLXFIWUpCeUszSzZNNGxMMEphSkVBUVFKeDdodUxCVE1ibHVnX1k1c3BMbTDSAbMBQVVfeXFMTXRyXzRwa0F4cWVkNHFLUUN5b3pPa3VxdUZnQ3FSVjJCbTROaFVBbl9VT0V4SUZ4U0ZEMURfVjBKZDlnd1R5Y3FRUFdvak5kMDk0TDJzcWVyUVdUSzZmWGhoMUVHbU9LN2FzQVVja2ZvZUZIMVhubUdpX2xjZURIanplTHZHdjlJTXpGVU5XdUJFZDd1TWtDa21iTHRNM0d0R3NZZTBlVko3bFB3S3RUeEdJMFk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQanpMRjRySTZPcTQydFUxQjVXUzhuTXJBT0VxWHh3REpmNFlDY2M4MVh5aV9HQUpoSGRuQ19NMTRXVGIxMXU1c0xCbWZ1VmdpUG01LVR5Znp0NmFtMW9GcUlpODNrSEFVbW55WEZpTG90ekpSb1BhRmJzWGZLLXNNc0YwUDZNNHNJUGdmWV9fdDVBVkt2LVBZdmJMcjJyazZBMUs1dzJET1FWYjdNb1VGMXJR?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46074.75547453704</v>
+        <v>46074.74791666667</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Yet Another Brussels Shooting: Gunfire Near Metro Station - The European Conservative</t>
+          <t>Berlaen viert jubileum als singer-songwriter met dubbel concert in Knipperlicht: “Mijn tweede thuis” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Yet Another Brussels Shooting: Gunfire Near Metro Station - The European Conservative</t>
+          <t>Berlaen celebrates his anniversary as a singer-songwriter with a double concert in Knipperlicht: “My second home” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 13:36:21 GMT</t>
+          <t>Sun, 22 Feb 2026 10:22:36 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPd25WaVVWZVRqMFFwU194S2gtVEpWUVJPbU5CLXFKVmR4QnJjcXczMzJHOGFzYjZGQlRfalgwTG1GV0lHcTZla3JWbHd5QmlNQmJCOWVIZFN0a0s2RTVQZkFrMkdMbjBqQWt5eDk2RnNjUUhBVkgtRm1Gd1RpUUdFZGlsWVpiOEd6cEY0SFNwb3lDVW1PWXp0M0wwLWd5RFlxNXVEY0R1R00ySHFkM0RocA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxOQ2ZNRUx5elg4NGlsbTI4UUdMM0tZZVgtYXpvXzhuUEtkLWN0dHJjeTdjTjVNUDU3bGJfSHNkdkFMMF9FSTBCdEpYVWtuRUpYajBjWHQ1TncxekloMFU4QzA3cV9vUEZlai1qRTNWbHJUcVA4WFFMVi12UG5GWmtBVndlQmcyY3FjaFV2SUVvamhqYkttYjQxSnVkUHJ4ZzUxNG9xclVXVVkwczNIcmJ6NTRnVTJYZTVjM3kzeXlFc2pJaFA3RTltS2pnNk1OWU5sYXhFWjZiYjF0WVBsWTBqVnBQa0tQU0VVcnM2VXpjelFkZjRreExBb2lDS0pQcW1QU1BzZ1FDYzI?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,11 +1020,11 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46074.56690972222</v>
+        <v>46075.43236111111</v>
       </c>
     </row>
     <row r="12">
@@ -1040,22 +1040,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
+          <t>American citizen killed by an immigration agent in Texas last year, records show - NBC 5 Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
+          <t>American citizen killed by an immigration agent in Texas last year, records show - NBC 5 Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 09:34:18 GMT</t>
+          <t>Sat, 21 Feb 2026 18:07:53 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNZlBCeEZXakZ5VVBhQWpxMEpCVzFtTm9CYlZ2emxsaXhUci1GUXRybGp0T2ZKRDJNYmFXYjFNZDRSS3NTLXBrRnVfS3RLRndzcFNTUU9rVGFmM3ZnV3hFbGNUN0JMVHRjSnpqWkVSWDFrS2pQa1JjeFZzN3luS2pqS1U3REhERHQ3dV9WUGVZeWl6Q014Sk5EenVfaGY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPQW54SkdIdzdMaXZsemJzZE1qTXRnV2c4cGdxSWFHdHRJOTROcGVjTlhWVzNBamJWNURMTHpWT00tVzQ2STNXb2JWTEZzbGlrVDdCWUVkMWxKSU1LTmwtdDRHaHUxMG9QMk9jUkMxV1REVlNvaDVvUUUwaVlmX3lRLXFIWUpCeUszSzZNNGxMMEphSkVBUVFKeDdodUxCVE1ibHVnX1k1c3BMbTDSAbMBQVVfeXFMTXRyXzRwa0F4cWVkNHFLUUN5b3pPa3VxdUZnQ3FSVjJCbTROaFVBbl9VT0V4SUZ4U0ZEMURfVjBKZDlnd1R5Y3FRUFdvak5kMDk0TDJzcWVyUVdUSzZmWGhoMUVHbU9LN2FzQVVja2ZvZUZIMVhubUdpX2xjZURIanplTHZHdjlJTXpGVU5XdUJFZDd1TWtDa21iTHRNM0d0R3NZZTBlVko3bFB3S3RUeEdJMFk?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46074.39881944445</v>
+        <v>46074.75547453704</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Nouvelle fusillade dans le centre de Bruxelles : ce que l’on sait - BruxellesToday</t>
+          <t>Fusillade rue d’Anderlecht à Bruxelles, les suspects en fuite - 7sur7.be</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>New shooting in the center of Brussels: what we know - BruxellesToday</t>
+          <t>Shooting on rue d'Anderlecht in Brussels, the suspects on the run - 7sur7.be</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 19:48:03 GMT</t>
+          <t>Sun, 22 Feb 2026 01:40:01 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOV1Q1Rjl3blc1OHpNQmFSeFNjMjlWeFN6MmpqeVBabkN6UExTald3eWVGd2JoZUQ2aFdBd1NRT0lieG1vcmxid0lqNmdlVE5IZmVvMFFRdHdiQXpMbHhIam93SzdWZTZlSkd4ZlVCNXNDU1ItM3BqWTdDZTRpbU43dUczSlVGMVN2enlTaDR3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPUEVSV3R2eHFabUEwaHNXYVMzOUI1R0pGb2JWZXpEODljRDdIbTZlT1E2aUxLbldLUW1yVW40WktaXzYyQV9QQ2xuMm9QSXhrRnZjUldIRlJMV013dXNIcHNZb2lESDY3ZVJkQzExRExCR3VVZzFPcWFCVzhVX01uTmkzMkVxeUJCVlFyaUVadFRoMkg1VWdIdWVUM1ZoTEoy?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46074.82503472222</v>
+        <v>46075.06945601852</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>La justice alerte contre le phishing via de fausses applications: “Impossible de distinguer le vrai du faux” - 7sur7.be</t>
+          <t>Un bébé de 16 mois retrouvé sans vie à Berchem, le parquet ouvre une enquête - BruxellesToday</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Justice warns against phishing via fake applications: “Impossible to distinguish real from fake” - 7sur7.be</t>
+          <t>A 16-month-old baby found lifeless in Berchem, the prosecution opens an investigation - BruxellesToday</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 06:20:52 GMT</t>
+          <t>Sun, 22 Feb 2026 12:40:00 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQOHpEb0RWNVpvS08zNmdON0xCMzUwN3VHZ21lcnFtS2syVEd6ZVAyNVJSdmduUy1vRVhpOUwtaV8xSksxVHA2UkNmRm4zQk5oMkpUVUplQzB4QU92SWRFTFNrQjZ6M0g3di1FeW1ZM1dXbmEweV9ISTRzZUR2ZUg5NVNabHdNajZRdE43bElzZVBodU5NUzl5OTZsMGJvam1fdTBVczE4RHc5UE9sd2NkdDFSNEdmNnF0X0ZLMUtzbllsZzhzbDhXVXB2UkF2S0RkN0FPcm1SaW9pNW93Z2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE0yMzAzNE9wYTFoTGJBLXdOWHpfRWJ5MUoxUGQxWHlMc09jQWZQY0l4Vm9FWlV0d2dRX2c2bWZTazRZRmg5cnZndmJzdmFXSi03eGhja0Y1NGR0TWIyeE5EcVN3T0RDUzdiYktDMERDZlJ6MTE4S2E0YQ?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46075.26449074074</v>
+        <v>46075.52777777778</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nouvelle stratégie de la Croix-Rouge de Flandre : « En cas de catastrophe majeure, il faudra pouvoir se débrouiller plus longtemps seul - De Standaard</t>
+          <t>Grisaille et pluie pour la 2e semaine des vacances, une belle journée printanière mercredi - 7sur7.be</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>New strategy of the Flanders Red Cross: “In the event of a major disaster, we will need to be able to manage alone for longer - De Standaard</t>
+          <t>Gray and rain for the 2nd week of the holidays, a beautiful spring day Wednesday - 7sur7.be</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 07:50:42 GMT</t>
+          <t>Sun, 22 Feb 2026 11:52:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPTjhOa3haWkhPQ1ZxbTVXWUJ5N2dwVXRlTy1aXzhmcllfbnBCREM3bE43eHNRRFZnYlE1UkxBMUJnVzFhbjVHaXNoZmlERnFydWpySmM2MVJKX3Bnd2R1ZTNpSFBhbjRNSFA2TFRZNWZxYzRnYzNpM1lnZzhBRVExUTJHTW81bVQ5bk1mNFVxY2FYY0RsTEZRV3FjZDNxeGhqekU1X1hLUnZhcXZKaGlOeHpRZ2lJOG5uaFRuXy1yWVZlY2Z4aU9aei1LNTJmbU5EV2R1bjhQWEJ1dlNtRXN2b0puNF8xTVRtYkRtWHQza0J1Ykx4N3JoQ1N2TWNPWHg3TEhEcFB6SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPY1NLZFc2MW8ySDZMNlo1LW1GQ0FRSG1jSjhrSHBrNmxtSmpELW15bkR0V0FfRnRzcVhTbXpqOWVieXlDNl9fVFEtUzFWWTRiVWJNcWRUMjZXcF9ZdXU2R19uendIajY5YkNOMG5ENzBZdlVKQnJ4OXpuSVBheHJPcGNkcVp3ZzByNUJoaWRVUUFlaHBqVnYwTXhSZGdfWG9nYmNvdzA0emVLa04wWmMyQUdlN21zODNyZlgyQUlGRUREZ084Z0ZxVg?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46074.326875</v>
+        <v>46075.49444444444</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dans son tracteur, il voulait faire peur à la police: le dépannage sera à sa charge - 7sur7.be</t>
+          <t>Agression sexuelle, contrats abusifs: une plainte secoue la finale de Miss Belgique 2026 - BruxellesToday</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>In his tractor, he wanted to scare the police: the repairs will be his responsibility - 7sur7.be</t>
+          <t>Sexual assault, abusive contracts: a complaint shakes up the Miss Belgium 2026 final - BruxellesToday</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 10:09:00 GMT</t>
+          <t>Sun, 22 Feb 2026 09:30:24 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQm5lT0FqYUZSUmQ3XzRORG04anAycUpGYmVTd1hiTXRCaGF1Sm51ZlRqQ2RqUU93Umhub0NtVmVXVzUzSDF1bHQtNDFpLV9VaGFJSXIzaU9ULVRDSUhIWDF2aWhRZTRET25mcFhNVElUN0NpdjBJRlp4Um1hQm5MWmN6T192RkxHelEwUHdPa0xDTVVaYXEyNmNXRjBxdlVVZzIyaEVLZVFacU1OZ090aFFmVWVQYlJPUHNrT1p3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNWDlJSDhHeGdmcjAwVGxLZU5LbXNtT2R2U3Y2cElYTm9GdUNmczVodkt5N2FDZXNBbFF5YkJCSjFFdXY3NzNEOTh4ZzY3US0yeThIaXMwOFVOeG9XeUxTYTFjVEh0VnEtODc5dTBkOUF2cXJ0cVlFMXZ5X0lYZTNNVWd3THd0ZEE?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46074.42291666667</v>
+        <v>46075.39611111111</v>
       </c>
     </row>
     <row r="17">
@@ -1315,22 +1315,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Alerte enlèvement en France pour trois enfants, dont un bébé prématuré - 7sur7.be</t>
+          <t>La justice alerte contre le phishing via de fausses applications: “Impossible de distinguer le vrai du faux” - 7sur7.be</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Kidnapping alert in France for three children, including a premature baby - 7sur7.be</t>
+          <t>Justice warns against phishing via fake applications: “Impossible to distinguish real from fake” - 7sur7.be</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 12:04:00 GMT</t>
+          <t>Sun, 22 Feb 2026 06:20:52 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOR3Q1ZnFQeUpnRlV0aHJwekVmejNYaFplR2xYTnRMcEdzYk9RU3RTak5uRklmYzB1Uk1RSnZfZGNSV3I0OFA5OU5tOE9FU1o4TU81bUZsejdkOE45UTM1bWdFaXVmajZMMDluSW5rTy1QRmprMUdsRmRkQ3dxNml3RjhESWFsbjhwM2VNNUp0RzVuTUo1aXJMQjRzSUJTUk5zLXRaSDItSWZNUnJ1YUxMNkRRaw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQOHpEb0RWNVpvS08zNmdON0xCMzUwN3VHZ21lcnFtS2syVEd6ZVAyNVJSdmduUy1vRVhpOUwtaV8xSksxVHA2UkNmRm4zQk5oMkpUVUplQzB4QU92SWRFTFNrQjZ6M0g3di1FeW1ZM1dXbmEweV9ISTRzZUR2ZUg5NVNabHdNajZRdE43bElzZVBodU5NUzl5OTZsMGJvam1fdTBVczE4RHc5UE9sd2NkdDFSNEdmNnF0X0ZLMUtzbllsZzhzbDhXVXB2UkF2S0RkN0FPcm1SaW9pNW93Z2c?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,38 +1354,38 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46074.50277777778</v>
+        <v>46075.26449074074</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Devant New York, Londres et Berlin : cette ville belge est une référence du street art mondial - RTL Info</t>
+          <t>Vakantiehuis voor mensen met beperking in Maasmechelen verliest half miljoen aan subsidies: toekomst onder druk - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ahead of New York, London and Berlin: this Belgian city is a reference in global street art - RTL Info</t>
+          <t>Holiday home for people with disabilities in Maasmechelen loses half a million in subsidies: future under pressure - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 18:30:00 GMT</t>
+          <t>Sun, 22 Feb 2026 10:53:39 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQeHFWdUhraEVFWEpncWVmUUR5b3ViTU9kN29PYzNJeXV5TjB0U0Vyc0t1UDRpUlhJejhULTN5eWJWcnNQd2drbnJZVFJFdDg1YlVZdVd5Z3EzXzQwVVdfaHBsZkRXd3FfTXpxU193bHBjM2wtdjNDSnRmMmNnYnpCYUFYR09KcHdtcEY4T210Z2R0OXh0Ym1ZVGlzdWsybXVZanFxX0MySjZaOFhBeDdQckJ2M0xlTkFybVA1VnRJUHJMeU9MMmdIMGxoNzU2Q0dmdjZEZkc1V0cydlFtakE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPSGxqbkRqNVpYNWk4RFVLN0hzNmZWY0hXMmN4RnRPeW4yZzd2LXlMeEhOWTB4TnhOSTJPSUR6VFVFVkJjeV9VUUZ4MEd5SGY3OHJBVGt5Q1lSdzAwTkh2clBVV2lhYWUyNFlrYTRkVDBhRTRPdEVpU2ZKVFZWSDhndHV6YlpRN056LVVlVjgweFhUVFJfTGdMYldJQmhROUlxRVZsci1lbGczR3BtRUo4R0FsNElrWk5RM0dYb0pUaFJzWXNhOEUxaGJyQ2dCUW9FcjlfUWhNb1VBdzc3ekJscFZDSlk0S0U?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1405,17 +1405,17 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46074.77083333334</v>
+        <v>46075.45392361111</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cultural Compass: Illumination at Atomium, exploration of nature and historical opera - belganewsagency.eu</t>
+          <t>“Misschien hadden we die uppercut van vorige week wel nodig?”: Sporting Hasselt weet weer wat winnen is - HBVL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Cultural Compass: Illumination at Atomium, exploration of nature and historical opera - belganewsagency.eu</t>
+          <t>“Maybe we needed that uppercut from last week?”: Sporting Hasselt knows what winning is again - HBVL</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 07:00:00 GMT</t>
+          <t>Sun, 22 Feb 2026 10:54:56 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOY3U5LTUtNXZGTG5qbHJmby1mR1dpOXJGVTF0aUI1NHBkYVZ6Skg1ZWRxWDZhRU00ek1aMzlvbTZwazAtcU5LZDNDM2I1NUl3MnlLUVRIUjdoVXZTYjZqWDNGRG5aQVVTNDFiZ0h6UDRHY2tSLVFGdkQ4Rzh4dVQ5T2h3UWNta0k3MHNqNnFBbi1SaHd6ZmVEVnk0YWN2Tm1URTBYeEp4X2taRW85Z1VMZUN0aEg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOY3o5T3d5emNMWXFhbW5Gdko0djNqZlhTSkZEVE1RQkp4U3hYN2xiQk1BU1FwWTZVelFrTjQ4Sm5tanBvZDcwanJUWDJrSjZrMk9mUWJwang0bC03bS15RVFQMEJBa0hJcGdIOFM0UEtVZWpZc1RqRVdxZlNBVklaVlJ5alRWWlNGSkpuTGRCZnlySTJ2bnBOZUZ4UGNCN1p2TWFYU21JelZBSHU4NHF1VS0wQkotNm12R25mTmpiLXRSeTZETWJzcWEwWWEwTHVPUzN2Y2NuN2xzTFNsakpkQ2FB?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,27 +1450,27 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46075.29166666666</v>
+        <v>46075.45481481482</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1480,22 +1480,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+          <t>KVK Tienen gaat in slotminuten van eerste helft onderuit tegen leider Sporting Hasselt: “Leuke ervaring om voor zoveel supporters te spelen” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+          <t>KVK Tienen loses to leader Sporting Hasselt in the final minutes of the first half: “Nice experience to play in front of so many supporters” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 11:03:22 GMT</t>
+          <t>Sun, 22 Feb 2026 13:09:58 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8waEpNdEZmMmtDMFhIVzRBZ0QteWtGc0JMUjRFT2hzUXNGa25Pa2FPNzRHSWtUZVVvcGNORnNvYjFVZ2dIeVBMNEs4dTBvdVhmYUt0UWx6T0RQR2daak9ZR2p2SFpZU3lRS2dNaXJ0M0pSMGM3bmcyeEJvT1Y?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAJBVV95cUxNZS1oMU9NNV9iOUVyeG41eHo2dzV1cUdMekJLWmJLVmJyMVR6aW95U0VkTUw2bVRfalUwcEZMRkpZU0NjNEJQd2RXQjVvc19HdlI4bzRleGd4eUIxQTRoWVNmWjJXQmh6MDBPdDJwYWNiMmkxTzhfVXk1bDA0RmFEYU9PVl9adDZuamhJWDF2YmFCUE1KSU5IQzl5VnJhcnZUQkJvMXZKSS1UTVp0MEROYkVpNklwdlYtLXFocy1aTG9FRUQ4MHpSNnV5MXdfc3A3LWlOSEZwcFR6ODRiaVVFblpHMWdXLWhQRFJ2cjduRGFZSHZVZnBZWktLVFUyMlRaNmNfVVB1V0tKNmd4R0wyRDBIbGtvQlM4TVg2bWVmWTY?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46074.4606712963</v>
+        <v>46075.54858796296</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Hasselt verhoogt ambitie sociale woningbouw - TV Limburg</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Hasselt increases ambition for social housing - TV Limburg</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 03:22:34 GMT</t>
+          <t>Sat, 21 Feb 2026 17:21:48 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxONWFSbE8zTHl0VVBBdnlMU1oydWVHMGU0cXY0cWtqRXdqeld4dXMxa0tMWDhmbC1pZV9aMUYxZlJOQ2R6RTZlb1FPVWdiQndWQUVyQ1BiWGQweTN4bUtxR1BWOUtzb3hZa1l4MFp2Y0M2Z1ZWVF8xUkhJR2Z6ME5MSEln?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46075.1406712963</v>
+        <v>46074.72347222222</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Beifahrerin lebensgefährlich verletzt: Stundenlanger Stau auf A9 nach Unfall mit Lastwagen - Augsburger Allgemeine</t>
+          <t>De Lijn moet 35,5 miljoen euro besparen: deze buslijnen in Hasselt zijn bedreigd - HLN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Passenger critically injured: hours-long traffic jam on the A9 after an accident with a truck - Augsburger Allgemeine</t>
+          <t>De Lijn must save 35.5 million euros: these bus lines in Hasselt are threatened - HLN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 07:47:00 GMT</t>
+          <t>Sun, 22 Feb 2026 07:33:32 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPVS12bm52YW9SWW0wYy1fTmt5WTN1YnZ0bFpJSFFaQlhNM0xIaHVpTTE3cFR5UjdsOGJTdXd6d3UwWVNWanQ3aVlBclZYM0pxaWxaVUthY3VUOThQeFN5QWpiZlhCUFh0ZERvRmtZX2dXYXI0NXotTDRNUDY0Z25yeGpZOWZlLTZ5MVJhaXBhUjVOaTNBWDVuU2VRQlNhc0dZM2JiRzRFamhtOFNTMWRHRDA2UDl6LVNTZE1aMmVrSGFmNEZOM004?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNSkgyWE83bXY1azFfX2NlZHFYaGNqT1JlNGotYmE0M3hTRHVzY3RFa3BPdEhXOWVnMGpWenBtTEJSSWNqUms4bTdsMHV3bDkxRDZNZEF2Z1V1MFFEVnFsYXYtazN1aWNRVjNOZGs0bG1PRjJVWEVDTjl1SWpnYUhhbWF1MkZEU0dJY1l0Zzd5bzRxbGk4bEhPdXhJYm5mam5CUXExOFFKck9DVEZoamtnMjR6NHpaM1k?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46074.32430555556</v>
+        <v>46075.3149537037</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>High Level City Spain Spanish</t>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Madrid" OR "Barcelona") AND ("amenaza de bomba" OR "paquete sospechoso" OR "paquete explosivo" OR "ataque con cuchillo" OR "tiroteo" OR "atentado" OR "operación policial" OR "evacuación" OR "artefacto explosivo") AND -fútbol AND -fichaje AND -Liga AND -transferencia</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Nuevo tiroteo en Barcelona: la víctima llevaba una bolsa con droga en plena calle - Crónica Global</t>
+          <t>Tafelschuimster teistert horecazaken in Eisden: “Serveer haar geen drank” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>New shooting in Barcelona: the victim was carrying a bag of drugs in the street - Global Chronicle</t>
+          <t>Table skimmer plagues catering establishments in Eisden: “Don't serve her drinks” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sat, 21 Feb 2026 13:14:29 GMT</t>
+          <t>Sun, 22 Feb 2026 13:56:34 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOVFJtSHl6bnVaM1g5V1lIdDNjTkR0TlZYUlNMejh4R3BpV3MtTThKRXh1RVhZWlV4aDMxdV9qbTRUc2dIa0E0OWhINnFMUk1lS1d5MW44MUxVLV9hQzc2cm9lb19Sa0RHTXBYZEstci1PR3I5aDJDZ1pZR2o2T01vQk12YjBjMExjazVNWnY5Tk5rWl9jb2pzdTJJVXJibmFIalRuS3UzY2NjSGRmblFYWGJvZFIxNEFCNDU0VWlfWdIBxAFBVV95cUxPMTN6OUUyR2c1YWREWDgzczZMMDdnd3g5dzVwRFhYWHdKazhuMU56dzBteENTQVMxVm9OU09MenRSWkE4ZVJCb0UxWEMtalVNUy0ySGVQWHZaQUF6dHBPbDVJZE1JNjhQYllBTmszRTgyNzg4OWZZdTRCZzJJVHFza28wOHE2bzJzSHlQc3R6YW1uR2RDNXpfMGlmdDBOVFZWazdlQkRvMGRlbzV2eFlhelVHLXZjbE00SUkwd21BMUZRcFJt?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxOLXR4Zm9rU1RXTFhMTFItYzc0Q1Z0RlBfNjFaMVUtNnhqTEI0T2ZCX2FlZ2dsa1RBNUdCTm53anl4QkVWWGNIOF81bl9BOWZiMV9RSnBZRVNtTzU3WmRDdkNXSjhmMk1xdUNxaVluTlNKdG9jdnY2Y1djUTN2bVEwTUNocTlmOHJFNXRrMUZKUzlyRVBqSTc2T0htMnBBcEY2ck01N2VnSThmNmxseHdiUnFlemQxa0RkMEZWNWgzR1RpcEwxZThLQkZNSGdCQWhrR3AyYQ?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,21 +1670,1066 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>ES:es</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46074.55172453704</v>
+        <v>46075.58094907407</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Niet alleen biathlon op de Winterspelen, ook in Hasselt wordt gestreden om het BK - TV Limburg</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Not only biathlon at the Winter Games, the BK - TV Limburg is also being competed in Hasselt</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sat, 21 Feb 2026 17:30:42 GMT</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxON29teHZNZ1hxY1QyX3NYSG1TZ3JOY1pYUzVsLWtwSTJmUkFqOVF1blg3T2NNLWdtdXVPY2lZbGJhZWJtcElZOXNXcUhMSjhrRC1yMFhlQW5aV3JxbG5iZDNJai1HeTBraDNRT3M4LWJaVUp1em9ibkJ5WnlVUDJBY0JXbzl6X2ZjMmkxaDFIWjRzNHVZa0Jzd1p5Z01CaC1UVUV2NFhZRDJKUE04VkZnUHVmWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>46074.72965277778</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Honderden bezoekers wanen zich op de Olympische Winterspelen tijdens het BK virtueel biatlon: “Toch moeilijker dan op tv” - HLN</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Hundreds of visitors imagine themselves at the Winter Olympics during the BK virtual biathlon: “Still more difficult than on TV” - HLN</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 13:45:43 GMT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxQTEpNOUxzazNpeFFOMF9ETVhxZGZQcFZacVFmX2xySU5HZThCVlFSLVdQMzhKRU5aMTMyelc5ajJyeFhHNlFhV2NpY3JQaC1oUGh6VGxxT3BQdlktS2VPRk52dFNzWmN4N2NSRjI4SURyTEJ6cW9Na3YwV3V1RF9wNlVFS0sxWjhQQUZFYUMzRG9GYlJ4dlpPVVJkc01FbndCVmFvdVcyZHZHNnJLUHNwVXprclR6aUFvQS16TWhac3R6aEJXN2JMT2g3cjhMUzE5QWVucnl2dGY2Uzg4YWZFOGVQV1RpNXF5Z3dv?oc=5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>46075.57341435185</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Loksbergen in spannend duel voorbij Juve Hasselt B - Nieuwsblad</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Loksbergen in exciting match over Juve Hasselt B - Nieuwsblad</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 03:26:01 GMT</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQNDJZeXhHbk9WMzhoYXZuVXhIOW9VWlpCdUhmR0xaZ0hGcGlneWN6UWZWTmVSdm9Bc2xHdkhjbTVNajc2bHk1bk5nX2d2SGN6ck5ORjd3bEpXUWRXeGI5M3RESmRvMm90eGhyRHI1bk1BYXVBUFp2N1pTMzlIVDBPX19SNHlvczFFR1pKOXpIU0xwbW9FYXRGYjIzN2pIcV9JaVNiQWdaT0twMTNkMG16Wg?oc=5</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>46075.14306712963</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Torpedo Hasselt B en E. Houthalen delen de punten - HBVL</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Torpedo Hasselt B and E. Houthalen share the points - HBVL</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sat, 21 Feb 2026 23:32:41 GMT</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxONDhpVVh2SUdFRnR1RHUzd0dXWlJSMFoxX3Z1UVRPSFhiNV82M3ZoYTJyMnF0aGY5bVlDUXcxTGswNlZVWnFmZUUtSS1lVnRWMlJEOTd2RXdNeFlyZTd3N2VBcDVxdWIwMEZidzdUbmM5RjljX0JON05MaTBHRElyRjhvYVZneTlaRUVWNzRfWWRvTlZ6Yjd3b2ktV1oySVd1YnJqZDg5dE11Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>46074.98103009259</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cash en juwelen gestolen bij inbraak in Stevoort - HBVL</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Cash and jewelry stolen during burglary in Stevoort - HBVL</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 11:09:32 GMT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOZUVNeG1OdjFmeERwdnZVSk14cjJ5SEFUazh0cDY4TEpnNnd2V1ZKQy1ZdEwtV0V5ME8tSW9uV0xYaEt3WG9EQk9JVWVyQ3JZa0dXeGpkZ0puemZkRDBfdzNQZDJxTmdoUTM5UmM2Ul9UekNINXphTzlRa2pQTURHM3dtUFZhSEpPUF8wXzJfWXpIZHBIeW83aVVkdFY2WlByekVlRnY0VUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>46075.4649537037</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Sporting Hasselt wint de wedstrijd tegen KVK Tienen en beslist in de eerste helft - Nieuwsblad</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Sporting Hasselt wins the match against KVK Tienen and decides in the first half - Nieuwsblad</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sat, 21 Feb 2026 23:23:01 GMT</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQaFNlS2hMaUVLWkQxR1FQcVV1ZE5Bay1kT2J5ODRDazRZNkZ2a0JSZWQ0SUx6TzlQQ0VycFdvN015SVZNZi1HSXFmclk5c0ZfRWMzd2E5dUdQbHl3MHZJSzhveVZPcU0zVmxaaFRneXFfZDJma3BEWThtYjNrSnQzNmQxVUVObzBFZlZkb3lHTHpvSlltSHM2QTh4MF9BeVB2TThBXzBJNkpKQUhJR1R2TmdLRF9WTUdydjZ4TzRrMVJaRXFObE9rTXRlckh3OF9wYkcxUnRURnluQkti?oc=5</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>46074.97431712963</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Ongeslagen reeks van Lanaken VV B tot een einde gebracht na 2-0 tegen KMR Biesen B - HBVL</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Undefeated series of Lanaken VV B ended after 2-0 against KMR Biesen B - HBVL</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sat, 21 Feb 2026 22:35:45 GMT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxNR3RsNTM5cnR0ZFZXdHdTYnM4dXpTTTRZejRpMWdvUjgwSXUxblNmOFVwdTBIdEZFREYtQnpRMHNLSThiVjV0OTNpYkdZNy1tcXFpWU5qVkFRY3pxNlBWWGxiWVpCOWNrbjVZOFl0RHlFRkRwV2RCNW54OHFQeHRpb0pwSERuQkZmQTViOGpUVUp2ZmpHa1VjaUU3SkFOQTBELVMyX3FNU2tIV3ZBMUNadjVOUGhsdDVfeENYVm0tSk9oa2tHdTQtWjdnUF9qcHNFdVo5SGViR0VwbThiWURN?oc=5</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>46074.94149305556</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Swinnen redt punt voor Juve Hasselt tegen Nieuwerkerken - HBVL</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Swinnen saves a point for Juve Hasselt against Nieuwerkerken - HBVL</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sat, 21 Feb 2026 21:50:44 GMT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPcGdBZ3ZRTko2WHRaaFlOUUM4VE5KeG84amJuQUcxblBrcVVCelhZODd6TWtNU1NoQUFOdURNOHFjV0d5ZjUzdHU4NkwzaHZNSE9CbkdjTkU5SUtSaWgtekphSXN1NUotb0tETXJMYlRlLTA1N0RxUVpnVVdZV1JCb2tGM2MtMDhmZ294LUstXzhEVV9oT0xuckVBQTc0YlY2ZHJ0cUlwNHBsX3hVd2N6aEpB?oc=5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>46074.91023148148</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch (fallback)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>De Spor herleeft: Is Erik Van Looy de geheime redder? - VoetbalNieuws.be</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>De Spor revives: Is Erik Van Looy the secret savior? - VoetbalNieuws.be</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 10:45:00 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOaGhEQlBKWGZsbElpQkZBZl95czJqVXVacmFxWFhpSFVHOXBYRGdnYnY0RkdIUTdoN0dTY04yUHJtdlB0amcteGdoSTFmOWljX3NoVkozTW53ZkYwZFRyMkJ2NGQ4S0lDSGlWM2tDQzdOY21jOWRnY1BEaHptZUZQSGpLdGdWeW9KSzM1WmFWX2NKSUNKMUFkcG11VQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46075.44791666666</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Devant New York, Londres et Berlin : cette ville belge est une référence du street art mondial - RTL Info</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Ahead of New York, London and Berlin: this Belgian city is a reference in global street art - RTL Info</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sat, 21 Feb 2026 18:30:00 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQeHFWdUhraEVFWEpncWVmUUR5b3ViTU9kN29PYzNJeXV5TjB0U0Vyc0t1UDRpUlhJejhULTN5eWJWcnNQd2drbnJZVFJFdDg1YlVZdVd5Z3EzXzQwVVdfaHBsZkRXd3FfTXpxU193bHBjM2wtdjNDSnRmMmNnYnpCYUFYR09KcHdtcEY4T210Z2R0OXh0Ym1ZVGlzdWsybXVZanFxX0MySjZaOFhBeDdQckJ2M0xlTkFybVA1VnRJUHJMeU9MMmdIMGxoNzU2Q0dmdjZEZkc1V0cydlFtakE?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46074.77083333334</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Cultural Compass: Illumination at Atomium, exploration of nature and historical opera - belganewsagency.eu</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Cultural Compass: Illumination at Atomium, exploration of nature and historical opera - belganewsagency.eu</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 07:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOY3U5LTUtNXZGTG5qbHJmby1mR1dpOXJGVTF0aUI1NHBkYVZ6Skg1ZWRxWDZhRU00ek1aMzlvbTZwazAtcU5LZDNDM2I1NUl3MnlLUVRIUjdoVXZTYjZqWDNGRG5aQVVTNDFiZ0h6UDRHY2tSLVFGdkQ4Rzh4dVQ5T2h3UWNta0k3MHNqNnFBbi1SaHd6ZmVEVnk0YWN2Tm1URTBYeEp4X2taRW85Z1VMZUN0aEg?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46075.29166666666</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 09:11:18 GMT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8waEpNdEZmMmtDMFhIVzRBZ0QteWtGc0JMUjRFT2hzUXNGa25Pa2FPNzRHSWtUZVVvcGNORnNvYjFVZ2dIeVBMNEs4dTBvdVhmYUt0UWx6T0RQR2daak9ZR2p2SFpZU3lRS2dNaXJ0M0pSMGM3bmcyeEJvT1Y?oc=5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>46075.38284722222</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Sparkx Antwerp or Pairi Daiza Edenya: Which Belgian Mega Attraction Is Really Worth Your Time and Money in 2026? - Travel And Tour World</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Sparkx Antwerp or Pairi Daiza Edenya: Which Belgian Mega Attraction Is Really Worth Your Time and Money in 2026? - Travel And Tour World</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 08:55:43 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxOTURZdURLM2hrTHotVTREVkg3RVdJRTFwdlpRWE9faEpydkxPLUVqTktyN2hsR3J2a2hxNUdkTFJZRlRRbk1EOUNEVFppbVFhX1pIYkhSY01kUWpwZUlucGE5OHloNjF6blRoQ3RRN0EzYncwMXVnNGJCdHpOYk5zN0xhRU9XUDhlNldjeTFwckt3Qm1JZkVCV056c0ZRd0xiNW1sU1dScVRXaTFwSGpoWS03bm9fU0RwN1lManNDSlkwUl8yOEVnZ1lVNUFCb2xqS2daUnlDMjdaTzQxeUxnalhqRHB3UDRyOEJlcnhqV0k?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46075.37202546297</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Lkr: Aschaffenburg: Nach Sturz: Radfahrer als mutmaßlicher Fahrraddieb entlarvt - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>District: Aschaffenburg: After a fall: cyclist exposed as suspected bicycle thief - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 12:24:00 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNb05tZ05NYVlVdmx5SmVWdXc3eERabUhHVEdyZjNFZ0V1S3BqMU5qNFBZN21rdmk0RTRiUHVOaUYzUWU0YV92NDJGZ2VJU0ZFVFNNNkVWSXFNRWJZNl8wNGJWVVlBdVI0ZlJTeEZzeWgtVXE1WTVYVmU3TmhwMzVhcVJFSjRIY202dThjYjNrWm5HRzIzZG1PQk5SdFFVUl9Zd1BFaWlLNmtBLTVRWTNCMA?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46075.51666666667</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Gestürzter Fahrradfahrer in Bessenbach als Dieb entlarvt | Foto: Bernd Setnik (dpa) - main-echo.de</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Fallen cyclist in Bessenbach exposed as a thief | Photo: Bernd Setnik (dpa) - main-echo.de</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 09:20:03 GMT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOaTZKZlVndVE3SGxUYlJRRnV4S2pSSm85SERZNEc3RWx6c2R2MW90YVZaVlVxcFU4S2tqeFcyRVBPVXFvQlhxSzJXZXBWd1J2c0VmSzdBbHdJRE5zcm42Z2VrRnBLWEI2bjA4MUpPZmE3QUQzRW14RXN0QUM4Q012eEtyQVJGZTZ6bDVIY0NVSUZzRTZNU29XWmRBeG9hYzVfY0tDMGEtencwYlZRMVZlaXpqTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>46075.38892361111</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>A3 bei Frankfurt gleicht nach Unfall Trümmerfeld – Mehrere Schwerverletzte - Frankfurter Rundschau</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>A3 near Frankfurt resembles a field of rubble after accident - several seriously injured - Frankfurter Rundschau</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 09:35:00 GMT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQRTlnZEV6ckd5ZE91N2JkT09DbEtvaXFJSG42c0lHOFk0blpOTXVDdXFwT2JRWHJjYjd2dFR2OFRxWmpac09FSGpHcHItM2xRdGlQQTFmWW9iRWpwcXBYbDFNaW1Td3lRVlJOVDZMSXdQSDVpb0dGSkdaRnNNQnFSU0lEemtoei1HeUNOQ0RZV2tZSlZwTFMyX3Nnc2Y5TWlqbWlvdnpvTC1LZmpFMTZBVjZVcXRLdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>46075.39930555555</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mobile Blitzer in Wertheim aktuell am Sonntag: Fuß vom Gas! Blitzer am 22.02.2026 - News.de</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Mobile speed cameras in Wertheim currently on Sunday: Take your foot off the gas! Speed ​​cameras on February 22, 2026 - News.de</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 09:28:15 GMT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingJBVV95cUxQS3NPNWtUalRJSHBfajA4X1FTQURMaUlRY08xMVUtX0FHY3FBbkc1ZktaMGlSRVZDMUdWMm5tanFCdjUtdC1UUjNHM1M4WVBYUU9vRFd3VXQ4TDhKSTliQzdtblpFZ2hOdWVCMVZsanVyT0ZKeE9ZTEswbHh3ODNWUlZYLXBjdUo0SVd6VjVYbWU5V190c0dBdG9NalJOMnhiVXBLYzJMSUFnNzdtSlNKMU9Db1htaFhBMl9PVHp2MW55OGczVFBHaUFTYk9uTndxWnIwYTVod25PcU9kUjRYRjRBVG5MNkw4THNFeF9YcGpRb2R2UWZHTW41aEVjZXFCUXVHaE4zLXRlZmRkMzhNWHR1dkNLN1dQWDhOREF30gGjAkFVX3lxTFBZM01kM0F6R3pYcVplVWhxaVNQM0xGYUM0bFdDQVJCaU44MzZzRlNwSlNEUnU5eTJUZFdJT3I1M0EyenVVR2xfSVRMd2JRaWZTZUFRdFE0TXY5NUNMMjUwYzNiNERwQnRRYjFlZXhsSGVPUWdBZ0I5em9aMG84VkxjN0tmaFNSVXRaQlQySEN1ejZDT2VMUDRFR2dTMHYxTzVRcGI2VTBuVkw3d3F6SWtQRGZqcnhGdTVoSTVJTlNWYUtCaHEzbmdaUnVfMlFOUTJNRlNNTjlPTmxDSE9HemhOZDM5aUFuWl9CX004MmRzQVpubm9Ub0Fhb0dkYUp4OTl2eFhsZkxPbnNYblQydFo0WEpQSTdaeWFyQXdad0tMbnFYdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>46075.39461805556</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Demo-Termine heute, 22.02.2026: Hier gibt's am Sonntag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Demo dates today, February 22nd, 2026: Here on Sunday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 03:10:00 GMT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxPbjg1bHBjNUY3b3BoMEZlQ2FyeU44dE53WVVQYXFKdk5iMDJGYnhyOGdGZ3oxeHFHMUJDTUxEWXRIczl6SVcxTlZ6WHctR2FRMThndTdLUnQydFotNW04WHV6TFBJN2FiMlRkWVBFdjFGcnYtcEFvb080WWk5eXJOSGNDam5aMTZGd3dBRXB3NGdjaTEzajZwTmNBZDJvd2lBTlUyeUtIXzd5ZURhdlJ3a2ZrOW1xNEl6eUhJTnc2eG9nU3ZrU3BfTWEwNWdDUTZqalRoNFNBY0dkOHppWWxrU1IwbHBROS1jNDV3T2ppaFgzZVBGaE8xam5EdXhxUXVrcklySNIBigJBVV95cUxPOFFPVE5JQmROaVRiTGNpQ0NQOXM0VGdNOC1PeE93Z2FnVDM3VDIxZFNnT1lvNWtIajhLQ2Zsam1JRUhUTkZQOVpabTFHM3ZYbThnR2Vic1F0TjBRZ3h2SmQxZTBRVlVEQTFwX0tQSTJ0THNkZzhSdFdmQkNpdFhtam1YLTZneVNmMnA3TXlYYkNpR0ttZklsOUpkUW9JY0VnWGVJNWk3dlY3cThubVZFZG4zOFFjVHhBZ0N3aDFCeHJVaTByQVZBQTd6NkwtUGl4MlB6RWI3TC1nQjZFOGt2b2tvUzU5WTZ5d1pWY2VqVnJ3Qmc1MWwtNk9PcjFIc09wSUF2R0xLTUhRZw?oc=5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>46075.13194444445</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>What is going on with the new FSU College of Business? - FSView &amp; Florida Flambeau</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>What is going on with the new FSU College of Business? - FSView &amp; Florida Flambeau</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Sun, 22 Feb 2026 14:01:00 GMT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOdGhlNk5VS041eFZaNXlCZElIOTNxVHpsbEVuLTVETEN5SzROZXVpc2NEX0tjdW9UQlBUR3RUY2JYWjBZWUsyOWgxaUFwWWJoWlBOYm53Tl9OakN5czlGanZLbEMzX3VWTkt6ZW1OdEdPb1ZMUEF5V0k3QTJsLUtPT090eElobUFBWnR4MVR3SjRWd1BMOUpIQU1nY180dTFPOWVBUTJ2MW5RRm8xaWV6Y3JqRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>46075.58402777778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-23 14:47 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Brand Protest</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nike Fortnite Shoes: Can You Get Them? - thedetroitbureau.com</t>
+          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Nike Fortnite Shoes: Can You Get Them? - thedetroitbureau.com</t>
+          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 00:04:32 GMT</t>
+          <t>Mon, 23 Feb 2026 08:35:59 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPSHg0Q0FVRTVtVWJtSlZUdnhOSTlyQzRPMUVPOG9wQU0wTXdIUXQ5VEV1UjNTODBWSGM1UzdKSHlLMk9udTAzZFhRUGFsVG9CSDV0Q3NBRGJ1N01Hcl9tbmVIRElQN0s1dW9DQVotVmNWTzc1M1RhMElia2ZmWE1kbmp3cmRBT3pDb0JIRUJueUVYQldpNUR0QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQOGNjVDdzNXFXVEZHMEFmaGdnaVZTN1UzZ0txV1BGYzc1dm5CLTg2dmEtSEdYSVBlN3drRUVGSmJrNmg4QWxkdUd3by0wN0ZIRVNJd3c2cDJqenFCTnNyWTJyZnlEUVZ4MWFaU3p5LUJXNzNRWEhBVEVjUTQ1U2o2aGJn?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46076.00314814815</v>
+        <v>46076.35832175926</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Brand Protest</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Moncler Down Jackets in 2026: Hype, Heat &amp; the Real Trade?Offs - AD HOC NEWS</t>
+          <t>Hof van beroep buigt zich over wrakingsverzoeken in zaak-Costa: “Mijn cliënt gelooft niet meer in een eerlijk proces” - HBVL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Moncler Down Jackets in 2026: Hype, Heat &amp; the Real Trade?Offs - AD HOC NEWS</t>
+          <t>Court of Appeal considers requests for recusal in Costa case: “My client no longer believes in a fair trial” - HBVL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 22:55:12 GMT</t>
+          <t>Mon, 23 Feb 2026 11:23:00 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOR3BaaVNqQ21ON2hBTnU3UThFRTdVT1B2V0ZwZHl1ZDFiWUJJRkRkOEg4ZHdVWVJKbWswdURiQklXaEt5cXQ3WW9PNjFMakVfbnpZV255b1ZjZ1BOaXM4WTNCOFR1VkEyNXMyWE1wdmVQYmt1UVBQSnFCLUV6QWdJSXRRTU1mczYwSm85Tk5UMFQ4LXg1OUM5YW5ZUmFrTi1QRHVwOHRsV21WX01TVFEyN05lNjZvV2R4UjJOX1dR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxQNlh2cU1lN1puZmpfZl9TblJvbVRMOWtxMU5QNzZ2aDloSXNOZHFQUHN0ZW81SzJlcnZxaXJSSzFoUWNNY2pJbThxVk5lRm8yMWRWcHhTTEtick1DLXN1WVBLZmdISXJJSWJ3WDBNNVJSRHVWOHJuZUF4dUZMLS1YaV9rdVB5cFBHRGpac1duQm0wQURWenlGN3F1Yl9yRW5yOUVmdWhrejhSSENKa2lfdURpRW9PaVp3VlFEb2hjbk9veUN5X1VtWFRWSDRTTmZFYm95YlJrSTRIWHNmQ1lvak8xQ2w0MjdCY2NheUVqMUZ3azY0Y0c4TW1rRGNqbUtaX1hJSUU1aU1WWE9IZVE?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46075.955</v>
+        <v>46076.47430555556</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tax refunds are about to give everyday Americans a boost. BofA says buy these 8 stocks to ride the wave of spending. - AOL.com</t>
+          <t>Ruben Van Gucht in shock: 'Bekentenis slaat in als een bom' - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tax refunds are about to give everyday Americans a boost. BofA says buy these 8 stocks to ride the wave of spending. - AOL.com</t>
+          <t>Ruben Van Gucht in shock: 'Confession hits like a bomb' - VoetbalNieuws.be</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 05:39:14 GMT</t>
+          <t>Sun, 22 Feb 2026 19:43:00 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxONDN6d0JBUncyN09RWE1HN05JQmxXVmdWTDJGUTJmUzhlRkVfT0hrWXcxWG9mdUdJWWlDRGZZQ3dhVm92NXJSYm9aeTJ0T2pJUzFJdEFHQVlScUUwX3Y4NUdaYUZtc2JSMnhhdkk5NnJZNVFqSXNEUnExUnE5cHZ5bTlkV1BvbEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQNTBkNjR2dWVMcWRqcEp5MmM0eHZSenlEOWVsejhsOXM2aDZsdHhKMlI5Vm16NHJreWM0MlA3WmQ3LW5WUTNxMVg0bS04dFFtYUdpbHNfT256QWhHM1kzVDQzS0ZtVjdQLTZlWjJvaTR3WjNDQWRzNEhyNzgxV3c5U0FpaUYxXy10alJUOFNCYk5GTWlTTlVVZkw5VFluM1lBVkE?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46076.2355787037</v>
+        <v>46075.82152777778</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>Explosief ontploft onder auto van volkszanger Frans Theunisz terwijl hij in Lanaken op het podium staat - Nieuwsblad</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Chiltern Railways to be disrupted by work on Tube - AOL.com</t>
+          <t>Explosive exploded under the car of folk singer Frans Theunisz while he was on stage in Lanaken - Nieuwsblad</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 08:35:59 GMT</t>
+          <t>Sun, 22 Feb 2026 23:10:54 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQOGNjVDdzNXFXVEZHMEFmaGdnaVZTN1UzZ0txV1BGYzc1dm5CLTg2dmEtSEdYSVBlN3drRUVGSmJrNmg4QWxkdUd3by0wN0ZIRVNJd3c2cDJqenFCTnNyWTJyZnlEUVZ4MWFaU3p5LUJXNzNRWEhBVEVjUTQ1U2o2aGJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxPS1Fvczk4VGdrakpKT1VxdVNfZGNJZXc2LWt1dHF4S184U0MxNXdYME5xOVNzbG9oT05wWkVKQnhnZDJVUy1BT08xbWVfZ2NoWVc0TVpieDBtTEt2eF9BNjQzNG0tZDVKVnV5ZDRpRFh4b0t0TUlfUVMwckZoYkp3Nk84SzVVVnJDWjgxY0hLWGdFd1FEZ0NjYXQxNllySlhuekVQbW5qRHdMVGs3bTdRVzZpdHNqM2hKN2hRQmY1al9EUnNCTlBhVEkyVjU0LVhuYXJiVnBZaFFDTmhzM3FDcUxKckdxZ1d1T3VPQzJFUHg4Nk1LeFItNW5R?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46076.35832175926</v>
+        <v>46075.96590277777</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Europese dag van het slachtoffer: Linda getuigt na steekpartij in Veerle-Laakdal: "Ik sta sterker in het leven nu" - rtv.be</t>
+          <t>Israel faces an internal time bomb - www.israelhayom.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>European Day of the Victim: Linda testifies after stabbing in Veerle-Laakdal: "I am stronger in life now" - rtv.be</t>
+          <t>Israel faces an internal time bomb - www.israelhayom.com</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 14:02:35 GMT</t>
+          <t>Mon, 23 Feb 2026 10:42:43 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxNLUxWTXZSNktaZVNZaFVhMlN0djhHazE0QVR0a0l0QTlLZUQ3a1ZUY1RyUFE3Wlc5aTZhN0ZXWmVFX3lXMWFqcUtESW1Pc3dOYVJVZTRsNnZXRVp1Z3ZmcUVpODJfWDVoc2YtODJjbVdRWEg5ZENRbHhnQkNZMURwNU1ZX2MxSVZDb2ZOYWZaTWlCUGI1RllSRkJ5ejJWZllBT3I2cU5UMWF1SUtJYWtyZkVVMW1sWnhH?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9UT1ZXandBRVdxaS1sbDVUNnVsVkhieWpMenNQLXlWZWxULWx0dUtUWHVDQUJpaWFzQUF0OFJBMHpRVXczTWxMVV9LWUhuSmUycFk0OVVqSWhQSVgzckVWcHBfQzhkcnYteC1VdGpiczd6cUMtZEFGeG93Zmc?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -745,42 +745,42 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46075.58512731481</v>
+        <v>46076.44633101852</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BBC tipt dit museum in Brussel bij ‘zes meest veelbelovende openingen ter wereld’: “Een absolute mijlpaal” - HLN</t>
+          <t>Air Force One fleet to be repainted in Trump colours - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BBC recommends this museum in Brussels among 'six most promising openings in the world': “An absolute milestone” - HLN</t>
+          <t>Air Force One fleet to be repainted in Trump colours - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 16:45:55 GMT</t>
+          <t>Mon, 23 Feb 2026 10:16:17 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNbWtyZ29waXdQa2VEaV9MZWZyTlJtclVEc3g1bk1oNGZsTjdoLVpXcGZwRFgxbnN4aXJvSl9BUi0ya0xETFhiRm9nRXUzRE5jclcwVG8zcHpveXFla3JQaFUyLU1EMFV4eWRmYWpRSF9ENVhkcDA4NlQzUXk4MzRiZVN4aGk4QXBzSXI3WWVfVnRIRjk5M3hiVkgwUlg4c204R1NoWDNHRG9vYTRFYXhzbnBpQVdFUktBYmFwX0RxVDVWOS1MbE9iaXZZWWhORS1wV2RLTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOeEwwd2VzTFZKaTJyblhmQXJONW9sNjVubTVtTmpEZjN1SW1XWXB4Qk9sMHNBZEhmdzh5OXZ3VUVhVUpGTWZsMTM1cTFuZ2VFQ0FjajlpejZwb3VrTllqY2NKWV85R3dmV0pBcUNrcFpDYmlzakpQTnotZmM5QXlBbHJaS2xGUEU?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -800,42 +800,42 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46075.69855324074</v>
+        <v>46076.42797453704</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Ruben Van Gucht in shock: 'Bekentenis slaat in als een bom' - VoetbalNieuws.be</t>
+          <t>Germany’s ruling CDU wants to stop Gaza payments via UNRWA - Brussels Signal</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ruben Van Gucht in shock: 'Confession hits like a bomb' - VoetbalNieuws.be</t>
+          <t>Germany’s ruling CDU wants to stop Gaza payments via UNRWA - Brussels Signal</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 19:43:00 GMT</t>
+          <t>Mon, 23 Feb 2026 13:37:46 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQNTBkNjR2dWVMcWRqcEp5MmM0eHZSenlEOWVsejhsOXM2aDZsdHhKMlI5Vm16NHJreWM0MlA3WmQ3LW5WUTNxMVg0bS04dFFtYUdpbHNfT256QWhHM1kzVDQzS0ZtVjdQLTZlWjJvaTR3WjNDQWRzNEhyNzgxV3c5U0FpaUYxXy10alJUOFNCYk5GTWlTTlVVZkw5VFluM1lBVkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxONTJpaS1CY1VFdHlVY0NtVzhNdTJmMG4wOHdydnY5MlM3bHVTZ2RRcVlzZ0dmX3JxdVEzNHFmM1VjWXZQOVlHVzdKU1I4TUMzeDJfZTAyNTJOVDgwcElQXzJfZzI0UFVZWGs3ZFdxMmlmNlF0N0pGa0pSY1hLWEw3WXFoVGx1WXFIaFZIeHM5VnVIVDNsMlFF?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -855,42 +855,42 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46075.82152777778</v>
+        <v>46076.56789351852</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Explosief ontploft onder auto van volkszanger Frans Theunisz terwijl hij in Lanaken op het podium staat - Nieuwsblad</t>
+          <t>"A deal is a deal": EU demands US to honour its trade commitments amid tariff uncertainty - lokmattimes.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Explosive exploded under the car of folk singer Frans Theunisz while he was on stage in Lanaken - Nieuwsblad</t>
+          <t>"A deal is a deal": EU demands US to honour its trade commitments amid tariff uncertainty - lokmattimes.com</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 23:10:54 GMT</t>
+          <t>Mon, 23 Feb 2026 04:53:47 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxPS1Fvczk4VGdrakpKT1VxdVNfZGNJZXc2LWt1dHF4S184U0MxNXdYME5xOVNzbG9oT05wWkVKQnhnZDJVUy1BT08xbWVfZ2NoWVc0TVpieDBtTEt2eF9BNjQzNG0tZDVKVnV5ZDRpRFh4b0t0TUlfUVMwckZoYkp3Nk84SzVVVnJDWjgxY0hLWGdFd1FEZ0NjYXQxNllySlhuekVQbW5qRHdMVGs3bTdRVzZpdHNqM2hKN2hRQmY1al9EUnNCTlBhVEkyVjU0LVhuYXJiVnBZaFFDTmhzM3FDcUxKckdxZ1d1T3VPQzJFUHg4Nk1LeFItNW5R?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQSEt2eExmVkxGQ2hINXRmaTdwYXJ5NnhmdVNOM2ZSdGlHb1dxaVdyMGpaYnBWWTVmVVd0WXh5SnVkaVdfdU5RMkh3TGVxVlFSS253MkNLZjM0NXZzQWlSeGQtQWN1ZW1SaUdfd0w3eEtqT1RwWThzb2tfWUNFdEV0NmYzUTRIQ3JuN1JENmZUSWgyMy1JZDNsYzlQQ3FXTXJvRnR1VmJ1VHRHVVd4dldqaDRZY2V5OTdtRzRobWhpdFhkYzdVWTVF0gHOAUFVX3lxTE9KUnZzY2U3d3A4eHBpY3ZXV0RiWkhEWFl0M2VkUUExNW1DOTM3WE94RjZtMUxod0U0UFdKRmZ1RUVLTzJhUEV1NFNkX1ZMTFhtTkVvaWlyWVJNenlLdjQ5ZkVpYXhaWmF4V0ZFRzV1X0Nnbks0NmZsVFNpOTJWVlJiSTZnVEIyT2Q4ZncwSngzNE5INTZGQkJha0I0R3ZvMzk1WDE3YS1nUy1jYm42UjBYbkt3amRvdEVHTmN4bFVYV3NWbGtkOXA4ZmpwV3RB?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46075.96590277777</v>
+        <v>46076.2040162037</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hoe deden de voetbalclubs uit Tervuren het afgelopen weekend in hun reeks? - HLN</t>
+          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>How did the football clubs from Tervuren do in their series last weekend? - HLN</t>
+          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 18:40:18 GMT</t>
+          <t>Sun, 22 Feb 2026 20:08:33 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxONS1jbXYyX0dkQ3JGVWViM29ndnp0dmZualdpMFBqbTR2NnpwdlJ6czlCbWdiTkV5emxzcEZHcjlRblFsM1lOX0lnX1pKa3NxNlFlMDBEV2J1VHhYSFljYTF0djZQZFdua0VPb2pHWjNfUEtYSTMtNm9PX1RfVnl3aVdGV0ExM2RxUVB2U29ybFN2blJRckZKRXVhdlZaZmZqdnNVVjZHNkJGcFQtLTRiRHdnYmduS1Iz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNZlBCeEZXakZ5VVBhQWpxMEpCVzFtTm9CYlZ2emxsaXhUci1GUXRybGp0T2ZKRDJNYmFXYjFNZDRSS3NTLXBrRnVfS3RLRndzcFNTUU9rVGFmM3ZnV3hFbGNUN0JMVHRjSnpqWkVSWDFrS2pQa1JjeFZzN3luS2pqS1U3REhERHQ3dV9WUGVZeWl6Q014Sk5EenVfaGY?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46075.77798611111</v>
+        <v>46075.83927083333</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Berlaen viert jubileum als singer-songwriter met dubbel concert in Knipperlicht: “Mijn tweede thuis” - Nieuwsblad</t>
+          <t>Explosion and Fire Reported on Container Ship MSC Giada III in Gulf of Finland - 112.ua</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Berlaen celebrates his anniversary as a singer-songwriter with a double concert in Knipperlicht: “My second home” - Nieuwsblad</t>
+          <t>Explosion and Fire Reported on Container Ship MSC Giada III in Gulf of Finland - 112.ua</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 10:22:36 GMT</t>
+          <t>Sun, 22 Feb 2026 20:17:56 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAJBVV95cUxOQ2ZNRUx5elg4NGlsbTI4UUdMM0tZZVgtYXpvXzhuUEtkLWN0dHJjeTdjTjVNUDU3bGJfSHNkdkFMMF9FSTBCdEpYVWtuRUpYajBjWHQ1TncxekloMFU4QzA3cV9vUEZlai1qRTNWbHJUcVA4WFFMVi12UG5GWmtBVndlQmcyY3FjaFV2SUVvamhqYkttYjQxSnVkUHJ4ZzUxNG9xclVXVVkwczNIcmJ6NTRnVTJYZTVjM3kzeXlFc2pJaFA3RTltS2pnNk1OWU5sYXhFWjZiYjF0WVBsWTBqVnBQa0tQU0VVcnM2VXpjelFkZjRreExBb2lDS0pQcW1QU1BzZ1FDYzI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOR1plTldVMXlJQTNVdkJ5YWlRNmJZU1VRZXlVb1Vpc2pad0plMEZxWkZXenRVcVVzRnk3OXlBb0JPUFhYUmx4Q2Z3LV9DbG00VmFsNnRKR1RNdjhZUER5a0FiYmdjNk5zdEFydWdZR29mbkl2bzByUHI0X3dDWUZoUUs2bW5wQ3ZReVpFVHJuRlRDODNHSzAxYTBn?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46075.43236111111</v>
+        <v>46075.84578703704</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>"A deal is a deal": EU demands US to honour its trade commitments amid tariff uncertainty - lokmattimes.com</t>
+          <t>Un homme de 79 ans tire des coups de feu sur une maison avant de se donner la mort à La Panne - 7sur7.be</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>"A deal is a deal": EU demands US to honour its trade commitments amid tariff uncertainty - lokmattimes.com</t>
+          <t>A 79-year-old man fires shots at a house before killing himself in La Panne - 7sur7.be</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 04:53:47 GMT</t>
+          <t>Mon, 23 Feb 2026 06:29:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQSEt2eExmVkxGQ2hINXRmaTdwYXJ5NnhmdVNOM2ZSdGlHb1dxaVdyMGpaYnBWWTVmVVd0WXh5SnVkaVdfdU5RMkh3TGVxVlFSS253MkNLZjM0NXZzQWlSeGQtQWN1ZW1SaUdfd0w3eEtqT1RwWThzb2tfWUNFdEV0NmYzUTRIQ3JuN1JENmZUSWgyMy1JZDNsYzlQQ3FXTXJvRnR1VmJ1VHRHVVd4dldqaDRZY2V5OTdtRzRobWhpdFhkYzdVWTVF0gHOAUFVX3lxTE9KUnZzY2U3d3A4eHBpY3ZXV0RiWkhEWFl0M2VkUUExNW1DOTM3WE94RjZtMUxod0U0UFdKRmZ1RUVLTzJhUEV1NFNkX1ZMTFhtTkVvaWlyWVJNenlLdjQ5ZkVpYXhaWmF4V0ZFRzV1X0Nnbks0NmZsVFNpOTJWVlJiSTZnVEIyT2Q4ZncwSngzNE5INTZGQkJha0I0R3ZvMzk1WDE3YS1nUy1jYm42UjBYbkt3amRvdEVHTmN4bFVYV3NWbGtkOXA4ZmpwV3RB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQaE1ZcmdIVzVhMVE3bkJxRXdkci1DN25Sa3VQczFQQjN2R2NvQU51S3JuaURxOGtHZ2RTREV5Wm1zT2JWWi1NWm1ydk91eUluWk5GWHpOeDNHZl9SVVJEVG9FVlNwak9mVFM1TVk2anc1WFdnY0RpeWYxZTlCTUhGejJiZ2pPd2lGd3NDaWx5QmZ6Vkh2VHFiTnRqWXhBNmdzN0k5RF9vR05DUHVWVFhYSXM4SWdPanlKa0VHLWdfNUNzSHk5S3ZzS2VUMjNaTnJWc1R3?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46076.2040162037</v>
+        <v>46076.27013888889</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
+          <t>Marc Uyttendaele ne donnera plus cours à l’ULB après un “geste inapproprié” envers une stagiaire - 7sur7.be</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ukrainian oil pipeline "Odesa-Brody" may replace Russian "Druzhba" - Online.UA</t>
+          <t>Marc Uyttendaele will no longer teach at ULB after an “inappropriate gesture” towards a trainee - 7sur7.be</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:08:33 GMT</t>
+          <t>Mon, 23 Feb 2026 10:32:00 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNZlBCeEZXakZ5VVBhQWpxMEpCVzFtTm9CYlZ2emxsaXhUci1GUXRybGp0T2ZKRDJNYmFXYjFNZDRSS3NTLXBrRnVfS3RLRndzcFNTUU9rVGFmM3ZnV3hFbGNUN0JMVHRjSnpqWkVSWDFrS2pQa1JjeFZzN3luS2pqS1U3REhERHQ3dV9WUGVZeWl6Q014Sk5EenVfaGY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQZzFuWjJVUFozaFJYUWEydER4aXlOX1ZILTZnNDFoY1VXaGY5UExQQktYcDlBa3hjZVNaZHJFYVRTWFJxeTM3dnJqTWlocGhIOHlBUlBzOW14emRnRlZ0a2JldXZQckVBcVgyajRIY0xEVGQ3cy1uQkhaQ3pNNlhublRzNUJwaXd1Z3BHN1ZseXhYbjNtTWFYbFFXdU5rR09OZTBLd0JxLWU0UGhuWFM4ZVpRcExHanNNQ2FQQ1ZYNkNJQkFEcVhiUmRaUkg2Z00?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46075.83927083333</v>
+        <v>46076.43888888889</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Explosion and Fire Reported on Container Ship MSC Giada III in Gulf of Finland - 112.ua</t>
+          <t>Tajani à Bruxelles pour le Conseil des affaires étrangères : Rassurez les entreprises concernant les droits de douane ; les guerres commerciales sont inutiles. - Agenzia Nova</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Explosion and Fire Reported on Container Ship MSC Giada III in Gulf of Finland - 112.ua</t>
+          <t>Tajani in Brussels for the Foreign Affairs Council: Reassure businesses about customs duties; trade wars are unnecessary. - Agenzia Nova</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:17:56 GMT</t>
+          <t>Mon, 23 Feb 2026 06:20:13 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOR1plTldVMXlJQTNVdkJ5YWlRNmJZU1VRZXlVb1Vpc2pad0plMEZxWkZXenRVcVVzRnk3OXlBb0JPUFhYUmx4Q2Z3LV9DbG00VmFsNnRKR1RNdjhZUER5a0FiYmdjNk5zdEFydWdZR29mbkl2bzByUHI0X3dDWUZoUUs2bW5wQ3ZReVpFVHJuRlRDODNHSzAxYTBn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAJBVV95cUxPdWVlY25DdEpZUGhvdF9ZZ0JPeGFzVl9sdEFfT2FaT1N6ZzFWWDJwNkh6bEtONXYxM2FlNHBKdTF1UXFEc09LVDI3V3RoLW9qdTdDWWpUMWItdzVOLXpyNkN2WUdUOE5QWjk3cnEwMlhKWmFZNTdjU0Y4M1FKUzZlODFmbkF6T1hTU3RnaWN4cHQxenI1RDNVRVBVcWJLcWs4YkJ3NmUxcHljbEJ3cVpOelpxVEE4S3F3dFQySE1CRU9xZnN5cHhRRVFhTTNrTUd2dVc0ejNzdUM5blUxVjBfa1dlYkJXTWplWVFKVWxXRUpQNWNicE1IZ3VPTUl5S1BJRmMzQ2QtNEZ3MWhBZDlPeW1KTUpMLVQ1b3JDLUphR1gxWFBi?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,11 +1185,11 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46075.84578703704</v>
+        <v>46076.26403935185</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Glatigny veut rendre l’apprentissage du néerlandais obligatoire dès la troisième primaire - 7sur7.be</t>
+          <t>Accusée de harcèlement, Elisabeth Degryse réagit: “Ces cris et jets de signataires ne figurent pas dans la plainte” - 7sur7.be</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Glatigny wants to make learning Dutch compulsory from third primary school - 7sur7.be</t>
+          <t>Accused of harassment, Elisabeth Degryse reacts: “These cries and throws of signatories do not appear in the complaint” - 7sur7.be</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 08:03:00 GMT</t>
+          <t>Mon, 23 Feb 2026 14:09:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOdW02WmNMX095RWFQc1dONmswazJhTEx1M1BWMUxVdnlRWVZpSURYYURndjFSSlN0OHdSVXZrSWZlM1NiQWliZjdvWUd3MkZVczVMc1lhMmxCdmh2OGF0R1E0R21TbjlZZklxVC1fVEhGX2VoRW1GVU9lMGFLMmwzREdzNElBZ1gzeVFqeVRTNk9adi1WSDhST3hLdmI1bUlDVlpFSzNZMFNyUFJ5SGxkRW9IRUpNTDItc2k4ZTVkS0JTbEptazhv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxNdE1zQmdaVE4xOWlKZE9memxWRldLYjZwaG9acmZPME8zOXk2ZE1xZXBlX1loaV9oeTJmdnJuWVVYcnZIaXhUNklkaml4YkNaakVqaW5UZWZ3WEt0blVmZVdqQ3lfVlNKTEdCMUU3TGppdl9jMHh0MXUyOGFETHk1YTdQN2pOd0JVeFBRbnZwQjlib0dBUFBRQkUwQnZFQVA0YzZYbGxibW1XWVJNNTBBWkpzVU1JRzYwN1oyMW1RTGZteHJ4eE9va09taHduMm1vbW1Sal84cUJQMjk0Y1Q1OVB0Rk1YZw?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46076.33541666667</v>
+        <v>46076.58958333333</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dix habitants sauvés lors d’un incendie dans un immeuble à Schaerbeek - 7sur7.be</t>
+          <t>Il a couru aux JO avant de combattre la bombe nucléaire : pourquoi l’histoire de Philip Noel-Baker dérange encore - Daily Geek Show</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ten residents saved during a fire in a building in Schaerbeek - 7sur7.be</t>
+          <t>He ran in the Olympics before fighting the nuclear bomb: why the story of Philip Noel-Baker is still disturbing - Daily Geek Show</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 22:01:00 GMT</t>
+          <t>Sun, 22 Feb 2026 20:31:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPdFlVQXdlMzVjOHE1SUxVZTR4am85NklKQzUyb2N6cXJNX2lvSUpjM0tIcDdXWVIyQTBDbUJIcHRMRE9jYzB1VkJSZkdoVnZUNEFVaUlfU3hqUklpOWpfX1cwSWJRcG10WHpXSVhRYXM1TFJJNEk3aGN5RTM4Y1FDYTlMcjFPMno1X3g1Vm5pbGZod3BuVjlHbU02WVVpOF80OWhkLTJ2YmY3SkJnenhoSXhB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE12aG1TZFZ1ZE43SkdRT1lfbTByMk1sS1NQQVAteEVGMWI0YmNpcWFtT0pwX1BXa3MtVm9UQ3dLbDhWaXZteXVVNTdGXzI?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,38 +1299,38 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46075.91736111111</v>
+        <v>46075.85486111111</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Un bébé de 16 mois retrouvé sans vie à Berchem, le parquet ouvre une enquête - BruxellesToday</t>
+          <t>220 oproepen in één weekend voor Politiezone - De Internetgazet</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>A 16-month-old baby found lifeless in Berchem, the prosecution opens an investigation - BruxellesToday</t>
+          <t>220 calls in one weekend for Police Zone - De Internetgazet</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 12:40:00 GMT</t>
+          <t>Mon, 23 Feb 2026 09:41:10 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE0yMzAzNE9wYTFoTGJBLXdOWHpfRWJ5MUoxUGQxWHlMc09jQWZQY0l4Vm9FWlV0d2dRX2c2bWZTazRZRmg5cnZndmJzdmFXSi03eGhja0Y1NGR0TWIyeE5EcVN3T0RDUzdiYktDMERDZlJ6MTE4S2E0YQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNYTBpdElMU1JKTjk3LXFvdXg0aG1LWVd4S1RZaEtXS3FfdzdCU0ZSQnE2NWJjX3JwU3VVNnlPRU9SN1VqTUtqYm9ON0FGVUY4STdEaFdWUno1WGxfTzRNc21wX3JkdUZ4c2p5LWZBVjhWcnRpXzVLekJaLXhyQnItY0NhcVo?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46075.52777777778</v>
+        <v>46076.40358796297</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Un homme de 79 ans tire des coups de feu sur une maison avant de se donner la mort à La Panne - 7sur7.be</t>
+          <t>Challenger Pro League : Renversant au Patro Maasmechelen, Beveren acte (déjà) sa montée en Jupiler Pro League - DHnet</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A 79-year-old man fires shots at a house before killing himself in La Panne - 7sur7.be</t>
+          <t>Challenger Pro League: Stunning at Patro Maasmechelen, Beveren (already) marks its rise in Jupiler Pro League - DHnet</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 06:29:00 GMT</t>
+          <t>Sun, 22 Feb 2026 17:31:00 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQaE1ZcmdIVzVhMVE3bkJxRXdkci1DN25Sa3VQczFQQjN2R2NvQU51S3JuaURxOGtHZ2RTREV5Wm1zT2JWWi1NWm1ydk91eUluWk5GWHpOeDNHZl9SVVJEVG9FVlNwak9mVFM1TVk2anc1WFdnY0RpeWYxZTlCTUhGejJiZ2pPd2lGd3NDaWx5QmZ6Vkh2VHFiTnRqWXhBNmdzN0k5RF9vR05DUHVWVFhYSXM4SWdPanlKa0VHLWdfNUNzSHk5S3ZzS2VUMjNaTnJWc1R3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAJBVV95cUxOMlhPQzRIdU1oWjk2ZXgtQmpiQmowckwwY256b2pINDRDb01YVlhZakJyYmJiWFpFdEVxZ0FxY1pESDNRbGNLQ3VKSzJwXzVDNU8wZDhBYXFTaGZSTHpzdEU2T2QwNTUxdWYxcS01WUw0M3BSYXNUaWFucXZhUFVvSlBYYkFaeUM2Y1FDVkhsYWdBTzhoSVFkYV9LNjlCWFQ3U0JXaGVQWEd4VjgwdjVvbndxTmo4OTlwTUdMQkdwbXdIb0RzZWpTVUxtV2xPMFRObWI1d1RuNmVrMFJTZXhUeGZNMTNKYXdMSF9lTGRHaEFoLTJieC11eVBGWDN5SUZFVlZ0Z29IeFgtSEVUWjU4YkpJZWxNYjdVZUNGRw?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,38 +1409,38 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46076.27013888889</v>
+        <v>46075.72986111111</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Il a couru aux JO avant de combattre la bombe nucléaire : pourquoi l’histoire de Philip Noel-Baker dérange encore - Daily Geek Show</t>
+          <t>Beveren a fêté sa montée sur la pelouse de Patro : la réaction de Stijn Stijnen a surpris tout le monde - Walfoot.be</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>He ran in the Olympics before fighting the nuclear bomb: why the story of Philip Noel-Baker is still disturbing - Daily Geek Show</t>
+          <t>Beveren celebrated his rise on the Patro pitch: Stijn Stijnen's reaction surprised everyone - Walfoot.be</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:31:00 GMT</t>
+          <t>Mon, 23 Feb 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE12aG1TZFZ1ZE43SkdRT1lfbTByMk1sS1NQQVAteEVGMWI0YmNpcWFtT0pwX1BXa3MtVm9UQ3dLbDhWaXZteXVVNTdGXzI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOMFZUdHIwV2NXVUVCZ2JjRVJ0d2Q2Q2ZOWUw1OFB5ZV9GNkt6eVNSS1h6RjhDbGtrNFg3eUhOU2NROWlxMkZ2ZVVxbTBaQ1dPTXZLYmMwcFVRaHNLOEdPVmZFYkptVWJxWDZiTGRlZjVPaHJTWGJ2UnhLaklhcW1TenlRd0FTUGZRZEtCdUoxUkFHNHpZamVYMGFSNFVyaDI2RUItaE5KeVN1dEZfQTRJNkdZUXp1TS1lRFNDUXVDZjhVZmRiTWsyVnlreUoyekVSUG5wWHVheVbSAd4BQVVfeXFMT2R1OWxYLVlQVHkxTkJOOFVTdVV4ZHA2Q2RiQXRpblVQdGV2Nlh2Q2xBMnBqSWxCaW43Y2ZKcTdIbWRDdEY2ZHVlN2NhRFNsaThCX0hpMDhsaXQ2U2lIZ1lWUGNvRTNndkJvWUUteXg1WWFIdnRXbGFhVC02aVc1RmtLdHU2dVd3RDliSHpndEg0ZzJyQXhacEl3LU05Mk5WWjZZUUdKRDVuS3IzN3NzdFQwX3VnbmctMV9QQWxtOElPT2Y1bFJXSFdKVTdvb3BibXFXQ25lLThqVW1CX0p3?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,38 +1464,38 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46075.85486111111</v>
+        <v>46076.5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>“Une erreur administrative”: des millions d’euros de pensions complémentaires “oubliés” - 7sur7.be</t>
+          <t>Toujours invaincu, coach de 33 ans : le premier promu en JPL vit une saison impressionnante - Walfoot.be</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>“An administrative error”: millions of euros in “forgotten” supplementary pensions - 7sur7.be</t>
+          <t>Still undefeated, 33-year-old coach: the first to be promoted to JPL is having an impressive season - Walfoot.be</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 05:17:00 GMT</t>
+          <t>Sun, 22 Feb 2026 21:26:00 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPSmZoYnBwQ2FJa0x6UTY5VERiRHJqeW91ZmxncHpQMVRmaDFLLU1JbTM3UDhKdlRTMHhvLXlBbVcwdXluQnRPcnZnQllxR2c4ME1venZ0VUxuN0szcjYyVjNQTzByZVBRYTA3M1pGeVFweV9YQ1dReTdvcFZzNUR4QlRuVGdudjBHTk5tcmUtbUhpQUJmTS1IVEVBcVJaWU9EWklBNkxKamU1SktIcnV6MVJSZ2ZZUlgtbkU0TDVn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPUm1aUHIzYkdJcldqSDFGdGJnV2dhR2ptNXpyb2Q3cmw2WnhJVEpHNGhycTU3Qng0MFozcThHdUFwbF91WjI2Rl9JT0dLUHpPX1k0VG5Vc0VrZWU2X1ZNZi1JalJ6dHZDSE8wNXJuMm03cUxHNjRBZHpna19tc1FhQnNISHJHbUZjTTNWZDUtVGFOTmtzNUx2NzZ6V2M4WFVQQkF0S0RUNk9DTmNMWGtaXzhQeHFGeXUzRFdwNlJEYXF1ajdocnhr0gHMAUFVX3lxTE5RSHcwUHQ5dWY5Rmk0RkRWSUhBSEdEMnJXTWh2bWIzYTY4N3hmWnZocm42cE9SaUNfb3d6Y3FsNkdPQUpLbUduMXB1WGRRNTFrc0NzVHdZYm5vaTRUOXdWYUhPczVHLTJYZDM1ajRrVWEzcldycExJdWNiWElhSXhmN1A3MnU2SUNTWk1Ta3VrdVA0cUlZSlZibGJGcWV3VHE0Q0tVZWZRTEQtdjllandwNFQwM09feDlabG1aMHBjWEdhNVBjYUlLQ3d2SQ?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1519,38 +1519,38 @@
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46076.22013888889</v>
+        <v>46075.89305555556</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Une enquête ouverte après le décès suspect d’un bébé de 16 mois à Anvers - 7sur7.be</t>
+          <t>Cambriolage au musée du Louvre : Rachida Dati finalement auditionnée à huis clos par l’Assemblée nationale - Ouest-France</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>An investigation opened after the suspicious death of a 16-month-old baby in Antwerp - 7sur7.be</t>
+          <t>Burglary at the Louvre Museum: Rachida Dati finally heard behind closed doors by the National Assembly - Ouest-France</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 13:04:00 GMT</t>
+          <t>Mon, 23 Feb 2026 14:01:49 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWlNZaUs0UnI4bmNvaDFjUDdieDV5RUszU09Ud3NGTV9DT3p0cUtBOUxrd0h3LXBnQzJ6U1YxcE4za3EyUGJBUWtFOFRtaHdrX3JzU0pWVFpLSlhjU3pBTkdfUXVINVhtZUd2LXFXUWpJUjBhTjZKLUkzUS1vdy1jcWJjTkFscEVqUkQydTUwY1JHdFB5ZnhQOUktbXR5bW1rak9Hc0NsQVN3RXVrV3piZmt2MmZKZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNZmw4eWxPU2NZRUF6aHJSSmZFYWx2STRHd1dSZFJSNVQwNXBzcFlSYlpWendqN2NKVmY5YWp4OW9rLV9IVVJhMzFJTG9USmRtTTR2ZnNTOGVzYzd3T3docUI3MTllcW03MVhHZ0NPTDVHN094OG5pLUdrbkNPRXpqajFEWFZDQTFGaFdLbU56akZYSENfem5qUGVDVGdtdmRTSjM2NHdfZ3ppZHNkbDh4N1E2R1h6V0o0bVpWSHF0RXlfbmdfVDI5cFFoUmFVZnFUY1VRTmgtNngyMHFIaVhYYWRNQ0tGQThxQXVBOUdfVGVZSlNwR0lUaklzc2pWa2hTanJRTnhjeGIwYmhNN2ZvZk53QVVua0pHeUxn?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1574,38 +1574,38 @@
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46075.54444444444</v>
+        <v>46076.58459490741</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Grisaille et pluie pour la 2e semaine des vacances, une belle journée printanière mercredi - 7sur7.be</t>
+          <t>Le Beerschot se loupe à la dernière minute : Beveren exulte et valide sa montée en Pro League - Walfoot.be</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Gray and rain for the 2nd week of the holidays, a beautiful spring day Wednesday - 7sur7.be</t>
+          <t>The Beerschot misses out at the last minute: Beveren exults and validates his rise to the Pro League - Walfoot.be</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 11:52:00 GMT</t>
+          <t>Sun, 22 Feb 2026 17:20:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPY1NLZFc2MW8ySDZMNlo1LW1GQ0FRSG1jSjhrSHBrNmxtSmpELW15bkR0V0FfRnRzcVhTbXpqOWVieXlDNl9fVFEtUzFWWTRiVWJNcWRUMjZXcF9ZdXU2R19uendIajY5YkNOMG5ENzBZdlVKQnJ4OXpuSVBheHJPcGNkcVp3ZzByNUJoaWRVUUFlaHBqVnYwTXhSZGdfWG9nYmNvdzA0emVLa04wWmMyQUdlN21zODNyZlgyQUlGRUREZ084Z0ZxVg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOMjM1SmJwVkRCWkx0aWwxVUpnYTA1dTcyMlpWTElWSTlQc1NGcHNaajRPTk9wVGxOMXl4clhJSWx2Z01XUXdPeFpCa3ZpT2c1T0pMam9GdG9jeDZENWlUWUt1cEV0SGozLTZDdmNaTWtaX3VaalRpd19jVHJyQmx6dlZIeDVhV09KSHN3NFllQmtaMElOWGVIcnFPVTd4QnFoUm9Wc09rbWpURXVYWkU4clRTQTJiNWxvVGlKSHJPN0VaSmxIOG5LUFJsVdIB0AFBVV95cUxQQmd0R2haLW1QSEM5WG4wVVZ1UFc4RWpVRFdka0pQQXM0QnVjMmVfQkdUSE5iejVKMmtFRHZ0dEJLWHk1VXJTeWNhVmJ0VTZEZWZoRy03aDJVQ2F3NlFfMnlTSFdZRHFvSW8yQkh4dG5HelFXNndaalZsYmJFS3dvSW9lTE5BMm1Ga3BlQ0VONUtjcno1Q25qaWxQak9oWG55VUpZMjV6U0ItdW9SMjJBcnRIM05tTllLMThMYXBkQmVIT0cyNl9kRXRSM1d5VHlI?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1629,38 +1629,38 @@
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46075.49444444444</v>
+        <v>46075.72222222222</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>220 oproepen in één weekend voor Politiezone - De Internetgazet</t>
+          <t>SA Winger Fires Beveren To Promotion In Belgium - iDiski Times</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>220 calls in one weekend for Police Zone - De Internetgazet</t>
+          <t>SA Winger Fires Beveren To Promotion In Belgium - iDiski Times</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 09:41:10 GMT</t>
+          <t>Mon, 23 Feb 2026 10:35:28 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNYTBpdElMU1JKTjk3LXFvdXg0aG1LWVd4S1RZaEtXS3FfdzdCU0ZSQnE2NWJjX3JwU3VVNnlPRU9SN1VqTUtqYm9ON0FGVUY4STdEaFdWUno1WGxfTzRNc21wX3JkdUZ4c2p5LWZBVjhWcnRpXzVLekJaLXhyQnItY0NhcVo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPS3ktRHpRekdhell6bG9ZVUdNeXhoQ2loT2RYMHl6eWNPNVFqd1p5Yk1wbGtPZGpzeGtkN0J3MGwtWVZhUm92NUFHSTk1bzR5WTlOTDgtbkZKWkpNbmgyUzFPS2ZJQXF4UnhRaGlwRW9jZldLNWdvU0FuOVdLVXMwMkJRaHlaVGdhUGZUY0YzX2V2Qkdrb0s5bHFB?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46076.40358796297</v>
+        <v>46076.4412962963</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Challenger Pro League : Renversant au Patro Maasmechelen, Beveren acte (déjà) sa montée en Jupiler Pro League - DHnet</t>
+          <t>Würzburg: Nach Angriff am Hauptbahnhof – Polizei sucht Zeugen - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Challenger Pro League: Stunning at Patro Maasmechelen, Beveren (already) marks its rise in Jupiler Pro League - DHnet</t>
+          <t>Würzburg: After the attack at the main train station – police are looking for witnesses - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:31:00 GMT</t>
+          <t>Mon, 23 Feb 2026 14:30:00 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAJBVV95cUxOMlhPQzRIdU1oWjk2ZXgtQmpiQmowckwwY256b2pINDRDb01YVlhZakJyYmJiWFpFdEVxZ0FxY1pESDNRbGNLQ3VKSzJwXzVDNU8wZDhBYXFTaGZSTHpzdEU2T2QwNTUxdWYxcS01WUw0M3BSYXNUaWFucXZhUFVvSlBYYkFaeUM2Y1FDVkhsYWdBTzhoSVFkYV9LNjlCWFQ3U0JXaGVQWEd4VjgwdjVvbndxTmo4OTlwTUdMQkdwbXdIb0RzZWpTVUxtV2xPMFRObWI1d1RuNmVrMFJTZXhUeGZNMTNKYXdMSF9lTGRHaEFoLTJieC11eVBGWDN5SUZFVlZ0Z29IeFgtSEVUWjU4YkpJZWxNYjdVZUNGRw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNUk1fcXRlQzR0TUx0eFZ4Rk1TMTBnQ2Z5RjJjeU02bGVXczhsQ0lfblVYOGJWRXRueExfZThlbTM2Smo3T25UQWs1TTNrZVRySUl6cl92NjJ1cktxVzltTTZmZGtJWXJVSWNWSmlDZVpYZFZiS1Q1WVgzRXFZbVBOT3lOUHlIbS1rMTBjQzNFNFhQdXFwLUNTZA?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46075.72986111111</v>
+        <v>46076.60416666666</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Toujours invaincu, coach de 33 ans : le premier promu en JPL vit une saison impressionnante - Walfoot.be</t>
+          <t>Schüsse in Kahl am Main – Polizei nimmt 19-Jährigen fest - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Still undefeated, 33-year-old coach: the first promoted to JPL is having an impressive season - Walfoot.be</t>
+          <t>Shots in Kahl am Main – police arrest 19-year-old - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 21:26:00 GMT</t>
+          <t>Mon, 23 Feb 2026 13:35:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPUm1aUHIzYkdJcldqSDFGdGJnV2dhR2ptNXpyb2Q3cmw2WnhJVEpHNGhycTU3Qng0MFozcThHdUFwbF91WjI2Rl9JT0dLUHpPX1k0VG5Vc0VrZWU2X1ZNZi1JalJ6dHZDSE8wNXJuMm03cUxHNjRBZHpna19tc1FhQnNISHJHbUZjTTNWZDUtVGFOTmtzNUx2NzZ6V2M4WFVQQkF0S0RUNk9DTmNMWGtaXzhQeHFGeXUzRFdwNlJEYXF1ajdocnhr0gHMAUFVX3lxTE5RSHcwUHQ5dWY5Rmk0RkRWSUhBSEdEMnJXTWh2bWIzYTY4N3hmWnZocm42cE9SaUNfb3d6Y3FsNkdPQUpLbUduMXB1WGRRNTFrc0NzVHdZYm5vaTRUOXdWYUhPczVHLTJYZDM1ajRrVWEzcldycExJdWNiWElhSXhmN1A3MnU2SUNTWk1Ta3VrdVA0cUlZSlZibGJGcWV3VHE0Q0tVZWZRTEQtdjllandwNFQwM09feDlabG1aMHBjWEdhNVBjYUlLQ3d2SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQdktzWkJUVTRINDl3TGRPNzVZUmJPYXRkWXlDbFJ1YUNMSWp6OUhNM1lrOGlHT3hiRm5OUXh5YTQzdk9aNDNMMERHTkNWMWQtYTZfdG5GdGRtSE92RE9DZkZ0N205d0FGUkx3N0VnV2haWkJVam5yN2xzTVc0RTl4TDRTUVdoTWNCeW0tbkkxU1VER0ZOZ0NMWFdzeUJ0ZWVOdjNqNXlqTXhFcDQwbnF2UW1WSHN5aUstTXlseWlGdkR3QQ?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46075.89305555556</v>
+        <v>46076.56597222222</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Une histoire d’autogoals permet à Beveren de retrouver officiellement la Pro League - RTBF</t>
+          <t>Demo-Termine heute, 23.02.2026: Hier gibt's am Montag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>A history of autogoals allows Beveren to officially return to the Pro League - RTBF</t>
+          <t>Demo dates today, February 23rd, 2026: Here on Monday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:54:11 GMT</t>
+          <t>Mon, 23 Feb 2026 06:09:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPbFhISjNiUHBBTk85aVdsYkFnS1RiQkxuZVZhNkRsU0hwbldROXVkaFpTckZxb2FhbUp4dXJ3NjBzWUlXY1ctX2xZUXRiUG9GNlVSNFY2R1NCZ2RoZGp6RVN2QmVnY21uUElQbm93X2owcHFUeDNvOGZKUnlVcGh0NzBZMzMyTnpyVm1YclE2VXVhNW1GWjJGUFllcFJSd3FNX1V6d2EyaFNtVmFXQkx3MTRUTnNpMmdKcWU5elluWUZLM1RmQUpz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxNcEw4UEFXTE9LZ3BUZHVRb0JhdDNVaTdaYUszLUdBam1CREwwRFN5NlUzUEdnYVZtN0dINC0xbTRudW5DSFR2QlY2QjhDVm5JMXJaN2F5SE5ubmMwWEZibXBFZ2tGM0c3dFZObV9FVGQ4dDlDam5GeDYzc09qWjJLdDBnMTdjTFJaamdheE1tX0FtaGt5WUkxdFVkZ0RXSWc2T2dlU3U0eXlhR2FhS2cxVU92OXVZcmpoUGs3allvX2h2S2s0ZWd1WW4yVGprekR2WUk1d2JPeEhhWFBnbHF1MG9xckV6dVppVEZKdnZvU05IQVRNdEZ0dGY0TDVoNmhrQ2tB0gGIAkFVX3lxTE1rWXg1LXplU3B4SGpfSG5LLXdwV0pGbEROYW5VUlJxWGRVVW9oZjgwY3djOENybFlTRDJMTUFmcVEtRmgwRGRNLV9vUWZ4M0tuenh1X190STlLX2FET09idW9Bak1JTFRtN2ZCM2NjeU9ZZElLY1A2V1Q4clNHZnhMR0NZVmFQMkpRUW1pckZuWnBNYmxicVpDZVNiMktDWUtVcHF4RGEycm5kOHN6dUJmMVdxdktDVTJLNzVsYm9vY1ZMOWh2YTRLdFcxRGFmZl9WdjNrRGR0c255SzB3R2pZZ1FTZUJlWWNHUWxwaTBmSEdYaTFXaFlRR3pEVDh5ZVJ2Y2cya1k2Sg?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46075.74596064815</v>
+        <v>46076.25625</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hippisme. He And Me drivé par Eric Raffin vainqueur du Prix de Paris - Ouest-France</t>
+          <t>Würzburg Hbf: Mann greift mehrere Personen mit Messer an - New-Facts.eu</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Horse racing. He And Me driven by Eric Raffin winner of the Prix de Paris - Ouest-France</t>
+          <t>Würzburg Hbf: Man attacks several people with a knife - New-Facts.eu</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 15:42:10 GMT</t>
+          <t>Mon, 23 Feb 2026 09:36:08 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQX3ZXcjVDbzRNblZfdE5yeDVDb0xKb1RGSnRhZ0J0Tk11akhzb0pCQzE1bUNEOU9mSTQ3N1Z3Mm5Ud2szV2M4b0hIT1BxR3djeUJyQ1JWak5PaHV1SFpvRVotQ2U0RFJXbDVhRWhJRnZXdzREMXFiM0FoN2gxQlZwbTBKQTZ2ZFBBZUpLNHkwX0xaNzdXdWh5UmE4MWkweVpaSVZzSUlvTEtybmlUb2NERkdhSERNeHJrQ2NZaDhzNE5zN0JNWjlOX0pMNnA1ejVGY19ZeFM3Ym9mZmlZNmR1OA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOM24zMzhrM2czdEk2MmF1TzJoSTdKNzZnZURodkdsRVFMZTIzakE2RDNTYWI3Wll6MzNNNUNsUDdsX09reEVwMF9nTGt6YzFaVkl4TnBfUzBvRzRKVGctdXpUUS1LTkJGMW1id1VFWFNsNm9ZT0FTMHM5LXA5MURHNnB5S1lPalRReDNtMWJOMTc0M1pUR05qN0tTckVhZS1Fa2ZpdElCaVlZMXUxaW93S3NFaEJHVGNuU1E?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46075.65428240741</v>
+        <v>46076.40009259259</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Le Beerschot se loupe à la dernière minute : Beveren exulte et valide sa montée en Pro League - Walfoot.be</t>
+          <t>Audi RS 5: A tonne (actually several) of talent - Motoringnz</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>The Beerschot misses out at the last minute: Beveren exults and validates his rise to the Pro League - Walfoot.be</t>
+          <t>Audi RS 5: A tonne (actually several) of talent - Motoringnz</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:20:00 GMT</t>
+          <t>Sun, 22 Feb 2026 20:59:44 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOMjM1SmJwVkRCWkx0aWwxVUpnYTA1dTcyMlpWTElWSTlQc1NGcHNaajRPTk9wVGxOMXl4clhJSWx2Z01XUXdPeFpCa3ZpT2c1T0pMam9GdG9jeDZENWlUWUt1cEV0SGozLTZDdmNaTWtaX3VaalRpd19jVHJyQmx6dlZIeDVhV09KSHN3NFllQmtaMElOWGVIcnFPVTd4QnFoUm9Wc09rbWpURXVYWkU4clRTQTJiNWxvVGlKSHJPN0VaSmxIOG5LUFJsVdIB0AFBVV95cUxQQmd0R2haLW1QSEM5WG4wVVZ1UFc4RWpVRFdka0pQQXM0QnVjMmVfQkdUSE5iejVKMmtFRHZ0dEJLWHk1VXJTeWNhVmJ0VTZEZWZoRy03aDJVQ2F3NlFfMnlTSFdZRHFvSW8yQkh4dG5HelFXNndaalZsYmJFS3dvSW9lTE5BMm1Ga3BlQ0VONUtjcno1Q25qaWxQak9oWG55VUpZMjV6U0ItdW9SMjJBcnRIM05tTllLMThMYXBkQmVIT0cyNl9kRXRSM1d5VHlI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNS2Z2ZDJ2cE43aWEyaEFvclJ2WG53ZkJzTk9TMHdfa2dGSDBYZWlrUkcxRnRBaUV0NjZVZkExNFRZR3cwUWdURlhMcVRPRkhIdHd0dlpfWi1ib2hnWndCQlZwYl9LMlYwaTg1dTZWQ1h4bFZjSHNDWml2QmxySXhSZ3J1Q3NPamVHRU1tUkk2Zw?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46075.72222222222</v>
+        <v>46075.87481481482</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>« Mon grand-père est fier de moi parce que je reprends le flambeau » : Gwenaëlle, 19 ans, candidate au service militaire - Ouest-France</t>
+          <t>Lamborghini Technology Boss To Head Audi R&amp;D - AutoSpies.com</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>“My grandfather is proud of me because I am taking up the torch”: Gwenaëlle, 19, candidate for military service - Ouest-France</t>
+          <t>Lamborghini Technology Boss To Head Audi R&amp;D - AutoSpies.com</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 11:07:25 GMT</t>
+          <t>Mon, 23 Feb 2026 13:01:28 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwJBVV95cUxPeXl3QTFDbzFpMDFsZGVYUG0xX0M5VW9QRDRMWVBNS1pBUVhCUFFmbUZ4cllPanNKVlpmcVk4b3MyVGdXUUdQRjVrWHpmVnBkTkN6cUtkTVpqQWZoeGRPa0xZNzRZekVrTmRrMUdpdl9OT0kzQW56VDlNVEh1aElkOUhfYTZqQUVCRHFMWVVlV3dSWnE4QUthNFp1VXh5clZ1RFBfYko1ek9EMTRTcE12NVFEQWJYX3NsQlVDQ3dWNjU4TG5mSzFTUkxpSGdMTGpJN1VEUWJYal8tMDlJMDE1WGFjSHlibzZtam45WmR0Rjd6c0ppN2RoWExpSUpWUGV0V2tZR3o3dERBT3Zzcllva1pZOExkVC1EMHlXUjdzenNaZDlyLXE4LUhpMzluUVoxNlhmbXA2Yw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE4zU1R5OU1XNHpNbXhaWHY3N0hFdFRKNTl1UTJnQU5fc1prNUw2VjU1QTlCcUp5d3BFcGNsc2VjaTBOalEtX2N6RHFXZVFUcnNkZGZBWVdmSXRYZFNxRjhSaGtrdjQ4cndUbVljMWVn?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46075.46348379629</v>
+        <v>46076.54268518519</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Las Rozas La Roca (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Messerangriff am Hauptbahnhof in Würzburg – Passanten greifen ein - Fränkische Nachrichten</t>
+          <t>Spain: Las Rozas Black Demons rally past Zaragoza Hurricanes in second-half thriller - American Football International</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Knife attack at the main train station in Würzburg – passers-by intervene - Fränkische Nachrichten</t>
+          <t>Spain: Las Rozas Black Demons rally past Zaragoza Hurricanes in second-half thriller - American Football International</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 09:38:00 GMT</t>
+          <t>Mon, 23 Feb 2026 05:45:33 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOR3d3NlFUUHNzd1FrdVZKTHdSc0xfendNTnJWNVRKeU10a3hjOVJpWmNkektEMkRYMnJJdTZHQ0E2SWJEbW0yS2hzUG5jdUlieGFIMDZkM3dSTTEtTHRDN2dwQ1VIeWRWS2ZfOE1aUnNWRU5aN2o4RjB0SG9mVXdfVnQ1M1YwUnFTT0ZTVVdUR3VLTlhGeERlekJVM3pBLTFkclVYSjRnZ3VaeVJBMFV0OW1Fd21yRU5uNUpBMEdEOXpSc1phME5RbURzd3FQSDVfNmJzMzBYQU0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxPcGUwMFYxdHY2dEZ6TXR6aFk2MlowaVV5bElVem9WRDBobjRld2wzR3dmWHBqZjBIVFdWQXVrWGM2VE4xSERvcnBTc3ltNFVCeEJlSXFMd2pIQ3kxMHIwWXFReU1KSnMtZGx6LUpFSE1iUzlXN1lUNGJfVnZPclVhM0ItN2h1SnVVNU9renpfVmlpTEJvMnhERElrR1JVZkdZeGRYV0ZKcjVuOC0xNGhrbXdsWjQtWHZtNHIxS3dJMm1TS0F1ZDB6TTZ4STl1dzTSAc8BQVVfeXFMT3BlMDBWMXR2NnRGek10emhZNjJaMGlVeWxJVXpvVkQwaG40ZXdsM0d3ZlhwamYwSFRXVkF1a1hjNlROMUhEb3JwU3N5bTRVQnhCZUlxTHdqSEN5MTByMFlxUXlNSkpzLWRsei1KRUhNYlM5VzdZVDRiX1Z2T3JVYTNCLTdodUp1VTVPa3p6X1ZpaUxCbzJ4RERJa0dSVWZHWXhkWFdGSnI1bjgtMTRoa213bFo0LVh2bTRyMUt3STJtU0tBdWQwek02eEk5dXc0?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46076.40138888889</v>
+        <v>46076.23996527777</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Las Rozas La Roca (fallback)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Demo-Termine heute, 23.02.2026: Hier gibt's am Montag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+          <t>Spain’s luxury mansions: where global buyers are investing - Idealista</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Demo dates today, February 23rd, 2026: Here on Monday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+          <t>Spain’s luxury mansions: where global buyers are investing - Idealista</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 06:09:00 GMT</t>
+          <t>Mon, 23 Feb 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxNcEw4UEFXTE9LZ3BUZHVRb0JhdDNVaTdaYUszLUdBam1CREwwRFN5NlUzUEdnYVZtN0dINC0xbTRudW5DSFR2QlY2QjhDVm5JMXJaN2F5SE5ubmMwWEZibXBFZ2tGM0c3dFZObV9FVGQ4dDlDam5GeDYzc09qWjJLdDBnMTdjTFJaamdheE1tX0FtaGt5WUkxdFVkZ0RXSWc2T2dlU3U0eXlhR2FhS2cxVU92OXVZcmpoUGs3allvX2h2S2s0ZWd1WW4yVGprekR2WUk1d2JPeEhhWFBnbHF1MG9xckV6dVppVEZKdnZvU05IQVRNdEZ0dGY0TDVoNmhrQ2tB0gGIAkFVX3lxTE1rWXg1LXplU3B4SGpfSG5LLXdwV0pGbEROYW5VUlJxWGRVVW9oZjgwY3djOENybFlTRDJMTUFmcVEtRmgwRGRNLV9vUWZ4M0tuenh1X190STlLX2FET09idW9Bak1JTFRtN2ZCM2NjeU9ZZElLY1A2V1Q4clNHZnhMR0NZVmFQMkpRUW1pckZuWnBNYmxicVpDZVNiMktDWUtVcHF4RGEycm5kOHN6dUJmMVdxdktDVTJLNzVsYm9vY1ZMOWh2YTRLdFcxRGFmZl9WdjNrRGR0c255SzB3R2pZZ1FTZUJlWWNHUWxwaTBmSEdYaTFXaFlRR3pEVDh5ZVJ2Y2cya1k2Sg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQR3djQzdWMVh1UWY0OWg5YVdaMno3OVpMbHVJUmxSVTRfVVRuZ1FfVHdkVzBoWFlRVV9TVldvS1A5a0xlVHdKT0NBZjhpUGprZ3VZOW9XMFBGWU5vb3VmZm9TRThGZkdPMTV1V29LTlZVZHdadWdiR0FmVUtrcXl4UV9aSVRLaHo4MzI3MWx6OXZfQ21kZjVjN1ljbE9aTHM2Z2ttaDNLX2h1QnEzempOY05MYzJpMHNZU0xzQVVPX1pmMmRUMGhFMHd5elduSUVPTW5DMWVQOUHSAdgBQVVfeXFMUEd3Y0M3VjFYdVFmNDloOWFXWjJ6NzlaTGx1SVJsUlU0X1VUbmdRX1R3ZFcwaFhZUVVfU1ZXb0tQOWtMZVR3Sk9DQWY4aVBqa2d1WTlvVzBQRllOb291ZmZvU0U4RmZHTzE1dVdvS05WVWR3WnVnYkdBZlVLa3F5eFFfWklUS2h6ODMyNzFsejl2X0NtZGY1YzdZY2xPWkxzNmdrbWgzS19odUJxM3pqTmNOTGMyaTBzWVNMc0FVT19aZjJkVDBoRTB3eXpXbklFT01uQzFlUDlB?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46076.25625</v>
+        <v>46076.29166666666</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Würzburg aktuell am Montag: Wo am 23.02.2026 Radarkontrollen stattfinden - News.de</t>
+          <t>Tributes paid to Kildare couple killed in road collision - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Würzburg currently on Monday: Where speed cameras will take place on February 23rd, 2026 - News.de</t>
+          <t>Tributes paid to Kildare couple killed in road collision - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 09:19:10 GMT</t>
+          <t>Mon, 23 Feb 2026 12:14:14 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxNODYyNHJkWS1RODBsQ1p0akJWNFdwaEIxWTJRR1A0YWFWSG9ZRVdzaGl2UmJxUnhGcXltaFpINjRnbmM1V25za2xucGpKSkxNcVVxaG1BLWR2YUpKQ1ZPWVJ2a0twemdnVzNGTWkxWm9HY09vTzlQYzJNNWZ1dllfQzlNOEk1N0thVUkxak4yNTV5OTZuWU5fdzhQZ2UzRjdkSEhSdFh5eDdKYjg0N0pYMkZIRGE2MGJFcU5RdV84cVpONzhOcUt1bndfTElSazFoLXVMek1ZOUNncmZWY2V5dTFpRjlOVHdKeEo0dlRMTkk0d1ZzcklqcDZkOTJaY2_SAYQCQVVfeXFMTmJnRHpQamItajJIS3o0TUY5RnVKbERDMXlCQ25paV9abTBHRUs3S3dYVkFYRU5YRVozd01idnp0N0Izdkw5MUVFRGVLd2plbWF3UG9VWU11M0lDVjhzSmRoaW1TTWdFajViOS1XS2VFS21pNUNVbnFabXpPenlDa2N3ajVVX3hma0Z5dGp5UDFUR19VM2loalg0ZEJ5US1SUTFGWXhfQTNnaHgydjU3aTQ3X1A5a1dDel9vbnByTUlpbjRGaV9hR1dFVHFmazR6czhzSE1MSENSQVZUUEJRcmp6TlloSjI2dF91Y1NpYWdwY0Z1UE42bmc4c1RIQ0pfODRTdDU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQYXB4b3ZvUklCZkNkMjdEaDRwN2FrN0JaaXJNQXpzV2tybENnb1ZjX2kyQUl2NU4yNUlTT1RXcXpTVVRIQktyTlpWUFNmMFFKX2pSR1B1WWUzMDkweGZoUWE4ZHkySlYzVUtRdFExUm1aTjNkcFdZY3IxNkxCV2k4VHc3a2EwUGtVajNBZWstc1ZDaXpkZUh0RG80dlV2eHg5OW8zc3pFRTBjLXFGeS1xdkR3?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46076.38831018518</v>
+        <v>46076.50988425926</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>What is going on with the new FSU College of Business? - FSView &amp; Florida Flambeau</t>
+          <t>Kildare workers being forced to give up right to work remotely - Cllr - Kildare Now</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>What is going on with the new FSU College of Business? - FSView &amp; Florida Flambeau</t>
+          <t>Kildare workers being forced to give up right to work remotely - Cllr - Kildare Now</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 14:01:00 GMT</t>
+          <t>Mon, 23 Feb 2026 12:30:00 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOdGhlNk5VS041eFZaNXlCZElIOTNxVHpsbEVuLTVETEN5SzROZXVpc2NEX0tjdW9UQlBUR3RUY2JYWjBZWUsyOWgxaUFwWWJoWlBOYm53Tl9OakN5czlGanZLbEMzX3VWTkt6ZW1OdEdPb1ZMUEF5V0k3QTJsLUtPT090eElobUFBWnR4MVR3SjRWd1BMOUpIQU1nY180dTFPOWVBUTJ2MW5RRm8xaWV6Y3JqRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQYTFHcVRLbTdXdW45dWlLR3l6ZkpCS0RtZVVDd2M1dGprU1ltY3Y3UXVjemlqLW9PNkw2Mm91eDdsU3liZTYzX3hPSXZYSEpsZG04dTFrREFaY3EtVlU3TG5YVFRfT2JSd2FDSlIybmNKN2ZfZ0NCazdpenZEdXhvS0RIYkExVzVxZWFQNFFHbmc0dHZtUUVVRFJ1SEFnbzZHT2hwOXg3ZnRQTl9FS1lnN29B?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2234,38 +2234,38 @@
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46075.58402777778</v>
+        <v>46076.52083333334</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Audi RS 5: A tonne (actually several) of talent - Motoringnz</t>
+          <t>Search operation underway in Kildare after reports person entered water - Irish Mirror</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Audi RS 5: A tonne (actually several) of talent - Motoringnz</t>
+          <t>Search operation underway in Kildare after reports person entered water - Irish Mirror</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:59:44 GMT</t>
+          <t>Sun, 22 Feb 2026 17:56:34 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNS2Z2ZDJ2cE43aWEyaEFvclJ2WG53ZkJzTk9TMHdfa2dGSDBYZWlrUkcxRnRBaUV0NjZVZkExNFRZR3cwUWdURlhMcVRPRkhIdHd0dlpfWi1ib2hnWndCQlZwYl9LMlYwaTg1dTZWQ1h4bFZjSHNDWml2QmxySXhSZ3J1Q3NPamVHRU1tUkk2Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNR0FNY0lDUjkxYTVDbjNBVFBEclA5cVpETmRzaHhqc2Y5VTMxMXBOeXJpOENFb3FqWFBUeVJpbW9CSUVsS1QtVDlIR0JZbFJRc011aVJJOWFmRUxEbGxob24telZKWFlVZGctcXlsM0Qya2h1MXFRQnVEZThoYy1WTGZqLVN5djZIakZqSU9tSjE3S0RIUGfSAZsBQVVfeXFMUHhNb1lyLS1qMkk5R3RibzdCWUJHNkEwOUdHZGRUOHFVb1VOal83VTNHWl9Pek1hVnRyMWNjVHJUcnEtYldjdFZCc3N1aDdNVTk2UjQyQVVFWGNLSUFaOERaQXJxSktHaW9XR0kzLVlQY1FOb25INm04eDlvUWs5cjlOTmdGVG81QzNVQTYxbVBLQ3ZlZFNNMnJqc0k?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2289,38 +2289,38 @@
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46075.87481481482</v>
+        <v>46075.74761574074</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Spain: Las Rozas Black Demons rally past Zaragoza Hurricanes in second-half thriller - American Football International</t>
+          <t>Search continues in Kildare along the Barrow - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Spain: Las Rozas Black Demons rally past Zaragoza Hurricanes in second-half thriller - American Football International</t>
+          <t>Search continues in Kildare along the Barrow - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 05:45:33 GMT</t>
+          <t>Mon, 23 Feb 2026 12:34:17 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxPcGUwMFYxdHY2dEZ6TXR6aFk2MlowaVV5bElVem9WRDBobjRld2wzR3dmWHBqZjBIVFdWQXVrWGM2VE4xSERvcnBTc3ltNFVCeEJlSXFMd2pIQ3kxMHIwWXFReU1KSnMtZGx6LUpFSE1iUzlXN1lUNGJfVnZPclVhM0ItN2h1SnVVNU9renpfVmlpTEJvMnhERElrR1JVZkdZeGRYV0ZKcjVuOC0xNGhrbXdsWjQtWHZtNHIxS3dJMm1TS0F1ZDB6TTZ4STl1dzTSAc8BQVVfeXFMT3BlMDBWMXR2NnRGek10emhZNjJaMGlVeWxJVXpvVkQwaG40ZXdsM0d3ZlhwamYwSFRXVkF1a1hjNlROMUhEb3JwU3N5bTRVQnhCZUlxTHdqSEN5MTByMFlxUXlNSkpzLWRsei1KRUhNYlM5VzdZVDRiX1Z2T3JVYTNCLTdodUp1VTVPa3p6X1ZpaUxCbzJ4RERJa0dSVWZHWXhkWFdGSnI1bjgtMTRoa213bFo0LVh2bTRyMUt3STJtU0tBdWQwek02eEk5dXc0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPQ0ZHNG9EZklpZHFCNEs3ZEJUOVpTM25ENmZKdEg5LWNQLWVuM2ZsWXZUZlRYQzRzb1cxQlRUVnUwZF85eFlvYm44Qklvb0RmcTJqMHNjU012VEVJY3J1M2RFZ2V4em1HUFlEZUN2TzZ0cDVZNHV4QzROaEJrWkwwMDd2QnlScVBWUW5VektiSlgta3kxVkdxLW5OYUV0eG9FcWc?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2344,38 +2344,38 @@
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46076.23996527777</v>
+        <v>46076.52380787037</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Spain’s luxury mansions: where global buyers are investing - Idealista</t>
+          <t>LGFA - Dubs secure victory over Kildare - dublingaa.ie</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Spain’s luxury mansions: where global buyers are investing - Idealista</t>
+          <t>LGFA - Dubs secure victory over Kildare - dublingaa.ie</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 07:00:00 GMT</t>
+          <t>Sun, 22 Feb 2026 17:24:44 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQR3djQzdWMVh1UWY0OWg5YVdaMno3OVpMbHVJUmxSVTRfVVRuZ1FfVHdkVzBoWFlRVV9TVldvS1A5a0xlVHdKT0NBZjhpUGprZ3VZOW9XMFBGWU5vb3VmZm9TRThGZkdPMTV1V29LTlZVZHdadWdiR0FmVUtrcXl4UV9aSVRLaHo4MzI3MWx6OXZfQ21kZjVjN1ljbE9aTHM2Z2ttaDNLX2h1QnEzempOY05MYzJpMHNZU0xzQVVPX1pmMmRUMGhFMHd5elduSUVPTW5DMWVQOUHSAdgBQVVfeXFMUEd3Y0M3VjFYdVFmNDloOWFXWjJ6NzlaTGx1SVJsUlU0X1VUbmdRX1R3ZFcwaFhZUVVfU1ZXb0tQOWtMZVR3Sk9DQWY4aVBqa2d1WTlvVzBQRllOb291ZmZvU0U4RmZHTzE1dVdvS05WVWR3WnVnYkdBZlVLa3F5eFFfWklUS2h6ODMyNzFsejl2X0NtZGY1YzdZY2xPWkxzNmdrbWgzS19odUJxM3pqTmNOTGMyaTBzWVNMc0FVT19aZjJkVDBoRTB3eXpXbklFT01uQzFlUDlB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE0tWDdBeWpTdkNBZVhiRXNuc3ZrcGQ4RHZpbzRGd0M0WTZzNDBVWUk0T2RsZWR4M3hSTWJZYUFZdzBFTF9yTzNfX08yN2Q1R21VYk1DYmdtTk1QaDd4MzBxNjdMYkk0Y18zbjhraC1LNXNUSTBzeFE?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2399,7 +2399,7 @@
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46076.29166666666</v>
+        <v>46075.72550925926</v>
       </c>
     </row>
     <row r="37">
@@ -2415,22 +2415,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Search operation underway in Kildare after reports person entered water - Irish Mirror</t>
+          <t>Former husband 'does not accept he is divorced', woman tells Kildare court - Kildare Now</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Search operation underway in Kildare after reports person entered water - Irish Mirror</t>
+          <t>Former husband 'does not accept he is divorced', woman tells Kildare court - Kildare Now</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 05:56:34 GMT</t>
+          <t>Sun, 22 Feb 2026 15:00:00 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNR0FNY0lDUjkxYTVDbjNBVFBEclA5cVpETmRzaHhqc2Y5VTMxMXBOeXJpOENFb3FqWFBUeVJpbW9CSUVsS1QtVDlIR0JZbFJRc011aVJJOWFmRUxEbGxob24telZKWFlVZGctcXlsM0Qya2h1MXFRQnVEZThoYy1WTGZqLVN5djZIakZqSU9tSjE3S0RIUGfSAZsBQVVfeXFMUHhNb1lyLS1qMkk5R3RibzdCWUJHNkEwOUdHZGRUOHFVb1VOal83VTNHWl9Pek1hVnRyMWNjVHJUcnEtYldjdFZCc3N1aDdNVTk2UjQyQVVFWGNLSUFaOERaQXJxSktHaW9XR0kzLVlQY1FOb25INm04eDlvUWs5cjlOTmdGVG81QzNVQTYxbVBLQ3ZlZFNNMnJqc0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQWmxiZWhLcV93VXNZcWFrQ3UxM29xVnJnNEVSZW9qVFdqc2dJY0xmd0d0SGZ4WHR3eWEtRmwzbnZUNi0yNmpnVTB3LXpRalpGOWZldmZOYjJkR3NQODdTY2FWU0xOSHVYWG5NWlBnRHduS1l1T05fZ1Q5Q1hrTUJ4czRPMFRvUWo5NWNubmVJNk9QLXNpMFZoaVRpeFBZT0x0RUVOcVFoSllnWVNlLTctLXpRRTJ5cl9ZemlDc2FoZEI2VTJVSlE?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2454,7 +2454,7 @@
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46076.24761574074</v>
+        <v>46075.625</v>
       </c>
     </row>
     <row r="38">
@@ -2470,22 +2470,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bicester Motion announces two new senior appointments - Yahoo News UK</t>
+          <t>Poor Kildare give way to Cavan in dismal affair - Kildare Live Leinster Leader</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Bicester Motion announces two new senior appointments - Yahoo News UK</t>
+          <t>Poor Kildare give way to Cavan in dismal affair - Kildare Live Leinster Leader</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 13:00:00 GMT</t>
+          <t>Sun, 22 Feb 2026 16:59:27 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNcFpYbFZXdUdYdzNvdl9od1RuMUdpWm9yMmhrUGs3dW1YMUVNenIyLVFMcnJiaGR3czhfTXM2TGh6ZUNvLUtjVDlqd1d6NmE5S2lWbS1Gc2dacEdjcmlBM2JFN1lRZU9pY3lGSzJYMTBIVE1pTEk4OGVqUzVnbWJ5aVFKRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQVml5ZlNRaEhfTi1WbEpTcC1VS3lGZnZyaDBPS2pPdWdRVFF6NXE2LWtwWHlCZENmSjM3bDhiMkE0NlN3OGJ3RHpreEswMUgyd0VKbk9qNEpnSjFjYWk4NTlVRGtHSlBQRjA2ZGRVaFE4YUFyY3JhaHN5LXYtNk11OVNhb0NvLWVib3c?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46075.54166666666</v>
+        <v>46075.70795138889</v>
       </c>
     </row>
     <row r="39">
@@ -2580,22 +2580,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Kildare County Council encouraged to progress rooftop solar panel installations - Kildare Now</t>
+          <t>McDonald’s drive-thru causing traffic jams in Kildare town - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Kildare County Council encouraged to progress rooftop solar panel installations - Kildare Now</t>
+          <t>McDonald’s drive-thru causing traffic jams in Kildare town - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 09:23:00 GMT</t>
+          <t>Sun, 22 Feb 2026 20:01:39 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxPWEUzLXlaX3pyNHY3M2tkUTZ1ZXpTaFlfM1FZSGhON2JoX2k2eEF6TUtfcWJlaE83ZUloRmNkX1haSmdGRmY2TERRVFJsa2dPTS1WNzdfN254NGxlaGNZNWhlTUM4UmN3d1lBUWhvejRXLUh0bmU4RU9kOU14SHZpUW9STWE1TmJPa1pyemJnT19EQkJfT3IyV003UHpnZ292RVhIaWZBMk41bUJ6T0dGSEU4LUpNUkhOZ0NlalZlTVo0VGp6eGJPdTkxMTNwczJuUnJSdkVwcEZsenRf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWElKdEpWUmpFTWczS2l5LWFob2pDaGdpbUJyWFM5elFGajFkQ21UM3hyeHc4NXJnZ2x3ZW1vdThhVVRjVW9jbXhjWHZ3YTRFQlpXY1VqQVdINFdLM3NvWmxOZ3pwZWNCLVB1MlVrYU11WExvWlY1YnZlbEVzcUw5RUhCUXJTekRMV2hBS2RJX3A0ZFRjQnlrTE40NjNBNnlQTE53ZTdEbWQ1RXNrTVE2RG1QVQ?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46076.39097222222</v>
+        <v>46075.83447916667</v>
       </c>
     </row>
     <row r="41">
@@ -2635,22 +2635,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Poor Kildare give way to Cavan - Leinster Leader</t>
+          <t>Kildare sucked back into relegation dogfight after dismal display in Cavan - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Poor Kildare give way to Cavan - Leinster Leader</t>
+          <t>Kildare sucked back into relegation dogfight after dismal display in Cavan - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 16:59:27 GMT</t>
+          <t>Sun, 22 Feb 2026 21:31:41 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxQVml5ZlNRaEhfTi1WbEpTcC1VS3lGZnZyaDBPS2pPdWdRVFF6NXE2LWtwWHlCZENmSjM3bDhiMkE0NlN3OGJ3RHpreEswMUgyd0VKbk9qNEpnSjFjYWk4NTlVRGtHSlBQRjA2ZGRVaFE4YUFyY3JhaHN5LXYtNk11OVNhb0NvLWVib3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQSnZwWEF3a2xxcGNSYXhhcFBIN1pnOHJ3TDlIY3BIeEdvX0R3WmZCVUJaem9WRmR0bVdqMHBsU1JvbGVsRUcxZDZMdGlyc2pvN1Y1SkEwMVE2NzNqNE1OTkIwSnBlSURnWWdpZ3d4OTRsMTAxV1JWUHprRUVKNXoxTG93TE9vMm45V2h4SjJ3R242Z1o4Y0pQcUU0NVVJNGhSWmszeXNWVHA1ZldGNTVFUDNzRVVPQ2x1Zl9rLVJpVERfRWZ5YlNwR2ZR?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46075.70795138889</v>
+        <v>46075.89700231481</v>
       </c>
     </row>
     <row r="42">
@@ -2690,22 +2690,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LGFA - Dubs secure victory over Kildare - dublingaa.ie</t>
+          <t>Pair sentenced for drug dealing and having an unlicenced air rifle - Oxford Mail</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>LGFA - Dubs secure victory over Kildare - dublingaa.ie</t>
+          <t>Pair sentenced for drug dealing and having an unlicenced air rifle - Oxford Mail</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:24:44 GMT</t>
+          <t>Mon, 23 Feb 2026 05:00:00 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE0tWDdBeWpTdkNBZVhiRXNuc3ZrcGQ4RHZpbzRGd0M0WTZzNDBVWUk0T2RsZWR4M3hSTWJZYUFZdzBFTF9yTzNfX08yN2Q1R21VYk1DYmdtTk1QaDd4MzBxNjdMYkk0Y18zbjhraC1LNXNUSTBzeFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNTHVNSDlCQ0ZlMUZwZTBKM2llc0hOR1lnRUc5blhOOWd2amxLYm01WlpReFF1cmpfU19CN3l3NGdmZ1VDRjJfSmhVazZISVB3ZDhWbk1aVHNEbGl6Y0tTUGVhQkwwR3BBcHQzWFJsdHgyay1QQ1JqUnFoSm1EM2JaM0ZiblRWUG5BRmtQclByN3ktNlFpaWdJ?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2729,7 +2729,7 @@
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46075.72550925926</v>
+        <v>46076.20833333334</v>
       </c>
     </row>
     <row r="43">
@@ -2745,22 +2745,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>McDonald’s drive-thru causing traffic jams in Kildare town - kildare-nationalist.ie</t>
+          <t>Road in Kildare ‘is like a patchwork quilt’, local rep claims - Kildare Now</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>McDonald’s drive-thru causing traffic jams in Kildare town - kildare-nationalist.ie</t>
+          <t>Road in Kildare ‘is like a patchwork quilt’, local rep claims - Kildare Now</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:01:39 GMT</t>
+          <t>Mon, 23 Feb 2026 13:05:00 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWElKdEpWUmpFTWczS2l5LWFob2pDaGdpbUJyWFM5elFGajFkQ21UM3hyeHc4NXJnZ2x3ZW1vdThhVVRjVW9jbXhjWHZ3YTRFQlpXY1VqQVdINFdLM3NvWmxOZ3pwZWNCLVB1MlVrYU11WExvWlY1YnZlbEVzcUw5RUhCUXJTekRMV2hBS2RJX3A0ZFRjQnlrTE40NjNBNnlQTE53ZTdEbWQ1RXNrTVE2RG1QVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQc0NBaUFXZlFwVlEtZnBFS3RlZF9walhsUHFLY1U1Vjl5ZTFsTGFSUGQzcHhGeHVyMDFWWEloUVMtSld3X1Z2VTIxS20xUGV0elE0c042TjMtSUxiUU9HcDdoSHozN1JrZ0ZtNzhXaVVJelplOWdmOWZXNFl4UFBKQVRDNVVvU1hQQTV1MXdYZ1Jzc0V1MjR5R1NrYlctbE10YlJSXzYzZWtVbDRjZlF3TkxoeGg?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2784,7 +2784,7 @@
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46075.83447916667</v>
+        <v>46076.54513888889</v>
       </c>
     </row>
     <row r="44">
@@ -2800,22 +2800,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Former husband 'does not accept he is divorced', woman tells Kildare court - Kildare Now</t>
+          <t>Claim that independent bookshop in Kildare is suffering because of parking dilemma - Kildare Now</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Former husband 'does not accept he is divorced', woman tells Kildare court - Kildare Now</t>
+          <t>Claim that independent bookshop in Kildare is suffering because of parking dilemma - Kildare Now</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 15:00:00 GMT</t>
+          <t>Mon, 23 Feb 2026 11:05:00 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQWmxiZWhLcV93VXNZcWFrQ3UxM29xVnJnNEVSZW9qVFdqc2dJY0xmd0d0SGZ4WHR3eWEtRmwzbnZUNi0yNmpnVTB3LXpRalpGOWZldmZOYjJkR3NQODdTY2FWU0xOSHVYWG5NWlBnRHduS1l1T05fZ1Q5Q1hrTUJ4czRPMFRvUWo5NWNubmVJNk9QLXNpMFZoaVRpeFBZT0x0RUVOcVFoSllnWVNlLTctLXpRRTJ5cl9ZemlDc2FoZEI2VTJVSlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxPTmVXT0ZBZG5sWE8xMk5IeFpPeFhHNUY5OHljdC1NX0ZUNV9fVGpIS094SS1QbGh3SEREc0hNcEh4MFZxYVE1UWxoaFBVWENPTk1XbHo3Yk1wWkpEdUNMLUFDalpZZzkxa1QzbWhiZVg4Zl9sNkhOTk5ZbUhPYl9zZ1A3RWVqY1ZyUmZPeE0wQnB3MnJSTC1XZ25GQTYxaDY1bGxzTzVfdlg1Y1R1OGVwSVBFdDBtc0p3cDFfdXlUdnFaY0x2cHBhRFVtZXltcmwwSHBRUQ?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2839,7 +2839,7 @@
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46075.625</v>
+        <v>46076.46180555555</v>
       </c>
     </row>
     <row r="45">
@@ -2855,22 +2855,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>UPDATED: Search in Athy stood down this evening - kildare-nationalist.ie</t>
+          <t>LATEST: Attractive apartments planned for this town in Kildare - Kildare Now</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>UPDATED: Search in Athy stood down this evening - kildare-nationalist.ie</t>
+          <t>LATEST: Attractive apartments planned for this town in Kildare - Kildare Now</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 20:52:30 GMT</t>
+          <t>Mon, 23 Feb 2026 10:30:00 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQZ0xWSkpYbVB2eGwxQVF1UzdtT2VBQUo2NHZGV19iTmVjaEtZZmFZcEp2cjAwaFJlTkFvejdsS0FFcTlTYVAzUml2TW5hUUEwT3FGMklWMWgwNTVoVzFwckdkWFVUQzJlMmdNaHFqTXdHVmh4VDJZY1BGeWRoQ0VVbHR2RC0ycWRIV0xzaENzcGRJa3dwTnFhSlJ6dVc2TWxNeWpHUw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNQUc3VkZBTTBTMjdpdm8yWEhlWjl6Q1JDUzA3XzFNQW5BQTE2WVlPb2pRVkdRNEZNTXpBSU0wSmVsMklXTXlOX0Z0STVtYUVPOVkzb01TUlJRY3k4cTd6VloybzhzUXA5V3ZKaUhWOFhCV1FkcW1vUW1BNFo4bUxkbTZQSHRrS0VybFRKSXFEaDMtVXZwbnAyRE12WU1rTnVtNUt4U1ZzOG9OZVhjTUNmLWhXaEhvUQ?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2894,7 +2894,7 @@
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46075.86979166666</v>
+        <v>46076.4375</v>
       </c>
     </row>
     <row r="46">
@@ -2910,22 +2910,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Emergency response in Athy following report of person in river - kildare-nationalist.ie</t>
+          <t>Kildare woman locked herself and children into bedroom after partner broke into her home, court told - Kildare Now</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Emergency response in Athy following report of person in river - kildare-nationalist.ie</t>
+          <t>Kildare woman locked herself and children into bedroom after partner broke into her home, court told - Kildare Now</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 14:16:14 GMT</t>
+          <t>Mon, 23 Feb 2026 13:47:00 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPZDJjWllad1pFWWp4UG9may1DV19rZEtISlpNTEZaSjU0Vm85ZUFOUW5rbExLdzRIY1JreWkyN3ZlOGVjTVQyc1ZhbVd0aVFGbGtoSDdhdldENTBNVmVpSlJyQXNwbUlLMEJ1aWpFNk90aGtFUWJsMEpEUDgwQUZLVkc5empYSkctbkFOdkZkczRVQTJrZE9razBGbElabjEza2t2bGdEMWk3alA2TjUtQ3IzVl9fS1Vab0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxONjl3Z1A5Ti1kcno5SkFmWlVJX3doZUVPMWQ3ZndrUHdfaDhUUENHTGdYQjJHRmExTjFVQlpnV29NV0puc0wyNXRzWklXMXI0OHZTdG1qbWdRSzhyZXROT3dGajNHeFltblJyS2Q0Z2JKMV9EdjI1dmVUWFJCZXNZSFpmMXFoZmFBcGppOV8yRE1QdnRiRkF2V2NUVkdVdHhpcUFDMlVSSGxXTXpLbmVIb2RYVjU5OTB2WXFRb2VHalR6cUlsd0tWU2NlWEkyYXZ5WThWMGNxTUFiM3gtLS1WTXBTRGRWMFo0dTJZ?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2949,7 +2949,7 @@
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46075.59460648148</v>
+        <v>46076.57430555556</v>
       </c>
     </row>
     <row r="47">
@@ -2965,22 +2965,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Kildare sucked back into relegation dogfight after dismal display in Cavan - kildare-nationalist.ie</t>
+          <t>Dowling 'immensely proud' of his Kildare side after close-run battle with Clare - Kildare Now</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Kildare sucked back into relegation dogfight after dismal display in Cavan - kildare-nationalist.ie</t>
+          <t>Dowling 'immensely proud' of his Kildare side after close-run battle with Clare - Kildare Now</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 21:31:41 GMT</t>
+          <t>Mon, 23 Feb 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxQSnZwWEF3a2xxcGNSYXhhcFBIN1pnOHJ3TDlIY3BIeEdvX0R3WmZCVUJaem9WRmR0bVdqMHBsU1JvbGVsRUcxZDZMdGlyc2pvN1Y1SkEwMVE2NzNqNE1OTkIwSnBlSURnWWdpZ3d4OTRsMTAxV1JWUHprRUVKNXoxTG93TE9vMm45V2h4SjJ3R242Z1o4Y0pQcUU0NVVJNGhSWmszeXNWVHA1ZldGNTVFUDNzRVVPQ2x1Zl9rLVJpVERfRWZ5YlNwR2ZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPcE1iMWVSLWRYTzZrdW12eDNBRFJDVHktTXE2aDFrSDR3S1BLNm9xc2VaUGdGWE9FX25kVDhwckZSdkJWWHhFNHJHT0VETUROaHlhZ1RHUjlZaTNRZHF5V1c2NHdNU1NGN3VlMjhUTk5hZjU2YUJiUnctZVFrYnNUTUEzSkNPT25mQVRIU0w4ZXM4VmhtaGtXeThwOXN5OHZPNnJJTzJLcmZ4RUtCakN6X2tNbktTUGlOMkRJRUZYNjZIVk5L?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3004,38 +3004,38 @@
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46075.89700231481</v>
+        <v>46076.5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Fidenza Italian</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Pair sentenced for drug dealing and having an unlicenced air rifle - Oxford Mail</t>
+          <t>Leao, polemica dopo Milan - Parma: la protesta social per gol di Troilo - Virgilio</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Pair sentenced for drug dealing and having an unlicenced air rifle - Oxford Mail</t>
+          <t>Leao, controversy after Milan - Parma: the social protest over goals from Troilo - Virgilio</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 05:00:00 GMT</t>
+          <t>Mon, 23 Feb 2026 13:23:00 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQMWtjaUYzcmRYMmpQLVdMc2l2cnVGSkJhMV9kbXRQeEJ4MDdoRTR2bXQxRjhnZ2o0VWtfczhOd245Tk9JY2pzOXYyU0xHbTFDaXVlc0xCS2MwdjgzckppZkJIdnREOEZ2WlN2Z2JwTmVXZHRDTENHanlNOW9jRzZZZVRlSHpzT1RDTDBPZlIxOFF4eFdYV0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxOV05fZEVJUUNKa3plVU9UWkVSS3BYRFBlNjZxUVo1OUJjTDdiSkFpOXBFZ0IxWDFYN3dseWt4dFVlVFZVbVp5UVFaVnM4azlpZVF5QXZZMXpmWGV2eUFsNU5pdGtIWHhzcC1UbldUTjZUR0pGaGJDeC1vajZseVBMbmlQLTdWbmp2dDlGMlRKUDlESW1jMm5zSDhUUVN6WDd0YzZtOXNNYjk4RFpYOU1SMC1QWU9ZS2hHcFVjeXZGaXAtYUwycGNrdldkUGRHV2fSAdQBQVVfeXFMT2dYVXJ1TG4yRVIwWmZ3ZnhVNTlDemh6b196NlB1eFVYSFRpa3czVTZ1TVdibW9LVURjZ2FEb1Ftc25hc0g5YkI1ZU4waGJFYU1HbG9tV3pmcEtERG1ZNzBJMkJtcGxza3k4V0g3U3ZkNU9OeTk1RHp3VnU2Ry1TMGtWTEpDeEVuVVdYS2ROZ2x5djlhSndhTDJvb3B5U19wYldQUkQxTm00ZEMtWjJscEgzUU5fTTlRYjBsbHV1N2poNWViVERTWFdIbkwxTTRBREhyNGg?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3045,52 +3045,52 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46076.20833333334</v>
+        <v>46076.55763888889</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Village Fidenza (fallback)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Fidenza Village" OR "Fidenza") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>All you need to know about the February 2026 Local Property Tax allocations for the Kildare-Newbridge Municipal District - Kildare Now</t>
+          <t>Fulgor Fidenza - Nuova Pallacanestro Vigevano: 89 - 94 tabellino campionato di Basket: Serie B Nazionale Girone A - basketmarche.it</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>All you need to know about the February 2026 Local Property Tax allocations for the Kildare-Newbridge Municipal District - Kildare Now</t>
+          <t>Fulgor Fidenza - Nuova Pallacanestro Vigevano: 89 - 94 Basketball championship scoreboard: National Serie B Group A - basketmarche.it</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Sun, 22 Feb 2026 17:05:00 GMT</t>
+          <t>Mon, 23 Feb 2026 03:57:00 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQdUlQZ01sYVdUQk5TZllvV2hVZVFlb3p4WHNueDd2RENsTTkxMDFWVGdGWVlrNjFwdnRwdEVFRHEzWFVjRGZyVXBmd3Y0dENTWFF5WXh4OGtDcFdIUW1kbE95U1VDa2RrSnc5UUd4MGtoYmw1N2tmcFlJUzhKemxyU3FwQUxsUHZOZkV1a21uOUVPWkhvLUpCYmt3aWVBdnV6TXRySzlVbk5Cb2JqYm51M2VxVnhDZTRCQTdBa1duVlF1Q0Zrdkg5WHhjZExWNVdGcnk4cmNIRnJSLTFVdEYxd3hMM2U5cHVOVzRTOHExVktPaWQwckdnYmFmZ3NSWHVBZmxiTU5sVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPVklxcUQyVFRfaXl4bmRWYWFubU9hZkNfRzFyYTVaamx1aDRrN1IyOER1cDZrcWV3QVdnVFlaQjQybnZ3SHRLVTBZdXFpeHJudkJsOC1ONWs2ZEZaNXNCd2N6WkQwa0J4SS1RMjdNS3AtZ0t6c3NKU0UyYkZieUtEeUYyd0RJZHpBOVJpV09ybkRpZXJ0dEJERHF0b1FMcVBVYndvQXZSanl3ejQ3ckhJSlZjYUxMNzkyVnJaR3NKeXhqSi1nVzZZdHZTeGJfeHVfUWdIWElMV1Bwdw?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3114,61 +3114,6 @@
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46075.71180555555</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Village Fidenza (fallback)</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>("Fidenza Village" OR "Fidenza") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Fulgor Fidenza - Nuova Pallacanestro Vigevano: 89 - 94 tabellino campionato di Basket: Serie B Nazionale Girone A - basketmarche.it</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Fulgor Fidenza - Nuova Pallacanestro Vigevano: 89 - 94 Basketball championship scoreboard: National Serie B Group A - basketmarche.it</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Mon, 23 Feb 2026 03:57:00 GMT</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPVklxcUQyVFRfaXl4bmRWYWFubU9hZkNfRzFyYTVaamx1aDRrN1IyOER1cDZrcWV3QVdnVFlaQjQybnZ3SHRLVTBZdXFpeHJudkJsOC1ONWs2ZEZaNXNCd2N6WkQwa0J4SS1RMjdNS3AtZ0t6c3NKU0UyYkZieUtEeUYyd0RJZHpBOVJpV09ybkRpZXJ0dEJERHF0b1FMcVBVYndvQXZSanl3ejQ3ckhJSlZjYUxMNzkyVnJaR3NKeXhqSi1nVzZZdHZTeGJfeHVfUWdIWElMV1Bwdw?oc=5</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K50" s="1" t="n">
         <v>46076.16458333333</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-24 14:45 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>REVIEW: 'It's longevity speaks for itself' Shan Shui at Bicester Village continues to prove its mettle - Ox In A Box</t>
+          <t>B&amp;M Executive Increases Stake with Share Purchase on London Market - TipRanks</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>REVIEW: 'It's longevity speaks for itself' Shan Shui at Bicester Village continues to prove its mettle - Ox In A Box</t>
+          <t>B&amp;M Executive Increases Stake with Share Purchase on London Market - TipRanks</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 06:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 13:07:26 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQNHhwYkgyd1ZmTnNNLVZCd3otNHlNa2VLRHhuYlN0VDZlQlk2Y1M2WFVLSUNJUDhVQW0yclppd01lNTU1N0JyUGhGb2ZfZ1hnWFJmUEhkZnZTd2Z3RW1ZbmFZeDBZMXlUTnVOWkFjbmdsdGx2TXEySDF3bF8yZVJTb3pvNVhVczVoTXdDbnBWSU14bTdyNW5GSW9zVEg5RU9FYlloWnltSkZtVURCT0JWNUdnQ0NlaUN3UEkyenZXNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOSHBZdkZJZGozM29XREZrVmJtdnREMjRRcGJTcnVsTkhNdlpwZHRUc0V4QUVWZE9QV3BnU2VJM0pJR2p5cURSMWVlNWRfQkNOQzAyNk9IcTd0ZXhEY3lvOFJxN2lwWVVmX1duc2pmNmRoMEptZGszeFU4MXp0NlFicG9sbjZoaDB0c2F0RS1mczhFN01nc0FuR19vSlExNkhEOWVuS3l2cVNteWZ4dDhEanFQUmZyZVdI?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46077.25</v>
+        <v>46077.5468287037</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>'Disgusting' bins and rubbish at Oxfordshire Sainsbury's condemned - Oxford Mail</t>
+          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>'Disgusting' bins and rubbish at Oxfordshire Sainsbury's condemned - Oxford Mail</t>
+          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 05:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 10:27:32 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOdXNXbzM5M1gwd1ZmUm5VWHdqYVZ4T0swWVNoaDlxaEk3dFNzWUxmODBnQklwNF9JOERhckV0RGVmNTF3aF9xcVVEQ3M2TzRORDBNVXJtcDdpeHV6ekVaMEVsWTUtVUZ2N2Y3THFrUmJMaVFMT29nNFNic2V5MmUwZ2pYUkc1dkhaakE1WjdkVFpQU2p1NFdpLUd3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQNHZxbGRlR01sS215TlJRRHpQcXAwRDZzdGRNTUc0SG43OFRLcmlhUHlQTHhKcEtmQm4xZWZ3Y3p4UzNPUUs4dk50cC1tNnlrYUxib0x0N0k2T3VVRW00ejNVWU9OREU0OGNxZXFka2FPaW9QUVVoMmE1Z0pnWk9uc1ZGek5Td0YzMEhJSklma0J1SUhuNFEzNWxYdE5fVGtrTWs4WExabw?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46077.20833333334</v>
+        <v>46077.43578703704</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Rising UK Engagement with Chinese Automakers and Asia-Pacific Industry - IDTechEx</t>
+          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rising UK Engagement with Chinese Automakers and Asia-Pacific Industry - IDTechEx</t>
+          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 04:33:36 GMT</t>
+          <t>Tue, 24 Feb 2026 11:06:48 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPeDRlc29GOWdqOVQwYm5ZLS1BYUhHbXE4ZWFLOEp3ZEp2NU9kSHF2LVFyZmN5WW5Vb3lnWDdCRTUtZkY5REQ5ZVNNd29MRHZKdmVMRzFUcHZNTFhNN1VvZUVvcGQ3UHFibWRENE1mZG5EcTB1ODZlT2ZNYVA5dDJZeGhJUVgtUGZZeFo5T003V1ItUmR2b294YzVESUhzUVEzeG55TWVVY2JSaDhKeFBUSklzSURvZW5nNUNkcjFR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNcWdvdkd5cGZ3QmRMYjFQaExNdUx0S3dVcmdEelVjcUpwNUhKbENHMlJRRVFCeWxoZjJQMko2UXhOaVV5d0N1aDF1SVdDZXBOUDJoRmFsV1AtLXFZdkpjdUdWNXlxTWNBb1lnZmNnQVMwLUJVak9JVGNJRWo4SmdBT1dQWGcwLWk4NlRLcTd0OVlHbXppYTJTSkx3WGYya2xmb21WbUFHd211Zw?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46077.19</v>
+        <v>46077.46305555556</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Changes announced for Oxford Tube services to and from London - Oxford Mail</t>
+          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Changes announced for Oxford Tube services to and from London - Oxford Mail</t>
+          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 07:29:15 GMT</t>
+          <t>Tue, 24 Feb 2026 10:28:00 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPaTRYa2NPSkxzZE1UWjRJSjU3eXZ3TkZka3VXdGd0YndMdHpscHJzSmJ6cWRRTGhNM2plYjFDX1hJeS00T1FMMGtnc3BsaEN1SmZ1dVYzSUFqc3pwTmtDSG12LWlRY3dkcXBxVTFUUjlubGs1dFhLMG9weGZYelhKcmZCYTQ5T1NoX292cHBWdGN4Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNaDlnYVhpRlVxSXcxQXpzRzhaZVBTZzdhRmxESzFScjBxanNhTHVkN3IyZTFZUXgxazRRU1RMV0pBUUpYZnkxZnFQYmU4VGkwdWJFdnE5ZzRHemtjWHFWMTY3dHpPOWdkaWR1UjZWcXZUWG5sYV9iemNMQXFkVWtkTmpUeGdyWlJTbHBOWXFtT3NDMFd5SE52eUQ2S0pKYXg3dG1OMlZXVEdzaldqcXQzX1p1MXJoLUpIU0J4b0JDQ1FvdXU1U3ljV0Qyc25QeE9PRGlYc1dDY0dlcXp1ZDRxVzg0dVBvLVk?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46077.31197916667</v>
+        <v>46077.43611111111</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>One of the UK’s biggest villages to become a new town – with cosy pubs and historic canal - The Sun</t>
+          <t>Politie Brussel West vindt bijna drie kilogram cannabis en plantagemateriaal - HLN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>One of the UK’s biggest villages to become a new town – with cosy pubs and historic canal - The Sun</t>
+          <t>Police Brussels West finds almost three kilograms of cannabis and plantation material - HLN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:11:00 GMT</t>
+          <t>Tue, 24 Feb 2026 13:58:28 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQTFdPODFXLUpCeFczUnFia3EtVG9wRmExQUV3cUppMmFkWEQ3Z1RzZFBHZVMxRl8yNThsc1JTajdfQjdzWmg2T2VSeDlSd1NWVWFjMmlxLXBaZ2dqVEhiR2FrMFhSTWV1dUNtbDF6SWpSZmtBRC1TWnh5Ykt1MDVESW5mR0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQVDNCRUxNSms1VFBKUXBxVTdkcGVlb2p3MGZiajBHcmFqN0oyR19uaDY5UnIwcXFQc3lQY3JncXR6blFKR0wyUVpSZ2d4UzRMeDh5UU50QllENEdBaEx3Nk1XbmNlZWE4d2Rnd2hMUVVoY3dqSjh2eWFTSnVzel9OTlV6dXBwZjVubXFWVWhhSTY3X2R1enUyM0J4bFRDYmNYTXF5U0k4aVMzRWlzaUl6UUVNNWI?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46076.63263888889</v>
+        <v>46077.58226851852</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Organised Retail Crime Surges in UK Costing Billions Annually - streamlinefeed.co.ke</t>
+          <t>Trio krijgt drie jaar cel voor schietpartij achter winkelcentrum, maar schutter gaat vrijuit - GVA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Organised Retail Crime Surges in UK Costing Billions Annually - streamlinefeed.co.ke</t>
+          <t>Trio gets three years in prison for shooting behind shopping center, but shooter goes free - GVA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 06:52:41 GMT</t>
+          <t>Tue, 24 Feb 2026 11:39:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQYXAwZGpoTUZsSlVHOUpRbDl3OUsycnA1RkEwNE9IdHE1S3FiZEhZbXdwcENSa3dSTEE4aDZIVTB6ZXJWZWx4LXN2N25WWUJrNzcySnlkV0dxWlhsQUI4aHUxalJ5LXhGSG1HeVZPMjRwWWE5Ykt1TUN1dFNZQVZDTXB0ZkVmbGFuNU5weEVZckJud0lRVkZZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOUXduU0hBQ2g5c0puak1mdjJQUzBfdEwxNk92RFdaemd6ZzZTTkI2dkdWWmlZV1RTTVV5cC1IdmZubHlNQTVuY0dmdlJDQ1hoRU9GSVBfNTFLQ0o4RmdoZHU0REptS3JBTVU2ek9JMmtTWFItbVpuSS0tM0o1MzVGSW9TNFFiRTFJY2VTalhyQkhsSmR1V0YtNkJCWDN2dFJIYms5cUlKUkZ4Rmh1Tm5zQVdJVVBoNUNpY2ZJOG5zNVI2YnJkRTlGdTAtbVRrekRqeWo3MEFrUkVCX04tZnZzQV80MUJKa2x4V2xxVkVweXN4ZGM?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46077.28658564815</v>
+        <v>46077.48541666667</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Farewell tour for 50-year-old trains raises £20,000 for charity - Chiltern Railways News</t>
+          <t>Voortvluchtige drugsbaas bestelt vanuit Turkije poging tot gijzeling in Berchem en moet 7 jaar naar cel - GVA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Farewell tour for 50-year-old trains raises £20,000 for charity - Chiltern Railways News</t>
+          <t>Fugitive drug boss orders an attempted hostage-taking in Berchem from Turkey and has to go to prison for 7 years - GVA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 12:36:24 GMT</t>
+          <t>Tue, 24 Feb 2026 11:28:25 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOOHVqT3VMZy1qWEJUZDQ3dU9nSWZnSmp1UDZmYjkzNlczRnpYRzJwWjRtWEdjNVF5TG55RUdPX2tuTjJEMWFWWG91T0dtVERUZTdQa2U4SmlaNGxfTlJtejg4Wjg5LWNTak1oVE9PNEhLM2lOVGxRZnVUT3Rmemd0SXhvbzBCTkx3bDBXdjVqS0V3TGdOUXI0N1UxZDg5bFRHWDZha28yc3ZCdnNj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogJBVV95cUxNZV9xLWN3R3ZhZHYwUEY4LTktS3hKTXNDbFhTMnRLSHByY1NKWDlUNlVtS1pwSDFhdDFidEl6NEJDbHNLZkJZcTJ3bUkxYzNSNnNPbktjUG9HaXpUNGI1TzBKc1J2c3Fld0pqNWtVWnRiSnd5b1NEcFY1b21oLWUyaVQzNXRIZkJza0RQdW1ici1QM0hfam92a1lHWFNIcXgxQnNvcklLMWwyOXpzci1wUWVtdXdMbmdGeTg4YldQMUx6amszckRuZHlCVEpBV0F1dkU3SEpzaXNiQmZtMzYtVzZTZllOTERxTFpqZUR3ZFVoTGNSZlZSVHp6c1NUNk8yMDIxZk9FdXZOYlZ6eE1Bd3N4bm0ySXhYdzM2NjVVd1IxUQ?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46076.52527777778</v>
+        <v>46077.47806712963</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Chiltern to use four Mk 5A sets until late-summer - modernrailways.com</t>
+          <t>Gravin Diana du Monceau de Bergendal opnieuw voor rechter voor verwaarlozing van 270 dieren: “Al zes inbeslagnames in 15 jaar” - HLN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Chiltern to use four Mk 5A sets until late-summer - modernrailways.com</t>
+          <t>Countess Diana du Monceau de Bergendal again in court for neglect of 270 animals: “Already six seizures in 15 years” - HLN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 12:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 13:07:30 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOblRHV1pybVdYR1lYOUYwVTEteFIyYVZiYXd4bzFTc21UMDlnZFJLWklDU0FValplQ0RndTJNTjV0cm1sZG5jUFpWTzE3a3huRTV3YWRiSkZpcWwwNDhPQ3I1WFlxanhUNlZuNy1RYjUyNVA5Zk92aHJ0aUd5WXlhdVFONFI2RjBQZVR0NGpn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxOVlFnbkZRT0RIRkNUQjYxNjFxWlkxX3RESk1NMHZremJEbmhYX3lNcEJYLTBnN0pkck5jeFdWQ2NkUVh0VFRCbWt3T2d6QkF5V1pBUFlkRmRrRGNmekJtYVBjMTl5a1hZZXBma0tRM25PWmwwQ3d3UDd0bEwybXNPZHVIeUV5R3pyNkdIc3d3V25VZVB4bE9TUmtxNU1heEVnUTZMYndkSUtnY2Y0cUg4N29FRF9RTEJzMklOVHlwbGRyTXpVOVVwLWh3bFl5UzlnRjIxc2I3bEk3MEJzb3NhNmhHXzRRUU14cWRBNVFHVjZGZw?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,21 +900,21 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46076.5</v>
+        <v>46077.546875</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Valse bommelding aan Grote Synagoge in Brussel: omgeving en tramverkeer tijdlang afgesloten - HLN</t>
+          <t>Antwerpen dooft verlichting aan 45 gebouwen en monumenten tijdens Earth Hour - HLN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>False bomb threat to Great Synagogue in Brussels: area and tram traffic closed for a while - HLN</t>
+          <t>Antwerp turns off lights on 45 buildings and monuments during Earth Hour - HLN</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 19:18:38 GMT</t>
+          <t>Tue, 24 Feb 2026 12:00:13 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNWTVCY1dETU45MTMzQ1l4YXhSaVQyWjhjQjRtd1E0OEdMNllTQnZ5SlJiN2Rod3JUaTlMMTU3bGM2U01jSkJuUkpCUlExQXl3MUFFcE1acFdpRVY4MnQtcVdoZW5zSHlGZDBIRWlGQTFtLWd6RzJraG9iWWd2RHdJSktMYkRfaWFBN3prOUFTQTZyS1F6OUdfOWs3RzFqSzlGRF9LbDFsUG5LM1pyOGxSbWJKamItVXRmMTM0UW5EbXlmeWc3eFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVzR6UXJtbHMtY1FGS0t6eVZOdjNvcEFlX21xOU1WdGZGb0tPaHpndGtwdXJ4bE5nV2prVG1xM0ZQbUlsTHhkbzVZX0p0cThqWU5XQkRRZk9pbXJrZGI2VjRCelEtaXpYYUhuZnY5WUY0WXhQOGdfWDB3QWF1QWR4NVFNVjM2NVkzUjdkTlJkcVNxQ01XMERzWWU1ajkxWmVBSVFWYTlvSmN2VElyNU1uOF9jbWdUdw?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46076.80460648148</v>
+        <v>46077.50015046296</v>
       </c>
     </row>
     <row r="11">
@@ -985,22 +985,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Vals bomalarm aan Grote Synagoge in Brussel: “Volgens eerste elementen weer zogenaamde grap” - Nieuwsblad</t>
+          <t>Antwerpse takelpionier failliet: takeldienst Viaene legt na meer dan 50 jaar de boeken neer - HLN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>False bomb alarm at Great Synagogue in Brussels: “According to first elements, another so-called joke” - Nieuwsblad</t>
+          <t>Antwerp towing pioneer bankrupt: towing service Viaene closes its books after more than 50 years - HLN</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 03:20:00 GMT</t>
+          <t>Tue, 24 Feb 2026 10:34:08 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPLVNGa1QzTEV5X253bFc0c0pCX0NmNVphY2tGVHJkN3BjS2tyd3BHSmo4cGtsY09FaTR5NjhKNU9Dd01rQjY1c0wwZUFQWVdlTlBSTjFMcDZaenRISzJqTUlTNTJmOFAzbVF0Ti14Vjl5aXZlNkhmSWM5NkNKcjlwNUxTWHJOUnBuQU01Q2tIUmVjdkhTd1V3S1F5dWNwd3NxQ0d2WTFwNlI3aVV5MjR6X3gxQVRRRmVmekllYTdoUUYxeG10cTRqb2hyZkI1eEtOMGRlLTllTmVUY2JPRFlXQUhYdEdIWnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNanBoV2o1anpZNlhuVEdxS29TaUh6VXdodFVkZTExeW1uUkZsZElSendqbzhoczRLTVdvOWRKcE9Wa2lINkVfQjRtRjBYSVdvck5wM0RPeFpMaFdpcjR5LWYxUndSNDczZGg3Tk5zbzVYQUdyWThVQVg3dEF5UEE3aVdoRFZIWFhINlFlN3NWM2V5YzQxU1FZSXJ1OThxcDMyeldEWk91MlFwbWRGb3ptNE9VbUZTcExhZWcyeU9SY00yYTF5alNaeA?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46077.13888888889</v>
+        <v>46077.44037037037</v>
       </c>
     </row>
     <row r="12">
@@ -1040,22 +1040,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Vals bomalarm aan Grote Synagoge - BRUZZ</t>
+          <t>Waarom laat je een vriend op straat achter om te sterven? Heerlenaar Johnny E. (43) moet na conflict binnen motorclub Kanun vijf jaar de cel in - De Limburger</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>False bomb alarm at Great Synagogue - BRUZZ</t>
+          <t>Why leave a friend on the street to die? Heerlen resident Johnny E. (43) has to go to prison for five years after a conflict within motorcycle club Kanun - De Limburger</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 18:42:22 GMT</t>
+          <t>Tue, 24 Feb 2026 14:01:37 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNUmhvam1VWGcxVmZOSEEwLXh4cHp0ZzBPa0dpR3dxRzJpcGFzRnY3Ylc5TlRPZVllcExRbnpBT0NhSVdiRUY5em1MZGFsdk1CcmVvQVphUkVxMG5nS29BT3FCWW1QWGN1QzVuT1lTVC1wZ0tSUmZQSTI4RjdHdmZYMkR0ZzlFb2dU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwJBVV95cUxPZUV2S0NpbC1iRTlwRlpBbXB0QnBqNnZkeE9SWUQxLVdWRHp4MXloQXBvMlhNTVhXaFZJVUZKN2o2NGh1b1VyOFFJYlBsb0I4ZjJieFl5MnBYcDhYQ2Q4ZUZUVUotOExudHBNYkZlT1doSmxDd3lLbjQ0Y2FlRVZoT1JJUmFfNnN6WXBFVnZLLVNSbE9tVUJ5WWRFMmlsSk9teVFsdkNUNDlVR244Q3RnUEpjWk1HbkhHaXNDWks4T0UzYTRxMmpRQlduTGNkTUZzWmZDTmJMNC1BSFlGV0FZVG1idS1aekR2OFFrblVkMTAwQWtZVVktclJXVjNzOVhBQ3EwVUI5ZW42OUZQNS1haGdTSTFFMlNXRHdDcWllRHdWck84dTIwYlBRbU1yY3c?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46076.7794212963</v>
+        <v>46077.58445601852</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>‘Spion van Poetin’ opgepakt in Brussel: zakenman zou militaire technologie aan Rusland leveren - De Morgen</t>
+          <t>Explosief gegooid naar woning in Eygelshoven: geen gewonden, wel flinke schrik en beschadigde auto - De Limburger</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>'Putin's spy' arrested in Brussels: businessman allegedly supplies military technology to Russia - De Morgen</t>
+          <t>Explosive thrown at home in Eygelshoven: no injuries, but quite a fright and damaged car - De Limburger</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 02:00:07 GMT</t>
+          <t>Tue, 24 Feb 2026 09:46:26 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQODlCWFZTUFlFb01fd2dRN05EWTBuT3YzVEN6YUhDWnRnR1FfN3Y5NjdXcWJaUGtjSzZ3bkJpWGFLVkd5VEpHNzF6ZElHSC1RUGZFZlRGZUkxTHJ2MXBJOWlVMkI1aUJGX2VqeEdHU2ZWUzhqMFJFNkxuSXgzcWFSR1Z0dmxrTUJmdmpacVZnTEplVDItbUp5WHoxbkFlcnRGYmVka1dMbGt1Wk5GeTZkb3Jma0swcDhJSkdiRy15bFNMQlFwV2hJNVBnOVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOd0xSOHdvOXluc2R6b0hTV3pfMnBqUXVULVo4TFhTYkNOVzBSc1F6bjJFY0hVRjRVSEJ4cEo0UDlONU9yenRORzFOSWR1U2hzYVJVbGNTMXNsLUdSMUlKZjhNOEFQNG54cm0zVVc3YjhlelJGSFI3N1pESHJ2RmFqSVZvb2pNU29nZjNHNm9id3l4Y08wQmNWNDFnekcwbklORVd0V2VFc0xaMzBkcU5YZENvVkNoYmpxMGZzelM2aXhTQzJTZmlEcEpvclNsWWkzbXN5Y3VUQnNkY09aLXlVWFVxSUw3dw?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46077.08341435185</v>
+        <v>46077.40724537037</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Papa zet zoontje af op school in Antwerpen. Wat later vliegen de kogels in het rond: “Hij zou 50 miljoen euro aan drugs hebben gestolen” - pzc.nl</t>
+          <t>Opnieuw incident aan Antwerpse gevangenis: politie grijpt in na mislukte poging om pakketjes over muur te gooien - HLN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Dad drops off son at school in Antwerp. A little later the bullets start flying: “He allegedly stole 50 million euros in drugs” - pzc.nl</t>
+          <t>Another incident at Antwerp prison: police intervene after failed attempt to throw packages over a wall - HLN</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 04:35:00 GMT</t>
+          <t>Tue, 24 Feb 2026 12:38:35 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxOR3ZBTk1uT2pkY0thS0FZNWZFbjR2c2gxWkhBUEgtZExhc0ptdHU3RHk3Z2tCNUZVYjVIbExCd1BMUXRkQnlZeTVLMVRZNllzQmlwaEZOc29kVG5venNocmlsa09wd2ZScGJWSEdCd0t1SnBlQnB4VDNzaTNTaGUtemN3el9DWFB0OEJnb0p1M1ZuRXd2bDRkUnVLajNtbGVsbGNfTGUzLTFObGpuRDhJNWhrUEZFV2JpXzFxeXRCeXluSEpXTDZOVlZKOVlVTWJ6TDBFZm80V2dvZHB5WWhudExNN3ZIbzFsMXdSeU4xc21jWWN6eGhGRFFad0JuYlQ4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPbGtHUkJLT01KeFFCU1ZHR3dTRUpOdlhVSVl3b2hKRXViSUNGZmJPRTJiMjZzemx1MjNzRGtRZzFDUElVMllrSDZoUWNnekNJU2hITWtDVlBobTRzSTB1c20wNnZoTklISm1qTEQ2N0YycmFvakZzY0xyT0NIRGxHaW5WWHpVWE5xYXFpYjRDalZPb01rMHFERWszOUx5U1Q4U1J2Uk9VU2NyY2ZvYVlJNjBVR2RyLWx5dURtU0x6clJfNXlFa2ctejRqS0NELTI5cVZfQ2pUN05PblVLRHltUG5WQWM?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46077.19097222222</v>
+        <v>46077.52679398148</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tiener móét van ‘Zero’ naar Antwerpen rijden... Wat later woedt brand bij juwelier en krijgen hotelgasten rook binnen - HLN</t>
+          <t>Beurtelings verkeer op de Kapelsesteenweg door bekabelingswerken - HLN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Teenager has to drive from 'Zero' to Antwerp... A little later, a fire rages at a jeweler and hotel guests ingest smoke - HLN</t>
+          <t>Alternating traffic on the Kapelsesteenweg due to cabling works - HLN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 04:36:58 GMT</t>
+          <t>Tue, 24 Feb 2026 12:05:04 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxQX21rWDN5aHZDUzI2X1hIb1JxaDRVRXlEYlhMaGt2Uld4RjIwWGhDWWl4aVZsTVBlMndIVUZ2UFg1WUhGM0tMVXJTc3N3cFctUWJVNl9QNHRmWXpRWHowTkljR2dtNnhFSHJaY04zS01WYl83Y0gzcG5famVkOUs0TGJWZlpTX201U2hvOEdPVmFCNVNpV1pxb2VkallKbEtfc3Z2NGEwdmRZSmxObEVDQXAyM0ZPeWpORXhWMUJNOGo4UDZDQ0dheDBCY3ktYlVVblNHQ2VGalpTZVNWZzRfQmtkaVEyQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPVVVoM3lVUzdhOWJUT2lGSi1HbDRHQmExeG1falVTUEt1WEdBRFgwRlJJWUJIV0xmd0M2UmlkdTN5X3RDa2Y4b1FjU2RzSGdFMmdXMHNsSGZhUXBIeHR0Mkh4MDhVdTREbTFsYXV6UUtxRzRIM2ZCM09MQkg0RXo5c1Y0YXcxZ3lSSmhyM3dpemoyMU13UlJNSVR0LTI1ek5sWGN6cWxn?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46077.19233796297</v>
+        <v>46077.50351851852</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hof van beroep buigt zich over wrakingsverzoeken in zaak-Costa: “Mijn cliënt gelooft niet meer in een eerlijk proces” - HBVL</t>
+          <t>Showing Off brengt visuele poëzie van Ziekenhuisschool Antwerpen naar M HKA: “Ik ben precies een echte kunstenaar!” - HLN</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Court of Appeal considers requests for recusal in Costa case: “My client no longer believes in a fair trial” - HBVL</t>
+          <t>Showing Off brings visual poetry from the Antwerp Hospital School to M HKA: “I am just a real artist!” - HLN</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 19:23:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:38:05 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxQNlh2cU1lN1puZmpfZl9TblJvbVRMOWtxMU5QNzZ2aDloSXNOZHFQUHN0ZW81SzJlcnZxaXJSSzFoUWNNY2pJbThxVk5lRm8yMWRWcHhTTEtick1DLXN1WVBLZmdISXJJSWJ3WDBNNVJSRHVWOHJuZUF4dUZMLS1YaV9rdVB5cFBHRGpac1duQm0wQURWenlGN3F1Yl9yRW5yOUVmdWhrejhSSENKa2lfdURpRW9PaVp3VlFEb2hjbk9veUN5X1VtWFRWSDRTTmZFYm95YlJrSTRIWHNmQ1lvak8xQ2w0MjdCY2NheUVqMUZ3azY0Y0c4TW1rRGNqbUtaX1hJSUU1aU1WWE9IZVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxQN0dJaG1VRGdjZWk1b0ljQWdTbmZtaDBxZU9UQU9CbFE0WHJaazJ2Y2k3S2RUVVdoN1NuRnJYejRVMkR2SlZ5UTlkaHdPcFZHRGpzdGtRQ3lLU29mcjhJVTlXWW9Ja2dPSXVmdlRnTTZnUkQwMHRHZUtPRUwtRWFwZkVuVVVCT3Y2VklTM3VHSGw5QnFHYWNPNHE1bnprQktCWlVrQXV5LWNWbUZGMVVVUk90T0oxaWhqSjZJU3hUM2NUUEliZDlKSzZvLWF3SlBGcVdSbFJpQTFVd21lNy1WU2JFc0c?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46076.80763888889</v>
+        <v>46077.60978009259</v>
       </c>
     </row>
     <row r="17">
@@ -1315,22 +1315,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Oefening Snelleresponsteam (SRT) levert indrukwekkende beelden op - GVA</t>
+          <t>Maart is Jeugdboekenmaand met meer dan 100 activiteiten - HLN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Rapid Response Team (SRT) exercise produces impressive images - GVA</t>
+          <t>March is Youth Book Month with more than 100 activities - HLN</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:23:01 GMT</t>
+          <t>Tue, 24 Feb 2026 11:16:34 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPbDZkSXpSOUlTSzA1SWtYdTZFUVZpaTN3UFAzdzZUQkplNEk1SkFvSEx1dWpweWdvdFA0VlBYcDJ3VzYwZFR4bnpjUzZkTllXOTA5c0YxS284bTBfS2ZFa3RZVmQ0cnZyMmdmTk1mc1NuUWNVc2p2QV9haTNyRXl2THIxZFoxQ2hnRXY0eHA3eUYyWng4cUJhMkwtakpxdy1XM1VxUGlYR3llcnBHcHBlUHFVYkctNlN4NTFpWVlBYjJMeEotUm51V21oVktmbV9SSFQtX2RR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNYnVLZVc1VjNxVmRLaVpZWTk1XzlLVTBrV1d3bmdOZlNELXpFZDNpS3BhQ25QcmMzX0doVUdMY0NsWU5YMzg5VlF0WThSQVpiTk1EdHdHelFuMXJjbkdadldvV1hQWW9ZTzZFNWRhSzhnbVZTSk4yS3ducjlpWHV4U1NkeEVoQ29fZjZPRlFUbzJlRmRyOUVMNHpB?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46076.64098379629</v>
+        <v>46077.46983796296</v>
       </c>
     </row>
     <row r="18">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Notoire drugsbaron ‘Flash’ gelinkt aan granaataanslag in Knokke-Heist - Nieuwsblad</t>
+          <t>19-jarige krijgt vier jaar cel voor brandstichting bij juwelierszaak in Antwerpen - GVA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Notorious drug lord 'Flash' linked to grenade attack in Knokke-Heist - Nieuwsblad</t>
+          <t>19-year-old gets four years in prison for arson at a jewelry store in Antwerp - GVA</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 01:45:00 GMT</t>
+          <t>Tue, 24 Feb 2026 11:25:42 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxOREMtU3Z3Q2ZUQmh2dTJKWHB5SDFYVklncFk0ZE1fUGRWUnJyUjN1OUktTGh1a29ma0ZFdFZYWENEQ3NwQUNrNEYwcW1JREdkTF9HaWlRR2pfOU04eHBXQXlHOFZKVUs3dzBvaFEyZll3eGNJUklvOFl1a0E0bnAybHFOT29YaGQyS21nUFYtd2c4VGVkZ19fb2FjQ2RtS29HZXdsLXp5R3F5RHh6VnFoTld6VTNOc3RXWlJ6dmhlTUJiTzRCTEpRVDBQdmxxYU1XbFhSdFJBTUNDLVQ0Y2Q0Qm5UTDdOekNqLWVGV2hlUWc0RVcwM0lnaQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQa0lwTTV0TjFWaE9SaWlLNFIzVzgzX2N6S2Uzekt3Z2tLWjhrRGZnRS1aWjRXWjU0dDF6VlZHelNiNkd1UmtjSE43MGN4VmVEeDFmX01GUTR0N0x0dmdvS3NiSFVVNEV6Ym1IVUg4WEFPb0paMWhCai12YU9Gd24tWHZPSm1GUzNXbUd6YUI2VE1xaURaYlA5QllGcGUwRnpuQ3JuWWNLbTc1MkJQX182Y19NN1FZTk9iTzctR3h4eDVnWkZIa1pSWHN1WkM0QkF6eFVBTzUtQ2VaRFk2Zm1VT2pRQl8yMGpqNEhTUWlB?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46077.07291666666</v>
+        <v>46077.47618055555</v>
       </c>
     </row>
     <row r="19">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Oplettende voorbijganger helpt politie inbreker te klissen op lijnbus richting Antwerpen - HLN</t>
+          <t>Drie personen proberen pakjes over gevangenismuur te gooien, politie rukt uit en rijdt wagen klem: “Ook minderjarige in auto” - HLN</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Attentive passerby helps police catch burglar on scheduled bus to Antwerp - HLN</t>
+          <t>Three people try to throw packages over the prison wall, police arrive and crash the car: “Also a minor in the car” - HLN</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 01:58:36 GMT</t>
+          <t>Tue, 24 Feb 2026 11:41:34 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPSVVWMEZtMTZNTVN3YnZYTjhHMGl5blBYNVVoZ2pTOWVzYlhKMm1hVkZRUWtmNEVIcWdRalJteGJuR3VSSU9IWEhUNTQ5aG9GWDBfYUNpb0dZdll4c2NJRTlCTXlIUDFNSkFMTWtQZ0I2SUU1b1Z1TGNhUzlUTWZ4dVlvd0lEQ0c0ZFVfbGZJellkNkFfSGdhU2pTSExLcUFod1JxMEZuVlE0UjExQnRQTHdQM1dTTUp4YldiazRYTmxTaVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxPOVNDVFlPaHBTcG1tMmc4SjlqZkFESUg0LUpFQ0hmbEhISGhva0I1Yl9IcTk0X2s3cVdFTGNkRXB5UDJvWGYtM3dzcDVKdVhmMkhJNlU1UG1YMXc3MkI5c3Z6U3pKeTBMTGUxZjN0LXBoT0lnbXpObFZEYmpGYkxkS29VUno3dTZrb2VNMFVJcFk0emhFUl8xVG90enZvRmdkeDZRWndiOWNZM2hZU0ptMFBrbVZGWThyRnpjb013RnM4MDNtdE5HdWpDM2VXcUFPNDY5M01qdjlPNXREMExQR3I5UlBpTk9EY1pCNkJIYWR0QQ?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46077.08236111111</v>
+        <v>46077.48719907407</v>
       </c>
     </row>
     <row r="20">
@@ -1480,22 +1480,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Jonge ondernemers lanceren app die Antwerps nachtleven bundelt: “Handig overzicht in plaats van onoverzichtelijke waas” - HLN</t>
+          <t>Stad Antwerpen genomineerd voor Vlaamse Verkeersveiligheidsprijs: “Minder verkeerslichten binnen zone 30” - HLN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Young entrepreneurs launch app that bundles Antwerp nightlife: “Handy overview instead of a confusing blur” - HLN</t>
+          <t>City of Antwerp nominated for Flemish Road Safety Award: “Fewer traffic lights within zone 30” - HLN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 07:01:06 GMT</t>
+          <t>Tue, 24 Feb 2026 09:48:33 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNMkRPZ0ZtVEpRMHVSYTZGMDhqY1RYRzZIck0zQjE4MzM5UmRmdE1VUFpPSWJZR0ZCOTI0Y0kxQXc5VTVIejNuQzJQOXdhRThUc1NqWTBPajFnelFuUjZ4VzdPUmpLaDg2TmtMSU1FTWZzRGtsWjJsWGlrQW45Z041Y0d1UXotNzVHcUd5ZDhwYjJ1SUt3WXhibGtSZ2gzYkFoaTFvM3diYWlCYnVyc1hMczIzOGk2UHlkNWMxa25zRGF0VEdHNVBMNXpWYkxrR3AwYUlZbHA4eld3WVNXVkNkR0xIamI4ZVZQdXFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQMmZMVXphNzNLM0ZZNjFUZXpLUjhwMEF3YjI1d3FrX3ViUG9UV1drOEFFYzZtaGdZX1BwajhRZHhrcUYxRVktNENzSVktUHVMTzZycDFOSG1jZ1NiR0E0Qnk2YXdxQURVOGRFeDVqX1NUb0hiSjdHZUZTRDVLNkhmLWdJekFUNkx5YlY2QzgySVJqYXlGSXBENUNTanptQi1YR0ViU1ljTDJ4SXVERHR6b2FrQ0MwXzJLQ1RPOHBGZ1dHNWhONXpHOGpDRHhyN2Y0MkR0Sm9XOW0?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46077.29243055556</v>
+        <v>46077.40871527778</v>
       </c>
     </row>
     <row r="21">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>“Ontruimd wegens zeer hoge CO-waarden”: burgemeester Els van Doesburg laat vier shishabars tijdelijk sluiten - HLN</t>
+          <t>AG Vespa zet Wolstraatcomplex in de markt: ateliers van vzw Ercola blijven tot 11 juli - HLN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>“Evacuated due to very high CO values”: Mayor Els van Doesburg temporarily closes four shisha bars - HLN</t>
+          <t>AG Vespa puts Wolstraat complex on the market: workshops of non-profit organization Ercola will remain until July 11 - HLN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 16:39:31 GMT</t>
+          <t>Tue, 24 Feb 2026 12:28:35 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxNY1BNank2aWc2R0RzV3ZpdUw4eVFYZTBwS2xrSVRHbERueXlIY3lTSGs5MFNVTkZnUVJpWXhnWE9vSC1FU3BUWkFFT2NuSVlzcHo4S29NYXJESENlQ19uMEVFdU1jTERFQjVvV1VGM2lGREZyTHRDUDZYdkZ2amVtSUJ5dlMxNUVpcS1jZTNma3ZmRnFkQ3NrLVNOdVlJVGZBQ0x2SWc5bVVKVFdKcjlVZ1pWSV84YU53elQxM09JcE5yeF9Ub2tFeW1DRGFaeVlmalhpaEpRU04xbXlW?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdm9fSkhTTFNrSUNnRnRYOWowZm1zUERzY2Q1M2xYdmZSOVg4RnctSnZveVBlSGlWZ1ZvYnRram52cTVjNW9La0RSSFFjQ2V2UXV1OGlqdTNibG9CUWZQSnA3aWZJNnBFNm9GcEtQQzhDVTVUSHBodG9rQnctaF9vNVdHWW81RW5zbXlKanV0QVJPeHYtNm50RTUxM2k1UHh1cVJIMzlIcmZGdF9lY2h2RkdKZnVTQVY5d2NWdEdUTnc5dw?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46076.6941087963</v>
+        <v>46077.51984953704</v>
       </c>
     </row>
     <row r="22">
@@ -1590,22 +1590,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Expo met juwelen start eind deze maand in DIVA: “Toont hoe we kijken, waarderen en betekenis geven” - HLN</t>
+          <t>Asbest vrijgekomen bij afbraakwerken in Markgravewijk, werf stilgelegd en pv opgesteld tegen aannemer - HLN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Expo with jewelry starts at the end of this month in DIVA: “Shows how we look, appreciate and give meaning” - HLN</t>
+          <t>Asbestos released during demolition works in Markgravewijk, site shut down and report drawn up against contractor - HLN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 19:13:33 GMT</t>
+          <t>Tue, 24 Feb 2026 11:22:43 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNaEtQeEJXd3g1aGZjNlZLampULUliUnNwUWIwMnpEdFhMdGozRWVTTzYtREpYNDlQVFdseElRb1JRMFV2Z2pXMEV0YnM5dGJaUzc3NzljQWxJdXFQd19NeVNxS0tBeUlLcjdEcGlQeFdsV1BoWThXcHhxV3Y1bndubjVlQ2VJcXFUTGJzMzNodUpPb2IzdVNDWjQ5aFE1S3ZLWFFBZ2ZuSThvU3hjODh1Rmc1eEJOdElDSUpnYk1zWEhPWXJTRXZZbWJ4dmRLOFU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOYklwVUNDTmRCUm5ZbldoWlJjMloyQjd6TENkajRIZGN0NHprRTFZM0dPdFJEYTE0VmJ2UGVlZFdDd3cyMlJFUEVFRUM0UVF0MmphUXpWeE9NaV9zRmZwenliaDFycmNxMUZlQkJjanhoQ3o0MWF4WS0wenFhSXk0R19qSjdWdjdTM1dKYUxrbWZEWksyamNUa2J1SkhvM3ZwTGRycndPUlBNOUExVnBvZEdQbXpYX203UG84TkJnMjJ2YnAzUkwtYUp1cEtyV2tTbkxTRURB?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46076.80107638889</v>
+        <v>46077.4741087963</v>
       </c>
     </row>
     <row r="23">
@@ -1645,22 +1645,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Modeketen IKKS in België failliet verklaard, tientallen banen op de tocht in Brussel - HLN</t>
+          <t>Wat betekenen de plannen van Antwerpen voor de stadskas? Zo evolueert de schuld de komende zes jaar - HLN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Fashion chain IKKS declared bankrupt in Belgium, dozens of jobs at risk in Brussels - HLN</t>
+          <t>What do Antwerp's plans mean for the city coffers? This is how the debt will evolve over the next six years - HLN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 17:13:38 GMT</t>
+          <t>Tue, 24 Feb 2026 08:31:33 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQSWhmNWVoTlRWSHN4Q0RaVTBVT1FxYXRIa1RuVG15cjdsS0Rsa2VXNFpCWW1xU2tTZEFlRGVfUkYzM056YWJ2RVlFZ0FnN3lzYkNWUDlwd0h6ZVl1VHhORzVrU2JaOTYyVWllbEJsalYxeWZzZENPX3k1RS02YWFzWGpMeTBYTVdyVFNZcFJtWUdYQzBzcHpLaHowYkhnR0RwOVNmNFhFZGRZcXJ2ODVQYXJvTWtjTFdnb3huRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOam9oWTQ1czAwZ2pWSTRYY291YkJ0bU5qUXcxV29jZWwtVTRMY1lBaTd2SWE3NXg4TlB1OTd0RFJ2Y1pXdldkUTVBOUZsWnc0LUtuVm1raVp3TURMUEYzYkNLU1UwRm1yOXhWZlRxaHpnZmhLZlI5cTJZOU1NS2dhTlk1MVM4b3drRkhodmp2Ynd5dXRqYlpZVEtseVhxNG1tUV82OUhIcXJiTVVEWGtNTlB3SUtMM3pvVWNpT1JPNTd3cXZQTE5tb3lsLWxkYXdMem9j?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1684,38 +1684,38 @@
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46076.71780092592</v>
+        <v>46077.35524305556</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>VUB lanceert app ‘Moment’ om onveiligheidsgevoel in Brussel in kaart te brengen - HLN</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>VUB launches app 'Moment' to map feelings of insecurity in Brussels - HLN</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 11:38:38 GMT</t>
+          <t>Tue, 24 Feb 2026 13:30:36 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPQ1RuNGMzWE1TNWZhc0xaOHI0STZsOXJzWW5EMW5rV1FMdzFWR1FqSHdEU0hNYm9wbXBaZkQyUzlzMm56M2tFQzRhWTdlWnBOMEFhanJIWFVVRGhiakF6SnpYWFpfeDgxTlktMUxlZ1hpeUVlMFc2NkFCSWphZVljWHFPMktpTW9tbWJwZ01UQ1htR2x0dVdsSDFvV1JORXh5TGdIcjBGVFVsUjlkSENZZXJ6VnQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOTVkweWFzUUNLdXBoYTJPUGNWeFI3c01LV1pqRWU2eExiOUFwOUE2MlZGaFBySWVJUmdUWGotM1BDS1lydWgwcEpZR3FlbHpuZmpDVVkyYWhNQnBSTEpMS1VscG9HOE1pREFTUlM0VHF4UV9UUjRybFNmaHpWMDlvdE5kZUt5d2lRYW9ENmFkQVFoMnZyRzY3VllEYVkzWEU?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1735,42 +1735,42 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46076.48516203704</v>
+        <v>46077.56291666667</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bommelding bij Grote Synagoge in Brussel zorgt voor kort oponthoud - P-magazine</t>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Bomb threat at Great Synagogue in Brussels causes short delay - P-magazine</t>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 19:28:46 GMT</t>
+          <t>Tue, 24 Feb 2026 10:27:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNT3c3X25ZLW1HMjlMQ0VDZjZ1RFFvNjFRZ0tSdkJ1TEFlY3RWMnh0c2p0cmVCemVpSGdxU0ZNckVsbEVoUVFiT1BnTmc1bTdSSk56SFN5bU1PNHNFVFhka19saDJGV2wtb0lkNlhTMHZiTUowaEdvY1FQMjkzX3M4NFN1ZGJUT0NyZl94ZDkzaGtveVFYQ0lubXJ5RndqZXZBZWVB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQZnNnQURka1FpeVppWjNTcnRjSmpQVHA1d0VQRXN3MkR5aWtqTW02SVduMExEbUJQYWp0X3dPbzVySndQZTBuQzlSOGF5V25pSFFVN2RNemFsU2Z1SzNpTzBfUU5HenlhREJtNGUydFpuNG1US1JtbE83NENfZ1RlY0dhSDY0TnRjeWU1bk0xOXJmNndmNE1VQnBJdUQ4VloyeE03YmdXTXpIUkZ4ZmZ0UEg4d2ZqaGwtdEh4UTFITExSWDhsZXZCclY1NEhZSHF5SmV1TlgyLU9oZw?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1790,42 +1790,42 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46076.81164351852</v>
+        <v>46077.43541666667</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Lijnbus belandt in gracht bij Pervijze: geen gewonden - P-magazine</t>
+          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Lijnbus ends up in a canal near Pervijze: no injuries - P-magazine</t>
+          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 21:03:59 GMT</t>
+          <t>Tue, 24 Feb 2026 12:16:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNTHhwSmNYRHNtX1ZYal9wM04yYWhsQ3dYaGhPVzhiUGttV0lORnNzVkZNLWFiR3hxLXQ2QkhUMldCTmN2X3RYWlQ1V29ZR0lQeHc1NHlQT1BhNlZuMFRiU1hnQkpPQW1qeUl1aUhLelEweDRIS2l6TTRSeHhLdG8wRDRJblRGaWJ0bVk2V1NhZno?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOOTRkZE1mSU1wNTNCODJ6TEt2WWtuTF9yMUR4c1BOb3ptMExaU0ZJSUFyek96ZnpGaHRGRFd6aElmLU9WeXN4ZEZZazVsLTRUNDREamdwTGlMLXhsSHZoLTYta2gxNlBzUlhmRkdCaWZub0xBQl94VTdDZmZhU2s5b1R5TWRpd3BZV3JDS1NTRWRsUjZtemdVLTdaTmkzVDJEVzRCNA?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1845,42 +1845,42 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46076.8777662037</v>
+        <v>46077.51111111111</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Obus ontdekt in Kortrijk tijdens graafwerken - P-magazine</t>
+          <t>Vakantiehuis Fabiola in Maasmechelen voor kinderen met een beperking krijgt toch nog 1 jaar subsidies van Vlaanderen - VRT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Obus discovered in Kortrijk during excavation works - P-magazine</t>
+          <t>Holiday home Fabiola in Maasmechelen for children with disabilities will still receive subsidies from Flanders for 1 year - VRT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:53:08 GMT</t>
+          <t>Tue, 24 Feb 2026 07:52:45 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxOSUc3UDRUeWljYlBzM1hETXpDTXZTekJ2SERQQlRMNE83RW51b3h3ZnVOdlBreXBqdUdRTTNxVF9RanlfTmNMaGpPb0oxc2E5Q09WU0k1NlpHckVpU0ptcHZjYnloRUFnTzF5X1R5bTlDQzRheG1LSWFWYzd1MGh6YllmZmRLdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5OenpKUkhrQ1AxTlBhUlRETGdRSFpRaVJKOW9TelBUUXdpU01tdmEwZ0VFM2dvR05IaFViZkVWM0YxLVlwU2ZETUxJbld6c3NrTm1DU1Z1SWlzZG9PNWFyZEJMSEVyX2hCY1BIa1RGaHdtQi1OQU9pR3ozdw?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1904,38 +1904,38 @@
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46076.66189814815</v>
+        <v>46077.32829861111</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Israel faces an internal time bomb - www.israelhayom.com</t>
+          <t>Halen keurt aangepast meerjarenplan goed na budgetfout van 5,4 miljoen euro - VRT</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Israel faces an internal time bomb - www.israelhayom.com</t>
+          <t>Halen approves adjusted multi-year plan after budget error of 5.4 million euros - VRT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:42:43 GMT</t>
+          <t>Tue, 24 Feb 2026 09:32:52 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9UT1ZXandBRVdxaS1sbDVUNnVsVkhieWpMenNQLXlWZWxULWx0dUtUWHVDQUJpaWFzQUF0OFJBMHpRVXczTWxMVV9LWUhuSmUycFk0OVVqSWhQSVgzckVWcHBfQzhkcnYteC1VdGpiczd6cUMtZEFGeG93Zmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPOTItcThiT1hZQjVXaDA5TEI5RUlVdmt5N1UzR2hEelF2aVBXemRfcTdNbk9xUk5sY2NfWkpJdmIycHN5TThoaVNnVVpCWjgzYXExeFpZUk91bVhhdFhiZ0szcDNRT3Nua3RCSTVUa1BTSGRUdU42TXJ3NzVYSXdFMTRZMkwwUVpqaURzNXJMMVIwbk1rNzNSQVdVaUVvdHRVNGNWcURCUzA?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1955,42 +1955,42 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46076.44633101852</v>
+        <v>46077.39782407408</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hungary Blocks EU’s 20th Russia Sanctions as Oil Row Sparks Explosive Brussels Showdown - The Times of India</t>
+          <t>Environ 50 emplois menacés par la faillite de IKKS Belgique - RTBF</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Hungary Blocks EU’s 20th Russia Sanctions as Oil Row Sparks Explosive Brussels Showdown - The Times of India</t>
+          <t>Around 50 jobs threatened by the bankruptcy of IKKS Belgium - RTBF</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 17:55:34 GMT</t>
+          <t>Tue, 24 Feb 2026 09:35:30 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOTlJDdnZJcUhhajNFWEtvMldrV0NBVDlQbThJYXI2MVBCbktZNWQ4dEtWVEc1bW9KT0RkRTFGcENzamNHQXd2STBjMVRQc1N5S3pvdHJ1TGFjeTc0STZMZ0t4MFY5RGJuNnowc3ZFcDRaV1VZQkNqNWF1Q21hcEcyc1VqTi05SUl0eF9nQ1lYYlFoQXNuWjdsM3c5TnNUeGliX3dvLUdwSWk0YzY0eENTb3hhNDJFN3VBMHZpRlViQ0lrcVkzLUFXS1BGdzNyZkd2ZDBMdzdEU1JSOUxHV0ZsdGZHRU9LSGl3SHpRQnd4RW5YdS1Udlp5S19jVdIBgAJBVV95cUxQSno4aUl4RDNXXzh6UXNFdWJyMHh3SkJzbEd5NFI4ZE5PRFRHWE10ZllZXzNVam1LdXZWYnBaeU9PYkJvcks2VXRLeEZlRFR0VFp1N21XZVdiMGZXaGszMER3OERaR0hHbDREYndvQ0ROdmFEa0l1dkFxemVRNkJBOGtNVFNWQjJpeW5DWjFneTBBMDlQbjlOVXRBanNybjNMR2ZZQkRyM1lRUDNHV0YtT3pYbVAwbTNuX1BBckZRa3RfeHd1SHhlOVZheldMTzh4eEZuWkZWa2VTWXNfaDV0TWx5a2lqcm4zZmhDaFpEQ09PMXhlYnRVRDJqRXNQdERG?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxQZE84MHM2aGc2b0JUc0dFQ0NzbXRhQTBKbDNILXRpN3o3Q1VxMmZnXzRIVXQxMlFUWjJ5U1ZWWjZFeFNCTEZ4bmlYN2VJOWpNLTRoRFREMlpITHhSTWFsN01STkN1THFxZmd3cEFPeFlSWVQyNm85Z0pVOW1LM2xnS29zeVJyUklsNGpDMDdJNDIxZENMbldhWXE1SHk?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2010,42 +2010,42 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46076.7469212963</v>
+        <v>46077.39965277778</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Germany’s ruling CDU wants to stop Gaza payments via UNRWA - Brussels Signal</t>
+          <t>Courtois va investir en Belgique : deux clubs mentionnés - FootNews.BE</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Germany’s ruling CDU wants to stop Gaza payments via UNRWA - Brussels Signal</t>
+          <t>Courtois will invest in Belgium: two clubs mentioned - FootNews.BE</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 13:37:46 GMT</t>
+          <t>Tue, 24 Feb 2026 12:39:21 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxONTJpaS1CY1VFdHlVY0NtVzhNdTJmMG4wOHdydnY5MlM3bHVTZ2RRcVlzZ0dmX3JxdVEzNHFmM1VjWXZQOVlHVzdKU1I4TUMzeDJfZTAyNTJOVDgwcElQXzJfZzI0UFVZWGs3ZFdxMmlmNlF0N0pGa0pSY1hLWEw3WXFoVGx1WXFIaFZIeHM5VnVIVDNsMlFF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNTlJDdTgzUm84dnhidVNwNUtTZGJqbWZZOVJmSHBzU1QyYmk4QV9ZanJ5TG12cXFKVDhVSHplR2dudWVsb3RlWjZUd0FpVmhHZFJfQzFnTlpvMnJwX2Y1Q3RLY1lzTlNWQ0JNSXAyalBMNm9YazVTenlGUXdranlMbjlwWUpSSlppbjF6SXU1aGJJd185?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2065,42 +2065,42 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46076.56789351852</v>
+        <v>46077.52732638889</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EU adds eight Russian officials to human rights sanctions list - The Straits Times</t>
+          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>EU adds eight Russian officials to human rights sanctions list - The Straits Times</t>
+          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:16:00 GMT</t>
+          <t>Tue, 24 Feb 2026 13:32:37 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQTU1vZDZ1QWVmS3RBUktpb3I4a3pkN1FFaGtkRkl3U0FKOUVQUF9Ec0VmVld3ZHJXQ3B6aGpZS3dxU3hzdms4Y2w5cGZWZGw5UlZmenVlRl9ZdkZidEd2OFUtRll3UlFIbXAzTGpUeVNhZUZlVUlBbUp2azdxYnROMDRFYmRYOFhVLTNMd3pWQXhmaUg2Qk9LNDdxd3BxM3BqelAtSVctWXNPVzRETmZySFZLcjdDcEpDR3BOTnJ4X1l1dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNRHZ4dm0tREV0cjFucHowcUNrWGlJTVljdlFXcjNtdFg0OUh4a2hWb25ucnlzMkNMdThqU25BNm1yaHhBRk8zTDRwcHdHRHZFRUNBSVlHcXZjdDJFQU95SEVCM20wQm1YNmFzczRjdzE5UmZUY2NpWldzMWRfdXpSVmo4ZlpsVHdNOWo1aVFGcVRBc0I5RjVyYkRGeXZmVTBGZkFvNy0xZFVxa2JNZ0RzeGt2dHJCZTZHUTU1RXRZbzNpQQ?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2115,47 +2115,47 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46076.63611111111</v>
+        <v>46077.56431712963</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Nadezhda Neynski and Mark Rutte discussed the changing security environment and transatlantic relations - fakti.bg</t>
+          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Nadezhda Neynski and Mark Rutte discussed the changing security environment and transatlantic relations - fakti.bg</t>
+          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 02:44:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:08:23 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPN1ZLQW9wZnR3UzM4bzVkNWZhbW1NS2g3WHRucjQ5RC1YZHNncWhzZ05VUWdOLWNSRnJhZ3FaMTlWVzRxLUhhTnBMYlh2VWF3V3dtSDBfaDNMdkZmN3JaaTdQUHhmQ0MwYVpLQmtTeVJzNjUwWEJVVUNpRmJsbnNzQjB2dFFUVktmREF2UEpSRm1XYmlPaWd5X3YxNGRVeWdoQUZlOEdjZmZMc09XaG9KMFN1ZEwxN1I2RHR3Y3JnMFk0aHYtaE9vYlFIMkxIU2NFeE9FVDNDU2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPNExOajRSMzJtQk9kOENCeXlHM25OUm5vVWQyUkszamgzQjVOMm92anAtdHN2QXhFLUVMLUptNVJ0YzV5dFJWTE5OeVNCMFVobnlyelUzeFBadlNFV3hCRVI0Y3pUTExVYU9TNFdwVUNsaXhyQjc2QW5MZlh3Rk9rejhZUDhEU1h3LUVQWHhBWHNHWG80NUltV2hxd1YwWmhRVVZyOHotOUdQeEp6UlVQYi1iVDZWcHFOanBzWWFB?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2170,47 +2170,47 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46077.11388888889</v>
+        <v>46077.5891550926</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Village Maasmechelen (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen Village" OR "Maasmechelen") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Fire breaks out after explosion at Baku flower shop - Latest news from Azerbaijan</t>
+          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Fire breaks out after explosion at Baku flower shop - Latest news from Azerbaijan</t>
+          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:27:55 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:27 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE1GUmdfSEw4Y0xPQnNwazNxWEY0cm56RjZIOWZ0R0lFVVZtanZuRXBOWUNZUWVURWdGaE9peWlud0NwZFYxbUhzTDZLcGxsM3pEWm9WM2ttbm9uczJkVzVEdTNFNm83NXFSQW1LSTBxeF9YLVRYUVZodmN3WFQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUW54aFlQc196RnJXM0FfVWU5a2JSN2w2MXdiZVg0Z2U2aXdKZENsNThtVWVvQjg3U0FwUUQ2Qk5SZF9rSnVqQWxrc1VzOUNzcVRfbWVXNWFCUW80ckl3MHJlaTZvUElidlBqZWNlSm85a1otTXNBMkpYTlQ1YzJBcDVNNkY1a2o2OUJtNG1HYnItU2RodXRXb1pXMVFOTkF6ejk3cEY4ZTdRbTA?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2225,47 +2225,47 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46076.43605324074</v>
+        <v>46077.5440625</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>La Grande Synagogue de Bruxelles visée par une fausse alerte à la bombe - BruxellesToday</t>
+          <t>Wertheim Village: Polizei stoppt mutmaßlichen Seriendieb - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>The Great Synagogue of Brussels targeted by a false bomb threat - BruxellesToday</t>
+          <t>Wertheim Village: Police stop suspected serial thief - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 18:51:00 GMT</t>
+          <t>Tue, 24 Feb 2026 09:34:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE5nRUxDNnpMb3JkTzgwMHV5YmVnMkY0M3JZWGIxMjhvNFBlTnQyXzBmdHFSU2x3LU5DTWw1Tm5sdjdSRDFSWVd5dmkyVWVOQzVMYkZwUWV5X3BhSmxXUTI1Qkp6aF9Wb2lnUHNQZjRqcjZ4MWFKWHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNempGdjdfTkxudlBkZnlNYlNUS3h0MEluS3JYU2tOVW9zamM4QUdCODMyNTAwc0ZDY0NCYXpReG9wOTVtOUY2eW9rWmhxT0RHaUdubGNoWVN3SjBCaE8tSlBpSTlneF9aQnNMdHR0VDI3Wjk4el80OU91akJGYWV4aVVuM01SejN5NC1rQlg0WElRd2VJbXVhZEtjZEVwdDAtYlZnSFFjazhjOExOcGszYmt1X0hEUlZyQjl3aTRWXzZxWHJ1NXlJ?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46076.78541666667</v>
+        <v>46077.39861111111</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Trafic de stupéfiants à Montignies-sur-Sambre: Un individu arrêté - Télésambre</t>
+          <t>Unfallfluchten in Aschaffenburg und Kleinostheim | Foto: Dirk Ceelen - main-echo.de</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Drug trafficking in Montignies-sur-Sambre: An individual arrested - Télésambre</t>
+          <t>Accident escapes in Aschaffenburg and Kleinostheim | Photo: Dirk Ceelen - main-echo.de</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:16:10 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:01 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNSXp2bmZ5TlN5YkZZLTBhalF5SmRHRGd4Mk50dWZZdW82WngwNXVXTDNSUXdfdWZET2t1dlNCcjZLTVdOY01DYTBQaVMzY3draDBabE13cHlYZ0xJeGNwYlhGdkNLU0JkMGZvSW5xZGZxX0FWLWtFRmF6N0R0TFlhdFVnZXNPczVNUG9zT0ZYMUl6TlFUQ09SbHFPeUZ2SFk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQMW02WVZqN19mTERhVXdiT194SUtPU2ZxVTJ3dGNKd2ZLQzVmM2lxb3lTdWpHVjBqOVlFTFVOYXE0d0czbUpZQzFFU19OT294MmdqVlU3d2M1QzFWUndPbm02SVBvakFlc0tVSnl6YXJjOUNaN2FvNUYwX1pOOGJ3aVJoZjlPOU9DWnFRZlBlZG5uNXN4N3ZvWnpYN21VX2M1Skppd2c4Zw?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46076.63622685185</v>
+        <v>46077.54376157407</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PostNL va installer des distributeurs automatiques de colis en Belgique - 7sur7.be</t>
+          <t>Marktheidenfeld: Polizei kontrolliert erfolgreich - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>PostNL to install parcel vending machines in Belgium - 7sur7.be</t>
+          <t>Marktheidenfeld: Police check successfully - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 09:39:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:09:08 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQUXVDZWdDN1M5TnNNUXptdEQ4UWFzdnRCcmVOZ1U3QnpaYzZkTGpybXlaTHRKV2s4eUF2YnNTbEU1MjIta0YwSTdaSXcyRHA5M0ZuU3lMY3FsU19VVWdwNGpwVjdYQjBPYzAwRXJNY191UU9oSmNsQ3k3N3ZRRjFKN2pEcjhHTDNhdzllYkVFYXhHQ3hoMjhvNmdBTWxnY0M2emk1b09QQUxSZk5ITGJsRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNM0F0V01ZMjFGbzFpQ0FldUNxRnI4UkplZ2daMUlzTXNvWGM2WnlUZGprenhxMXBfSkRrLTFkWUU2c2VFODdxRTU1bWF2bVNZeW9zWWVPaEtGU0ZfdUdGbVBKOGt3dEdmaUszMTdlZnFuNUV6b0JWUEFtVjBlTmdFQXh5SXhuZTN2eVVzelU2Z29RUU9wNGw2Z1Vn?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46076.40208333333</v>
+        <v>46077.58967592593</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Elisabeth Degryse répond aux accusations de harcèlement: “Ces cris et jets de signataires ne figurent pas dans la plainte” - 7sur7.be</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Elisabeth Degryse responds to accusations of harassment: “These cries and throwing of signatories do not appear in the complaint” - 7sur7.be</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 14:09:00 GMT</t>
+          <t>Tue, 24 Feb 2026 12:52:25 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNSWJoWVlHOGJFNi03b2w5Y1p6UmxvSndnOF9pTHBZOVBMZnNoN2RweXBoN0hKamlQSFZFSklRNUY3NGp4aktrUDExbjBObDQ5ZkoyeGliZTcyMC1iZTJYTE05eEZMbUVmb2lEWmpxb3RhRlo5cVRHbjJtTVRkR2JBeDRxc29veThvdWRDaUZjcER5WEM3QTZyNWZHanZjbjBVb244bC1KUmNMU1VYVXVVNndRU1ZBUC1xdFJhTlowa3ZoeTBjU0FaemVVdzNoelhaektaUTZrSVZ2QmNzRHNXN0o2LUwwT0xQY1FUbnJEN1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46076.58958333333</v>
+        <v>46077.53640046297</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Marc Uyttendaele ne donnera plus cours à l’ULB après un “geste inapproprié” envers une stagiaire - 7sur7.be</t>
+          <t>Streit bei Auto-Kauf in Aschaffenburg: Männer gehen aufeinander los | Foto: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Marc Uyttendaele will no longer teach at ULB after an “inappropriate gesture” towards a trainee - 7sur7.be</t>
+          <t>Dispute when buying a car in Aschaffenburg: Men attack each other | Photo: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:32:00 GMT</t>
+          <t>Tue, 24 Feb 2026 12:34:53 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQZzFuWjJVUFozaFJYUWEydER4aXlOX1ZILTZnNDFoY1VXaGY5UExQQktYcDlBa3hjZVNaZHJFYVRTWFJxeTM3dnJqTWlocGhIOHlBUlBzOW14emRnRlZ0a2JldXZQckVBcVgyajRIY0xEVGQ3cy1uQkhaQ3pNNlhublRzNUJwaXd1Z3BHN1ZseXhYbjNtTWFYbFFXdU5rR09OZTBLd0JxLWU0UGhuWFM4ZVpRcExHanNNQ2FQQ1ZYNkNJQkFEcVhiUmRaUkg2Z00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQNXA4Vkl0TlZ2Ui1SOTgxNWVUcF8xdXdtOUJsODFOalIybVlxTkU3SURZVHc5aTFsdHNHMGR1SXNvNWZGdlgyT0dzbHZmbmtQMklfbERteC1yMWw4WFVvUzhGSWQyb1J6X3hPcmRBVkFfVkxMbEtkWDMtbGZWckV4LTZVLXBvUUk5ZEFNMlJ3SE80TXZ0V2JEakttUjJkWmtoX3djX01wY2dUbDhoLXQtRm1qVXpwZzlfM2UxWXRTYng?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46076.43888888889</v>
+        <v>46077.52422453704</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Opnieuw laadkabels gestolen, nu in Maasmechelen en Lanaken - VRT</t>
+          <t>Kleiderdieb in Untersuchungshaft - NOKZEIT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Charging cables stolen again, now in Maasmechelen and Lanaken - VRT</t>
+          <t>Clothes thief in custody - NOKZEIT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 16:16:31 GMT</t>
+          <t>Tue, 24 Feb 2026 08:58:15 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQLXpEcnVvUUFXZTVvb0o3cEl0bG8taUR5R3ZmT1RybVhhNDBXeHFaNHZ3TWlabXpySzljU3JiTTlPc09uaElITUlISDhBTERBcW10ZEdvV3otMG4xZm50R1IzOEpzX05sVzVMb3VwMGNyenk0MWNIYlY3andhSWpNdWQ4d3NNTlowbGZDV0FXYTNLRHc4RjdaczdLaTJiRG8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBKUUNfaWVwNkcxMmtpalVDTWxaMGNYQl8zZEVkWlFUMVk0UjFYa0Y0OEpFMERfaGMtSUI1dlU4cHVxLUJJMWxnV3FMcFdnNnQzc2s4RVVnamxfLXRxRjR3a3VYNkd0Q2pTcGVPb0lpTFE2ZE9KZUE?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46076.67813657408</v>
+        <v>46077.37378472222</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Vakantiehuis Fabiola in Maasmechelen voor kinderen met een beperking krijgt toch nog 1 jaar subsidies van Vlaanderen - VRT</t>
+          <t>Herrmann begrüßt deutliches Personalplus für die Bayerische Polizei - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Holiday home Fabiola in Maasmechelen for children with disabilities will still receive subsidies from Flanders for 1 year - VRT</t>
+          <t>Herrmann welcomes a significant increase in personnel for the Bavarian Police - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 07:52:45 GMT</t>
+          <t>Tue, 24 Feb 2026 11:06:28 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5OenpKUkhrQ1AxTlBhUlRETGdRSFpRaVJKOW9TelBUUXdpU01tdmEwZ0VFM2dvR05IaFViZkVWM0YxLVlwU2ZETUxJbld6c3NrTm1DU1Z1SWlzZG9PNWFyZEJMSEVyX2hCY1BIa1RGaHdtQi1OQU9pR3ozdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNU0FPOVFwS1pZal9xUnlUNDVjT0wzY2xwRG5TUmdob3JERkNFdld6ZHdVTHJBdnAxOGl6VW5jeTNxMmxtWjZfSVdkczVTaVdTNFBIaEN0VzBTbUkzRHk0QlBJSEU0bEk0aVJIT0lsdnV6VE91WUZDMGRybGhMSmVMWEM1R2hId1pvN3E2Z3BOT2xYZk5vMm03Vjk3dHNfV3ZhS05OM3RqX3J0b25uUTRadzZLaDJXWk5KbzdmLTZ0OA?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46077.32829861111</v>
+        <v>46077.46282407407</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Filipijnse oud-president Rodrigo Duterte staat terecht voor Internationaal Strafhof - MSN</t>
+          <t>Unfallflucht an Rastanlage Spessart: Schaden an Kleintransporter | Foto: Stephan Jansen (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Former Philippine President Rodrigo Duterte is on trial before the International Criminal Court - MSN</t>
+          <t>Accident escape at Spessart rest area: damage to small van | Photo: Stephan Jansen (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 23:49:19 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:26 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxQSlN1U2R4azRIVFo0b0lNbUhzbjBDWFJpemk0eFIxcDN0NF81bXgxS2U0dDZUb1ExdThSVXhJd1hyQmZvVGtYNHpNVTNfTXR3WEprc1N6cUk0WGZkeXVpVVRsR0FwS0RyLUtXV2w3TWVCU1hidGJFRXN2X0hNcG1LSUl5SmNodUNib2M1NHRyWC1kTzNBNGxhR0hDcUNXcmlaM0t6ZlNhVXphcFFOajY4RDlpSjlBN3VHOURfYUhVYnJUNzdNbFRsT2ptZXdQeWdCX08zeDFDWkR6LUtZWVljSlRzaS1HSnlZdjFlbDBhdll6Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOQkJUQUtFSW5nMU05Unk5Vmx5ZkJXem1XV2JHVEFKSjBISGN6OU5wZElaUjlWZ0pZMGc0MHlJcEJqcDRSNy1od1dCY0dQdUZVX1VWdHJwSk9aMUljaXoxLWxmbWdZSnhMU0EtcE9DXzlRQVEyNVlpd1R5NnVvSElCVVF5TjB2VHZpLVpOUTJvYkdTVHlSTVhudzI4YmI0YnUycUpFLWtFMndDby04OU1aRWVZY2MwQmVKTE44?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46076.99258101852</v>
+        <v>46077.54405092593</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>220 oproepen in één weekend voor Politiezone - De Internetgazet</t>
+          <t>Helmstadt: Nach Einbruch in Einfamilienhaus – Zeugen gesucht - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>220 calls in one weekend for Police Zone - De Internetgazet</t>
+          <t>Helmstadt: Witnesses wanted after a break-in in a single-family home - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 09:41:10 GMT</t>
+          <t>Tue, 24 Feb 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNYTBpdElMU1JKTjk3LXFvdXg0aG1LWVd4S1RZaEtXS3FfdzdCU0ZSQnE2NWJjX3JwU3VVNnlPRU9SN1VqTUtqYm9ON0FGVUY4STdEaFdWUno1WGxfTzRNc21wX3JkdUZ4c2p5LWZBVjhWcnRpXzVLekJaLXhyQnItY0NhcVo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOeHEydHhfR29sSVFqWENkVEU5ekVMTnRTcmFoZXhIeFJNVTMzSGN5dzNjZjVtZVk0TnhtSjRNUmRTRC1OdndqNVV1MDJadHZUdlU5UjBtTVV1b2k0TC0wX25XXzdGQnk4VVR5Rno1akhMM19aOGRNZURrcmJ4cEh2Z05UVFpqQURvalNLcU8zcWZ4RG1PdWc?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46076.40358796297</v>
+        <v>46077.58333333334</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Beveren a fêté sa montée sur la pelouse de Patro : la réaction de Stijn Stijnen a surpris tout le monde - Walfoot.be</t>
+          <t>Würzburg: Messerattacke auf Zeugen Jehovas - Idea.de</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Beveren celebrated his rise on the Patro pitch: Stijn Stijnen's reaction surprised everyone - Walfoot.be</t>
+          <t>Würzburg: Knife attack on Jehovah's Witnesses - Idea.de</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 12:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:00:03 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOMFZUdHIwV2NXVUVCZ2JjRVJ0d2Q2Q2ZOWUw1OFB5ZV9GNkt6eVNSS1h6RjhDbGtrNFg3eUhOU2NROWlxMkZ2ZVVxbTBaQ1dPTXZLYmMwcFVRaHNLOEdPVmZFYkptVWJxWDZiTGRlZjVPaHJTWGJ2UnhLaklhcW1TenlRd0FTUGZRZEtCdUoxUkFHNHpZamVYMGFSNFVyaDI2RUItaE5KeVN1dEZfQTRJNkdZUXp1TS1lRFNDUXVDZjhVZmRiTWsyVnlreUoyekVSUG5wWHVheVbSAd4BQVVfeXFMT2R1OWxYLVlQVHkxTkJOOFVTdVV4ZHA2Q2RiQXRpblVQdGV2Nlh2Q2xBMnBqSWxCaW43Y2ZKcTdIbWRDdEY2ZHVlN2NhRFNsaThCX0hpMDhsaXQ2U2lIZ1lWUGNvRTNndkJvWUUteXg1WWFIdnRXbGFhVC02aVc1RmtLdHU2dVd3RDliSHpndEg0ZzJyQXhacEl3LU05Mk5WWjZZUUdKRDVuS3IzN3NzdFQwX3VnbmctMV9QQWxtOElPT2Y1bFJXSFdKVTdvb3BibXFXQ25lLThqVW1CX0p3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE55UThGQWVSVnBMUGM3RFpMeDJJbjc2Zi00aVhuV1lVeW9rZmw0WXdNdmZFY0REWGpQZUtUelROVXl5RE9KMkhJNlRoNUNvN09sS3Z3aTVjMWp3N0ZWc05CZmdGeWVPUzR3VXhBMFNkTnVWWWNTOFlwcnJ3?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46076.5</v>
+        <v>46077.58336805556</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SA Winger Fires Beveren To Promotion In Belgium - iDiski Times</t>
+          <t>Erfolgreicher Callcenterbetrug: Falscher Polizist holt Wertgegenstände ab, Kripo ermittelt - Mainfranken News</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>SA Winger Fires Beveren To Promotion In Belgium - iDiski Times</t>
+          <t>Successful call center fraud: Fake police officer picks up valuables, police investigate - Mainfranken News</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 10:35:28 GMT</t>
+          <t>Tue, 24 Feb 2026 14:06:37 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPS3ktRHpRekdhell6bG9ZVUdNeXhoQ2loT2RYMHl6eWNPNVFqd1p5Yk1wbGtPZGpzeGtkN0J3MGwtWVZhUm92NUFHSTk1bzR5WTlOTDgtbkZKWkpNbmgyUzFPS2ZJQXF4UnhRaGlwRW9jZldLNWdvU0FuOVdLVXMwMkJRaHlaVGdhUGZUY0YzX2V2Qkdrb0s5bHFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNRkZoQVNGWmlQVjB6c210V3RQRjYzeWxmU1RkQmJURFJhajlmQkVvRjI4V3d4U3AyQm1GajFjYUlteHcyYV9LcTQ3Z3ZMdklUbm9DemlqMkdvRnlTeHJJd1AzejlhMjlFOGJGYklWQlZ6cHRYekZYNkttNUFReWlieW5WVGY0aTRuVWRVZUZIRlpSZ1B5clJnMEh5VWtqVXZXbHZ3SnN5T0ZvSEJVa3h5X3hGdmxyV2pfSDVCejJ3Smd0NE9s?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,21 +2825,21 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46076.4412962963</v>
+        <v>46077.58792824074</v>
       </c>
     </row>
     <row r="45">
@@ -2855,22 +2855,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Würzburg: Nach Angriff am Hauptbahnhof – Polizei sucht Zeugen - Radio Gong Würzburg</t>
+          <t>Frammersbach: Falsche Spendensammler - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Würzburg: After the attack at the main train station – police are looking for witnesses - Radio Gong Würzburg</t>
+          <t>Frammersbach: Fake fundraisers - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 14:30:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:06:56 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNUk1fcXRlQzR0TUx0eFZ4Rk1TMTBnQ2Z5RjJjeU02bGVXczhsQ0lfblVYOGJWRXRueExfZThlbTM2Smo3T25UQWs1TTNrZVRySUl6cl92NjJ1cktxVzltTTZmZGtJWXJVSWNWSmlDZVpYZFZiS1Q1WVgzRXFZbVBOT3lOUHlIbS1rMTBjQzNFNFhQdXFwLUNTZA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQmphdE5lMlFNZTFQYTdWTzBNU1pHMUc2YWlxZXFPc1BZWlBWZ2lnME9Xa29OcmFCeE5XeTlZS21YRTVSeGU1OEUtOHdCZTNwZE1CWHoyQkl1VlZfcDJQQmphOGh6V1J5YWs3cmhLSmU5Z2tFbGJuWGJBQlZxbEJPYXo4T2stUlVW?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2894,7 +2894,7 @@
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46076.60416666666</v>
+        <v>46077.58814814815</v>
       </c>
     </row>
     <row r="46">
@@ -2910,22 +2910,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Reichenberg: Frontalzusammenstoß auf der B19 bei Würzburg: Zwei Autofahrerinnen schwer verletzt - Main-Post</t>
+          <t>Obernburg: Unfallflucht schnell geklärt - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Reichenberg: Head-on collision on the B19 near Würzburg: Two drivers seriously injured - Main-Post</t>
+          <t>Obernburg: Escape accident quickly resolved - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 20:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:07:44 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxON0VPNERZb21RaF8xWTQtUzVObjNuUUw5LXpNbEVyOGtLQ3I2eWc2STlOUEd2OTU3UUVMNlVhNlRvTGFSQmxvb181ZkxJNzFtQXI5NGoxZHJPZ0gtbUVBd0l6Wm96UjREZ3JnV3dfNjYyQklGWVlSUTVLRjZrRE5mU3E5dVFaNU5WdE0yblAxWHIzR1hJdU1JVFEyZnEyMFVneGhHTl9UVF8zYnZPTVM2bTQtT3l1RUg4WFc2WHhVekMxVTZCRmo4eXA5THhKRzRibTE1UkpFaGJqYW1qaXhZZ3VJcFpVYUVrNGh6Qkc2NDQyS19FMFItR2E4V3k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQWDdoMzlzRi04dVVnRzU4ZmFHbElQdTh1SFVrZWFJakZUYUVRQlk4MExVam5lb3U3XzFWVy1keWczZzJ1a3pBai1GR0E4bDRYR3JiMWY0UVVtb0ZDaFdaR3NCa1ItcjRSajg1Ny1kOFJFaFI4VWVnd0pBR1FfMndCNFV5SFFIQVgtVml3ZFUwc3kwX0hvUzRURDNwVDdkVHV3czBQVTlR?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2949,7 +2949,7 @@
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46076.83333333334</v>
+        <v>46077.5887037037</v>
       </c>
     </row>
     <row r="47">
@@ -2965,22 +2965,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Schüsse in Kahl: Polizei nimmt 19-Jährigen fest | Foto: Oliver Killig (dpa-Zentralbild) - main-echo.de</t>
+          <t>Blitzer in Aschaffenburg aktuell am Dienstag: Hier nimmt die Polizei am 24.02.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Shots in Kahl: Police arrest 19-year-old | Photo: Oliver Killig (dpa-Zentralbild) - main-echo.de</t>
+          <t>Speed ​​cameras in Aschaffenburg currently on Tuesday: Here the police are targeting speeders on February 24th, 2026 - News.de</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 11:01:41 GMT</t>
+          <t>Tue, 24 Feb 2026 09:18:00 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOTjJHN2xRN1Y3emR3c2pkRG9uMjJIYjhKZnY2d19ObFJuS1dHRVJ1UFc5aHdRWFpVUS1oYUpjdE5mWUhZRmF4cG5iVzN3R2pzWGxRekJiS0J4WWZCcnF1YXpzX0l1LVdRTjIzcTZQSzExS25kRXA3S2kzN2ZobkxRTkU2ZTlHQjlrcW5FRVZHSFRfYXFIRERVQWJLVkNybXlSQUJXVnFPUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPTVBpWlNVVWhJQTJIZ0xMUkVmR2dOWmtjZkxfaDJIcDJXUHo1Z2d0T0RGOVJXdmVmRV9PQ0p1ZUg2dlVaYXhqVERySGpCM00zeGlxNnZWMjZfQzRPZzhHTFRrODVTNUlLcFRGTnpQQzJFa3pZaDNjQzRaOGpMWno3Z3ZZaEpma0xtbDVzU3I5TV9EaGVnbmpHdzlWRUxmY3NMeFg3RnhxWDRfZElOeXVDeXVXZnpaaXNwTjNWc1IyaXNTQmZMbVlZa09qVURBYTJsQmlUdDZXUEVEeDFXZHNPZE9TQmtiSmk2M3puY9IB8gFBVV95cUxOeHd5dHFsS0VxRHViWnMwbzlwYjl2VFhheTA4a0xFTjNCcWM0S0VQR1ZkRms1eVFWdzVrcUp0RFhhSkZqRE1fUmFVd3VQVVZWVkNrNHE5Y2g5U20yMlNKb0h0T0MwTVRsRkxoa1pvdU52MzFNUE9ac0FBdjRQTE5Xbko3cjNGaTkwX190N2wxUjljcGRsLTJJZEZfM2h1aHVFcTBkYUJLaExSMm9zUXQwRE5hd00wVVc4YVMyQ0ZfQWlJU3B5Y09obzh0bHFBUGpsWmw4VC1mUFd3dmVxUS14b09IRGhxeEhzLXQwV1MzdnVZZw?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3004,7 +3004,7 @@
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46076.45950231481</v>
+        <v>46077.3875</v>
       </c>
     </row>
     <row r="48">
@@ -3020,22 +3020,22 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Corona-Zahlen im Landkreis Aschaffenburg aktuell: Die Coronavirus-News aus der Region - News.de</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Current Corona numbers in the Aschaffenburg district: The coronavirus news from the region - News.de</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 05:25:22 GMT</t>
+          <t>Tue, 24 Feb 2026 10:39:00 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxQaUEzVnI1RndRNXNjVEEzZ1phUmhtempTcElXZld6R1lVQTZuYmFKQWdYN25qclF5TE54T0UzTU9iWnZSc0RydTlpMGRjZ3ZyM1hWZDh2SlBHLXJPTTN2T0d1SDJkT1RSU1FpckR2bGQ3MHlTU2MzWU1WdUVtTnRvdzN5LTJSRVJ1Q1dqMFlOS2lia1E2bWNxZ2RUMzhzS3Z3Q1ExcHlyYUxydTFkU0lIZ2hIMlZNRDZXZmlOREFzVUs2YmxrN0lOZ0FDWGxCZzIxY1djYl9RLUJGeExvOG9VZ0gyTF9WODdVdVp5LS1WOTZRNkNlQkwxZWdBZG01VmPSAYQCQVVfeXFMTUphRTNneGpNMmxrczR4aGUtLS1PT0swYXJ4T2RWOWVvZU5XNG4xckFrSm8wT2RSVUNCSG5GQlJCcm9vX1p0THJITHAtN0xldjhacjR2VXFfUWVCdXg5SjFlSEpTN2lQLVE5M1AzcjhVdEVTa3ROV0tFbmNhWlVmcXBjUUw5ZzFfZkE1amdCdFZxRkd2c2x3dk1DbXRYR1FBWW9sY1g5ZjhPNXE5WXF0U204Z3RHWlVGVDlKdG1YeVAtYXB6ZGhoZ3pXMEp0cTNyS0o2dXhGRDFDV2JCYWlWbDFfXzZVVmJ1RjRKV09aZzNqZ3pETERxU2cxUUhYM0dNZ0xlSV8?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3059,38 +3059,38 @@
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46077.22594907408</v>
+        <v>46077.44375</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Demo-Termine heute, 24.02.2026: Hier gibt's am Dienstag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Demo dates today, February 24th, 2026: Here on Tuesday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 06:04:43 GMT</t>
+          <t>Tue, 24 Feb 2026 13:17:11 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPTGdUUkg2a1JYTDFRNDFrZTJfejZYeTZZc1dOeC1sYkNIOVQ4eXFXU2t2X1BXaTJsaHlsSmJXcUM1MWlpVmdXZXpBZ3ZiOUpPd2NhOG1OSUNfZWRhR1o0dEVWX2hZT0pCVk1WMmV6T1BmaFI3V0lEYjdrTUlPMUZvM1hMdHd1UWdnak13VFlMa1FydXF0cUZWd2ZTRjJWaTBCNmMyelAtdlI1Z3kyNndzZ0NSRjNkeTYwZWludW9WNVVPWThLbWw2ZXRpU2ZMdUxXcTZZOUllbG42OGp1dDBpbXlWeGE2X0xOakFnYnpxbXoyWE1HVks5bDZoVUs2QTMzbXpTWVh4a9IBjAJBVV95cUxNVlA5c1FOUjBhdmxMUWhDQk8xbDhPTFlENjAtM0hCS2pmX0M1VUZxcC1WblZQTWdhRjlhT2NWbUZWSG5NZWpLby1sYlJMTnA0X2JFeWNNcVFvNHpqQlJBcmY2VHc1QTYtc2xnTEVFRlFGTXRnZDFRNktpTFFVTG1vRmhtSGtvdTRDX0ktZm9QanY3SzBLTFo3enRWc3hSODJIejdMcGFqdGVpU3owaF92NmdKNkd4ek9OMFlfcE5pNldoNExVOGU5VjIxUDB3alBORWFRM0pRWXJVT0JlSkR3TmJOaTZhOWxQUncybTNxZGFpN2NGRWdCU0N5dE81blBrSUxjbld6cHBRc25X?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOYl8yTkRYaUVVaUU4eE4wZk1aSTVxbkNEVzg5MHF5aTI1bGZnZkxweHgzM3MwUU9BekdUVVNlV3pPV0J4NkJuM0ptYzlsa1JxNUNCZjNqdmdldHkzRnNMSnpidGhTb2h3LUYwR3VXU3BnX1Z4ZDY0dkJRd3JiMUpYT0FZbjVyNzJf?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3100,52 +3100,52 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46077.25327546296</v>
+        <v>46077.55359953704</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Jon Wertheim suggests the reason why Serena Williams may return to the WTA Tour - Tennishead</t>
+          <t>Sexueller Übergriff am Bahnhof: Kripo Ingolstadt sucht Zeugen - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Jon Wertheim suggests the reason why Serena Williams may return to the WTA Tour - Tennishead</t>
+          <t>Sexual assault at the train station: Ingolstadt police are looking for witnesses - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 22:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:34:12 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNdXRXQ1JpcjVLX3Vkd3RzbW5VMWR1SW1qQ1hwc0RfUi0xZG5nQktYRXhYcEstZ3BSb1pMVU8yeklCS3dycGdhMW14WVZKVUdyOUtjN2YwMllOQ3JxOGo0VVhCX1VCM3AyLUFQVHMwZzZDbXNKb0prSkJITVlJbm1ka0ZDY2g5X3hJQ2llel9EM01mdjRaYklTazA5dHA0WGU0LUdmeHVn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOYVpQc2ZubWFubEFJeVhURXhHUWlPa24td1QzXzVWS0dmdEJCN0VVRGNfNjEyZjNuTEZyN3IwWWo0cFQ0SjRYQUs2VXBJWGUwMXY2ZG9wc2V3UmM2WW5ZaUZkVTNWXy1mcVpNcXd2NE5SRklKSDh3aklIcUMwWDJnSGxyNms4N2ZETzg5QTQxZzd6Q1dJQ1B3akVZMkR6UElYenU3clBPOXRLaTNmTGVxYjdLU0NsQmY1ZXJEcVBSWmVlZGpmZS1BeFBqeUFZQXdJaWZKRHBKbw?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3155,21 +3155,21 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46076.91666666666</v>
+        <v>46077.60708333334</v>
       </c>
     </row>
     <row r="51">
@@ -3185,22 +3185,22 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Betrunkener Autofahrer wird in Ingolstadt auf Heimweg von Polizei erwischt - Augsburger Allgemeine</t>
+          <t>Schwerer Auffahrunfall am Brückenkopf Ingolstadt: Beifahrer eingeklemmt und schwer verletzt - RegionalReporter</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Drunk driver is caught by police in Ingolstadt on the way home - Augsburger Allgemeine</t>
+          <t>Serious rear-end collision at the Ingolstadt bridgehead: passenger trapped and seriously injured - RegionalReporter</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 11:49:59 GMT</t>
+          <t>Tue, 24 Feb 2026 07:57:13 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPWjhucDdvek5HMVVQUWR4LVhhbnFzUmNVeGVrbzQ1b2p6TDdST0ZNcENYejA3RGdNZ3h1aGlESzhnRHVuTHRzMmJIMGRVNjdhdlZ4TkdaVjVjWGExUjFOWS03YVdHT2NqSmRkbXM0RUh5dVlpUzNPOVM5LXFDVnBmMG5Gb2lVQmluM0d3V0ZibWtMSmNKX2Q1LUZjYXNVYWlQSUl5QkFNRXROOS00VngwbUNFWVdkdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNb2w4ekV5aHlhNHcwSEJKaUlBN2hpd0ZVUW56eHFPTXlFMGVLYjkyMVRPT0hUTjllLUdONnY1bExmUUJnSk9SR1lmQTBjZV9oV1JHNWQwV0RnTXB2Q3ZPdFR1di1IZjBETzFJd2FTY05aYmE5LWpsdC1nSGI4X05ENkMyelJvazdFeVFJSkN2SUZWSUZLWm9fSk1NRXFjOFhhV3I5cXRLZmJJNkFyRDVSS3Z5Q1ByMVFpV0V4VHVKVXUzalJIQ2pHSkl4WU1YZU5xbjdYbldYYlJHV3R2Z2JtSDYyazE?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3224,38 +3224,38 @@
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46076.49304398148</v>
+        <v>46077.33140046296</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Village Las Rozas La Roca</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Las Rozas outlet" OR "La Roca outlet" OR "Las Rozas Village" OR "La Roca Village")</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Polizei stoppt 66-jährige Autofahrerin mit 1,6 Promille - RegionalReporter</t>
+          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Police stop 66-year-old driver with 1.6 per mille - RegionalReporter</t>
+          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 03:38:40 GMT</t>
+          <t>Tue, 24 Feb 2026 09:21:06 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNZ01KNnczSFRPLTlLZUNzb1pXWTBqbGR0LWxFTXR0ZHZWb1pza0ctYmFSd3VmRUhLcjdsVXZDS1d5NUsteUN3b01FSW9lZ213MndZMWxnUDlFTkVYcnJZQjg2Mkg2WmdOSGpSUmZNeERVd3pHUlhwMjJva0JQWlNfS1lFREcyVmZfbzMzMkprZ3dlRWVWbzRKd3ZQLWhVS0FrMFVDUnRMMXRNdDN6NDhRbFhndzE3Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPd0dBclgxSVlFV1dtaEgzNklSZENrcDBPVF9kbEZOWUZhMGtfS3BsS01WWlpwMERQMHVtUUcxaG1EaFlyV3NONy05ZlQ1TzRPTG9lVDUtZE5xVVZEbUdBTFdkNlB5TEhTb0FmSWJlOFpqTXVVLWhvd1JaYzkzNGNMaVBmaGpSaWZ0dHJ1cnBXQndERXZMN2ZhSWJSNlFPNHQ5MFMwbUF1WHRIXzBXOUxpQmtYdWgyNlpDaVhEdjcwYXBGLUtQNzQwdw?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3265,52 +3265,52 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46077.15185185185</v>
+        <v>46077.38965277778</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Unter Vorwand ins Haus gelassen: Täter stiehlt Geldbörse einer Seniorin - Augsburger Allgemeine</t>
+          <t>Zola Predosa (Bologna), sparatoria al campo nomadi: «Un pregiudicato colpito alle gambe» - Corriere di Bologna</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Let into the house under pretext: perpetrator steals wallet from senior citizen - Augsburger Allgemeine</t>
+          <t>Zola Predosa (Bologna), shooting at the nomad camp: «A criminal hit in the legs» - Corriere di Bologna</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 06:42:59 GMT</t>
+          <t>Tue, 24 Feb 2026 08:41:43 GMT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOUzZOZmpZeWJ4MGZ6Z003ZG5oYVIwZDhtN2k1VU9BM2FSLTgxWXlxcDc3eXBBOUxVY2h4SzVXU29tRXpxZzBZZW9mNFhGbXg1TWVRWUIyQzgzaGZac2N5c28wZ0pyV2hUWEhfblk2cUpGMFZmNDV2QTk3a0JZNXZfTFRqTUppSU1rSVRQa2NvSTlTX3ZEdE56U29HWTdSUmM1QXAyS2JGNkZzZ0llNm8xY1hLNWN5MXVsRHhLV1J5bGhmN3pRczRQZ3BLZXBSbVFETkZ3UkUzRURrNk0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTXZ3cFF6NURKMDl5cGZSWFJWQ2ZRWk95Z2ItemVwYmlVd1BhMm9LX2Z5YmJiOFp5b2lNVE00TVdpWUlnb2VLd3B2VnJnckU1R096NU5nTFM0dmFlU2o1WUlWakN2dkttY2Z3YlZ6akF5TnhZb3g5QkV2ZXRXSnRvR0IxZ1dRMjMxWmVaNUNTcXJIaUVYVXp5eXdwdUN6ek54Z2o2dVdybmwzUC1MS1pBMjQ1d1g5UWZFSXQtMi1MeXhleU9LWlBMeV9HaUhDczQ1bmRIMVVxaHZKR3hsWWZ0c05rUTZ5ZXFpWFdV0gHwAUFVX3lxTFBIZXFtcm93OHQ3bmZIcTdUcXV1VmN1Tm56S0dld3pCVDEtS2ZYdVB1bHYwNzBqUjhyc3ZhSUM0S3p6b09JQmtiOWI3ZmlfOUs5OWxMci0tX2NFckV2V0VKQ3Uxam1rWWtEa1dpdWdZcHA1T0JVLTVneS16d05NVmxJVjBOMDdDcHJaUW5lYS1JamdtcGFlMHhneTJkTE4zeWZtbXhNZWRtWUZQbHpIR09sNWxGZ3ktLVVVSVZlWG55eXYzX3BQV0M0MkppUVlNWU1PU3czUnRMTUNRVkVzWUlyYWhPZGs2MUFULTU2RnNFcw?oc=5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3320,461 +3320,21 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K53" s="1" t="n">
-        <v>46077.27984953704</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Alin Coen live in Regensburg: „Du bedeutest mir die Welt“ – Ein Konzert voller Emotionen - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Alin Coen live in Regensburg: “You mean the world to me” – A concert full of emotions - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 03:47:07 GMT</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNaGZyR041TjVBbXZOa0NudVppUlh4Zm1Gc1BFNmwzRmFaZjNvMExzaHBoMmh4Y1plTUk5QW1VM0lWTHNSMmN0NmJsZmlkbHpZa0dxdGhzMzNvYnhlOU1BRnlOeHdUclJKLWNjaUhHMWNFWFFxMDBjYlJWcUtidGJKQVNLOFNia1laaWVXbjR1N3JkUlQyS2dLTGZ5Uk56SThmQXFRMzYwaTVYam9wdnUxZndURUxSSEx2cDl3S1RDVGhub1dob2pxeWx0TTltXzN2bWpFVWR3?oc=5</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K54" s="1" t="n">
-        <v>46077.15771990741</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Beifahrerin lebensgefährlich verletzt: Stundenlanger Stau auf A9 nach Unfall mit Lastwagen - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Passenger critically injured: hours-long traffic jam on the A9 after an accident with a truck - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 05:08:22 GMT</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQRXl1MWhlRzRsY0RRYVZPdTBPWG9FLW9TdGl2QmdMenY2b3EyeFNGZGdZMVNoajRVc3FWeTBUeEZqanVrOEpmUTF1SDdtblFVYXRhOG5RYTcteGZqRnBLUVJ4ZTgxU2hIZ2x4dGxfaFRYN3ZIYVplS3A4VjBHVnBrU1AyRGhtNV95VDVkREo1LTJYSThBUHRJTS0weENUekpNaU9ySUlUY1g2YnJVa2E3RnZhRnV6OHQ2VnNJT2VpZ2M2SklKdmZN?oc=5</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K55" s="1" t="n">
-        <v>46077.21414351852</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>SPD Frauen Ingolstadt fordern gerechte Gesundheitsversorgung für Frauen - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>SPD women in Ingolstadt demand fair health care for women - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 04:53:13 GMT</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQWTVvZndQRWxzYWswTXQtRHNrV01FQUwwRlRsQXlqS1h4V3NPZVNsRlMyelVnd2FPV3dJSHY0UGk4cExDb0FIYkV0aGhRX184WUxRLTdpRFB5dXR2WUQxYm00RlNiU09lN050cFptMU5MRDRXSXg1cXNqZnNpUGNsOVUyazhqQTJZQmEzckI3Qy1KbWVKSzYwa2tSWVhjM0hLR0pFSktqOS1kazFDSXNXd2lWaF9BaEtBZ0Y5ZUdnVXhXUE0?oc=5</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K56" s="1" t="n">
-        <v>46077.20362268519</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Solidarischer Hochwasserschutz: Regionale Allianz setzt auf dezentrale Maßnahmen und Echtzeit-Frühwarnsystem - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Solidarity flood protection: Regional alliance relies on decentralized measures and real-time early warning system - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 05:04:48 GMT</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQbGI4VVlKYUJfeGhaTGpqVXg3ZDZqTzBnUXBqUngwQ1l2dkxFakRZN2QwTm9HTDVORC03bnpaNGVaV2FBWlNXS2VBY0dqNlRmdXpiNGVKdGR6aGxUSkJwelhkMUdTU0lUVktmSTNmcVI0NHBBbGpXZUowZnpRT2hKWHJlSFhKa1VJYVMxTkZ2VjRBVTR0dUFKVnlqNF9rdllKYndwRW5hdUNGUVZfVDhMb3BUNFJqcFQxZVhueXJVT2dZUm1iU1Z6VUNoV3MwUkhsd3BZVi1oZEdpZXlHR1NvYVppckZrLU5IZEp4SEdHWjVvcEFMODg0?oc=5</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K57" s="1" t="n">
-        <v>46077.21166666667</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Important note: Municipal construction work restricts access to the parking lot - EHC Red Bull München</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Important note: Municipal construction work restricts access to the parking lot - EHC Red Bull München</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Mon, 23 Feb 2026 16:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNdUdtZFdTODlzV1RXU2NEWGRNeGwtWjRtODUtYWI3bkZfRXVNVjhNWTBhWnNYcGVmZUtYdHJsOWYtX0NRV0xteEwxTFlJU3J4VVUxREFmaDB3dTVTaTRjdG5YM2t6VE5yZUFKRV90MnN4WURuRERQeW9CYzZaZlZhS0lOS2lHTUZvZml2RzVIc0dmdFVHemlTVjJLcV9pTjk5RkxUYnF4UFNoNlptU2c?oc=5</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K58" s="1" t="n">
-        <v>46076.66666666666</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Lamborghini Technology Boss To Head Audi R&amp;D - AutoSpies.com</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Lamborghini Technology Boss To Head Audi R&amp;D - AutoSpies.com</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Mon, 23 Feb 2026 13:01:28 GMT</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE1YYnl0N0FVLXZlckdFZVVPUE1VaGZqSmp3VTg0Y1BzWjlqN3pVams4QVYxZV9IQTVYZTEyWUFzSjE3UjRJQ3RIMjBXUEFnQ2JFVllwa0c0WUVXMXI2MUh1NnF3VG96U2xpTFpDbg?oc=5</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K59" s="1" t="n">
-        <v>46076.54268518519</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Sparatoria al campo nomadi di Zola Predosa (Bologna): giovane ferito alle gambe - Il Resto del Carlino</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Shooting at the Zola Predosa gypsy camp (Bologna): young man wounded in the legs - Il Resto del Carlino</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Mon, 23 Feb 2026 22:54:30 GMT</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQNENFR2txSTcwcFdrc01hbnRrSVZ1N19nNHZ2N3A3WUxsSzNHTkVBNnJUY3loUTN6QjBmc1Z3QjVyN2tqZS15UGpHdi1NbnFtTFh3TFFlTm9ITjNzMnVibXhDX1lKdUlMcFAyMl9jWk5MOXRISFQzVWdYZFhHdXA4QktBcWRfTk84MnpyNGt0WQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K60" s="1" t="n">
-        <v>46076.95451388889</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Local Town Fidenza Italian</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Leao, polemica dopo Milan - Parma: la protesta social per gol di Troilo - Virgilio</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Leao, controversy after Milan - Parma: the social protest over goals from Troilo - Virgilio</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Mon, 23 Feb 2026 13:23:00 GMT</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxOV05fZEVJUUNKa3plVU9UWkVSS3BYRFBlNjZxUVo1OUJjTDdiSkFpOXBFZ0IxWDFYN3dseWt4dFVlVFZVbVp5UVFaVnM4azlpZVF5QXZZMXpmWGV2eUFsNU5pdGtIWHhzcC1UbldUTjZUR0pGaGJDeC1vajZseVBMbmlQLTdWbmp2dDlGMlRKUDlESW1jMm5zSDhUUVN6WDd0YzZtOXNNYjk4RFpYOU1SMC1QWU9ZS2hHcFVjeXZGaXAtYUwycGNrdldkUGRHV2fSAdQBQVVfeXFMT2dYVXJ1TG4yRVIwWmZ3ZnhVNTlDemh6b196NlB1eFVYSFRpa3czVTZ1TVdibW9LVURjZ2FEb1Ftc25hc0g5YkI1ZU4waGJFYU1HbG9tV3pmcEtERG1ZNzBJMkJtcGxza3k4V0g3U3ZkNU9OeTk1RHp3VnU2Ry1TMGtWTEpDeEVuVVdYS2ROZ2x5djlhSndhTDJvb3B5U19wYldQUkQxTm00ZEMtWjJscEgzUU5fTTlRYjBsbHV1N2poNWViVERTWFdIbkwxTTRBREhyNGg?oc=5</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K61" s="1" t="n">
-        <v>46076.55763888889</v>
+        <v>46077.36230324074</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-24 15:18 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,32 +535,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>REVIEW: 'It's longevity speaks for itself' Shan Shui at Bicester Village continues to prove its mettle - Ox In A Box</t>
+          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>REVIEW: 'It's longevity speaks for itself' Shan Shui at Bicester Village continues to prove its mettle - Ox In A Box</t>
+          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 06:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 10:37:32 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQNHhwYkgyd1ZmTnNNLVZCd3otNHlNa2VLRHhuYlN0VDZlQlk2Y1M2WFVLSUNJUDhVQW0yclppd01lNTU1N0JyUGhGb2ZfZ1hnWFJmUEhkZnZTd2Z3RW1ZbmFZeDBZMXlUTnVOWkFjbmdsdGx2TXEySDF3bF8yZVJTb3pvNVhVczVoTXdDbnBWSU14bTdyNW5GSW9zVEg5RU9FYlloWnltSkZtVURCT0JWNUdnQ0NlaUN3UEkyenZXNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPQ0JBbVhreXY3QjZCanZWU1VSYnlMNDg3NHBrbG5VV2Q5WG9VS1dLdHFmbmtjaEh1a2RlRHNtcXRPWHVxdEtMZDNsMnhNR3hYbXAzUEFoZVo4WF82RTVGR3ZHT1hyU2pWNTFlRFdYTHFtUG1EYTV5ZkNhQmZabndXWFFiYmI2ZTA?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46077.25</v>
+        <v>46077.44273148148</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>'Disgusting' bins and rubbish at Oxfordshire Sainsbury's condemned - Oxford Mail</t>
+          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>'Disgusting' bins and rubbish at Oxfordshire Sainsbury's condemned - Oxford Mail</t>
+          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 05:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 11:06:48 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOdXNXbzM5M1gwd1ZmUm5VWHdqYVZ4T0swWVNoaDlxaEk3dFNzWUxmODBnQklwNF9JOERhckV0RGVmNTF3aF9xcVVEQ3M2TzRORDBNVXJtcDdpeHV6ekVaMEVsWTUtVUZ2N2Y3THFrUmJMaVFMT29nNFNic2V5MmUwZ2pYUkc1dkhaakE1WjdkVFpQU2p1NFdpLUd3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNcWdvdkd5cGZ3QmRMYjFQaExNdUx0S3dVcmdEelVjcUpwNUhKbENHMlJRRVFCeWxoZjJQMko2UXhOaVV5d0N1aDF1SVdDZXBOUDJoRmFsV1AtLXFZdkpjdUdWNXlxTWNBb1lnZmNnQVMwLUJVak9JVGNJRWo4SmdBT1dQWGcwLWk4NlRLcTd0OVlHbXppYTJTSkx3WGYya2xmb21WbUFHd211Zw?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46077.20833333334</v>
+        <v>46077.46305555556</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rising UK Engagement with Chinese Automakers and Asia-Pacific Industry - IDTechEx</t>
+          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rising UK Engagement with Chinese Automakers and Asia-Pacific Industry - IDTechEx</t>
+          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 04:33:36 GMT</t>
+          <t>Tue, 24 Feb 2026 10:28:00 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPeDRlc29GOWdqOVQwYm5ZLS1BYUhHbXE4ZWFLOEp3ZEp2NU9kSHF2LVFyZmN5WW5Vb3lnWDdCRTUtZkY5REQ5ZVNNd29MRHZKdmVMRzFUcHZNTFhNN1VvZUVvcGQ3UHFibWRENE1mZG5EcTB1ODZlT2ZNYVA5dDJZeGhJUVgtUGZZeFo5T003V1ItUmR2b294YzVESUhzUVEzeG55TWVVY2JSaDhKeFBUSklzSURvZW5nNUNkcjFR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNaDlnYVhpRlVxSXcxQXpzRzhaZVBTZzdhRmxESzFScjBxanNhTHVkN3IyZTFZUXgxazRRU1RMV0pBUUpYZnkxZnFQYmU4VGkwdWJFdnE5ZzRHemtjWHFWMTY3dHpPOWdkaWR1UjZWcXZUWG5sYV9iemNMQXFkVWtkTmpUeGdyWlJTbHBOWXFtT3NDMFd5SE52eUQ2S0pKYXg3dG1OMlZXVEdzaldqcXQzX1p1MXJoLUpIU0J4b0JDQ1FvdXU1U3ljV0Qyc25QeE9PRGlYc1dDY0dlcXp1ZDRxVzg0dVBvLVk?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46077.19</v>
+        <v>46077.43611111111</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Changes announced for Oxford Tube services to and from London - Oxford Mail</t>
+          <t>Politie Brussel West vindt bijna drie kilogram cannabis en plantagemateriaal - HLN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Changes announced for Oxford Tube services to and from London - Oxford Mail</t>
+          <t>Police Brussels West finds almost three kilograms of cannabis and plantation material - HLN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 07:29:15 GMT</t>
+          <t>Tue, 24 Feb 2026 13:58:28 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPaTRYa2NPSkxzZE1UWjRJSjU3eXZ3TkZka3VXdGd0YndMdHpscHJzSmJ6cWRRTGhNM2plYjFDX1hJeS00T1FMMGtnc3BsaEN1SmZ1dVYzSUFqc3pwTmtDSG12LWlRY3dkcXBxVTFUUjlubGs1dFhLMG9weGZYelhKcmZCYTQ5T1NoX292cHBWdGN4Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQVDNCRUxNSms1VFBKUXBxVTdkcGVlb2p3MGZiajBHcmFqN0oyR19uaDY5UnIwcXFQc3lQY3JncXR6blFKR0wyUVpSZ2d4UzRMeDh5UU50QllENEdBaEx3Nk1XbmNlZWE4d2Rnd2hMUVVoY3dqSjh2eWFTSnVzel9OTlV6dXBwZjVubXFWVWhhSTY3X2R1enUyM0J4bFRDYmNYTXF5U0k4aVMzRWlzaUl6UUVNNWI?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46077.31197916667</v>
+        <v>46077.58226851852</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>One of the UK’s biggest villages to become a new town – with cosy pubs and historic canal - The Sun</t>
+          <t>Trio krijgt drie jaar cel voor schietpartij achter winkelcentrum, maar schutter gaat vrijuit - GVA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>One of the UK’s biggest villages to become a new town – with cosy pubs and historic canal - The Sun</t>
+          <t>Trio gets three years in prison for shooting behind shopping center, but shooter goes free - GVA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:11:00 GMT</t>
+          <t>Tue, 24 Feb 2026 11:39:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQTFdPODFXLUpCeFczUnFia3EtVG9wRmExQUV3cUppMmFkWEQ3Z1RzZFBHZVMxRl8yNThsc1JTajdfQjdzWmg2T2VSeDlSd1NWVWFjMmlxLXBaZ2dqVEhiR2FrMFhSTWV1dUNtbDF6SWpSZmtBRC1TWnh5Ykt1MDVESW5mR0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOUXduU0hBQ2g5c0puak1mdjJQUzBfdEwxNk92RFdaemd6ZzZTTkI2dkdWWmlZV1RTTVV5cC1IdmZubHlNQTVuY0dmdlJDQ1hoRU9GSVBfNTFLQ0o4RmdoZHU0REptS3JBTVU2ek9JMmtTWFItbVpuSS0tM0o1MzVGSW9TNFFiRTFJY2VTalhyQkhsSmR1V0YtNkJCWDN2dFJIYms5cUlKUkZ4Rmh1Tm5zQVdJVVBoNUNpY2ZJOG5zNVI2YnJkRTlGdTAtbVRrekRqeWo3MEFrUkVCX04tZnZzQV80MUJKa2x4V2xxVkVweXN4ZGM?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46076.63263888889</v>
+        <v>46077.48541666667</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Organised Retail Crime Surges in UK Costing Billions Annually - streamlinefeed.co.ke</t>
+          <t>Het opruimen van rondslingerende flessen lachgas kan dure grap zijn: bij onjuiste verwerking risico op ontploffing - De Limburger</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Organised Retail Crime Surges in UK Costing Billions Annually - streamlinefeed.co.ke</t>
+          <t>Cleaning up bottles of laughing gas lying around can be expensive: there is a risk of explosion if handled incorrectly - De Limburger</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 06:52:41 GMT</t>
+          <t>Tue, 24 Feb 2026 14:22:57 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQYXAwZGpoTUZsSlVHOUpRbDl3OUsycnA1RkEwNE9IdHE1S3FiZEhZbXdwcENSa3dSTEE4aDZIVTB6ZXJWZWx4LXN2N25WWUJrNzcySnlkV0dxWlhsQUI4aHUxalJ5LXhGSG1HeVZPMjRwWWE5Ykt1TUN1dFNZQVZDTXB0ZkVmbGFuNU5weEVZckJud0lRVkZZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPNmtxRU80QmdSV2tTNlRrRHd0QVJCNDBXVnFKQWVOdkp2OEtlM3podGY1LTViTm5hWDl3aWRIY3ViU3R0dUMxbndTSGZWS2FjdmJhM2xiN1MwS0RnNTdGQVE3cGlrU2duaTkwSnBFU1lqX2xBdi1yeDh3WVhXVmVDazl0eW1KMEdKbXJURHFyQXAyYW12ODF0R2pkRWhjUjJ0bmhQQlhLQUpma1lJN1R2SldGNnBhdlo2UkNyOUtGWWVHYzRaRDFJRHhBMkVJYU9CcGZPcDJERVJSLXB4YmhTQlhfV3B5TDdtQlktRjgxZy01ak0yOXhPY3MxYw?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46077.28658564815</v>
+        <v>46077.59927083334</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
+          <t>Voortvluchtige drugsbaas bestelt vanuit Turkije poging tot gijzeling in Berchem en moet 7 jaar naar cel - GVA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
+          <t>Fugitive drug boss orders attempted hostage-taking in Berchem from Turkey and has to go to prison for 7 years - GVA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:27:32 GMT</t>
+          <t>Tue, 24 Feb 2026 11:28:25 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQNHZxbGRlR01sS215TlJRRHpQcXAwRDZzdGRNTUc0SG43OFRLcmlhUHlQTHhKcEtmQm4xZWZ3Y3p4UzNPUUs4dk50cC1tNnlrYUxib0x0N0k2T3VVRW00ejNVWU9OREU0OGNxZXFka2FPaW9QUVVoMmE1Z0pnWk9uc1ZGek5Td0YzMEhJSklma0J1SUhuNFEzNWxYdE5fVGtrTWs4WExabw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogJBVV95cUxNZV9xLWN3R3ZhZHYwUEY4LTktS3hKTXNDbFhTMnRLSHByY1NKWDlUNlVtS1pwSDFhdDFidEl6NEJDbHNLZkJZcTJ3bUkxYzNSNnNPbktjUG9HaXpUNGI1TzBKc1J2c3Fld0pqNWtVWnRiSnd5b1NEcFY1b21oLWUyaVQzNXRIZkJza0RQdW1ici1QM0hfam92a1lHWFNIcXgxQnNvcklLMWwyOXpzci1wUWVtdXdMbmdGeTg4YldQMUx6amszckRuZHlCVEpBV0F1dkU3SEpzaXNiQmZtMzYtVzZTZllOTERxTFpqZUR3ZFVoTGNSZlZSVHp6c1NUNk8yMDIxZk9FdXZOYlZ6eE1Bd3N4bm0ySXhYdzM2NjVVd1IxUQ?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,52 +900,52 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46077.43578703704</v>
+        <v>46077.47806712963</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
+          <t>Gravin Diana du Monceau de Bergendal opnieuw voor rechter voor verwaarlozing van 270 dieren: “Al zes inbeslagnames in 15 jaar” - HLN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
+          <t>Countess Diana du Monceau de Bergendal again in court for neglect of 270 animals: “Already six seizures in 15 years” - HLN</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:28:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:18:39 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNaDlnYVhpRlVxSXcxQXpzRzhaZVBTZzdhRmxESzFScjBxanNhTHVkN3IyZTFZUXgxazRRU1RMV0pBUUpYZnkxZnFQYmU4VGkwdWJFdnE5ZzRHemtjWHFWMTY3dHpPOWdkaWR1UjZWcXZUWG5sYV9iemNMQXFkVWtkTmpUeGdyWlJTbHBOWXFtT3NDMFd5SE52eUQ2S0pKYXg3dG1OMlZXVEdzaldqcXQzX1p1MXJoLUpIU0J4b0JDQ1FvdXU1U3ljV0Qyc25QeE9PRGlYc1dDY0dlcXp1ZDRxVzg0dVBvLVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxOVlFnbkZRT0RIRkNUQjYxNjFxWlkxX3RESk1NMHZremJEbmhYX3lNcEJYLTBnN0pkck5jeFdWQ2NkUVh0VFRCbWt3T2d6QkF5V1pBUFlkRmRrRGNmekJtYVBjMTl5a1hZZXBma0tRM25PWmwwQ3d3UDd0bEwybXNPZHVIeUV5R3pyNkdIc3d3V25VZVB4bE9TUmtxNU1heEVnUTZMYndkSUtnY2Y0cUg4N29FRF9RTEJzMklOVHlwbGRyTXpVOVVwLWh3bFl5UzlnRjIxc2I3bEk3MEJzb3NhNmhHXzRRUU14cWRBNVFHVjZGZw?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,52 +955,52 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46077.43611111111</v>
+        <v>46077.59628472223</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
+          <t>Stad Antwerpen genomineerd voor Vlaamse Verkeersveiligheidsprijs: “Minder verkeerslichten binnen zone 30” - HLN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
+          <t>City of Antwerp nominated for Flemish Road Safety Award: “Fewer traffic lights within zone 30” - HLN</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:06:48 GMT</t>
+          <t>Tue, 24 Feb 2026 09:48:33 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNcWdvdkd5cGZ3QmRMYjFQaExNdUx0S3dVcmdEelVjcUpwNUhKbENHMlJRRVFCeWxoZjJQMko2UXhOaVV5d0N1aDF1SVdDZXBOUDJoRmFsV1AtLXFZdkpjdUdWNXlxTWNBb1lnZmNnQVMwLUJVak9JVGNJRWo4SmdBT1dQWGcwLWk4NlRLcTd0OVlHbXppYTJTSkx3WGYya2xmb21WbUFHd211Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQMmZMVXphNzNLM0ZZNjFUZXpLUjhwMEF3YjI1d3FrX3ViUG9UV1drOEFFYzZtaGdZX1BwajhRZHhrcUYxRVktNENzSVktUHVMTzZycDFOSG1jZ1NiR0E0Qnk2YXdxQURVOGRFeDVqX1NUb0hiSjdHZUZTRDVLNkhmLWdJekFUNkx5YlY2QzgySVJqYXlGSXBENUNTanptQi1YR0ViU1ljTDJ4SXVERHR6b2FrQ0MwXzJLQ1RPOHBGZ1dHNWhONXpHOGpDRHhyN2Y0MkR0Sm9XOW0?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,52 +1010,52 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46077.46305555556</v>
+        <v>46077.40871527778</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Farewell tour for mark III trains raises £20,000 for charity - RailAdvent</t>
+          <t>Waarom laat je een vriend op straat achter om te sterven? Heerlenaar Johnny E. (43) moet na conflict binnen motorclub Kanun vijf jaar de cel in - De Limburger</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Farewell tour for mark III trains raises £20,000 for charity - RailAdvent</t>
+          <t>Why leave a friend on the street to die? Heerlen resident Johnny E. (43) has to go to jail for five years after a conflict within motorcycle club Kanun - De Limburger</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:56:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:01:37 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNQlVtd1h0QVIyR2VBYkFsR2RoN1lUd0UzMWZPMDVydUtCdEVvUEpNRGdHWG1IaHBjRzUxdGJvQ19FRVQxXzhQbGRCd2tLMGViaUZ6WVN5UThidXBGVnBUT3FsS3A5dGJJS0R5S2ZFeVR0UGNjSnd4NGpfQVBhSHVES0ZhTlZvaVVITDFQNXpYazd5N3VUWkllNW5OeWJYRk1jZFBuN21n?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwJBVV95cUxPZUV2S0NpbC1iRTlwRlpBbXB0QnBqNnZkeE9SWUQxLVdWRHp4MXloQXBvMlhNTVhXaFZJVUZKN2o2NGh1b1VyOFFJYlBsb0I4ZjJieFl5MnBYcDhYQ2Q4ZUZUVUotOExudHBNYkZlT1doSmxDd3lLbjQ0Y2FlRVZoT1JJUmFfNnN6WXBFVnZLLVNSbE9tVUJ5WWRFMmlsSk9teVFsdkNUNDlVR244Q3RnUEpjWk1HbkhHaXNDWks4T0UzYTRxMmpRQlduTGNkTUZzWmZDTmJMNC1BSFlGV0FZVG1idS1aekR2OFFrblVkMTAwQWtZVVktclJXVjNzOVhBQ3EwVUI5ZW42OUZQNS1haGdTSTFFMlNXRHdDcWllRHdWck84dTIwYlBRbU1yY3c?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,21 +1065,21 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46076.66388888889</v>
+        <v>46077.58445601852</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Drugsbaas bestelt vanuit Turkije aanslag op papa die zoontje afzet op school in Berchem: “Voor 50 miljoen euro aan drugs gestolen” - HLN</t>
+          <t>Explosief gegooid naar woning in Eygelshoven: geen gewonden, wel flinke schrik en beschadigde auto - De Limburger</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Drug boss orders attack from Turkey on father who drops son off at school in Berchem: “50 million euros worth of drugs stolen” - HLN</t>
+          <t>Explosive thrown at home in Eygelshoven: no injuries, but quite a fright and damaged car - De Limburger</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:28:51 GMT</t>
+          <t>Tue, 24 Feb 2026 09:46:26 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxNX1NManE1aGM0dUxmMXhDYUEyX19pdFRGcmZPWGtCN0U4QTFzSkVLQjRaODI2aWNqWkd1cVA0U3AyeloyRVo0aUgtQkpxaGtEY3JzMzBZUjdHMGhyUmxGT081NG1RSDdKdXJQa2tWSEpub1BSUk1IY0VRSUhrZTBySVJPTm9XSjBFSmlBTTdkbzBBRkpfc0FNdU1UX21jNER5eXJleHBJcFA5Z05JWkdMeXRpOVVGU2FzOWYycEtCak53MzdFeVdIakwyVnVKdXh4MmZiUFlDV3ViemJfc29ncWczOWhiV1lDVm03V1RLSDROYWFrLWFkcXFn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOd0xSOHdvOXluc2R6b0hTV3pfMnBqUXVULVo4TFhTYkNOVzBSc1F6bjJFY0hVRjRVSEJ4cEo0UDlONU9yenRORzFOSWR1U2hzYVJVbGNTMXNsLUdSMUlKZjhNOEFQNG54cm0zVVc3YjhlelJGSFI3N1pESHJ2RmFqSVZvb2pNU29nZjNHNm9id3l4Y08wQmNWNDFnekcwbklORVd0V2VFc0xaMzBkcU5YZENvVkNoYmpxMGZzelM2aXhTQzJTZmlEcEpvclNsWWkzbXN5Y3VUQnNkY09aLXlVWFVxSUw3dw?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46077.47836805556</v>
+        <v>46077.40724537037</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Vals bomalarm aan Grote Synagoge in Brussel: “Volgens eerste elementen weer zogenaamde grap” - Nieuwsblad</t>
+          <t>Opnieuw incident aan Antwerpse gevangenis: politie grijpt in na mislukte poging om pakketjes over muur te gooien - HLN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>False bomb alarm at Great Synagogue in Brussels: “According to first elements, another so-called joke” - Nieuwsblad</t>
+          <t>Another incident at Antwerp prison: police intervene after failed attempt to throw packages over a wall - HLN</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 03:20:00 GMT</t>
+          <t>Tue, 24 Feb 2026 12:38:35 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPLVNGa1QzTEV5X253bFc0c0pCX0NmNVphY2tGVHJkN3BjS2tyd3BHSmo4cGtsY09FaTR5NjhKNU9Dd01rQjY1c0wwZUFQWVdlTlBSTjFMcDZaenRISzJqTUlTNTJmOFAzbVF0Ti14Vjl5aXZlNkhmSWM5NkNKcjlwNUxTWHJOUnBuQU01Q2tIUmVjdkhTd1V3S1F5dWNwd3NxQ0d2WTFwNlI3aVV5MjR6X3gxQVRRRmVmekllYTdoUUYxeG10cTRqb2hyZkI1eEtOMGRlLTllTmVUY2JPRFlXQUhYdEdIWnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPbGtHUkJLT01KeFFCU1ZHR3dTRUpOdlhVSVl3b2hKRXViSUNGZmJPRTJiMjZzemx1MjNzRGtRZzFDUElVMllrSDZoUWNnekNJU2hITWtDVlBobTRzSTB1c20wNnZoTklISm1qTEQ2N0YycmFvakZzY0xyT0NIRGxHaW5WWHpVWE5xYXFpYjRDalZPb01rMHFERWszOUx5U1Q4U1J2Uk9VU2NyY2ZvYVlJNjBVR2RyLWx5dURtU0x6clJfNXlFa2ctejRqS0NELTI5cVZfQ2pUN05PblVLRHltUG5WQWM?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46077.13888888889</v>
+        <v>46077.52679398148</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Trio krijgt drie jaar cel voor schietpartij achter winkelcentrum, maar schutter gaat vrijuit - GVA</t>
+          <t>Antwerpen dooft verlichting aan 45 gebouwen en monumenten tijdens Earth Hour - HLN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Trio gets three years in prison for shooting behind shopping center, but shooter goes free - GVA</t>
+          <t>Antwerp turns off lights on 45 buildings and monuments during Earth Hour - HLN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:39:00 GMT</t>
+          <t>Tue, 24 Feb 2026 12:00:13 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOUXduU0hBQ2g5c0puak1mdjJQUzBfdEwxNk92RFdaemd6ZzZTTkI2dkdWWmlZV1RTTVV5cC1IdmZubHlNQTVuY0dmdlJDQ1hoRU9GSVBfNTFLQ0o4RmdoZHU0REptS3JBTVU2ek9JMmtTWFItbVpuSS0tM0o1MzVGSW9TNFFiRTFJY2VTalhyQkhsSmR1V0YtNkJCWDN2dFJIYms5cUlKUkZ4Rmh1Tm5zQVdJVVBoNUNpY2ZJOG5zNVI2YnJkRTlGdTAtbVRrekRqeWo3MEFrUkVCX04tZnZzQV80MUJKa2x4V2xxVkVweXN4ZGM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVzR6UXJtbHMtY1FGS0t6eVZOdjNvcEFlX21xOU1WdGZGb0tPaHpndGtwdXJ4bE5nV2prVG1xM0ZQbUlsTHhkbzVZX0p0cThqWU5XQkRRZk9pbXJrZGI2VjRCelEtaXpYYUhuZnY5WUY0WXhQOGdfWDB3QWF1QWR4NVFNVjM2NVkzUjdkTlJkcVNxQ01XMERzWWU1ajkxWmVBSVFWYTlvSmN2VElyNU1uOF9jbWdUdw?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46077.48541666667</v>
+        <v>46077.50015046296</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Vals bomalarm aan Grote Synagoge - BRUZZ</t>
+          <t>Antwerpse Vervoerregioraad verwerpt besparingsplannen van De Lijn - HLN</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>False bomb alarm at Great Synagogue - BRUZZ</t>
+          <t>Antwerp Transport Regional Council rejects De Lijn's savings plans - HLN</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 18:42:22 GMT</t>
+          <t>Tue, 24 Feb 2026 11:05:43 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNUmhvam1VWGcxVmZOSEEwLXh4cHp0ZzBPa0dpR3dxRzJpcGFzRnY3Ylc5TlRPZVllcExRbnpBT0NhSVdiRUY5em1MZGFsdk1CcmVvQVphUkVxMG5nS29BT3FCWW1QWGN1QzVuT1lTVC1wZ0tSUmZQSTI4RjdHdmZYMkR0ZzlFb2dU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPMDBYSXlQbWhUYXJYNTU0VHpqbEsxdTVYSnM5dk05UHlSSlJCSS1CMXh1UnFVcm1VZ0tWOVMtb1JFSlJQUnpyVTI0Ul9hQk5hQkdITEF6X3lfZjRFU2Rncm9sNzBhY0Zqdzdpcml4c3JmdVhobTVNUFJyTDJnZ2ExTWNxQTU5cE13dzlJNHIyV1BFRklKNl8yM18yQzlMQU5jbWlrYlpENA?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46076.7794212963</v>
+        <v>46077.46230324074</v>
       </c>
     </row>
     <row r="17">
@@ -1315,22 +1315,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>‘Spion van Poetin’ opgepakt in Brussel: zakenman zou militaire technologie aan Rusland leveren - De Morgen</t>
+          <t>Maart is Jeugdboekenmaand met meer dan 100 activiteiten - HLN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>'Putin's spy' arrested in Brussels: businessman allegedly supplies military technology to Russia - De Morgen</t>
+          <t>March is Youth Book Month with more than 100 activities - HLN</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 02:00:07 GMT</t>
+          <t>Tue, 24 Feb 2026 11:16:34 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQODlCWFZTUFlFb01fd2dRN05EWTBuT3YzVEN6YUhDWnRnR1FfN3Y5NjdXcWJaUGtjSzZ3bkJpWGFLVkd5VEpHNzF6ZElHSC1RUGZFZlRGZUkxTHJ2MXBJOWlVMkI1aUJGX2VqeEdHU2ZWUzhqMFJFNkxuSXgzcWFSR1Z0dmxrTUJmdmpacVZnTEplVDItbUp5WHoxbkFlcnRGYmVka1dMbGt1Wk5GeTZkb3Jma0swcDhJSkdiRy15bFNMQlFwV2hJNVBnOVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNYnVLZVc1VjNxVmRLaVpZWTk1XzlLVTBrV1d3bmdOZlNELXpFZDNpS3BhQ25QcmMzX0doVUdMY0NsWU5YMzg5VlF0WThSQVpiTk1EdHdHelFuMXJjbkdadldvV1hQWW9ZTzZFNWRhSzhnbVZTSk4yS3ducjlpWHV4U1NkeEVoQ29fZjZPRlFUbzJlRmRyOUVMNHpB?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46077.08341435185</v>
+        <v>46077.46983796296</v>
       </c>
     </row>
     <row r="18">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Politie Brussel West vindt bijna drie kilogram cannabis en plantagemateriaal - HLN</t>
+          <t>Beurtelings verkeer op de Kapelsesteenweg door bekabelingswerken - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Police Brussels West finds almost three kilograms of cannabis and plantation material - HLN</t>
+          <t>Alternating traffic on the Kapelsesteenweg due to cabling works - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:58:28 GMT</t>
+          <t>Tue, 24 Feb 2026 12:05:04 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQVDNCRUxNSms1VFBKUXBxVTdkcGVlb2p3MGZiajBHcmFqN0oyR19uaDY5UnIwcXFQc3lQY3JncXR6blFKR0wyUVpSZ2d4UzRMeDh5UU50QllENEdBaEx3Nk1XbmNlZWE4d2Rnd2hMUVVoY3dqSjh2eWFTSnVzel9OTlV6dXBwZjVubXFWVWhhSTY3X2R1enUyM0J4bFRDYmNYTXF5U0k4aVMzRWlzaUl6UUVNNWI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPVVVoM3lVUzdhOWJUT2lGSi1HbDRHQmExeG1falVTUEt1WEdBRFgwRlJJWUJIV0xmd0M2UmlkdTN5X3RDa2Y4b1FjU2RzSGdFMmdXMHNsSGZhUXBIeHR0Mkh4MDhVdTREbTFsYXV6UUtxRzRIM2ZCM09MQkg0RXo5c1Y0YXcxZ3lSSmhyM3dpemoyMU13UlJNSVR0LTI1ek5sWGN6cWxn?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46077.58226851852</v>
+        <v>46077.50351851852</v>
       </c>
     </row>
     <row r="19">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Waarom laat je een vriend op straat achter om te sterven? Heerlenaar Johnny E. (43) moet na conflict binnen motorclub Kanun vijf jaar de cel in - De Limburger</t>
+          <t>19-jarige krijgt vier jaar cel voor brandstichting bij juwelierszaak in Antwerpen - GVA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Why leave a friend on the street to die? Heerlen resident Johnny E. (43) has to go to jail for five years after a conflict within motorcycle club Kanun - De Limburger</t>
+          <t>19-year-old gets four years in prison for arson at a jewelry store in Antwerp - GVA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:01:37 GMT</t>
+          <t>Tue, 24 Feb 2026 11:25:42 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwJBVV95cUxPZUV2S0NpbC1iRTlwRlpBbXB0QnBqNnZkeE9SWUQxLVdWRHp4MXloQXBvMlhNTVhXaFZJVUZKN2o2NGh1b1VyOFFJYlBsb0I4ZjJieFl5MnBYcDhYQ2Q4ZUZUVUotOExudHBNYkZlT1doSmxDd3lLbjQ0Y2FlRVZoT1JJUmFfNnN6WXBFVnZLLVNSbE9tVUJ5WWRFMmlsSk9teVFsdkNUNDlVR244Q3RnUEpjWk1HbkhHaXNDWks4T0UzYTRxMmpRQlduTGNkTUZzWmZDTmJMNC1BSFlGV0FZVG1idS1aekR2OFFrblVkMTAwQWtZVVktclJXVjNzOVhBQ3EwVUI5ZW42OUZQNS1haGdTSTFFMlNXRHdDcWllRHdWck84dTIwYlBRbU1yY3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQa0lwTTV0TjFWaE9SaWlLNFIzVzgzX2N6S2Uzekt3Z2tLWjhrRGZnRS1aWjRXWjU0dDF6VlZHelNiNkd1UmtjSE43MGN4VmVEeDFmX01GUTR0N0x0dmdvS3NiSFVVNEV6Ym1IVUg4WEFPb0paMWhCai12YU9Gd24tWHZPSm1GUzNXbUd6YUI2VE1xaURaYlA5QllGcGUwRnpuQ3JuWWNLbTc1MkJQX182Y19NN1FZTk9iTzctR3h4eDVnWkZIa1pSWHN1WkM0QkF6eFVBTzUtQ2VaRFk2Zm1VT2pRQl8yMGpqNEhTUWlB?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46077.58445601852</v>
+        <v>46077.47618055555</v>
       </c>
     </row>
     <row r="20">
@@ -1480,22 +1480,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Valse bommelding aan Grote Synagoge in Brussel: omgeving en tramverkeer tijdlang afgesloten - HLN</t>
+          <t>Radio Minerva eert Frank Boekhoff op dinsdag 24 februari tijdens een twaalf uur durend radioprogramma: “We zullen hem nooit vergeten!” - HLN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>False bomb threat to Great Synagogue in Brussels: area and tram traffic closed for a while - HLN</t>
+          <t>Radio Minerva honors Frank Boekhoff on Tuesday, February 24 during a twelve-hour radio program: “We will never forget him!” - HLN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 19:18:38 GMT</t>
+          <t>Tue, 24 Feb 2026 14:07:41 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNWTVCY1dETU45MTMzQ1l4YXhSaVQyWjhjQjRtd1E0OEdMNllTQnZ5SlJiN2Rod3JUaTlMMTU3bGM2U01jSkJuUkpCUlExQXl3MUFFcE1acFdpRVY4MnQtcVdoZW5zSHlGZDBIRWlGQTFtLWd6RzJraG9iWWd2RHdJSktMYkRfaWFBN3prOUFTQTZyS1F6OUdfOWs3RzFqSzlGRF9LbDFsUG5LM1pyOGxSbWJKamItVXRmMTM0UW5EbXlmeWc3eFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPMnFVMngxOEFlSUpuc1B1TzBsZHk4b2stc3EyeDYxV1VhNGlXV2hDTlJTUmFPTjlvdTcxQWFuU0JfZTZMT18zYVFPMHFBS0RIZTVJZ3BsX1dRUHU4cnlYcGtGbDBwd2hsQ0lGQjdlSHhEZDBIbXNKTVNQcFlBanhCbFRXNUlJVnVFdm1HV3I2d2pYaGtpZHRjZFV3NmltWVFzT3BmWFpQaWdVVEoyMFk2LUtDWG9wRE9JRmNoSl80bDd3T1JLN0p5cU5lcWxfZ0hINk8xTVRDSktTMUxuT2NBRTUyY1Y5VHVlRmJzSnRuQkxtbEwwVWNHS2VCdFhsZw?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46076.80460648148</v>
+        <v>46077.58866898148</v>
       </c>
     </row>
     <row r="21">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Gravin opnieuw voor rechter voor verwaarlozing van 270 dieren in Brussel: “Zes inbeslagnames in 15 jaar” - HLN</t>
+          <t>AG Vespa zet Wolstraatcomplex in de markt: ateliers van vzw Ercola blijven tot 11 juli - HLN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Countess again in court for neglect of 270 animals in Brussels: “Six seizures in 15 years” - HLN</t>
+          <t>AG Vespa puts Wolstraat complex on the market: workshops of non-profit organization Ercola will remain until July 11 - HLN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:03:38 GMT</t>
+          <t>Tue, 24 Feb 2026 12:28:35 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNTmVTUGtHaF84MHFKTnpoVFprUC05R0Zvb3ZjdlNFcWFVYmt1TTJZYXRIZDd3bGtDMk1UTmxDSkE4V3ktRll5dkEyeVhqamxRSk40OUg1NVVJOFhCM09uWUsxaDNhMUNGZng3TFU3ZDg5cmtwYndNY2UwRGR5bUJwNVJWek1jbFFhX1JGaERGdmh4RnAxdWJJckMwQ0JTcjdIVzBOalpDemNjYnB0d0RwVHU1YUg3aE5FeEJoVU1WYkNsQXl2NURKX2k2UVhJdElpWE9CTml5eVlUUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdm9fSkhTTFNrSUNnRnRYOWowZm1zUERzY2Q1M2xYdmZSOVg4RnctSnZveVBlSGlWZ1ZvYnRram52cTVjNW9La0RSSFFjQ2V2UXV1OGlqdTNibG9CUWZQSnA3aWZJNnBFNm9GcEtQQzhDVTVUSHBodG9rQnctaF9vNVdHWW81RW5zbXlKanV0QVJPeHYtNm50RTUxM2k1UHh1cVJIMzlIcmZGdF9lY2h2RkdKZnVTQVY5d2NWdEdUTnc5dw?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46077.54418981481</v>
+        <v>46077.51984953704</v>
       </c>
     </row>
     <row r="22">
@@ -1590,22 +1590,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Notoire drugsbaron ‘Flash’ gelinkt aan granaataanslag in Knokke-Heist - Nieuwsblad</t>
+          <t>Asbest vrijgekomen bij afbraakwerken in Markgravewijk, werf stilgelegd en pv opgesteld tegen aannemer - HLN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Notorious drug lord 'Flash' linked to grenade attack in Knokke-Heist - Nieuwsblad</t>
+          <t>Asbestos released during demolition works in Markgravewijk, site shut down and notice drawn up against contractor - HLN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 01:45:00 GMT</t>
+          <t>Tue, 24 Feb 2026 11:22:43 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxOREMtU3Z3Q2ZUQmh2dTJKWHB5SDFYVklncFk0ZE1fUGRWUnJyUjN1OUktTGh1a29ma0ZFdFZYWENEQ3NwQUNrNEYwcW1JREdkTF9HaWlRR2pfOU04eHBXQXlHOFZKVUs3dzBvaFEyZll3eGNJUklvOFl1a0E0bnAybHFOT29YaGQyS21nUFYtd2c4VGVkZ19fb2FjQ2RtS29HZXdsLXp5R3F5RHh6VnFoTld6VTNOc3RXWlJ6dmhlTUJiTzRCTEpRVDBQdmxxYU1XbFhSdFJBTUNDLVQ0Y2Q0Qm5UTDdOekNqLWVGV2hlUWc0RVcwM0lnaQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOYklwVUNDTmRCUm5ZbldoWlJjMloyQjd6TENkajRIZGN0NHprRTFZM0dPdFJEYTE0VmJ2UGVlZFdDd3cyMlJFUEVFRUM0UVF0MmphUXpWeE9NaV9zRmZwenliaDFycmNxMUZlQkJjanhoQ3o0MWF4WS0wenFhSXk0R19qSjdWdjdTM1dKYUxrbWZEWksyamNUa2J1SkhvM3ZwTGRycndPUlBNOUExVnBvZEdQbXpYX203UG84TkJnMjJ2YnAzUkwtYUp1cEtyV2tTbkxTRURB?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46077.07291666666</v>
+        <v>46077.4741087963</v>
       </c>
     </row>
     <row r="23">
@@ -1645,22 +1645,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Antwerpen dooft verlichting aan 45 gebouwen en monumenten tijdens Earth Hour - HLN</t>
+          <t>Wat betekenen de plannen van Antwerpen voor de stadskas? Zo evolueert de schuld de komende zes jaar - HLN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Antwerp turns off lights on 45 buildings and monuments during Earth Hour - HLN</t>
+          <t>What do Antwerp's plans mean for the city coffers? This is how the debt will evolve over the next six years - HLN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:00:13 GMT</t>
+          <t>Tue, 24 Feb 2026 08:31:33 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVzR6UXJtbHMtY1FGS0t6eVZOdjNvcEFlX21xOU1WdGZGb0tPaHpndGtwdXJ4bE5nV2prVG1xM0ZQbUlsTHhkbzVZX0p0cThqWU5XQkRRZk9pbXJrZGI2VjRCelEtaXpYYUhuZnY5WUY0WXhQOGdfWDB3QWF1QWR4NVFNVjM2NVkzUjdkTlJkcVNxQ01XMERzWWU1ajkxWmVBSVFWYTlvSmN2VElyNU1uOF9jbWdUdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOam9oWTQ1czAwZ2pWSTRYY291YkJ0bU5qUXcxV29jZWwtVTRMY1lBaTd2SWE3NXg4TlB1OTd0RFJ2Y1pXdldkUTVBOUZsWnc0LUtuVm1raVp3TURMUEYzYkNLU1UwRm1yOXhWZlRxaHpnZmhLZlI5cTJZOU1NS2dhTlk1MVM4b3drRkhodmp2Ynd5dXRqYlpZVEtseVhxNG1tUV82OUhIcXJiTVVEWGtNTlB3SUtMM3pvVWNpT1JPNTd3cXZQTE5tb3lsLWxkYXdMem9j?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1684,38 +1684,38 @@
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46077.50015046296</v>
+        <v>46077.35524305556</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tiener móét van ‘Zero’ naar Antwerpen rijden... Wat later woedt brand bij juwelier en krijgen hotelgasten rook binnen - HLN</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Teenager has to drive from 'Zero' to Antwerp... A little later, a fire rages at a jeweler and hotel guests ingest smoke - HLN</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 04:36:58 GMT</t>
+          <t>Tue, 24 Feb 2026 13:30:36 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxQX21rWDN5aHZDUzI2X1hIb1JxaDRVRXlEYlhMaGt2Uld4RjIwWGhDWWl4aVZsTVBlMndIVUZ2UFg1WUhGM0tMVXJTc3N3cFctUWJVNl9QNHRmWXpRWHowTkljR2dtNnhFSHJaY04zS01WYl83Y0gzcG5famVkOUs0TGJWZlpTX201U2hvOEdPVmFCNVNpV1pxb2VkallKbEtfc3Z2NGEwdmRZSmxObEVDQXAyM0ZPeWpORXhWMUJNOGo4UDZDQ0dheDBCY3ktYlVVblNHQ2VGalpTZVNWZzRfQmtkaVEyQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOTVkweWFzUUNLdXBoYTJPUGNWeFI3c01LV1pqRWU2eExiOUFwOUE2MlZGaFBySWVJUmdUWGotM1BDS1lydWgwcEpZR3FlbHpuZmpDVVkyYWhNQnBSTEpMS1VscG9HOE1pREFTUlM0VHF4UV9UUjRybFNmaHpWMDlvdE5kZUt5d2lRYW9ENmFkQVFoMnZyRzY3VllEYVkzWEU?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1735,42 +1735,42 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46077.19233796297</v>
+        <v>46077.56291666667</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Antwerpse takelpionier failliet: takeldienst Viaene legt na meer dan 50 jaar de boeken neer - HLN</t>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Antwerp towing pioneer bankrupt: towing service Viaene closes its books after more than 50 years - HLN</t>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:34:08 GMT</t>
+          <t>Tue, 24 Feb 2026 10:27:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNanBoV2o1anpZNlhuVEdxS29TaUh6VXdodFVkZTExeW1uUkZsZElSendqbzhoczRLTVdvOWRKcE9Wa2lINkVfQjRtRjBYSVdvck5wM0RPeFpMaFdpcjR5LWYxUndSNDczZGg3Tk5zbzVYQUdyWThVQVg3dEF5UEE3aVdoRFZIWFhINlFlN3NWM2V5YzQxU1FZSXJ1OThxcDMyeldEWk91MlFwbWRGb3ptNE9VbUZTcExhZWcyeU9SY00yYTF5alNaeA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNM185ekl4N3lkY3FGV2xtcHpCRDZicWFIVWpxeXZuVUVzNGc4SFpCa292cnVnaElFMUtnYlMyeVRXWnpnNWNfQmxFVEdzTk9ZVnFob3RqaDgxMTZmWlNaa3ZPWWtVeVU1YVI4SG1vUGdvdmVNUENkdy1fTUJPZTBkcUZGaW5BblhDSHFfbENWLUtoemlqREJHUjB3ZjBnS3AxNHZfZzdOTGdEYk1KV3ZNcVl4R0prelRHVW82SE1n?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1790,42 +1790,42 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46077.44037037037</v>
+        <v>46077.43541666667</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Oplettende voorbijganger helpt politie inbreker te klissen op lijnbus richting Antwerpen - HLN</t>
+          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Attentive passerby helps police catch burglar on scheduled bus to Antwerp - HLN</t>
+          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 01:58:36 GMT</t>
+          <t>Tue, 24 Feb 2026 12:16:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPSVVWMEZtMTZNTVN3YnZYTjhHMGl5blBYNVVoZ2pTOWVzYlhKMm1hVkZRUWtmNEVIcWdRalJteGJuR3VSSU9IWEhUNTQ5aG9GWDBfYUNpb0dZdll4c2NJRTlCTXlIUDFNSkFMTWtQZ0I2SUU1b1Z1TGNhUzlUTWZ4dVlvd0lEQ0c0ZFVfbGZJellkNkFfSGdhU2pTSExLcUFod1JxMEZuVlE0UjExQnRQTHdQM1dTTUp4YldiazRYTmxTaVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOOTRkZE1mSU1wNTNCODJ6TEt2WWtuTF9yMUR4c1BOb3ptMExaU0ZJSUFyek96ZnpGaHRGRFd6aElmLU9WeXN4ZEZZazVsLTRUNDREamdwTGlMLXhsSHZoLTYta2gxNlBzUlhmRkdCaWZub0xBQl94VTdDZmZhU2s5b1R5TWRpd3BZV3JDS1NTRWRsUjZtemdVLTdaTmkzVDJEVzRCNA?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1845,42 +1845,42 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46077.08236111111</v>
+        <v>46077.51111111111</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Antwerpse Vervoerregioraad verwerpt besparingsplannen van De Lijn: “Terug naar de tekentafel” - HLN</t>
+          <t>La Ville de Bruxelles supprime une taxe pour l’installation de panneaux photovoltaïques - 7sur7.be</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Antwerp Transport Regional Council rejects De Lijn's savings plans: “Back to the drawing board” - HLN</t>
+          <t>The City of Brussels removes a tax for the installation of photovoltaic panels - 7sur7.be</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:08:51 GMT</t>
+          <t>Tue, 24 Feb 2026 08:50:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNZ2hxaTJvZkxLVUJBOUt5d28yc2dPMmpaZ0lueFc3WHVYd01WMWlweDBQVTk5OFRTMVlJQUxFUXpwRFFfSEJEWGtkcnJPTi1zelo5T1pvelFOTTQ1V3J2cnlaY21saUFUMHU0QTlSeC1xMk4tTzRFNndIek84QmxrS0FLbThyek1yU09ueVlhemZiaWF4OGc4VE44SnM3cXE3RDlqSkxwSy1XUzlVVGtuTXhWb29ETm9zNmRYbTJiRlpfdHlyTVl1Qg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPRWg0V2dNa1lZdG1wUWp4V181cklFS3JlWnc0VkRIOEN3STFyRUtURmRRSlQ2U04xQlVMWERsbE12eXpqUDE4QjZPTFl1TDBOVzk4N0YtQzRGSXVYcE9QZDJnem0yZ0xGSkRLN0RWQzJfSDJYbDl6VmktQUQzMFZGRXBYcWpIX3J5SnVlWVlIeXlQVW0zbHNCQ0NNWXZyN2VXVWdLTWVYTU9BOGkwMGhWUmZDQ0o0aUg3bVd0ay04TjBWLWxo?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1900,42 +1900,42 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46077.5478125</v>
+        <v>46077.36805555555</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Beurtelings verkeer op de Kapelsesteenweg door bekabelingswerken - HLN</t>
+          <t>Halen keurt aangepast meerjarenplan goed na budgetfout van 5,4 miljoen euro - VRT</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Alternating traffic on the Kapelsesteenweg due to cabling works - HLN</t>
+          <t>Halen approves adjusted multi-year plan after budget error of 5.4 million euros - VRT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:05:04 GMT</t>
+          <t>Tue, 24 Feb 2026 09:32:52 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPVVVoM3lVUzdhOWJUT2lGSi1HbDRHQmExeG1falVTUEt1WEdBRFgwRlJJWUJIV0xmd0M2UmlkdTN5X3RDa2Y4b1FjU2RzSGdFMmdXMHNsSGZhUXBIeHR0Mkh4MDhVdTREbTFsYXV6UUtxRzRIM2ZCM09MQkg0RXo5c1Y0YXcxZ3lSSmhyM3dpemoyMU13UlJNSVR0LTI1ek5sWGN6cWxn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPOTItcThiT1hZQjVXaDA5TEI5RUlVdmt5N1UzR2hEelF2aVBXemRfcTdNbk9xUk5sY2NfWkpJdmIycHN5TThoaVNnVVpCWjgzYXExeFpZUk91bVhhdFhiZ0szcDNRT3Nua3RCSTVUa1BTSGRUdU42TXJ3NzVYSXdFMTRZMkwwUVpqaURzNXJMMVIwbk1rNzNSQVdVaUVvdHRVNGNWcURCUzA?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,38 +1959,38 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46077.50351851852</v>
+        <v>46077.39782407408</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Maart is Jeugdboekenmaand met meer dan 100 activiteiten - HLN</t>
+          <t>Environ 50 emplois menacés par la faillite de IKKS Belgique - 7sur7.be</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>March is Youth Book Month with more than 100 activities - HLN</t>
+          <t>Around 50 jobs threatened by the bankruptcy of IKKS Belgium - 7sur7.be</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:16:34 GMT</t>
+          <t>Tue, 24 Feb 2026 10:07:00 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNYnVLZVc1VjNxVmRLaVpZWTk1XzlLVTBrV1d3bmdOZlNELXpFZDNpS3BhQ25QcmMzX0doVUdMY0NsWU5YMzg5VlF0WThSQVpiTk1EdHdHelFuMXJjbkdadldvV1hQWW9ZTzZFNWRhSzhnbVZTSk4yS3ducjlpWHV4U1NkeEVoQ29fZjZPRlFUbzJlRmRyOUVMNHpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOem83dERqcmRmSmtFWjNqa2Y3NnBpVldLaEJVbWY0Q1FTNTRiRktXS1BVd01WQVNvQVp2VVFRUWdzdjk5RV91bXgtbFZweWdYeXNGbHU1QTl2ZzJuV09lMUdmVDNMTVVRMlBzQ3lJVS1SM3dWLUVLZ0FwTlVmZXpsdWJYbUtDNWtBY0xnUngwSEkySmwyWTFsSFFhZ1JWRUVJ?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2010,42 +2010,42 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46077.46983796296</v>
+        <v>46077.42152777778</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>19-jarige krijgt vier jaar cel voor brandstichting bij juwelierszaak in Antwerpen - GVA</t>
+          <t>Courtois va investir en Belgique : deux clubs mentionnés - FootNews.BE</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>19-year-old gets four years in prison for arson at a jewelry store in Antwerp - GVA</t>
+          <t>Courtois will invest in Belgium: two clubs mentioned - FootNews.BE</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:25:42 GMT</t>
+          <t>Tue, 24 Feb 2026 12:39:21 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQa0lwTTV0TjFWaE9SaWlLNFIzVzgzX2N6S2Uzekt3Z2tLWjhrRGZnRS1aWjRXWjU0dDF6VlZHelNiNkd1UmtjSE43MGN4VmVEeDFmX01GUTR0N0x0dmdvS3NiSFVVNEV6Ym1IVUg4WEFPb0paMWhCai12YU9Gd24tWHZPSm1GUzNXbUd6YUI2VE1xaURaYlA5QllGcGUwRnpuQ3JuWWNLbTc1MkJQX182Y19NN1FZTk9iTzctR3h4eDVnWkZIa1pSWHN1WkM0QkF6eFVBTzUtQ2VaRFk2Zm1VT2pRQl8yMGpqNEhTUWlB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNTlJDdTgzUm84dnhidVNwNUtTZGJqbWZZOVJmSHBzU1QyYmk4QV9ZanJ5TG12cXFKVDhVSHplR2dudWVsb3RlWjZUd0FpVmhHZFJfQzFnTlpvMnJwX2Y1Q3RLY1lzTlNWQ0JNSXAyalBMNm9YazVTenlGUXdranlMbjlwWUpSSlppbjF6SXU1aGJJd185?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2065,42 +2065,42 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46077.47618055555</v>
+        <v>46077.52732638889</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Stad Antwerpen genomineerd voor Vlaamse Verkeersveiligheidsprijs: “Minder verkeerslichten binnen zone 30” - HLN</t>
+          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>City of Antwerp nominated for Flemish Road Safety Award: “Fewer traffic lights within zone 30” - HLN</t>
+          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:48:33 GMT</t>
+          <t>Tue, 24 Feb 2026 13:32:37 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQMmZMVXphNzNLM0ZZNjFUZXpLUjhwMEF3YjI1d3FrX3ViUG9UV1drOEFFYzZtaGdZX1BwajhRZHhrcUYxRVktNENzSVktUHVMTzZycDFOSG1jZ1NiR0E0Qnk2YXdxQURVOGRFeDVqX1NUb0hiSjdHZUZTRDVLNkhmLWdJekFUNkx5YlY2QzgySVJqYXlGSXBENUNTanptQi1YR0ViU1ljTDJ4SXVERHR6b2FrQ0MwXzJLQ1RPOHBGZ1dHNWhONXpHOGpDRHhyN2Y0MkR0Sm9XOW0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNRHZ4dm0tREV0cjFucHowcUNrWGlJTVljdlFXcjNtdFg0OUh4a2hWb25ucnlzMkNMdThqU25BNm1yaHhBRk8zTDRwcHdHRHZFRUNBSVlHcXZjdDJFQU95SEVCM20wQm1YNmFzczRjdzE5UmZUY2NpWldzMWRfdXpSVmo4ZlpsVHdNOWo1aVFGcVRBc0I5RjVyYkRGeXZmVTBGZkFvNy0xZFVxa2JNZ0RzeGt2dHJCZTZHUTU1RXRZbzNpQQ?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46077.40871527778</v>
+        <v>46077.56431712963</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Halfuur file op E313 richting Antwerpen na ongeval op aansluiting met Antwerpse Ring - HLN</t>
+          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Half-hour traffic jam on E313 towards Antwerp after accident on connection with Antwerp Ring - HLN</t>
+          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 07:35:25 GMT</t>
+          <t>Tue, 24 Feb 2026 14:08:23 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxPOHNXVzE2SUxteEFZb21NakZYTTBBNmlvRGJDTWwzVjF1Ykh1d1pFNTZpcjQ2VWFqc1dwMEpWMm1mWFZkVk0talpZOUx0dnBWUEhqMlA3WkFDUWo5SkRTVlhoeVZTSXFsT3RfVU5UTkpKWEM2bC1kdGw4eUdVNmRIaXZyR0xKQVgwTnJrTG5pYTV3ZDRwdHBJZ0hlR0hreGlORnNjbjRhMExHRDJaYnVvRE5saUV5amFQWV9kUVpFby0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPNExOajRSMzJtQk9kOENCeXlHM25OUm5vVWQyUkszamgzQjVOMm92anAtdHN2QXhFLUVMLUptNVJ0YzV5dFJWTE5OeVNCMFVobnlyelUzeFBadlNFV3hCRVI0Y3pUTExVYU9TNFdwVUNsaXhyQjc2QW5MZlh3Rk9rejhZUDhEU1h3LUVQWHhBWHNHWG80NUltV2hxd1YwWmhRVVZyOHotOUdQeEp6UlVQYi1iVDZWcHFOanBzWWFB?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46077.31626157407</v>
+        <v>46077.5891550926</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Village Maasmechelen (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen Village" OR "Maasmechelen") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Wat betekenen de plannen van Antwerpen voor de stadskas? Zo evolueert de schuld de komende zes jaar - HLN</t>
+          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>What do Antwerp's plans mean for the city coffers? This is how the debt will evolve over the next six years - HLN</t>
+          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 08:31:33 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:27 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOam9oWTQ1czAwZ2pWSTRYY291YkJ0bU5qUXcxV29jZWwtVTRMY1lBaTd2SWE3NXg4TlB1OTd0RFJ2Y1pXdldkUTVBOUZsWnc0LUtuVm1raVp3TURMUEYzYkNLU1UwRm1yOXhWZlRxaHpnZmhLZlI5cTJZOU1NS2dhTlk1MVM4b3drRkhodmp2Ynd5dXRqYlpZVEtseVhxNG1tUV82OUhIcXJiTVVEWGtNTlB3SUtMM3pvVWNpT1JPNTd3cXZQTE5tb3lsLWxkYXdMem9j?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUW54aFlQc196RnJXM0FfVWU5a2JSN2w2MXdiZVg0Z2U2aXdKZENsNThtVWVvQjg3U0FwUUQ2Qk5SZF9rSnVqQWxrc1VzOUNzcVRfbWVXNWFCUW80ckl3MHJlaTZvUElidlBqZWNlSm85a1otTXNBMkpYTlQ1YzJBcDVNNkY1a2o2OUJtNG1HYnItU2RodXRXb1pXMVFOTkF6ejk3cEY4ZTdRbTA?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,52 +2220,52 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46077.35524305556</v>
+        <v>46077.5440625</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Asbest vrijgekomen bij afbraakwerken in Markgravewijk, werf stilgelegd en pv opgesteld tegen aannemer - HLN</t>
+          <t>​Mainfranken: Polizei warnt vor verschiedenen Betrügern - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Asbestos released during demolition works in Markgravewijk, site shut down and report drawn up against contractor - HLN</t>
+          <t>​Mainfranken: Police warn of various fraudsters - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:22:43 GMT</t>
+          <t>Tue, 24 Feb 2026 15:00:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOYklwVUNDTmRCUm5ZbldoWlJjMloyQjd6TENkajRIZGN0NHprRTFZM0dPdFJEYTE0VmJ2UGVlZFdDd3cyMlJFUEVFRUM0UVF0MmphUXpWeE9NaV9zRmZwenliaDFycmNxMUZlQkJjanhoQ3o0MWF4WS0wenFhSXk0R19qSjdWdjdTM1dKYUxrbWZEWksyamNUa2J1SkhvM3ZwTGRycndPUlBNOUExVnBvZEdQbXpYX203UG84TkJnMjJ2YnAzUkwtYUp1cEtyV2tTbkxTRURB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOWDNkYUtDak02bnA4LXVTd0lXVFpaeVNRTnVVNGk0VndJUy1oeXVkWm9IbTdtMWV5NnRCdXVSWmQ4LWotUEg1LVc4WVJ0Qk1GZHBDMVUtYlk1VjROTlpwM2R1RHhIX2cyX2xDWG9FNm1DN0hlYVZQWVJEbkRtUkpsTnlzTndjUnMwWm85Vy1USE8xZw?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46077.4741087963</v>
+        <v>46077.625</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Royal Caribbean bets on flexibility with new Discovery Class vessels - Travel Tomorrow</t>
+          <t>Wertheim Village: Polizei stoppt mutmaßlichen Seriendieb - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Royal Caribbean bets on flexibility with new Discovery Class vessels - Travel Tomorrow</t>
+          <t>Wertheim Village: Police stop suspected serial thief - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:53:01 GMT</t>
+          <t>Tue, 24 Feb 2026 09:34:00 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNXzV4T21XbFJaMGdnTnl0X2FFTzhwUk9aZ0Q1TWRVTENZRXpWU1hWRGJnY3VzcGZQNFRHcmg3TFpLTVN5NnBDZ3ZhX19wcmhtT1VncmtlcGFIYTRKRUxYd2R0d0R3dDM4eUN2Vk9GWHdFWVZ1NnBpV0drZkxXRGtUN2FBejJyNng1ak5iMTVWeUx5ampWcnBVanlMU3Q?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNempGdjdfTkxudlBkZnlNYlNUS3h0MEluS3JYU2tOVW9zamM4QUdCODMyNTAwc0ZDY0NCYXpReG9wOTVtOUY2eW9rWmhxT0RHaUdubGNoWVN3SjBCaE8tSlBpSTlneF9aQnNMdHR0VDI3Wjk4el80OU91akJGYWV4aVVuM01SejN5NC1rQlg0WElRd2VJbXVhZEtjZEVwdDAtYlZnSFFjazhjOExOcGszYmt1X0hEUlZyQjl3aTRWXzZxWHJ1NXlJ?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46077.57848379629</v>
+        <v>46077.39861111111</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
+          <t>Unfallfluchten in Aschaffenburg und Kleinostheim | Foto: Dirk Ceelen - main-echo.de</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
+          <t>Accident escapes in Aschaffenburg and Kleinostheim | Photo: Dirk Ceelen - main-echo.de</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:30:36 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:01 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOTVkweWFzUUNLdXBoYTJPUGNWeFI3c01LV1pqRWU2eExiOUFwOUE2MlZGaFBySWVJUmdUWGotM1BDS1lydWgwcEpZR3FlbHpuZmpDVVkyYWhNQnBSTEpMS1VscG9HOE1pREFTUlM0VHF4UV9UUjRybFNmaHpWMDlvdE5kZUt5d2lRYW9ENmFkQVFoMnZyRzY3VllEYVkzWEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQMW02WVZqN19mTERhVXdiT194SUtPU2ZxVTJ3dGNKd2ZLQzVmM2lxb3lTdWpHVjBqOVlFTFVOYXE0d0czbUpZQzFFU19OT294MmdqVlU3d2M1QzFWUndPbm02SVBvakFlc0tVSnl6YXJjOUNaN2FvNUYwX1pOOGJ3aVJoZjlPOU9DWnFRZlBlZG5uNXN4N3ZvWnpYN21VX2M1Skppd2c4Zw?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46077.56291666667</v>
+        <v>46077.54376157407</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
+          <t>Marktheidenfeld: Polizei kontrolliert erfolgreich - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
+          <t>Marktheidenfeld: Police check successfully - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:27:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:09:08 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQZnNnQURka1FpeVppWjNTcnRjSmpQVHA1d0VQRXN3MkR5aWtqTW02SVduMExEbUJQYWp0X3dPbzVySndQZTBuQzlSOGF5V25pSFFVN2RNemFsU2Z1SzNpTzBfUU5HenlhREJtNGUydFpuNG1US1JtbE83NENfZ1RlY0dhSDY0TnRjeWU1bk0xOXJmNndmNE1VQnBJdUQ4VloyeE03YmdXTXpIUkZ4ZmZ0UEg4d2ZqaGwtdEh4UTFITExSWDhsZXZCclY1NEhZSHF5SmV1TlgyLU9oZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNM0F0V01ZMjFGbzFpQ0FldUNxRnI4UkplZ2daMUlzTXNvWGM2WnlUZGprenhxMXBfSkRrLTFkWUU2c2VFODdxRTU1bWF2bVNZeW9zWWVPaEtGU0ZfdUdGbVBKOGt3dEdmaUszMTdlZnFuNUV6b0JWUEFtVjBlTmdFQXh5SXhuZTN2eVVzelU2Z29RUU9wNGw2Z1Vn?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46077.43541666667</v>
+        <v>46077.58967592593</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Landmark Scottish museum set to reopen in 2026 after major renovations - Travel Tomorrow</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Landmark Scottish museum set to reopen in 2026 after major renovations - Travel Tomorrow</t>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:37:51 GMT</t>
+          <t>Tue, 24 Feb 2026 12:52:25 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxORGJ2bWpnWEhuN0JwZ3pXU1FBQzYwWWxWRGZOTUFleFlQZmt1d3NKd0FwWjdzal83cXZLS3hxV201SmU5NHRyOGQzeURSampqR19yYnFfR2NSSnFSWllIYk9adGdBM25ndGFzTnc5LXk5MlVNdEllY05VUXh3YXJqbjk5eDVMTGxTZ3I4a1NacjF3bFUzTTZCZFVQT3BneEk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46077.48461805555</v>
+        <v>46077.53640046297</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Hungary Blocks EU’s 20th Russia Sanctions as Oil Row Sparks Explosive Brussels Showdown - The Times of India</t>
+          <t>Streit bei Auto-Kauf in Aschaffenburg: Männer gehen aufeinander los | Foto: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Hungary Blocks EU’s 20th Russia Sanctions as Oil Row Sparks Explosive Brussels Showdown - The Times of India</t>
+          <t>Dispute when buying a car in Aschaffenburg: Men attack each other | Photo: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 17:55:34 GMT</t>
+          <t>Tue, 24 Feb 2026 12:34:53 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOTlJDdnZJcUhhajNFWEtvMldrV0NBVDlQbThJYXI2MVBCbktZNWQ4dEtWVEc1bW9KT0RkRTFGcENzamNHQXd2STBjMVRQc1N5S3pvdHJ1TGFjeTc0STZMZ0t4MFY5RGJuNnowc3ZFcDRaV1VZQkNqNWF1Q21hcEcyc1VqTi05SUl0eF9nQ1lYYlFoQXNuWjdsM3c5TnNUeGliX3dvLUdwSWk0YzY0eENTb3hhNDJFN3VBMHZpRlViQ0lrcVkzLUFXS1BGdzNyZkd2ZDBMdzdEU1JSOUxHV0ZsdGZHRU9LSGl3SHpRQnd4RW5YdS1Udlp5S19jVdIBgAJBVV95cUxQSno4aUl4RDNXXzh6UXNFdWJyMHh3SkJzbEd5NFI4ZE5PRFRHWE10ZllZXzNVam1LdXZWYnBaeU9PYkJvcks2VXRLeEZlRFR0VFp1N21XZVdiMGZXaGszMER3OERaR0hHbDREYndvQ0ROdmFEa0l1dkFxemVRNkJBOGtNVFNWQjJpeW5DWjFneTBBMDlQbjlOVXRBanNybjNMR2ZZQkRyM1lRUDNHV0YtT3pYbVAwbTNuX1BBckZRa3RfeHd1SHhlOVZheldMTzh4eEZuWkZWa2VTWXNfaDV0TWx5a2lqcm4zZmhDaFpEQ09PMXhlYnRVRDJqRXNQdERG?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQNXA4Vkl0TlZ2Ui1SOTgxNWVUcF8xdXdtOUJsODFOalIybVlxTkU3SURZVHc5aTFsdHNHMGR1SXNvNWZGdlgyT0dzbHZmbmtQMklfbERteC1yMWw4WFVvUzhGSWQyb1J6X3hPcmRBVkFfVkxMbEtkWDMtbGZWckV4LTZVLXBvUUk5ZEFNMlJ3SE80TXZ0V2JEakttUjJkWmtoX3djX01wY2dUbDhoLXQtRm1qVXpwZzlfM2UxWXRTYng?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46076.7469212963</v>
+        <v>46077.52422453704</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>EU adds eight Russian officials to human rights sanctions list - The Straits Times</t>
+          <t>Kleiderdieb in Untersuchungshaft - NOKZEIT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>EU adds eight Russian officials to human rights sanctions list - The Straits Times</t>
+          <t>Clothes thief in custody - NOKZEIT</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:16:00 GMT</t>
+          <t>Tue, 24 Feb 2026 08:58:15 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQTU1vZDZ1QWVmS3RBUktpb3I4a3pkN1FFaGtkRkl3U0FKOUVQUF9Ec0VmVld3ZHJXQ3B6aGpZS3dxU3hzdms4Y2w5cGZWZGw5UlZmenVlRl9ZdkZidEd2OFUtRll3UlFIbXAzTGpUeVNhZUZlVUlBbUp2azdxYnROMDRFYmRYOFhVLTNMd3pWQXhmaUg2Qk9LNDdxd3BxM3BqelAtSVctWXNPVzRETmZySFZLcjdDcEpDR3BOTnJ4X1l1dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBKUUNfaWVwNkcxMmtpalVDTWxaMGNYQl8zZEVkWlFUMVk0UjFYa0Y0OEpFMERfaGMtSUI1dlU4cHVxLUJJMWxnV3FMcFdnNnQzc2s4RVVnamxfLXRxRjR3a3VYNkd0Q2pTcGVPb0lpTFE2ZE9KZUE?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46076.63611111111</v>
+        <v>46077.37378472222</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
+          <t>Herrmann begrüßt deutliches Personalplus für die Bayerische Polizei - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
+          <t>Herrmann welcomes a significant increase in personnel for the Bavarian Police - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:16:00 GMT</t>
+          <t>Tue, 24 Feb 2026 11:06:28 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOOTRkZE1mSU1wNTNCODJ6TEt2WWtuTF9yMUR4c1BOb3ptMExaU0ZJSUFyek96ZnpGaHRGRFd6aElmLU9WeXN4ZEZZazVsLTRUNDREamdwTGlMLXhsSHZoLTYta2gxNlBzUlhmRkdCaWZub0xBQl94VTdDZmZhU2s5b1R5TWRpd3BZV3JDS1NTRWRsUjZtemdVLTdaTmkzVDJEVzRCNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNU0FPOVFwS1pZal9xUnlUNDVjT0wzY2xwRG5TUmdob3JERkNFdld6ZHdVTHJBdnAxOGl6VW5jeTNxMmxtWjZfSVdkczVTaVdTNFBIaEN0VzBTbUkzRHk0QlBJSEU0bEk0aVJIT0lsdnV6VE91WUZDMGRybGhMSmVMWEM1R2hId1pvN3E2Z3BOT2xYZk5vMm03Vjk3dHNfV3ZhS05OM3RqX3J0b25uUTRadzZLaDJXWk5KbzdmLTZ0OA?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46077.51111111111</v>
+        <v>46077.46282407407</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>La Ville de Bruxelles supprime une taxe pour l’installation de panneaux photovoltaïques - 7sur7.be</t>
+          <t>Würzburg: Messerattacke auf Zeugen Jehovas - Idea.de</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>The City of Brussels removes a tax for the installation of photovoltaic panels - 7sur7.be</t>
+          <t>Würzburg: Knife attack on Jehovah's Witnesses - Idea.de</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 08:48:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:00:03 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPRWg0V2dNa1lZdG1wUWp4V181cklFS3JlWnc0VkRIOEN3STFyRUtURmRRSlQ2U04xQlVMWERsbE12eXpqUDE4QjZPTFl1TDBOVzk4N0YtQzRGSXVYcE9QZDJnem0yZ0xGSkRLN0RWQzJfSDJYbDl6VmktQUQzMFZGRXBYcWpIX3J5SnVlWVlIeXlQVW0zbHNCQ0NNWXZyN2VXVWdLTWVYTU9BOGkwMGhWUmZDQ0o0aUg3bVd0ay04TjBWLWxo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE55UThGQWVSVnBMUGM3RFpMeDJJbjc2Zi00aVhuV1lVeW9rZmw0WXdNdmZFY0REWGpQZUtUelROVXl5RE9KMkhJNlRoNUNvN09sS3Z3aTVjMWp3N0ZWc05CZmdGeWVPUzR3VXhBMFNkTnVWWWNTOFlwcnJ3?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46077.36666666667</v>
+        <v>46077.58336805556</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Trafic de stupéfiants à Montignies-sur-Sambre: Un individu arrêté - Télésambre</t>
+          <t>Erfolgreicher Callcenterbetrug: Falscher Polizist holt Wertgegenstände ab, Kripo ermittelt - Mainfranken News</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Drug trafficking in Montignies-sur-Sambre: An individual arrested - Télésambre</t>
+          <t>Successful call center fraud: Fake police officer picks up valuables, police investigate - Mainfranken News</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:16:10 GMT</t>
+          <t>Tue, 24 Feb 2026 14:06:37 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNSXp2bmZ5TlN5YkZZLTBhalF5SmRHRGd4Mk50dWZZdW82WngwNXVXTDNSUXdfdWZET2t1dlNCcjZLTVdOY01DYTBQaVMzY3draDBabE13cHlYZ0xJeGNwYlhGdkNLU0JkMGZvSW5xZGZxX0FWLWtFRmF6N0R0TFlhdFVnZXNPczVNUG9zT0ZYMUl6TlFUQ09SbHFPeUZ2SFk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNRkZoQVNGWmlQVjB6c210V3RQRjYzeWxmU1RkQmJURFJhajlmQkVvRjI4V3d4U3AyQm1GajFjYUlteHcyYV9LcTQ3Z3ZMdklUbm9DemlqMkdvRnlTeHJJd1AzejlhMjlFOGJGYklWQlZ6cHRYekZYNkttNUFReWlieW5WVGY0aTRuVWRVZUZIRlpSZ1B5clJnMEh5VWtqVXZXbHZ3SnN5T0ZvSEJVa3h5X3hGdmxyV2pfSDVCejJ3Smd0NE9s?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46076.63622685185</v>
+        <v>46077.58792824074</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>La justice alerte contre le phishing via de fausses applications: “Impossible de distinguer le vrai du faux” - 7sur7.be</t>
+          <t>Helmstadt: Nach Einbruch in Einfamilienhaus – Zeugen gesucht - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Justice warns against phishing via fake applications: “Impossible to distinguish real from fake” - 7sur7.be</t>
+          <t>Helmstadt: Witnesses wanted after a break-in in a single-family home - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 06:20:46 GMT</t>
+          <t>Tue, 24 Feb 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxQOHpEb0RWNVpvS08zNmdON0xCMzUwN3VHZ21lcnFtS2syVEd6ZVAyNVJSdmduUy1vRVhpOUwtaV8xSksxVHA2UkNmRm4zQk5oMkpUVUplQzB4QU92SWRFTFNrQjZ6M0g3di1FeW1ZM1dXbmEweV9ISTRzZUR2ZUg5NVNabHdNajZRdE43bElzZVBodU5NUzl5OTZsMGJvam1fdTBVczE4RHc5UE9sd2NkdDFSNEdmNnF0X0ZLMUtzbllsZzhzbDhXVXB2UkF2S0RkN0FPcm1SaW9pNW93Z2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOeHEydHhfR29sSVFqWENkVEU5ekVMTnRTcmFoZXhIeFJNVTMzSGN5dzNjZjVtZVk0TnhtSjRNUmRTRC1OdndqNVV1MDJadHZUdlU5UjBtTVV1b2k0TC0wX25XXzdGQnk4VVR5Rno1akhMM19aOGRNZURrcmJ4cEh2Z05UVFpqQURvalNLcU8zcWZ4RG1PdWc?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,52 +2825,52 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46077.2644212963</v>
+        <v>46077.58333333334</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Opnieuw laadkabels gestolen, nu in Maasmechelen en Lanaken - VRT</t>
+          <t>Unfallflucht an Rastanlage Spessart: Schaden an Kleintransporter | Foto: Stephan Jansen (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Charging cables stolen again, now in Maasmechelen and Lanaken - VRT</t>
+          <t>Accident escape at Spessart rest area: damage to small van | Photo: Stephan Jansen (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 16:16:31 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:26 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQLXpEcnVvUUFXZTVvb0o3cEl0bG8taUR5R3ZmT1RybVhhNDBXeHFaNHZ3TWlabXpySzljU3JiTTlPc09uaElITUlISDhBTERBcW10ZEdvV3otMG4xZm50R1IzOEpzX05sVzVMb3VwMGNyenk0MWNIYlY3andhSWpNdWQ4d3NNTlowbGZDV0FXYTNLRHc4RjdaczdLaTJiRG8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOQkJUQUtFSW5nMU05Unk5Vmx5ZkJXem1XV2JHVEFKSjBISGN6OU5wZElaUjlWZ0pZMGc0MHlJcEJqcDRSNy1od1dCY0dQdUZVX1VWdHJwSk9aMUljaXoxLWxmbWdZSnhMU0EtcE9DXzlRQVEyNVlpd1R5NnVvSElCVVF5TjB2VHZpLVpOUTJvYkdTVHlSTVhudzI4YmI0YnUycUpFLWtFMndDby04OU1aRWVZY2MwQmVKTE44?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2880,52 +2880,52 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46076.67813657408</v>
+        <v>46077.54405092593</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Vakantiehuis Fabiola in Maasmechelen voor kinderen met een beperking krijgt toch nog 1 jaar subsidies van Vlaanderen - VRT</t>
+          <t>Frammersbach: Falsche Spendensammler - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Holiday home Fabiola in Maasmechelen for children with disabilities will still receive subsidies from Flanders for 1 year - VRT</t>
+          <t>Frammersbach: Fake fundraisers - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 07:52:45 GMT</t>
+          <t>Tue, 24 Feb 2026 14:06:56 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5OenpKUkhrQ1AxTlBhUlRETGdRSFpRaVJKOW9TelBUUXdpU01tdmEwZ0VFM2dvR05IaFViZkVWM0YxLVlwU2ZETUxJbld6c3NrTm1DU1Z1SWlzZG9PNWFyZEJMSEVyX2hCY1BIa1RGaHdtQi1OQU9pR3ozdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQmphdE5lMlFNZTFQYTdWTzBNU1pHMUc2YWlxZXFPc1BZWlBWZ2lnME9Xa29OcmFCeE5XeTlZS21YRTVSeGU1OEUtOHdCZTNwZE1CWHoyQkl1VlZfcDJQQmphOGh6V1J5YWs3cmhLSmU5Z2tFbGJuWGJBQlZxbEJPYXo4T2stUlVW?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46077.32829861111</v>
+        <v>46077.58814814815</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Halen keurt aangepast meerjarenplan goed na budgetfout van 5,4 miljoen euro - VRT</t>
+          <t>Obernburg: Unfallflucht schnell geklärt - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Halen approves adjusted multi-year plan after budget error of 5.4 million euros - VRT</t>
+          <t>Obernburg: Escape accident quickly resolved - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:32:52 GMT</t>
+          <t>Tue, 24 Feb 2026 14:07:44 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPOTItcThiT1hZQjVXaDA5TEI5RUlVdmt5N1UzR2hEelF2aVBXemRfcTdNbk9xUk5sY2NfWkpJdmIycHN5TThoaVNnVVpCWjgzYXExeFpZUk91bVhhdFhiZ0szcDNRT3Nua3RCSTVUa1BTSGRUdU42TXJ3NzVYSXdFMTRZMkwwUVpqaURzNXJMMVIwbk1rNzNSQVdVaUVvdHRVNGNWcURCUzA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQWDdoMzlzRi04dVVnRzU4ZmFHbElQdTh1SFVrZWFJakZUYUVRQlk4MExVam5lb3U3XzFWVy1keWczZzJ1a3pBai1GR0E4bDRYR3JiMWY0UVVtb0ZDaFdaR3NCa1ItcjRSajg1Ny1kOFJFaFI4VWVnd0pBR1FfMndCNFV5SFFIQVgtVml3ZFUwc3kwX0hvUzRURDNwVDdkVHV3czBQVTlR?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46077.39782407408</v>
+        <v>46077.5887037037</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Booba : un procès requis contre le rappeur pour le cyberharcèlement de Magali Berdah - CNews</t>
+          <t>Blitzer in Aschaffenburg aktuell am Dienstag: Hier nimmt die Polizei am 24.02.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Booba: a trial required against the rapper for the cyberharassment of Magali Berdah - CNews</t>
+          <t>Speed ​​cameras in Aschaffenburg currently on Tuesday: Here the police are targeting speeders on February 24th, 2026 - News.de</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mon, 23 Feb 2026 15:03:57 GMT</t>
+          <t>Tue, 24 Feb 2026 09:18:00 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPOFUyODdiVzRYWEh6cWZKWlY2M2UxQjZJcy1PSEJ5TDNDQ1dhVDVfSjUyOWcxQlNsaEF4Z3NVZDJTc2J5eEpCZ0hyZjFYYTY1a1RKbWtTUTdFellXWndJOTZZckROSzNsekdYM2k3VzBJc3htS0t6djc3S185RUJSZl9fanMtNVVDWXlQb2RkbjRZQy1tbDJhQ2Jxcm1RbE92UFRONDlOZmlDRTRES014NjB3SVZtSkM1U1FQTXp4R0F2UdIBwgFBVV95cUxPOFUyODdiVzRYWEh6cWZKWlY2M2UxQjZJcy1PSEJ5TDNDQ1dhVDVfSjUyOWcxQlNsaEF4Z3NVZDJTc2J5eEpCZ0hyZjFYYTY1a1RKbWtTUTdFellXWndJOTZZckROSzNsekdYM2k3VzBJc3htS0t6djc3S185RUJSZl9fanMtNVVDWXlQb2RkbjRZQy1tbDJhQ2Jxcm1RbE92UFRONDlOZmlDRTRES014NjB3SVZtSkM1U1FQTXp4R0F2UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPTVBpWlNVVWhJQTJIZ0xMUkVmR2dOWmtjZkxfaDJIcDJXUHo1Z2d0T0RGOVJXdmVmRV9PQ0p1ZUg2dlVaYXhqVERySGpCM00zeGlxNnZWMjZfQzRPZzhHTFRrODVTNUlLcFRGTnpQQzJFa3pZaDNjQzRaOGpMWno3Z3ZZaEpma0xtbDVzU3I5TV9EaGVnbmpHdzlWRUxmY3NMeFg3RnhxWDRfZElOeXVDeXVXZnpaaXNwTjNWc1IyaXNTQmZMbVlZa09qVURBYTJsQmlUdDZXUEVEeDFXZHNPZE9TQmtiSmk2M3puY9IB8gFBVV95cUxOeHd5dHFsS0VxRHViWnMwbzlwYjl2VFhheTA4a0xFTjNCcWM0S0VQR1ZkRms1eVFWdzVrcUp0RFhhSkZqRE1fUmFVd3VQVVZWVkNrNHE5Y2g5U20yMlNKb0h0T0MwTVRsRkxoa1pvdU52MzFNUE9ac0FBdjRQTE5Xbko3cjNGaTkwX190N2wxUjljcGRsLTJJZEZfM2h1aHVFcTBkYUJLaExSMm9zUXQwRE5hd00wVVc4YVMyQ0ZfQWlJU3B5Y09obzh0bHFBUGpsWmw4VC1mUFd3dmVxUS14b09IRGhxeEhzLXQwV1MzdnVZZw?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3045,52 +3045,52 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46076.62774305556</v>
+        <v>46077.3875</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Courtois va investir en Belgique : deux clubs mentionnés - FootNews.BE</t>
+          <t>Corona-Zahlen im Landkreis Aschaffenburg aktuell: Die Coronavirus-News aus der Region - News.de</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Courtois will invest in Belgium: two clubs mentioned - FootNews.BE</t>
+          <t>Current Corona numbers in the Aschaffenburg district: The coronavirus news from the region - News.de</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:39:21 GMT</t>
+          <t>Tue, 24 Feb 2026 10:39:00 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNTlJDdTgzUm84dnhidVNwNUtTZGJqbWZZOVJmSHBzU1QyYmk4QV9ZanJ5TG12cXFKVDhVSHplR2dudWVsb3RlWjZUd0FpVmhHZFJfQzFnTlpvMnJwX2Y1Q3RLY1lzTlNWQ0JNSXAyalBMNm9YazVTenlGUXdranlMbjlwWUpSSlppbjF6SXU1aGJJd185?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxQaUEzVnI1RndRNXNjVEEzZ1phUmhtempTcElXZld6R1lVQTZuYmFKQWdYN25qclF5TE54T0UzTU9iWnZSc0RydTlpMGRjZ3ZyM1hWZDh2SlBHLXJPTTN2T0d1SDJkT1RSU1FpckR2bGQ3MHlTU2MzWU1WdUVtTnRvdzN5LTJSRVJ1Q1dqMFlOS2lia1E2bWNxZ2RUMzhzS3Z3Q1ExcHlyYUxydTFkU0lIZ2hIMlZNRDZXZmlOREFzVUs2YmxrN0lOZ0FDWGxCZzIxY1djYl9RLUJGeExvOG9VZ0gyTF9WODdVdVp5LS1WOTZRNkNlQkwxZWdBZG01VmPSAYQCQVVfeXFMTUphRTNneGpNMmxrczR4aGUtLS1PT0swYXJ4T2RWOWVvZU5XNG4xckFrSm8wT2RSVUNCSG5GQlJCcm9vX1p0THJITHAtN0xldjhacjR2VXFfUWVCdXg5SjFlSEpTN2lQLVE5M1AzcjhVdEVTa3ROV0tFbmNhWlVmcXBjUUw5ZzFfZkE1amdCdFZxRkd2c2x3dk1DbXRYR1FBWW9sY1g5ZjhPNXE5WXF0U204Z3RHWlVGVDlKdG1YeVAtYXB6ZGhoZ3pXMEp0cTNyS0o2dXhGRDFDV2JCYWlWbDFfXzZVVmJ1RjRKV09aZzNqZ3pETERxU2cxUUhYM0dNZ0xlSV8?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3100,52 +3100,52 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46077.52732638889</v>
+        <v>46077.44375</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
+          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
+          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:32:37 GMT</t>
+          <t>Tue, 24 Feb 2026 13:17:11 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNRHZ4dm0tREV0cjFucHowcUNrWGlJTVljdlFXcjNtdFg0OUh4a2hWb25ucnlzMkNMdThqU25BNm1yaHhBRk8zTDRwcHdHRHZFRUNBSVlHcXZjdDJFQU95SEVCM20wQm1YNmFzczRjdzE5UmZUY2NpWldzMWRfdXpSVmo4ZlpsVHdNOWo1aVFGcVRBc0I5RjVyYkRGeXZmVTBGZkFvNy0xZFVxa2JNZ0RzeGt2dHJCZTZHUTU1RXRZbzNpQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOYl8yTkRYaUVVaUU4eE4wZk1aSTVxbkNEVzg5MHF5aTI1bGZnZkxweHgzM3MwUU9BekdUVVNlV3pPV0J4NkJuM0ptYzlsa1JxNUNCZjNqdmdldHkzRnNMSnpidGhTb2h3LUYwR3VXU3BnX1Z4ZDY0dkJRd3JiMUpYT0FZbjVyNzJf?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3169,38 +3169,38 @@
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46077.56431712963</v>
+        <v>46077.55359953704</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
+          <t>Sexueller Übergriff am Bahnhof: Kripo Ingolstadt sucht Zeugen - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
+          <t>Sexual assault at the train station: Ingolstadt police are looking for witnesses - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:08:23 GMT</t>
+          <t>Tue, 24 Feb 2026 14:34:12 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPNExOajRSMzJtQk9kOENCeXlHM25OUm5vVWQyUkszamgzQjVOMm92anAtdHN2QXhFLUVMLUptNVJ0YzV5dFJWTE5OeVNCMFVobnlyelUzeFBadlNFV3hCRVI0Y3pUTExVYU9TNFdwVUNsaXhyQjc2QW5MZlh3Rk9rejhZUDhEU1h3LUVQWHhBWHNHWG80NUltV2hxd1YwWmhRVVZyOHotOUdQeEp6UlVQYi1iVDZWcHFOanBzWWFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOYVpQc2ZubWFubEFJeVhURXhHUWlPa24td1QzXzVWS0dmdEJCN0VVRGNfNjEyZjNuTEZyN3IwWWo0cFQ0SjRYQUs2VXBJWGUwMXY2ZG9wc2V3UmM2WW5ZaUZkVTNWXy1mcVpNcXd2NE5SRklKSDh3aklIcUMwWDJnSGxyNms4N2ZETzg5QTQxZzd6Q1dJQ1B3akVZMkR6UElYenU3clBPOXRLaTNmTGVxYjdLU0NsQmY1ZXJEcVBSWmVlZGpmZS1BeFBqeUFZQXdJaWZKRHBKbw?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3210,52 +3210,52 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46077.5891550926</v>
+        <v>46077.60708333334</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Village Maasmechelen (fallback)</t>
+          <t>Village Las Rozas La Roca</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Maasmechelen Village" OR "Maasmechelen") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Las Rozas outlet" OR "La Roca outlet" OR "Las Rozas Village" OR "La Roca Village")</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
+          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
+          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:03:27 GMT</t>
+          <t>Tue, 24 Feb 2026 09:21:06 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUW54aFlQc196RnJXM0FfVWU5a2JSN2w2MXdiZVg0Z2U2aXdKZENsNThtVWVvQjg3U0FwUUQ2Qk5SZF9rSnVqQWxrc1VzOUNzcVRfbWVXNWFCUW80ckl3MHJlaTZvUElidlBqZWNlSm85a1otTXNBMkpYTlQ1YzJBcDVNNkY1a2o2OUJtNG1HYnItU2RodXRXb1pXMVFOTkF6ejk3cEY4ZTdRbTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPd0dBclgxSVlFV1dtaEgzNklSZENrcDBPVF9kbEZOWUZhMGtfS3BsS01WWlpwMERQMHVtUUcxaG1EaFlyV3NONy05ZlQ1TzRPTG9lVDUtZE5xVVZEbUdBTFdkNlB5TEhTb0FmSWJlOFpqTXVVLWhvd1JaYzkzNGNMaVBmaGpSaWZ0dHJ1cnBXQndERXZMN2ZhSWJSNlFPNHQ5MFMwbUF1WHRIXzBXOUxpQmtYdWgyNlpDaVhEdjcwYXBGLUtQNzQwdw?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3279,38 +3279,38 @@
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46077.5440625</v>
+        <v>46077.38965277778</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Wertheim Village: Polizei stoppt mutmaßlichen Seriendieb - Fränkische Nachrichten</t>
+          <t>Zola Predosa (Bologna), sparatoria al campo nomadi: «Un pregiudicato colpito alle gambe» - Corriere di Bologna</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Wertheim Village: Police stop suspected serial thief - Fränkische Nachrichten</t>
+          <t>Zola Predosa (Bologna), shooting at the nomad camp: «A criminal hit in the legs» - Corriere di Bologna</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:34:00 GMT</t>
+          <t>Tue, 24 Feb 2026 08:41:43 GMT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNempGdjdfTkxudlBkZnlNYlNUS3h0MEluS3JYU2tOVW9zamM4QUdCODMyNTAwc0ZDY0NCYXpReG9wOTVtOUY2eW9rWmhxT0RHaUdubGNoWVN3SjBCaE8tSlBpSTlneF9aQnNMdHR0VDI3Wjk4el80OU91akJGYWV4aVVuM01SejN5NC1rQlg0WElRd2VJbXVhZEtjZEVwdDAtYlZnSFFjazhjOExOcGszYmt1X0hEUlZyQjl3aTRWXzZxWHJ1NXlJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTXZ3cFF6NURKMDl5cGZSWFJWQ2ZRWk95Z2ItemVwYmlVd1BhMm9LX2Z5YmJiOFp5b2lNVE00TVdpWUlnb2VLd3B2VnJnckU1R096NU5nTFM0dmFlU2o1WUlWakN2dkttY2Z3YlZ6akF5TnhZb3g5QkV2ZXRXSnRvR0IxZ1dRMjMxWmVaNUNTcXJIaUVYVXp5eXdwdUN6ek54Z2o2dVdybmwzUC1MS1pBMjQ1d1g5UWZFSXQtMi1MeXhleU9LWlBMeV9HaUhDczQ1bmRIMVVxaHZKR3hsWWZ0c05rUTZ5ZXFpWFdV0gHwAUFVX3lxTFBIZXFtcm93OHQ3bmZIcTdUcXV1VmN1Tm56S0dld3pCVDEtS2ZYdVB1bHYwNzBqUjhyc3ZhSUM0S3p6b09JQmtiOWI3ZmlfOUs5OWxMci0tX2NFckV2V0VKQ3Uxam1rWWtEa1dpdWdZcHA1T0JVLTVneS16d05NVmxJVjBOMDdDcHJaUW5lYS1JamdtcGFlMHhneTJkTE4zeWZtbXhNZWRtWUZQbHpIR09sNWxGZ3ktLVVVSVZlWG55eXYzX3BQV0M0MkppUVlNWU1PU3czUnRMTUNRVkVzWUlyYWhPZGs2MUFULTU2RnNFcw?oc=5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3320,1120 +3320,20 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K53" s="1" t="n">
-        <v>46077.39861111111</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Reichenberg: Frontalzusammenstoß auf der B19 bei Würzburg: Zwei Autofahrerinnen schwer verletzt - Main-Post</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Reichenberg: Head-on collision on the B19 near Würzburg: Two drivers seriously injured - Main-Post</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Mon, 23 Feb 2026 20:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxON0VPNERZb21RaF8xWTQtUzVObjNuUUw5LXpNbEVyOGtLQ3I2eWc2STlOUEd2OTU3UUVMNlVhNlRvTGFSQmxvb181ZkxJNzFtQXI5NGoxZHJPZ0gtbUVBd0l6Wm96UjREZ3JnV3dfNjYyQklGWVlSUTVLRjZrRE5mU3E5dVFaNU5WdE0yblAxWHIzR1hJdU1JVFEyZnEyMFVneGhHTl9UVF8zYnZPTVM2bTQtT3l1RUg4WFc2WHhVekMxVTZCRmo4eXA5THhKRzRibTE1UkpFaGJqYW1qaXhZZ3VJcFpVYUVrNGh6Qkc2NDQyS19FMFItR2E4V3k?oc=5</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K54" s="1" t="n">
-        <v>46076.83333333334</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Streit bei Auto-Kauf in Aschaffenburg: Männer gehen aufeinander los | Foto: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Dispute when buying a car in Aschaffenburg: Men attack each other | Photo: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 12:34:53 GMT</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQNXA4Vkl0TlZ2Ui1SOTgxNWVUcF8xdXdtOUJsODFOalIybVlxTkU3SURZVHc5aTFsdHNHMGR1SXNvNWZGdlgyT0dzbHZmbmtQMklfbERteC1yMWw4WFVvUzhGSWQyb1J6X3hPcmRBVkFfVkxMbEtkWDMtbGZWckV4LTZVLXBvUUk5ZEFNMlJ3SE80TXZ0V2JEakttUjJkWmtoX3djX01wY2dUbDhoLXQtRm1qVXpwZzlfM2UxWXRTYng?oc=5</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K55" s="1" t="n">
-        <v>46077.52422453704</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Herrmann begrüßt deutliches Personalplus für die Bayerische Polizei - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Herrmann welcomes a significant increase in personnel for the Bavarian Police - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 11:06:28 GMT</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNU0FPOVFwS1pZal9xUnlUNDVjT0wzY2xwRG5TUmdob3JERkNFdld6ZHdVTHJBdnAxOGl6VW5jeTNxMmxtWjZfSVdkczVTaVdTNFBIaEN0VzBTbUkzRHk0QlBJSEU0bEk0aVJIT0lsdnV6VE91WUZDMGRybGhMSmVMWEM1R2hId1pvN3E2Z3BOT2xYZk5vMm03Vjk3dHNfV3ZhS05OM3RqX3J0b25uUTRadzZLaDJXWk5KbzdmLTZ0OA?oc=5</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K56" s="1" t="n">
-        <v>46077.46282407407</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 05:25:22 GMT</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K57" s="1" t="n">
-        <v>46077.22594907408</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Unfallfluchten in Aschaffenburg und Kleinostheim | Foto: Dirk Ceelen - main-echo.de</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Accident escapes in Aschaffenburg and Kleinostheim | Photo: Dirk Ceelen - main-echo.de</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 13:03:01 GMT</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQMW02WVZqN19mTERhVXdiT194SUtPU2ZxVTJ3dGNKd2ZLQzVmM2lxb3lTdWpHVjBqOVlFTFVOYXE0d0czbUpZQzFFU19OT294MmdqVlU3d2M1QzFWUndPbm02SVBvakFlc0tVSnl6YXJjOUNaN2FvNUYwX1pOOGJ3aVJoZjlPOU9DWnFRZlBlZG5uNXN4N3ZvWnpYN21VX2M1Skppd2c4Zw?oc=5</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K58" s="1" t="n">
-        <v>46077.54376157407</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Marktheidenfeld: Polizei kontrolliert erfolgreich - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Marktheidenfeld: Police check successfully - aschaffenburg.news</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 14:09:08 GMT</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNM0F0V01ZMjFGbzFpQ0FldUNxRnI4UkplZ2daMUlzTXNvWGM2WnlUZGprenhxMXBfSkRrLTFkWUU2c2VFODdxRTU1bWF2bVNZeW9zWWVPaEtGU0ZfdUdGbVBKOGt3dEdmaUszMTdlZnFuNUV6b0JWUEFtVjBlTmdFQXh5SXhuZTN2eVVzelU2Z29RUU9wNGw2Z1Vn?oc=5</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K59" s="1" t="n">
-        <v>46077.58967592593</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Blitzer in Aschaffenburg aktuell am Dienstag: Hier nimmt die Polizei am 24.02.2026 Raser ins Visier - News.de</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Speed ​​cameras in Aschaffenburg currently on Tuesday: Here the police are targeting speeders on February 24th, 2026 - News.de</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 09:18:00 GMT</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPTVBpWlNVVWhJQTJIZ0xMUkVmR2dOWmtjZkxfaDJIcDJXUHo1Z2d0T0RGOVJXdmVmRV9PQ0p1ZUg2dlVaYXhqVERySGpCM00zeGlxNnZWMjZfQzRPZzhHTFRrODVTNUlLcFRGTnpQQzJFa3pZaDNjQzRaOGpMWno3Z3ZZaEpma0xtbDVzU3I5TV9EaGVnbmpHdzlWRUxmY3NMeFg3RnhxWDRfZElOeXVDeXVXZnpaaXNwTjNWc1IyaXNTQmZMbVlZa09qVURBYTJsQmlUdDZXUEVEeDFXZHNPZE9TQmtiSmk2M3puY9IB8gFBVV95cUxOeHd5dHFsS0VxRHViWnMwbzlwYjl2VFhheTA4a0xFTjNCcWM0S0VQR1ZkRms1eVFWdzVrcUp0RFhhSkZqRE1fUmFVd3VQVVZWVkNrNHE5Y2g5U20yMlNKb0h0T0MwTVRsRkxoa1pvdU52MzFNUE9ac0FBdjRQTE5Xbko3cjNGaTkwX190N2wxUjljcGRsLTJJZEZfM2h1aHVFcTBkYUJLaExSMm9zUXQwRE5hd00wVVc4YVMyQ0ZfQWlJU3B5Y09obzh0bHFBUGpsWmw4VC1mUFd3dmVxUS14b09IRGhxeEhzLXQwV1MzdnVZZw?oc=5</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K60" s="1" t="n">
-        <v>46077.3875</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Demo-Termine heute, 24.02.2026: Hier gibt's am Dienstag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Demo dates today, February 24th, 2026: Here on Tuesday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 06:04:00 GMT</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPTGdUUkg2a1JYTDFRNDFrZTJfejZYeTZZc1dOeC1sYkNIOVQ4eXFXU2t2X1BXaTJsaHlsSmJXcUM1MWlpVmdXZXpBZ3ZiOUpPd2NhOG1OSUNfZWRhR1o0dEVWX2hZT0pCVk1WMmV6T1BmaFI3V0lEYjdrTUlPMUZvM1hMdHd1UWdnak13VFlMa1FydXF0cUZWd2ZTRjJWaTBCNmMyelAtdlI1Z3kyNndzZ0NSRjNkeTYwZWludW9WNVVPWThLbWw2ZXRpU2ZMdUxXcTZZOUllbG42OGp1dDBpbXlWeGE2X0xOakFnYnpxbXoyWE1HVks5bDZoVUs2QTMzbXpTWVh4a9IBjAJBVV95cUxNVlA5c1FOUjBhdmxMUWhDQk8xbDhPTFlENjAtM0hCS2pmX0M1VUZxcC1WblZQTWdhRjlhT2NWbUZWSG5NZWpLby1sYlJMTnA0X2JFeWNNcVFvNHpqQlJBcmY2VHc1QTYtc2xnTEVFRlFGTXRnZDFRNktpTFFVTG1vRmhtSGtvdTRDX0ktZm9QanY3SzBLTFo3enRWc3hSODJIejdMcGFqdGVpU3owaF92NmdKNkd4ek9OMFlfcE5pNldoNExVOGU5VjIxUDB3alBORWFRM0pRWXJVT0JlSkR3TmJOaTZhOWxQUncybTNxZGFpN2NGRWdCU0N5dE81blBrSUxjbld6cHBRc25X?oc=5</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K61" s="1" t="n">
-        <v>46077.25277777778</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Village Wertheim (fallback)</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Jon Wertheim suggests the reason why Serena Williams may return to the WTA Tour - Tennishead</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Jon Wertheim suggests the reason why Serena Williams may return to the WTA Tour - Tennishead</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Mon, 23 Feb 2026 22:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNdXRXQ1JpcjVLX3Vkd3RzbW5VMWR1SW1qQ1hwc0RfUi0xZG5nQktYRXhYcEstZ3BSb1pMVU8yeklCS3dycGdhMW14WVZKVUdyOUtjN2YwMllOQ3JxOGo0VVhCX1VCM3AyLUFQVHMwZzZDbXNKb0prSkJITVlJbm1ka0ZDY2g5X3hJQ2llel9EM01mdjRaYklTazA5dHA0WGU0LUdmeHVn?oc=5</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K62" s="1" t="n">
-        <v>46076.91666666666</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Unter Vorwand ins Haus gelassen: Täter stiehlt Geldbörse einer Seniorin - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Let into the house under pretext: perpetrator steals wallet from senior citizen - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 06:42:59 GMT</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOUzZOZmpZeWJ4MGZ6Z003ZG5oYVIwZDhtN2k1VU9BM2FSLTgxWXlxcDc3eXBBOUxVY2h4SzVXU29tRXpxZzBZZW9mNFhGbXg1TWVRWUIyQzgzaGZac2N5c28wZ0pyV2hUWEhfblk2cUpGMFZmNDV2QTk3a0JZNXZfTFRqTUppSU1rSVRQa2NvSTlTX3ZEdE56U29HWTdSUmM1QXAyS2JGNkZzZ0llNm8xY1hLNWN5MXVsRHhLV1J5bGhmN3pRczRQZ3BLZXBSbVFETkZ3UkUzRURrNk0?oc=5</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K63" s="1" t="n">
-        <v>46077.27984953704</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Polizei stoppt 66-jährige Autofahrerin mit 1,6 Promille - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Police stop 66-year-old driver with 1.6 per mille - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 03:38:40 GMT</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNZ01KNnczSFRPLTlLZUNzb1pXWTBqbGR0LWxFTXR0ZHZWb1pza0ctYmFSd3VmRUhLcjdsVXZDS1d5NUsteUN3b01FSW9lZ213MndZMWxnUDlFTkVYcnJZQjg2Mkg2WmdOSGpSUmZNeERVd3pHUlhwMjJva0JQWlNfS1lFREcyVmZfbzMzMkprZ3dlRWVWbzRKd3ZQLWhVS0FrMFVDUnRMMXRNdDN6NDhRbFhndzE3Zw?oc=5</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K64" s="1" t="n">
-        <v>46077.15185185185</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Schwerer Auffahrunfall am Brückenkopf Ingolstadt: Beifahrer eingeklemmt und schwer verletzt - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Serious rear-end collision at the Ingolstadt bridgehead: passenger trapped and seriously injured - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 07:57:13 GMT</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNb2w4ekV5aHlhNHcwSEJKaUlBN2hpd0ZVUW56eHFPTXlFMGVLYjkyMVRPT0hUTjllLUdONnY1bExmUUJnSk9SR1lmQTBjZV9oV1JHNWQwV0RnTXB2Q3ZPdFR1di1IZjBETzFJd2FTY05aYmE5LWpsdC1nSGI4X05ENkMyelJvazdFeVFJSkN2SUZWSUZLWm9fSk1NRXFjOFhhV3I5cXRLZmJJNkFyRDVSS3Z5Q1ByMVFpV0V4VHVKVXUzalJIQ2pHSkl4WU1YZU5xbjdYbldYYlJHV3R2Z2JtSDYyazE?oc=5</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K65" s="1" t="n">
-        <v>46077.33140046296</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Sexueller Übergriff am Bahnhof: Kripo Ingolstadt sucht Zeugen - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Sexual assault at the train station: Ingolstadt police are looking for witnesses - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 14:34:12 GMT</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOYVpQc2ZubWFubEFJeVhURXhHUWlPa24td1QzXzVWS0dmdEJCN0VVRGNfNjEyZjNuTEZyN3IwWWo0cFQ0SjRYQUs2VXBJWGUwMXY2ZG9wc2V3UmM2WW5ZaUZkVTNWXy1mcVpNcXd2NE5SRklKSDh3aklIcUMwWDJnSGxyNms4N2ZETzg5QTQxZzd6Q1dJQ1B3akVZMkR6UElYenU3clBPOXRLaTNmTGVxYjdLU0NsQmY1ZXJEcVBSWmVlZGpmZS1BeFBqeUFZQXdJaWZKRHBKbw?oc=5</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K66" s="1" t="n">
-        <v>46077.60708333334</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Alin Coen live in Regensburg: „Du bedeutest mir die Welt“ – Ein Konzert voller Emotionen - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Alin Coen live in Regensburg: “You mean the world to me” – A concert full of emotions - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 03:47:07 GMT</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNaGZyR041TjVBbXZOa0NudVppUlh4Zm1Gc1BFNmwzRmFaZjNvMExzaHBoMmh4Y1plTUk5QW1VM0lWTHNSMmN0NmJsZmlkbHpZa0dxdGhzMzNvYnhlOU1BRnlOeHdUclJKLWNjaUhHMWNFWFFxMDBjYlJWcUtidGJKQVNLOFNia1laaWVXbjR1N3JkUlQyS2dLTGZ5Uk56SThmQXFRMzYwaTVYam9wdnUxZndURUxSSEx2cDl3S1RDVGhub1dob2pxeWx0TTltXzN2bWpFVWR3?oc=5</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K67" s="1" t="n">
-        <v>46077.15771990741</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Beifahrerin lebensgefährlich verletzt: Stundenlanger Stau auf A9 nach Unfall mit Lastwagen - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Passenger critically injured: hours-long traffic jam on the A9 after an accident with a truck - Augsburger Allgemeine</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 05:08:22 GMT</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQRXl1MWhlRzRsY0RRYVZPdTBPWG9FLW9TdGl2QmdMenY2b3EyeFNGZGdZMVNoajRVc3FWeTBUeEZqanVrOEpmUTF1SDdtblFVYXRhOG5RYTcteGZqRnBLUVJ4ZTgxU2hIZ2x4dGxfaFRYN3ZIYVplS3A4VjBHVnBrU1AyRGhtNV95VDVkREo1LTJYSThBUHRJTS0weENUekpNaU9ySUlUY1g2YnJVa2E3RnZhRnV6OHQ2VnNJT2VpZ2M2SklKdmZN?oc=5</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K68" s="1" t="n">
-        <v>46077.21414351852</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>SPD Frauen Ingolstadt fordern gerechte Gesundheitsversorgung für Frauen - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>SPD women in Ingolstadt demand fair health care for women - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 04:53:13 GMT</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQWTVvZndQRWxzYWswTXQtRHNrV01FQUwwRlRsQXlqS1h4V3NPZVNsRlMyelVnd2FPV3dJSHY0UGk4cExDb0FIYkV0aGhRX184WUxRLTdpRFB5dXR2WUQxYm00RlNiU09lN050cFptMU5MRDRXSXg1cXNqZnNpUGNsOVUyazhqQTJZQmEzckI3Qy1KbWVKSzYwa2tSWVhjM0hLR0pFSktqOS1kazFDSXNXd2lWaF9BaEtBZ0Y5ZUdnVXhXUE0?oc=5</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K69" s="1" t="n">
-        <v>46077.20362268519</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Solidarischer Hochwasserschutz: Regionale Allianz setzt auf dezentrale Maßnahmen und Echtzeit-Frühwarnsystem - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Solidarity flood protection: Regional alliance relies on decentralized measures and real-time early warning system - RegionalReporter</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 05:04:48 GMT</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxQbGI4VVlKYUJfeGhaTGpqVXg3ZDZqTzBnUXBqUngwQ1l2dkxFakRZN2QwTm9HTDVORC03bnpaNGVaV2FBWlNXS2VBY0dqNlRmdXpiNGVKdGR6aGxUSkJwelhkMUdTU0lUVktmSTNmcVI0NHBBbGpXZUowZnpRT2hKWHJlSFhKa1VJYVMxTkZ2VjRBVTR0dUFKVnlqNF9rdllKYndwRW5hdUNGUVZfVDhMb3BUNFJqcFQxZVhueXJVT2dZUm1iU1Z6VUNoV3MwUkhsd3BZVi1oZEdpZXlHR1NvYVppckZrLU5IZEp4SEdHWjVvcEFMODg0?oc=5</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K70" s="1" t="n">
-        <v>46077.21166666667</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Village Ingolstadt (fallback)</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Important note: Municipal construction work restricts access to the parking lot - EHC Red Bull München</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Important note: Municipal construction work restricts access to the parking lot - EHC Red Bull München</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Mon, 23 Feb 2026 16:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNdUdtZFdTODlzV1RXU2NEWGRNeGwtWjRtODUtYWI3bkZfRXVNVjhNWTBhWnNYcGVmZUtYdHJsOWYtX0NRV0xteEwxTFlJU3J4VVUxREFmaDB3dTVTaTRjdG5YM2t6VE5yZUFKRV90MnN4WURuRERQeW9CYzZaZlZhS0lOS2lHTUZvZml2RzVIc0dmdFVHemlTVjJLcV9pTjk5RkxUYnF4UFNoNlptU2c?oc=5</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K71" s="1" t="n">
-        <v>46076.66666666666</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Village Las Rozas La Roca</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>("Las Rozas outlet" OR "La Roca outlet" OR "Las Rozas Village" OR "La Roca Village")</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 09:21:06 GMT</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPd0dBclgxSVlFV1dtaEgzNklSZENrcDBPVF9kbEZOWUZhMGtfS3BsS01WWlpwMERQMHVtUUcxaG1EaFlyV3NONy05ZlQ1TzRPTG9lVDUtZE5xVVZEbUdBTFdkNlB5TEhTb0FmSWJlOFpqTXVVLWhvd1JaYzkzNGNMaVBmaGpSaWZ0dHJ1cnBXQndERXZMN2ZhSWJSNlFPNHQ5MFMwbUF1WHRIXzBXOUxpQmtYdWgyNlpDaVhEdjcwYXBGLUtQNzQwdw?oc=5</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K72" s="1" t="n">
-        <v>46077.38965277778</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Zola Predosa (Bologna), sparatoria al campo nomadi: «Un pregiudicato colpito alle gambe» - Corriere di Bologna</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Zola Predosa (Bologna), shooting at the nomad camp: «A criminal hit in the legs» - Corriere di Bologna</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Tue, 24 Feb 2026 08:41:43 GMT</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTXZ3cFF6NURKMDl5cGZSWFJWQ2ZRWk95Z2ItemVwYmlVd1BhMm9LX2Z5YmJiOFp5b2lNVE00TVdpWUlnb2VLd3B2VnJnckU1R096NU5nTFM0dmFlU2o1WUlWakN2dkttY2Z3YlZ6akF5TnhZb3g5QkV2ZXRXSnRvR0IxZ1dRMjMxWmVaNUNTcXJIaUVYVXp5eXdwdUN6ek54Z2o2dVdybmwzUC1MS1pBMjQ1d1g5UWZFSXQtMi1MeXhleU9LWlBMeV9HaUhDczQ1bmRIMVVxaHZKR3hsWWZ0c05rUTZ5ZXFpWFdV0gHwAUFVX3lxTFBIZXFtcm93OHQ3bmZIcTdUcXV1VmN1Tm56S0dld3pCVDEtS2ZYdVB1bHYwNzBqUjhyc3ZhSUM0S3p6b09JQmtiOWI3ZmlfOUs5OWxMci0tX2NFckV2V0VKQ3Uxam1rWWtEa1dpdWdZcHA1T0JVLTVneS16d05NVmxJVjBOMDdDcHJaUW5lYS1JamdtcGFlMHhneTJkTE4zeWZtbXhNZWRtWUZQbHpIR09sNWxGZ3ktLVVVSVZlWG55eXYzX3BQV0M0MkppUVlNWU1PU3czUnRMTUNRVkVzWUlyYWhPZGs2MUFULTU2RnNFcw?oc=5</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K73" s="1" t="n">
         <v>46077.36230324074</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-25 07:59 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>Brand Protest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M Executive Increases Stake with Share Purchase on London Market - TipRanks</t>
+          <t>CANADA GOOSE HOLDINGS INC. INVESTOR ALERT: Kirby McInerney LLP Announces Investigation Into Potential Securities Fraud - Business Wire</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M Executive Increases Stake with Share Purchase on London Market - TipRanks</t>
+          <t>CANADA GOOSE HOLDINGS INC. INVESTOR ALERT: Kirby McInerney LLP Announces Investigation Into Potential Securities Fraud - Business Wire</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:07:26 GMT</t>
+          <t>Wed, 25 Feb 2026 01:00:00 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOSHBZdkZJZGozM29XREZrVmJtdnREMjRRcGJTcnVsTkhNdlpwZHRUc0V4QUVWZE9QV3BnU2VJM0pJR2p5cURSMWVlNWRfQkNOQzAyNk9IcTd0ZXhEY3lvOFJxN2lwWVVmX1duc2pmNmRoMEptZGszeFU4MXp0NlFicG9sbjZoaDB0c2F0RS1mczhFN01nc0FuR19vSlExNkhEOWVuS3l2cVNteWZ4dDhEanFQUmZyZVdI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxNSWdGWEV1YjFJb3FVS0h2alBPemlnSTMyUVlOTkhGaFNUQV9vZW1aS09nVHNJNGxsZ180SFFvVm9ibVNWTUZfVENNbEJVYlo3ZXlhdXFpWGVDYWJKcVNGZUxYaFRSaGEzQXN2eW1vWjhpU1FSWlJ0TlRqMWFjTUdMb0Nram1tUFc4VGJycW9IZnlLdXNxeThXUG1QeFVnN3A1MndfVUFmcFA3MTB1MW0tNVhMSzFhX0xZaWd1MDg5eERiYkIyQkVKYTdWelZnUzFZRW1vTm11VmVYMmRPcktIeHJmUC0tS2xfX3gxNk54WUw3bkl6ckk2ZWpiLUttRVlveTBWRA?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46077.5468287037</v>
+        <v>46078.04166666666</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
+          <t>B&amp;M Executive Increases Stake with Share Purchase on London Market - TipRanks</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Retailers sound alarm as shoplifting reaches 5.5 million incidents across UK - EasternEye</t>
+          <t>B&amp;M Executive Increases Stake with Share Purchase on London Market - TipRanks</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:37:32 GMT</t>
+          <t>Tue, 24 Feb 2026 13:07:26 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPQ0JBbVhreXY3QjZCanZWU1VSYnlMNDg3NHBrbG5VV2Q5WG9VS1dLdHFmbmtjaEh1a2RlRHNtcXRPWHVxdEtMZDNsMnhNR3hYbXAzUEFoZVo4WF82RTVGR3ZHT1hyU2pWNTFlRFdYTHFtUG1EYTV5ZkNhQmZabndXWFFiYmI2ZTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOSHBZdkZJZGozM29XREZrVmJtdnREMjRRcGJTcnVsTkhNdlpwZHRUc0V4QUVWZE9QV3BnU2VJM0pJR2p5cURSMWVlNWRfQkNOQzAyNk9IcTd0ZXhEY3lvOFJxN2lwWVVmX1duc2pmNmRoMEptZGszeFU4MXp0NlFicG9sbjZoaDB0c2F0RS1mczhFN01nc0FuR19vSlExNkhEOWVuS3l2cVNteWZ4dDhEanFQUmZyZVdI?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46077.44273148148</v>
+        <v>46077.5468287037</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
+          <t>U.K. shares lower at close of trade; Investing.com United Kingdom 100 down 0.03% By Investing.com - Investing.com UK</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
+          <t>U.K. shares lower at close of trade; Investing.com United Kingdom 100 down 0.03% By Investing.com - Investing.com UK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:06:48 GMT</t>
+          <t>Tue, 24 Feb 2026 17:28:26 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNcWdvdkd5cGZ3QmRMYjFQaExNdUx0S3dVcmdEelVjcUpwNUhKbENHMlJRRVFCeWxoZjJQMko2UXhOaVV5d0N1aDF1SVdDZXBOUDJoRmFsV1AtLXFZdkpjdUdWNXlxTWNBb1lnZmNnQVMwLUJVak9JVGNJRWo4SmdBT1dQWGcwLWk4NlRLcTd0OVlHbXppYTJTSkx3WGYya2xmb21WbUFHd211Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPX1E0aWNNVzZlX0lpb29OUnFVenZNSk11UmU0T25UeHFXS3gwdFZ6SWZCc3E1a1Iwb3NnV0FFNHY1ejdLcFFTekpqUmlNQzRPaE9sZlJZRk5LcTB2cDlSYjk1Mk1kelhKakNoV082dzBwWmNiWVVIb3lEN3I1OWN4OXNHcjBtMUdObmEwWkNjNmlHZHNRZmpUU1JhbDgyc1cxMFM2bllyRXlMUDd6OGNDSUJyZW81QU5YYVFjTHNUX18zbkhWZ1V1M2RvdVRTOWZhMGRDOUF4OFVLQQ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46077.46305555556</v>
+        <v>46077.7280787037</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>London Marylebone Incident (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
+          <t>IRFC shares falls 4% after OFS opens for subscription today — Here's what investors should know - CNBC TV18</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
+          <t>IRFC shares falls 4% after OFS opens for subscription today — Here's what investors should know - CNBC TV18</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:28:00 GMT</t>
+          <t>Tue, 24 Feb 2026 23:18:47 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNaDlnYVhpRlVxSXcxQXpzRzhaZVBTZzdhRmxESzFScjBxanNhTHVkN3IyZTFZUXgxazRRU1RMV0pBUUpYZnkxZnFQYmU4VGkwdWJFdnE5ZzRHemtjWHFWMTY3dHpPOWdkaWR1UjZWcXZUWG5sYV9iemNMQXFkVWtkTmpUeGdyWlJTbHBOWXFtT3NDMFd5SE52eUQ2S0pKYXg3dG1OMlZXVEdzaldqcXQzX1p1MXJoLUpIU0J4b0JDQ1FvdXU1U3ljV0Qyc25QeE9PRGlYc1dDY0dlcXp1ZDRxVzg0dVBvLVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxONklGTzgxZkEtS0padGhMcTBPRm5GRndzR25DX1dWN2pYU21md2hVRW5tdFBVSUxNOTBlQWpSTVhKUnRYUWNyRnNjb3NUdXoxM2lfNlFzdGVtUXBYVkUtbnBZc3EtWmtFR0xuUlJETl9uVmp3NmZCc0VOb24tRHdRclk5YWoxQzFlSlBBMDhzamEzQzdZU21qUWVjSGU1aFQ0M09qaEcwOWxaWUZmb04xTE1aeW90eTVNclRESGpFcjY3LWhLWkQycW85S2k1djRpNE1WbmpDNjRnSzdfZXpTeEhlWDI1bHk5YVFwYm1R0gHzAUFVX3lxTFBSSnVqYlZqN1RFcVhTZDhRazRvYzNQX0V0VWNhTHBKTHhnZzlwX2c3dDF1c0E1emJ4bGJ0Yzl1Vm5rTVNoSWtEOEp6N2pYT2FuT2J1VkhHNXRKcE8zSE9GWENIdXBMX0dJS0p6clhyeGNfVS1WbUExWmFEekhrYnd1LUNKNTQtR0VrMGJqZ25KWEhZMjdKQkxRU0pvNUpjV01INUx0QjQwYnFTTGtDbGdGbEhFcVg2V3JDZ3lhdzJGYUlRZXkwTlRJdXRCbnJEZzByQXB0NWpNUnRkNDRlbzhpRUdmQnJ1SlJjeU1xMWR5Tm1JZw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46077.43611111111</v>
+        <v>46077.97137731482</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Politie Brussel West vindt bijna drie kilogram cannabis en plantagemateriaal - HLN</t>
+          <t>Bicester fire: Explosions heard as blaze rips through former RAF base - with smoke seen for miles - MSN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Police Brussels West finds almost three kilograms of cannabis and plantation material - HLN</t>
+          <t>Bicester fire: Explosions heard as blaze rips through former RAF base - with smoke seen for miles - MSN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:58:28 GMT</t>
+          <t>Wed, 25 Feb 2026 00:46:40 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQVDNCRUxNSms1VFBKUXBxVTdkcGVlb2p3MGZiajBHcmFqN0oyR19uaDY5UnIwcXFQc3lQY3JncXR6blFKR0wyUVpSZ2d4UzRMeDh5UU50QllENEdBaEx3Nk1XbmNlZWE4d2Rnd2hMUVVoY3dqSjh2eWFTSnVzel9OTlV6dXBwZjVubXFWVWhhSTY3X2R1enUyM0J4bFRDYmNYTXF5U0k4aVMzRWlzaUl6UUVNNWI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gJBVV95cUxQelBnWW5WSTRCRElaaVplcXVobDRVZWctMUtzMWk5aWtTLXA5U3B2cENlQjBFdkdWRjFhLXRHbkJZZUhCeXBzODFhb2txR0hWc1M0Z2Z5SDhLNTcwNFYxTHlXMDU2VENsRWlmZE9faXpZaldTcG5QVExGWURaY05EX2lOM3dZZzAzTVFTdmI3TW5wMDF4enVnWktGYXZYaGkxbkxoa1I5NmNhdXFRZ1o0M3NXcElBZHE3ZDJkaXZ2VGRidzZTeXAtMXFscDg5R0lSbnVWUFpyQ2dZOUZHOEh2UXdkaHlYTGZUY0dmTTRreDRuUmhMdV9jM0VIM1h4b2h3Y2JnaGFwZC0zX3hFTF80UWtxWE1yVnFCN3N2R2I5LXZucDg1RjlOdm5NMTRDUWlWU2VfTjJSb1hOd0p3Skh3MTU2a0JpaGFMZ0ZmaGwtdjlmQk1LTk5jTkpzNl82cDc5S1I4eW5tSnZqYjRjdlFycWR3?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46077.58226851852</v>
+        <v>46078.03240740741</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Trio krijgt drie jaar cel voor schietpartij achter winkelcentrum, maar schutter gaat vrijuit - GVA</t>
+          <t>UK trips go digital: What tourists must know about 2026 E-visas - Lifestyle Asia</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Trio gets three years in prison for shooting behind shopping center, but shooter goes free - GVA</t>
+          <t>UK trips go digital: What tourists must know about 2026 E-visas - Lifestyle Asia</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:39:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:33:24 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOUXduU0hBQ2g5c0puak1mdjJQUzBfdEwxNk92RFdaemd6ZzZTTkI2dkdWWmlZV1RTTVV5cC1IdmZubHlNQTVuY0dmdlJDQ1hoRU9GSVBfNTFLQ0o4RmdoZHU0REptS3JBTVU2ek9JMmtTWFItbVpuSS0tM0o1MzVGSW9TNFFiRTFJY2VTalhyQkhsSmR1V0YtNkJCWDN2dFJIYms5cUlKUkZ4Rmh1Tm5zQVdJVVBoNUNpY2ZJOG5zNVI2YnJkRTlGdTAtbVRrekRqeWo3MEFrUkVCX04tZnZzQV80MUJKa2x4V2xxVkVweXN4ZGM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQWjV6bjJBVXFyM2NheXlXTFVVMHlPRm80dmZCcEJZUkcxUU5zS2ZReWJSd01Oa3RKUFl3bGYwMjlVaWMwYkgzQ0s0QlpITXV3ZTBhTTNzdUh5NV9jNFo2ejR4NGstWjhYWkJlOUtOR1FNR0JSbUx4Ml94MmZFTF9jMFYyTDMxZ0pGQmhVcEVKN2QyNVpEaGZIazdSb081WnRlUVdMdFREOF81Y190dzZFNFRB0gG3AUFVX3lxTE9fNVo0NUpneVZtTFN4ajVaSjBGNjlpNENRWjZDNTh6dzlDWE94YjhOSFlyTHR5NzBIQTJ6Z3NIVElZM1ZHZldpenRJb1FmQzVxbEZ6Q182OTU2Tl9weTVNTk1XRU4zRGQyZDBYakJsRjBsWkRoNjFJVE8wS2FXdkQweXNiRW5ER1pJZlgxNlY1c0Jpam1FTWxUVEIxSVdkOWR3U1IyRHBzVjZtTlliUm55VTNSOTRqUQ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46077.48541666667</v>
+        <v>46077.60652777777</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Logistics Disruption</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("DHL" OR "UPS" OR "DPD" OR "FedEx" OR "Royal Mail" OR "Parcelforce" OR "EVRI" OR "Dropit") AND (disruption OR strike OR failure OR delay) AND ("UK" OR "United Kingdom" OR "Britain") AND -dental AND -"pay dispute" AND -"postal vote"</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Het opruimen van rondslingerende flessen lachgas kan dure grap zijn: bij onjuiste verwerking risico op ontploffing - De Limburger</t>
+          <t>Royal Mail warns 44 UK postcodes they won’t receive mail on time — full list - The Mirror</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cleaning up bottles of laughing gas lying around can be expensive: there is a risk of explosion if handled incorrectly - De Limburger</t>
+          <t>Royal Mail warns 44 UK postcodes they won’t receive mail on time — full list - The Mirror</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:22:57 GMT</t>
+          <t>Tue, 24 Feb 2026 10:20:00 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxPNmtxRU80QmdSV2tTNlRrRHd0QVJCNDBXVnFKQWVOdkp2OEtlM3podGY1LTViTm5hWDl3aWRIY3ViU3R0dUMxbndTSGZWS2FjdmJhM2xiN1MwS0RnNTdGQVE3cGlrU2duaTkwSnBFU1lqX2xBdi1yeDh3WVhXVmVDazl0eW1KMEdKbXJURHFyQXAyYW12ODF0R2pkRWhjUjJ0bmhQQlhLQUpma1lJN1R2SldGNnBhdlo2UkNyOUtGWWVHYzRaRDFJRHhBMkVJYU9CcGZPcDJERVJSLXB4YmhTQlhfV3B5TDdtQlktRjgxZy01ak0yOXhPY3MxYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTFAwTkduWUExczlmMmo4TGlCYTQzNEtwU2tPQTNnNGs1Q3ozSFFEQVpHN3kySGFVVDh6Ykc1WEt0VkxpU3BUYkJjVVNiM1h2WkQ4RlVERzBNYk9KX2lZUjJLUXRBbWtPWEdWdy1wakR2VnNZWVFPOVFqN1VBUm44d9IBgwFBVV95cUxPWV9sUDFrQ0xOcHd4WUlxNGI4UWt3c0lqQ1hKalRIQmlnVFZNd1dxd3kzTkxTWDl4QWI3dkV6clZtazBhVmN2QnVqX3htcUZ4WUMxejFkRlU5SzRSZ25td3pWUEpBWnlSRDlDdlIwMHlnUTZfTmFzMHFCWkxoX1V4bFZMQQ?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46077.59927083334</v>
+        <v>46077.43055555555</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>PETA Broad Search</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"PETA" AND ("Italy" OR "UK" OR "Germany" OR "Belgium" OR "Spain" OR "France") AND ("fashion" OR "designer" OR "outlet" OR "luxury retail" OR "shopping village") AND (protest OR rally OR demonstration OR campaign OR action)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Voortvluchtige drugsbaas bestelt vanuit Turkije poging tot gijzeling in Berchem en moet 7 jaar naar cel - GVA</t>
+          <t>Italy Fashion Protest - the-messenger.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Fugitive drug boss orders attempted hostage-taking in Berchem from Turkey and has to go to prison for 7 years - GVA</t>
+          <t>Italy Fashion Protest - the-messenger.com</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:28:25 GMT</t>
+          <t>Wed, 25 Feb 2026 04:04:46 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogJBVV95cUxNZV9xLWN3R3ZhZHYwUEY4LTktS3hKTXNDbFhTMnRLSHByY1NKWDlUNlVtS1pwSDFhdDFidEl6NEJDbHNLZkJZcTJ3bUkxYzNSNnNPbktjUG9HaXpUNGI1TzBKc1J2c3Fld0pqNWtVWnRiSnd5b1NEcFY1b21oLWUyaVQzNXRIZkJza0RQdW1ici1QM0hfam92a1lHWFNIcXgxQnNvcklLMWwyOXpzci1wUWVtdXdMbmdGeTg4YldQMUx6amszckRuZHlCVEpBV0F1dkU3SEpzaXNiQmZtMzYtVzZTZllOTERxTFpqZUR3ZFVoTGNSZlZSVHp6c1NUNk8yMDIxZk9FdXZOYlZ6eE1Bd3N4bm0ySXhYdzM2NjVVd1IxUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPQkxKREQ3LWFXRTV0dlpHTWJsVHJwZnBuMmdNUTFTbFctbzhjRE12cUNzUUlUQlVJTzdVSjhZZDZKNkR3MEJWczBUUUR6VFNlalJKRWwyUERadTE4Vm84Z2g3bkYzRTEwVmtwUHRCNWJHa3N4TWRjWFp0N2s5T01LMkVmNmNlaVprR3d6RzBLV1NCdw?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,52 +900,52 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46077.47806712963</v>
+        <v>46078.16997685185</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Gravin Diana du Monceau de Bergendal opnieuw voor rechter voor verwaarlozing van 270 dieren: “Al zes inbeslagnames in 15 jaar” - HLN</t>
+          <t>UK Retail Crime: Is the Surge Finally Easing? - International Business Times UK</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Countess Diana du Monceau de Bergendal again in court for neglect of 270 animals: “Already six seizures in 15 years” - HLN</t>
+          <t>UK Retail Crime: Is the Surge Finally Easing? - International Business Times UK</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:18:39 GMT</t>
+          <t>Tue, 24 Feb 2026 16:29:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxOVlFnbkZRT0RIRkNUQjYxNjFxWlkxX3RESk1NMHZremJEbmhYX3lNcEJYLTBnN0pkck5jeFdWQ2NkUVh0VFRCbWt3T2d6QkF5V1pBUFlkRmRrRGNmekJtYVBjMTl5a1hZZXBma0tRM25PWmwwQ3d3UDd0bEwybXNPZHVIeUV5R3pyNkdIc3d3V25VZVB4bE9TUmtxNU1heEVnUTZMYndkSUtnY2Y0cUg4N29FRF9RTEJzMklOVHlwbGRyTXpVOVVwLWh3bFl5UzlnRjIxc2I3bEk3MEJzb3NhNmhHXzRRUU14cWRBNVFHVjZGZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE9CanphNm90dWFQeXVqS081SVZWZG5zSF9XNWR3NEFCVmZRU2J1MWM4Nkw5dUU2bkZXZVcwekcycTBlQmVsQ3NpU1VDQUd5Z0FvU1M5NVFmSWd1SFdMV3Y1UXBqWWNEbjl3alpGeVYtOA?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,52 +955,52 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46077.59628472223</v>
+        <v>46077.68680555555</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Stad Antwerpen genomineerd voor Vlaamse Verkeersveiligheidsprijs: “Minder verkeerslichten binnen zone 30” - HLN</t>
+          <t>Retailers sound alarm as shoplifting incidents reach 5.5 million across UK - EasternEye</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>City of Antwerp nominated for Flemish Road Safety Award: “Fewer traffic lights within zone 30” - HLN</t>
+          <t>Retailers sound alarm as shoplifting incidents reach 5.5 million across UK - EasternEye</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:48:33 GMT</t>
+          <t>Tue, 24 Feb 2026 10:37:32 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQMmZMVXphNzNLM0ZZNjFUZXpLUjhwMEF3YjI1d3FrX3ViUG9UV1drOEFFYzZtaGdZX1BwajhRZHhrcUYxRVktNENzSVktUHVMTzZycDFOSG1jZ1NiR0E0Qnk2YXdxQURVOGRFeDVqX1NUb0hiSjdHZUZTRDVLNkhmLWdJekFUNkx5YlY2QzgySVJqYXlGSXBENUNTanptQi1YR0ViU1ljTDJ4SXVERHR6b2FrQ0MwXzJLQ1RPOHBGZ1dHNWhONXpHOGpDRHhyN2Y0MkR0Sm9XOW0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPQ0JBbVhreXY3QjZCanZWU1VSYnlMNDg3NHBrbG5VV2Q5WG9VS1dLdHFmbmtjaEh1a2RlRHNtcXRPWHVxdEtMZDNsMnhNR3hYbXAzUEFoZVo4WF82RTVGR3ZHT1hyU2pWNTFlRFdYTHFtUG1EYTV5ZkNhQmZabndXWFFiYmI2ZTA?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,52 +1010,52 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46077.40871527778</v>
+        <v>46077.44273148148</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Waarom laat je een vriend op straat achter om te sterven? Heerlenaar Johnny E. (43) moet na conflict binnen motorclub Kanun vijf jaar de cel in - De Limburger</t>
+          <t>Michelin-starred Lita names Kostas Papathanasiou culinary director - The Drinks Business</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Why leave a friend on the street to die? Heerlen resident Johnny E. (43) has to go to jail for five years after a conflict within motorcycle club Kanun - De Limburger</t>
+          <t>Michelin-starred Lita names Kostas Papathanasiou culinary director - The Drinks Business</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:01:37 GMT</t>
+          <t>Tue, 24 Feb 2026 17:42:57 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwJBVV95cUxPZUV2S0NpbC1iRTlwRlpBbXB0QnBqNnZkeE9SWUQxLVdWRHp4MXloQXBvMlhNTVhXaFZJVUZKN2o2NGh1b1VyOFFJYlBsb0I4ZjJieFl5MnBYcDhYQ2Q4ZUZUVUotOExudHBNYkZlT1doSmxDd3lLbjQ0Y2FlRVZoT1JJUmFfNnN6WXBFVnZLLVNSbE9tVUJ5WWRFMmlsSk9teVFsdkNUNDlVR244Q3RnUEpjWk1HbkhHaXNDWks4T0UzYTRxMmpRQlduTGNkTUZzWmZDTmJMNC1BSFlGV0FZVG1idS1aekR2OFFrblVkMTAwQWtZVVktclJXVjNzOVhBQ3EwVUI5ZW42OUZQNS1haGdTSTFFMlNXRHdDcWllRHdWck84dTIwYlBRbU1yY3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNeTM0UkM5dW1EMUZyYVp2Vk01WEdNWHRXU005by1wNTZaZ0h0VjRHeDVYaXU3ZXdHRW5YMWNsQnRxS2MxbGJNMG96TWRCX0RKcEtkN1lkR01odzBSY1hKYy1XdlhaZzJKdm95Tm5pYy1CVktuclpZZXJHSy0wQUd5MlhBMDAwejBRZy15U1o5LWNodFpaSjJIdllOaGRhdjJWYmpFaGJhWW0tZzBvcGc?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,52 +1065,52 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46077.58445601852</v>
+        <v>46077.73815972222</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Explosief gegooid naar woning in Eygelshoven: geen gewonden, wel flinke schrik en beschadigde auto - De Limburger</t>
+          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Explosive thrown at home in Eygelshoven: no injuries, but quite a fright and damaged car - De Limburger</t>
+          <t>Railway enthusiasts flock to Banbury to watch as 50-year-old train sets off on farewell journey - Banbury Guardian</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:46:26 GMT</t>
+          <t>Tue, 24 Feb 2026 10:28:00 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOd0xSOHdvOXluc2R6b0hTV3pfMnBqUXVULVo4TFhTYkNOVzBSc1F6bjJFY0hVRjRVSEJ4cEo0UDlONU9yenRORzFOSWR1U2hzYVJVbGNTMXNsLUdSMUlKZjhNOEFQNG54cm0zVVc3YjhlelJGSFI3N1pESHJ2RmFqSVZvb2pNU29nZjNHNm9id3l4Y08wQmNWNDFnekcwbklORVd0V2VFc0xaMzBkcU5YZENvVkNoYmpxMGZzelM2aXhTQzJTZmlEcEpvclNsWWkzbXN5Y3VUQnNkY09aLXlVWFVxSUw3dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNaDlnYVhpRlVxSXcxQXpzRzhaZVBTZzdhRmxESzFScjBxanNhTHVkN3IyZTFZUXgxazRRU1RMV0pBUUpYZnkxZnFQYmU4VGkwdWJFdnE5ZzRHemtjWHFWMTY3dHpPOWdkaWR1UjZWcXZUWG5sYV9iemNMQXFkVWtkTmpUeGdyWlJTbHBOWXFtT3NDMFd5SE52eUQ2S0pKYXg3dG1OMlZXVEdzaldqcXQzX1p1MXJoLUpIU0J4b0JDQ1FvdXU1U3ljV0Qyc25QeE9PRGlYc1dDY0dlcXp1ZDRxVzg0dVBvLVk?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,52 +1120,52 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46077.40724537037</v>
+        <v>46077.43611111111</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Opnieuw incident aan Antwerpse gevangenis: politie grijpt in na mislukte poging om pakketjes over muur te gooien - HLN</t>
+          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Another incident at Antwerp prison: police intervene after failed attempt to throw packages over a wall - HLN</t>
+          <t>Railway veteran of 64 years returns to Flying Scotsman footplate - Chiltern Railways News</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:38:35 GMT</t>
+          <t>Tue, 24 Feb 2026 11:06:48 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPbGtHUkJLT01KeFFCU1ZHR3dTRUpOdlhVSVl3b2hKRXViSUNGZmJPRTJiMjZzemx1MjNzRGtRZzFDUElVMllrSDZoUWNnekNJU2hITWtDVlBobTRzSTB1c20wNnZoTklISm1qTEQ2N0YycmFvakZzY0xyT0NIRGxHaW5WWHpVWE5xYXFpYjRDalZPb01rMHFERWszOUx5U1Q4U1J2Uk9VU2NyY2ZvYVlJNjBVR2RyLWx5dURtU0x6clJfNXlFa2ctejRqS0NELTI5cVZfQ2pUN05PblVLRHltUG5WQWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNcWdvdkd5cGZ3QmRMYjFQaExNdUx0S3dVcmdEelVjcUpwNUhKbENHMlJRRVFCeWxoZjJQMko2UXhOaVV5d0N1aDF1SVdDZXBOUDJoRmFsV1AtLXFZdkpjdUdWNXlxTWNBb1lnZmNnQVMwLUJVak9JVGNJRWo4SmdBT1dQWGcwLWk4NlRLcTd0OVlHbXppYTJTSkx3WGYya2xmb21WbUFHd211Zw?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,21 +1175,21 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46077.52679398148</v>
+        <v>46077.46305555556</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Antwerpen dooft verlichting aan 45 gebouwen en monumenten tijdens Earth Hour - HLN</t>
+          <t>Brussels Airport opgeschrikt door valse bommelding - VRT</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Antwerp turns off lights on 45 buildings and monuments during Earth Hour - HLN</t>
+          <t>Brussels Airport shocked by false bomb threat - VRT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:00:13 GMT</t>
+          <t>Tue, 24 Feb 2026 19:33:53 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVzR6UXJtbHMtY1FGS0t6eVZOdjNvcEFlX21xOU1WdGZGb0tPaHpndGtwdXJ4bE5nV2prVG1xM0ZQbUlsTHhkbzVZX0p0cThqWU5XQkRRZk9pbXJrZGI2VjRCelEtaXpYYUhuZnY5WUY0WXhQOGdfWDB3QWF1QWR4NVFNVjM2NVkzUjdkTlJkcVNxQ01XMERzWWU1ajkxWmVBSVFWYTlvSmN2VElyNU1uOF9jbWdUdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNVU9yZ2VyOGoyU2FaVk9XbnZVenpiTko2NE43bVBlLW15WEpKUG1DLU56VXRoNHFwZ2ZnZVAzWHdCNlhtUGowUkhrVjUyajZPUEJHT3pOOVFGUnZxY012bFNTVG1wYkNuMkIwcVVrTnZWQU11SUg3QllGdmt1Y29ycURHdE9PZlN6SnRybWtJRE5DbDNqUWc?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46077.50015046296</v>
+        <v>46077.81519675926</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Antwerpse Vervoerregioraad verwerpt besparingsplannen van De Lijn - HLN</t>
+          <t>Trio krijgt drie jaar cel voor schietpartij achter winkelcentrum, maar schutter gaat vrijuit - GVA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Antwerp Transport Regional Council rejects De Lijn's savings plans - HLN</t>
+          <t>Trio gets three years in prison for shooting behind shopping center, but shooter goes free - GVA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:05:43 GMT</t>
+          <t>Tue, 24 Feb 2026 18:48:37 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPMDBYSXlQbWhUYXJYNTU0VHpqbEsxdTVYSnM5dk05UHlSSlJCSS1CMXh1UnFVcm1VZ0tWOVMtb1JFSlJQUnpyVTI0Ul9hQk5hQkdITEF6X3lfZjRFU2Rncm9sNzBhY0Zqdzdpcml4c3JmdVhobTVNUFJyTDJnZ2ExTWNxQTU5cE13dzlJNHIyV1BFRklKNl8yM18yQzlMQU5jbWlrYlpENA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOUXduU0hBQ2g5c0puak1mdjJQUzBfdEwxNk92RFdaemd6ZzZTTkI2dkdWWmlZV1RTTVV5cC1IdmZubHlNQTVuY0dmdlJDQ1hoRU9GSVBfNTFLQ0o4RmdoZHU0REptS3JBTVU2ek9JMmtTWFItbVpuSS0tM0o1MzVGSW9TNFFiRTFJY2VTalhyQkhsSmR1V0YtNkJCWDN2dFJIYms5cUlKUkZ4Rmh1Tm5zQVdJVVBoNUNpY2ZJOG5zNVI2YnJkRTlGdTAtbVRrekRqeWo3MEFrUkVCX04tZnZzQV80MUJKa2x4V2xxVkVweXN4ZGM?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46077.46230324074</v>
+        <v>46077.78376157407</v>
       </c>
     </row>
     <row r="17">
@@ -1315,22 +1315,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Maart is Jeugdboekenmaand met meer dan 100 activiteiten - HLN</t>
+          <t>Nog twee minderjarigen aangehouden voor explosie sportschool Fitletic in Roermond - De Limburger</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>March is Youth Book Month with more than 100 activities - HLN</t>
+          <t>Two more minors arrested for explosion at Fitletic gym in Roermond - De Limburger</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:16:34 GMT</t>
+          <t>Tue, 24 Feb 2026 16:22:20 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNYnVLZVc1VjNxVmRLaVpZWTk1XzlLVTBrV1d3bmdOZlNELXpFZDNpS3BhQ25QcmMzX0doVUdMY0NsWU5YMzg5VlF0WThSQVpiTk1EdHdHelFuMXJjbkdadldvV1hQWW9ZTzZFNWRhSzhnbVZTSk4yS3ducjlpWHV4U1NkeEVoQ29fZjZPRlFUbzJlRmRyOUVMNHpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxOY1lITEdQUDN5cm9DTzhnVnRIN2l1Q0QtY2ZsaWo2OS10SDlrNkNTMWI1R0xoOHl6V19aNXRsLXNtSnBiX2RIa0J0ekZuWTNGSXR2THV6TXNaMjRtdmg4Tmx1VlhGZm10Sl85bHJzb3RKbmN2ZnVfTWNBS2J2TWIwVEk4X1FjckVLNmpZeHkwVFZDbVQxT3dneFQwRUk3X01Oc2dsSllEdWl3RkJUUXctbVFWNm1IX056dW9zSWJOdjU1YUkzdHVYTnk0OVZBS3JDRlpzWEk3aU5zZjEwQUE?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46077.46983796296</v>
+        <v>46077.68217592593</v>
       </c>
     </row>
     <row r="18">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Beurtelings verkeer op de Kapelsesteenweg door bekabelingswerken - HLN</t>
+          <t>Drugsbaas bestelt vanuit Turkije aanslag op papa die zoontje afzet op school in Berchem: “Voor 50 miljoen euro aan drugs gestolen” - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Alternating traffic on the Kapelsesteenweg due to cabling works - HLN</t>
+          <t>Drug boss orders attack from Turkey on dad who drops son off at school in Berchem: “50 million euros worth of drugs stolen” - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:05:04 GMT</t>
+          <t>Tue, 24 Feb 2026 11:28:51 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPVVVoM3lVUzdhOWJUT2lGSi1HbDRHQmExeG1falVTUEt1WEdBRFgwRlJJWUJIV0xmd0M2UmlkdTN5X3RDa2Y4b1FjU2RzSGdFMmdXMHNsSGZhUXBIeHR0Mkh4MDhVdTREbTFsYXV6UUtxRzRIM2ZCM09MQkg0RXo5c1Y0YXcxZ3lSSmhyM3dpemoyMU13UlJNSVR0LTI1ek5sWGN6cWxn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxNX1NManE1aGM0dUxmMXhDYUEyX19pdFRGcmZPWGtCN0U4QTFzSkVLQjRaODI2aWNqWkd1cVA0U3AyeloyRVo0aUgtQkpxaGtEY3JzMzBZUjdHMGhyUmxGT081NG1RSDdKdXJQa2tWSEpub1BSUk1IY0VRSUhrZTBySVJPTm9XSjBFSmlBTTdkbzBBRkpfc0FNdU1UX21jNER5eXJleHBJcFA5Z05JWkdMeXRpOVVGU2FzOWYycEtCak53MzdFeVdIakwyVnVKdXh4MmZiUFlDV3ViemJfc29ncWczOWhiV1lDVm03V1RLSDROYWFrLWFkcXFn?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46077.50351851852</v>
+        <v>46077.47836805556</v>
       </c>
     </row>
     <row r="19">
@@ -1425,22 +1425,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>19-jarige krijgt vier jaar cel voor brandstichting bij juwelierszaak in Antwerpen - GVA</t>
+          <t>Waarom laat je een vriend op straat achter om te sterven? Heerlenaar Johnny E. (43) moet na conflict binnen motorclub Kanun vijf jaar de cel in - De Limburger</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>19-year-old gets four years in prison for arson at a jewelry store in Antwerp - GVA</t>
+          <t>Why leave a friend on the street to die? Heerlen resident Johnny E. (43) has to go to prison for five years after a conflict within motorcycle club Kanun - De Limburger</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:25:42 GMT</t>
+          <t>Tue, 24 Feb 2026 14:50:06 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQa0lwTTV0TjFWaE9SaWlLNFIzVzgzX2N6S2Uzekt3Z2tLWjhrRGZnRS1aWjRXWjU0dDF6VlZHelNiNkd1UmtjSE43MGN4VmVEeDFmX01GUTR0N0x0dmdvS3NiSFVVNEV6Ym1IVUg4WEFPb0paMWhCai12YU9Gd24tWHZPSm1GUzNXbUd6YUI2VE1xaURaYlA5QllGcGUwRnpuQ3JuWWNLbTc1MkJQX182Y19NN1FZTk9iTzctR3h4eDVnWkZIa1pSWHN1WkM0QkF6eFVBTzUtQ2VaRFk2Zm1VT2pRQl8yMGpqNEhTUWlB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwJBVV95cUxPZUV2S0NpbC1iRTlwRlpBbXB0QnBqNnZkeE9SWUQxLVdWRHp4MXloQXBvMlhNTVhXaFZJVUZKN2o2NGh1b1VyOFFJYlBsb0I4ZjJieFl5MnBYcDhYQ2Q4ZUZUVUotOExudHBNYkZlT1doSmxDd3lLbjQ0Y2FlRVZoT1JJUmFfNnN6WXBFVnZLLVNSbE9tVUJ5WWRFMmlsSk9teVFsdkNUNDlVR244Q3RnUEpjWk1HbkhHaXNDWks4T0UzYTRxMmpRQlduTGNkTUZzWmZDTmJMNC1BSFlGV0FZVG1idS1aekR2OFFrblVkMTAwQWtZVVktclJXVjNzOVhBQ3EwVUI5ZW42OUZQNS1haGdTSTFFMlNXRHdDcWllRHdWck84dTIwYlBRbU1yY3c?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46077.47618055555</v>
+        <v>46077.618125</v>
       </c>
     </row>
     <row r="20">
@@ -1480,22 +1480,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Radio Minerva eert Frank Boekhoff op dinsdag 24 februari tijdens een twaalf uur durend radioprogramma: “We zullen hem nooit vergeten!” - HLN</t>
+          <t>Politie Brussel West vindt bijna drie kilogram cannabis en plantagemateriaal - HLN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Radio Minerva honors Frank Boekhoff on Tuesday, February 24 during a twelve-hour radio program: “We will never forget him!” - HLN</t>
+          <t>Police Brussels West finds almost three kilograms of cannabis and plantation material - HLN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:07:41 GMT</t>
+          <t>Tue, 24 Feb 2026 13:58:38 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxPMnFVMngxOEFlSUpuc1B1TzBsZHk4b2stc3EyeDYxV1VhNGlXV2hDTlJTUmFPTjlvdTcxQWFuU0JfZTZMT18zYVFPMHFBS0RIZTVJZ3BsX1dRUHU4cnlYcGtGbDBwd2hsQ0lGQjdlSHhEZDBIbXNKTVNQcFlBanhCbFRXNUlJVnVFdm1HV3I2d2pYaGtpZHRjZFV3NmltWVFzT3BmWFpQaWdVVEoyMFk2LUtDWG9wRE9JRmNoSl80bDd3T1JLN0p5cU5lcWxfZ0hINk8xTVRDSktTMUxuT2NBRTUyY1Y5VHVlRmJzSnRuQkxtbEwwVWNHS2VCdFhsZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQVDNCRUxNSms1VFBKUXBxVTdkcGVlb2p3MGZiajBHcmFqN0oyR19uaDY5UnIwcXFQc3lQY3JncXR6blFKR0wyUVpSZ2d4UzRMeDh5UU50QllENEdBaEx3Nk1XbmNlZWE4d2Rnd2hMUVVoY3dqSjh2eWFTSnVzel9OTlV6dXBwZjVubXFWVWhhSTY3X2R1enUyM0J4bFRDYmNYTXF5U0k4aVMzRWlzaUl6UUVNNWI?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46077.58866898148</v>
+        <v>46077.58238425926</v>
       </c>
     </row>
     <row r="21">
@@ -1535,22 +1535,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AG Vespa zet Wolstraatcomplex in de markt: ateliers van vzw Ercola blijven tot 11 juli - HLN</t>
+          <t>Gravin opnieuw voor rechter voor verwaarlozing van 270 dieren in Brussel: “Zes inbeslagnames in 15 jaar” - HLN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AG Vespa puts Wolstraat complex on the market: workshops of non-profit organization Ercola will remain until July 11 - HLN</t>
+          <t>Countess again in court for neglect of 270 animals in Brussels: “Six seizures in 15 years” - HLN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:28:35 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:38 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPdm9fSkhTTFNrSUNnRnRYOWowZm1zUERzY2Q1M2xYdmZSOVg4RnctSnZveVBlSGlWZ1ZvYnRram52cTVjNW9La0RSSFFjQ2V2UXV1OGlqdTNibG9CUWZQSnA3aWZJNnBFNm9GcEtQQzhDVTVUSHBodG9rQnctaF9vNVdHWW81RW5zbXlKanV0QVJPeHYtNm50RTUxM2k1UHh1cVJIMzlIcmZGdF9lY2h2RkdKZnVTQVY5d2NWdEdUTnc5dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNTmVTUGtHaF84MHFKTnpoVFprUC05R0Zvb3ZjdlNFcWFVYmt1TTJZYXRIZDd3bGtDMk1UTmxDSkE4V3ktRll5dkEyeVhqamxRSk40OUg1NVVJOFhCM09uWUsxaDNhMUNGZng3TFU3ZDg5cmtwYndNY2UwRGR5bUJwNVJWek1jbFFhX1JGaERGdmh4RnAxdWJJckMwQ0JTcjdIVzBOalpDemNjYnB0d0RwVHU1YUg3aE5FeEJoVU1WYkNsQXl2NURKX2k2UVhJdElpWE9CTml5eVlUUQ?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46077.51984953704</v>
+        <v>46077.54418981481</v>
       </c>
     </row>
     <row r="22">
@@ -1590,22 +1590,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Asbest vrijgekomen bij afbraakwerken in Markgravewijk, werf stilgelegd en pv opgesteld tegen aannemer - HLN</t>
+          <t>Maart is Jeugdboekenmaand met meer dan 100 activiteiten - HLN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Asbestos released during demolition works in Markgravewijk, site shut down and notice drawn up against contractor - HLN</t>
+          <t>March is Youth Book Month with more than 100 activities - HLN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:22:43 GMT</t>
+          <t>Tue, 24 Feb 2026 11:16:34 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOYklwVUNDTmRCUm5ZbldoWlJjMloyQjd6TENkajRIZGN0NHprRTFZM0dPdFJEYTE0VmJ2UGVlZFdDd3cyMlJFUEVFRUM0UVF0MmphUXpWeE9NaV9zRmZwenliaDFycmNxMUZlQkJjanhoQ3o0MWF4WS0wenFhSXk0R19qSjdWdjdTM1dKYUxrbWZEWksyamNUa2J1SkhvM3ZwTGRycndPUlBNOUExVnBvZEdQbXpYX203UG84TkJnMjJ2YnAzUkwtYUp1cEtyV2tTbkxTRURB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNYnVLZVc1VjNxVmRLaVpZWTk1XzlLVTBrV1d3bmdOZlNELXpFZDNpS3BhQ25QcmMzX0doVUdMY0NsWU5YMzg5VlF0WThSQVpiTk1EdHdHelFuMXJjbkdadldvV1hQWW9ZTzZFNWRhSzhnbVZTSk4yS3ducjlpWHV4U1NkeEVoQ29fZjZPRlFUbzJlRmRyOUVMNHpB?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46077.4741087963</v>
+        <v>46077.46983796296</v>
       </c>
     </row>
     <row r="23">
@@ -1645,22 +1645,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Wat betekenen de plannen van Antwerpen voor de stadskas? Zo evolueert de schuld de komende zes jaar - HLN</t>
+          <t>Antwerpen dooft verlichting aan 45 gebouwen en monumenten tijdens Earth Hour - HLN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>What do Antwerp's plans mean for the city coffers? This is how the debt will evolve over the next six years - HLN</t>
+          <t>Antwerp turns off lights on 45 buildings and monuments during Earth Hour - HLN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 08:31:33 GMT</t>
+          <t>Tue, 24 Feb 2026 12:00:13 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOam9oWTQ1czAwZ2pWSTRYY291YkJ0bU5qUXcxV29jZWwtVTRMY1lBaTd2SWE3NXg4TlB1OTd0RFJ2Y1pXdldkUTVBOUZsWnc0LUtuVm1raVp3TURMUEYzYkNLU1UwRm1yOXhWZlRxaHpnZmhLZlI5cTJZOU1NS2dhTlk1MVM4b3drRkhodmp2Ynd5dXRqYlpZVEtseVhxNG1tUV82OUhIcXJiTVVEWGtNTlB3SUtMM3pvVWNpT1JPNTd3cXZQTE5tb3lsLWxkYXdMem9j?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOVzR6UXJtbHMtY1FGS0t6eVZOdjNvcEFlX21xOU1WdGZGb0tPaHpndGtwdXJ4bE5nV2prVG1xM0ZQbUlsTHhkbzVZX0p0cThqWU5XQkRRZk9pbXJrZGI2VjRCelEtaXpYYUhuZnY5WUY0WXhQOGdfWDB3QWF1QWR4NVFNVjM2NVkzUjdkTlJkcVNxQ01XMERzWWU1ajkxWmVBSVFWYTlvSmN2VElyNU1uOF9jbWdUdw?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1684,38 +1684,38 @@
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46077.35524305556</v>
+        <v>46077.50015046296</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
+          <t>Sociaal assistent die mesaanval overleefde, loopt van Luik naar Brussel voor goed doel: “Belangrijk om op te komen voor minderheden” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
+          <t>Social worker who survived knife attack walks from Liège to Brussels for charity: “Important to stand up for minorities” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:30:36 GMT</t>
+          <t>Wed, 25 Feb 2026 00:46:57 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOTVkweWFzUUNLdXBoYTJPUGNWeFI3c01LV1pqRWU2eExiOUFwOUE2MlZGaFBySWVJUmdUWGotM1BDS1lydWgwcEpZR3FlbHpuZmpDVVkyYWhNQnBSTEpMS1VscG9HOE1pREFTUlM0VHF4UV9UUjRybFNmaHpWMDlvdE5kZUt5d2lRYW9ENmFkQVFoMnZyRzY3VllEYVkzWEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxOV002bEs5aGRYNWtZNmRSMFo1RTV6NExtUEhzX3ZpREJxWkE3c1I3U2JJMEtHbnEtdjVEeGVCenROX0VFdC1TYklmV0JfcXZPNzlZb2hKcFpDaThOQnI0X2N0WnoyRy1wRUhiVHVnUWNDOEZaZE5CWmhJampsbHRMcXFJaEhKdmhBWG5qbU1PVDBjOHZGT0NGLWhtV3JvT0dCWTIwdGNaaTV4LW1LWGotWlRoRUdWc3NJT3VFZU1YeUpLWG9TalF2M1JtalBDMG1RTTZQWmJhS2RneE5PVE5ITFJ3VUJ4WkpOeVI0SGREWHVjQThiYUFJcTduUEx0cEh6NExvcWg5OE9QY3hMdlprdXpkSnMwQW1QZ0ln?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1735,42 +1735,42 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46077.56291666667</v>
+        <v>46078.03260416666</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
+          <t>Opnieuw incident aan Antwerpse gevangenis: politie grijpt in na mislukte poging om pakketjes over muur te gooien - HLN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
+          <t>Another incident at Antwerp prison: police intervene after failed attempt to throw packages over a wall - HLN</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:27:00 GMT</t>
+          <t>Tue, 24 Feb 2026 12:33:15 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNM185ekl4N3lkY3FGV2xtcHpCRDZicWFIVWpxeXZuVUVzNGc4SFpCa292cnVnaElFMUtnYlMyeVRXWnpnNWNfQmxFVEdzTk9ZVnFob3RqaDgxMTZmWlNaa3ZPWWtVeVU1YVI4SG1vUGdvdmVNUENkdy1fTUJPZTBkcUZGaW5BblhDSHFfbENWLUtoemlqREJHUjB3ZjBnS3AxNHZfZzdOTGdEYk1KV3ZNcVl4R0prelRHVW82SE1n?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxPNUdBQlVyWENiaFpub3YwM2l5U3U3WGJhbEpPY21YWUhCOWJiZ29xX1pjYkpDclJyUzBrd29QaW9vUmJfNGlyRUhXX2xlaEtpM2lWanNXaFljX2VuTUFPcGNqZmxROUdfUHBJRGZ2bXRKVk4ybXE2R3lSUnFPOG1HT3psZGZSTVpEUTdiUEl0X25HYVNNYTlfVGZ6YXJSdUNMdEtFcmhhY2MtRTlkdHoxVEFfbzNLUFhOczFWZnNUbGdkMDI1R1VocjBDNkQyUXplZlhjU0Z5TFBsMlozaGpFaWZR?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1790,42 +1790,42 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46077.43541666667</v>
+        <v>46077.52309027778</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
+          <t>Radio Minerva eert Frank Boekhoff op dinsdag 24 februari tijdens een twaalf uur durend radioprogramma: “We zullen hem nooit vergeten!” - HLN</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
+          <t>Radio Minerva honors Frank Boekhoff on Tuesday, February 24 during a twelve-hour radio program: “We will never forget him!” - HLN</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:16:00 GMT</t>
+          <t>Tue, 24 Feb 2026 23:46:26 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOOTRkZE1mSU1wNTNCODJ6TEt2WWtuTF9yMUR4c1BOb3ptMExaU0ZJSUFyek96ZnpGaHRGRFd6aElmLU9WeXN4ZEZZazVsLTRUNDREamdwTGlMLXhsSHZoLTYta2gxNlBzUlhmRkdCaWZub0xBQl94VTdDZmZhU2s5b1R5TWRpd3BZV3JDS1NTRWRsUjZtemdVLTdaTmkzVDJEVzRCNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNQWozbzdiclNmZmRDU3VJLVZtTXBzSS1ZWHR1YTR4WU55aHhLdHdVcXRUeFIwbTI0NXZIdjlYejV3UlJhejUyOHVxMnV5djJhNHg5NHlUN241TjRLeDI1LUwxMVhsT0dZa2Vxdzd3NWxPbjFGZXBYbG50SmNrSVFRUmZpSGxJQVpzeW5iOWpSQUtXcXB4TUJKdmdEOXZzanhWMFhrVWNPbTUzbnc5R1VWNG0xTnVtRC1yQTBoR2tuQWZrSmNtOGx4UGt6VmkzeHkyRGU2SFZ3MA?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1845,42 +1845,42 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46077.51111111111</v>
+        <v>46077.99057870371</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>La Ville de Bruxelles supprime une taxe pour l’installation de panneaux photovoltaïques - 7sur7.be</t>
+          <t>19-jarige krijgt vier jaar cel voor brandstichting bij juwelierszaak in Antwerpen - GVA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>The City of Brussels removes a tax for the installation of photovoltaic panels - 7sur7.be</t>
+          <t>19-year-old gets four years in prison for arson at a jewelry store in Antwerp - GVA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 08:50:00 GMT</t>
+          <t>Tue, 24 Feb 2026 11:25:42 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPRWg0V2dNa1lZdG1wUWp4V181cklFS3JlWnc0VkRIOEN3STFyRUtURmRRSlQ2U04xQlVMWERsbE12eXpqUDE4QjZPTFl1TDBOVzk4N0YtQzRGSXVYcE9QZDJnem0yZ0xGSkRLN0RWQzJfSDJYbDl6VmktQUQzMFZGRXBYcWpIX3J5SnVlWVlIeXlQVW0zbHNCQ0NNWXZyN2VXVWdLTWVYTU9BOGkwMGhWUmZDQ0o0aUg3bVd0ay04TjBWLWxo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQa0lwTTV0TjFWaE9SaWlLNFIzVzgzX2N6S2Uzekt3Z2tLWjhrRGZnRS1aWjRXWjU0dDF6VlZHelNiNkd1UmtjSE43MGN4VmVEeDFmX01GUTR0N0x0dmdvS3NiSFVVNEV6Ym1IVUg4WEFPb0paMWhCai12YU9Gd24tWHZPSm1GUzNXbUd6YUI2VE1xaURaYlA5QllGcGUwRnpuQ3JuWWNLbTc1MkJQX182Y19NN1FZTk9iTzctR3h4eDVnWkZIa1pSWHN1WkM0QkF6eFVBTzUtQ2VaRFk2Zm1VT2pRQl8yMGpqNEhTUWlB?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1900,42 +1900,42 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46077.36805555555</v>
+        <v>46077.47618055555</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Halen keurt aangepast meerjarenplan goed na budgetfout van 5,4 miljoen euro - VRT</t>
+          <t>Wat betekenen de plannen van Antwerpen voor de stadskas? Zo evolueert de schuld de komende zes jaar - HLN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Halen approves adjusted multi-year plan after budget error of 5.4 million euros - VRT</t>
+          <t>What do Antwerp's plans mean for the city coffers? This is how the debt will evolve over the next six years - HLN</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:32:52 GMT</t>
+          <t>Tue, 24 Feb 2026 08:31:33 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPOTItcThiT1hZQjVXaDA5TEI5RUlVdmt5N1UzR2hEelF2aVBXemRfcTdNbk9xUk5sY2NfWkpJdmIycHN5TThoaVNnVVpCWjgzYXExeFpZUk91bVhhdFhiZ0szcDNRT3Nua3RCSTVUa1BTSGRUdU42TXJ3NzVYSXdFMTRZMkwwUVpqaURzNXJMMVIwbk1rNzNSQVdVaUVvdHRVNGNWcURCUzA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOam9oWTQ1czAwZ2pWSTRYY291YkJ0bU5qUXcxV29jZWwtVTRMY1lBaTd2SWE3NXg4TlB1OTd0RFJ2Y1pXdldkUTVBOUZsWnc0LUtuVm1raVp3TURMUEYzYkNLU1UwRm1yOXhWZlRxaHpnZmhLZlI5cTJZOU1NS2dhTlk1MVM4b3drRkhodmp2Ynd5dXRqYlpZVEtseVhxNG1tUV82OUhIcXJiTVVEWGtNTlB3SUtMM3pvVWNpT1JPNTd3cXZQTE5tb3lsLWxkYXdMem9j?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,38 +1959,38 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46077.39782407408</v>
+        <v>46077.35524305556</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Environ 50 emplois menacés par la faillite de IKKS Belgique - 7sur7.be</t>
+          <t>Antwerpse Vervoerregioraad verwerpt besparingsplannen van De Lijn: “Terug naar de tekentafel” - HLN</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Around 50 jobs threatened by the bankruptcy of IKKS Belgium - 7sur7.be</t>
+          <t>Antwerp Transport Regional Council rejects De Lijn's savings plans: “Back to the drawing board” - HLN</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:07:00 GMT</t>
+          <t>Tue, 24 Feb 2026 13:00:24 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOem83dERqcmRmSmtFWjNqa2Y3NnBpVldLaEJVbWY0Q1FTNTRiRktXS1BVd01WQVNvQVp2VVFRUWdzdjk5RV91bXgtbFZweWdYeXNGbHU1QTl2ZzJuV09lMUdmVDNMTVVRMlBzQ3lJVS1SM3dWLUVLZ0FwTlVmZXpsdWJYbUtDNWtBY0xnUngwSEkySmwyWTFsSFFhZ1JWRUVJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPMDBYSXlQbWhUYXJYNTU0VHpqbEsxdTVYSnM5dk05UHlSSlJCSS1CMXh1UnFVcm1VZ0tWOVMtb1JFSlJQUnpyVTI0Ul9hQk5hQkdITEF6X3lfZjRFU2Rncm9sNzBhY0Zqdzdpcml4c3JmdVhobTVNUFJyTDJnZ2ExTWNxQTU5cE13dzlJNHIyV1BFRklKNl8yM18yQzlMQU5jbWlrYlpENA?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2010,42 +2010,42 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46077.42152777778</v>
+        <v>46077.54194444444</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Courtois va investir en Belgique : deux clubs mentionnés - FootNews.BE</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Courtois will invest in Belgium: two clubs mentioned - FootNews.BE</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:39:21 GMT</t>
+          <t>Tue, 24 Feb 2026 17:56:40 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNTlJDdTgzUm84dnhidVNwNUtTZGJqbWZZOVJmSHBzU1QyYmk4QV9ZanJ5TG12cXFKVDhVSHplR2dudWVsb3RlWjZUd0FpVmhHZFJfQzFnTlpvMnJwX2Y1Q3RLY1lzTlNWQ0JNSXAyalBMNm9YazVTenlGUXdranlMbjlwWUpSSlppbjF6SXU1aGJJd185?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOTVkweWFzUUNLdXBoYTJPUGNWeFI3c01LV1pqRWU2eExiOUFwOUE2MlZGaFBySWVJUmdUWGotM1BDS1lydWgwcEpZR3FlbHpuZmpDVVkyYWhNQnBSTEpMS1VscG9HOE1pREFTUlM0VHF4UV9UUjRybFNmaHpWMDlvdE5kZUt5d2lRYW9ENmFkQVFoMnZyRzY3VllEYVkzWEU?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2065,42 +2065,42 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46077.52732638889</v>
+        <v>46077.74768518518</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
+          <t>France’s ailing winemakers to get $60m in aid: EU farming chief - The Straits Times</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Official | Ousmane Dembélé and Fabián Ruiz out of PSG’s Champions League return leg - Get French Football News</t>
+          <t>France’s ailing winemakers to get $60m in aid: EU farming chief - The Straits Times</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:32:37 GMT</t>
+          <t>Wed, 25 Feb 2026 04:49:00 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNRHZ4dm0tREV0cjFucHowcUNrWGlJTVljdlFXcjNtdFg0OUh4a2hWb25ucnlzMkNMdThqU25BNm1yaHhBRk8zTDRwcHdHRHZFRUNBSVlHcXZjdDJFQU95SEVCM20wQm1YNmFzczRjdzE5UmZUY2NpWldzMWRfdXpSVmo4ZlpsVHdNOWo1aVFGcVRBc0I5RjVyYkRGeXZmVTBGZkFvNy0xZFVxa2JNZ0RzeGt2dHJCZTZHUTU1RXRZbzNpQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPYXV2clhjQ0RuS2RqY1B6clVlMEd3akNmekRNMWN3NUdUb2NGM1ZRWmk3Z0xGa3h0dS1UZTgyT0dwVVdCSXU1TTZPZWFHRVVEZThHRUJrdnF1dmw3UHNzRDh3ZkFhU0RvQ21MR3JfRUkzYzBnTDV5UjQ3ckl6MWQwZVNTbHJFZEF5QlIySEFiUlpDbWdXbWNBOUZ6SWllVW1sWkVLR2dtaVlrQXhLSUE3LXNkSQ?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2115,47 +2115,47 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46077.56431712963</v>
+        <v>46078.20069444444</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
+          <t>NATO Secretary-General calls for increased military, humanitarian aid to Ukraine - irishsun.com</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>LolaLiza acquired by three board members following management buyout - fashionunited.uk</t>
+          <t>NATO Secretary-General calls for increased military, humanitarian aid to Ukraine - irishsun.com</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:08:23 GMT</t>
+          <t>Tue, 24 Feb 2026 11:19:00 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxPNExOajRSMzJtQk9kOENCeXlHM25OUm5vVWQyUkszamgzQjVOMm92anAtdHN2QXhFLUVMLUptNVJ0YzV5dFJWTE5OeVNCMFVobnlyelUzeFBadlNFV3hCRVI0Y3pUTExVYU9TNFdwVUNsaXhyQjc2QW5MZlh3Rk9rejhZUDhEU1h3LUVQWHhBWHNHWG80NUltV2hxd1YwWmhRVVZyOHotOUdQeEp6UlVQYi1iVDZWcHFOanBzWWFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNLWpIMS1uWlZQRVVHWjFOUFBwcDhFYU1zdWhqSjRUMkFxU016cVRIZXlLVXQzWU9pQ0x6bmxLOFFUSlNlZGE0WG1pbDRaTzlNWDRxa1pvQ3NvMEpPZWhBRW9WUFhKUGRzVkZ5eHd0RlpBOWdZT0k1ZC01RWx2UFhBNDJURHplcV9IdFdKSzlJUHNTaG50MFlvRFg3T05iTGxpR2g4OFh3OVNYTVRNLWJ2Q1dIT1B2SG5TME9F?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2170,47 +2170,47 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46077.5891550926</v>
+        <v>46077.47152777778</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Village Maasmechelen (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Maasmechelen Village" OR "Maasmechelen") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
+          <t>Rute: Ukraine needs ammunition today and every day until the massacre ends - vijesti.me</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
+          <t>Rute: Ukraine needs ammunition today and every day until the massacre ends - vijesti.me</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:03:27 GMT</t>
+          <t>Tue, 24 Feb 2026 15:51:31 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUW54aFlQc196RnJXM0FfVWU5a2JSN2w2MXdiZVg0Z2U2aXdKZENsNThtVWVvQjg3U0FwUUQ2Qk5SZF9rSnVqQWxrc1VzOUNzcVRfbWVXNWFCUW80ckl3MHJlaTZvUElidlBqZWNlSm85a1otTXNBMkpYTlQ1YzJBcDVNNkY1a2o2OUJtNG1HYnItU2RodXRXb1pXMVFOTkF6ejk3cEY4ZTdRbTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNNkF0OEpmaXVhOVNvVnJOZVhOMFZCTzBrWTlHdjdOMUlwdVVBMHIxV2lFUkx6MjgxM3VDNlFlcy1uR2lYNzlCRFRlRzk4ajlXOHV4N1dNVC1fWGdlakJHbzZQc1NPSV9KZ2V2UFM3RGNidXEteDA1TGstcDBrUVF6QWVpQ0JFZHIxTU1wZEpqbWJ0Ykgtc1hQVngyWUsyTm1VamRaTDdoQmpUd9IBqgFBVV95cUxNNkF0OEpmaXVhOVNvVnJOZVhOMFZCTzBrWTlHdjdOMUlwdVVBMHIxV2lFUkx6MjgxM3VDNlFlcy1uR2lYNzlCRFRlRzk4ajlXOHV4N1dNVC1fWGdlakJHbzZQc1NPSV9KZ2V2UFM3RGNidXEteDA1TGstcDBrUVF6QWVpQ0JFZHIxTU1wZEpqbWJ0Ykgtc1hQVngyWUsyTm1VamRaTDdoQmpUdw?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2225,47 +2225,47 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46077.5440625</v>
+        <v>46077.66077546297</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>​Mainfranken: Polizei warnt vor verschiedenen Betrügern - Radio Gong Würzburg</t>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>​Mainfranken: Police warn of various fraudsters - Radio Gong Würzburg</t>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 15:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 17:16:59 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOWDNkYUtDak02bnA4LXVTd0lXVFpaeVNRTnVVNGk0VndJUy1oeXVkWm9IbTdtMWV5NnRCdXVSWmQ4LWotUEg1LVc4WVJ0Qk1GZHBDMVUtYlk1VjROTlpwM2R1RHhIX2cyX2xDWG9FNm1DN0hlYVZQWVJEbkRtUkpsTnlzTndjUnMwWm85Vy1USE8xZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNM185ekl4N3lkY3FGV2xtcHpCRDZicWFIVWpxeXZuVUVzNGc4SFpCa292cnVnaElFMUtnYlMyeVRXWnpnNWNfQmxFVEdzTk9ZVnFob3RqaDgxMTZmWlNaa3ZPWWtVeVU1YVI4SG1vUGdvdmVNUENkdy1fTUJPZTBkcUZGaW5BblhDSHFfbENWLUtoemlqREJHUjB3ZjBnS3AxNHZfZzdOTGdEYk1KV3ZNcVl4R0prelRHVW82SE1n?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46077.625</v>
+        <v>46077.72012731482</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Wertheim Village: Polizei stoppt mutmaßlichen Seriendieb - Fränkische Nachrichten</t>
+          <t>Alerte à la bombe levée à la Grande Synagogue de Bruxelles - 7sur7.be</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Wertheim Village: Police stop suspected serial thief - Fränkische Nachrichten</t>
+          <t>Bomb alert lifted at the Great Synagogue of Brussels - 7sur7.be</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:34:00 GMT</t>
+          <t>Tue, 24 Feb 2026 12:16:00 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNempGdjdfTkxudlBkZnlNYlNUS3h0MEluS3JYU2tOVW9zamM4QUdCODMyNTAwc0ZDY0NCYXpReG9wOTVtOUY2eW9rWmhxT0RHaUdubGNoWVN3SjBCaE8tSlBpSTlneF9aQnNMdHR0VDI3Wjk4el80OU91akJGYWV4aVVuM01SejN5NC1rQlg0WElRd2VJbXVhZEtjZEVwdDAtYlZnSFFjazhjOExOcGszYmt1X0hEUlZyQjl3aTRWXzZxWHJ1NXlJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOOTRkZE1mSU1wNTNCODJ6TEt2WWtuTF9yMUR4c1BOb3ptMExaU0ZJSUFyek96ZnpGaHRGRFd6aElmLU9WeXN4ZEZZazVsLTRUNDREamdwTGlMLXhsSHZoLTYta2gxNlBzUlhmRkdCaWZub0xBQl94VTdDZmZhU2s5b1R5TWRpd3BZV3JDS1NTRWRsUjZtemdVLTdaTmkzVDJEVzRCNA?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46077.39861111111</v>
+        <v>46077.51111111111</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Unfallfluchten in Aschaffenburg und Kleinostheim | Foto: Dirk Ceelen - main-echo.de</t>
+          <t>Le DJ set bruxellois d’Odymel annulé après des accusations d’agression sexuelle - 7sur7.be</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Accident escapes in Aschaffenburg and Kleinostheim | Photo: Dirk Ceelen - main-echo.de</t>
+          <t>Odymel's Brussels DJ set canceled after sexual assault accusations - 7sur7.be</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:03:01 GMT</t>
+          <t>Tue, 24 Feb 2026 19:06:00 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQMW02WVZqN19mTERhVXdiT194SUtPU2ZxVTJ3dGNKd2ZLQzVmM2lxb3lTdWpHVjBqOVlFTFVOYXE0d0czbUpZQzFFU19OT294MmdqVlU3d2M1QzFWUndPbm02SVBvakFlc0tVSnl6YXJjOUNaN2FvNUYwX1pOOGJ3aVJoZjlPOU9DWnFRZlBlZG5uNXN4N3ZvWnpYN21VX2M1Skppd2c4Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQTzBLc1Etdk9JRF9KVFBnV1hkd1dKVlFkekg0WlJaSzhGSkNsdTZ0bjBoZ3NVWnA3c1BxM0pnZ3JfQ1B0NFE1RjRXN2hsY0xEdlVZLUxmdDVnbjh5YTRHeUJnUkFUNVpzRl8zZFdXS2wtejliVW9tMkw0bzR4OXB6ZUxRQlBvdVBCamlBc2pSZVVXS1FZbWNzRFg4NV9MTHl4ejEwSnhFbFNsY3lZR3d5UGFSRHNhWk0?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2385,52 +2385,52 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46077.54376157407</v>
+        <v>46077.79583333333</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Marktheidenfeld: Polizei kontrolliert erfolgreich - aschaffenburg.news</t>
+          <t>Tribunal spécial pour le crime d’agression contre l’Ukraine - Le Club de Mediapart</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Marktheidenfeld: Police check successfully - aschaffenburg.news</t>
+          <t>Special tribunal for the crime of aggression against Ukraine - Le Club de Mediapart</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:09:08 GMT</t>
+          <t>Tue, 24 Feb 2026 13:42:46 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNM0F0V01ZMjFGbzFpQ0FldUNxRnI4UkplZ2daMUlzTXNvWGM2WnlUZGprenhxMXBfSkRrLTFkWUU2c2VFODdxRTU1bWF2bVNZeW9zWWVPaEtGU0ZfdUdGbVBKOGt3dEdmaUszMTdlZnFuNUV6b0JWUEFtVjBlTmdFQXh5SXhuZTN2eVVzelU2Z29RUU9wNGw2Z1Vn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQY09Xa2ROeU5aR3hzV0k2S1NHNS13MkhqUzJleTZLY0tQV08zcEk0MVcxYzJPTjRJMnFSY3pmUXQ3cTllSWFhaENkOTdJVlk3NDRRRF8yMkFrRmhteGR4VkE0VHExUXFxM0dudUdDemRlaW41OXJoNFlWTF9jVXlmT3FrOXZTT1gtNUF4c3RUbFNBZ2daSFNCRXptVkY2dUxZM0JBRGVzNGZjY0VrdlM2RTdB?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46077.58967592593</v>
+        <v>46077.57136574074</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>La Ville de Bruxelles supprime une taxe pour l’installation de panneaux photovoltaïques - 7sur7.be</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>The City of Brussels removes a tax for the installation of photovoltaic panels - 7sur7.be</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:52:25 GMT</t>
+          <t>Tue, 24 Feb 2026 08:50:00 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPRWg0V2dNa1lZdG1wUWp4V181cklFS3JlWnc0VkRIOEN3STFyRUtURmRRSlQ2U04xQlVMWERsbE12eXpqUDE4QjZPTFl1TDBOVzk4N0YtQzRGSXVYcE9QZDJnem0yZ0xGSkRLN0RWQzJfSDJYbDl6VmktQUQzMFZGRXBYcWpIX3J5SnVlWVlIeXlQVW0zbHNCQ0NNWXZyN2VXVWdLTWVYTU9BOGkwMGhWUmZDQ0o0aUg3bVd0ay04TjBWLWxo?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46077.53640046297</v>
+        <v>46077.36805555555</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Streit bei Auto-Kauf in Aschaffenburg: Männer gehen aufeinander los | Foto: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
+          <t>Halen keurt aangepast meerjarenplan goed na budgetfout van 5,4 miljoen euro - VRT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Dispute when buying a car in Aschaffenburg: Men attack each other | Photo: Karl-Josef Hildenbrand/dpa - main-echo.de</t>
+          <t>Halen approves adjusted multi-year plan after budget error of 5.4 million euros - VRT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 12:34:53 GMT</t>
+          <t>Tue, 24 Feb 2026 09:32:52 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQNXA4Vkl0TlZ2Ui1SOTgxNWVUcF8xdXdtOUJsODFOalIybVlxTkU3SURZVHc5aTFsdHNHMGR1SXNvNWZGdlgyT0dzbHZmbmtQMklfbERteC1yMWw4WFVvUzhGSWQyb1J6X3hPcmRBVkFfVkxMbEtkWDMtbGZWckV4LTZVLXBvUUk5ZEFNMlJ3SE80TXZ0V2JEakttUjJkWmtoX3djX01wY2dUbDhoLXQtRm1qVXpwZzlfM2UxWXRTYng?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPOTItcThiT1hZQjVXaDA5TEI5RUlVdmt5N1UzR2hEelF2aVBXemRfcTdNbk9xUk5sY2NfWkpJdmIycHN5TThoaVNnVVpCWjgzYXExeFpZUk91bVhhdFhiZ0szcDNRT3Nua3RCSTVUa1BTSGRUdU42TXJ3NzVYSXdFMTRZMkwwUVpqaURzNXJMMVIwbk1rNzNSQVdVaUVvdHRVNGNWcURCUzA?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46077.52422453704</v>
+        <v>46077.39782407408</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Kleiderdieb in Untersuchungshaft - NOKZEIT</t>
+          <t>Le printemps est déjà à nos portes : pas moins de 18 degrés attendus ce mercredi en Belgique - parismatch.be</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Clothes thief in custody - NOKZEIT</t>
+          <t>Spring is already upon us: no less than 18 degrees expected this Wednesday in Belgium - parismatch.be</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 08:58:15 GMT</t>
+          <t>Tue, 24 Feb 2026 19:13:00 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBKUUNfaWVwNkcxMmtpalVDTWxaMGNYQl8zZEVkWlFUMVk0UjFYa0Y0OEpFMERfaGMtSUI1dlU4cHVxLUJJMWxnV3FMcFdnNnQzc2s4RVVnamxfLXRxRjR3a3VYNkd0Q2pTcGVPb0lpTFE2ZE9KZUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxOdks2b214NE5TQ0g5LWg1RFd4QXpBVjVUWHJEOG90ai1VMnQ5RVd2V0JSeWZqbU4tVnRwOFphQmhTWVhLb2lCWjRVSk82RHI0OTBMRnNYMkQydU04OGRobTBHaE5VYnNrU05YRnJNR1B2YS1SSlZrWTBMSDdhRFh0SUtSYlpseTdySHFiNDZiM1RZY3E1NmJFLVlUWmZsY09tQmkzc1ZsQ2RMTmtXaEFaeFVVZ1dvNUFtMGwxRmJvaU4xaUsxN20xalBLZlNrUW1iWHo2dDRnRlltWE5ZMEx6cjltWXdPWHhMY09BZDRTTkYtS3p0d1RQS0VEQ3pDVktzZ3Vud29SMzNpV1h4?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46077.37378472222</v>
+        <v>46077.80069444444</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Herrmann begrüßt deutliches Personalplus für die Bayerische Polizei - aschaffenburg.news</t>
+          <t>La présidente du musée du Louvre Laurence des Cars a remis sa démission à Emmanuel Macron, qui l’a acceptée - Ouest-France</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Herrmann welcomes a significant increase in personnel for the Bavarian Police - aschaffenburg.news</t>
+          <t>The president of the Louvre museum Laurence des Cars submitted her resignation to Emmanuel Macron, who accepted it - Ouest-France</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 11:06:28 GMT</t>
+          <t>Tue, 24 Feb 2026 17:02:46 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNU0FPOVFwS1pZal9xUnlUNDVjT0wzY2xwRG5TUmdob3JERkNFdld6ZHdVTHJBdnAxOGl6VW5jeTNxMmxtWjZfSVdkczVTaVdTNFBIaEN0VzBTbUkzRHk0QlBJSEU0bEk0aVJIT0lsdnV6VE91WUZDMGRybGhMSmVMWEM1R2hId1pvN3E2Z3BOT2xYZk5vMm03Vjk3dHNfV3ZhS05OM3RqX3J0b25uUTRadzZLaDJXWk5KbzdmLTZ0OA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxQdEN5bFdMbTV2UVhqWlJUVV9xQWZxUkNFTmdLQUQxNklGcDgzZzBmRlFTaWMwLVBkeV9CY0pBLXdfZm9SSEdMOHdpbjVuWGRwNjRoTDFBN2hsQmQ0MzZmSHNEbUlyVWtqckJwNFdncklLWXJjTGd5NkpBdS1yamV4eUw4Qm8zZTBjaDVqMVNnR2VlNmU3OWY1X28wWi15cE9tSGZyc1VQaTdPN0lsR290N1NrdWd2TF9xcEhhTFFvVEtEWHNyZDNtNlYzQ0ZTWF81S05lbGZmOFRTSFZPMldETlVTYUl2U0g5RzNyZDVOTXlWYzNhMHhwTzNB?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46077.46282407407</v>
+        <v>46077.71025462963</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Würzburg: Messerattacke auf Zeugen Jehovas - Idea.de</t>
+          <t>Le Contre-pied de Jean-Marc Ghéraille : Beveren champion : l'ivresse même avec un Bob - DHnet</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Würzburg: Knife attack on Jehovah's Witnesses - Idea.de</t>
+          <t>The Against of Jean-Marc Ghéraille: Beveren champion: drunkenness even with a Bob - DHnet</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:00:03 GMT</t>
+          <t>Tue, 24 Feb 2026 15:34:00 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE55UThGQWVSVnBMUGM3RFpMeDJJbjc2Zi00aVhuV1lVeW9rZmw0WXdNdmZFY0REWGpQZUtUelROVXl5RE9KMkhJNlRoNUNvN09sS3Z3aTVjMWp3N0ZWc05CZmdGeWVPUzR3VXhBMFNkTnVWWWNTOFlwcnJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQMHJua1RueGFMeXhQSmRTN3dLalZiMmZaVVpydVhnS3JmNXpPSnZVZVd4X1VPQ2RkcllGTHhYLUFMWktIclZRS2lzTG9PLUpFbExiWlhfUWN1VU1IMVJjbjlGYlI3SGdPb25xd0RwN3dNck1yTFFsVy1yenBRZlZPZ3dnRTVmS1hpZTZXdzBjdTU2emxlZlM1QkdDVjA2VDc3RTZiTWZkcXVDVzdIVl9RblJ4TzZKZkhDTndVXzVoTkU0UlRqNE1zN2lPUWJpOXduTzZjWVRfMzV6QnR4Z2M0Rw?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46077.58336805556</v>
+        <v>46077.64861111111</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Erfolgreicher Callcenterbetrug: Falscher Polizist holt Wertgegenstände ab, Kripo ermittelt - Mainfranken News</t>
+          <t>Courtois va investir en Belgique : deux clubs mentionnés - FootNews.BE</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Successful call center fraud: Fake police officer picks up valuables, police investigate - Mainfranken News</t>
+          <t>Courtois will invest in Belgium: two clubs mentioned - FootNews.BE</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:06:37 GMT</t>
+          <t>Tue, 24 Feb 2026 12:39:21 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNRkZoQVNGWmlQVjB6c210V3RQRjYzeWxmU1RkQmJURFJhajlmQkVvRjI4V3d4U3AyQm1GajFjYUlteHcyYV9LcTQ3Z3ZMdklUbm9DemlqMkdvRnlTeHJJd1AzejlhMjlFOGJGYklWQlZ6cHRYekZYNkttNUFReWlieW5WVGY0aTRuVWRVZUZIRlpSZ1B5clJnMEh5VWtqVXZXbHZ3SnN5T0ZvSEJVa3h5X3hGdmxyV2pfSDVCejJ3Smd0NE9s?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNTlJDdTgzUm84dnhidVNwNUtTZGJqbWZZOVJmSHBzU1QyYmk4QV9ZanJ5TG12cXFKVDhVSHplR2dudWVsb3RlWjZUd0FpVmhHZFJfQzFnTlpvMnJwX2Y1Q3RLY1lzTlNWQ0JNSXAyalBMNm9YazVTenlGUXdranlMbjlwWUpSSlppbjF6SXU1aGJJd185?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46077.58792824074</v>
+        <v>46077.52732638889</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen English</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bomb OR explosion OR shooting OR stabbing OR evacuation OR police OR arrest OR threat) AND -sport AND -football</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Helmstadt: Nach Einbruch in Einfamilienhaus – Zeugen gesucht - Radio Gong Würzburg</t>
+          <t>Louvre president hands in resignation to Macron: Elysee - foxbangor.com</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Helmstadt: Witnesses wanted after a break-in in a single-family home - Radio Gong Würzburg</t>
+          <t>Louvre president hands in resignation to Macron: Elysee - foxbangor.com</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:00:00 GMT</t>
+          <t>Tue, 24 Feb 2026 19:31:08 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOeHEydHhfR29sSVFqWENkVEU5ekVMTnRTcmFoZXhIeFJNVTMzSGN5dzNjZjVtZVk0TnhtSjRNUmRTRC1OdndqNVV1MDJadHZUdlU5UjBtTVV1b2k0TC0wX25XXzdGQnk4VVR5Rno1akhMM19aOGRNZURrcmJ4cEh2Z05UVFpqQURvalNLcU8zcWZ4RG1PdWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxOU1hWMW5PLUJZZU4xTWIxSGxzUkZfVVZLcHJ5OE1UQnd2UGtiY2tia0VzLUpybmk2WU5hTXowTVVSbzVXX1hEQlJrLVdwTU9fRFNWSVN2MXlMZnNIcEtncGo3LXVfOTJDTmJyMmpkeFpDUU9rX0hUanVDcTdFQXdaYlR0Y0FHQ19sMW53V0dtZGZnLWZNc0taSEF2am56UUhaYThURWIzdmhJSThmNkJ2WnR2NXJQS09TbjB6eTlheHhjbWViWlplZHVTLWVJNnE0WVhWZEx1UVZCZGpF?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,52 +2825,52 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46077.58333333334</v>
+        <v>46077.81328703704</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Maasmechelen (fallback)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen Village" OR "Maasmechelen") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Unfallflucht an Rastanlage Spessart: Schaden an Kleintransporter | Foto: Stephan Jansen (dpa) - main-echo.de</t>
+          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Accident escape at Spessart rest area: damage to small van | Photo: Stephan Jansen (dpa) - main-echo.de</t>
+          <t>IKKS declared bankrupt in Belgium: dozens of jobs at risk - fashionunited.uk</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:03:26 GMT</t>
+          <t>Tue, 24 Feb 2026 13:32:25 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOQkJUQUtFSW5nMU05Unk5Vmx5ZkJXem1XV2JHVEFKSjBISGN6OU5wZElaUjlWZ0pZMGc0MHlJcEJqcDRSNy1od1dCY0dQdUZVX1VWdHJwSk9aMUljaXoxLWxmbWdZSnhMU0EtcE9DXzlRQVEyNVlpd1R5NnVvSElCVVF5TjB2VHZpLVpOUTJvYkdTVHlSTVhudzI4YmI0YnUycUpFLWtFMndDby04OU1aRWVZY2MwQmVKTE44?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOUW54aFlQc196RnJXM0FfVWU5a2JSN2w2MXdiZVg0Z2U2aXdKZENsNThtVWVvQjg3U0FwUUQ2Qk5SZF9rSnVqQWxrc1VzOUNzcVRfbWVXNWFCUW80ckl3MHJlaTZvUElidlBqZWNlSm85a1otTXNBMkpYTlQ1YzJBcDVNNkY1a2o2OUJtNG1HYnItU2RodXRXb1pXMVFOTkF6ejk3cEY4ZTdRbTA?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2880,21 +2880,21 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46077.54405092593</v>
+        <v>46077.56417824074</v>
       </c>
     </row>
     <row r="46">
@@ -2910,22 +2910,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Frammersbach: Falsche Spendensammler - aschaffenburg.news</t>
+          <t>​Mainfranken: Polizei warnt vor verschiedenen Betrügern - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Frammersbach: Fake fundraisers - aschaffenburg.news</t>
+          <t>​Mainfranken: Police warn of various fraudsters - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:06:56 GMT</t>
+          <t>Tue, 24 Feb 2026 15:00:00 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQmphdE5lMlFNZTFQYTdWTzBNU1pHMUc2YWlxZXFPc1BZWlBWZ2lnME9Xa29OcmFCeE5XeTlZS21YRTVSeGU1OEUtOHdCZTNwZE1CWHoyQkl1VlZfcDJQQmphOGh6V1J5YWs3cmhLSmU5Z2tFbGJuWGJBQlZxbEJPYXo4T2stUlVW?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOWDNkYUtDak02bnA4LXVTd0lXVFpaeVNRTnVVNGk0VndJUy1oeXVkWm9IbTdtMWV5NnRCdXVSWmQ4LWotUEg1LVc4WVJ0Qk1GZHBDMVUtYlk1VjROTlpwM2R1RHhIX2cyX2xDWG9FNm1DN0hlYVZQWVJEbkRtUkpsTnlzTndjUnMwWm85Vy1USE8xZw?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2949,7 +2949,7 @@
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46077.58814814815</v>
+        <v>46077.625</v>
       </c>
     </row>
     <row r="47">
@@ -2965,22 +2965,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Obernburg: Unfallflucht schnell geklärt - aschaffenburg.news</t>
+          <t>Wertheim Village: Polizei stoppt mutmaßlichen Seriendieb - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Obernburg: Escape accident quickly resolved - aschaffenburg.news</t>
+          <t>Wertheim Village: Police stop suspected serial thief - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:07:44 GMT</t>
+          <t>Tue, 24 Feb 2026 09:34:00 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQWDdoMzlzRi04dVVnRzU4ZmFHbElQdTh1SFVrZWFJakZUYUVRQlk4MExVam5lb3U3XzFWVy1keWczZzJ1a3pBai1GR0E4bDRYR3JiMWY0UVVtb0ZDaFdaR3NCa1ItcjRSajg1Ny1kOFJFaFI4VWVnd0pBR1FfMndCNFV5SFFIQVgtVml3ZFUwc3kwX0hvUzRURDNwVDdkVHV3czBQVTlR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxNempGdjdfTkxudlBkZnlNYlNUS3h0MEluS3JYU2tOVW9zamM4QUdCODMyNTAwc0ZDY0NCYXpReG9wOTVtOUY2eW9rWmhxT0RHaUdubGNoWVN3SjBCaE8tSlBpSTlneF9aQnNMdHR0VDI3Wjk4el80OU91akJGYWV4aVVuM01SejN5NC1rQlg0WElRd2VJbXVhZEtjZEVwdDAtYlZnSFFjazhjOExOcGszYmt1X0hEUlZyQjl3aTRWXzZxWHJ1NXlJ?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3004,7 +3004,7 @@
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46077.5887037037</v>
+        <v>46077.39861111111</v>
       </c>
     </row>
     <row r="48">
@@ -3020,22 +3020,22 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Blitzer in Aschaffenburg aktuell am Dienstag: Hier nimmt die Polizei am 24.02.2026 Raser ins Visier - News.de</t>
+          <t>Marktheidenfeld: Polizei kontrolliert erfolgreich - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Speed ​​cameras in Aschaffenburg currently on Tuesday: Here the police are targeting speeders on February 24th, 2026 - News.de</t>
+          <t>Marktheidenfeld: Police check successfully - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:18:00 GMT</t>
+          <t>Tue, 24 Feb 2026 14:09:08 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPTVBpWlNVVWhJQTJIZ0xMUkVmR2dOWmtjZkxfaDJIcDJXUHo1Z2d0T0RGOVJXdmVmRV9PQ0p1ZUg2dlVaYXhqVERySGpCM00zeGlxNnZWMjZfQzRPZzhHTFRrODVTNUlLcFRGTnpQQzJFa3pZaDNjQzRaOGpMWno3Z3ZZaEpma0xtbDVzU3I5TV9EaGVnbmpHdzlWRUxmY3NMeFg3RnhxWDRfZElOeXVDeXVXZnpaaXNwTjNWc1IyaXNTQmZMbVlZa09qVURBYTJsQmlUdDZXUEVEeDFXZHNPZE9TQmtiSmk2M3puY9IB8gFBVV95cUxOeHd5dHFsS0VxRHViWnMwbzlwYjl2VFhheTA4a0xFTjNCcWM0S0VQR1ZkRms1eVFWdzVrcUp0RFhhSkZqRE1fUmFVd3VQVVZWVkNrNHE5Y2g5U20yMlNKb0h0T0MwTVRsRkxoa1pvdU52MzFNUE9ac0FBdjRQTE5Xbko3cjNGaTkwX190N2wxUjljcGRsLTJJZEZfM2h1aHVFcTBkYUJLaExSMm9zUXQwRE5hd00wVVc4YVMyQ0ZfQWlJU3B5Y09obzh0bHFBUGpsWmw4VC1mUFd3dmVxUS14b09IRGhxeEhzLXQwV1MzdnVZZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNM0F0V01ZMjFGbzFpQ0FldUNxRnI4UkplZ2daMUlzTXNvWGM2WnlUZGprenhxMXBfSkRrLTFkWUU2c2VFODdxRTU1bWF2bVNZeW9zWWVPaEtGU0ZfdUdGbVBKOGt3dEdmaUszMTdlZnFuNUV6b0JWUEFtVjBlTmdFQXh5SXhuZTN2eVVzelU2Z29RUU9wNGw2Z1Vn?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3059,7 +3059,7 @@
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46077.3875</v>
+        <v>46077.58967592593</v>
       </c>
     </row>
     <row r="49">
@@ -3075,22 +3075,22 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Corona-Zahlen im Landkreis Aschaffenburg aktuell: Die Coronavirus-News aus der Region - News.de</t>
+          <t>Herrmann begrüßt deutliches Personalplus für die Bayerische Polizei - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Current Corona numbers in the Aschaffenburg district: The coronavirus news from the region - News.de</t>
+          <t>Herrmann welcomes a significant increase in personnel for the Bavarian Police - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 10:39:00 GMT</t>
+          <t>Tue, 24 Feb 2026 11:06:28 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxQaUEzVnI1RndRNXNjVEEzZ1phUmhtempTcElXZld6R1lVQTZuYmFKQWdYN25qclF5TE54T0UzTU9iWnZSc0RydTlpMGRjZ3ZyM1hWZDh2SlBHLXJPTTN2T0d1SDJkT1RSU1FpckR2bGQ3MHlTU2MzWU1WdUVtTnRvdzN5LTJSRVJ1Q1dqMFlOS2lia1E2bWNxZ2RUMzhzS3Z3Q1ExcHlyYUxydTFkU0lIZ2hIMlZNRDZXZmlOREFzVUs2YmxrN0lOZ0FDWGxCZzIxY1djYl9RLUJGeExvOG9VZ0gyTF9WODdVdVp5LS1WOTZRNkNlQkwxZWdBZG01VmPSAYQCQVVfeXFMTUphRTNneGpNMmxrczR4aGUtLS1PT0swYXJ4T2RWOWVvZU5XNG4xckFrSm8wT2RSVUNCSG5GQlJCcm9vX1p0THJITHAtN0xldjhacjR2VXFfUWVCdXg5SjFlSEpTN2lQLVE5M1AzcjhVdEVTa3ROV0tFbmNhWlVmcXBjUUw5ZzFfZkE1amdCdFZxRkd2c2x3dk1DbXRYR1FBWW9sY1g5ZjhPNXE5WXF0U204Z3RHWlVGVDlKdG1YeVAtYXB6ZGhoZ3pXMEp0cTNyS0o2dXhGRDFDV2JCYWlWbDFfXzZVVmJ1RjRKV09aZzNqZ3pETERxU2cxUUhYM0dNZ0xlSV8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNU0FPOVFwS1pZal9xUnlUNDVjT0wzY2xwRG5TUmdob3JERkNFdld6ZHdVTHJBdnAxOGl6VW5jeTNxMmxtWjZfSVdkczVTaVdTNFBIaEN0VzBTbUkzRHk0QlBJSEU0bEk0aVJIT0lsdnV6VE91WUZDMGRybGhMSmVMWEM1R2hId1pvN3E2Z3BOT2xYZk5vMm03Vjk3dHNfV3ZhS05OM3RqX3J0b25uUTRadzZLaDJXWk5KbzdmLTZ0OA?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3114,38 +3114,38 @@
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46077.44375</v>
+        <v>46077.46282407407</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
+          <t>Unfallfluchten in Aschaffenburg und Kleinostheim | Foto: Dirk Ceelen - main-echo.de</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
+          <t>Accident escapes in Aschaffenburg and Kleinostheim | Photo: Dirk Ceelen - main-echo.de</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 13:17:11 GMT</t>
+          <t>Tue, 24 Feb 2026 13:03:01 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOYl8yTkRYaUVVaUU4eE4wZk1aSTVxbkNEVzg5MHF5aTI1bGZnZkxweHgzM3MwUU9BekdUVVNlV3pPV0J4NkJuM0ptYzlsa1JxNUNCZjNqdmdldHkzRnNMSnpidGhTb2h3LUYwR3VXU3BnX1Z4ZDY0dkJRd3JiMUpYT0FZbjVyNzJf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQMW02WVZqN19mTERhVXdiT194SUtPU2ZxVTJ3dGNKd2ZLQzVmM2lxb3lTdWpHVjBqOVlFTFVOYXE0d0czbUpZQzFFU19OT294MmdqVlU3d2M1QzFWUndPbm02SVBvakFlc0tVSnl6YXJjOUNaN2FvNUYwX1pOOGJ3aVJoZjlPOU9DWnFRZlBlZG5uNXN4N3ZvWnpYN21VX2M1Skppd2c4Zw?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3155,52 +3155,52 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46077.55359953704</v>
+        <v>46077.54376157407</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Sexueller Übergriff am Bahnhof: Kripo Ingolstadt sucht Zeugen - Augsburger Allgemeine</t>
+          <t>„Messer in der Hand und gebrüllt“: Mann griff am Montag am Würzburger Hauptbahnhof Zeugen Jehovas an - Main-Post</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Sexual assault at the train station: Ingolstadt police are looking for witnesses - Augsburger Allgemeine</t>
+          <t>“Knife in hand and shouting”: Man attacked Jehovah's Witnesses at Würzburg main station on Monday - Main-Post</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 14:34:12 GMT</t>
+          <t>Tue, 24 Feb 2026 14:35:00 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOYVpQc2ZubWFubEFJeVhURXhHUWlPa24td1QzXzVWS0dmdEJCN0VVRGNfNjEyZjNuTEZyN3IwWWo0cFQ0SjRYQUs2VXBJWGUwMXY2ZG9wc2V3UmM2WW5ZaUZkVTNWXy1mcVpNcXd2NE5SRklKSDh3aklIcUMwWDJnSGxyNms4N2ZETzg5QTQxZzd6Q1dJQ1B3akVZMkR6UElYenU3clBPOXRLaTNmTGVxYjdLU0NsQmY1ZXJEcVBSWmVlZGpmZS1BeFBqeUFZQXdJaWZKRHBKbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQYlNWeWdpWVoyVW5tMkJSWlBDTDRsNW16Q09RQUFsMTQyVXFObUE2YTZHZUxsUXA3YllJbWRKYnlLb2kxMmlpRld4T1dKZ0dsWWFycHhxb1RUem1VTzZqNW51MDh6c2RBcEt3SjZaNlhDOC1acDNJXzhWSFRTMWROWHdsWFUtbXg3cjBrY05rUEE5YlUtWW5lakVNNmUxOFowSmRmbVRqTjZiWWRoV01CcXZTMkZHdjZHZWtDRWNTYmh1bU13eFFESFFGOERZR2ZXNDhtOVJBdzk?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3224,38 +3224,38 @@
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46077.60708333334</v>
+        <v>46077.60763888889</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Village Las Rozas La Roca</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Las Rozas outlet" OR "La Roca outlet" OR "Las Rozas Village" OR "La Roca Village")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
+          <t>Demo-Termine heute, 25.02.2026: Hier gibt's am Mittwoch Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
+          <t>Demo dates today, February 25th, 2026: Here on Wednesday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Tue, 24 Feb 2026 09:21:06 GMT</t>
+          <t>Wed, 25 Feb 2026 05:55:29 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPd0dBclgxSVlFV1dtaEgzNklSZENrcDBPVF9kbEZOWUZhMGtfS3BsS01WWlpwMERQMHVtUUcxaG1EaFlyV3NONy05ZlQ1TzRPTG9lVDUtZE5xVVZEbUdBTFdkNlB5TEhTb0FmSWJlOFpqTXVVLWhvd1JaYzkzNGNMaVBmaGpSaWZ0dHJ1cnBXQndERXZMN2ZhSWJSNlFPNHQ5MFMwbUF1WHRIXzBXOUxpQmtYdWgyNlpDaVhEdjcwYXBGLUtQNzQwdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxQNFdodW8waDJhejU0ZGtoemRUWV9YRlZ1TEtMeVk4WU1RT2doLTBsOEZ1Z29mZS12dFJoYXF3dDVBSHM2eFg5NzloLUVsYjdycDRsc0FnZmtxeExBb0ctcmxyR3FwRXYxbmhDSmRQYXRJUGNPRnQ2cmRzMDJQazZTMUd4RWNlV0NSbU5NUWlYNTROMnZqbllmUnpicHU5RFZscHVjR09rV2pYLWVxck5UTzY2d29aeXd5WUhjQTRfZ1dERXZGNHpxNHlIWXh1SHFBOVcxTDRzS0Q0bmtDdHZuS3FSQlpydDg4WDdVU0pGTFRXUTdvalJkS3N6VVVPVWvSAYQCQVVfeXFMTWNydll2dWxMbEUwa2RNY1V3RVVER2ZjTmZFbGUzdk42M25oYUtONnhPWGV1SXVtcDNUYVlZVVUwVkk1ak1FME9RTWI4aFZtYU9uMHZqRHZkZGtfRFRwTzhnU3NKMEJISHNNaG5XXzdBOXZVQnhZMjY2RnRNZTZWRlpXenRWVWVaVGxYTTBxbmtqRlBPMjktSlBlLXQxOTgwRGZacW9IZTRScFduX0hCaWc5ZGJWc193RWxmd2NkZjFRYVJ6MF96RkhNRGpVRnVsQ3RBUzlLM1VaalRpREdjaFZEY3BrdXZwc25sUXRTNWJ3R3ZsUHhmNUJNSkNpeVRWZmdoaVE?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3265,76 +3265,846 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46077.38965277778</v>
+        <v>46078.24686342593</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Giving | Staff - FIU Herbert Wertheim College of Medicine</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Giving | Staff - FIU Herbert Wertheim College of Medicine</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 21:09:35 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE9od1VFYUdJaUw5WmNDdFZBaEtfY3F5WWNfRWNrRmpyc0F2V01OTnFVV3ppY1pqYU0yTGpNN29uUWdpcjIxOUprWTJOVG9vZHV6Ym9MU1BGRnNGM0ta?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46077.88165509259</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ESPN Signs Andy Roddick As An Analyst, Andy Murray Reacts - Last Word On Sports</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ESPN Signs Andy Roddick As An Analyst, Andy Murray Reacts - Last Word On Sports</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 16:55:39 GMT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxQd0NveEJPVzlTRG9uTzFEcGt2a2Z4OTBfeGU2dWJsMHE0ei1abXdXQS1TM1NKS1BwdS1seHA2b3VQaHFaYWI4QjVpUExLZGNKVWRLbU1UcGVUYTgwR3BHS3pNbk1LTXdqdEdkNTZIWElLTkpMQVlIQUxuOVNFdDFnS0xiYlVnSjF5bVc4?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>46077.7053125</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Jon Wertheim suggests the reason why Serena Williams might be planning a WTA Tour return - Yahoo Sports</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 13:17:11 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOYl8yTkRYaUVVaUU4eE4wZk1aSTVxbkNEVzg5MHF5aTI1bGZnZkxweHgzM3MwUU9BekdUVVNlV3pPV0J4NkJuM0ptYzlsa1JxNUNCZjNqdmdldHkzRnNMSnpidGhTb2h3LUYwR3VXU3BnX1Z4ZDY0dkJRd3JiMUpYT0FZbjVyNzJf?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46077.55359953704</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Andy Roddick says whether Serena Williams should return to tennis at Indian Wells next month - The Tennis Gazette</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Andy Roddick says whether Serena Williams should return to tennis at Indian Wells next month - The Tennis Gazette</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 01:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNemVFRjNiSDAwYnFfVjBWRnk3Z01tOUtaenQ4UWo4aXQ5NlRpS3BFZU9MQTlNZUVqZm1wT1ZkUjVkY0hOeER2WDE4TUVkS3pBMWtfSHFLMVhlaXF6cVJ5bm5reU5wVlR0dXpPTktaZ2FBOVpNZFNIQmdJTDdLOU9EUkVzcEVvSTliUzhXQnBqOTRienJaYkIyeWd6cVhFNXVyR2t4QndsWDJ3RUdlMWZvUk80NzFnczEzLWhuMmRkVFVMaV9UWFc0d24wMA?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46078.04166666666</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>FSU auditing scholar ranks among world’s most prolific researchers - Florida State University News</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>FSU auditing scholar ranks among world’s most prolific researchers - Florida State University News</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 18:53:47 GMT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNWnZRdlpabjN4UmRMTWhtTmtrU3lpVVhES3Zpei1aWEJhTGFxOHppY2V5R05MUGs1Z25BcS1CX3hvNTF6M0hFVWVIZ2V1VEpNUHh4dC0yRzZmWllKNlFZaXNTTXhIVURRLXRtV1dBdk9wT2FNZ0F2UjZJMF9RVVJlN2UzM1lZMzB1VlFDYU5qTlJIMHhjbE9fVnFROHlIN05sdWtmWWNrNUp1eW9ZVHNsV3dUSWJhSFBKeHlpcDBGdDM?oc=5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>46077.78734953704</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Sexueller Übergriff am Bahnhof: Kripo Ingolstadt sucht Zeugen - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Sexual assault at the train station: Ingolstadt police are looking for witnesses - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 14:34:12 GMT</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxOYVpQc2ZubWFubEFJeVhURXhHUWlPa24td1QzXzVWS0dmdEJCN0VVRGNfNjEyZjNuTEZyN3IwWWo0cFQ0SjRYQUs2VXBJWGUwMXY2ZG9wc2V3UmM2WW5ZaUZkVTNWXy1mcVpNcXd2NE5SRklKSDh3aklIcUMwWDJnSGxyNms4N2ZETzg5QTQxZzd6Q1dJQ1B3akVZMkR6UElYenU3clBPOXRLaTNmTGVxYjdLU0NsQmY1ZXJEcVBSWmVlZGpmZS1BeFBqeUFZQXdJaWZKRHBKbw?oc=5</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="n">
+        <v>46077.60708333334</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Restart after the break: Red Bulls host Ingolstadt in top match - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Restart after the break: Red Bulls host Ingolstadt in top match - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 17:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNUFljMGRGOVlqSlNXT2ZCYTFGSVJMNllmTF9LVFhFVWJhb0NnZ1lWZTY1cmdKejZRbi1nV19zdjVKUGs5d1ExZHdwZEl1aXdkQ0s5eXBUT1lYY3BtZ1V5MjdxeG5jZzJvaWpURWVORTQ0eVExSFBoMHBuSE1mazhVa280M19FNXpETU0tNkpJSEM4ZkM5VU8tOVFyX3M2c2FVWHkweDZ5MGVhYzkteTVPQ2hya1o?oc=5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>46077.70833333334</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Germany's FC Ingolstadt makes special collaboration with Kashmir's design house Pumposh - India TV News</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Germany's FC Ingolstadt makes special collaboration with Kashmir's design house Pumposh - India TV News</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 07:15:30 GMT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxOaDJGeFRzT00tVDBFTzU0bW9IeFFHOUdGa3A4Wk1kVG1Ed1VIbi1tSVdEd2tfdTRIcFRVU19oVkRWUG11OHVBUnVtMHRpMnpmcldxTzUxQmUyX3FxVm5XVWhGMXJZMHZ2Um95RVVKVDlLYkFselFaODBPTmdVUFlqRm1EU3hzaEFQcGc0VENqdmNmYVItZ1ktOVFITG9EbjJQVW9wN2xNejJJTllobXhBV016MF9ROTRHRXh6THlQMy0zdE5IT2V4ZVhqb0UyY1JoZDNxZnE4bmxKSHVhbU85bnpHU2Z4Z9IB6wFBVV95cUxNUTdkcE9MOUlfSndGTER2U0Z3anVFMWxqM1RDYThNZ1lNQm0tLTc3MHRlNVRRanpyU3pyRGFYUXZQTE4wUEszaDFkVHNJUzRUTlczUGxNSHJQS191ZnRoOUVoVVZGMWZMME1rdGFpaFVOSzZNNEl1cm5aUEFpMkNwWUJDZk9KNGZGSmlaWHZySXd1bE1KNHVJdDNyN0xRYWdYUWExM2ZpZS16M3ZwYUdmTTczeklEQUR1NHhkRVd5ZGFYT0lGcUk4SGtfNml0TjZ2RnZFSGVRLU95dGE2V2JfZjR0RXQ1a05aaFpv?oc=5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>46078.30243055556</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Kashmir’s Sozni embroidery scores international tie-up - Greater Kashmir</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Kashmir’s Sozni embroidery scores international tie-up - Greater Kashmir</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 18:13:16 GMT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPRFpzbUVlOEdhUXpURGZlRHdXZENLSW5RbHlua0lWY1gtajI5Y3dVTllfZGo2amdKXy15emZuQTlTcWJhUWFnNXVSVFZTQ2JaMU5TTi1GbzZCcV9KY2ZDYVFYTEplOFVobktnRzVTWTU0Z2ZEc1NhRnc5c09uYnd6RHBjNVVJNXRSTkpkdzZFNk5xUVFLM3NTcjRqNTk3UTFYUFlr0gGjAUFVX3lxTE9EWnNtRWU4R2FRelREZmVEd1dkQ0tJblFseW5rSVZjWC1qMjljd1VOWV9kajZqZ0pfLXl6Zm5BOVNxYmFRYWc1dVJUVlNDYloxTlNOLUZvNkJxX0pjZkNhUVhMSmU4VWhuS2dHNVNZNTRnZkRzU2FGdzlzT25id3pEcGM1VUk1dFJOSmR3NkU2TnFRUUszc1NyNGo1OTdRMVhQWWs?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>46077.75921296296</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>In Defense Of Car Bloat: Why Performance Cars Must Get Fatter To Survive - inkl</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>In Defense Of Car Bloat: Why Performance Cars Must Get Fatter To Survive - inkl</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 13:00:08 GMT</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNbTJrRkMyM0hCTDRZXzhicnVUTVRaUmRGSkNPMXBLejN2cnl4MS1RSkVhOHlfbzVtUHhEVkwtOUpLTGNPN1Z0d1JvVG1fX19tYWR5dzF5RGlRQ3FDa05jbUc5NGVMRzIxNWxneGpLR0xJcU15T056VjRuSzFKdHRLNnR2TFlzVjd2YTR2VGhfVUJtVmhNLVBUenhIcF9uQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>46077.54175925926</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>PENNY DEL gibt Termine der Playoffs bekannt – alle Runden in der Übersicht - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>PENNY DEL announces the dates of the playoffs – all rounds at a glance - EHC Red Bull Munich</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 13:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQZ3Rhb09IdTNSaUxZTWRmYXhsTWY3V1IxN042WkJPZUQwZk43SDJ5MmNfa3hIT2hvU2hYT1hneUt2TlhSWFVQV3cwNS1iQnVfbk42Ty1UckkwcXdRSU5FbVNvcWR3M2J3eVhTNkdvUkdVODhGY2NxLXJUTmNzLTIyT2pHb2g5NW5mQ0t2MGx5bUVoOUYxWlhvQXNyMHZZd0tTQjhkN3RXUU5kZl81U3NJNTBB?oc=5</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>46077.54166666666</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Village Las Rozas La Roca</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>("Las Rozas outlet" OR "La Roca outlet" OR "Las Rozas Village" OR "La Roca Village")</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Movie-style robbery in Catalonia: in just a few minutes, 120 e-bikes worth over 300,000 euros are stolen - Brujulabike.com</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 09:21:06 GMT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPd0dBclgxSVlFV1dtaEgzNklSZENrcDBPVF9kbEZOWUZhMGtfS3BsS01WWlpwMERQMHVtUUcxaG1EaFlyV3NONy05ZlQ1TzRPTG9lVDUtZE5xVVZEbUdBTFdkNlB5TEhTb0FmSWJlOFpqTXVVLWhvd1JaYzkzNGNMaVBmaGpSaWZ0dHJ1cnBXQndERXZMN2ZhSWJSNlFPNHQ5MFMwbUF1WHRIXzBXOUxpQmtYdWgyNlpDaVhEdjcwYXBGLUtQNzQwdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>46077.38965277778</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Bus stop in this Kildare village may be moved - as new route is built - Kildare Now</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Bus stop in this Kildare village may be moved - as new route is built - Kildare Now</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 20:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPX1ItOE1UMVNYQTlkVzBtT2RiNWwwd214SFNKOEFobWoweGt0M3B1eTFfU09sNGNWM01YNVNYQ1VHN243UXNrTU1LdG03Vk41SUtmTnBoOUtYQ044ejdoVlFacm13dEVoRlZhTmY2NmJCNm5SbGJOdGpiUGxlbEVsMWppSV9CeVVURDRNUWJvQjYwaEVvN3NncXo3M09QUm1lVnhTbTN5di1GNU9sbUE4dlF5eXRXZlZmbHZYTl9mcw?oc=5</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>46077.83333333334</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>High Level City Italy Italian</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>Zola Predosa (Bologna), sparatoria al campo nomadi: «Un pregiudicato colpito alle gambe» - Corriere di Bologna</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>Zola Predosa (Bologna), shooting at the nomad camp: «A criminal hit in the legs» - Corriere di Bologna</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>Tue, 24 Feb 2026 08:41:43 GMT</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTXZ3cFF6NURKMDl5cGZSWFJWQ2ZRWk95Z2ItemVwYmlVd1BhMm9LX2Z5YmJiOFp5b2lNVE00TVdpWUlnb2VLd3B2VnJnckU1R096NU5nTFM0dmFlU2o1WUlWakN2dkttY2Z3YlZ6akF5TnhZb3g5QkV2ZXRXSnRvR0IxZ1dRMjMxWmVaNUNTcXJIaUVYVXp5eXdwdUN6ek54Z2o2dVdybmwzUC1MS1pBMjQ1d1g5UWZFSXQtMi1MeXhleU9LWlBMeV9HaUhDczQ1bmRIMVVxaHZKR3hsWWZ0c05rUTZ5ZXFpWFdV0gHwAUFVX3lxTFBIZXFtcm93OHQ3bmZIcTdUcXV1VmN1Tm56S0dld3pCVDEtS2ZYdVB1bHYwNzBqUjhyc3ZhSUM0S3p6b09JQmtiOWI3ZmlfOUs5OWxMci0tX2NFckV2V0VKQ3Uxam1rWWtEa1dpdWdZcHA1T0JVLTVneS16d05NVmxJVjBOMDdDcHJaUW5lYS1JamdtcGFlMHhneTJkTE4zeWZtbXhNZWRtWUZQbHpIR09sNWxGZ3ktLVVVSVZlWG55eXYzX3BQV0M0MkppUVlNWU1PU3czUnRMTUNRVkVzWUlyYWhPZGs2MUFULTU2RnNFcw?oc=5</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
         <is>
           <t>it</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I66" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="J66" t="inlineStr">
         <is>
           <t>IT:it</t>
         </is>
       </c>
-      <c r="K53" s="1" t="n">
+      <c r="K66" s="1" t="n">
         <v>46077.36230324074</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Local Town Fidenza English</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>("Fidenza outlet" OR "Designer Outlet Fidenza" OR "Fidenza Village" OR "Parma" OR "Piacenza" OR "Cremona") AND (protest OR bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR evacuation OR "police operation") AND -football AND -transfer</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Parma police welfare check on man who made 'suicidal statements' ends with deadly shooting - News 5 Cleveland WEWS</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Parma police welfare check on man who made 'suicidal statements' ends with deadly shooting - News 5 Cleveland WEWS</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 21:46:19 GMT</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQbTJBbWl5WFE4TTZJLU5XcDd6c3FYM0Z3OE8zQjNJUHE5c0FibWdKb0dJbk9VYjViMDBsUFhMZmUxQVdsVkVralpIS1l0cnFTQ2tYazdYTDNDX1VMX2RxWURSbjVXdWlIbHYzWGNVbkNyVEJ0d1hlMzFJZGFUMlV1b0t2eDB2UkNfS2VGcGtvTmwtRzVPbnFFYm1TcjI3N1ZoYldnenVZXzExR2hzUlE?oc=5</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K67" s="1" t="n">
+        <v>46077.90716435185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-25 14:49 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,32 +590,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - Yicai Global</t>
+          <t>U.K. shares lower at close of trade; Investing.com United Kingdom 100 down 0.03% By Investing.com - Investing.com UK</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - Yicai Global</t>
+          <t>U.K. shares lower at close of trade; Investing.com United Kingdom 100 down 0.03% By Investing.com - Investing.com UK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:52:27 GMT</t>
+          <t>Tue, 24 Feb 2026 17:28:26 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQQVhnQ0Y1UWRwRmdlb3JBNlR3NG9RYzhSZ0thTkhtWHRKWW1rbjdRYmJKeXJzeE8wMUpiVTZ5aV8tWTVZQnA1LU5NejhlREM2SmluVjI4T0dKMk5kdjBtQkQ1WXhmWkJHVFV6YlgzcXBfaTdKME45SVFZV1Aya3pfRTZPVFBBSTFrd0JBZHNlbmd3R0lNa1VTZ2NFcS1QTmhvVy00S2p4Mmt6SkVwTXU2QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxPX1E0aWNNVzZlX0lpb29OUnFVenZNSk11UmU0T25UeHFXS3gwdFZ6SWZCc3E1a1Iwb3NnV0FFNHY1ejdLcFFTekpqUmlNQzRPaE9sZlJZRk5LcTB2cDlSYjk1Mk1kelhKakNoV082dzBwWmNiWVVIb3lEN3I1OWN4OXNHcjBtMUdObmEwWkNjNmlHZHNRZmpUU1JhbDgyc1cxMFM2bllyRXlMUDd6OGNDSUJyZW81QU5YYVFjTHNUX18zbkhWZ1V1M2RvdVRTOWZhMGRDOUF4OFVLQQ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46078.36975694444</v>
+        <v>46077.7280787037</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
+          <t>IRFC shares falls 4% after OFS opens for subscription today — Here's what investors should know - CNBC TV18</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
+          <t>IRFC shares falls 4% after OFS opens for subscription today — Here's what investors should know - CNBC TV18</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:32:50 GMT</t>
+          <t>Tue, 24 Feb 2026 23:18:47 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOY1NoSnNJUHdDZVlIYkRJazd4c01fay1YMjNDQU83U0pPczJYdmRwbUFKQzV3S21sTFBnQXNoWmhhNjVoWG03N1ZZUnJRSnpzdC0wamFZY3lRWWpBMmFzTmh1LVlzT3RlYlZabDYzWG81emRxRnFxUWVZVGNuU0xDSTJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxONklGTzgxZkEtS0padGhMcTBPRm5GRndzR25DX1dWN2pYU21md2hVRW5tdFBVSUxNOTBlQWpSTVhKUnRYUWNyRnNjb3NUdXoxM2lfNlFzdGVtUXBYVkUtbnBZc3EtWmtFR0xuUlJETl9uVmp3NmZCc0VOb24tRHdRclk5YWoxQzFlSlBBMDhzamEzQzdZU21qUWVjSGU1aFQ0M09qaEcwOWxaWUZmb04xTE1aeW90eTVNclRESGpFcjY3LWhLWkQycW85S2k1djRpNE1WbmpDNjRnSzdfZXpTeEhlWDI1bHk5YVFwYm1R0gHzAUFVX3lxTFBSSnVqYlZqN1RFcVhTZDhRazRvYzNQX0V0VWNhTHBKTHhnZzlwX2c3dDF1c0E1emJ4bGJ0Yzl1Vm5rTVNoSWtEOEp6N2pYT2FuT2J1VkhHNXRKcE8zSE9GWENIdXBMX0dJS0p6clhyeGNfVS1WbUExWmFEekhrYnd1LUNKNTQtR0VrMGJqZ25KWEhZMjdKQkxRU0pvNUpjV01INUx0QjQwYnFTTGtDbGdGbEhFcVg2V3JDZ3lhdzJGYUlRZXkwTlRJdXRCbnJEZzByQXB0NWpNUnRkNDRlbzhpRUdmQnJ1SlJjeU1xMWR5Tm1JZw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46078.35613425926</v>
+        <v>46077.97137731482</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Verdachte van taximoord in Geel probeert tevergeefs vrij te komen: ook in beroep blijft A.B. (20) aangehouden - pzc.nl</t>
+          <t>Bicester fire: Explosions heard as blaze rips through former RAF base - with smoke seen for miles - MSN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Suspect of taxi murder in Geel tries in vain to be released: A.B. also remains on appeal. (20) arrested - pzc.nl</t>
+          <t>Bicester fire: Explosions heard as blaze rips through former RAF base - with smoke seen for miles - MSN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:40:00 GMT</t>
+          <t>Wed, 25 Feb 2026 00:46:40 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQV3Jwel9IeFZBTEN1d1hoME4tRkYwQVJqUkM2SFZNLWlKbU9wdUZsa3pFMHh3bXJmUEpQRld2UHhXZ2hUSmRJZ2ZXeFdsYXNPS2lKZFFOeDFhd24tWDUwMERCbjdEUS1KMHkzLVAwdkd1eGpUVjdfYURRQklXQ0JxNUJ1TDNkWk9VOE0yU2tEYmVPUS1CdVB5OWN0U0ZvNG1PUzdfZjdXT05LQ1g3NHdCYjlnMW1wX3M4VTZfanYwcFNLaWUzcnBlckxiZzc2MmFYQVMzb1V5MkRieDVO?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gJBVV95cUxQelBnWW5WSTRCRElaaVplcXVobDRVZWctMUtzMWk5aWtTLXA5U3B2cENlQjBFdkdWRjFhLXRHbkJZZUhCeXBzODFhb2txR0hWc1M0Z2Z5SDhLNTcwNFYxTHlXMDU2VENsRWlmZE9faXpZaldTcG5QVExGWURaY05EX2lOM3dZZzAzTVFTdmI3TW5wMDF4enVnWktGYXZYaGkxbkxoa1I5NmNhdXFRZ1o0M3NXcElBZHE3ZDJkaXZ2VGRidzZTeXAtMXFscDg5R0lSbnVWUFpyQ2dZOUZHOEh2UXdkaHlYTGZUY0dmTTRreDRuUmhMdV9jM0VIM1h4b2h3Y2JnaGFwZC0zX3hFTF80UWtxWE1yVnFCN3N2R2I5LXZucDg1RjlOdm5NMTRDUWlWU2VfTjJSb1hOd0p3Skh3MTU2a0JpaGFMZ0ZmaGwtdjlmQk1LTk5jTkpzNl82cDc5S1I4eW5tSnZqYjRjdlFycWR3?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46078.40277777778</v>
+        <v>46078.03240740741</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Staatssecretaris Erkens snel naar Brussel voor beschikbaarheid CO2 in de kas - Nieuwe Oogst</t>
+          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - 一财全球Yicai Global</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>State Secretary Erkens quickly goes to Brussels for the availability of CO2 in the greenhouse - Nieuwe Oogst</t>
+          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - 一财全球Yicai Global</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:00:00 GMT</t>
+          <t>Wed, 25 Feb 2026 08:52:27 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQWZDWTliTDZRMU1Ub3BtNHhTSDFXTWRmUzBZNlpVZV9LRDhZeU9DOWY4b0Q5STc0U1ZNb2NON2tDY1NoR29GdXdxRTNIUGZXcUI1NEJJUzlIV2dubl9kUGdvYjNiN1NYZDRpY05PUmZVWTFpR2d6Yk5kZXZHejZVVXN5a1U0Zkxpa3lwZU5SbGN4eUZ1OS1MRm1fbjlzMENkc2NyNHVGT3FxdkQ4bDMweV9ITVpBeWluSXFpenln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQQVhnQ0Y1UWRwRmdlb3JBNlR3NG9RYzhSZ0thTkhtWHRKWW1rbjdRYmJKeXJzeE8wMUpiVTZ5aV8tWTVZQnA1LU5NejhlREM2SmluVjI4T0dKMk5kdjBtQkQ1WXhmWkJHVFV6YlgzcXBfaTdKME45SVFZV1Aya3pfRTZPVFBBSTFrd0JBZHNlbmd3R0lNa1VTZ2NFcS1QTmhvVy00S2p4Mmt6SkVwTXU2QQ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46078.41666666666</v>
+        <v>46078.36975694444</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>PETA Broad Search</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"PETA" AND ("Italy" OR "UK" OR "Germany" OR "Belgium" OR "Spain" OR "France") AND ("fashion" OR "designer" OR "outlet" OR "luxury retail" OR "shopping village") AND (protest OR rally OR demonstration OR campaign OR action)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bom barst in dancewereld: top-dj’s beschuldigd van seksueel wangedrag, optredens in sneltempo geschrapt - HLN</t>
+          <t>Italy Fashion Protest - the-messenger.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bombshell explodes in the dance world: top DJs accused of sexual misconduct, performances quickly canceled - HLN</t>
+          <t>Italy Fashion Protest - the-messenger.com</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 07:57:50 GMT</t>
+          <t>Wed, 25 Feb 2026 04:06:54 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQaTJaVF9JOXJmVjVHcndLMzM4TThwWjBSV3hkbG10VTlUTFBJU1NfdGVvZC1XdHVxOWZJOW9jU0FLRTJ0a0RIbnVueFBoNEZtQlgwdlo4b0ZJdEk1NkcyNS1jbU1QQjNHMHlSaE94azd6QTgzc2xkMzlSSjIyN09CeXZDel9xNmRWVTJfQm5FQV9zb3JrUzdwNkZjNTVCdjZrRmxKZTlKdkFmQzVkWVdSOFFQQkJHMjBUaTdydUpUbF9MLW1GcjNxRV9zMWlxdEtNeFZn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPQkxKREQ3LWFXRTV0dlpHTWJsVHJwZnBuMmdNUTFTbFctbzhjRE12cUNzUUlUQlVJTzdVSjhZZDZKNkR3MEJWczBUUUR6VFNlalJKRWwyUERadTE4Vm84Z2g3bkYzRTEwVmtwUHRCNWJHa3N4TWRjWFp0N2s5T01LMkVmNmNlaVprR3d6RzBLV1NCdw?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46078.3318287037</v>
+        <v>46078.17145833333</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>France’s ailing winemakers to get $60m in aid: EU farming chief - The Straits Times</t>
+          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>France’s ailing winemakers to get $60m in aid: EU farming chief - The Straits Times</t>
+          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 04:49:00 GMT</t>
+          <t>Wed, 25 Feb 2026 08:32:50 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPYXV2clhjQ0RuS2RqY1B6clVlMEd3akNmekRNMWN3NUdUb2NGM1ZRWmk3Z0xGa3h0dS1UZTgyT0dwVVdCSXU1TTZPZWFHRVVEZThHRUJrdnF1dmw3UHNzRDh3ZkFhU0RvQ21MR3JfRUkzYzBnTDV5UjQ3ckl6MWQwZVNTbHJFZEF5QlIySEFiUlpDbWdXbWNBOUZ6SWllVW1sWkVLR2dtaVlrQXhLSUE3LXNkSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOY1NoSnNJUHdDZVlIYkRJazd4c01fay1YMjNDQU83U0pPczJYdmRwbUFKQzV3S21sTFBnQXNoWmhhNjVoWG03N1ZZUnJRSnpzdC0wamFZY3lRWWpBMmFzTmh1LVlzT3RlYlZabDYzWG81emRxRnFxUWVZVGNuU0xDSTJn?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -905,47 +905,47 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46078.20069444444</v>
+        <v>46078.35613425926</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>"Un scooter faisait des roues arrière" : un couple s'est fait passer à tabac devant le centre commercial Basilix à Berchem-Sainte-Agathe - BruxellesToday</t>
+          <t>UK Retail Crime: Is the Surge Finally Easing? - International Business Times UK</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>“A scooter was spinning backwards”: a couple was beaten up in front of the Basilix shopping center in Berchem-Sainte-Agathe - BrusselsToday</t>
+          <t>UK Retail Crime: Is the Surge Finally Easing? - International Business Times UK</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:06:02 GMT</t>
+          <t>Tue, 24 Feb 2026 16:29:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbUtkQ2xUMFo0NUdZR1NDNGdBU2V3bzhURWt4Q2tBSXZib1AzX01ZQmI0V21CbExjZ3M3bTdoekQ4eTJicmpLVVFaanUtN3lDTDRicFpqQ3pPTG1wWi00S1dud09hM3RDSGg4QnJmc1cwTkJIRDVtc3dUbjJZZmFMN1g3Umk0YWt0UnJ3am5RcllkdWJJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE9CanphNm90dWFQeXVqS081SVZWZG5zSF9XNWR3NEFCVmZRU2J1MWM4Nkw5dUU2bkZXZVcwekcycTBlQmVsQ3NpU1VDQUd5Z0FvU1M5NVFmSWd1SFdMV3Y1UXBqWWNEbjl3alpGeVYtOA?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,52 +955,52 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46078.33752314815</v>
+        <v>46077.68680555555</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Le CPAS de Bruxelles victime de 26 incidents violents en 2025 - 7sur7.be</t>
+          <t>Michelin-starred Lita names Kostas Papathanasiou culinary director - The Drinks Business</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>The Brussels CPAS victim of 26 violent incidents in 2025 - 7sur7.be</t>
+          <t>Michelin-starred Lita names Kostas Papathanasiou culinary director - The Drinks Business</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:04:00 GMT</t>
+          <t>Tue, 24 Feb 2026 17:42:57 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQMXhzcDN3dmtBX25uRkppaVJkQ09CZnVZem42ZUd4WUhmUDRSTUpmTVRiM1E5VUdoVl96U2FlczJYSU42TEVkaXpCTmdGVVVVQXFGMXE5ZEdjZGc3NWpncjFmX29ZckV0aTJOS3pwX2NHSmk3b3dFQnZWdjQ4N3hsWklTOFlxWl91cFNraVVFRGJFeldWNHFjc3Vqbnk4WGFNWE9r?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNeTM0UkM5dW1EMUZyYVp2Vk01WEdNWHRXU005by1wNTZaZ0h0VjRHeDVYaXU3ZXdHRW5YMWNsQnRxS2MxbGJNMG96TWRCX0RKcEtkN1lkR01odzBSY1hKYy1XdlhaZzJKdm95Tm5pYy1CVktuclpZZXJHSy0wQUd5MlhBMDAwejBRZy15U1o5LWNodFpaSjJIdllOaGRhdjJWYmpFaGJhWW0tZzBvcGc?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,52 +1010,52 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46078.37777777778</v>
+        <v>46077.73815972222</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dour déprogramme plusieurs artistes suite à de "graves accusations" - BruxellesToday</t>
+          <t>Brussels Airport opgeschrikt door valse bommelding - VRT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Dour deprograms several artists following “serious accusations” - BruxellesToday</t>
+          <t>Brussels Airport shocked by false bomb threat - VRT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 07:28:05 GMT</t>
+          <t>Tue, 24 Feb 2026 19:33:53 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPRXo1VnI3UDJVTzVudTNJU1A2LUNySGxjY0VTMFpsT21PVG9ubjJCVEhhQzNDVUxvQTBTWVlYZ0wyYTktY3UtSVZNc1dxVExCWWZDWFhvZkljS1Y1MzFINzYwNGtkdHItR1BzWkV2Ny1Ib1dCS1JxZDd2N1FoRVFYUmZIOG1udGxFUGZ2OGMzSTFVX1k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNVU9yZ2VyOGoyU2FaVk9XbnZVenpiTko2NE43bVBlLW15WEpKUG1DLU56VXRoNHFwZ2ZnZVAzWHdCNlhtUGowUkhrVjUyajZPUEJHT3pOOVFGUnZxY012bFNTVG1wYkNuMkIwcVVrTnZWQU11SUg3QllGdmt1Y29ycURHdE9PZlN6SnRybWtJRE5DbDNqUWc?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46078.31116898148</v>
+        <v>46077.81519675926</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Lait infantile contaminé: désormais huit cas confirmés en Flandre - 7sur7.be</t>
+          <t>Voortvluchtige drugsbaas bestelt vanuit Turkije poging tot gijzeling in Berchem en moet 7 jaar naar cel - GVA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Contaminated infant milk: now eight confirmed cases in Flanders - 7sur7.be</t>
+          <t>Fugitive drug boss orders attempted hostage-taking in Berchem from Turkey and has to go to prison for 7 years - GVA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:53:00 GMT</t>
+          <t>Tue, 24 Feb 2026 19:28:25 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNUWF2Tl85Z0lyTVhDY29SOW9IaThCMUJseXUzVzhOQXpsX1JZalVhZVkyRnlXUzBmRExpUUFreDAtV0QtQU1xSFNZZ204S0Jsenhucl90X0FaTk12MDNtQW1kY3dCdWNsVWFORmFJODJ1bHpOcV8wOHpka1J4NnBwZXVPSktiN0RXV29ZQnUtZm1qRVRDRVJZSF9uY2lyNjMxYU4yaU9LNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxQVTdOS2hnamVfSDF5SURJd1pCM3h2UGYzb2ZYRGlVdlB3d3dRaUU3ekJKak93ZE9xa0laRERmMms0QU5WbmV1NTdpdXFWbGM0eXJzODFBVHZ1ZG5HNFlYc2V4YnRqS2FZaEFHQXItcENKYVZFNDUtM3NBRXFNb21nMnRURVA3TTJ1T2MwSzVkMm1oZlhtRHFPRzZ0UU5xWEEycFI3YzBmMXlBa08xWGdsai1OOWc3R0FUdW85b0ctUDV3cnJvOW00dTU2SkFxX3k3Zl9hSTNqeTN5eWk5QVZDQ3lZWkdWZ1kyVFQtNzVjWmo4a05rOTBNUTJLZWluVzA5SlBoNWNnU3dPNFU?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46078.41180555556</v>
+        <v>46077.81140046296</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Twee auto's branden uit op privéterrein achter huis in Stevoort, oorzaak nog onduidelijk - VRT</t>
+          <t>Trio krijgt drie jaar cel voor schietpartij achter winkelcentrum, maar schutter gaat vrijuit - GVA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Two cars burn out on private property behind a house in Stevoort, cause still unclear - VRT</t>
+          <t>Trio gets three years in prison for shooting behind shopping center, but shooter goes free - GVA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:01:15 GMT</t>
+          <t>Tue, 24 Feb 2026 18:48:37 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPS1ZUaU5WUzRCU0tiM3BRRTYtNXpFSlFSeUs3UjYzMHg1TDhheGJwQk1HMDNBSVNhRXh2aEFOaFZqNnpZdTlJSHRfQm1aVzNlamZ2R0tIM0NycGZVOHoyVmF5TUotM0M0RHd1dTRzTkdDNXlVZTN5UERuZHBFdlNhYUVZSnJGN3NtZHp0YkRUc1drVXViSkRKM3ZCOFc5ak4tNmxPZDh3bw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxOUXduU0hBQ2g5c0puak1mdjJQUzBfdEwxNk92RFdaemd6ZzZTTkI2dkdWWmlZV1RTTVV5cC1IdmZubHlNQTVuY0dmdlJDQ1hoRU9GSVBfNTFLQ0o4RmdoZHU0REptS3JBTVU2ek9JMmtTWFItbVpuSS0tM0o1MzVGSW9TNFFiRTFJY2VTalhyQkhsSmR1V0YtNkJCWDN2dFJIYms5cUlKUkZ4Rmh1Tm5zQVdJVVBoNUNpY2ZJOG5zNVI2YnJkRTlGdTAtbVRrekRqeWo3MEFrUkVCX04tZnZzQV80MUJKa2x4V2xxVkVweXN4ZGM?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,38 +1189,38 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46078.33420138889</v>
+        <v>46077.78376157407</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Afin de retrouver la croissance, Seb envisage «jusqu'à 2.100» suppressions de postes dont 500 en France - Europe 1</t>
+          <t>Nog twee minderjarigen aangehouden voor explosie sportschool Fitletic in Roermond - De Limburger</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>In order to regain growth, Seb plans “up to 2,100” job cuts, including 500 in France – Europe 1</t>
+          <t>Two more minors arrested for explosion at Fitletic gym in Roermond - De Limburger</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:58:00 GMT</t>
+          <t>Tue, 24 Feb 2026 16:22:20 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxNX2E4Qlo0dG9hczljSTJaTG80NjBqX2s1WFlKZE9waUFLQllFaHNoamZfSlpaV09vajdta3cyT1BBWi15NklsNlc3R3B1a0pTWmMwdEk5LTc3ZlgzTVd2WFFzNHlWbXZ6Q2x2eW1OV2VZZ0tieGo4aGg5NTY2dEhFZnlVQnY4WGpuNW55ak92WW5zMFF2RzRWdUJlTE9tdHpmWVRCeXFreDhSY29laGo0UTJUQmZSYV80SnFQX04zRlhiX0ZnalZXTVA4YzlDaG1IcDlr0gHYAUFVX3lxTE82VU4tNjdDdXpyQy1NMmVZZTZOS0xIczFSTW41MHptWHUybktTaXBfcHFuX3hHX0YxY3Y4UW1QYXB0NzBsWXE1NFZVcEduVHhOeEZ3c0hTVWp2VThGYjBPNjR4dzdISXI3MFNMYThfUy0yZUFsOTdScWU0LXFUQ0E1NUxfVE5XcTFoQVN1MTdjdG9iV09nQTU2TmI4NUxvTlBId0tJVW9aNW82TGJ1SzRwOGRSU3NTQ0ctZWtVSFh2eTRkbUlmajdJNG9NVmtiWENqVUlCdU1nQg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxOY1lITEdQUDN5cm9DTzhnVnRIN2l1Q0QtY2ZsaWo2OS10SDlrNkNTMWI1R0xoOHl6V19aNXRsLXNtSnBiX2RIa0J0ekZuWTNGSXR2THV6TXNaMjRtdmg4Tmx1VlhGZm10Sl85bHJzb3RKbmN2ZnVfTWNBS2J2TWIwVEk4X1FjckVLNmpZeHkwVFZDbVQxT3dneFQwRUk3X01Oc2dsSllEdWl3RkJUUXctbVFWNm1IX056dW9zSWJOdjU1YUkzdHVYTnk0OVZBS3JDRlpzWEk3aU5zZjEwQUE?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46078.45694444444</v>
+        <v>46077.68217592593</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>38-Jähriger nach Öl-Diebstahl auf A3 bei Bessenbach festgenommen - Fränkische Nachrichten</t>
+          <t>Staatssecretaris Erkens snel naar Brussel voor beschikbaarheid CO2 in de kas - Nieuwe Oogst</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>38-year-old arrested after oil theft on A3 near Bessenbach - Fränkische Nachrichten</t>
+          <t>State Secretary Erkens quickly goes to Brussels for the availability of CO2 in the greenhouse - New Harvest</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:06:00 GMT</t>
+          <t>Wed, 25 Feb 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxPQXdHZDdJdGhkcGZOeFQyZVBhbUY2eTk0YnNvZnlFWkdKZHdYNXR6dW10U0FkZkRpWTViQnVrNFNvVnpoMk9HbkkwbE5uNDZiR3ZEYzVhQkpPODA1Z0N6OHRrRjE4LXY1VlR4WHRlNXJfWmxzWDNQcmxDQXpLWVpTSGU2U05ab2RSTDhJRVpPQ1Y3THA2cm1veVE1Yk05NnhlckdGY1JxZmx5NUpNN3V3Q0I4MHIxZXJaeHVnVmUybXo3OGpvd1pPdWV6QUI3c00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQWZDWTliTDZRMU1Ub3BtNHhTSDFXTWRmUzBZNlpVZV9LRDhZeU9DOWY4b0Q5STc0U1ZNb2NON2tDY1NoR29GdXdxRTNIUGZXcUI1NEJJUzlIV2dubl9kUGdvYjNiN1NYZDRpY05PUmZVWTFpR2d6Yk5kZXZHejZVVXN5a1U0Zkxpa3lwZU5SbGN4eUZ1OS1MRm1fbjlzMENkc2NyNHVGT3FxdkQ4bDMweV9ITVpBeWluSXFpenln?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,52 +1285,52 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46078.37916666667</v>
+        <v>46078.41666666666</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Autobahn 3 in Unterfranken: Überladener Transporter gestoppt - Ladung war gestohlen - Neue Presse Coburg</t>
+          <t>Verdachte van taximoord in Geel probeert tevergeefs vrij te komen: ook in beroep blijft A.B. (20) aangehouden - HLN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Autobahn 3 in Lower Franconia: Overloaded van stopped - load was stolen - Neue Presse Coburg</t>
+          <t>Suspect of taxi murder in Geel tries in vain to be released: A.B. also remains on appeal. (20) arrested - HLN</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:15:49 GMT</t>
+          <t>Wed, 25 Feb 2026 09:43:43 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxQc3ZDRmViNExNZE9zRTAzU09PN3hNYzZBZnlvbTVheG84T05KWFduM2plUHJiVXlzX0h4d0VtS1BQWElnRUlrZ25mOXlia0ZZM3dOYy1ha3NpaDF0UmNXZkpKbHBWRGw3V3V0aXgwNWhWTV9sRVh2MGdHemVPYWVnX3R5YV9zMzNXb1lsc1VXWnpzMlJlb3VCQ1pZODI4SEFSMV85Vy1uRVVWQmRkdzBpb3lxdURnWFFfSzBxVmFLOTQwSThQdTJjZ2JWOXR2SU51YUxlMHRSNTdndXYwSXNLeDR0SnRhZmJhelVj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNS2pxcUxaMEF6Nm96R3p0Z2VzSVhGblZfTktvV0VGVlJXb0tMU2FVLVJ4YU5kYTFEakdZRVJ4aU1ZcmdWMkYwd1FNVThPUDQ1SG1tXzd2YndKRTVxSnZ0aEN6ajlXSHdqdUI3RWV1aHVMcTJoZlBpVmhLaUsxUWpYXzR1aVNWNGpVbWZNNmhaZEFZYWRUdF9Eay1FWXdHWmozYzVhRVBSV09zdmtJU25fUmN1bTFEMzBoUmZKVHNfWURnWTc0YXd0M2FfM1JYZ0ZLNXNZeU5R?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46078.42765046296</v>
+        <v>46078.4053587963</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Demo-Termine heute, 25.02.2026: Hier gibt's am Mittwoch Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+          <t>Bom barst in dancewereld: top-dj’s beschuldigd van seksueel wangedrag, optredens in sneltempo geschrapt - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Demo dates today, February 25th, 2026: Here on Wednesday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+          <t>Bombshell explodes in the dance world: top DJs accused of sexual misconduct, performances quickly canceled - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 05:55:29 GMT</t>
+          <t>Wed, 25 Feb 2026 07:57:50 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxQNFdodW8waDJhejU0ZGtoemRUWV9YRlZ1TEtMeVk4WU1RT2doLTBsOEZ1Z29mZS12dFJoYXF3dDVBSHM2eFg5NzloLUVsYjdycDRsc0FnZmtxeExBb0ctcmxyR3FwRXYxbmhDSmRQYXRJUGNPRnQ2cmRzMDJQazZTMUd4RWNlV0NSbU5NUWlYNTROMnZqbllmUnpicHU5RFZscHVjR09rV2pYLWVxck5UTzY2d29aeXd5WUhjQTRfZ1dERXZGNHpxNHlIWXh1SHFBOVcxTDRzS0Q0bmtDdHZuS3FSQlpydDg4WDdVU0pGTFRXUTdvalJkS3N6VVVPVWvSAYQCQVVfeXFMTWNydll2dWxMbEUwa2RNY1V3RVVER2ZjTmZFbGUzdk42M25oYUtONnhPWGV1SXVtcDNUYVlZVVUwVkk1ak1FME9RTWI4aFZtYU9uMHZqRHZkZGtfRFRwTzhnU3NKMEJISHNNaG5XXzdBOXZVQnhZMjY2RnRNZTZWRlpXenRWVWVaVGxYTTBxbmtqRlBPMjktSlBlLXQxOTgwRGZacW9IZTRScFduX0hCaWc5ZGJWc193RWxmd2NkZjFRYVJ6MF96RkhNRGpVRnVsQ3RBUzlLM1VaalRpREdjaFZEY3BrdXZwc25sUXRTNWJ3R3ZsUHhmNUJNSkNpeVRWZmdoaVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQaTJaVF9JOXJmVjVHcndLMzM4TThwWjBSV3hkbG10VTlUTFBJU1NfdGVvZC1XdHVxOWZJOW9jU0FLRTJ0a0RIbnVueFBoNEZtQlgwdlo4b0ZJdEk1NkcyNS1jbU1QQjNHMHlSaE94azd6QTgzc2xkMzlSSjIyN09CeXZDel9xNmRWVTJfQm5FQV9zb3JrUzdwNkZjNTVCdjZrRmxKZTlKdkFmQzVkWVdSOFFQQkJHMjBUaTdydUpUbF9MLW1GcjNxRV9zMWlxdEtNeFZn?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46078.24686342593</v>
+        <v>46078.3318287037</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Blitzer in Estenfeld aktuell am Mittwoch: Hier nimmt die Polizei am 25.02.2026 Raser ins Visier - News.de</t>
+          <t>Sociaal assistent die mesaanval overleefde, loopt van Luik naar Brussel voor goed doel: “Belangrijk om op te komen voor minderheden” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Speed ​​cameras in Estenfeld currently on Wednesday: Here the police are targeting speeders on February 25th, 2026 - News.de</t>
+          <t>Social worker who survived knife attack walks from Liège to Brussels for charity: “Important to stand up for minorities” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 05:15:05 GMT</t>
+          <t>Wed, 25 Feb 2026 00:46:57 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxOQnU4UnRoVkVsSm1rdndna2ljQVFld3VyakZxSTRXY2dJcHBXQkhfZE02bF90UFA1RllzYXVJamlKbklDOGRkb0NaWVhPR3p2ZXJMUWxfQTlhZHhSVXNST0t6YWExSzdsNVFZQXdELXhXWElFOHBSNC02N2tDRENsdk9iZlZ2SEJ4X056dENxaFFrd0JJVzVTODlrZzBENmFEZ3p4S0I1OFdIcTg1QklqQ3hMWnpTdk5JLUhIX1lZVVhZcmtCZGd6YlFzQ2k5WW43dUZ4dXpqZmRsbGJwZ2RmR0N0VWl0UnplRXBIVGR0TFRzX3ZfWFhjStIB_gFBVV95cUxNS3paT3VfNkhyeWdjSEo1TXB0VlVnZmVZX0JpeTB3SVJRbHNoaEs1ZVRmZ3NGbFctTk16SGNkem8tVmg0d3hXM0lmLUhSa05ic2M5UGUyZkZsMXplWG5TUk54alp5TUd6RDVCUDgzVmlVWTYya0hRZXBwemYwUXdMakNDczRhRFc3UVVSLUUwdnI3X0RGVHFsOU8tVnhfZkxsTmM1dGJOY2EwT0JxaGdINTRkLUFLa2hkRUUwcjJRd1lycVEtNHZqZlZPd3JmVEZteTdISE5Gc0tENU14VjNMU1gyUnlOSjg3dDl6TWxBNDA2dlJTcjJHOTBnbERJdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxOV002bEs5aGRYNWtZNmRSMFo1RTV6NExtUEhzX3ZpREJxWkE3c1I3U2JJMEtHbnEtdjVEeGVCenROX0VFdC1TYklmV0JfcXZPNzlZb2hKcFpDaThOQnI0X2N0WnoyRy1wRUhiVHVnUWNDOEZaZE5CWmhJampsbHRMcXFJaEhKdmhBWG5qbU1PVDBjOHZGT0NGLWhtV3JvT0dCWTIwdGNaaTV4LW1LWGotWlRoRUdWc3NJT3VFZU1YeUpLWG9TalF2M1JtalBDMG1RTTZQWmJhS2RneE5PVE5ITFJ3VUJ4WkpOeVI0SGREWHVjQThiYUFJcTduUEx0cEh6NExvcWg5OE9QY3hMdlprdXpkSnMwQW1QZ0ln?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46078.21880787037</v>
+        <v>46078.03260416666</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mit 2,4 Promille durch Lindach: 33-Jähriger verursacht Unfall und fährt davon - Augsburger Allgemeine</t>
+          <t>Radio Minerva eert Frank Boekhoff op dinsdag 24 februari tijdens een twaalf uur durend radioprogramma: “We zullen hem nooit vergeten!” - HLN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>With 2.4 per mille through Lindach: 33-year-old causes accident and drives away - Augsburger Allgemeine</t>
+          <t>Radio Minerva honors Frank Boekhoff on Tuesday, February 24 during a twelve-hour radio program: “We will never forget him!” - HLN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:56:42 GMT</t>
+          <t>Tue, 24 Feb 2026 23:46:26 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPWVFzbGJzMDlkWXkzaFVmZzMwbzB2aVFpcFd4WFdMdFpfLUJ6OF9wWlg0NmJzOXdQVnd3RmQ4QXFrQ3hpUHl4QlExaWJyQWxkQ3JEZHlRQ0tQUW9vZ2R3ZVJadzJvUjdJZEk1X2ZNLU5DSmViTnd5aGhKbXVWaWRKcm5xQzJuOE1BVFFCUnFvZ1AzeGozWEtZczEyQmtDWUJNbjAyM21Vb2hWNUhMMjB0UFZkek5aWWFwT0VoVHJDTXNZUi12VW1DSFVsYmNMZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNQWozbzdiclNmZmRDU3VJLVZtTXBzSS1ZWHR1YTR4WU55aHhLdHdVcXRUeFIwbTI0NXZIdjlYejV3UlJhejUyOHVxMnV5djJhNHg5NHlUN241TjRLeDI1LUwxMVhsT0dZa2Vxdzd3NWxPbjFGZXBYbG50SmNrSVFRUmZpSGxJQVpzeW5iOWpSQUtXcXB4TUJKdmdEOXZzanhWMFhrVWNPbTUzbnc5R1VWNG0xTnVtRC1yQTBoR2tuQWZrSmNtOGx4UGt6VmkzeHkyRGU2SFZ3MA?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46078.37270833334</v>
+        <v>46077.99057870371</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Nächtlicher Feuerwehreinsatz im Hotel - RegionalReporter</t>
+          <t>False bomb threat at Brussels Airport prompts security response, no evacuation required - Aviation24.be</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Nighttime fire brigade operation in the hotel - RegionalReporter</t>
+          <t>False bomb threat at Brussels Airport prompts security response, no evacuation required - Aviation24.be</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:53:21 GMT</t>
+          <t>Wed, 25 Feb 2026 10:40:50 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNOWpPNjE5YUFuc0F6TnJYR1RwMi03Vlk1TTYyM19zTTkzSkF6R2JxcGtNeWpOc0YtM1hwa3JmR1RlQV9Ub0RXMXYwRFBiZS11MDhtalVKNENaQlItQ3RSN05zZklUcDJzLWxsQWVveTd3Q3ZRRTZpaWlsaTFwbm4weGxJLXFjaW5WbEtVOVd2c3dTZjVtSGo2al85c1U4WTNs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxNSFFvV1Itc3d0a2YtTS1zQzBpLTRta2RQWnBZU2c4akI4Um1tSXNabVhWb2doeWI5T1BCM0taSVdFY3kwUDV2UkZJRFFYejJ1STBtcWRDRjRDUmlvX2kzZWVNN3NyOENzQkdBR0JLUXJpZlc5ckM5Z3Y3T0RSaXhwNjAyTXF1M1ljemVaczdOZHo4SXpaVUlLYnUzN3E2NEh0T05xM0lSSTRJVmJ2cS1vT25SbzI4Mkd5UDZCQ2RtYlZrSTlabFg1TW5MdGtBTHo5ekhfY1JwdF9Sdlk?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46078.41204861111</v>
+        <v>46078.44502314815</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Flucht nach Suff-Crash bei Manching: 33-Jähriger hatte mehr als 2,4 Promille - Pfaffenhofen Today</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Escape after drinking crash near Manching: 33-year-old had more than 2.4 per mille - Pfaffenhofen Today</t>
+          <t>Brussels shines Ukrainian colors on buildings as EU marks four years of Russia's full-scale war - Euromaidan Press</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:06:55 GMT</t>
+          <t>Tue, 24 Feb 2026 17:56:40 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9LSFBSM1d2QkVZeEE5clBhSzMtbmhxTVpVejFlXy1WbTFDa2FkSHgxWl9McjRXMnFJeGdhTEFpcXpjQVpVTkpjN3MxMjRsOW5BRkY2dG1yRUhyNVUtRmVzYzNn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOTVkweWFzUUNLdXBoYTJPUGNWeFI3c01LV1pqRWU2eExiOUFwOUE2MlZGaFBySWVJUmdUWGotM1BDS1lydWgwcEpZR3FlbHpuZmpDVVkyYWhNQnBSTEpMS1VscG9HOE1pREFTUlM0VHF4UV9UUjRybFNmaHpWMDlvdE5kZUt5d2lRYW9ENmFkQVFoMnZyRzY3VllEYVkzWEU?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46078.46313657407</v>
+        <v>46077.74768518518</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Germany's FC Ingolstadt makes special collaboration with Kashmir's design house Pumposh - India TV News</t>
+          <t>Ukraine war latest: UK and Ukraine respond to Moscow's 'absurd' nuclear bomb claim - as Trump sets new peace deal deadline - Sky News</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Germany's FC Ingolstadt makes special collaboration with Kashmir's design house Pumposh - India TV News</t>
+          <t>Ukraine war latest: UK and Ukraine respond to Moscow's 'absurd' nuclear bomb claim - as Trump sets new peace deal deadline - Sky News</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 07:15:30 GMT</t>
+          <t>Wed, 25 Feb 2026 02:53:27 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNUTdkcE9MOUlfSndGTER2U0Z3anVFMWxqM1RDYThNZ1lNQm0tLTc3MHRlNVRRanpyU3pyRGFYUXZQTE4wUEszaDFkVHNJUzRUTlczUGxNSHJQS191ZnRoOUVoVVZGMWZMME1rdGFpaFVOSzZNNEl1cm5aUEFpMkNwWUJDZk9KNGZGSmlaWHZySXd1bE1KNHVJdDNyN0xRYWdYUWExM2ZpZS16M3ZwYUdmTTczeklEQUR1NHhkRVd5ZGFYT0lGcUk4SGtfNml0TjZ2RnZFSGVRLU95dGE2V2JfZjR0RXQ1a05aaFpv0gHrAUFVX3lxTE1RN2RwT0w5SV9Kd0ZMRHZTRndqdUUxbGozVENhOE1nWU1CbS0tNzcwdGU1VFFqenJTenJEYVhRdlBMTjBQSzNoMWRUc0lTNFROVzNQbE1IclBLX3VmdGg5RWhVVkYxZkwwTWt0YWloVU5LNk00SXVyblpQQWkyQ3BZQkNmT0o0ZkZKaVpYdnJJd3VsTUo0dUl0M3I3TFFhZ1hRYTEzZmllLXozdnBhR2ZNNzN6SURBRHU0eGRFV3lkYVhPSUZxSThIa182aXRONnZGdkVIZVEtT3l0YTZXYl9mNHRFdDVrTlpoWm8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwJBVV95cUxQdjRuNUJlWFNXZWx4QWZqT3piekRnSUZWeVg1TEdpX2hPbDNxRGJ5allwV0hBQmNXS1ctV3MtY3pHV29rbXA4ZDBCSjk2bEpfZ0FUUTV4YzMxNXhLalZfb1ZWZ2VUQUFzcVJQejNsZE1qWlpxUWFKd3I5Yjl6WlZaRGpfSk50cGlnT29jdUg5SUozZzRLLXFLWFNPWHREeFk0eUNaUmJudE1hQkZ6MHN1SFVleXNVajR2Q0lWclc0YkhFdXJobFZZdHY5T19FQVdKSGI4anpSeElpYkw2NEdSMXR0bmpDaFVTcTlGLVBBS1RhVGlNR09WMVFvR3IwWXgzRmtyOGhoRnMzVmdpUlVEQzUyRExqc1FMX19vaVlJZVhfX0xfcjZV?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1675,70 +1675,1940 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46078.30243055556</v>
+        <v>46078.12045138889</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>High Level City Belgium English</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>France’s ailing winemakers to get $60m in aid: EU farming chief - The Straits Times</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>France’s ailing winemakers to get $60m in aid: EU farming chief - The Straits Times</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 04:49:00 GMT</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPYXV2clhjQ0RuS2RqY1B6clVlMEd3akNmekRNMWN3NUdUb2NGM1ZRWmk3Z0xGa3h0dS1UZTgyT0dwVVdCSXU1TTZPZWFHRVVEZThHRUJrdnF1dmw3UHNzRDh3ZkFhU0RvQ21MR3JfRUkzYzBnTDV5UjQ3ckl6MWQwZVNTbHJFZEF5QlIySEFiUlpDbWdXbWNBOUZ6SWllVW1sWkVLR2dtaVlrQXhLSUE3LXNkSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>BE:en</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>46078.20069444444</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>High Level City Belgium English</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Rute: Ukraine needs ammunition today and every day until the massacre ends - vijesti.me</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Rute: Ukraine needs ammunition today and every day until the massacre ends - vijesti.me</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 15:51:31 GMT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNNkF0OEpmaXVhOVNvVnJOZVhOMFZCTzBrWTlHdjdOMUlwdVVBMHIxV2lFUkx6MjgxM3VDNlFlcy1uR2lYNzlCRFRlRzk4ajlXOHV4N1dNVC1fWGdlakJHbzZQc1NPSV9KZ2V2UFM3RGNidXEteDA1TGstcDBrUVF6QWVpQ0JFZHIxTU1wZEpqbWJ0Ykgtc1hQVngyWUsyTm1VamRaTDdoQmpUd9IBqgFBVV95cUxNNkF0OEpmaXVhOVNvVnJOZVhOMFZCTzBrWTlHdjdOMUlwdVVBMHIxV2lFUkx6MjgxM3VDNlFlcy1uR2lYNzlCRFRlRzk4ajlXOHV4N1dNVC1fWGdlakJHbzZQc1NPSV9KZ2V2UFM3RGNidXEteDA1TGstcDBrUVF6QWVpQ0JFZHIxTU1wZEpqbWJ0Ykgtc1hQVngyWUsyTm1VamRaTDdoQmpUdw?oc=5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>BE:en</t>
+        </is>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>46077.66077546297</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>High Level City Belgium English</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>West must support Ukraine ‘every day until bloodshed stops’: NATO chief Mark Rutte - The Straits Times</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 17:16:59 GMT</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNM185ekl4N3lkY3FGV2xtcHpCRDZicWFIVWpxeXZuVUVzNGc4SFpCa292cnVnaElFMUtnYlMyeVRXWnpnNWNfQmxFVEdzTk9ZVnFob3RqaDgxMTZmWlNaa3ZPWWtVeVU1YVI4SG1vUGdvdmVNUENkdy1fTUJPZTBkcUZGaW5BblhDSHFfbENWLUtoemlqREJHUjB3ZjBnS3AxNHZfZzdOTGdEYk1KV3ZNcVl4R0prelRHVW82SE1n?oc=5</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>BE:en</t>
+        </is>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>46077.72012731482</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Plus d’une vingtaine d’agressions au CPAS de la Ville de Bruxelles : des sanctions sur le RIS envisagées - BruxellesToday</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>More than twenty attacks at the CPAS of the City of Brussels: sanctions on the RIS envisaged - BruxellesToday</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 11:32:00 GMT</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNblV2Mk45V3MtT0hiU0J4cEVLSkk0QVFOOXFRS05TTUVwZVk2NVFmWG9COV9Od001MDcxdzBnTWpydVlnWVFEOUk4MlNOLUMySGJkZFFpM3hPNVZJMExmSXVkVS1mQW0zQ3E0d1pLTjFwMjZ5a0tqQ1RJLVRjc1NrdE55eGVJMDFSMkYyWQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>46078.48055555556</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>18,9°C à Bruxelles: record de chaleur battu pour un 25 février - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>18.9°C in Brussels: heat record broken for February 25 - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 13:24:03 GMT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVUxQbFR1U2NjQXJ0bWFIbEx6REd1YlhFZFJ2eVpmQkRveFFZNU5jdWVoUFM4U3FhTl95eXVRMTlYb1lKcEhTNDRGYXoybUZOQ0dhNFZkMHdHdGRYTkNJd0UxbjlxN09KSE80a2FmQ095d0pWczY4TzMwZXBZTjVySEQ2cnYzY3pKMnJYWUwtTEhXQ0ZLUlR4VF8wRFh3cFlTOUE?oc=5</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>46078.55836805556</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Le CPAS de la Ville de Bruxelles a recensé 26 incidents violents en 2025 - BX1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>The CPAS of the City of Brussels recorded 26 violent incidents in 2025 - BX1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 08:01:00 GMT</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOanBUYWg1T3JISGlCRU9qdlhJNXJjaXpxeVM0RG95eWNGS1NHUHRITDN1dFQyWVJreG9WdEw2OTBndEJQXy1QWXF4Nm0zS0JZRUFRUWprYy13MFRTdlJDdEF4czJ3Y1BfYnpBME14UGU0Rmpyc3I3VER2eU40aDJweDBXODB6VE5wc2JNUFNsekNNNDUzZXl1Q05QWG9HNXpPc24tUnhXUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>46078.33402777778</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>"Un scooter faisait des roues arrière" : un couple s'est fait passer à tabac devant le centre commercial Basilix à Berchem-Sainte-Agathe - BruxellesToday</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>“A scooter was spinning backwards”: a couple was beaten up in front of the Basilix shopping center in Berchem-Sainte-Agathe - BrusselsToday</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 08:06:02 GMT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbUtkQ2xUMFo0NUdZR1NDNGdBU2V3bzhURWt4Q2tBSXZib1AzX01ZQmI0V21CbExjZ3M3bTdoekQ4eTJicmpLVVFaanUtN3lDTDRicFpqQ3pPTG1wWi00S1dud09hM3RDSGg4QnJmc1cwTkJIRDVtc3dUbjJZZmFMN1g3Umk0YWt0UnJ3am5RcllkdWJJ?oc=5</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>46078.33752314815</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>La CGSP Cheminots dépose un préavis de grève de trois jours sur le rail en mars - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>The CGSP Cheminots files a three-day strike notice on the rail in March - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 14:29:00 GMT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQeUhLZk83MmROZnNOYmVrMVhkRWdUWWtQTExucWItbEVHUm4wMFp3bzJ4U3dWN09XSUt5bDNEanQ4YTZFVHhDdFZsR3gzc1oxYzVyX3ltU0RCVVI2b00wSTc1S1BfX09rZGVDR0ZrUjhvV0o5dEFTU0lYUDNzbDFmVFJ0eXV1cU8tMlRGOWVZX0VZMHBNaUpSVnpRaDZRbnJrQkk2WXNmY2ZXTmVTUUlCOGo0WGhsTE1WMUl3?oc=5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>46078.60347222222</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Dour déprogramme plusieurs artistes suite à de "graves accusations" - BruxellesToday</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Dour deprograms several artists following “serious accusations” - BruxellesToday</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 07:28:05 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPRXo1VnI3UDJVTzVudTNJU1A2LUNySGxjY0VTMFpsT21PVG9ubjJCVEhhQzNDVUxvQTBTWVlYZ0wyYTktY3UtSVZNc1dxVExCWWZDWFhvZkljS1Y1MzFINzYwNGtkdHItR1BzWkV2Ny1Ib1dCS1JxZDd2N1FoRVFYUmZIOG1udGxFUGZ2OGMzSTFVX1k?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46078.31116898148</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Les syndicats de police claquent la porte des négociations avec le ministre Quintin: “On ne peut que se cogner à un mur” - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Police unions slam the door on negotiations with Minister Quintin: “We can only hit a wall” - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 12:24:00 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxPU1VJWjRjUXIzdWxuLWh5VWgyMVJuOXJMSEFvX3YzSzB4YUhSYm5iczBKb3JBWHhKSml3cC1iVEpiVVdOX0piX2lKWlhWNUZ5cUFvOEd0Y3I3US1xdVRlRW13MkVva1VMQnJHOG1GVHl0REduVThUSmdyR04zdGtnU1RManVVZFpaUl9hckxFc1JKS1FJcld0b0VxYTlxZXJWamxPWGVHVHlaakxJbUpiY21uRDJDZDRhcDFVd25lSVAzY192cWgtcmJwRlZ3VW5yUUdfMnQzRHF5ZXI0eVJpZ0VTUFp2MmVoLXRLT09B?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46078.51666666667</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Lait infantile contaminé: désormais huit cas confirmés en Flandre - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Contaminated infant milk: now eight confirmed cases in Flanders - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 09:53:00 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNUWF2Tl85Z0lyTVhDY29SOW9IaThCMUJseXUzVzhOQXpsX1JZalVhZVkyRnlXUzBmRExpUUFreDAtV0QtQU1xSFNZZ204S0Jsenhucl90X0FaTk12MDNtQW1kY3dCdWNsVWFORmFJODJ1bHpOcV8wOHpka1J4NnBwZXVPSktiN0RXV29ZQnUtZm1qRVRDRVJZSF9uY2lyNjMxYU4yaU9LNA?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46078.41180555556</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Le DJ set bruxellois d’Odymel annulé après des accusations d’agression sexuelle - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Odymel's Brussels DJ set canceled after sexual assault accusations - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 19:06:00 GMT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQTzBLc1Etdk9JRF9KVFBnV1hkd1dKVlFkekg0WlJaSzhGSkNsdTZ0bjBoZ3NVWnA3c1BxM0pnZ3JfQ1B0NFE1RjRXN2hsY0xEdlVZLUxmdDVnbjh5YTRHeUJnUkFUNVpzRl8zZFdXS2wtejliVW9tMkw0bzR4OXB6ZUxRQlBvdVBCamlBc2pSZVVXS1FZbWNzRFg4NV9MTHl4ejEwSnhFbFNsY3lZR3d5UGFSRHNhWk0?oc=5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>46077.79583333333</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Twee auto's branden uit op privéterrein achter huis in Stevoort, oorzaak nog onduidelijk - VRT</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Two cars burn out on private property behind a house in Stevoort, cause still unclear - VRT</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 08:01:15 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPS1ZUaU5WUzRCU0tiM3BRRTYtNXpFSlFSeUs3UjYzMHg1TDhheGJwQk1HMDNBSVNhRXh2aEFOaFZqNnpZdTlJSHRfQm1aVzNlamZ2R0tIM0NycGZVOHoyVmF5TUotM0M0RHd1dTRzTkdDNXlVZTN5UERuZHBFdlNhYUVZSnJGN3NtZHp0YkRUc1drVXViSkRKM3ZCOFc5ak4tNmxPZDh3bw?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46078.33420138889</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Vrai ou faux. Le député LFI Raphaël Arnault a-t-il été condamné pour avoir protégé une manifestation LGBT ciblée par l'ultradroite ? - Radio France</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>True or false. Was LFI MP Raphaël Arnault convicted for protecting an LGBT demonstration targeted by the ultra-right? - Radio France</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 11:23:03 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPd0hMVEw5NlBKdXdBMlVrWk4xREZZZnU5RmxDUVpwUHJqTndLeWZ5ODV3dUozZndOTDFpLUpBWHJkMjA3Z1p5TVM0TVNzOHBYbURfSnl6NzJSeWdJazJKYko0NW1MVXdKTmo3cVNjYWxYaGZLX2RNZXctVVlGaDhlYWNNc25VQUJWZ2pXZVA3NjdnSkRqMGtLczZOdjRKNzM0aThJeUVzai1fX2E2d1BpdVY4ZHQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46078.47434027777</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bomb OR explosion OR shooting OR stabbing OR evacuation OR police OR arrest OR threat) AND -sport AND -football</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Louvre president hands in resignation to Macron: Elysee - foxbangor.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Louvre president hands in resignation to Macron: Elysee - foxbangor.com</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 19:31:08 GMT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxOU1hWMW5PLUJZZU4xTWIxSGxzUkZfVVZLcHJ5OE1UQnd2UGtiY2tia0VzLUpybmk2WU5hTXowTVVSbzVXX1hEQlJrLVdwTU9fRFNWSVN2MXlMZnNIcEtncGo3LXVfOTJDTmJyMmpkeFpDUU9rX0hUanVDcTdFQXdaYlR0Y0FHQ19sMW53V0dtZGZnLWZNc0taSEF2am56UUhaYThURWIzdmhJSThmNkJ2WnR2NXJQS09TbjB6eTlheHhjbWViWlplZHVTLWVJNnE0WVhWZEx1UVZCZGpF?oc=5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>46077.81328703704</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Mellrichstadt: Polizei ermittelt wegen Jagdwilderei - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Mellrichstadt: Police are investigating hunting poaching - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 12:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQRS1wU0U3U3dQSTlMOWFiOU9vRHI3NEhFZUxGOGUtTzhKUi1DV3h1SEZNV1VnMDNEVVBVUHFzbUlFdkRMR3BQWmlHTEVjRlU5ZXgtWkF1Q3NKekI3TGp6UW41Y1BqMlR0aUxWbjNaRTVQQmkxaWtua1BiT3NWdXFfWnd3QjFXX3hSR0dfUw?oc=5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>46078.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Frontalzusammenstoß auf B19 – Zwei Personen schwer verletzt - TV Mainfranken</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Head-on collision on B19 – two people seriously injured - TV Mainfranken</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 16:05:00 GMT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPdVBZMUhFUmM0ZXl1U09WQXI0eHVKR1FvMlkxSU5PVzI4YWJLdlJSYWZVa2doRXpOV3B6aVRKLUZNWEUzVmVBa1h3QV9IY1BvSGtDYUp4MkVnT3JBTzVTTkFFTG81cDVmeERscVhUMmVtVm9PUHd5MVB2bDdzZk1vWC1QUm81ekhPeWVyczhWbm1aT01OelRRUEVnSGl2VGdxMmxGZkh2Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>46077.67013888889</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Mainfranken: Trotz Warnung – Callcenterbetrüger wieder erfolgreich - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Mainfranken: Despite warnings – call center fraudsters successful again - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 14:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNZllFZWRoOW5GS1hkdmxITUFlenF6Nm1mYlVob01rN2Q3TEx3emlzRU1GaE0xVWE1UWJ2ZUVzLUlJS21pa3NyMkhVdmhXWWVJUzVLTUlMWEhlaFJjWEthZUJaYy1tYVVsRGhWOEZiWTJodGx3QWVwTGR1WlNkVEZKdkFQYkpOMVdUYTg2bHhCS0tGNmRKX1lKT1RvM1U2QkZfQXMw?oc=5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>46078.58333333334</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>A7 nach Lkw-Unfall stundenlang gesperrt - Zeitungsverlag Waiblingen</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>A7 closed for hours after truck accident - Waiblingen newspaper publisher</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 02:45:00 GMT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOZHU4RjZSa2l1Sy1IT3RUSzJxWFVYWUtzVEQ4NHdkb2lKR0Z5aWhZUG9LSGFSSkhyVkd2R3dfNlhvVzJ4Z3dTWWVLaE9jeDRHMXFEenQ1UHNnR28zTDZqazhPLTB2SG5iMlhGLVRHNTNqY1BDbVpUanNVbVBHSUp6cXhhWkZxTG9sb0NiQ2NBa3oyTnVucHI0QzJB?oc=5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>46078.11458333334</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Herrmann: Wechsel an der Spitze des Polizeipräsidiums Unterfranken - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Herrmann: Change at the top of the Lower Franconia police headquarters - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 12:29:43 GMT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPblZ5bjRhZmwxUjdVbElESmtfSkxtSmZyZmpKWDc3ekVUTXYwWmRjMVk2aDVGc0FRa0YtcmNudzJVdUNSc3EzSk8zeWhvSGdJTkRTQzA1SDdCbDBGRUZ4RjU5WkpGYXhHb3ZpUUFrVEtrZWJLNkpfM1g5QzhSQTZaeWE2Tmk4cmJNTWxscS1KYkFXMTRrR0hFa3YwcDB1RmtSTl9OM2RsNXZrcnFZdFBZ?oc=5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>46078.52063657407</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Nach Streitigkeit unter Unbekannten - Schaden an Glastür - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>After a dispute between strangers - damage to the glass door - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 12:23:36 GMT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOZnI4UW9KcU5SM0ltNnFWakhJeXpvdGgxdHQxMXRyR2RMak9objhiZkY2VUJUSEpvZkZXNHBzNm1zSzE2d2pvN0hFT0ZsbEhXZzN1N1hGMUo1MXhXY3BneVhWbjVMUEdjdnNyZU9WMGlMY2RmVFFzUlNQSW11VVdTcVJXdWduaUw5Q1ktWDY5b0xTcGZFSTh3ZEZxVmVDck1CZnVsRkV2LVYxMEFZUklBTEZwVGt1NEFtb1d0Um93eHI0eVJGVlBjTjFDOHF0QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>46078.51638888889</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Demo-Termine heute, 25.02.2026: Hier gibt's am Mittwoch Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Demo dates today, February 25th, 2026: Here on Wednesday there will be demos against AfD, misanthropy and the shift to the right - News.de</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 05:55:29 GMT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxQNFdodW8waDJhejU0ZGtoemRUWV9YRlZ1TEtMeVk4WU1RT2doLTBsOEZ1Z29mZS12dFJoYXF3dDVBSHM2eFg5NzloLUVsYjdycDRsc0FnZmtxeExBb0ctcmxyR3FwRXYxbmhDSmRQYXRJUGNPRnQ2cmRzMDJQazZTMUd4RWNlV0NSbU5NUWlYNTROMnZqbllmUnpicHU5RFZscHVjR09rV2pYLWVxck5UTzY2d29aeXd5WUhjQTRfZ1dERXZGNHpxNHlIWXh1SHFBOVcxTDRzS0Q0bmtDdHZuS3FSQlpydDg4WDdVU0pGTFRXUTdvalJkS3N6VVVPVWvSAYQCQVVfeXFMTWNydll2dWxMbEUwa2RNY1V3RVVER2ZjTmZFbGUzdk42M25oYUtONnhPWGV1SXVtcDNUYVlZVVUwVkk1ak1FME9RTWI4aFZtYU9uMHZqRHZkZGtfRFRwTzhnU3NKMEJISHNNaG5XXzdBOXZVQnhZMjY2RnRNZTZWRlpXenRWVWVaVGxYTTBxbmtqRlBPMjktSlBlLXQxOTgwRGZacW9IZTRScFduX0hCaWc5ZGJWc193RWxmd2NkZjFRYVJ6MF96RkhNRGpVRnVsQ3RBUzlLM1VaalRpREdjaFZEY3BrdXZwc25sUXRTNWJ3R3ZsUHhmNUJNSkNpeVRWZmdoaVE?oc=5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>46078.24686342593</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ESPN Signs Andy Roddick As An Analyst, Andy Murray Reacts - Last Word On Sports</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ESPN Signs Andy Roddick As An Analyst, Andy Murray Reacts - Last Word On Sports</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 16:55:39 GMT</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxQd0NveEJPVzlTRG9uTzFEcGt2a2Z4OTBfeGU2dWJsMHE0ei1abXdXQS1TM1NKS1BwdS1seHA2b3VQaHFaYWI4QjVpUExLZGNKVWRLbU1UcGVUYTgwR3BHS3pNbk1LTXdqdEdkNTZIWElLTkpMQVlIQUxuOVNFdDFnS0xiYlVnSjF5bVc4?oc=5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>46077.7053125</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Andy Roddick says whether Serena Williams should return to tennis at Indian Wells next month - The Tennis Gazette</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Andy Roddick says whether Serena Williams should return to tennis at Indian Wells next month - The Tennis Gazette</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 01:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNemVFRjNiSDAwYnFfVjBWRnk3Z01tOUtaenQ4UWo4aXQ5NlRpS3BFZU9MQTlNZUVqZm1wT1ZkUjVkY0hOeER2WDE4TUVkS3pBMWtfSHFLMVhlaXF6cVJ5bm5reU5wVlR0dXpPTktaZ2FBOVpNZFNIQmdJTDdLOU9EUkVzcEVvSTliUzhXQnBqOTRienJaYkIyeWd6cVhFNXVyR2t4QndsWDJ3RUdlMWZvUk80NzFnczEzLWhuMmRkVFVMaV9UWFc0d24wMA?oc=5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="n">
+        <v>46078.04166666666</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>FSU auditing scholar ranks among world’s most prolific researchers - Florida State University News</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>FSU auditing scholar ranks among world’s most prolific researchers - Florida State University News</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 18:53:47 GMT</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNWnZRdlpabjN4UmRMTWhtTmtrU3lpVVhES3Zpei1aWEJhTGFxOHppY2V5R05MUGs1Z25BcS1CX3hvNTF6M0hFVWVIZ2V1VEpNUHh4dC0yRzZmWllKNlFZaXNTTXhIVURRLXRtV1dBdk9wT2FNZ0F2UjZJMF9RVVJlN2UzM1lZMzB1VlFDYU5qTlJIMHhjbE9fVnFROHlIN05sdWtmWWNrNUp1eW9ZVHNsV3dUSWJhSFBKeHlpcDBGdDM?oc=5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="n">
+        <v>46077.78734953704</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Giving | Staff - FIU Herbert Wertheim College of Medicine</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Giving | Staff - FIU Herbert Wertheim College of Medicine</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 21:09:35 GMT</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE9od1VFYUdJaUw5WmNDdFZBaEtfY3F5WWNfRWNrRmpyc0F2V01OTnFVV3ppY1pqYU0yTGpNN29uUWdpcjIxOUprWTJOVG9vZHV6Ym9MU1BGRnNGM0ta?oc=5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>46077.88165509259</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Mit 2,4 Promille durch Lindach: 33-Jähriger verursacht Unfall und fährt davon - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>With 2.4 per mille through Lindach: 33-year-old causes accident and drives away - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 08:56:42 GMT</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPWVFzbGJzMDlkWXkzaFVmZzMwbzB2aVFpcFd4WFdMdFpfLUJ6OF9wWlg0NmJzOXdQVnd3RmQ4QXFrQ3hpUHl4QlExaWJyQWxkQ3JEZHlRQ0tQUW9vZ2R3ZVJadzJvUjdJZEk1X2ZNLU5DSmViTnd5aGhKbXVWaWRKcm5xQzJuOE1BVFFCUnFvZ1AzeGozWEtZczEyQmtDWUJNbjAyM21Vb2hWNUhMMjB0UFZkek5aWWFwT0VoVHJDTXNZUi12VW1DSFVsYmNMZw?oc=5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>46078.37270833334</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Amtsbekannter 25-Jähriger nach Fahrrad-Diebstahl in Ingolstadt verhaftet - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Well-known 25-year-old arrested after bicycle theft in Ingolstadt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 12:29:11 GMT</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE11TExybWZ1aEs3c0hXekZBWDhLVEIyQTJhUW9zbEw5SVVXODFLLVk3cmdKa1NrZTFHeFJhd1lDbzNCVFVCdFdBNHhLa19mS0xXa2tSRkVMa05CZl9LM2N6RGxwOUwteVNqREk4UV9VaVU?oc=5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>46078.5202662037</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Nächtlicher Feuerwehreinsatz im Hotel - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Nighttime fire brigade operation in the hotel - RegionalReporter</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 09:53:21 GMT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNOWpPNjE5YUFuc0F6TnJYR1RwMi03Vlk1TTYyM19zTTkzSkF6R2JxcGtNeWpOc0YtM1hwa3JmR1RlQV9Ub0RXMXYwRFBiZS11MDhtalVKNENaQlItQ3RSN05zZklUcDJzLWxsQWVveTd3Q3ZRRTZpaWlsaTFwbm4weGxJLXFjaW5WbEtVOVd2c3dTZjVtSGo2al85c1U4WTNs?oc=5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>46078.41204861111</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Bekifft auf der Autobahn: Polizei stoppt Autofahrer bei Holledau - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Stoned on the highway: Police stop drivers near Holledau - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 09:11:53 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTFVxM1lJN0FVcHFqLTRvNmdZME9mT1lwTVJpWFgzU0dVa0lWMWxrSlNMVzhUSjZCaFd2VlF2MG9CTHlsVUY2QTVGaENQdUFWSm95aWFzQmltUUZWaWs0S2hTS09COGdXOWdpdHBoYUhzQnZKdzJrUFprNWtCNi1IQUtvZnNCY1JuVUxOWUhJa0pKdmFscWFlcWtQWGZfVkNlMXZWNlJIRVdXa1Q3UHpONlhBYzFHVkZyVjFOeQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46078.38325231482</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Germany's FC Ingolstadt makes special collaboration with Kashmir's design house Pumposh - India TV News</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Germany's FC Ingolstadt makes special collaboration with Kashmir's design house Pumposh - India TV News</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 07:15:30 GMT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNUTdkcE9MOUlfSndGTER2U0Z3anVFMWxqM1RDYThNZ1lNQm0tLTc3MHRlNVRRanpyU3pyRGFYUXZQTE4wUEszaDFkVHNJUzRUTlczUGxNSHJQS191ZnRoOUVoVVZGMWZMME1rdGFpaFVOSzZNNEl1cm5aUEFpMkNwWUJDZk9KNGZGSmlaWHZySXd1bE1KNHVJdDNyN0xRYWdYUWExM2ZpZS16M3ZwYUdmTTczeklEQUR1NHhkRVd5ZGFYT0lGcUk4SGtfNml0TjZ2RnZFSGVRLU95dGE2V2JfZjR0RXQ1a05aaFpv0gHrAUFVX3lxTE1RN2RwT0w5SV9Kd0ZMRHZTRndqdUUxbGozVENhOE1nWU1CbS0tNzcwdGU1VFFqenJTenJEYVhRdlBMTjBQSzNoMWRUc0lTNFROVzNQbE1IclBLX3VmdGg5RWhVVkYxZkwwTWt0YWloVU5LNk00SXVyblpQQWkyQ3BZQkNmT0o0ZkZKaVpYdnJJd3VsTUo0dUl0M3I3TFFhZ1hRYTEzZmllLXozdnBhR2ZNNzN6SURBRHU0eGRFV3lkYVhPSUZxSThIa182aXRONnZGdkVIZVEtT3l0YTZXYl9mNHRFdDVrTlpoWm8?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>46078.30243055556</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Restart after the break: Red Bulls host Ingolstadt in top match - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Restart after the break: Red Bulls host Ingolstadt in top match - EHC Red Bull München</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 17:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNUFljMGRGOVlqSlNXT2ZCYTFGSVJMNllmTF9LVFhFVWJhb0NnZ1lWZTY1cmdKejZRbi1nV19zdjVKUGs5d1ExZHdwZEl1aXdkQ0s5eXBUT1lYY3BtZ1V5MjdxeG5jZzJvaWpURWVORTQ0eVExSFBoMHBuSE1mazhVa280M19FNXpETU0tNkpJSEM4ZkM5VU8tOVFyX3M2c2FVWHkweDZ5MGVhYzkteTVPQ2hya1o?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46077.70833333334</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Kashmir’s Sozni embroidery scores international tie-up - Greater Kashmir</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Kashmir’s Sozni embroidery scores international tie-up - Greater Kashmir</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 18:13:16 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPRFpzbUVlOEdhUXpURGZlRHdXZENLSW5RbHlua0lWY1gtajI5Y3dVTllfZGo2amdKXy15emZuQTlTcWJhUWFnNXVSVFZTQ2JaMU5TTi1GbzZCcV9KY2ZDYVFYTEplOFVobktnRzVTWTU0Z2ZEc1NhRnc5c09uYnd6RHBjNVVJNXRSTkpkdzZFNk5xUVFLM3NTcjRqNTk3UTFYUFlr0gGjAUFVX3lxTE9EWnNtRWU4R2FRelREZmVEd1dkQ0tJblFseW5rSVZjWC1qMjljd1VOWV9kajZqZ0pfLXl6Zm5BOVNxYmFRYWc1dVJUVlNDYloxTlNOLUZvNkJxX0pjZkNhUVhMSmU4VWhuS2dHNVNZNTRnZkRzU2FGdzlzT25id3pEcGM1VUk1dFJOSmR3NkU2TnFRUUszc1NyNGo1OTdRMVhQWWs?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46077.75921296296</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Bus stop in this Kildare village may be moved - as new route is built - Kildare Now</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Bus stop in this Kildare village may be moved - as new route is built - Kildare Now</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Tue, 24 Feb 2026 20:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPX1ItOE1UMVNYQTlkVzBtT2RiNWwwd214SFNKOEFobWoweGt0M3B1eTFfU09sNGNWM01YNVNYQ1VHN243UXNrTU1LdG03Vk41SUtmTnBoOUtYQ044ejdoVlFacm13dEVoRlZhTmY2NmJCNm5SbGJOdGpiUGxlbEVsMWppSV9CeVVURDRNUWJvQjYwaEVvN3NncXo3M09QUm1lVnhTbTN5di1GNU9sbUE4dlF5eXRXZlZmbHZYTl9mcw?oc=5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>46077.83333333334</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>Local Town Fidenza English</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>("Fidenza outlet" OR "Designer Outlet Fidenza" OR "Fidenza Village" OR "Parma" OR "Piacenza" OR "Cremona") AND (protest OR bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR evacuation OR "police operation") AND -football AND -transfer</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>Parma police welfare check on man who made 'suicidal statements' ends with deadly shooting - News 5 Cleveland WEWS</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>Parma police welfare check on man who made 'suicidal statements' ends with deadly shooting - News 5 Cleveland WEWS</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Wed, 25 Feb 2026 04:43:14 GMT</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQbTJBbWl5WFE4TTZJLU5XcDd6c3FYM0Z3OE8zQjNJUHE5c0FibWdKb0dJbk9VYjViMDBsUFhMZmUxQVdsVkVralpIS1l0cnFTQ2tYazdYTDNDX1VMX2RxWURSbjVXdWlIbHYzWGNVbkNyVEJ0d1hlMzFJZGFUMlV1b0t2eDB2UkNfS2VGcGtvTmwtRzVPbnFFYm1TcjI3N1ZoYldnenVZXzExR2hzUlE?oc=5</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
         <is>
           <t>en-GB</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J58" t="inlineStr">
         <is>
           <t>GB:en</t>
         </is>
       </c>
-      <c r="K24" s="1" t="n">
+      <c r="K58" s="1" t="n">
         <v>46078.19668981482</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-26 07:57 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail (LON:BME) Share Price Crosses Above 50-Day Moving Average - Should You Sell? - MarketBeat</t>
+          <t>B&amp;M European Value Retail S A : Prospectus - Migration - marketscreener.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail (LON:BME) Share Price Crosses Above 50-Day Moving Average - Should You Sell? - MarketBeat</t>
+          <t>B&amp;M European Value Retail S A : Prospectus - Migration - marketscreener.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:18:55 GMT</t>
+          <t>Wed, 25 Feb 2026 11:51:05 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQcHFXTEZaaGNtSW1ibVVBT0NDaGpEZUxpOTU3d09xRElNX29wbEJBaU1Jc05NUUZobWg0REtXY3d6MU9Xci1sU0JNRVRzQUg2dnYxVFpiSy1DNGxUV2FBRmh1T3JhdWN5bnJxc2dySEppY2lmUnpZZHV2TVBTWjRMcUVrMUxWUzBaaDZmMjhPaWxSa0l1UFJHczFOaHJ2dk9rdzMzVGJacFpURkVfSjEtNzNwekhJOUJ2LWd5d2pHSll4RDU5c2N0UGcxdm5WWkZlWkc1LTB0bzFjdWVxbmYwb1dqWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxORnRLQnN2cTNWWW1pT0RGT01Hc3ZCRXNxZmdWZzZaaVZVMDdpYzRpQnB0ZDNNbWVsdEFxSnhYSGk1RC1YNkNwWVRSc1Y1cUZUcUpuNVhMQ3lpQUdwTUlRT1o5d1pfZVdQSE5aRlZNMHZER0hrOWRQS25MYkQ2T1JyQUVOYnZ3OFZqM1BiTGJYaklNTXFRNGtGMG1nalJkOWxTU0lLdndn?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46078.47146990741</v>
+        <v>46078.49380787037</v>
       </c>
     </row>
     <row r="3">
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B&amp;M Publishes Prospectus Ahead of Jersey Migration and London Listing Move - TipRanks</t>
+          <t>B&amp;M European Value Retail (LON:BME) Share Price Crosses Above 50-Day Moving Average - Should You Sell? - MarketBeat</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B&amp;M Publishes Prospectus Ahead of Jersey Migration and London Listing Move - TipRanks</t>
+          <t>B&amp;M European Value Retail (LON:BME) Share Price Crosses Above 50-Day Moving Average - Should You Sell? - MarketBeat</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:05:35 GMT</t>
+          <t>Wed, 25 Feb 2026 11:18:55 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPNElkenJwY0R3U1AyNnpVeU1VclhkejRWUFhEOVlPUXY1VTJ3azBhRVI5eVc1T3ZQRG5vN1hMMy05MUJPQUkzRGdreUNVWmd4VnBPYVRScTFoSkFvUGVjMWExZjg2bDZXWms0a1Q2anpjWTNSZC1nTXU3WDJwbDJVMW5BVmhvRk9kYXo4WXoyVHVmTHJiSE8zM0ZZT2t3QVAtY09KOUpxUEpReFR5NVU1SGZiQ2p6SkJ4a1pzMUtqVFVPcTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQcHFXTEZaaGNtSW1ibVVBT0NDaGpEZUxpOTU3d09xRElNX29wbEJBaU1Jc05NUUZobWg0REtXY3d6MU9Xci1sU0JNRVRzQUg2dnYxVFpiSy1DNGxUV2FBRmh1T3JhdWN5bnJxc2dySEppY2lmUnpZZHV2TVBTWjRMcUVrMUxWUzBaaDZmMjhPaWxSa0l1UFJHczFOaHJ2dk9rdzMzVGJacFpURkVfSjEtNzNwekhJOUJ2LWd5d2pHSll4RDU5c2N0UGcxdm5WWkZlWkc1LTB0bzFjdWVxbmYwb1dqWQ?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46078.46221064815</v>
+        <v>46078.47146990741</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - 一财全球Yicai Global</t>
+          <t>B&amp;M Publishes Prospectus Ahead of Jersey Migration and London Listing Move - TipRanks</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - 一财全球Yicai Global</t>
+          <t>B&amp;M Publishes Prospectus Ahead of Jersey Migration and London Listing Move - TipRanks</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:52:27 GMT</t>
+          <t>Wed, 25 Feb 2026 11:37:09 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQQVhnQ0Y1UWRwRmdlb3JBNlR3NG9RYzhSZ0thTkhtWHRKWW1rbjdRYmJKeXJzeE8wMUpiVTZ5aV8tWTVZQnA1LU5NejhlREM2SmluVjI4T0dKMk5kdjBtQkQ1WXhmWkJHVFV6YlgzcXBfaTdKME45SVFZV1Aya3pfRTZPVFBBSTFrd0JBZHNlbmd3R0lNa1VTZ2NFcS1QTmhvVy00S2p4Mmt6SkVwTXU2QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxPNElkenJwY0R3U1AyNnpVeU1VclhkejRWUFhEOVlPUXY1VTJ3azBhRVI5eVc1T3ZQRG5vN1hMMy05MUJPQUkzRGdreUNVWmd4VnBPYVRScTFoSkFvUGVjMWExZjg2bDZXWms0a1Q2anpjWTNSZC1nTXU3WDJwbDJVMW5BVmhvRk9kYXo4WXoyVHVmTHJiSE8zM0ZZT2t3QVAtY09KOUpxUEpReFR5NVU1SGZiQ2p6SkJ4a1pzMUtqVFVPcTg?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46078.36975694444</v>
+        <v>46078.48413194445</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shoplifting UK</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
+          <t>Cotswolds described as the Hamptons of London: top hotels, restaurants and shops - artthreat.net</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
+          <t>Cotswolds described as the Hamptons of London: top hotels, restaurants and shops - artthreat.net</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:32:50 GMT</t>
+          <t>Wed, 25 Feb 2026 23:29:44 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOY1NoSnNJUHdDZVlIYkRJazd4c01fay1YMjNDQU83U0pPczJYdmRwbUFKQzV3S21sTFBnQXNoWmhhNjVoWG03N1ZZUnJRSnpzdC0wamFZY3lRWWpBMmFzTmh1LVlzT3RlYlZabDYzWG81emRxRnFxUWVZVGNuU0xDSTJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxQVzJVSmc0ZVMxQ0NnU1lBREZSRjIydFo0VzVjdDNqTGFOWmhIZ0pPakEyX081b3dVcUF4bHBHZ3lkQnk3Y1dZcnNQNEh1NXZ1V3ZmaWYtd0Jua0V4aGhuYTU3MGtjY1FpVGlRYW1GMnY3YXZzMmtYdFZjMlZPQklrOURZWDMzWmlxQmFrT1hIRTVzMVZiaGpqTjhJTWczYUVYaUlZVmxpSDJVdw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46078.35613425926</v>
+        <v>46078.97898148148</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Staatssecretaris Erkens snel naar Brussel voor beschikbaarheid CO2 in de kas - Nieuwe Oogst</t>
+          <t>Latest update on closure from city centre sandwich bar - Oxford Mail</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>State Secretary Erkens quickly goes to Brussels for the availability of CO2 in the greenhouse - New Harvest</t>
+          <t>Latest update on closure from city centre sandwich bar - Oxford Mail</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:00:00 GMT</t>
+          <t>Wed, 25 Feb 2026 16:00:00 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQWZDWTliTDZRMU1Ub3BtNHhTSDFXTWRmUzBZNlpVZV9LRDhZeU9DOWY4b0Q5STc0U1ZNb2NON2tDY1NoR29GdXdxRTNIUGZXcUI1NEJJUzlIV2dubl9kUGdvYjNiN1NYZDRpY05PUmZVWTFpR2d6Yk5kZXZHejZVVXN5a1U0Zkxpa3lwZU5SbGN4eUZ1OS1MRm1fbjlzMENkc2NyNHVGT3FxdkQ4bDMweV9ITVpBeWluSXFpenln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQRlp2RTlpNXNRZkl4eEdMMzF2cVZVbDBJRC1nQjAyQnhobUN0SkcxMEE2OFItdnlBalptekFQeTJRWTNJcUl4RlhTbFBsSUVTekhYbmQxNlhRLVhxZmpFbk9SWE5EQ3pnajdyV3JWdFkzMV9Oa2oyVGl5SnY1RE8wZ3lIZmR6QUo1R0QzMTZFVU01R1U?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46078.41666666666</v>
+        <v>46078.66666666666</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Verdachte van taximoord in Geel probeert tevergeefs vrij te komen: ook in beroep blijft A.B. (20) aangehouden - HLN</t>
+          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - 一财全球Yicai Global</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Suspect of taxi murder in Geel tries in vain to be released: A.B. also remains on appeal. (20) arrested - HLN</t>
+          <t>From Bargain Bins to “Mini-Vacations”: China’s Outlet Boom Deepens as Sales Rise 9% - 一财全球Yicai Global</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:43:43 GMT</t>
+          <t>Wed, 25 Feb 2026 09:13:54 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNS2pxcUxaMEF6Nm96R3p0Z2VzSVhGblZfTktvV0VGVlJXb0tMU2FVLVJ4YU5kYTFEakdZRVJ4aU1ZcmdWMkYwd1FNVThPUDQ1SG1tXzd2YndKRTVxSnZ0aEN6ajlXSHdqdUI3RWV1aHVMcTJoZlBpVmhLaUsxUWpYXzR1aVNWNGpVbWZNNmhaZEFZYWRUdF9Eay1FWXdHWmozYzVhRVBSV09zdmtJU25fUmN1bTFEMzBoUmZKVHNfWURnWTc0YXd0M2FfM1JYZ0ZLNXNZeU5R?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQQVhnQ0Y1UWRwRmdlb3JBNlR3NG9RYzhSZ0thTkhtWHRKWW1rbjdRYmJKeXJzeE8wMUpiVTZ5aV8tWTVZQnA1LU5NejhlREM2SmluVjI4T0dKMk5kdjBtQkQ1WXhmWkJHVFV6YlgzcXBfaTdKME45SVFZV1Aya3pfRTZPVFBBSTFrd0JBZHNlbmd3R0lNa1VTZ2NFcS1QTmhvVy00S2p4Mmt6SkVwTXU2QQ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46078.4053587963</v>
+        <v>46078.38465277778</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Shoplifting UK</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("shoplifting" OR "retail theft" OR "retail crime" OR "shop theft" OR "pickpocket") AND ("UK" OR "England" OR "Britain") AND ("gang" OR "organised" OR "trend" OR "rise" OR "survey" OR "report")</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>False bomb threat at Brussels Airport prompts security response, no evacuation required - Aviation24.be</t>
+          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>False bomb threat at Brussels Airport prompts security response, no evacuation required - Aviation24.be</t>
+          <t>Shoplifting on the rise in Scotland - Scottish Grocer &amp; Convenience Retailer</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:40:50 GMT</t>
+          <t>Wed, 25 Feb 2026 08:32:50 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxNSFFvV1Itc3d0a2YtTS1zQzBpLTRta2RQWnBZU2c4akI4Um1tSXNabVhWb2doeWI5T1BCM0taSVdFY3kwUDV2UkZJRFFYejJ1STBtcWRDRjRDUmlvX2kzZWVNN3NyOENzQkdBR0JLUXJpZlc5ckM5Z3Y3T0RSaXhwNjAyTXF1M1ljemVaczdOZHo4SXpaVUlLYnUzN3E2NEh0T05xM0lSSTRJVmJ2cS1vT25SbzI4Mkd5UDZCQ2RtYlZrSTlabFg1TW5MdGtBTHo5ekhfY1JwdF9Sdlk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOY1NoSnNJUHdDZVlIYkRJazd4c01fay1YMjNDQU83U0pPczJYdmRwbUFKQzV3S21sTFBnQXNoWmhhNjVoWG03N1ZZUnJRSnpzdC0wamFZY3lRWWpBMmFzTmh1LVlzT3RlYlZabDYzWG81emRxRnFxUWVZVGNuU0xDSTJn?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -850,47 +850,47 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46078.44502314815</v>
+        <v>46078.35613425926</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Plus d’une vingtaine d’agressions au CPAS de la Ville de Bruxelles : des sanctions sur le RIS envisagées - BruxellesToday</t>
+          <t>Explosie aan openbare camera’s baart privacywaakhond zorgen - De Standaard</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>More than twenty attacks at the CPAS of the City of Brussels: sanctions on the RIS envisaged - BruxellesToday</t>
+          <t>Explosion of public cameras worries privacy watchdog - De Standaard</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:32:00 GMT</t>
+          <t>Thu, 26 Feb 2026 05:30:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNblV2Mk45V3MtT0hiU0J4cEVLSkk0QVFOOXFRS05TTUVwZVk2NVFmWG9COV9Od001MDcxdzBnTWpydVlnWVFEOUk4MlNOLUMySGJkZFFpM3hPNVZJMExmSXVkVS1mQW0zQ3E0d1pLTjFwMjZ5a0tqQ1RJLVRjc1NrdE55eGVJMDFSMkYyWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPTUJmTFZIODZ3UWpNWlJXNVQ2NTZlcDF3M2xtam9BTUlHWDZPYUFFU0pGRGlYOXJKVXNDT1BKMTVrMUxwQUlNNHB4anZkeFc2aE1TOHg5emlQSDBQQ1N3LVRsWS02QmJwWWtZZHNWYVB1SDJKOURaWDNvckdjMHVKLU9ZMm5uYnhtTjc1eEVpa3p0R3YwZDZ2MmZvbmFNY2ZxbTdxaHFPbEZlR0k?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46078.48055555556</v>
+        <v>46079.22916666666</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Un couple violemment agressé dans le parking du Basilix Shopping Center - 7sur7.be</t>
+          <t>Jens Grieten (Kompass Klub): "Goed dat technocommunity duidelijk zegt wat niet kan" - VRT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A couple violently attacked in the parking lot of the Basilix Shopping Center - 7sur7.be</t>
+          <t>Jens Grieten (Kompass Klub): "It's good that the techno community clearly says what is not possible" - VRT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 14:12:00 GMT</t>
+          <t>Wed, 25 Feb 2026 23:00:29 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOUnZUY0VBMTBiVVZHZzJJVmEtZHBoZTlGaDN2azJQNV9mejN3Nms0TVJja292Z0JrNTRZSjFiR25EdlY5UTNES1Y4azJzV0RpMWNFYXFUMUZoUmZqV0U1NmlnRkV5ak9EVHRybVRSZUg5dFFUZ1pjcEV0WkFnRXNab0oxQm9PdUV0QklCbk9ONFhOQ3NtRFFBTmtIdUx5UTI4ZEhnN3lVSnFaQTBaR1Z3c1gtWi1sQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNaEpjUlo2Q04wMV9Vam9XdlRBdTdRQlUybmhrTlJjei0tTHRhbENIRHB5UmhsaUxuZjltM2NzaEFReWRwNWFsbEszRFFrYzhYNktvVnhoaTgyUkdXREgtLVRCVFBVX0dkd3FNNkVXUGQyVVBHTzV1MmVvVkh1cm1mQXVJeXVfZ0kzWHVUNDJYaENnVkw1YkgxNVppYjJDREpLaGY0?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46078.59166666667</v>
+        <v>46078.95866898148</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>18,9°C à Bruxelles: record de chaleur battu pour un 25 février - 7sur7.be</t>
+          <t>Staatssecretaris Erkens snel naar Brussel voor beschikbaarheid CO2 in de kas - Nieuwe Oogst</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>18.9°C in Brussels: heat record broken for February 25 - 7sur7.be</t>
+          <t>State Secretary Erkens quickly goes to Brussels for the availability of CO2 in the greenhouse - New Harvest</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 13:24:03 GMT</t>
+          <t>Wed, 25 Feb 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVUxQbFR1U2NjQXJ0bWFIbEx6REd1YlhFZFJ2eVpmQkRveFFZNU5jdWVoUFM4U3FhTl95eXVRMTlYb1lKcEhTNDRGYXoybUZOQ0dhNFZkMHdHdGRYTkNJd0UxbjlxN09KSE80a2FmQ095d0pWczY4TzMwZXBZTjVySEQ2cnYzY3pKMnJYWUwtTEhXQ0ZLUlR4VF8wRFh3cFlTOUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNQWZDWTliTDZRMU1Ub3BtNHhTSDFXTWRmUzBZNlpVZV9LRDhZeU9DOWY4b0Q5STc0U1ZNb2NON2tDY1NoR29GdXdxRTNIUGZXcUI1NEJJUzlIV2dubl9kUGdvYjNiN1NYZDRpY05PUmZVWTFpR2d6Yk5kZXZHejZVVXN5a1U0Zkxpa3lwZU5SbGN4eUZ1OS1MRm1fbjlzMENkc2NyNHVGT3FxdkQ4bDMweV9ITVpBeWluSXFpenln?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46078.55836805556</v>
+        <v>46078.41666666666</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>La CGSP Cheminots dépose un préavis de grève de trois jours sur le rail en mars - 7sur7.be</t>
+          <t>Verdachte van taximoord in Geel probeert tevergeefs vrij te komen: ook in beroep blijft A.B. (20) aangehouden - HLN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The CGSP Cheminots files a three-day strike notice on the rail in March - 7sur7.be</t>
+          <t>Suspect of taxi murder in Geel tries in vain to be released: A.B. also remains on appeal. (20) arrested - HLN</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 14:29:00 GMT</t>
+          <t>Wed, 25 Feb 2026 09:43:43 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQeUhLZk83MmROZnNOYmVrMVhkRWdUWWtQTExucWItbEVHUm4wMFp3bzJ4U3dWN09XSUt5bDNEanQ4YTZFVHhDdFZsR3gzc1oxYzVyX3ltU0RCVVI2b00wSTc1S1BfX09rZGVDR0ZrUjhvV0o5dEFTU0lYUDNzbDFmVFJ0eXV1cU8tMlRGOWVZX0VZMHBNaUpSVnpRaDZRbnJrQkk2WXNmY2ZXTmVTUUlCOGo0WGhsTE1WMUl3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNS2pxcUxaMEF6Nm96R3p0Z2VzSVhGblZfTktvV0VGVlJXb0tMU2FVLVJ4YU5kYTFEakdZRVJ4aU1ZcmdWMkYwd1FNVThPUDQ1SG1tXzd2YndKRTVxSnZ0aEN6ajlXSHdqdUI3RWV1aHVMcTJoZlBpVmhLaUsxUWpYXzR1aVNWNGpVbWZNNmhaZEFZYWRUdF9Eay1FWXdHWmozYzVhRVBSV09zdmtJU25fUmN1bTFEMzBoUmZKVHNfWURnWTc0YXd0M2FfM1JYZ0ZLNXNZeU5R?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46078.60347222222</v>
+        <v>46078.4053587963</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Le Fuse, mythique discothèque bruxelloise, bannit les smartphones - 7sur7.be</t>
+          <t>Bom barst in dancewereld: top-dj’s beschuldigd van seksueel wangedrag, optredens in sneltempo geschrapt - HLN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Le Fuse, legendary Brussels nightclub, bans smartphones - 7sur7.be</t>
+          <t>Bombshell explodes in the dance world: top DJs accused of sexual misconduct, performances quickly canceled - HLN</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 14:45:00 GMT</t>
+          <t>Wed, 25 Feb 2026 07:57:50 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNUUlsblRkYlJOTjhrWEpkX253MEh4S1ZfcUtIUm1qQVkzRnQ5XzI3MmpIY05nVDBlSFVxS052amU2TWczSVBWLUc5WEVtSEhZZU5ma3Y0bkZLY0dCal8xU2k3OEw0NWlCbUZLaVlWOVYydGJadlBlMHEwOUJRdGlId0plMEFpaUNZaTZ1Y0JpSHQzYTJBVTNZQVRUOFlFcVVOYzJMREpB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQaTJaVF9JOXJmVjVHcndLMzM4TThwWjBSV3hkbG10VTlUTFBJU1NfdGVvZC1XdHVxOWZJOW9jU0FLRTJ0a0RIbnVueFBoNEZtQlgwdlo4b0ZJdEk1NkcyNS1jbU1QQjNHMHlSaE94azd6QTgzc2xkMzlSSjIyN09CeXZDel9xNmRWVTJfQm5FQV9zb3JrUzdwNkZjNTVCdjZrRmxKZTlKdkFmQzVkWVdSOFFQQkJHMjBUaTdydUpUbF9MLW1GcjNxRV9zMWlxdEtNeFZn?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46078.61458333334</v>
+        <v>46078.3318287037</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Le CPAS de Bruxelles victime de 26 incidents violents en 2025 - 7sur7.be</t>
+          <t>Man op elektrische step slaat op de vlucht na routinecontrole in Brussel-West: politie vindt meer dan 1 kilo marihuana - HLN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>The Brussels CPAS victim of 26 violent incidents in 2025 - 7sur7.be</t>
+          <t>Man on electric scooter flees after routine check in Brussels West: police find more than 1 kilo of marijuana - HLN</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:04:00 GMT</t>
+          <t>Wed, 25 Feb 2026 15:18:41 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQMXhzcDN3dmtBX25uRkppaVJkQ09CZnVZem42ZUd4WUhmUDRSTUpmTVRiM1E5VUdoVl96U2FlczJYSU42TEVkaXpCTmdGVVVVQXFGMXE5ZEdjZGc3NWpncjFmX29ZckV0aTJOS3pwX2NHSmk3b3dFQnZWdjQ4N3hsWklTOFlxWl91cFNraVVFRGJFeldWNHFjc3Vqbnk4WGFNWE9r?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxNMnlETE5uMDVNNFA4R3FWT2EtNUFXSlJkdERxZHhHZ1prSHhiUVlUVWJDdWE2bnV1NzgyYl9oYVRHd09QcmV3NjkwcHVpbGd0dEdEdG9rRHBhUmlaWkZRcW51dVpnb081MkpFRlgtQTJXYzZRVlhXenFkZ0dEM3BwbGROTTBaS0RTZUxvMDhERGo1eGJtczktZU42aEFtRjl1UGVkZ2d0Q0NjVWE3TkVsSXJlUXhkWUx0OGxLSHg5ZGxUY2VXN1NNRF9Nd1Ytb3pVVmktZjQ0Um4zS3BRaXZfeGU5ZEVwWmhoM1E?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46078.37777777778</v>
+        <v>46078.63797453704</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Engie propose de l’électricité “gratuite” en cas de surplus d’énergie renouvelable - 7sur7.be</t>
+          <t>False bomb threat at Brussels Airport prompts security response, no evacuation required - Aviation24.be</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Engie offers “free” electricity in the event of a surplus of renewable energy - 7sur7.be</t>
+          <t>False bomb threat at Brussels Airport prompts security response, no evacuation required - Aviation24.be</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:18:00 GMT</t>
+          <t>Wed, 25 Feb 2026 10:40:50 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPeXlMTUppZ1lhWFQ1cG5QOFo0S1pMQWlVZEg3TFNqaUtQNFk1N1IyM0pLbFRTWmE4dkE5RWNBTjhZOGRwR0l2S05yZjlEZXpEdXprMTg3ek1UVjBVejc5RTAzWmxkeVdybEdnMU9qVHpoRFJXV0praWo4ZG9RZXJfX3JBRkFkdEJEanA5NU9kZVlGTzdfeTJKaVVJTUZaZmlrTU4zeXIxdF9GV1E3eGQ5QnNMZ2RSYXh0VFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxNSFFvV1Itc3d0a2YtTS1zQzBpLTRta2RQWnBZU2c4akI4Um1tSXNabVhWb2doeWI5T1BCM0taSVdFY3kwUDV2UkZJRFFYejJ1STBtcWRDRjRDUmlvX2kzZWVNN3NyOENzQkdBR0JLUXJpZlc5ckM5Z3Y3T0RSaXhwNjAyTXF1M1ljemVaczdOZHo4SXpaVUlLYnUzN3E2NEh0T05xM0lSSTRJVmJ2cS1vT25SbzI4Mkd5UDZCQ2RtYlZrSTlabFg1TW5MdGtBTHo5ekhfY1JwdF9Sdlk?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46078.42916666667</v>
+        <v>46078.44502314815</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Vrai ou faux. Le député LFI Raphaël Arnault a-t-il été condamné pour avoir protégé une manifestation LGBT ciblée par l'ultradroite ? - Radio France</t>
+          <t>Ireland eyes closer cooperation with NATO neighbours to handle maritime threats - The Straits Times</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>True or false. Was LFI MP Raphaël Arnault convicted for protecting an LGBT demonstration targeted by the ultra-right? - Radio France</t>
+          <t>Ireland eyes closer cooperation with NATO neighbours to handle maritime threats - The Straits Times</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:23:03 GMT</t>
+          <t>Wed, 25 Feb 2026 15:22:16 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPd0hMVEw5NlBKdXdBMlVrWk4xREZZZnU5RmxDUVpwUHJqTndLeWZ5ODV3dUozZndOTDFpLUpBWHJkMjA3Z1p5TVM0TVNzOHBYbURfSnl6NzJSeWdJazJKYko0NW1MVXdKTmo3cVNjYWxYaGZLX2RNZXctVVlGaDhlYWNNc25VQUJWZ2pXZVA3NjdnSkRqMGtLczZOdjRKNzM0aThJeUVzai1fX2E2d1BpdVY4ZHQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQM2ppZS1xNFdnNTZlbFBVazZoUWRVblpDbnVVVGlvWmJuMlJqamJEdzY3UnY1eFQwMC1sV0o2dl9nZE9WODNnVXpybDA2Ym5YRjJmN29YczBwR2VheEdZUFpnWXFVTXdlVTd5cU91Zm5zb3I1R1VLakJrQVVDX0ltQ1lGZHh3eGZMZUNyZmxYWE1wRkkxb0xXVWRJNTAzQVBFMzBsbUFzN2RsRWF2QUFmNHFkYjVYcHdKczBDVDBoWUpFOU5oM1BZRHAyUjI0UUNBNC10aFZWc0IyUQ?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46078.47434027777</v>
+        <v>46078.64046296296</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mellrichstadt: Polizei ermittelt wegen Jagdwilderei - Radio Gong Würzburg</t>
+          <t>Spirit Airlines to exit second bankruptcy as smaller, restructured carrier - Aviation24.be</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Mellrichstadt: Police are investigating hunting poaching - Radio Gong Würzburg</t>
+          <t>Spirit Airlines to exit second bankruptcy as smaller, restructured carrier - Aviation24.be</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 12:00:00 GMT</t>
+          <t>Wed, 25 Feb 2026 15:34:21 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQRS1wU0U3U3dQSTlMOWFiOU9vRHI3NEhFZUxGOGUtTzhKUi1DV3h1SEZNV1VnMDNEVVBVUHFzbUlFdkRMR3BQWmlHTEVjRlU5ZXgtWkF1Q3NKekI3TGp6UW41Y1BqMlR0aUxWbjNaRTVQQmkxaWtua1BiT3NWdXFfWnd3QjFXX3hSR0dfUw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPU18ydTBZVGxoYWJ2cjRvQk45UHNGZE1GNVRfczhTenoydTA1ZlgxaUVrdXgtQXp6ZWs0Mmd4bWhGVHY5cy1QMXdxMkJSb0tDTlg4anJzTnFpT2FUMnZ4ejV3V2ZPV3RCOGlkTWRpUTRjMHZSbWpxUXo4M28xemVzeDhTSVNqV3NnT0R2VWtYZzk3OGZGbU5zMGtBQnVDTUY1OGViOExRMTNYbk1uRF92VHdJalVKRmxzZE1lUHVRdy1sNDM0UHF4dg?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46078.5</v>
+        <v>46078.64885416667</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>U.S. Airforwarders Association criticises 10% import surcharge, warns of supply chain disruption - Aviation24.be</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>U.S. Airforwarders Association criticises 10% import surcharge, warns of supply chain disruption - Aviation24.be</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 12:50:41 GMT</t>
+          <t>Wed, 25 Feb 2026 16:06:30 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxORERBYk5UUzVzUC13Q1R3SktnQ2gxN0F4SjFxR0dfZmt1cGtCNDRTMnUzYU9oeUlUYmpFZkRWT25FU3ppa1d4X2E5ZlFEUHllMEU3aW9WTlZKQUZPdVJvQVJyNkE0U2RwdDFsbDJtQUlEMUlNaER0M2hseDFCTmFhb0tiNmJNM1l4MmVsd0JGQzF2YXZzVzJZRFEtN21HczdtNmxmdVBmQ3pmR19WNVNJVTFCMU9WMnBXMTVKVXlsWHM5b0MzUTg2X01zbzZpMGhreHY3Y1VCODZKcDFhYldCYmw2cXpCQzVHSEtCY015UFNpU3hUdHRB?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46078.53519675926</v>
+        <v>46078.67118055555</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Herrmann: Wechsel an der Spitze des Polizeipräsidiums Unterfranken - aschaffenburg.news</t>
+          <t>Etihad deploys A380 to Bangkok from October 2026, bringing The Residence to Thailand - Aviation24.be</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Herrmann: Change at the top of the Lower Franconia police headquarters - aschaffenburg.news</t>
+          <t>Etihad deploys A380 to Bangkok from October 2026, bringing The Residence to Thailand - Aviation24.be</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 12:29:43 GMT</t>
+          <t>Wed, 25 Feb 2026 14:42:33 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPblZ5bjRhZmwxUjdVbElESmtfSkxtSmZyZmpKWDc3ekVUTXYwWmRjMVk2aDVGc0FRa0YtcmNudzJVdUNSc3EzSk8zeWhvSGdJTkRTQzA1SDdCbDBGRUZ4RjU5WkpGYXhHb3ZpUUFrVEtrZWJLNkpfM1g5QzhSQTZaeWE2Tmk4cmJNTWxscS1KYkFXMTRrR0hFa3YwcDB1RmtSTl9OM2RsNXZrcnFZdFBZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNRkhFdmhYaC1PTG9YcERvYVNtVEVHWG1nbWVoQW80Y1J6ZldzckNkRVVHYjhvdUpTVUxHcVF2bDVZQ1QyaWQweDBQdUw3eTRxaGJIV0lFZHg3Tk5CVEM5N18tbkNtRTcwNnJRbENya29IZDY0Njk3bXVIcWJqTEhMN285SWtMMzZ0ZWFMRkIzekVvczdWbW5uV29QY2ItQml6UGVJc2wxWjVpS3VrWUxzUDhxVE9KYVUtTzBjcU9VZmNXNXJUNkN5RlRZZEZ0ajZFLVJBRA?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46078.52063657407</v>
+        <v>46078.61288194444</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Würzburg und Kitzingen: Zahlreiche Fälle von Telefonbetrug - inFranken.de</t>
+          <t>IAG Cargo launches 24/7 global AOG service as demand for rapid aircraft recovery grows - Aviation24.be</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Würzburg and Kitzingen: Numerous cases of telephone fraud - inFranken.de</t>
+          <t>IAG Cargo launches 24/7 global AOG service as demand for rapid aircraft recovery grows - Aviation24.be</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 12:14:00 GMT</t>
+          <t>Wed, 25 Feb 2026 15:56:28 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNUnhNMDF3d3l3S0tqeWlNdEJraVlaaXVXSTFBdFFrcUIzNHRXcEYtcFNoLVlVS3BMZzFNY1hjWlQ5b183eGFYdHVrUDhvbG9CWC1HTGhibTlRRXhrMnlLMUlBWFMxY3l6MUpuc3VJdUtkSGh2R2ExOEp1d2hEdUpJX2M0RklFeHVGOVRZUkF6V0lES1Z4Y0s1LTVHb1dXdGp5bVBESVNDcnFaalV5MTJyN01OUW5odldvaGRB0gG7AUFVX3lxTE1SeE0wMXd3eXdLS2p5aU10QmtpWVppdVdJMUF0UWtxQjM0dFdwRi1wU2gtWVVLcExnMU1jWGNaVDlvXzd4YVh0dWtQOG9sb0JYLUdMaGJtOVFFeGsyeUsxSUFYUzFjeXoxSm5zdUl1S2RIaHZHYTE4SnV3aER1SklfYzRGSUV4dUY5VFlSQXpXSURLVnhjSzUtNUdvV1d0anltUERJU0NycVpqVXkxMnI3TU5Rbmh2V29oZEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxQQVF1ZEFLLWJqNWdoTFVkQVhZX1JiNlNyTlBndDRNekZwYzhKdlQ4VDhMWFZYXy1XZFRpeTU5Ylg3UTVoLXhZNlRJN011RGZvR041SVNmTkdnQnNyZVRkTjFQYl84TGVLekRMSjQ4V0xWTjBwOEhibTlydVlBZkxEU2Nodi1kdlEtZUxYRll5Zk1kVXN4a0JXVVplbGFTQ0Nva0dsVTB1V042Y3NpaTM0MjFNSWt0M1loNW5XQm1WMzczd29KWTNUZ0xlM3VBcEpzc1JfTldDOVJzbzhuZUVUYXFYUzhVQkNCcldyX3VXUERxUEpwMFczOHdEamwyUQ?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46078.50972222222</v>
+        <v>46078.66421296296</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Nach Streitigkeit unter Unbekannten - Schaden an Glastür - aschaffenburg.news</t>
+          <t>Federal Ombudsman: 6,000+ regulatory breaches recorded around Brussels Airport in 2025 - Aviation24.be</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>After a dispute between strangers - damage to the glass door - aschaffenburg.news</t>
+          <t>Federal Ombudsman: 6,000+ regulatory breaches recorded around Brussels Airport in 2025 - Aviation24.be</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 12:23:36 GMT</t>
+          <t>Wed, 25 Feb 2026 15:26:22 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOZnI4UW9KcU5SM0ltNnFWakhJeXpvdGgxdHQxMXRyR2RMak9objhiZkY2VUJUSEpvZkZXNHBzNm1zSzE2d2pvN0hFT0ZsbEhXZzN1N1hGMUo1MXhXY3BneVhWbjVMUEdjdnNyZU9WMGlMY2RmVFFzUlNQSW11VVdTcVJXdWduaUw5Q1ktWDY5b0xTcGZFSTh3ZEZxVmVDck1CZnVsRkV2LVYxMEFZUklBTEZwVGt1NEFtb1d0Um93eHI0eVJGVlBjTjFDOHF0QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQQ1RrV1ZyX0pjRUVNV1pJX3dLT0NDX1AwWnJwZkJJSzZjNFdwdWVBRmtXQm11UzhSVXRUUG9tS2FWX0I1bFdKQWpfbzdGc2lNOXpGSHUtNU9pYVZNSHdBQll6Zmg1dlg4Mzd0eDdXdElvZnZ2UGpDQTMxX0NvbHlGeXA3U2ctaFkxeUNqcm0tZDdrek9aUTVPM2VtZ2pPZk9GY1Y4NTN3TV9xVUtqX2k0c0dRM1BkaXlMSUN6cXBYZWhmVDZGOTQxY09MdGNGWjhZZlZoWVVsaVpZbkFo?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46078.51638888889</v>
+        <v>46078.64331018519</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mainfranken: Trotz Warnung – Callcenterbetrüger wieder erfolgreich - Charivari Würzburg</t>
+          <t>TUI fly Amsterdam–Montego Bay flight diverts to Bermuda, and afterwards to Cancun - Aviation24.be</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mainfranken: Despite warnings – call center fraudsters successful again - Charivari Würzburg</t>
+          <t>TUI fly Amsterdam–Montego Bay flight diverts to Bermuda, and afterwards to Cancun - Aviation24.be</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 14:00:00 GMT</t>
+          <t>Wed, 25 Feb 2026 17:09:14 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNZllFZWRoOW5GS1hkdmxITUFlenF6Nm1mYlVob01rN2Q3TEx3emlzRU1GaE0xVWE1UWJ2ZUVzLUlJS21pa3NyMkhVdmhXWWVJUzVLTUlMWEhlaFJjWEthZUJaYy1tYVVsRGhWOEZiWTJodGx3QWVwTGR1WlNkVEZKdkFQYkpOMVdUYTg2bHhCS0tGNmRKX1lKT1RvM1U2QkZfQXMw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQdlhkNkwwOG1xN3BkdWY0S2Y0WkFqZU10SzFfTVc5aXNmdG12WHppZmZUdGJDdnhmSTluQjRObWNvQXYzMFhqNW1SUnIwbE5qRlg4RFZhSm1JMDA5c05XdldMSEpGNzlQNVo4cmxiQXhjUGpzOG1LR1JOeVQtNktqck0tVlZxUXlOaFBxTTBsbzQ1Q3FZem9MaE5saDM4VGFIN3VuRkhDalhfcG13QXVjX1ZWNC13SWx6bG1GbGo5WV9EUkZ1dlFQNHhVTDR0b0dYYjFQS2k2S0ZFWWJrb05hcjFzVQ?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46078.58333333334</v>
+        <v>46078.71474537037</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Überladener Transporter gestoppt – Ladung war gestohlen - Radio Plassenburg</t>
+          <t>Plus d’une vingtaine d’agressions au CPAS de la Ville de Bruxelles : des sanctions sur le RIS envisagées - BruxellesToday</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Overloaded van stopped - load was stolen - Radio Plassenburg</t>
+          <t>More than twenty attacks at the CPAS of the City of Brussels: sanctions on the RIS envisaged - BruxellesToday</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 10:09:00 GMT</t>
+          <t>Wed, 25 Feb 2026 11:32:00 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPZ3BrbkJNUzdNREFLOWt2TDVaUUVQTUVUeFlrR3BjYndnbk9ZUmhyT2lFYk1tNmk1VmQ2SHRLRlFVVnZfUktHZy05RkFScmVFTGRwQm5adEdJYjBHeEhVcmVBQi1aZlBSdkRsR1cyNDhqcWNvVzU2b3hKeDRwNDlINDg4Qm04ZC1lRlZGMW5zMTlsOE1CaDJseVd2SXFGUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxNblV2Mk45V3MtT0hiU0J4cEVLSkk0QVFOOXFRS05TTUVwZVk2NVFmWG9COV9Od001MDcxdzBnTWpydVlnWVFEOUk4MlNOLUMySGJkZFFpM3hPNVZJMExmSXVkVS1mQW0zQ3E0d1pLTjFwMjZ5a0tqQ1RJLVRjc1NrdE55eGVJMDFSMkYyWQ?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46078.42291666667</v>
+        <v>46078.48055555556</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>38-Jähriger nach Öl-Diebstahl auf A3 bei Bessenbach festgenommen - Fränkische Nachrichten</t>
+          <t>Le CPAS de la Ville de Bruxelles a recensé 26 incidents violents en 2025 - BX1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>38-year-old arrested after oil theft on A3 near Bessenbach - Fränkische Nachrichten</t>
+          <t>The CPAS of the City of Brussels recorded 26 violent incidents in 2025 - BX1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:06:00 GMT</t>
+          <t>Wed, 25 Feb 2026 15:36:56 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxPQXdHZDdJdGhkcGZOeFQyZVBhbUY2eTk0YnNvZnlFWkdKZHdYNXR6dW10U0FkZkRpWTViQnVrNFNvVnpoMk9HbkkwbE5uNDZiR3ZEYzVhQkpPODA1Z0N6OHRrRjE4LXY1VlR4WHRlNXJfWmxzWDNQcmxDQXpLWVpTSGU2U05ab2RSTDhJRVpPQ1Y3THA2cm1veVE1Yk05NnhlckdGY1JxZmx5NUpNN3V3Q0I4MHIxZXJaeHVnVmUybXo3OGpvd1pPdWV6QUI3c00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOanBUYWg1T3JISGlCRU9qdlhJNXJjaXpxeVM0RG95eWNGS1NHUHRITDN1dFQyWVJreG9WdEw2OTBndEJQXy1QWXF4Nm0zS0JZRUFRUWprYy13MFRTdlJDdEF4czJ3Y1BfYnpBME14UGU0Rmpyc3I3VER2eU40aDJweDBXODB6VE5wc2JNUFNsekNNNDUzZXl1Q05QWG9HNXpPc24tUnhXUQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46078.37916666667</v>
+        <v>46078.65064814815</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Schöllkrippen: Kabeldiebstahl - aschaffenburg.news</t>
+          <t>Les trams 4 et 10 interrompus brièvement - BruxellesToday</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Schöllkrippen: Cable theft - aschaffenburg.news</t>
+          <t>Trams 4 and 10 briefly interrupted - BruxellesToday</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 12:22:06 GMT</t>
+          <t>Wed, 25 Feb 2026 16:44:02 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNazd0TW0zZ3pRWlFZMl9OS2kyN2VzQ1lOUld0ZlRMMXZGUFo0TEhnS2s4UG5LU0gxRzBrOEJPMVlsOHhSTXl2ZXZXbmk2NUpWSkNpdmVseGVpeUFQWkFaVnpUNEc2MmtNREtZSmtCcVYwakdvc3l1ZVEybE9OZWVJSnVEZ2U4UG1QRmJFQWU5T3VhZlBZRmxJYzdNbkN2RFpWUUc5cXlGTk5DWGtHcVlsaFNn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQZFh5dEZoX2dFSEhWcXNiTThkek9ISEx6SXRJbDJHOWs0VHh0RmVMQmRoblc1NjhzMXBVbE1KR2FFUEFlc3V2UXpJMmlQZDJKN0p1cGF6TlRkcVFHLWU4YVZlWWx5UEt3cGUzNGdDQ3h4eDVGQWtYSkZqc1FCLVJrUkhGTQ?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46078.51534722222</v>
+        <v>46078.69724537037</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mit 2,4 Promille durch Lindach: 33-Jähriger verursacht Unfall und fährt davon - Augsburger Allgemeine</t>
+          <t>18,9°C à Bruxelles: record de chaleur battu pour un 25 février - 7sur7.be</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>With 2.4 per mille through Lindach: 33-year-old causes accident and drives away - Augsburger Allgemeine</t>
+          <t>18.9°C in Brussels: heat record broken for February 25 - 7sur7.be</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 08:56:42 GMT</t>
+          <t>Wed, 25 Feb 2026 13:24:03 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPWVFzbGJzMDlkWXkzaFVmZzMwbzB2aVFpcFd4WFdMdFpfLUJ6OF9wWlg0NmJzOXdQVnd3RmQ4QXFrQ3hpUHl4QlExaWJyQWxkQ3JEZHlRQ0tQUW9vZ2R3ZVJadzJvUjdJZEk1X2ZNLU5DSmViTnd5aGhKbXVWaWRKcm5xQzJuOE1BVFFCUnFvZ1AzeGozWEtZczEyQmtDWUJNbjAyM21Vb2hWNUhMMjB0UFZkek5aWWFwT0VoVHJDTXNZUi12VW1DSFVsYmNMZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNVUxQbFR1U2NjQXJ0bWFIbEx6REd1YlhFZFJ2eVpmQkRveFFZNU5jdWVoUFM4U3FhTl95eXVRMTlYb1lKcEhTNDRGYXoybUZOQ0dhNFZkMHdHdGRYTkNJd0UxbjlxN09KSE80a2FmQ095d0pWczY4TzMwZXBZTjVySEQ2cnYzY3pKMnJYWUwtTEhXQ0ZLUlR4VF8wRFh3cFlTOUE?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46078.37270833334</v>
+        <v>46078.55836805556</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nächtlicher Feuerwehreinsatz im Hotel - RegionalReporter</t>
+          <t>"Un scooter faisait des roues arrière" : un couple s'est fait passer à tabac devant le centre commercial Basilix à Berchem-Sainte-Agathe - BruxellesToday</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Nighttime fire brigade operation in the hotel - RegionalReporter</t>
+          <t>“A scooter was spinning backwards”: a couple was beaten up in front of the Basilix shopping center in Berchem-Sainte-Agathe - BrusselsToday</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:53:21 GMT</t>
+          <t>Wed, 25 Feb 2026 08:06:02 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNOWpPNjE5YUFuc0F6TnJYR1RwMi03Vlk1TTYyM19zTTkzSkF6R2JxcGtNeWpOc0YtM1hwa3JmR1RlQV9Ub0RXMXYwRFBiZS11MDhtalVKNENaQlItQ3RSN05zZklUcDJzLWxsQWVveTd3Q3ZRRTZpaWlsaTFwbm4weGxJLXFjaW5WbEtVOVd2c3dTZjVtSGo2al85c1U4WTNs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQbUtkQ2xUMFo0NUdZR1NDNGdBU2V3bzhURWt4Q2tBSXZib1AzX01ZQmI0V21CbExjZ3M3bTdoekQ4eTJicmpLVVFaanUtN3lDTDRicFpqQ3pPTG1wWi00S1dud09hM3RDSGg4QnJmc1cwTkJIRDVtc3dUbjJZZmFMN1g3Umk0YWt0UnJ3am5RcllkdWJJ?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46078.41204861111</v>
+        <v>46078.33752314815</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Amtsbekannter 25-Jähriger nach Fahrrad-Diebstahl in Ingolstadt verhaftet - Pfaffenhofen Today</t>
+          <t>La CGSP Cheminots dépose un préavis de grève de trois jours sur le rail en mars - 7sur7.be</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Well-known 25-year-old arrested after bicycle theft in Ingolstadt - Pfaffenhofen Today</t>
+          <t>The CGSP Cheminots files a three-day strike notice on the rail in March - 7sur7.be</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 12:29:11 GMT</t>
+          <t>Wed, 25 Feb 2026 14:26:00 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE11TExybWZ1aEs3c0hXekZBWDhLVEIyQTJhUW9zbEw5SVVXODFLLVk3cmdKa1NrZTFHeFJhd1lDbzNCVFVCdFdBNHhLa19mS0xXa2tSRkVMa05CZl9LM2N6RGxwOUwteVNqREk4UV9VaVU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNeTJ0Y1BCeXZpRjlQZmNJWFE3NTRGTWFHUE11U0lpaHVvSElGN0dCd25NX1hONXVPQ2Z0MHI3V1AtemVoRXd1ek0zeXdmTUlWcU9yLVVHV0c0NmYyTlQ0X1JibkJwNzFKTFpGRFU4eWRWXzlrZ3RMSWJuNS1pRHlOVkZ2NnBOR1FRNk9YSlpPUQ?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46078.5202662037</v>
+        <v>46078.60138888889</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Augsburg/Kempten/Lindau/Ingolstadt/Schwaben/Oberbayern - Am Donnerstag, Freitag und Samstag der verg - AD HOC NEWS</t>
+          <t>Politiezone Limburg Regio Hoofdstad ijvert voor eigen TikTokaccount: "Jongeren bereiken in hun eigen leefwereld" - VRT</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Augsburg/Kempten/Lindau/Ingolstadt/Swabia/Upper Bavaria - On Thursday, Friday and Saturday the forg - AD HOC NEWS</t>
+          <t>Police zone Limburg Capital Region is working towards its own TikTok account: "Reaching young people in their own living environment" - VRT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 13:57:49 GMT</t>
+          <t>Thu, 26 Feb 2026 07:37:41 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQYjR2V0ExRkdOVEd3Y3lzZHY0YmhtWTFYUDM5NjNOZC1wODl0Zkx1bUlqSXRBTllWRGVyX2NIV0V4dnUtdHB1Z1RvT3dKSWg4MmtJeTJwSENObVNJbWJWNnpCUjhKdl9HbVZDeWQ0ZGlDYXZvUXd5YU8zSmN0VENnNGtDZmVOak5MamlDZzNDWTRlblpSMElxYWN5cV9XYkdfS2MwalFFdDI2RFIyOTVNUjB2U2lCenZjUHB3SjVB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNai1yalVwN0dOTG1mbU1heHFLTEVLYzhPaDBNVndkd1A3S29YRk5XeGVoTk1wdzNZRTNNX05xa2d3TmtqRVhMbzVoYXFUR3dsaThPNm1Fdll0OFFfNEZqS1VzM0I1dUZBQUR1R0NpbFMxUXNKVmMwRXBFLXBuZWZxNg?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46078.58181712963</v>
+        <v>46079.31783564815</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bekifft auf der Autobahn: Polizei stoppt Autofahrer bei Holledau - Augsburger Allgemeine</t>
+          <t>Minister van Binnenlandse Zaken Quintin (MR) pleit bij bezoek aan politiezone LRH in Hasselt opnieuw voor fusies van zones - VRT</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Stoned on the highway: Police stop drivers near Holledau - Augsburger Allgemeine</t>
+          <t>Minister of the Interior Quintin (MR) again calls for mergers of zones during a visit to the LRH police zone in Hasselt - VRT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 09:11:53 GMT</t>
+          <t>Wed, 25 Feb 2026 17:04:05 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTFVxM1lJN0FVcHFqLTRvNmdZME9mT1lwTVJpWFgzU0dVa0lWMWxrSlNMVzhUSjZCaFd2VlF2MG9CTHlsVUY2QTVGaENQdUFWSm95aWFzQmltUUZWaWs0S2hTS09COGdXOWdpdHBoYUhzQnZKdzJrUFprNWtCNi1IQUtvZnNCY1JuVUxOWUhJa0pKdmFscWFlcWtQWGZfVkNlMXZWNlJIRVdXa1Q3UHpONlhBYzFHVkZyVjFOeQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNbWgyV2ZETTdWd1lWZjA0eEkxU0lud29pV0Q5dWFqdmpTTFVhaWJBTTBJdTJmZmxUc2ZxUUhlcXc3VVR5Vm96b3ZoelVYNGY4OGZ4SUk1ZW05Y0VUeUJEUjNtN1FHb0ozZ2Q4TWxtLS1rUHVTcEF5MG80VVByNW9fN0p0dlU3TlExRTVKREZVRldWR3pTZ1ZpTElZbzNnT1d5Vl9hS0NmcTI?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46078.38325231482</v>
+        <v>46078.71116898148</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Flucht nach Suff-Crash bei Manching: 33-Jähriger hatte mehr als 2,4 Promille - Pfaffenhofen Today</t>
+          <t>Twee auto's branden uit op privéterrein achter huis in Stevoort, oorzaak nog onduidelijk - VRT</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Escape after drinking crash near Manching: 33-year-old had more than 2.4 per mille - Pfaffenhofen Today</t>
+          <t>Two cars burn out on private property behind a house in Stevoort, cause still unclear - VRT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Wed, 25 Feb 2026 11:06:55 GMT</t>
+          <t>Wed, 25 Feb 2026 08:01:15 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9LSFBSM1d2QkVZeEE5clBhSzMtbmhxTVpVejFlXy1WbTFDa2FkSHgxWl9McjRXMnFJeGdhTEFpcXpjQVpVTkpjN3MxMjRsOW5BRkY2dG1yRUhyNVUtRmVzYzNn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPS1ZUaU5WUzRCU0tiM3BRRTYtNXpFSlFSeUs3UjYzMHg1TDhheGJwQk1HMDNBSVNhRXh2aEFOaFZqNnpZdTlJSHRfQm1aVzNlamZ2R0tIM0NycGZVOHoyVmF5TUotM0M0RHd1dTRzTkdDNXlVZTN5UERuZHBFdlNhYUVZSnJGN3NtZHp0YkRUc1drVXViSkRKM3ZCOFc5ak4tNmxPZDh3bw?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,76 +2110,1396 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46078.46313657407</v>
+        <v>46078.33420138889</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Local Town Maasmechelen French</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Après la France, Thibaut Courtois s'attaque à la Belgique : le Diable Rouge va devenir actionnaire d'un club - Walfoot.be</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>After France, Thibaut Courtois attacks Belgium: the Red Devil will become a shareholder of a club - Walfoot.be</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 19:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOd2R4T3hFY1laTzNheVhhYmptRGFyNzdLdG1HNFZNSTRRY016dG03UTJ2MGhoRFZoUmZpdThjem5nNURLaEs4YnVIRV80OEVMd0tEem1vdWVjdVJub1VPMnFIUXRub2dSUVMwYThDcHhJZk1COGtvOUtxb0E5blpIR0JSQ1JLRVNtNERJOC1sNFRua3JGRXZ5WDBqR3ZNWk93aDUteXN1dElNQWZQMC1mUXYxRUlYQ2JsSnpyWEpSVElFN1E4Ry1ldWRZZjZxLTI4OXpBRy1JYVRvMVnSAeABQVVfeXFMTXhOMUR2WkRnOW4xcGVBVl9KZ3U4Y3JLU2lqV096aV94MDgxWUxGcjk1WGdIbDFVdEdZMUVfY1Rka0tUbGR4ZVc1ZDFUQ2xCTFhPUjVCczRrTVdYNHd4VEVXamxDWGNGRnBIay1VM0htT2hWWUc0SWJvLVBNY2ZKdjhIWnQ4UWk4NUhPdEFNbkI4U3ZmZXEyamdpVXQ3NVZQZWt2a0RIUzJEMUhvRG5ETS1NOER2VXUyVnE1M1hIbVFmWHh3T3A1RnpQMWJjb0NSRjNITXdFMzBHY25CcWxWQ3M?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46078.79166666666</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Vrai ou faux. Le député LFI Raphaël Arnault a-t-il été condamné pour avoir protégé une manifestation LGBT ciblée par l'ultradroite ? - Radio France</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>True or false. Was LFI MP Raphaël Arnault convicted for protecting an LGBT demonstration targeted by the ultra-right? - Radio France</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 11:23:03 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPd0hMVEw5NlBKdXdBMlVrWk4xREZZZnU5RmxDUVpwUHJqTndLeWZ5ODV3dUozZndOTDFpLUpBWHJkMjA3Z1p5TVM0TVNzOHBYbURfSnl6NzJSeWdJazJKYko0NW1MVXdKTmo3cVNjYWxYaGZLX2RNZXctVVlGaDhlYWNNc25VQUJWZ2pXZVA3NjdnSkRqMGtLczZOdjRKNzM0aThJeUVzai1fX2E2d1BpdVY4ZHQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46078.47434027777</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Le fisc belge réclame 1,5 milliard d’euros à Nike: le procès s’ouvre jeudi - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Belgian tax authorities demand 1.5 billion euros from Nike: trial opens Thursday - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 05:49:00 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNYWFMblVnV2JUSndYZVA1TjJtcU1FbTJSVlFKMmFRR29KSmd5V1ZVRkI1YVZ3NWdNRlB6Rzl4ZDRPaFJmZ294bW9wLUp3V01DdVVkZmtXTnBzSlMzMGpCWGE0SUM5TmhsNzJkVmduTlJTeFZhTnVId1N2T1paZUc5OG5SRDJyMVdkd0NPbi1iMG5pTnZNS3JJaTMyQTBpTmhNQ2ltV0FlOEtUYTVWTTdycA?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46079.24236111111</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Main-Spessart: Polizei nimmt falsche Spendensammler fest - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Main-Spessart: Police arrest fake fundraisers - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 15:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQTlBoR3NYVDh4bkpwUHhmLXdlcHZpZ0VpLVE4eW1WYTBiajFMMHdhMmF0a2xCcllSb0VrT0d4eUUxVFo3aXh5ck1uQkkzUkl5VzdQQWVxNVNIUXM3U3dqQUl4X3hVQ3dYWFJqYkJjRm1YWFJ1V24wYXVJWTVtQm1ydDNEVEU2bXZBZjVQejBfcktqcE0?oc=5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>46078.625</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Herrmann: Wechsel an der Spitze des Polizeipräsidiums Unterfranken - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Herrmann: Change at the top of the Lower Franconia police headquarters - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 12:29:43 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPblZ5bjRhZmwxUjdVbElESmtfSkxtSmZyZmpKWDc3ekVUTXYwWmRjMVk2aDVGc0FRa0YtcmNudzJVdUNSc3EzSk8zeWhvSGdJTkRTQzA1SDdCbDBGRUZ4RjU5WkpGYXhHb3ZpUUFrVEtrZWJLNkpfM1g5QzhSQTZaeWE2Tmk4cmJNTWxscS1KYkFXMTRrR0hFa3YwcDB1RmtSTl9OM2RsNXZrcnFZdFBZ?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46078.52063657407</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Unterfranken: Mehr Verletzte auf den Straßen 2025 - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Lower Franconia: More injured people on the roads 2025 - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 04:29:00 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOdVBiVzJ1Unh3MlJlYlpITGhBSTgtN3FmcUZFVHVCT3pCRm9kRUp1a0hGYXRlOFpHRmZzRkhlLXotOHJydDRSOENkQUdLa2tRMEMtSUZ1aDVqYlhuY251b2VPWEhHRGp5Qmw2dmVPRklWR2x6bV9xNHpyT1FFRDZ0VkdlVmVXTUUzYWRPVHJjVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46079.18680555555</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Würzburg/Kitzingen: Zahlreiche Anrufe von Betrügern in Mainfranken: Falscher Arzt oder Polizist ruft an - Main-Post</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Würzburg/Kitzingen: Numerous calls from fraudsters in Mainfranken: Fake doctor or police officer calls - Main-Post</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 13:06:09 GMT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxQczVZTXVxaElDRlgtcGl3emlESGNYdFh5LW1fSlFMcmNSZXZNZlBGeEYwOFA3N0pVR1ZLeEpsZ3NpejdXa29VYThvblBRa2xUWWg1T0JWdXE1RkVydERCQ3hqTHlhelpBWU5hREp5U1BGMG5jZlJHYlc3MVJ5R0oyekliUF96Ml8ySFdPYzBjeGl6dUZLZUt3b21FbEdDN1cyQklCc1hHbHFVc1BXWHBnV2ZEaURidlhnV0pMSzBHelRWbHRSOFdna3puWVpuV3QyZ1ppaHpxMTNjVEtZbmZIaGZ5LW9OZi1tS2lYa1JIeE9QVGR3RUtoQXJB?oc=5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>46078.5459375</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Würzburg und Kitzingen: Zahlreiche Fälle von Telefonbetrug - inFranken.de</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Würzburg and Kitzingen: Numerous cases of telephone fraud - inFranken.de</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 12:14:00 GMT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNUnhNMDF3d3l3S0tqeWlNdEJraVlaaXVXSTFBdFFrcUIzNHRXcEYtcFNoLVlVS3BMZzFNY1hjWlQ5b183eGFYdHVrUDhvbG9CWC1HTGhibTlRRXhrMnlLMUlBWFMxY3l6MUpuc3VJdUtkSGh2R2ExOEp1d2hEdUpJX2M0RklFeHVGOVRZUkF6V0lES1Z4Y0s1LTVHb1dXdGp5bVBESVNDcnFaalV5MTJyN01OUW5odldvaGRB0gG7AUFVX3lxTE1SeE0wMXd3eXdLS2p5aU10QmtpWVppdVdJMUF0UWtxQjM0dFdwRi1wU2gtWVVLcExnMU1jWGNaVDlvXzd4YVh0dWtQOG9sb0JYLUdMaGJtOVFFeGsyeUsxSUFYUzFjeXoxSm5zdUl1S2RIaHZHYTE4SnV3aER1SklfYzRGSUV4dUY5VFlSQXpXSURLVnhjSzUtNUdvV1d0anltUERJU0NycVpqVXkxMnI3TU5Rbmh2V29oZEE?oc=5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>46078.50972222222</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mainfranken: Trotz Warnung – Callcenterbetrüger wieder erfolgreich - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Mainfranken: Despite warnings – call center fraudsters successful again - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 14:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNZllFZWRoOW5GS1hkdmxITUFlenF6Nm1mYlVob01rN2Q3TEx3emlzRU1GaE0xVWE1UWJ2ZUVzLUlJS21pa3NyMkhVdmhXWWVJUzVLTUlMWEhlaFJjWEthZUJaYy1tYVVsRGhWOEZiWTJodGx3QWVwTGR1WlNkVEZKdkFQYkpOMVdUYTg2bHhCS0tGNmRKX1lKT1RvM1U2QkZfQXMw?oc=5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>46078.58333333334</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Aschaffenburg: Schleierfahndung deckt mutmaßlichen Einbruchsdiebstahl auf - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Aschaffenburg: Veil manhunt uncovers suspected burglary - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 16:14:47 GMT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxNMVZ1dmtOc0hzMVJjWkIwV3ZvQ3dudHBncUZ1a2tSNjd4RGpjWEVXX0FVWWhHUDM4N21ub0s5NXZRcDBlMkZYdV9mNDNGT0hlbnd1bXoxeUo1UGx4UThmRUp1Vy14ZEpxeFBYNk5ocXM1NS1STXk2ZDRUSGFTUGFSNENtMUJJMFFQUW5QTDdGWlViWjMxR0hrVDV2UlVaWHRTYWRZN0lXeUlGRVRETEF4alBBRzEyTVk3TVM4?oc=5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>46078.67693287037</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Nach Streitigkeit unter Unbekannten - Schaden an Glastür - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>After a dispute between strangers - damage to the glass door - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 12:23:36 GMT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxOZnI4UW9KcU5SM0ltNnFWakhJeXpvdGgxdHQxMXRyR2RMak9objhiZkY2VUJUSEpvZkZXNHBzNm1zSzE2d2pvN0hFT0ZsbEhXZzN1N1hGMUo1MXhXY3BneVhWbjVMUEdjdnNyZU9WMGlMY2RmVFFzUlNQSW11VVdTcVJXdWduaUw5Q1ktWDY5b0xTcGZFSTh3ZEZxVmVDck1CZnVsRkV2LVYxMEFZUklBTEZwVGt1NEFtb1d0Um93eHI0eVJGVlBjTjFDOHF0QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>46078.51638888889</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>'What excellence looks like': FSU trustees extend president's contract - Tallahassee Democrat</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>'What excellence looks like': FSU trustees extend president's contract - Tallahassee Democrat</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 20:54:00 GMT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQRlhsRjR3dXRfZ3ZhazdmX1FpVjZLbEJMdEdrZmNBVW05REpfNjBvR1JRb3dLUkVMNDlfekdzbkFEOWp4QVZIQ3A3eVV6cFNVb1Z4NTlMRWRDTUcycjQ2SDc3bU1KVDJMbkhSSHV3WmFvZUJ5ZVp6SnlNN2JIa210MHFkZW4weUVLM3J4aGViNXJiczVqNVlHWEw4aGkydXlBTlFnQ1BwMWNyU1YwM0hWUmFFejhjcjM3UlUwRGhXSk1VckduWlNtRFg2SmIxSXRodGZWMw?oc=5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>46078.87083333333</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Jon Wertheim says Serena’s unfinished business at Wimbledon fuels speculation - Tennis Tonic</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Jon Wertheim says Serena’s unfinished business at Wimbledon fuels speculation - Tennis Tonic</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 19:15:51 GMT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOMjVOSGZuWVNUbzFTN0JLUWJaZVp0b2lzYnQwVkIzNFVHV1psZ2l2VXFRTEdlWXZ1ek1BYVpUMnA0dDlKMGVTTDZGRXNUVUhGekFTRExEelpJVHBIZ3d1TVN0Y2V5M1JwenBqUHVuc0NqY2dMaUFURmZrQmNxQUJnVGVTZ1BRSTk5cGZWY2FVU1hGcUx3bDVrZXc5OFdhcGdjaG91OHRvNzJGRzhKbks2bGZ2VUhSWjdRTlY1Qw?oc=5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>46078.80267361111</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Local Town Ingolstadt German</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Bekifft auf der Autobahn: Polizei stoppt Autofahrer bei Holledau - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Stoned on the highway: Police stop drivers near Holledau - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 09:11:53 GMT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTFVxM1lJN0FVcHFqLTRvNmdZME9mT1lwTVJpWFgzU0dVa0lWMWxrSlNMVzhUSjZCaFd2VlF2MG9CTHlsVUY2QTVGaENQdUFWSm95aWFzQmltUUZWaWs0S2hTS09COGdXOWdpdHBoYUhzQnZKdzJrUFprNWtCNi1IQUtvZnNCY1JuVUxOWUhJa0pKdmFscWFlcWtQWGZfVkNlMXZWNlJIRVdXa1Q3UHpONlhBYzFHVkZyVjFOeQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>46078.38325231482</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Mit 2,4 Promille durch Lindach: 33-Jähriger verursacht Unfall und fährt davon - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>With 2.4 per mille through Lindach: 33-year-old causes accident and drives away - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 08:56:42 GMT</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPWVFzbGJzMDlkWXkzaFVmZzMwbzB2aVFpcFd4WFdMdFpfLUJ6OF9wWlg0NmJzOXdQVnd3RmQ4QXFrQ3hpUHl4QlExaWJyQWxkQ3JEZHlRQ0tQUW9vZ2R3ZVJadzJvUjdJZEk1X2ZNLU5DSmViTnd5aGhKbXVWaWRKcm5xQzJuOE1BVFFCUnFvZ1AzeGozWEtZczEyQmtDWUJNbjAyM21Vb2hWNUhMMjB0UFZkek5aWWFwT0VoVHJDTXNZUi12VW1DSFVsYmNMZw?oc=5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>46078.37270833334</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Augsburg/Kempten/Lindau/Ingolstadt/Schwaben/Oberbayern - Am Donnerstag, Freitag und Samstag der verg - AD HOC NEWS</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Augsburg/Kempten/Lindau/Ingolstadt/Swabia/Upper Bavaria - On Thursday, Friday and Saturday the forg - AD HOC NEWS</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 13:57:49 GMT</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQYjR2V0ExRkdOVEd3Y3lzZHY0YmhtWTFYUDM5NjNOZC1wODl0Zkx1bUlqSXRBTllWRGVyX2NIV0V4dnUtdHB1Z1RvT3dKSWg4MmtJeTJwSENObVNJbWJWNnpCUjhKdl9HbVZDeWQ0ZGlDYXZvUXd5YU8zSmN0VENnNGtDZmVOak5MamlDZzNDWTRlblpSMElxYWN5cV9XYkdfS2MwalFFdDI2RFIyOTVNUjB2U2lCenZjUHB3SjVB?oc=5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="n">
+        <v>46078.58181712963</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Mann klaut Mountainbike – nun sitzt er im Gefängnis - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Man steals mountain bike - now he's in prison - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Thu, 26 Feb 2026 07:11:33 GMT</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQdG9hTURrQkdSQzRveWFBV25xTlFHSEQtenktcG5YbFpqcFc3Mm5MUnA5WHNNTS1nNU91TGNxWkhoZzV6S09wSHlXUmU1Vk53RmlhSkNFR2tBY3ZTYVZjM3JVUTREX0REb0QwT2RGMjdFUF9GNXByNnJ6VkdDZDZ0d09NNlBtd3NlcWtEelNYWG0wMlYwa0VWTnpYS3ZMVEY5SXAyR1dxNEdLQ3EzSnhycUwwNA?oc=5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="n">
+        <v>46079.2996875</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
         <is>
           <t>Illegales Fischen am Kapellbuck: Polizei Eichstätt sucht Zeugen - Augsburger Allgemeine</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Illegal fishing on the Kapellbuck: Eichstätt police are looking for witnesses - Augsburger Allgemeine</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Wed, 25 Feb 2026 13:13:05 GMT</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPYWZORTQxZWRJZTJtS0tIRGVmanhNMkcwWmhJMDNTWTFjeVViWXBTRmsyY25HRGx3dHQtSGxET3hFN0hBVElXU3VJdk5wOFoxaWtlSXBzbkV5eG9jYUh3T0NIaEF2SE5VdkdLT3pvdVJrVFVHYVcxN3I1UjJrR05hLXJWNUpNNndCRXF4Njlma3duNVQya0UtTV9GTGQxWGVnT2c4Vjd3R2p4VExvZjRNUlQ5YkxBWUhvZGc?oc=5</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>DE:de</t>
         </is>
       </c>
-      <c r="K32" s="1" t="n">
+      <c r="K49" s="1" t="n">
         <v>46078.55075231481</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Granit Stein set for WBA Continental super-middleweight title fight in May - British Boxing News</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Granit Stein set for WBA Continental super-middleweight title fight in May - British Boxing News</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 18:36:29 GMT</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9lZ2ctMEFpRDZMTmthLVZSajRYal91QW5sM0xTVXhKU3otd2lyZDQ4U3V5SXJwbXpZd3d3Sk1wSnAyRDlaVkJXMjNzSkIxQXZkcV9fMDNKOG8xYmNOR0E4Qkd0Z2VsdkdjNFNoRGMtTTFfNGZXbk5vcVduSE0?oc=5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>46078.77533564815</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>German regulator spots competitive broadband markets in Munich, Cologne, Ingolstadt and Wolfsburg - Telecompaper</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>German regulator spots competitive broadband markets in Munich, Cologne, Ingolstadt and Wolfsburg - Telecompaper</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 14:32:36 GMT</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQdXl6S25JZHZnbmNhYTdUZGp1ZWdDejB4bnQ3T19lUHBNNHhNeWl6Z09BNVRlMGlha0NfZ1IzSGhXN0h5dGRYM1VUbEdWQXdBdVUteFdZdVRGTFRPTjUzSzRqdUN0RkNxRGg1cVlTeTBEclBIZ3JVU0I5Yk8zRGJMR3BVTUJZZnJtMlBwRjBlemkzLS1BMklNVDJaSlFEVnVTSzE5X0FhcWN0cWlDdWNjNEV5Y1NUaF9wRThkX1YyOHNPZUNvelBmOVpVSTZfaFFXVk9vTg?oc=5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>46078.60597222222</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Naas Book Club welcomes renowned Irish author to celebrate International Women’s Day - Ireland Live</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Naas Book Club welcomes renowned Irish author to celebrate International Women’s Day - Ireland Live</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 18:35:15 GMT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOTzZhUFpjUjNqTWRfNnhqcmR6MjJ2RGprVHVoX05QZE9SaHUxUmJib3R2cElHcUJpZmpDcEUzbXowYW9fUGRuTmpHV3ZHSWY2dDM3dU1ycEY3QXlmM3NpdXpXNHc3RG0wVmtWUmJOM2VKYzR6dGZFS2xjZlVEc21zbTBDYkZ0RHpYZVRxdms2N2tkRk1EbXg1LUJrcTNDQjFqWE9oYVM3UzBsRGYtUzFFQTZSMXJrTnhjSHdYeFVlYU53M2FHeGthbzFxUVJ2LTEwMUY4dFpTc1c?oc=5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>46078.77447916667</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>3,200 people per GP in Kildare 'unsustainable' - TD - Ireland Live</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>3,200 people per GP in Kildare 'unsustainable' - TD - Ireland Live</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 21:40:38 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPd09GbXg4WGJMWXRLTnRudjgxVVlMcEhtcGt3a0h3WHhoMktNQnRPNDc0ckVwdjFYOGdHWnB4UVk0eUMyYmM2Q3ZpWXpIeUxVWDItWVZKbjZyMFl0SUhHUG1feWY3TWtscHk4NERHQnBhMWNPRG9OcVhlcjh0VGJvT0VndDVZTUR1WmZTVTZQZ252NVBBRVFxcDZsTTRWUnMtazdWMTBDQlY?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46078.90321759259</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Steal Her Style: Karen Koster's chic Sandro sundress as she reunites with Alan Hughes - MSN</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Steal Her Style: Karen Koster's chic Sandro sundress as she reunites with Alan Hughes - MSN</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 09:35:11 GMT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7wJBVV95cUxORGlaU2xKMmxhdmZVS2EyNk9odjNmQ2NNUmQtY3ZhWW1RODN1N1AyS0xZZzVGWVlud1kzOUJ1RzQzZnVTcmRDMlY5Q0hUNEp2aldieUV4U1dQMHIwUGtnVndLV1lDY3VkUWtjNFZvVEFKbURFdHNRMjNTVWtSRHFvUmlaSXdYeWZWdmlGVDFMdDhZcjRqUXRzdEtqNTF6ZWxiYXRpclhnYzRwVUQ2Sm5xUFcxYlhNUktLU2JrZDZkNE5MVWJudjVyVVQtN09WTHMzNFBFSC1LRXZ0NzFmV2tibWctazVVX1c2RS1HemJNb3pteDFEa2Q4RWtDUks3TTBWUkJmN1A5dnJ4MWRhcGxObWtLSzZHTEw3d1UzV0M5NWp5cTNPY1JKdTdnQVJGRlB4T2xzVktIN0UtVU9uaDBnUGRldm12YjQ0elh5UzM3cXpZYjJqY0M4clVlM3VEdXdKQXhJdkNKblluQ0hHZEgw?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="n">
+        <v>46078.39943287037</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>High Level City UK Ireland</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("London" OR "Dublin") AND ("terror" OR "bomb threat" OR "suspicious package" OR "police operation" OR "counter terrorism" OR "stabbing attack" OR "shooting incident") AND -"bomb squad" AND -film AND -movie AND -filming AND -"New London" AND -Connecticut</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>What are school officials instructed to do (and not do) amid a bomb threat? - London Free Press</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>What are school officials instructed to do (and not do) amid a bomb threat? - London Free Press</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 19:49:14 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNbXc2MTViTVZjQUpDd1FxVy16MXdnZ2NjV1ZEYkQ5VDd4YTVLMWFob09SeS1fT3Z6a3lDb3pQajI5NWJ0c2I3VGVTbGZnTUZfREMzNnpfY3I3RGhndktPaG54YW5tNXotclI3VTZER3VjTVlod3ZUMElveUpLNlVMOERmZXVuRGF5YkFDMWxwdHhOU3B3MHg0eHloYlpQSGxi?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46078.82585648148</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Local Town Fidenza English</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Fidenza outlet" OR "Designer Outlet Fidenza" OR "Fidenza Village" OR "Parma" OR "Piacenza" OR "Cremona") AND (protest OR bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR evacuation OR "police operation") AND -football AND -transfer</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Man shot, killed by Parma police identified - FOX 8 News</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Man shot, killed by Parma police identified - FOX 8 News</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Wed, 25 Feb 2026 14:49:58 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBES0ZWdG1QWXpjTVVqVVRoNGdzN1lDWXhRQ1pPX2lMdW1WdFhnSklSZUlGQmV1ck9KUXA1Y05NYUdjSmFDd2sxYl84aG9DZmw1elowS3BQNklmV0VQY2g0dHNtVEtDS0ZJVlhkSDU1UXpYVzDSAXhBVV95cUxPUGZsdmZUNUNlS3hJQ3JsdzVHc2VZQXRULXY4TlUyV0dqYmVMLTZFT0NpQ1pWX2NHc09tOGpyVDVIb0JaelI5N1ljb2gxZG5KOHpybTVyUGpvVVRWdlItQ0dBX0NNZnBfUGpYS1Q0anRWQUs5WEgwWTM?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46078.61803240741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-28 07:37 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Brand Protest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lululemon founder Wilson ramps up pressure on board amid proxy fight - Reuters</t>
+          <t>Demna debuts with body con Gucci in Roman temple - FashionNetwork USA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Lululemon founder Wilson ramps up pressure on board amid proxy fight - Reuters</t>
+          <t>Demna debuts with body con Gucci in Roman temple - FashionNetwork USA</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 13:15:13 GMT</t>
+          <t>Fri, 27 Feb 2026 16:44:30 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxOQW1JMEhQWXZMSVhwSDRsNFRuTUhoUm1idnJFTjdhV0xMamRZTWV5S1MtRFF0U2RDUjVEM1lmV0ItSkowSFNydTlFbUdlN016bnpvMDJTRE1NTTdTNlNqQXYzQmFpYmFEbmNKcDVDeHhjSGdKLWtJR29WSFFOdW00UU9sSjdwQnZJbF9XdEFjWmNsdXdraVN1LW5CbnZQUVpDakdNOGdqc09XYXFxTVlfbnhPSk1JV0ZScm5QdGNXUUZudVNxOGV3YlVUSGpJRVJMcUhjZExFNmJvOWxHclVXS0tDdGtUWVVudHJaUzA5dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNSjEyV25FYkdjQldydExXQXR3VkJ1allCT0NkSDRTMURkSWVIMTZ5amZqQVVja1NvTFlucEMwNnRhUlNZVWRXTTNfTlZITS1TNW8tSERRRWZoYWpiVk9ULUJkU1A0UGh5NzlZeUgxRnhIN3JoNW55bFdMUmF4M0V5NG5kMmNybWo4YTQ4dHhocUlvaXpHQWNQdGNZS0k?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46080.5522337963</v>
+        <v>46080.69756944444</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Twee jongeren gearresteerd na drugsactie: “Cocaïne, geld en gsm-toestellen in beslag” - HLN</t>
+          <t>B&amp;M European Value Retail S A : Inside Information / Ad Hoc Information - B&amp;M EUROPEAN VALUE RETAIL S.A. - marketscreener.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Two young people arrested after drug action: “Cocaine, money and mobile phone devices seized” - HLN</t>
+          <t>B&amp;M European Value Retail S A : Inside Information / Ad Hoc Information - B&amp;M EUROPEAN VALUE RETAIL S.A. - marketscreener.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 09:07:19 GMT</t>
+          <t>Fri, 27 Feb 2026 17:03:11 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPbUg2N2ZHT1M3THRKTHA2LU1MbDkxRG01Y2pDSm4xVURHMl9tR2FsbExMdEQyRW1OcEhRRzlXRWEyUTVEN21IRUZfZzNhOHNCWDA4OVlWY2JIc2k2eEVwWGloRF9QYkFzWm9kRzdaSldSQk0tMzUxSHR2MWFUeDE4M3pCTndHcWJQeHAtWExpeEV0MUZ6QkVrVEFYZUowbk9RUGF3bDBxNDY4V3hsUkptQkdrWW8xc0RNLTJSdA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxPNGMxSFIzZjFJLUVqRWpwSkFqdUgzeHZWOWlfblZMVU1wMFlXTjMyTm01Z0NDV1lMajV1cTFlMi01QmktV2FZd0NqdHU5djNrQTNGcUllZE1DS0ViaGFnS3RSdkZyRTZ5VU11Yk50QmNUY1AtTmFjNHE0NHp0ZDRlLXFqeW9hRHBwanhuTF9tY2FBQ0FCTWFMTU5iUGV2b01aTGFwY05qSTk3cENjSjhaQzZ4bDB2bWl2NV95eG9JRk12ZVdmLW1GSktpUUNvZFpYVTB5M1A4UkRvRzllLUFZ?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46080.38008101852</v>
+        <v>46080.71054398148</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Justitie wil ‘terreurambtenaar’ van provincie Limburg langer vasthouden, rechtbank stuurt Maastrichtse verdachte naar huis - De Limburger</t>
+          <t>B&amp;M Completes Jersey Migration and Prepares London Listing of New Shares - TipRanks</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Justice wants to detain 'terror official' from the province of Limburg longer, court sends Maastricht suspect home - De Limburger</t>
+          <t>B&amp;M Completes Jersey Migration and Prepares London Listing of New Shares - TipRanks</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 13:03:20 GMT</t>
+          <t>Fri, 27 Feb 2026 16:59:50 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPSXh3aHJsRzRjWko1SS1JUnB0Ym1fQTBRelIxZ2pjcjlENFB0V09jVzRGckJia3p2WGNReXFNajFZWTRuUF9KdElUdUtkTnJsOWtEZ3M2MzhOcThkLWJfOVJfdi03TFlKQTNqR0dDUE11b0k1WnppbW1kUFJnOGhyeURyN2RfZTZWdjZYb2ZYaWNTNHNmcGhzS0FqWUhWVTcxU2VfQ2l2QzdHZDl4MUVoMzdKN3JpSWRjcGt4bFdQZjVIdFlLWVBTbmFBQVJYTDAzY1BORmNSRmRrRGNWX3hxMG5NaHVhR1BUNFVRRGc5NjNYVDhIM05QQnp4NmFDeDhZV1lqbG5DMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNZEdFSFRreEduaWlhTEhiLThKM2QxdC1wTjVVYWFCNjhEcWphd2IxR0RDT2NJdEhpbl9UUnNXTGpvN0lEaFExeW9ZMzVad3FScmVGYVVZRTJfZ01RSmFxQjM5NFM3SXhRT3NSVktrRmlNRTVuSFhtTjN2QUR6TDB5cjNrbnNNWEVBTnJwSWdMWF8xTWRMWnVweHN5SGxYdzZBQVkydFFOdVBMVFlnYnRFM0tRVVZyY1Exc1RrLWx0OUo?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46080.54398148148</v>
+        <v>46080.70821759259</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Brussel laat Mercosur-deal ingaan, ondanks verzet van het Parlement - Het Financieele Dagblad</t>
+          <t>Promoter pares 14% stake in Vishal Mega Mart; HDFC MF, Govt of Singapore among 3 investors pick up over 6% shares - TradingView</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Brussels allows Mercosur deal to take effect, despite opposition from Parliament - Het Financieele Dagblad</t>
+          <t>Promoter pares 14% stake in Vishal Mega Mart; HDFC MF, Govt of Singapore among 3 investors pick up over 6% shares - TradingView</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 11:22:40 GMT</t>
+          <t>Fri, 27 Feb 2026 15:13:14 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQYlpwQ2JtcURVTkVOYVR1Skh1b3VKUDYwTkFsZGxJck9kS2pIU1VQdE55OURUblAzamdrbENJNDMtYnVGRURuOFdsd2NCLXNobVZQaVN4Yk9GcGNlLVhTMUMzRlhnU1lfS19YVjRxdzY3d18wWmhaVVpOOThhT2JfVHM5Q0hqVzhFdmQ3dWJzV2YzX0VON0gzUVEwNGZmdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxPTlNtUkNVUm5RS3czMkhjT2FNbVA1dXpRU3pVVTd1WnBmcHlkcUtxQVBYV2FmNEI3MzNLdVlNOHQyMUtFY0gzRkhTWXA0cVhnWjZteTRsNm9fU3VSUnVja3UyZTNaU1hjaTB2UGJheENtYjdscFJaSXA0VDlxcFk5QTQ1NkpDV1JiWVFvME9sclNyZVpwUUp2cTUtSHVvWk5OTXhEOW03d1dEVXlsLV9DV2RMWlo1U0JoSXlCb0FzcjN1U2xxZ2RRRTgtTVRKaFR2UkZtOXlSb2hpcGRvS1ZSUTNfMVdHZldheWNrdDkzaVlvUVRtNmE0aTk3eFFDX0NDSlE?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46080.47407407407</v>
+        <v>46080.63418981482</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Brussel laat Mercosur-handelsverdrag ingaan en wacht niet op handtekening Europarlement - De Telegraaf</t>
+          <t>Lululemon founder Wilson ramps up pressure on board amid proxy fight - Reuters</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Brussels allows Mercosur trade agreement to enter into force and does not wait for European Parliament signature - De Telegraaf</t>
+          <t>Lululemon founder Wilson ramps up pressure on board amid proxy fight - Reuters</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 12:16:46 GMT</t>
+          <t>Fri, 27 Feb 2026 13:15:13 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQYld5NGlfWXlJa1lwcXZZMkJ5UEZYS3hxdXpPZktrSlNjeUZJRHJ2T0JjRWplWFdJajY4RDQtUGpoZl9zSzh6YWwzR193ZXkxMVRsc0JmSDRHUmtmQVd6VThqdGVOSWFwdW5jUWtTT3NyR25zV1luRkh4UW9ZTjd5MXJBSWdubHFRNXQxLVh1S2h1YldNVHZ3aE1sNlVqRE1yNGZEYWZuUHcwTnhPUHRYN0lHLVlIc0k0aUh2TnZodWxWaXVQbWNCN05saWVDUkk5MU9KbQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxOQW1JMEhQWXZMSVhwSDRsNFRuTUhoUm1idnJFTjdhV0xMamRZTWV5S1MtRFF0U2RDUjVEM1lmV0ItSkowSFNydTlFbUdlN016bnpvMDJTRE1NTTdTNlNqQXYzQmFpYmFEbmNKcDVDeHhjSGdKLWtJR29WSFFOdW00UU9sSjdwQnZJbF9XdEFjWmNsdXdraVN1LW5CbnZQUVpDakdNOGdqc09XYXFxTVlfbnhPSk1JV0ZScm5QdGNXUUZudVNxOGV3YlVUSGpJRVJMcUhjZExFNmJvOWxHclVXS0tDdGtUWVVudHJaUzA5dw?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46080.51164351852</v>
+        <v>46080.5522337963</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Zo liep het negentiende seizoen van Flikken Maastricht af - Televizier.nl</t>
+          <t>'We're crowdfunding to stay open and are humbled by the response' The Duck On The Pond's Hendrik and Julie on keeping afloat and being proactive! - Ox In A Box</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>This is how the nineteenth season of Flikken Maastricht ended - Televizier.nl</t>
+          <t>'We're crowdfunding to stay open and are humbled by the response' The Duck On The Pond's Hendrik and Julie on keeping afloat and being proactive! - Ox In A Box</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 09:08:02 GMT</t>
+          <t>Fri, 27 Feb 2026 14:59:25 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNaGpEXzZDcDMwQUdxM1VpN0M4dWVXUjhGN3cxNGpJa0NkU0R2Rkw0LUVIRzlYLVlpZXY3Wk9TZWhQdXo0cVBtaVUzNzhyNFlzZXhfdDIxN1NWMlRraWtRcXpnYWJMeVp3TjlycHlocmMwRGlWa3QwWkJybkh5eHZaczk5em5GY1k0bGI4anNWQ3NQaVpXY3NLYjRFd3d1QnVI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOOVBBX1UyTU9oQ3pFdHdya2xyZ2ZfYmhDVXNMMDJncnUxYU8zVmQ2NEhYNnN1dlZCZndUMDZsWnNXZmNuOGI1aFhkVHNGUWtVQjQwOEdlWnJMQ25sOTdYRXBSdHZGY2hZOV9TaldwWUh3Mm9YOTFtNUpqeHdua1hkSm9zNHNaTnRWM25iOWFfLWhHU0Jjd0dLZDF2T1BzOG52RXF5QmhwSXZiSFRLdGdzbVVBN3ZUMldZRUlWMWRqekRYMTRBdG1BTURNOWlwMXFuMW10cTFGSlNxUVMzdGUxWU1nd3lRQlM1VTFxUllJZDNHSzhhRUEw?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46080.38057870371</v>
+        <v>46080.62459490741</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>XR JSO Village Search</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Extinction Rebellion" OR "Just Stop Oil" OR "climate protest" OR "environmental protest") AND ("Ingolstadt" OR "Kildare" OR "Vallee" OR "Bicester" OR "Wertheim" OR "Las Rozas" OR "La Roca" OR "Fidenza" OR "Maasmechelen")</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Onboarding in Automotive: met nieuwe cursus in één dag klaargestoomd voor baan in de autobranche - Automotive Online</t>
+          <t>Winston Churchill statue daubed with graffiti calling him ‘Zionist war criminal’ - Bicester Advertiser</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Onboarding in Automotive: prepared for a job in the automotive industry in one day with a new course - Automotive Online</t>
+          <t>Winston Churchill statue daubed with graffiti calling him ‘Zionist war criminal’ - Bicester Advertiser</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 09:01:34 GMT</t>
+          <t>Fri, 27 Feb 2026 13:01:46 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOZzJCSkFmOUxMeXVlTFBxU3VEMmtGdmt1Y0VXczh3VlZiS0VhUW1JYlRrSkFCN0Z6czF0QXprUEw1aFlLZWlKNjZfU1NfNlB5UEVxU2YzemtIM0QySjR1cDNQNUVQbEwxbmtXT1ZCVUhOdlNnNXFZUUxxNzM5elktREhzOGh3b2RaTTV4azl4NTQ4S1FHM2ZwTUszRkNnOWJHMHIxM2VmSkJEb0NnUVZERko1Y1J0ckdWbko5aVBSYkwtcG5namdpYXJ0ZnhQVHNwU2xlenQ1em52NEJPSjVEdGVrZ0dVWmFKd3kwcnlHWGpLbUFS?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQV2k2eHhuOGstTm1DWElsejVQdjhfQjJOZUF5YmVPM3F6OXhHNklFbmwweF9wZVlvempUc3pNU2c3QWhiem05ZEFBeldIUklUdlN6LUR4UzdpYUxEa081UC1jaHlJSXhTU3d3MWxyM0lQLWdoMjNLa1p0TFpoMkJOSHN3R1ZsU0VjSzZWTmwwa29JekZIczVnNHIyaWdwdExIUlFoc3Z0WnFiMTN4SjhpUGdPbi1TRXRiajhzTV9VaGdmV1R6VFo0?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46080.37608796296</v>
+        <v>46080.54289351852</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Brussels orders probe of Mandelson's Epstein ties while EU trade rep - Yakima Herald-Republic</t>
+          <t>Organisatie Kuurne-Brussel-Kuurne treft laatste voorbereidingen - Focus en WTV</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Brussels orders probe of Mandelson's Epstein ties while EU trade rep - Yakima Herald-Republic</t>
+          <t>Organization Kuurne-Brussels-Kuurne is making final preparations - Focus and WTV</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 10:19:46 GMT</t>
+          <t>Fri, 27 Feb 2026 16:12:22 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxQOTkxQkkzaTA4TGF0U3o1Tmp1dEJpWnZKVDNuaGFFRldZRXdwT0VYLVpZNlpGVEtmbmJXaDRCSkNzNmhNTk91eGt6bTJNbEl3NDl3QzRhQ2Fsdk14QkR1U1VRT0J2RDBMZFZGRGptZ3BqOWpETDhhRVVWai1VRjVBVWJaQ2diOFhqSVhnOTFfNHlVcEwtOTBhSGpWdjluR0tpT0liTnkzc0JYMWxpX0s4UWNvd0JsNl9uNWlDSEdXMTY2NVJ4c1dsazFBU2lQODg3cWJfYk4wYnlVYy11MHFfbE9KUGdTLUdwSVNLN3hjcF9BZ2FUbFg1MUtSRUZzMlhIRERMQtIBigJBVV95cUxPemJzLWRsMnIyNDY3c3JnOEZxT1ZFV3ZjMzRaTkxIS0dkY1Nua0Vvd1QwQnRsZW9pZUdTQWZjaHBiemJwNGJsSlhaMHFKQ0tWMjlMQUdxUkhsaVdNanZ0UW41Rnh5NGotNVpTUG1ISXdYZjN2cEttX0hZZ0ZlUjdNVlFyc1k2STJCUG5OOVI0M0xQa0RlaWgzdUtvSGhmcHplV1daWkNfT2NmNWs3OHBfbUNpakRtWGV4c1BGN293MkZXVERQcjVfMWxLdnhMcWp3NnhPTFVHYjhLUFRsaTZiQk5FZG1wQVF3d1V5c0tUX2FVNnlwM3JESW4xX1VfUlYzaDVaUTRlam1ZQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNeFhLZFBtdmU5d2NBRS1ZV0d0QV9XZDIwUGpGQlYzT0c3a1NjR1IzaGxKeXc1aXM1Yy1zTFhqazNTS25pay1OdmNVV01QbS1ZMnFpcGVYZDRRbDRNbzZLLXhjMnFCRy1VMEhjdERuNFBfc29BM0w2OGxrX0tCcUc0ZXhXemFXc1hlMy10TVZHVDRUTHRQ?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46080.43039351852</v>
+        <v>46080.67525462963</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Plus de 1.200 condamnations, 224 millions d’euros saisis: l’impressionnant bilan du dossier Sky ECC - 7sur7.be</t>
+          <t>Brussel laat Mercosur-handelsverdrag ingaan en wacht niet op handtekening Europarlement - De Telegraaf</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>More than 1,200 convictions, 224 million euros seized: the impressive results of the Sky ECC case - 7sur7.be</t>
+          <t>Brussels allows Mercosur trade agreement to enter into force and does not wait for European Parliament signature - De Telegraaf</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 11:33:00 GMT</t>
+          <t>Fri, 27 Feb 2026 20:06:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOVkdlQ1ZzWlY4UEhKbWo2M3FMSHFyaG11LUFXbXFEQmdpbDVOT0NJbVNCdnlRa1hkbkdVQ2JNd0FHZTVUY1VFZF94WWdwcEtJU1FjVko2TVI3TGc2YnNxa2tNeklKQlhUQ2Q3Nkp0ZTRaZ0RvZDhwWENPVUNGRWRldWRPaXcwbnJxZEpXekUyYVJDVnZQQlhpSEhvcW5sVDNXRzViY19FLUFzV2U1UHdjUVV5UGFEQkxnZV9tbWtkQXdlRkNOdV84QVVTNUR2WjdkSExzNHVR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQYld5NGlfWXlJa1lwcXZZMkJ5UEZYS3hxdXpPZktrSlNjeUZJRHJ2T0JjRWplWFdJajY4RDQtUGpoZl9zSzh6YWwzR193ZXkxMVRsc0JmSDRHUmtmQVd6VThqdGVOSWFwdW5jUWtTT3NyR25zV1luRkh4UW9ZTjd5MXJBSWdubHFRNXQxLVh1S2h1YldNVHZ3aE1sNlVqRE1yNGZEYWZuUHcwTnhPUHRYN0lHLVlIc0k0aUh2TnZodWxWaXVQbWNCN05saWVDUkk5MU9KbQ?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46080.48125</v>
+        <v>46080.8375</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Buurtbewoner die mollen wil verjagen met gasgeurmiddel zorgt voor evacuatie van school door sterke geurhinder - VRT</t>
+          <t>Twee jongeren gearresteerd na drugsactie: “Cocaïne, geld en gsm-toestellen in beslag” - HLN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Local resident who wants to chase away moles with gas odorant causes evacuation from school due to strong odor nuisance - VRT</t>
+          <t>Two young people arrested after drug action: “Cocaine, money and mobile phone devices seized” - HLN</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 11:31:23 GMT</t>
+          <t>Fri, 27 Feb 2026 09:07:19 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNQk1IcU50a1AyNGxpaTFGWmFqZ3RkbFJURjZISHcwYlRlWEg3amRkRWU0TEFQVDJGeWsxQTZZeG5nVkQ4RHItRmVhSjhaQWc4eDQ0VDkyZzdBM0syYm5IVklnYlF4N1NFRXg0aEhvcTRZY1dCSHNZMTd2UlNDMDVFMF9WSWplb0k3WjJOakNEUDJ1QnB4Y1FsVlptcUxmS3dUQXk0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPbUg2N2ZHT1M3THRKTHA2LU1MbDkxRG01Y2pDSm4xVURHMl9tR2FsbExMdEQyRW1OcEhRRzlXRWEyUTVEN21IRUZfZzNhOHNCWDA4OVlWY2JIc2k2eEVwWGloRF9QYkFzWm9kRzdaSldSQk0tMzUxSHR2MWFUeDE4M3pCTndHcWJQeHAtWExpeEV0MUZ6QkVrVEFYZUowbk9RUGF3bDBxNDY4V3hsUkptQkdrWW8xc0RNLTJSdA?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,38 +1024,38 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46080.48012731481</v>
+        <v>46080.38008101852</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TC Hasselt - Un homme de 21 ans risque dix ans de prison pour tentative d'assassinat - DHnet</t>
+          <t>Justitie wil ‘terreurambtenaar’ van provincie Limburg langer vasthouden, rechtbank stuurt Maastrichtse verdachte naar huis - De Limburger</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>TC Hasselt - 21-year-old man faces ten years in prison for attempted murder - DHnet</t>
+          <t>Justice wants to detain 'terror official' from the province of Limburg longer, court sends Maastricht suspect home - De Limburger</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 12:15:00 GMT</t>
+          <t>Fri, 27 Feb 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxPMHEtTjFPMk1xSXRqWFdWLUZJbVBOOGJmbDlmNm5RU0dfclJKV014SUJYdWZuRXkwVGlmUDNPejRsclFFeGRVVnVOdkpCOThNbWpJWDZFaDVEMlVHT2xTUXQ3M3ZEeHBWUER0S2RBWFEyQlFXMlhNZTVDdWtqYV9NYWQ0T0dlME5CWmtqWG02NC1ScjVNUFRXd0FmZFF6cWZkd3JhdDdDelZkOUxybVFaS1liRy1UUWdPRWdleENOUVBvek1rVGNiQURJOUloeXNlRlBCQXUtdFNMVkdvOXpWRHFRUFEzdXdzTl9ia01iVmNIUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPSXh3aHJsRzRjWko1SS1JUnB0Ym1fQTBRelIxZ2pjcjlENFB0V09jVzRGckJia3p2WGNReXFNajFZWTRuUF9KdElUdUtkTnJsOWtEZ3M2MzhOcThkLWJfOVJfdi03TFlKQTNqR0dDUE11b0k1WnppbW1kUFJnOGhyeURyN2RfZTZWdjZYb2ZYaWNTNHNmcGhzS0FqWUhWVTcxU2VfQ2l2QzdHZDl4MUVoMzdKN3JpSWRjcGt4bFdQZjVIdFlLWVBTbmFBQVJYTDAzY1BORmNSRmRrRGNWX3hxMG5NaHVhR1BUNFVRRGc5NjNYVDhIM05QQnp4NmFDeDhZV1lqbG5DMA?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46080.51041666666</v>
+        <v>46080.58333333334</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Poppy Ackroyd unveils new album Liminal, lead track The Unknown - Live4ever Media</t>
+          <t>Brussel laat Mercosur-deal ingaan, ondanks verzet van het Parlement - Het Financieele Dagblad</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Poppy Ackroyd unveils new album Liminal, lead track The Unknown - Live4ever Media</t>
+          <t>Brussels allows Mercosur deal to take effect, despite opposition from Parliament - Het Financieele Dagblad</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 08:49:51 GMT</t>
+          <t>Fri, 27 Feb 2026 11:22:11 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE42WEFhTXNKR2E1QUpyRjhKSzVZUkhvSUc2RGdUMjhyeGxWQUNIbVdHc1ZaNDZCZ2NDTjFvTGhJZ19vSkZyWEpibmpOYXdUZ0UwRWJUSTFqRzhkTlR0UEdFYlMxNlRObU5naUlTTEhaR3k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQYlpwQ2JtcURVTkVOYVR1Skh1b3VKUDYwTkFsZGxJck9kS2pIU1VQdE55OURUblAzamdrbENJNDMtYnVGRURuOFdsd2NCLXNobVZQaVN4Yk9GcGNlLVhTMUMzRlhnU1lfS19YVjRxdzY3d18wWmhaVVpOOThhT2JfVHM5Q0hqVzhFdmQ3dWJzV2YzX0VON0gzUVEwNGZmdw?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,52 +1120,52 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46080.36795138889</v>
+        <v>46080.47373842593</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
+          <t>Onboarding in Automotive: met nieuwe cursus in één dag klaargestoomd voor baan in de autobranche - Automotive Online</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
+          <t>Onboarding in Automotive: prepared for a job in the automotive industry in one day with a new course - Automotive Online</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 11:12:30 GMT</t>
+          <t>Fri, 27 Feb 2026 09:01:34 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNT1h3QWd4eHNRQlFGRDh4UExSNTZiUHp4d1R4c0lxcG5LWEhsQU5sZklnUWlBYzlOV2hNREZ1Uk9haW1WdlQ0MUF5c3E5Y3pPTFc4czRwd3dBOGpCS0M1RkdvaHNXSUZNRi1fT19xZHVJYThNRk9fNmZwQXIxc1l5Umxn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOZzJCSkFmOUxMeXVlTFBxU3VEMmtGdmt1Y0VXczh3VlZiS0VhUW1JYlRrSkFCN0Z6czF0QXprUEw1aFlLZWlKNjZfU1NfNlB5UEVxU2YzemtIM0QySjR1cDNQNUVQbEwxbmtXT1ZCVUhOdlNnNXFZUUxxNzM5elktREhzOGh3b2RaTTV4azl4NTQ4S1FHM2ZwTUszRkNnOWJHMHIxM2VmSkJEb0NnUVZERko1Y1J0ckdWbko5aVBSYkwtcG5namdpYXJ0ZnhQVHNwU2xlenQ1em52NEJPSjVEdGVrZ0dVWmFKd3kwcnlHWGpLbUFS?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,52 +1175,52 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46080.46701388889</v>
+        <v>46080.37608796296</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Marktbreit: 79-Jähriger vermisst - Radio Gong Würzburg</t>
+          <t>Euorpees Parlementslid Rihards Kols reageert fel op open brief van Orban: “Richt u tot het Kremlin, niet tot Kiev” - P-magazine</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Marktbreit: 79-year-old missing - Radio Gong Würzburg</t>
+          <t>European Member of Parliament Rihards Kols reacts strongly to Orban's open letter: “Aim to the Kremlin, not to Kiev” - P-magazine</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 13:05:00 GMT</t>
+          <t>Fri, 27 Feb 2026 18:56:32 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBZeTVpOWVYbVhHeGxaSkV4SVUzRWJTcUJURl81alBxT0NTQUtVenhSQ2s4VHJjMHdsS2JuOVFUTnhscjdUcUNacmFyUnRkeHdWc2hQRUFnSFZiTXMxZTJXTWtZRXFQbnpLSGxsTVdjVkp5T1JZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxOeFRubVZ0dkQ3WnlCaDIyRkNhdW5ZeFFhTVZHZmhwUGR6ZldHYlh4c3YzaW40RmlaTlJRdG1EUGFub1dMZ3FUQ2o0N1ZYTUNfTWg3ZU5PaW5lWlFjRnZUUUNKVjBzbHh0THBZNU9lLVVjUE9GWkhLbFJ5QWMyT1dob0h6MHpfWDFEbkxyYVF2Vmx2V0dScXRmbjgwMEJ5d0FxNVFuRmVnZUtuY2dBLWYtUnlHQ2FBVnNSS0ZlM1U4dWlHcHkzdE16VWI4cmZUbldGUEtWRmFNdEVGcEhHU0E?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,52 +1230,52 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46080.54513888889</v>
+        <v>46080.78925925926</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Kitzingen: Baufortschritt an der Klinik - Charivari Würzburg</t>
+          <t>Mandelson geconfronteerd met EU-onderzoek naar handelsrol in Brussel vanwege Epstein-banden - ekhbary.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Kitzingen: Construction progress at the clinic - Charivari Würzburg</t>
+          <t>Mandelson faces EU investigation into Brussels trading role over Epstein ties - ekhbary.com</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 14:30:00 GMT</t>
+          <t>Fri, 27 Feb 2026 19:33:05 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQM0sybjNfLVc2Q2FNVmRHUWRoeXlaTW9RYXA5LXktbTBaU0FLTGVWa3JNN0V1QzJJVW14Q0NwLTRuTkRjZ25ES2prd3FKcUFNS0lBNl84ZGdpUmlCT1VkVDNNQ1M0TFBIVUZEOHoyZU1wRktndVRqUHhKSW4zNG8yWA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNbThmazN2dEstYTc4M0s2UFc5ODBTRkw2UmhwdmhwTTAtSUYzVHdRZFU5dkMzVUxZRTZPcmFSYkJxTEsyREdULV9zSGVabVBjX09wSDU0dGxlcHd1ZmhhaFdJdWxyX0ZETjNrRlRJY0VRakJOVmlDY2piMFVKMUxON3IyRXBmTVdLcEZmLXF5TzZSOXN2R3diVHJ4YXduXzROQ0hFMUc2LVNSUkQ2bFlzVHJnMFpzWnQ3VnlLX2pXdC1kVzJ1SG5FNWNGbm4?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,52 +1285,52 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46080.60416666666</v>
+        <v>46080.8146412037</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Brussels orders probe of Mandelson's Epstein ties while EU trade rep - Yakima Herald-Republic</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Brussels orders probe of Mandelson's Epstein ties while EU trade rep - Yakima Herald-Republic</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 12:51:46 GMT</t>
+          <t>Fri, 27 Feb 2026 10:19:46 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxQOTkxQkkzaTA4TGF0U3o1Tmp1dEJpWnZKVDNuaGFFRldZRXdwT0VYLVpZNlpGVEtmbmJXaDRCSkNzNmhNTk91eGt6bTJNbEl3NDl3QzRhQ2Fsdk14QkR1U1VRT0J2RDBMZFZGRGptZ3BqOWpETDhhRVVWai1VRjVBVWJaQ2diOFhqSVhnOTFfNHlVcEwtOTBhSGpWdjluR0tpT0liTnkzc0JYMWxpX0s4UWNvd0JsNl9uNWlDSEdXMTY2NVJ4c1dsazFBU2lQODg3cWJfYk4wYnlVYy11MHFfbE9KUGdTLUdwSVNLN3hjcF9BZ2FUbFg1MUtSRUZzMlhIRERMQtIBigJBVV95cUxPemJzLWRsMnIyNDY3c3JnOEZxT1ZFV3ZjMzRaTkxIS0dkY1Nua0Vvd1QwQnRsZW9pZUdTQWZjaHBiemJwNGJsSlhaMHFKQ0tWMjlMQUdxUkhsaVdNanZ0UW41Rnh5NGotNVpTUG1ISXdYZjN2cEttX0hZZ0ZlUjdNVlFyc1k2STJCUG5OOVI0M0xQa0RlaWgzdUtvSGhmcHplV1daWkNfT2NmNWs3OHBfbUNpakRtWGV4c1BGN293MkZXVERQcjVfMWxLdnhMcWp3NnhPTFVHYjhLUFRsaTZiQk5FZG1wQVF3d1V5c0tUX2FVNnlwM3JESW4xX1VfUlYzaDVaUTRlam1ZQQ?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46080.53594907407</v>
+        <v>46080.43039351852</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Polizei-News Schweinfurt / Würzburg / Nürnberg, 27.02.26: Schweinfurter Zoll stoppt Lebensmittel-Kurier mit ungekühlten Pizzen im Kofferraum - News.de</t>
+          <t>EU THREATENS TO HALT FUNDS FOR SERBIA: Emergency debate in Brussels over adoption of Mrdić’s laws! - Serbiantimes.info</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Police News Schweinfurt / Würzburg / Nuremberg, February 27, 2026: Schweinfurt customs stops food courier with unrefrigerated pizzas in the trunk - News.de</t>
+          <t>EU THREATENS TO HALT FUNDS FOR SERBIA: Emergency debate in Brussels over adoption of Mrdić’s laws! - Serbiantimes.info</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 09:36:02 GMT</t>
+          <t>Fri, 27 Feb 2026 10:06:28 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPM1RDOTB3eGxGY1ZOa2NmZVhXX28wWHZBZjhmUVBaVVlseGtWa1BtSjZVNDM3YUlSMFVoQ3kzTldhRjFQOFI3WWFwRVJEcWpvU2M3aG9fVUtzSzJvOXFfSmkzUTMwelJBcXFramhneGxuZ19GNFpUY1d5c2VKSW9UZ09wSWNuVEhZODJySl83cHNXVWJrWlI0S294NUV2Y2U0SG03bEV2ZjJDYUJpUF8wdUlBem5KbEZjR0xrcGlGeFR5Qy1kRXU4ckZZN3o3aWNyRFNad1plMDFWMnFBZFHSAeMBQVVfeXFMTmc0UGhYTEdaalNuQUpjSXJfaXY0T1kxY1AycVI3c0FqNWozaUZVTzRVV1c2aXYxaTNsSk5fYjdqSENtNVR3TUJtR0dOUGwwUTZsbTBmeWhHY2xiRUs4Q1kzV0lUTjBrYVlSVlNxZUE2U2V6RHJOQi16eUN4SDhtbzBXTU5sU3ZUUkYxVDZKVDI0NGpfOFhJQnY3ZDJuN255Rm1SVTA5WEVZOGJraXNkYjhsX3FkV2dmRXhIQkhydkdBcGg3SVduV3hkcDFxd3JqRkVIaXhJTi1fUlpSa083TzQ1bXM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOYzVLRnJnam1rRFB4T2hoSFUyRTZjLUhlZlBsTEM0VDRySW55UGtRUVFydVdsbGFrTElESHBCN1NTZzBpV1NPbUs0Q2wxMVh0N0xPMDBPaThmZWpNNzBmdkR3T3lCYkxaQTFqOVl3Rjd0eFkxSXU1a2pqZjZ3eG5Nd1dDbHhMRXNaQUVmMDJFRVQzeGtKVXAzS3dHbEE2YUJlSllOR3Z3QzdsRWdDVjd5c09waVAwOHVJbFpTRm1KQ0l6eDA?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46080.40002314815</v>
+        <v>46080.42115740741</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Bessenbach aktuell am Freitag: Hier nimmt die Polizei am 27.02.2026 Raser ins Visier - News.de</t>
+          <t>Alertes à la bombe: la tour Montparnasse et Sciences Po Paris évacués - 7sur7.be</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Bessenbach currently on Friday: Here the police are targeting speeders on February 27th, 2026 - News.de</t>
+          <t>Bomb threats: the Montparnasse tower and Sciences Po Paris evacuated - 7sur7.be</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 09:19:07 GMT</t>
+          <t>Fri, 27 Feb 2026 16:57:59 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxQN3loSDQweXZybkRTSHlpM3k5eEdMZThLVTZGcWJIRGV4OURiMTBxOThwdUFGcEdiLURKOHluU0hJRVo5Q29vZnRoYTNKRVhsM1NURW56SDY2TGVRSVhQV1lTU0I3a19yYjZyUkduQS1yXzFMVGM1c1BHNjNhMlRiQy1pNFNmN2xuZW1JeEJkb3gxdVBaUk41ZHRGejFoWWhkdEMxcEtwQmY0dWMzcmR4RkdROHBZdjc4NFVUYzlOYVNtaHgyRUVha1BoQ1dlWjBFcU5RdlpROVRkTUdmeXBkcG12cFNjU2VBcVllR244bUpKTkRFZV9GT25B0gH_AUFVX3lxTFBaNGU3anh2QW95X0J3aTVubTJiOVdEeFZjUFhFZjdyRVAwV1J0TW5oMlRVaXRhV29JSi1HbDM0OWJyaGx4QTIxQnJUa1RnZjlCQkdTX0lqdW1HZjl1LUtMcFYtOFhwaG8xcEZHUS1RbGNwVjE4VGZVZy14aGJEQlNqVGVDTnpOLWFvR1d2TWNzRTNLQ1ZzZm12MDdhN3RZc0hwck5seXBuS3FxbENvV1NxY3laSWt5WDZUUVdDOXZBTzZFbnJlWG1jM04ySEVhdURWclgxVVV2ajJrSW5BMGlDdW15YWwzZTdsbERJUnVtUHpoTDJfZFNlSDYwXzM1SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQVzBXYjBsbHhQa09jeElaeEVUR2JYdFlza1NFUzIzeVpLT1JnbzNRaDRZaG1WYUxNemg2eE5BVzNYZi1CZWZGcGlWMEgyUjRuTk5QOE9XX2x4bnN3dFlHUThIMklYUWg0c2EwVG9xNkxWdmwxN3RNOWNvb1RMeHB6UHpBRWVnTkU5QVJtYmtuaXE1V1I5enVHWFN2czNDaHhyRFBVTXZES1lmY0lNOG5zWVN3?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46080.38827546296</v>
+        <v>46080.70693287037</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Corona-Zahlen im Landkreis Aschaffenburg aktuell: Inzidenz für Landkreis Aschaffenburg, Bayern und Deutschland - News.de</t>
+          <t>Buurtbewoner die mollen wil verjagen met gasgeurmiddel zorgt voor evacuatie van school door sterke geurhinder - VRT</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Current Corona numbers in the Aschaffenburg district: Incidence for the Aschaffenburg district, Bavaria and Germany - News.de</t>
+          <t>Local resident who wants to chase away moles with gas odorant causes evacuation from school due to strong odor nuisance - VRT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 10:35:43 GMT</t>
+          <t>Fri, 27 Feb 2026 11:31:23 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_wFBVV95cUxObGwzMFZ6N242bWREWWdvZVNrYVVrclRSVFlPM1lvaVYyRHFpTXNlSHUyUHE4SnNfenJ6clUwNnZkcFdMVHdsb3hwVUh6d2pqNVdWYlpydVNOZ2xTdVBEMnY3VnBRMUUtaGVLc3dxQWxPLVBpVDhrc29ST1hhaVJHMWJXOFBLWmJ4RU9WdTZUODNob1dZRmxHSXdZY0Fpc2E0LW5USDRUX1hKWWZSVTN5TU16RXZvTDRWNHZaVmJTOGhWTGRjTloxWm5uaWgyZTJ0YUF3Rk82ak1WbzBOUy1CbEM5Q0wwX1Z6X3MycHJMOEpaY0c1R3M4VjdqNGpjamfSAYQCQVVfeXFMTXc3WWI2TDV5aG4zZENUNWEtQ1QxbFJ6Z1VMbE9aT3ZxRHNvUnR1YWdLN0E5ZTdDNjZTOWdobzdudTIwRWdRR1hEZWU0bTJJb3JxZE5VQVI4c09ZcDlablRSQVRVQ1d6d0JHSlBHUWxhR0lVbkNTMnByRzFVT3BKUjVwWGZvcnpYdGtLaDdfUC1iNktJYldpRUZ3Rlk4N3hCaDFFYTUxbTMtTEFhd1k3aG9kT3pBdDEzZkZzaENqc3RHV21mNU11TU9adWk0bmV3NktyWDUteFdjT2dJOFd1THZWR2hUdGc2QmtGZm5qMUFrYTJDWXVsMVJrSkhBckl4eUNkbU0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNQk1IcU50a1AyNGxpaTFGWmFqZ3RkbFJURjZISHcwYlRlWEg3amRkRWU0TEFQVDJGeWsxQTZZeG5nVkQ4RHItRmVhSjhaQWc4eDQ0VDkyZzdBM0syYm5IVklnYlF4N1NFRXg0aEhvcTRZY1dCSHNZMTd2UlNDMDVFMF9WSWplb0k3WjJOakNEUDJ1QnB4Y1FsVlptcUxmS3dUQXk0?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46080.4414699074</v>
+        <v>46080.48012731481</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Polizei-News Main-Tauber-Kreis, 27.02.26: Körperverletzung und Missbrauch von Notrufen - News.de</t>
+          <t>TC Hasselt - Un homme de 21 ans risque dix ans de prison pour tentative d'assassinat - DHnet</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Police news Main-Tauber district, February 27, 2026: Assault and misuse of emergency calls - News.de</t>
+          <t>TC Hasselt - 21-year-old man faces ten years in prison for attempted murder - DHnet</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 11:06:02 GMT</t>
+          <t>Fri, 27 Feb 2026 12:15:00 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQQWhNV2VQeURtamFMNnBaOEpHRm1KaE1feEVuMmc4RnJVWTdlZ1VZOFBJMTVnbjgwVjVCWjJvUVpmMGRFZGxtck9IbTNiRjF1V21vQkllQTNGMVFDWER2eU5CUEJpNEhlOFdKZHR1TGhjakEtVkNfd29aRUVya1ZJLU9PWWxLU0lRQUxlN3h1OHQ0d3FERm1ZOW1OMXJFVWpM0gGmAUFVX3lxTE4tc09YRUZjVHNycGtZa2tFWHoxdXp1RFBQc1pEOVUwYU5ISW5hSFMxZWJfdXNIT0t1ZDhVVElYX3J2MmFOdWJCTVdUU05qQ1R4N1M0d1dFRjh2ZjRuRlBSYm9uX0lUblpXcldYV19xdF91M3Iwa2IybTV2VmpzTlhEdFB4aVRiVU1xbUtyQzhlck8wcVVnYmV0elhqTVQxQ2VoWjdwa3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxPMHEtTjFPMk1xSXRqWFdWLUZJbVBOOGJmbDlmNm5RU0dfclJKV014SUJYdWZuRXkwVGlmUDNPejRsclFFeGRVVnVOdkpCOThNbWpJWDZFaDVEMlVHT2xTUXQ3M3ZEeHBWUER0S2RBWFEyQlFXMlhNZTVDdWtqYV9NYWQ0T0dlME5CWmtqWG02NC1ScjVNUFRXd0FmZFF6cWZkd3JhdDdDelZkOUxybVFaS1liRy1UUWdPRWdleENOUVBvek1rVGNiQURJOUloeXNlRlBCQXUtdFNMVkdvOXpWRHFRUFEzdXdzTl9ia01iVmNIUQ?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46080.46252314815</v>
+        <v>46080.51041666666</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Paysafe Announces Changes to its Board of Directors - Business Wire</t>
+          <t>Jong Gent - Patro Eisden Maasmechelen - Bulinews</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Paysafe Announces Changes to its Board of Directors - Business Wire</t>
+          <t>Jong Gent - Patro Eisden Maasmechelen - Bulinews</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 12:00:00 GMT</t>
+          <t>Fri, 27 Feb 2026 18:17:48 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQbktaX2NKdnB5YXpUTDNzendZSE5BaGRtcUE5SXEtOGZCZk55SzBwWUt2VFgxdjlvMlFGNnpWakt0dmV0MnpreU5lTTF3UnVfZkdrTERwSmxvNmxIUVVqQXgwbW5TR2R5bkNMLW9rYzlwaUxWQ0hDczA1bXpCVHlXRVhEOFI1N1E0WlNmSkRGZU1kd3pBcDZmcDZrQVJ6akY2UWt3UnI0RDh2bENB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxORXp5bGdmTllvNE5KUW16Q21Zd0NQUUREU0phUVMxMnpKQmk2dmFQT3hOZ2M2TklESks4cXRNbzQ2WXV3TmRXNHZXYVVrX0V1cEM3VU9hZy04VXV2RnJPZklLX2R6SEZkZTR1Qk9qcFREOXkwb2M3Mk05NW9iSnZnanh6TUFza2s?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1629,62 +1629,832 @@
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46080.5</v>
+        <v>46080.76236111111</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Match Centre - Transfermarkt</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Match Centre - Transfermarkt</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 18:54:07 GMT</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBIQ0R4X1lzd0Y0R25OX050b3RSSFdoRld3ZDk0Smd3YTJxU3JCeHJrSkxUYXAwRnAzenhJbWNPYnE2dTlXQndLVnFBcGU1elp1Z2F4LVRrTDdhVHYyZW9fR1RkUTc5NWM5Yk5V?oc=5</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>46080.78758101852</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Poppy Ackroyd unveils new album Liminal, lead track The Unknown - Live4ever Media</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Poppy Ackroyd unveils new album Liminal, lead track The Unknown - Live4ever Media</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 08:49:51 GMT</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE42WEFhTXNKR2E1QUpyRjhKSzVZUkhvSUc2RGdUMjhyeGxWQUNIbVdHc1ZaNDZCZ2NDTjFvTGhJZ19vSkZyWEpibmpOYXdUZ0UwRWJUSTFqRzhkTlR0UEdFYlMxNlRObU5naUlTTEhaR3k?oc=5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>46080.36795138889</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 11:12:30 GMT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNT1h3QWd4eHNRQlFGRDh4UExSNTZiUHp4d1R4c0lxcG5LWEhsQU5sZklnUWlBYzlOV2hNREZ1Uk9haW1WdlQ0MUF5c3E5Y3pPTFc4czRwd3dBOGpCS0M1RkdvaHNXSUZNRi1fT19xZHVJYThNRk9fNmZwQXIxc1l5Umxn?oc=5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>46080.46701388889</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 07:40:40 GMT</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8waEpNdEZmMmtDMFhIVzRBZ0QteWtGc0JMUjRFT2hzUXNGa25Pa2FPNzRHSWtUZVVvcGNORnNvYjFVZ2dIeVBMNEs4dTBvdVhmYUt0UWx6T0RQR2daak9ZR2p2SFpZU3lRS2dNaXJ0M0pSMGM3bmcyeEJvT1Y?oc=5</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>46080.31990740741</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>79-Jähriger vermisst: Polizei vermutet Ausnahmezustand - Nordbayern</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>79-year-old missing: Police suspect state of emergency - Northern Bavaria</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 17:24:40 GMT</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNaTZUazctejdYd0p0VUQybmYxWDJlZE9ocnZjRVdMOTlHVTRnbWZVeVo3NmR5WTNNR3BJNi16QkZ3V25oWTJWLW5CRVVwOU9QQXU4X0ZpM3UzX2tJTzNIdXZtalVSSTkyZHVKZldDcVBPbGNkR2Rab1pLX0FKVGc2cEFqc0ltRkwxSF9PNXZ4bm9vRV93ZWxuaEZKbHBESVhXZDJiV3BsV2V1Ync2U2g5WTBaOXRVZzlxZ25WZThJemY?oc=5</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>46080.72546296296</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Würzburg: Gewerkschaft der Polizei traf sich zur Versammlung - Main-Post</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Würzburg: Police union met for a meeting - Main-Post</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 15:13:17 GMT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxORXY4Y3Yteko5T00wam1IbXhyNk1FSE9IVkNZeThtUkNORzFQS0x2MUczUm9jdUVNLTFZNUVfUFk4Qlo5NURWLWpGVkVDdVNSZlNNcFJEd1hJS0dwRUg0ZWg0VGZ0cTEyUHAwSEZTWGlqaDBSMnhkM0lqT2xuNUp6eXRjRFh1dUpXX1JscVVSUUJ0Z2E5VlBHVUVBeU42ZWNnNmVVZF9NQy0zeFlfN1VlQW12WWVELU42LXR0M3VZRUo2MHY3?oc=5</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>46080.63422453704</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Marktbreit: 79-Jähriger vermisst - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Marktbreit: 79-year-old missing - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 13:05:00 GMT</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBZeTVpOWVYbVhHeGxaSkV4SVUzRWJTcUJURl81alBxT0NTQUtVenhSQ2s4VHJjMHdsS2JuOVFUTnhscjdUcUNacmFyUnRkeHdWc2hQRUFnSFZiTXMxZTJXTWtZRXFQbnpLSGxsTVdjVkp5T1JZ?oc=5</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>46080.54513888889</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Polizeimeldung Kitzingen, 27.02.2026: +++ Aktuelle Öffentlichkeitsfahndung +++ - News.de</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Police report Kitzingen, February 27th, 2026: +++ Current public search +++ - News.de</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 14:35:02 GMT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNY2JRazRGcUxpZXhTNlNhNW5Lam1HSDFzLUlLLU50NmZ5MFgyLU1RM2tPYTI5Mnc3b29pcS1fM01WQTFlSzlsSUJUc0VybDIxTnU4T09DOGNpbDRwbXV6Q0hEcUxrS2xYNm5neUt3N2c0b3pKeV9TcmIybDNYUmFodDlhdDk0aERtczRlZkJKd3Z2cElaY3A2TV90U25QMTNPcjNlcU5ROGREQ2JabnfSAbMBQVVfeXFMT0piOUtlSUJHaThhRmpwUEowdldVY3p5MHMxR1hYM3ZmQXRFR1lzX3g2R2N0OW9nM002WDhHT0Z3bW5IVlMtQlJrY29EYlAxSmdQY0h4T2dxMTlTbXl5a3lIdVVXV3BKVnROXzZ0TkVsUmFNd2o1T2JOaFRydkVhNnJmRzJORFlfMW12dHZiaEx0Vy1pUzRVMGhoOHRhVTBOeFNScjFWYnpTUDdod21XMUo5T0E?oc=5</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>46080.60766203704</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Polizei-News Schweinfurt / Würzburg / Nürnberg, 27.02.26: Schweinfurter Zoll stoppt Lebensmittel-Kurier mit ungekühlten Pizzen im Kofferraum - News.de</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Police News Schweinfurt / Würzburg / Nuremberg, February 27, 2026: Schweinfurt customs stops food courier with unrefrigerated pizzas in the trunk - News.de</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 09:36:02 GMT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPM1RDOTB3eGxGY1ZOa2NmZVhXX28wWHZBZjhmUVBaVVlseGtWa1BtSjZVNDM3YUlSMFVoQ3kzTldhRjFQOFI3WWFwRVJEcWpvU2M3aG9fVUtzSzJvOXFfSmkzUTMwelJBcXFramhneGxuZ19GNFpUY1d5c2VKSW9UZ09wSWNuVEhZODJySl83cHNXVWJrWlI0S294NUV2Y2U0SG03bEV2ZjJDYUJpUF8wdUlBem5KbEZjR0xrcGlGeFR5Qy1kRXU4ckZZN3o3aWNyRFNad1plMDFWMnFBZFHSAeMBQVVfeXFMTmc0UGhYTEdaalNuQUpjSXJfaXY0T1kxY1AycVI3c0FqNWozaUZVTzRVV1c2aXYxaTNsSk5fYjdqSENtNVR3TUJtR0dOUGwwUTZsbTBmeWhHY2xiRUs4Q1kzV0lUTjBrYVlSVlNxZUE2U2V6RHJOQi16eUN4SDhtbzBXTU5sU3ZUUkYxVDZKVDI0NGpfOFhJQnY3ZDJuN255Rm1SVTA5WEVZOGJraXNkYjhsX3FkV2dmRXhIQkhydkdBcGg3SVduV3hkcDFxd3JqRkVIaXhJTi1fUlpSa083TzQ1bXM?oc=5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>46080.40002314815</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Demo-Termine heute, 28.02.2026: Hier gibt's am Samstag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Demo dates today, February 28th, 2026: There will be demos here on Saturday against AfD, misanthropy and the shift to the right - News.de</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sat, 28 Feb 2026 05:26:59 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxPNThVQm5RUm9BYU5RaVAtMTRuMzhNUV82NFlJRVZidVZqOGZ4ZWFnN2NEdGk2cUxIbzRmbUNhWXJtalhqVUxsU3ZqM2wzeTBLd0pScFB4TTlLblJLZ20xaWo4OTJBWXRrYmJYR2dSRnRyZDViT2gwTmNXdGNHT2xHeW00MG9ERjJpRVBWNU1Lak9PTldOWHNxSW1ZVmhVVmlrdndtSFlLMEpLTUpiX0xNZG54bDZwbnBUSE5ZY250VVZidUFYc1RRSXVBZVJhVW44cFhWLXdOQWNVTkhvaTA5T0RFTjZWVnROS19MekFWV1J4N1lnTHY2by00R3IweHo5YXpZ0gGIAkFVX3lxTFB5dmV1aEkwUGx4TExoWUJ6Z2FTbm1tTGtRNU1IVnBZUGNNV0F3TkpKbTc2UDVrdzI1Y1hZbDZvVnB5SlBQMF96YVhUbG10dDJoUVc5RVBSa2ZQNWZSZWhmaXh3YjZQcmtwd3BoXzNJZXdHa0UtMno0RkFGaXhmVlRuQ2p2Qlk1STdjVlVtcnVlcXJ5WjBMN2laZkZvU3RuX1ZBTDFMSkRZYXV1emFJYXd4cjdJM1hiNkd4bVpCX09rcWN6ZmUxdEtJaVlzS1pZT3pfZXVhTTlLV2JocGozUFBndEk5QVI1SVhoNDhJRmdVZENCVDZIUjd1aFp3Tm5fX29JeWU0UFhoeQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46081.22707175926</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Mobile Blitzer in Bessenbach aktuell am Freitag: Hier nimmt die Polizei am 27.02.2026 Raser ins Visier - News.de</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Mobile speed cameras in Bessenbach currently on Friday: Here the police are targeting speeders on February 27th, 2026 - News.de</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 09:19:07 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxQN3loSDQweXZybkRTSHlpM3k5eEdMZThLVTZGcWJIRGV4OURiMTBxOThwdUFGcEdiLURKOHluU0hJRVo5Q29vZnRoYTNKRVhsM1NURW56SDY2TGVRSVhQV1lTU0I3a19yYjZyUkduQS1yXzFMVGM1c1BHNjNhMlRiQy1pNFNmN2xuZW1JeEJkb3gxdVBaUk41ZHRGejFoWWhkdEMxcEtwQmY0dWMzcmR4RkdROHBZdjc4NFVUYzlOYVNtaHgyRUVha1BoQ1dlWjBFcU5RdlpROVRkTUdmeXBkcG12cFNjU2VBcVllR244bUpKTkRFZV9GT25B0gH_AUFVX3lxTFBaNGU3anh2QW95X0J3aTVubTJiOVdEeFZjUFhFZjdyRVAwV1J0TW5oMlRVaXRhV29JSi1HbDM0OWJyaGx4QTIxQnJUa1RnZjlCQkdTX0lqdW1HZjl1LUtMcFYtOFhwaG8xcEZHUS1RbGNwVjE4VGZVZy14aGJEQlNqVGVDTnpOLWFvR1d2TWNzRTNLQ1ZzZm12MDdhN3RZc0hwck5seXBuS3FxbENvV1NxY3laSWt5WDZUUVdDOXZBTzZFbnJlWG1jM04ySEVhdURWclgxVVV2ajJrSW5BMGlDdW15YWwzZTdsbERJUnVtUHpoTDJfZFNlSDYwXzM1SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46080.38827546296</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Paysafe Announces Changes to its Board of Directors - Financial Times</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Paysafe Announces Changes to its Board of Directors - Financial Times</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 12:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPc3N3ZWlYLUFIeVg3VGFjZlpKdlNEaVJ0azlRRW10cW5ENHltbkVVZEVCNkhWaWt4ald6V2VvRW9kXzRqbklrc2tWUXhSQTZ1eGtxcGt4Z2dud1h6ZXoyTVVMaGFLT25nQzNfUW1pMVR6UWZmMmRFeWFISURSTl9GaWtTQU44ZlVkMjRSbHE2VlFRY1NSY0VsU1pUbDUxREpKbTZrbGl3?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46080.5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Local Town Ingolstadt German</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Suff-Fahrt bei Manching: Kleintransporter-Lenker hatte über zwei Promille intus - Pfaffenhofen Today</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Drunk driving near Manching: van driver had over two per mille alcohol consumption - Pfaffenhofen Today</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Drunk driving near Manching: van driver had over two per mille ingestion - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>Fri, 27 Feb 2026 14:11:55 GMT</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DMGk1UjJFUjlIc0RzOW1wUDBvRmJHRmR1MjFxYXFkTzJyX1IwNTlTRVktMVhweklRQkh3UGJoVzJvUEZ2dC0wdU1QUHNQRFl0U1A3ei1PMVlYNng2WG93YVB3?oc=5</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>DE:de</t>
         </is>
       </c>
-      <c r="K23" s="1" t="n">
+      <c r="K35" s="1" t="n">
         <v>46080.5916087963</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Desire Lines: As Mother's Day approaches this one of a kind keepsake is a must buy - Irish Examiner</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Desire Lines: As Mother's Day approaches this one of a kind keepsake is a must buy - Irish Examiner</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sat, 28 Feb 2026 01:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNZ3l3cDJxM012NVc3M1dodV9uNWdjZG9zeGNHX3FHcU5mNllnR2tVSmxySlltVXhDZTQyZ2RrYnVFVllhNEdpRERZTzY2SGxMQ25oRWJZdUxKX1ZEQkRCM0R6eVM2TUpUdnJTcy1zY1FSZjd4emk2X3F2TF9HZ2VIRg?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46081.04166666666</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Village La Vallee (fallback)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("La Vallee Village" OR "La Vallée Village" OR "Serris" OR "Chessy") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Elaine Hendrix Reveals Lisa Ann Walter, A.K.A. Chessy, Is Joining Her on 'DWTS' to Perform 'a Song from “The Parent Trap”' (Exclusive) - AOL.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Elaine Hendrix Reveals Lisa Ann Walter, A.K.A. Chessy, Is Joining Her on 'DWTS' to Perform 'a Song from “The Parent Trap”' (Exclusive) - AOL.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Fri, 27 Feb 2026 20:49:28 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNYWpLTjZGdUdzMXdlTFhjTzZaeDU2X0JySkU5UGRpX0l6T3gxd05CdTNKRFpRRHNUVE14RVFKQVFYQy1peFhDT1UwR25SY21UMkxmSGNSMm00TkhpRGp1NGVLNjByM25WTG0xc1ZlWjRsU0k5WEN2Q0ZZSHRQX2ItNg?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46080.86768518519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-02-28 14:22 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Brand Protest</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Demna debuts with body con Gucci in Roman temple - FashionNetwork USA</t>
+          <t>B&amp;M European Value Retail S A : Creates 30 Jobs for Locals with Brand New Diss, Norfolk Store - marketscreener.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Demna debuts with body con Gucci in Roman temple - FashionNetwork USA</t>
+          <t>B&amp;M European Value Retail S A : Creates 30 Jobs for Locals with Brand New Diss, Norfolk Store - marketscreener.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 16:44:30 GMT</t>
+          <t>Sat, 28 Feb 2026 08:53:04 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNSjEyV25FYkdjQldydExXQXR3VkJ1allCT0NkSDRTMURkSWVIMTZ5amZqQVVja1NvTFlucEMwNnRhUlNZVWRXTTNfTlZITS1TNW8tSERRRWZoYWpiVk9ULUJkU1A0UGh5NzlZeUgxRnhIN3JoNW55bFdMUmF4M0V5NG5kMmNybWo4YTQ4dHhocUlvaXpHQWNQdGNZS0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxObHRuQUhqcllSTUotUXlXVElTTFgwbERBZjBpUkFBaWtDZUhHSkgxZ1dDcjFHalllaXI5bWh6cHUzdWM4MXgwS2lpbURUWHNkMEppajMtd1dwSnJMNWRqWERNU1I0NllrQnFMd3A2clcxWjFrQlZ6RER4WVVtVGxwd3lETzlqMXQ4OFBXNGZMWlB6ODFjejNvZGh1UmpFUU1INmMxVjI4bWRIVTZ2RGtydl9SdHo3dV9Da295M3g0ZjRrcTYwUXVndV8zdDY2UGpCVGgwb3BkOUJISWM?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46080.69756944444</v>
+        <v>46081.37018518519</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>BV Logistics Disruption</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("DHL" OR "UPS" OR "DPD" OR "FedEx" OR "Royal Mail" OR "Parcelforce" OR "EVRI" OR "Dropit") AND (disruption OR strike OR failure OR delay) AND ("UK" OR "United Kingdom" OR "Britain") AND -dental AND -"pay dispute" AND -"postal vote"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail S A : Inside Information / Ad Hoc Information - B&amp;M EUROPEAN VALUE RETAIL S.A. - marketscreener.com</t>
+          <t>Royal Mail warns 20 UK areas won't receive post on time this weekend – full list - Express.co.uk</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail S A : Inside Information / Ad Hoc Information - B&amp;M EUROPEAN VALUE RETAIL S.A. - marketscreener.com</t>
+          <t>Royal Mail warns 20 UK areas won't receive post on time this weekend – full list - Express.co.uk</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 17:03:11 GMT</t>
+          <t>Sat, 28 Feb 2026 10:47:00 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3wFBVV95cUxPNGMxSFIzZjFJLUVqRWpwSkFqdUgzeHZWOWlfblZMVU1wMFlXTjMyTm01Z0NDV1lMajV1cTFlMi01QmktV2FZd0NqdHU5djNrQTNGcUllZE1DS0ViaGFnS3RSdkZyRTZ5VU11Yk50QmNUY1AtTmFjNHE0NHp0ZDRlLXFqeW9hRHBwanhuTF9tY2FBQ0FCTWFMTU5iUGV2b01aTGFwY05qSTk3cENjSjhaQzZ4bDB2bWl2NV95eG9JRk12ZVdmLW1GSktpUUNvZFpYVTB5M1A4UkRvRzllLUFZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNdWFkbzRSX2hQT1J5cjFJazJoQno1LV9tOEtaTExvYnJZVkF2ck5MOXRLQUg1TjdnTG9GQlZuQ3dIN2llaXRNU1I5MzNVS3ZyNEY3cFVCa3JISTQwWmdvdTBqZFl5REhkSHl2T2x2ZE40cjZLc0xNRnVWV2k0aVd2SzVYRXJwd1HSAYwBQVVfeXFMTWVRUmVlRHZxajY2Q0czS01XMDQ2M01TN3p1bnEyTGZXS0NwMFNad1VmbndpME1uTU9OR0tVMVA5OTQ1b2JiZFNSN3RONk9JVzZ6OUhyVmllTVZJdVBlQ0VRaWtDWnBTblZNMTJjS3pTWURYZDZiZDBqbTliM0RNaTJVdXFBOGVoU05hWlM?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46080.71054398148</v>
+        <v>46081.44930555556</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>B&amp;M Completes Jersey Migration and Prepares London Listing of New Shares - TipRanks</t>
+          <t>Explosie in Anderlecht: appartementsgebouw en voormalig tankstation onbewoonbaar - HLN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B&amp;M Completes Jersey Migration and Prepares London Listing of New Shares - TipRanks</t>
+          <t>Explosion in Anderlecht: apartment building and former gas station uninhabitable - HLN</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 16:59:50 GMT</t>
+          <t>Sat, 28 Feb 2026 10:40:17 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNZEdFSFRreEduaWlhTEhiLThKM2QxdC1wTjVVYWFCNjhEcWphd2IxR0RDT2NJdEhpbl9UUnNXTGpvN0lEaFExeW9ZMzVad3FScmVGYVVZRTJfZ01RSmFxQjM5NFM3SXhRT3NSVktrRmlNRTVuSFhtTjN2QUR6TDB5cjNrbnNNWEVBTnJwSWdMWF8xTWRMWnVweHN5SGxYdzZBQVkydFFOdVBMVFlnYnRFM0tRVVZyY1Exc1RrLWx0OUo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOdmFTNmVmeVFpRC13MENWemxqWE8tSlR5RE1PaF9ZY0FkcFk1OGd0U1Vnb0NvUDBlRXhPR1huWHh1cWh1NGZkVTJZZmdTT2R4a1NEVDVwRGtzX2dvUmExeTRKdVMwclphOXNaUVdBTHBXcjlneHNiZ3dJWjJmMlpIZEFtSk16R0c1RkRvOUdFT210RGJtd2lWT1ByZ2duTnhtc3dMTTVtSkhEbHJJcm85YUxVNy0tcG5m?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46080.70821759259</v>
+        <v>46081.44464120371</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Promoter pares 14% stake in Vishal Mega Mart; HDFC MF, Govt of Singapore among 3 investors pick up over 6% shares - TradingView</t>
+          <t>Raad van State legt bom onder voorstel voor lagere LEZ-boetes - BRUZZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Promoter pares 14% stake in Vishal Mega Mart; HDFC MF, Govt of Singapore among 3 investors pick up over 6% shares - TradingView</t>
+          <t>Council of State puts bomb under proposal for lower LEZ fines - BRUZZ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 15:13:14 GMT</t>
+          <t>Sat, 28 Feb 2026 11:16:08 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxPTlNtUkNVUm5RS3czMkhjT2FNbVA1dXpRU3pVVTd1WnBmcHlkcUtxQVBYV2FmNEI3MzNLdVlNOHQyMUtFY0gzRkhTWXA0cVhnWjZteTRsNm9fU3VSUnVja3UyZTNaU1hjaTB2UGJheENtYjdscFJaSXA0VDlxcFk5QTQ1NkpDV1JiWVFvME9sclNyZVpwUUp2cTUtSHVvWk5OTXhEOW03d1dEVXlsLV9DV2RMWlo1U0JoSXlCb0FzcjN1U2xxZ2RRRTgtTVRKaFR2UkZtOXlSb2hpcGRvS1ZSUTNfMVdHZldheWNrdDkzaVlvUVRtNmE0aTk3eFFDX0NDSlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPWDl4MjB2WS00b1VZZk92cjNFNWhIdEZCY2tPQXhET0N3cFY3NlhSTmRQdl9GcFlLQW9oWnpzUUZtQ0ZYcnJXQ0YwdUdPbW5FMldxNXR5R1hNQzV5MW8yY0xfcW5RMTNsdWRCanZnUVAzNHhXWkY0OFkzYUVmZFZHZGtidFdjTkx4dDYtMkFPM1VRNkxpUDI1RnpqWllLYzFuZFdqcjF3bTE0dw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46080.63418981482</v>
+        <v>46081.46953703704</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Lululemon founder Wilson ramps up pressure on board amid proxy fight - Reuters</t>
+          <t>Former petrol station explodes in Anderlecht - The Brussels Times</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Lululemon founder Wilson ramps up pressure on board amid proxy fight - Reuters</t>
+          <t>Former petrol station explodes in Anderlecht - The Brussels Times</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 13:15:13 GMT</t>
+          <t>Sat, 28 Feb 2026 11:15:00 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxOQW1JMEhQWXZMSVhwSDRsNFRuTUhoUm1idnJFTjdhV0xMamRZTWV5S1MtRFF0U2RDUjVEM1lmV0ItSkowSFNydTlFbUdlN016bnpvMDJTRE1NTTdTNlNqQXYzQmFpYmFEbmNKcDVDeHhjSGdKLWtJR29WSFFOdW00UU9sSjdwQnZJbF9XdEFjWmNsdXdraVN1LW5CbnZQUVpDakdNOGdqc09XYXFxTVlfbnhPSk1JV0ZScm5QdGNXUUZudVNxOGV3YlVUSGpJRVJMcUhjZExFNmJvOWxHclVXS0tDdGtUWVVudHJaUzA5dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOeWFacnRqcHFrSERIbnNXbFV3QmJqSFI3RGpWcjdvQXNvWHN4YUdoTVFOdG1jYUcxbl9lLTNyNFNqMUNaekZoWkJ3Z01tZS1RMTQyeWh6TnhDV01mZ3RoTWkwdkRUZHZBMXVPcm1HdzdtaGJ5YlNLRE9hbnVoTWJNb1p0eHgzQXZmQURNQVBQaGJDX2FE?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -740,47 +740,47 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46080.5522337963</v>
+        <v>46081.46875</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>'We're crowdfunding to stay open and are humbled by the response' The Duck On The Pond's Hendrik and Julie on keeping afloat and being proactive! - Ox In A Box</t>
+          <t>EU withdraws Middle East personnel after US-Israel strike Iran - The Straits Times</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>'We're crowdfunding to stay open and are humbled by the response' The Duck On The Pond's Hendrik and Julie on keeping afloat and being proactive! - Ox In A Box</t>
+          <t>EU withdraws Middle East personnel after US-Israel strike Iran - The Straits Times</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 14:59:25 GMT</t>
+          <t>Sat, 28 Feb 2026 10:57:48 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOOVBBX1UyTU9oQ3pFdHdya2xyZ2ZfYmhDVXNMMDJncnUxYU8zVmQ2NEhYNnN1dlZCZndUMDZsWnNXZmNuOGI1aFhkVHNGUWtVQjQwOEdlWnJMQ25sOTdYRXBSdHZGY2hZOV9TaldwWUh3Mm9YOTFtNUpqeHdua1hkSm9zNHNaTnRWM25iOWFfLWhHU0Jjd0dLZDF2T1BzOG52RXF5QmhwSXZiSFRLdGdzbVVBN3ZUMldZRUlWMWRqekRYMTRBdG1BTURNOWlwMXFuMW10cTFGSlNxUVMzdGUxWU1nd3lRQlM1VTFxUllJZDNHSzhhRUEw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPWGpNTTQ1UHdHTlBFcEN0UjFybUlMUEVMbjRLVlJ4bkFHME0xQUcyd1FoY2V0NUNuOFlkd0xBNFptMkRQR244Sm52czhXeEJCZXNGR0s2ODJacmhyRk9ZVXZSMVZpWW9jM2tFMWxrVy1IdlZNYUJFdG5HTnV5by0zUXo2T0dFb0FIcTY2RkdZM0F3aENZVDNmdXhMWFhCQQ?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -795,47 +795,47 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46080.62459490741</v>
+        <v>46081.45680555556</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>XR JSO Village Search</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Extinction Rebellion" OR "Just Stop Oil" OR "climate protest" OR "environmental protest") AND ("Ingolstadt" OR "Kildare" OR "Vallee" OR "Bicester" OR "Wertheim" OR "Las Rozas" OR "La Roca" OR "Fidenza" OR "Maasmechelen")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Winston Churchill statue daubed with graffiti calling him ‘Zionist war criminal’ - Bicester Advertiser</t>
+          <t>World leaders fear broader escalation after attack on Iran - Manila Bulletin</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Winston Churchill statue daubed with graffiti calling him ‘Zionist war criminal’ - Bicester Advertiser</t>
+          <t>World leaders fear broader escalation after attack on Iran - Manila Bulletin</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 13:01:46 GMT</t>
+          <t>Sat, 28 Feb 2026 13:52:47 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQV2k2eHhuOGstTm1DWElsejVQdjhfQjJOZUF5YmVPM3F6OXhHNklFbmwweF9wZVlvempUc3pNU2c3QWhiem05ZEFBeldIUklUdlN6LUR4UzdpYUxEa081UC1jaHlJSXhTU3d3MWxyM0lQLWdoMjNLa1p0TFpoMkJOSHN3R1ZsU0VjSzZWTmwwa29JekZIczVnNHIyaWdwdExIUlFoc3Z0WnFiMTN4SjhpUGdPbi1TRXRiajhzTV9VaGdmV1R6VFo0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxOellfbDBWTVl2QTE1R3FWZzdEcEk1UG5TRHBjaVZHWlBYbmJXSUxxYmRkOEhRblluTk9FNEhwTjR0b0s3SzNKdG5DMkRPYlFud0R6N01nNjNXbHN4OGdyWDdzeDZDSDdTV2dvTGNvTXhiSXo2Z1YzcEVHcmRHT05reWJSVVJYUnE3SWdYTTlaRGU?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -850,47 +850,47 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46080.54289351852</v>
+        <v>46081.57832175926</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Organisatie Kuurne-Brussel-Kuurne treft laatste voorbereidingen - Focus en WTV</t>
+          <t>EU Leaders Urge Restraint on Iran Situation - Devdiscourse</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Organization Kuurne-Brussels-Kuurne is making final preparations - Focus and WTV</t>
+          <t>EU Leaders Urge Restraint on Iran Situation - Devdiscourse</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 16:12:22 GMT</t>
+          <t>Sat, 28 Feb 2026 10:41:48 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNeFhLZFBtdmU5d2NBRS1ZV0d0QV9XZDIwUGpGQlYzT0c3a1NjR1IzaGxKeXc1aXM1Yy1zTFhqazNTS25pay1OdmNVV01QbS1ZMnFpcGVYZDRRbDRNbzZLLXhjMnFCRy1VMEhjdERuNFBfc29BM0w2OGxrX0tCcUc0ZXhXemFXc1hlMy10TVZHVDRUTHRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPVmxfVHFUUUJvbm1wcGdwYWdFQmo3alprRC1JWHUwVnJfaDdYeUMza2hDQWkzQnI2WmpHQUhfMGlvNmNhUGZ2UGptRjBJMV9pNEV0WWF3d2g5ZjJBN3lfWmhDTngtUWZlX2VvOHBwUU8yOW5RUTlTVGlZN2dkb2gxZWtXX2xnSFozRnltOXhjTEIyQ1I1WTBreFowMXZISzJob0F1T9IBpAFBVV95cUxPVmxfVHFUUUJvbm1wcGdwYWdFQmo3alprRC1JWHUwVnJfaDdYeUMza2hDQWkzQnI2WmpHQUhfMGlvNmNhUGZ2UGptRjBJMV9pNEV0WWF3d2g5ZjJBN3lfWmhDTngtUWZlX2VvOHBwUU8yOW5RUTlTVGlZN2dkb2gxZWtXX2xnSFozRnltOXhjTEIyQ1I1WTBreFowMXZISzJob0F1Tw?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46080.67525462963</v>
+        <v>46081.44569444445</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Brussel laat Mercosur-handelsverdrag ingaan en wacht niet op handtekening Europarlement - De Telegraaf</t>
+          <t>Explosion à Anderlecht : un immeuble à appartements temporairement inhabitable, aucun blessé - BX1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Brussels allows Mercosur trade agreement to enter into force and does not wait for European Parliament signature - De Telegraaf</t>
+          <t>Explosion in Anderlecht: apartment building temporarily uninhabitable, no injuries - BX1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 20:06:00 GMT</t>
+          <t>Sat, 28 Feb 2026 10:28:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxQYld5NGlfWXlJa1lwcXZZMkJ5UEZYS3hxdXpPZktrSlNjeUZJRHJ2T0JjRWplWFdJajY4RDQtUGpoZl9zSzh6YWwzR193ZXkxMVRsc0JmSDRHUmtmQVd6VThqdGVOSWFwdW5jUWtTT3NyR25zV1luRkh4UW9ZTjd5MXJBSWdubHFRNXQxLVh1S2h1YldNVHZ3aE1sNlVqRE1yNGZEYWZuUHcwTnhPUHRYN0lHLVlIc0k0aUh2TnZodWxWaXVQbWNCN05saWVDUkk5MU9KbQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQalp1ODR5WVRrQVhPTmJpOFVaUnFnZDNQaC02bEhQTDkwRnJNcG04Z3VnVWYxOHFsQ2p0RnNScmtCN1NVV01OWXd1RDQ3S1lhNWxFUjE5OTR5d2FqSnBFZkgyellMUVRvR1gwUVMzV0Jfa1l5RFd1UDUzOUxPeW01TXJqbU5VZ3dfcjBOMXpMWWZMSTlUU2JQV2V5dTIxYmZ6WE5hQ3Uzc2pxN3pNem4zRzJ5V0NLeUFpc0d1WDBB?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46080.8375</v>
+        <v>46081.43611111111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Twee jongeren gearresteerd na drugsactie: “Cocaïne, geld en gsm-toestellen in beslag” - HLN</t>
+          <t>L’OTAN examine le renforcement de ses capacités nucléaires - سانا</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Two young people arrested after drug action: “Cocaine, money and mobile phone devices seized” - HLN</t>
+          <t>NATO examines strengthening its nuclear capabilities - سانا</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 09:07:19 GMT</t>
+          <t>Sat, 28 Feb 2026 11:04:15 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPbUg2N2ZHT1M3THRKTHA2LU1MbDkxRG01Y2pDSm4xVURHMl9tR2FsbExMdEQyRW1OcEhRRzlXRWEyUTVEN21IRUZfZzNhOHNCWDA4OVlWY2JIc2k2eEVwWGloRF9QYkFzWm9kRzdaSldSQk0tMzUxSHR2MWFUeDE4M3pCTndHcWJQeHAtWExpeEV0MUZ6QkVrVEFYZUowbk9RUGF3bDBxNDY4V3hsUkptQkdrWW8xc0RNLTJSdA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE5Wa0oyYTdqZXhoNFRESmxsaXFaVlZtVlV0cnc4bHdRRUhwSGQ1ajFBTHZ2b05RYWFyMFQ0aFYtektuX3h4a21vZ1NwVE9UaVlsYW1J?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46080.38008101852</v>
+        <v>46081.46128472222</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Justitie wil ‘terreurambtenaar’ van provincie Limburg langer vasthouden, rechtbank stuurt Maastrichtse verdachte naar huis - De Limburger</t>
+          <t>Accord UE-Mercosur : Emmanuel Macron critique l’application provisoire décidée par Bruxelles - Capital.fr</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Justice wants to detain 'terror official' from the province of Limburg longer, court sends Maastricht suspect home - De Limburger</t>
+          <t>EU-Mercosur agreement: Emmanuel Macron criticizes the provisional application decided by Brussels - Capital.fr</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 14:00:00 GMT</t>
+          <t>Sat, 28 Feb 2026 08:49:40 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPSXh3aHJsRzRjWko1SS1JUnB0Ym1fQTBRelIxZ2pjcjlENFB0V09jVzRGckJia3p2WGNReXFNajFZWTRuUF9KdElUdUtkTnJsOWtEZ3M2MzhOcThkLWJfOVJfdi03TFlKQTNqR0dDUE11b0k1WnppbW1kUFJnOGhyeURyN2RfZTZWdjZYb2ZYaWNTNHNmcGhzS0FqWUhWVTcxU2VfQ2l2QzdHZDl4MUVoMzdKN3JpSWRjcGt4bFdQZjVIdFlLWVBTbmFBQVJYTDAzY1BORmNSRmRrRGNWX3hxMG5NaHVhR1BUNFVRRGc5NjNYVDhIM05QQnp4NmFDeDhZV1lqbG5DMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPVmJieGlWamItX1hMSGVCczVyRmRYR0hZcGRONldodE5leXozQlJjY0pySTQzcEtGNU5VUF9PMTMydWVjcDR5QUo0bUo4cDIyZXVUOVhzVEdJVHFZS0FHVjNrNjNNcHZYNWJESzFqNDQyWWZIaWlzV1hhVnV2Nzl1bGYwb3IwT2pzbVpwRDY3WUduSnNwX094Yk84U1lsdVVJQk1DSDhQWTdfN3YzZ0pYal9kNllab01BcFZHb2FfZmJhTEFodXF2UE40QzA4VzFJMVRPQ2tWNA?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46080.58333333334</v>
+        <v>46081.36782407408</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Brussel laat Mercosur-deal ingaan, ondanks verzet van het Parlement - Het Financieele Dagblad</t>
+          <t>Meurtre de David Polfliet : crime homophobe ou "chasse au pédophile" - BruxellesToday</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Brussels allows Mercosur deal to take effect, despite opposition from Parliament - Het Financieele Dagblad</t>
+          <t>Murder of David Polfliet: homophobic crime or “pedophile hunt” - BruxellesToday</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 11:22:11 GMT</t>
+          <t>Sat, 28 Feb 2026 12:04:37 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQYlpwQ2JtcURVTkVOYVR1Skh1b3VKUDYwTkFsZGxJck9kS2pIU1VQdE55OURUblAzamdrbENJNDMtYnVGRURuOFdsd2NCLXNobVZQaVN4Yk9GcGNlLVhTMUMzRlhnU1lfS19YVjRxdzY3d18wWmhaVVpOOThhT2JfVHM5Q0hqVzhFdmQ3dWJzV2YzX0VON0gzUVEwNGZmdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQQlNSV3ZjX2FYSm1xTUI5TWJfSnVJVzRxdEZzRnU3azNQUkNPMUJwQnVFR21OLXdWQ2g1YmRQTHBaTndNWDBBRndvREVjRUxRdExNOXptbjIyT2o3Y1JXWmRCWFFQTWxRLTFBQlFCTlFSdlg0OV9ucUc3NEJ4eVRIYTU5RDdTM1RGWEhKS2pOeHpRcVMzcU1nQWd3WQ?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46080.47373842593</v>
+        <v>46081.50320601852</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Onboarding in Automotive: met nieuwe cursus in één dag klaargestoomd voor baan in de autobranche - Automotive Online</t>
+          <t>Warme maaltijd moet rust en verbondenheid brengen in wijk Ter Hilst in Hasselt - VRT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Onboarding in Automotive: prepared for a job in the automotive industry in one day with a new course - Automotive Online</t>
+          <t>Hot meal should bring peace and solidarity to the Ter Hilst district in Hasselt - VRT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 09:01:34 GMT</t>
+          <t>Sat, 28 Feb 2026 10:26:04 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOZzJCSkFmOUxMeXVlTFBxU3VEMmtGdmt1Y0VXczh3VlZiS0VhUW1JYlRrSkFCN0Z6czF0QXprUEw1aFlLZWlKNjZfU1NfNlB5UEVxU2YzemtIM0QySjR1cDNQNUVQbEwxbmtXT1ZCVUhOdlNnNXFZUUxxNzM5elktREhzOGh3b2RaTTV4azl4NTQ4S1FHM2ZwTUszRkNnOWJHMHIxM2VmSkJEb0NnUVZERko1Y1J0ckdWbko5aVBSYkwtcG5namdpYXJ0ZnhQVHNwU2xlenQ1em52NEJPSjVEdGVrZ0dVWmFKd3kwcnlHWGpLbUFS?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPZlNReUNVMGNsV3ZNRlE5YXMwcDRuYnppMWlQUmxVT3VDNzNfYW9tVGFyTlBaUHFocFhKQ3BjMlotMHJOR2h3Mmw4WWhnaldSZnVNY3FwZHo0VFB1NEpLVVQwU0ctbk1iZVZyYXRaOTJ3OGJYeEJiMmhMVmxhWUN5c0hVT3pPU010SlMyOUE5NzdORDJYTGZZWFlhbEhLQ2VwcXVvSzdUdEo?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,38 +1189,38 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46080.37608796296</v>
+        <v>46081.43476851852</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen French</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Euorpees Parlementslid Rihards Kols reageert fel op open brief van Orban: “Richt u tot het Kremlin, niet tot Kiev” - P-magazine</t>
+          <t>Handball (SHL) | Visé, la révolte avec du sang neuf, à Hasselt : « On va disposer d’un groupe plus étoffé pour les prochains matchs » - Sudinfo</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>European Member of Parliament Rihards Kols reacts strongly to Orban's open letter: “Aim to the Kremlin, not to Kiev” - P-magazine</t>
+          <t>Handball (SHL) | Visé, the revolt with new blood, in Hasselt: “We will have a larger group for the next matches” - Sudinfo</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 18:56:32 GMT</t>
+          <t>Sat, 28 Feb 2026 11:00:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxOeFRubVZ0dkQ3WnlCaDIyRkNhdW5ZeFFhTVZHZmhwUGR6ZldHYlh4c3YzaW40RmlaTlJRdG1EUGFub1dMZ3FUQ2o0N1ZYTUNfTWg3ZU5PaW5lWlFjRnZUUUNKVjBzbHh0THBZNU9lLVVjUE9GWkhLbFJ5QWMyT1dob0h6MHpfWDFEbkxyYVF2Vmx2V0dScXRmbjgwMEJ5d0FxNVFuRmVnZUtuY2dBLWYtUnlHQ2FBVnNSS0ZlM1U4dWlHcHkzdE16VWI4cmZUbldGUEtWRmFNdEVGcEhHU0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPV3RvZjJUUnJ3dW1oSHhBUlliNDBFS0ZHUkZmWEZsT1lIWlVXZVZMRlU5QmdRS3ZZSjV3SXR3bzJUa19SaDdPd3VRNFdhS25YM25nTGVJRFFFeFIzZk5FdGliNmhfb1B2MThMNGJjSk14cnJVVlNFckVLSDN3NWJQcFd2ODJKTUx1VXh0M1ZsS3B3Q2Vjd3lQb3BNN0xHbEJHanU2b2ZBMktqMm82Nnozb2d0OF80ZURGdURmMHU4YVh0MTlKclhlUg?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46080.78925925926</v>
+        <v>46081.45833333334</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mandelson geconfronteerd met EU-onderzoek naar handelsrol in Brussel vanwege Epstein-banden - ekhbary.com</t>
+          <t>Highlights: RSCA Futsal 21-1 Sensei Sushi Anderlecht (Futsal League) - Anderlecht</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Mandelson faces EU investigation into Brussels trading role over Epstein ties - ekhbary.com</t>
+          <t>Highlights: RSCA Futsal 21-1 Sensei Sushi Anderlecht (Futsal League) - Anderlecht</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 19:33:05 GMT</t>
+          <t>Sat, 28 Feb 2026 14:10:27 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNbThmazN2dEstYTc4M0s2UFc5ODBTRkw2UmhwdmhwTTAtSUYzVHdRZFU5dkMzVUxZRTZPcmFSYkJxTEsyREdULV9zSGVabVBjX09wSDU0dGxlcHd1ZmhhaFdJdWxyX0ZETjNrRlRJY0VRakJOVmlDY2piMFVKMUxON3IyRXBmTVdLcEZmLXF5TzZSOXN2R3diVHJ4YXduXzROQ0hFMUc2LVNSUkQ2bFlzVHJnMFpzWnQ3VnlLX2pXdC1kVzJ1SG5FNWNGbm4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxOZW9SV3hPdlpHN0hfaVFlR3h0aVlVMlA3ZzYtLTFObWY3a2FpdnRYOUVNZktHMUtleGRaMF9va1ZsZ3NpR3BTd2hkMS1fMUl1elhrQ3IwTmNqN2xQWWhLYzlGTldiLVd2RTZCTnlieFdQUWVGM3c2SkE0d3NfVDVXMmZHOEhJQ2xfc04wNnB2d05MYnEtUzdEQg?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,52 +1285,52 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46080.8146412037</v>
+        <v>46081.59059027778</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Brussels orders probe of Mandelson's Epstein ties while EU trade rep - Yakima Herald-Republic</t>
+          <t>Waldaschaff: Polizei sucht Zeugen nach Angriff nach Faschingsparty - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Brussels orders probe of Mandelson's Epstein ties while EU trade rep - Yakima Herald-Republic</t>
+          <t>Waldaschaff: Police are looking for witnesses after an attack after a carnival party - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 10:19:46 GMT</t>
+          <t>Sat, 28 Feb 2026 10:06:38 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxQOTkxQkkzaTA4TGF0U3o1Tmp1dEJpWnZKVDNuaGFFRldZRXdwT0VYLVpZNlpGVEtmbmJXaDRCSkNzNmhNTk91eGt6bTJNbEl3NDl3QzRhQ2Fsdk14QkR1U1VRT0J2RDBMZFZGRGptZ3BqOWpETDhhRVVWai1VRjVBVWJaQ2diOFhqSVhnOTFfNHlVcEwtOTBhSGpWdjluR0tpT0liTnkzc0JYMWxpX0s4UWNvd0JsNl9uNWlDSEdXMTY2NVJ4c1dsazFBU2lQODg3cWJfYk4wYnlVYy11MHFfbE9KUGdTLUdwSVNLN3hjcF9BZ2FUbFg1MUtSRUZzMlhIRERMQtIBigJBVV95cUxPemJzLWRsMnIyNDY3c3JnOEZxT1ZFV3ZjMzRaTkxIS0dkY1Nua0Vvd1QwQnRsZW9pZUdTQWZjaHBiemJwNGJsSlhaMHFKQ0tWMjlMQUdxUkhsaVdNanZ0UW41Rnh5NGotNVpTUG1ISXdYZjN2cEttX0hZZ0ZlUjdNVlFyc1k2STJCUG5OOVI0M0xQa0RlaWgzdUtvSGhmcHplV1daWkNfT2NmNWs3OHBfbUNpakRtWGV4c1BGN293MkZXVERQcjVfMWxLdnhMcWp3NnhPTFVHYjhLUFRsaTZiQk5FZG1wQVF3d1V5c0tUX2FVNnlwM3JESW4xX1VfUlYzaDVaUTRlam1ZQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPT2JycGhsRDBGX19melROOXNVUXNVWE9VTGszVC1JOG5lU2x4UHZBT19hU0w5a3RQenFwendXc2pPem9DMTdRc21RZDZUS1JFWnpMaElhcUlxUV8yVXhTcmNtOGZIcTFHQWhmNlhZc0JJWlBTS3M4WThRY1JqbTlfbVVwRGp2VE9OeUkxVlF6ZGQxLW5RejJIM2FhNjFpSURBQXV2SmJXWUFmbjl5QmlXN1diS1FoWVNpYnNOSTZsaEVSQQ?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46080.43039351852</v>
+        <v>46081.42127314815</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EU THREATENS TO HALT FUNDS FOR SERBIA: Emergency debate in Brussels over adoption of Mrdić’s laws! - Serbiantimes.info</t>
+          <t>Streit am Morgen: Nach Messerangriff in Würzburg keine Hinweise auf Psychose - Bayern - Neue Presse Coburg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EU THREATENS TO HALT FUNDS FOR SERBIA: Emergency debate in Brussels over adoption of Mrdić’s laws! - Serbiantimes.info</t>
+          <t>Argument in the morning: No evidence of psychosis after knife attack in Würzburg - Bavaria - Neue Presse Coburg</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 10:06:28 GMT</t>
+          <t>Sat, 28 Feb 2026 09:15:48 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOYzVLRnJnam1rRFB4T2hoSFUyRTZjLUhlZlBsTEM0VDRySW55UGtRUVFydVdsbGFrTElESHBCN1NTZzBpV1NPbUs0Q2wxMVh0N0xPMDBPaThmZWpNNzBmdkR3T3lCYkxaQTFqOVl3Rjd0eFkxSXU1a2pqZjZ3eG5Nd1dDbHhMRXNaQUVmMDJFRVQzeGtKVXAzS3dHbEE2YUJlSllOR3Z3QzdsRWdDVjd5c09waVAwOHVJbFpTRm1KQ0l6eDA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxPZXhycWdQbTY3cC1kWTVIMXk5ektJb1FwMkZHRkt5NE5JcDkyNWxxZU1qbHB6R25VdWpUWFU1YWdGVnVKQzZ0RjRyM3RQX2xQcm1lZklFQ29KLWE5MUpuenpiLTVpS1RCQldOX2xPcjNyajl4Y2pPNnJ5SjRabm5zNU5YMHhiMlRqUTV5R2dnY3VVbU9rS0JtX1FUeXZVYV9IQWNvWnIzVzMwelRvZTdEZmpvNkcxY0ZvR3V0NEJzcXFnWi1pM2JscmRQRXVhb1dPaTgwLXg5cnJfLVAwcV9lOGNsM2g?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46080.42115740741</v>
+        <v>46081.38597222222</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Alertes à la bombe: la tour Montparnasse et Sciences Po Paris évacués - 7sur7.be</t>
+          <t>Weibersbrunn: Ausweichmanöver wegen ausschwenkendem Lkw - aschaffenburg.news</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Bomb threats: the Montparnasse tower and Sciences Po Paris evacuated - 7sur7.be</t>
+          <t>Weibersbrunn: Evasive maneuvers due to truck swerving - aschaffenburg.news</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 16:57:59 GMT</t>
+          <t>Sat, 28 Feb 2026 10:09:22 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQVzBXYjBsbHhQa09jeElaeEVUR2JYdFlza1NFUzIzeVpLT1JnbzNRaDRZaG1WYUxNemg2eE5BVzNYZi1CZWZGcGlWMEgyUjRuTk5QOE9XX2x4bnN3dFlHUThIMklYUWg0c2EwVG9xNkxWdmwxN3RNOWNvb1RMeHB6UHpBRWVnTkU5QVJtYmtuaXE1V1I5enVHWFN2czNDaHhyRFBVTXZES1lmY0lNOG5zWVN3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOSVRRVGwzbGUxTU1zaE05RWRzYWdvMTFONWYzOThvNHg0TjdPbXM0ci0ya1BCNllwdnhTT1lhcXluLWM0eEVNWTVsRXZOYnlBeE1hOWZiMVU2Q28tblg1S3pRNkxPWmc0ZjJWUWdZVFJ3UFI3Mkxaakc1TEJBenNQekRnU1lsaDhNMzB2amx0T0dvM0lPRmRLakc2VVVWNHY1dXBHaWVVQ240Q1p5V2h5Yk5JLTViMkVqV1E?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46080.70693287037</v>
+        <v>46081.42317129629</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Buurtbewoner die mollen wil verjagen met gasgeurmiddel zorgt voor evacuatie van school door sterke geurhinder - VRT</t>
+          <t>Livecenter - Adler Mannheim</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Local resident who wants to chase away moles with gas odorant causes evacuation from school due to strong odor nuisance - VRT</t>
+          <t>Livecenter - Adler Mannheim</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 11:31:23 GMT</t>
+          <t>Sat, 28 Feb 2026 11:42:36 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNQk1IcU50a1AyNGxpaTFGWmFqZ3RkbFJURjZISHcwYlRlWEg3amRkRWU0TEFQVDJGeWsxQTZZeG5nVkQ4RHItRmVhSjhaQWc4eDQ0VDkyZzdBM0syYm5IVklnYlF4N1NFRXg0aEhvcTRZY1dCSHNZMTd2UlNDMDVFMF9WSWplb0k3WjJOakNEUDJ1QnB4Y1FsVlptcUxmS3dUQXk0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiTEFVX3lxTE9YM3hUZnd3U2M4OXZHTFNnY3BpdV9Cb0c5UnFWOUd4U2cydVQ4QldYZVpITTUwV3JYaXBKcUFKdDhFUHFEZDExWmhkZ3U?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46080.48012731481</v>
+        <v>46081.48791666667</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TC Hasselt - Un homme de 21 ans risque dix ans de prison pour tentative d'assassinat - DHnet</t>
+          <t>Liveticker | SV Wehen Wiesbaden - FC Ingolstadt 04 : | 26. Spieltag | 3. Liga 2025/26 - kicker.ch</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TC Hasselt - 21-year-old man faces ten years in prison for attempted murder - DHnet</t>
+          <t>Live ticker | SV Wehen Wiesbaden - FC Ingolstadt 04: | 26th matchday | 3rd League 2025/26 - kicker.ch</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 12:15:00 GMT</t>
+          <t>Sat, 28 Feb 2026 12:31:44 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxPMHEtTjFPMk1xSXRqWFdWLUZJbVBOOGJmbDlmNm5RU0dfclJKV014SUJYdWZuRXkwVGlmUDNPejRsclFFeGRVVnVOdkpCOThNbWpJWDZFaDVEMlVHT2xTUXQ3M3ZEeHBWUER0S2RBWFEyQlFXMlhNZTVDdWtqYV9NYWQ0T0dlME5CWmtqWG02NC1ScjVNUFRXd0FmZFF6cWZkd3JhdDdDelZkOUxybVFaS1liRy1UUWdPRWdleENOUVBvek1rVGNiQURJOUloeXNlRlBCQXUtdFNMVkdvOXpWRHFRUFEzdXdzTl9ia01iVmNIUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE96UlJjV091cnBqbDNKWXVDaTNQdnhrVnZpOFNFTnQwdm0yME9WRkx4ZXh6SXlROWtvNDJ3MEdIWDVkelhHNGtqV0gyUEs3YjhJVVh6QTFsNmFYNFZUcEVYbGJLMzJvWDNqVlNEX3ZKb0NDcEYydVNBQTgtVDAxQQ?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46080.51041666666</v>
+        <v>46081.52203703704</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Jong Gent - Patro Eisden Maasmechelen - Bulinews</t>
+          <t>Neues Projekt im Tierheim Ingolstadt: Kinder lesen Hunden vor - Donaukurier</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Jong Gent - Patro Eisden Maasmechelen - Bulinews</t>
+          <t>New project at the Ingolstadt animal shelter: Children read to dogs - Donaukurier</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 18:17:48 GMT</t>
+          <t>Sat, 28 Feb 2026 12:05:20 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxORXp5bGdmTllvNE5KUW16Q21Zd0NQUUREU0phUVMxMnpKQmk2dmFQT3hOZ2M2TklESks4cXRNbzQ2WXV3TmRXNHZXYVVrX0V1cEM3VU9hZy04VXV2RnJPZklLX2R6SEZkZTR1Qk9qcFREOXkwb2M3Mk05NW9iSnZnanh6TUFza2s?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQb01ZY3MtWUtzYnpZNmMzUGlhV21HRmMzNVhLcnFnRlcyZm9wRnZQZUl3cU5pcXlrTW5xSUJBWHA1djh4TjVoUkV3UDh6QU9nVDFJdDc2OThSVEtadWNnbGtuWVVISGlsSmlhRENIcDZaUTBfZEpWcmxibkxGTXdITVJwYlpERTZ3OWc4aU1wbWpkTndCRXdKbkpQbDVzUF9XdUgwNHYtcGtUbUNuSEdXRjhGVnpRUQ?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46080.76236111111</v>
+        <v>46081.5037037037</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Match Centre - Transfermarkt</t>
+          <t>ÖPNV-Streik: Auch Passau, Landshut, Regensburg und Ingolstadt am Samstag betroffen - Wochenblatt.de</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Match Centre - Transfermarkt</t>
+          <t>Public transport strike: Passau, Landshut, Regensburg and Ingolstadt also affected on Saturday - Wochenblatt.de</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 18:54:07 GMT</t>
+          <t>Sat, 28 Feb 2026 08:25:21 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBIQ0R4X1lzd0Y0R25OX050b3RSSFdoRld3ZDk0Smd3YTJxU3JCeHJrSkxUYXAwRnAzenhJbWNPYnE2dTlXQndLVnFBcGU1elp1Z2F4LVRrTDdhVHYyZW9fR1RkUTc5NWM5Yk5V?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOTzNQVm1lMVVuZWdyaXRJbzhSMTJ1RTMzcmxBWHNXZTdsMzZ1bXYzRlpUYVhwRHlEMTVjT1VYMFJDeVFMcmpPS0Q5eWRlZjhoaFNsN2NYaGlzaGVhZ1VCMDE0b0d0XzNGSU92Sy0yUkRRN3ZzMVRkaFpIYzhydmtTUk9PMmowWWVPeFE0ZmpFUEdKd0lEV1kzWjRsQ3kxNkhsNEJWU1lUU3JVd25SZ3ROWTY4RzZCQ2NXVFhjc3pMOTZLbUtHT0hLLVBMajgxOFR4T3M3eXZqU3BHSmc?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46080.78758101852</v>
+        <v>46081.3509375</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Poppy Ackroyd unveils new album Liminal, lead track The Unknown - Live4ever Media</t>
+          <t>Kölner Haie - ERC Ingolstadt (Highlights) - SPORT1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Poppy Ackroyd unveils new album Liminal, lead track The Unknown - Live4ever Media</t>
+          <t>Kölner Haie - ERC Ingolstadt (highlights) - SPORT1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 08:49:51 GMT</t>
+          <t>Sat, 28 Feb 2026 10:00:40 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE42WEFhTXNKR2E1QUpyRjhKSzVZUkhvSUc2RGdUMjhyeGxWQUNIbVdHc1ZaNDZCZ2NDTjFvTGhJZ19vSkZyWEpibmpOYXdUZ0UwRWJUSTFqRzhkTlR0UEdFYlMxNlRObU5naUlTTEhaR3k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQOVhMT0tOZUdKeW8yQ0IxZVFYSmoyTE1Ec1g2cnV5Nnd0bThZSnZJTldyZkRMVHlFWDllOHhEaXR6YngzSWxSbDhGVjZkT0wxUTJRVWtnajh4cnRjazc0OXVsN3NWSzJyWk5JTHlVNGMyWWdNYnh3c2FDNklNb3JvdUJNR3N2b2ZlaXVYZzV4MlplSnJtNXlLNkdfRmdZY1VvYWtJbnZhT1dITUwtZGhaYmd3?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46080.36795138889</v>
+        <v>46081.41712962963</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
+          <t>SV Wehen Wiesbaden - FC Ingolstadt 04 im Live-Stream und TV: Wohin gehen heute die Punkte bei SV Wehen gegen Ingolstadt? - News.de</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Assassin’s Creed maker Ubisoft cuts jobs, sparks strike - AOL.com</t>
+          <t>SV Wehen Wiesbaden - FC Ingolstadt 04 in the live stream and TV: Where do the points go at SV Wehen against Ingolstadt today? - News.de</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 11:12:30 GMT</t>
+          <t>Sat, 28 Feb 2026 08:56:34 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNT1h3QWd4eHNRQlFGRDh4UExSNTZiUHp4d1R4c0lxcG5LWEhsQU5sZklnUWlBYzlOV2hNREZ1Uk9haW1WdlQ0MUF5c3E5Y3pPTFc4czRwd3dBOGpCS0M1RkdvaHNXSUZNRi1fT19xZHVJYThNRk9fNmZwQXIxc1l5Umxn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxQQ083NUlVRlV6TmROOF9FeUtwRm9YRFUxM1F0R3VwY3JIbkxtcGRLY3Z2XzZwWThnSkF6QngydUcxSXZqU1RVTUp1UnkxMjFwVG9VUVA5eTdmWDd6SnN2M0hhenJrdEhmZ3ZqV2lWeXd3cXZWNkNuQ1liZFU4NzhZbXVxODNRM24xeUtUbFZqbXFxNXB1TnJUeU42MVI4VGpISFhKRUpfQnhUOE5Vd1lrUjRYZlRrc041ZnROUDVZcHYyN3NGcWNFS1pNRC1wMEdDOUxZTjRLOTVKalNJd2VoM3BFSXZ3OFUzRTMwSjhoMmpUZm1jM3JYZnZlMlrSAYICQVVfeXFMTm9hY2p6RzlrVG1VcnQxSmJPNklqREFXRWpKa2RWbjI0anFlSzFoY28zajc3ZGNEcEd0OE05VWxIQkJqTFQ4NFFfd1F3VUlWVXRDWGU0MEtwanVkLWRyWEFna2REZnFLWHNuM2thb3VqZXhDYVVPbXp4WVFuclFVdXY4VW1MNFA1VWNiV3JSVmlYUThXajhZRkRwNWR6RGlKa1owdUtoMTUwZWlnQnRwTFM5T3EzTlRWZTdZQ1UwLU8xTGtvN0k5OUQ5blpJQmNHTGI5dE54azJQcVFFRnA5aXB6WXFpaWF6VHI3UXE4VWh2TXFSUk5QV2ptSDAtRzJNRlpB?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46080.46701388889</v>
+        <v>46081.37261574074</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+          <t>Verein Schanzer Wildparkfreunde in Ingolstadt gegründet - Donaukurier</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Margot Robbie Stuns in Red Gown at Wuthering Heights Premiere - AOL.com</t>
+          <t>Schanzer Wildlife Park Friends Association founded in Ingolstadt - Donaukurier</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 07:40:40 GMT</t>
+          <t>Sat, 28 Feb 2026 12:38:02 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE8waEpNdEZmMmtDMFhIVzRBZ0QteWtGc0JMUjRFT2hzUXNGa25Pa2FPNzRHSWtUZVVvcGNORnNvYjFVZ2dIeVBMNEs4dTBvdVhmYUt0UWx6T0RQR2daak9ZR2p2SFpZU3lRS2dNaXJ0M0pSMGM3bmcyeEJvT1Y?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNVmtlZTRTTnVZTUJsQ3FVMU1uY0xnMzBXcXFweHBJSmhVMm5pLUZ3MXhOejk1eXA3dUh2YTN6dDRabXJTbFQ5WHpsUThDdmNxSTNKZkwwdmZVYVA3dGdhSlh4U1hoaWx4VGt3aDhmV0x1OHFoTEZ4YlVsU0NZQXozbEpMSi1MazEyN2JuSmtIb2FfOXduZXUybXN0dGZWWUxBWjFhMm5VbXhZWUJKNzVTNQ?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46080.31990740741</v>
+        <v>46081.52641203703</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>79-Jähriger vermisst: Polizei vermutet Ausnahmezustand - Nordbayern</t>
+          <t>„Die Milchstraße“: Kammerphilharmonie Ingolstadt spielt Piccolokonzerte in der Fronte - Donaukurier</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>79-year-old missing: Police suspect state of emergency - Northern Bavaria</t>
+          <t>“The Milky Way”: Kammerphilharmonie Ingolstadt plays piccolo concerts in the Fronte - Donaukurier</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 17:24:40 GMT</t>
+          <t>Sat, 28 Feb 2026 13:07:52 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNaTZUazctejdYd0p0VUQybmYxWDJlZE9ocnZjRVdMOTlHVTRnbWZVeVo3NmR5WTNNR3BJNi16QkZ3V25oWTJWLW5CRVVwOU9QQXU4X0ZpM3UzX2tJTzNIdXZtalVSSTkyZHVKZldDcVBPbGNkR2Rab1pLX0FKVGc2cEFqc0ltRkwxSF9PNXZ4bm9vRV93ZWxuaEZKbHBESVhXZDJiV3BsV2V1Ync2U2g5WTBaOXRVZzlxZ25WZThJemY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiS0FVX3lxTFB3amdWVGdjblNUdGNEWDFBc1JqRGpRazVvUTE2WEpDQ29IV281alc1MUt1bGdZZ21fYzFFUTlrM0lmdzNET0xaZ21iZw?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1904,38 +1904,38 @@
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46080.72546296296</v>
+        <v>46081.54712962963</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Würzburg: Gewerkschaft der Polizei traf sich zur Versammlung - Main-Post</t>
+          <t>Eishockey | Spiele - Tabellen - News - Live-Ticker - Kicker</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Würzburg: Police union met for a meeting - Main-Post</t>
+          <t>Ice hockey | Games - Tables - News - Live Ticker - Kicker</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 15:13:17 GMT</t>
+          <t>Sat, 28 Feb 2026 07:48:37 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxORXY4Y3Yteko5T00wam1IbXhyNk1FSE9IVkNZeThtUkNORzFQS0x2MUczUm9jdUVNLTFZNUVfUFk4Qlo5NURWLWpGVkVDdVNSZlNNcFJEd1hJS0dwRUg0ZWg0VGZ0cTEyUHAwSEZTWGlqaDBSMnhkM0lqT2xuNUp6eXRjRFh1dUpXX1JscVVSUUJ0Z2E5VlBHVUVBeU42ZWNnNmVVZF9NQy0zeFlfN1VlQW12WWVELU42LXR0M3VZRUo2MHY3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiVEFVX3lxTE1NN2pCNzRrN3VGS1NHOFFoZXJqeFQtMDJ4QUh6MmJ4ZGZUeXpvM1pub1JZTGJPcktsbXUzbGR2X09uWTMzNGh6ODlONmotb0Q5SDlySA?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1959,38 +1959,38 @@
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46080.63422453704</v>
+        <v>46081.32542824074</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Ingolstadt German (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt")</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Marktbreit: 79-Jähriger vermisst - Radio Gong Würzburg</t>
+          <t>Gitarrist Michael Schenker gibt ein Konzert in der Eventhalle am Westpark in Ingolstadt - Donaukurier</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Marktbreit: 79-year-old missing - Radio Gong Würzburg</t>
+          <t>Guitarist Michael Schenker gives a concert in the event hall at Westpark in Ingolstadt - Donaukurier</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fri, 27 Feb 2026 13:05:00 GMT</t>
+          <t>Sat, 28 Feb 2026 07:37:58 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBZeTVpOWVYbVhHeGxaSkV4SVUzRWJTcUJURl81alBxT0NTQUtVenhSQ2s4VHJjMHdsS2JuOVFUTnhscjdUcUNacmFyUnRkeHdWc2hQRUFnSFZiTXMxZTJXTWtZRXFQbnpLSGxsTVdjVkp5T1JZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiS0FVX3lxTE5mcW5KRUJxa1FfYmZGMU16SkIyVXdKYkh5Q1Q3dm5sVWxHY1UxVW8tZ3RRSmpLeGFQOEVmU3VvUFEzQU9kNV9yWkNTNA?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2014,447 +2014,7 @@
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46080.54513888889</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Polizeimeldung Kitzingen, 27.02.2026: +++ Aktuelle Öffentlichkeitsfahndung +++ - News.de</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Police report Kitzingen, February 27th, 2026: +++ Current public search +++ - News.de</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Fri, 27 Feb 2026 14:35:02 GMT</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNY2JRazRGcUxpZXhTNlNhNW5Lam1HSDFzLUlLLU50NmZ5MFgyLU1RM2tPYTI5Mnc3b29pcS1fM01WQTFlSzlsSUJUc0VybDIxTnU4T09DOGNpbDRwbXV6Q0hEcUxrS2xYNm5neUt3N2c0b3pKeV9TcmIybDNYUmFodDlhdDk0aERtczRlZkJKd3Z2cElaY3A2TV90U25QMTNPcjNlcU5ROGREQ2JabnfSAbMBQVVfeXFMT0piOUtlSUJHaThhRmpwUEowdldVY3p5MHMxR1hYM3ZmQXRFR1lzX3g2R2N0OW9nM002WDhHT0Z3bW5IVlMtQlJrY29EYlAxSmdQY0h4T2dxMTlTbXl5a3lIdVVXV3BKVnROXzZ0TkVsUmFNd2o1T2JOaFRydkVhNnJmRzJORFlfMW12dHZiaEx0Vy1pUzRVMGhoOHRhVTBOeFNScjFWYnpTUDdod21XMUo5T0E?oc=5</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K30" s="1" t="n">
-        <v>46080.60766203704</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Polizei-News Schweinfurt / Würzburg / Nürnberg, 27.02.26: Schweinfurter Zoll stoppt Lebensmittel-Kurier mit ungekühlten Pizzen im Kofferraum - News.de</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Police News Schweinfurt / Würzburg / Nuremberg, February 27, 2026: Schweinfurt customs stops food courier with unrefrigerated pizzas in the trunk - News.de</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Fri, 27 Feb 2026 09:36:02 GMT</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPM1RDOTB3eGxGY1ZOa2NmZVhXX28wWHZBZjhmUVBaVVlseGtWa1BtSjZVNDM3YUlSMFVoQ3kzTldhRjFQOFI3WWFwRVJEcWpvU2M3aG9fVUtzSzJvOXFfSmkzUTMwelJBcXFramhneGxuZ19GNFpUY1d5c2VKSW9UZ09wSWNuVEhZODJySl83cHNXVWJrWlI0S294NUV2Y2U0SG03bEV2ZjJDYUJpUF8wdUlBem5KbEZjR0xrcGlGeFR5Qy1kRXU4ckZZN3o3aWNyRFNad1plMDFWMnFBZFHSAeMBQVVfeXFMTmc0UGhYTEdaalNuQUpjSXJfaXY0T1kxY1AycVI3c0FqNWozaUZVTzRVV1c2aXYxaTNsSk5fYjdqSENtNVR3TUJtR0dOUGwwUTZsbTBmeWhHY2xiRUs4Q1kzV0lUTjBrYVlSVlNxZUE2U2V6RHJOQi16eUN4SDhtbzBXTU5sU3ZUUkYxVDZKVDI0NGpfOFhJQnY3ZDJuN255Rm1SVTA5WEVZOGJraXNkYjhsX3FkV2dmRXhIQkhydkdBcGg3SVduV3hkcDFxd3JqRkVIaXhJTi1fUlpSa083TzQ1bXM?oc=5</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K31" s="1" t="n">
-        <v>46080.40002314815</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Demo-Termine heute, 28.02.2026: Hier gibt's am Samstag Demos gegen AfD, Menschenhass und Rechtsruck - News.de</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Demo dates today, February 28th, 2026: There will be demos here on Saturday against AfD, misanthropy and the shift to the right - News.de</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Sat, 28 Feb 2026 05:26:59 GMT</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxPNThVQm5RUm9BYU5RaVAtMTRuMzhNUV82NFlJRVZidVZqOGZ4ZWFnN2NEdGk2cUxIbzRmbUNhWXJtalhqVUxsU3ZqM2wzeTBLd0pScFB4TTlLblJLZ20xaWo4OTJBWXRrYmJYR2dSRnRyZDViT2gwTmNXdGNHT2xHeW00MG9ERjJpRVBWNU1Lak9PTldOWHNxSW1ZVmhVVmlrdndtSFlLMEpLTUpiX0xNZG54bDZwbnBUSE5ZY250VVZidUFYc1RRSXVBZVJhVW44cFhWLXdOQWNVTkhvaTA5T0RFTjZWVnROS19MekFWV1J4N1lnTHY2by00R3IweHo5YXpZ0gGIAkFVX3lxTFB5dmV1aEkwUGx4TExoWUJ6Z2FTbm1tTGtRNU1IVnBZUGNNV0F3TkpKbTc2UDVrdzI1Y1hZbDZvVnB5SlBQMF96YVhUbG10dDJoUVc5RVBSa2ZQNWZSZWhmaXh3YjZQcmtwd3BoXzNJZXdHa0UtMno0RkFGaXhmVlRuQ2p2Qlk1STdjVlVtcnVlcXJ5WjBMN2laZkZvU3RuX1ZBTDFMSkRZYXV1emFJYXd4cjdJM1hiNkd4bVpCX09rcWN6ZmUxdEtJaVlzS1pZT3pfZXVhTTlLV2JocGozUFBndEk5QVI1SVhoNDhJRmdVZENCVDZIUjd1aFp3Tm5fX29JeWU0UFhoeQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K32" s="1" t="n">
-        <v>46081.22707175926</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Local Town Wertheim German</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Mobile Blitzer in Bessenbach aktuell am Freitag: Hier nimmt die Polizei am 27.02.2026 Raser ins Visier - News.de</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Mobile speed cameras in Bessenbach currently on Friday: Here the police are targeting speeders on February 27th, 2026 - News.de</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Fri, 27 Feb 2026 09:19:07 GMT</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxQN3loSDQweXZybkRTSHlpM3k5eEdMZThLVTZGcWJIRGV4OURiMTBxOThwdUFGcEdiLURKOHluU0hJRVo5Q29vZnRoYTNKRVhsM1NURW56SDY2TGVRSVhQV1lTU0I3a19yYjZyUkduQS1yXzFMVGM1c1BHNjNhMlRiQy1pNFNmN2xuZW1JeEJkb3gxdVBaUk41ZHRGejFoWWhkdEMxcEtwQmY0dWMzcmR4RkdROHBZdjc4NFVUYzlOYVNtaHgyRUVha1BoQ1dlWjBFcU5RdlpROVRkTUdmeXBkcG12cFNjU2VBcVllR244bUpKTkRFZV9GT25B0gH_AUFVX3lxTFBaNGU3anh2QW95X0J3aTVubTJiOVdEeFZjUFhFZjdyRVAwV1J0TW5oMlRVaXRhV29JSi1HbDM0OWJyaGx4QTIxQnJUa1RnZjlCQkdTX0lqdW1HZjl1LUtMcFYtOFhwaG8xcEZHUS1RbGNwVjE4VGZVZy14aGJEQlNqVGVDTnpOLWFvR1d2TWNzRTNLQ1ZzZm12MDdhN3RZc0hwck5seXBuS3FxbENvV1NxY3laSWt5WDZUUVdDOXZBTzZFbnJlWG1jM04ySEVhdURWclgxVVV2ajJrSW5BMGlDdW15YWwzZTdsbERJUnVtUHpoTDJfZFNlSDYwXzM1SQ?oc=5</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K33" s="1" t="n">
-        <v>46080.38827546296</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Village Wertheim (fallback)</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Paysafe Announces Changes to its Board of Directors - Financial Times</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Paysafe Announces Changes to its Board of Directors - Financial Times</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Fri, 27 Feb 2026 12:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPc3N3ZWlYLUFIeVg3VGFjZlpKdlNEaVJ0azlRRW10cW5ENHltbkVVZEVCNkhWaWt4ald6V2VvRW9kXzRqbklrc2tWUXhSQTZ1eGtxcGt4Z2dud1h6ZXoyTVVMaGFLT25nQzNfUW1pMVR6UWZmMmRFeWFISURSTl9GaWtTQU44ZlVkMjRSbHE2VlFRY1NSY0VsU1pUbDUxREpKbTZrbGl3?oc=5</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K34" s="1" t="n">
-        <v>46080.5</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Local Town Ingolstadt German</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Suff-Fahrt bei Manching: Kleintransporter-Lenker hatte über zwei Promille intus - Pfaffenhofen Today</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Drunk driving near Manching: van driver had over two per mille ingestion - Pfaffenhofen Today</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Fri, 27 Feb 2026 14:11:55 GMT</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9DMGk1UjJFUjlIc0RzOW1wUDBvRmJHRmR1MjFxYXFkTzJyX1IwNTlTRVktMVhweklRQkh3UGJoVzJvUEZ2dC0wdU1QUHNQRFl0U1A3ei1PMVlYNng2WG93YVB3?oc=5</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>DE:de</t>
-        </is>
-      </c>
-      <c r="K35" s="1" t="n">
-        <v>46080.5916087963</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Village Bicester Kildare</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Desire Lines: As Mother's Day approaches this one of a kind keepsake is a must buy - Irish Examiner</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Desire Lines: As Mother's Day approaches this one of a kind keepsake is a must buy - Irish Examiner</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Sat, 28 Feb 2026 01:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNZ3l3cDJxM012NVc3M1dodV9uNWdjZG9zeGNHX3FHcU5mNllnR2tVSmxySlltVXhDZTQyZ2RrYnVFVllhNEdpRERZTzY2SGxMQ25oRWJZdUxKX1ZEQkRCM0R6eVM2TUpUdnJTcy1zY1FSZjd4emk2X3F2TF9HZ2VIRg?oc=5</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K36" s="1" t="n">
-        <v>46081.04166666666</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Village La Vallee (fallback)</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>("La Vallee Village" OR "La Vallée Village" OR "Serris" OR "Chessy") AND (shopping OR outlet OR luxury OR retail OR news)</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Elaine Hendrix Reveals Lisa Ann Walter, A.K.A. Chessy, Is Joining Her on 'DWTS' to Perform 'a Song from “The Parent Trap”' (Exclusive) - AOL.com</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Elaine Hendrix Reveals Lisa Ann Walter, A.K.A. Chessy, Is Joining Her on 'DWTS' to Perform 'a Song from “The Parent Trap”' (Exclusive) - AOL.com</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Fri, 27 Feb 2026 20:49:28 GMT</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNYWpLTjZGdUdzMXdlTFhjTzZaeDU2X0JySkU5UGRpX0l6T3gxd05CdTNKRFpRRHNUVE14RVFKQVFYQy1peFhDT1UwR25SY21UMkxmSGNSMm00TkhpRGp1NGVLNjByM25WTG0xc1ZlWjRsU0k5WEN2Q0ZZSHRQX2ItNg?oc=5</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>en-GB</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>GB:en</t>
-        </is>
-      </c>
-      <c r="K37" s="1" t="n">
-        <v>46080.86768518519</v>
+        <v>46081.31803240741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-02 07:55 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>Brand Protest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail: The UK Discount Beast US Traders Are Watching - AD HOC NEWS</t>
+          <t>Milan Fashion Week 2026: Gucci, Bottega Veneta, Tod’s and Ferragamo - South China Morning Post</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail: The UK Discount Beast US Traders Are Watching - AD HOC NEWS</t>
+          <t>Milan Fashion Week 2026: Gucci, Bottega Veneta, Tod’s and Ferragamo - South China Morning Post</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 13:19:09 GMT</t>
+          <t>Mon, 02 Mar 2026 03:59:42 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOV2NhNXFZcmFfUnVVYXUwMGRKbVFNZ3BhU0RqTmVKOWt4Q0FSNXRvcW1KQUkzREYyUzNxUXpBVUZGeV9Ldktwc1o1TllYcXRLcjdTNUx0MWZkZWlQZ3JNdno1eEhHcjJxSXJGTm52cjFKb0FkZ3hFVTVOTFdYVnRLY1FqODVIT09mYmxBRTNXX2xCMWZCQWFHMnRvV0VPRXl0aWw5NzVQZmYxUWJMQm01UzlnSDNzbVdxZTFreG8zMC0xVVU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxOMy1ZT3pEWHFmU3R0eXFoZ3dTd3ZpVjcxaW1XaW05aVp3X0dRNTBJS3VaZ2U1bmdUQXJYNkM3b0RRUmtFR0xvaGlubFhLcjZBeXk5SXZqWVZ5LW5uakdnSTFad0dBcnR5bXJ6cWRVQmZJbGFKaVhmOHVQOHhWSjhZdm9nWjNRbjNfc3FOM2NrOEdEMDJXeHpKZENCdEtNMDlJbEJ1aVhOeFFtSjRTXzM1VGg4MEdFelI4RGRNM1dTRGptYlVzY0Nydzg0bHg0dlEwbkxORWh5NEJKQdIB2gFBVV95cUxNTTg2ZEtHYlBHc1JqUHN3d3hrb19UMVpHOEhkRmJZekR3ZFlfOXYyUUhYUFE5MnpVLXRnQnNfeVRXMlBNekNjRW40MnBYZlhoek0zUVVOTS1SVDFKRGVuaHBhcllQeGVYRHRSTV85TU5EUFdGQXJ2RGluYTczWDNzLWhjOVhFLXBKZVc4ZEYwRVU1STdJbDNWSjR3ZHVwdHZyMlo2M3NpVC1uVTIybXlqTTFIbU1pZ2MzZDJJTGVLYVNnZndaWU01WXRVOURsWW5PaXFJYzJIX09MUQ?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46082.55496527778</v>
+        <v>46083.16645833333</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Explosie bij woning in Venlo, politie doet onderzoek - De Limburger</t>
+          <t>B&amp;M European Value Retail: The UK Discount Beast US Traders Are Watching - AD HOC NEWS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Explosion at home in Venlo, police are investigating - De Limburger</t>
+          <t>B&amp;M European Value Retail: The UK Discount Beast US Traders Are Watching - AD HOC NEWS</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 13:55:21 GMT</t>
+          <t>Sun, 01 Mar 2026 13:19:09 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPN0dXMDBnX0lwakEzbHQySHhLd1BUOElucDZWc1ZiczlVOXYzMWdOVXJDZktkN2c4QjR5aHZjMHpCS1FQQldPSzZqdUY3c2VDSkpjeXVIRTJ3QUtFbzdyODkyTTRyU3FzY1gwWmJ1a1FYYzAwNnd3czBOZzBUU3B1TFI4cmxLc3Azd2ZseHlKNU95bWdwMExQa0gxZlpPYjRLTXV1TTB5N29pdE1DYUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQY2JmcDBvWTNrdHZ0UF9kU0p4eGRBalAyQnlPQVpYdHNmM0toWi0yRjdocXVBbmt1dnhpZUlWNmtVZFJNMHp2bDQyYWZoMG1ibWJDWFo4ZDdGdWlwWFJGd0tIRlMwVy1UTk44TE1xaGxBZUVkamJRZkp0ckZROVRVeGYtVTVJYjMzdFVGeEhLWWFvYk9jYTBHeGNTVElNM3VhZTdLcXRYcEt0Y0haTGRFMHdjRk44dng1UU1mRg?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,52 +570,52 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46082.58010416666</v>
+        <v>46082.55496527778</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Leslie &amp; Agnes treden op in 50+ Ontmoetingspunt - De Gelderlander</t>
+          <t>Foxx Development (NASDAQ:FOXX) and B&amp;M European Value Retail (OTCMKTS:BMRRY) Critical Analysis - Defense World</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Leslie &amp; Agnes perform in 50+ Meeting Point - De Gelderlander</t>
+          <t>Foxx Development (NASDAQ:FOXX) and B&amp;M European Value Retail (OTCMKTS:BMRRY) Critical Analysis - Defense World</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 11:51:00 GMT</t>
+          <t>Mon, 02 Mar 2026 07:17:04 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxONW5pM29Fd0N3YURZcDVodU4yQXhhMnZwWDVYZl9yOEtPVmFGVHVTUGZmTDJWQVNsSllNSzhBQTdHNUV5eHZIQVY3OVIweFBwQUZhQWxEX29HWWJCanh1U2JzdnVqbkZ3eVpaci1sc1h4UHUzbktNU3NaU1JYTkNYVC1kMlp4UmFOMlRsMFZwWXk4cEp0YWNCM1daMlg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxNMnZKMno5dmM3ZkE2MVhaSG5Sbm42Q1psY2pMcF9VVS1iaVNYZ0pQRmtHaDRUeXFkR1ptZlNfX0d5b0NTTWhZVks0dTZvek1vcmpfVmx3SVA5OXhuT2JtYnBBTHFpNEcyMlpSVmo1QVFXTGdVQU1EV183clVMd09EeUg4Wkoxc1dVbGZXZDhjT0xUWWplNHBKSVhtcXJkWlVXQ2ZHM0Nzd1JBdE50a0JhTHIwaDh1VnQ4dk4yTW5hYU5OYmpHWXpqUDdfNzg?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,21 +625,21 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46082.49375</v>
+        <v>46083.30351851852</v>
       </c>
     </row>
     <row r="5">
@@ -655,22 +655,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>‘Domme fout’ leidde liquidatie Khamenei in: zo kwam geheime operatie opeens in stroomversnelling - De Limburger</t>
+          <t>Explosie in Anderlecht: appartementen in voormalig tankstation onbewoonbaar | Foto - HLN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>'Stupid mistake' led to Khamenei's liquidation: this is how the secret operation suddenly gained momentum - De Limburger</t>
+          <t>Explosion in Anderlecht: apartments in former gas station uninhabitable | Photo - HLN</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 10:49:29 GMT</t>
+          <t>Mon, 02 Mar 2026 02:43:28 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxNd0w3QVZQdXpoR2xGSmwwaGUyU0R4M0pmRFo0dTZyS0g5UHNCa2xDeEVrcC1YMzROakliOGRsYTlTZl9ZNU5UOTlrNXlJM2pfS2lJakMwWWU5d0s0VFlkR3VMcHFuVm1odTBEX1ZwWmVGcXNidHNNeGZfck1RVjFCcE0yRGNua0dvbEFNNEZfTkluREVTSUYwVjNQVmJnWml5SnJwWWhteUtyMldiaXo2SGhIZ25Gc1VHbEw5Q21CVF9mRzVQV1lVSno3c0RySWt2ZmVTcjFPelFvMV9v?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOYzlIMnhzM0pZZG8xQU9MVDdyQTJJQUJicUoyS3JNZ0R1MFpxMXJTTWZOeHlJZmVVTjZkcjI4VEQzTVcyNHRLbnpuakRoWk1aUVR1WHlNLWlNQTBteWJEWkhzUFA2TF8zN0dpZXhlbkp4ZkI1NElocl9UY1IyeVBtTjhlaXplNDhmZG1aM195ZkJGcGRTS2l3Tk9NbWlGbWhzN19UMWx6TlZhRDVPcHFkTEV6YXAwaDJXVDV5UmlHbw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46082.45103009259</v>
+        <v>46083.11351851852</v>
       </c>
     </row>
     <row r="6">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Poging tot brandstichting van auto in Venlo - De Limburger</t>
+          <t>Matteo Jorgenson moet ook in Faun Drôme Classic hoofd buigen voor jonge Fransman - wielerflits.be</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Attempted arson of car in Venlo - De Limburger</t>
+          <t>Matteo Jorgenson also has to bow his head to young Frenchman in Faun Drôme Classic - wielerflits.be</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 07:26:49 GMT</t>
+          <t>Sun, 01 Mar 2026 15:16:53 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPTDd2Sk0tSG5TaEEyZmJSdEh5UjJsUGE1bGdZZ0tOQVM4Q050eGp2T09leUI1Z0hrV2NXTjVZazhtbXZZc0hyYUhtWmw3ZHZxc202SzZod043RUJiYXZCX2NnclJMVllEM2NTekhqNFdSc08yM0pXdi11TDdjT1cyc0RfTVNVaGNFWGhfWXowa2k0ZzRVVkpLd09mdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQbjV6cENuVFc2c216dzNwVmNwZkkzaWRaMFQ3MHVsaUpnVnFyUFRwSmhocHZtcE9wbVlCWWJZVDE3RXFpeURyZFBtdmdjU3NaT25BRjh0c3J1MnNiek1waUVoNjh2Y2VVRG1UaFUyWTRWdkZMMlAxVVliZl9RU0poQ2d6V3lWNUV4eDAzMUloUjNnMG52UzRTcjRoV2Q4a2xzc3NV?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,38 +749,38 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46082.31028935185</v>
+        <v>46082.63672453703</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>World leaders urge return to talks after U.S. and Israeli strikes kill Iran leader Ali Khamenei - WRDW</t>
+          <t>Vučić: In Brussel waren er ook fysieke confrontaties, Tača op Dačić, Bisljima op Petković, dus ik spring ook - KoSSev</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>World leaders urge return to talks after U.S. and Israeli strikes kill Iran leader Ali Khamenei - WRDW</t>
+          <t>Vučić: In Brussels there were also physical confrontations, Tača on Dačić, Bisljima on Petković, so I jump too - KoSSev</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 11:38:00 GMT</t>
+          <t>Sun, 01 Mar 2026 22:11:13 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQcmZXbmpXeWQ4cC1kTXNGVFk5eVZtREpLdUNzb0d3WjFqd001eVVra3lDRVVuREdMWGxFa1NaUDhXS1FyNGZMaDh5VG5vU2gwS0JYN00tQU9rSUhRVVZHbjBUWG1td3piOERTblNzRHFiVjNBampXd2l5M2NtU21PNENfTjVfNVRlb3F5c2Mzc0tFUG9VWUdWVmVhM3p5dUhFbWtYYjY2N3poRHNHVmoxanJ6dmktbXdOMkloOTFjZzRiXzlyX29YVVZXelRTWknSAc8BQVVfeXFMUHJmV25qV3lkOHAtZE1zRlRZOXlWbURKS3VDc29Hd1oxandNNXlVa2t5Q0VVbkRHTFhsRWtTWlA4V0tRcjRmTGg4eVRub1NoMEtCWDdNLUFPa0lIUVVWR24wVFhtbXd6YjhEU25Tc0RxYlYzQWpqV3dpeTNjbVNtTzRDX041XzVUZW9xeXNjM3NLRVBvVVlHVlZlYTN6eXVIRW1rWGI2Njd6aERzR1ZqMWpyenZpLW13TjJJaDkxY2c0Yl85cl9vWFVWV3pUU1pJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPQjVSNGlfS0JvOXM3ZFY3ODdDX2lHLXgtX0tlV2VQNEMzT1kwYUZjSVFqbUpadl9vT0h2Z1N5QktnTzlDTlEtSDRxQmFxTTBzZXVrcTcxSjhqWV9ZLWdqVHhUN2hiSnpkUGVpV0RzOUtqbVkzdFhXZUU4WnNaMFNjV1FET2l2bVBvWmNMQ21EejNVVVgtVkxoTkZJQ0NoNVdjRWVrOElDbW9qNURmb3BTdW1CYjl3NDA?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -800,42 +800,42 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46082.48472222222</v>
+        <v>46082.92445601852</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Latest developments after US, Israeli strikes kill Iran’s Khamenei - Brussels Signal</t>
+          <t>Explosie bij woning in Venlo, politie doet onderzoek - De Limburger</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Latest developments after US, Israeli strikes kill Iran’s Khamenei - Brussels Signal</t>
+          <t>Explosion at home in Venlo, police are investigating - De Limburger</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 10:03:46 GMT</t>
+          <t>Sun, 01 Mar 2026 13:55:21 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNM2cyc0hkVVN6OWl4b015NEg5OE9WRDFCTURIczFfenZ3ZzFWQzlpdk84dW1fYkhSTDhvcXliQW92cWJLODlEbUplV1JZS0VPWDdBMWNfTFdOTFU3dUpLZm9TdkdnQXRtdzhkYk5ReTJyLU1rb3VaMGFKSkhSR2F1eWt3cTV1NFRtMXFfbGllMmZlT084dkZlNjBTNzcxUjFY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxPN0dXMDBnX0lwakEzbHQySHhLd1BUOElucDZWc1ZiczlVOXYzMWdOVXJDZktkN2c4QjR5aHZjMHpCS1FQQldPSzZqdUY3c2VDSkpjeXVIRTJ3QUtFbzdyODkyTTRyU3FzY1gwWmJ1a1FYYzAwNnd3czBOZzBUU3B1TFI4cmxLc3Azd2ZseHlKNU95bWdwMExQa0gxZlpPYjRLTXV1TTB5N29pdE1DYUE?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -855,42 +855,42 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46082.41928240741</v>
+        <v>46082.58010416666</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>"C'était pour l'aider à se préparer à un copain" : 30 mois requis contre l'oncle qui a initié sa nièce de 11 ans aux sextoys - BruxellesToday</t>
+          <t>Vučić: Pristina geniet "stilzwijgende steun van het Westen" na de arrestatie van vijf Kosovaarse Serviërs - KoSSev</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>“It was to help her prepare for a boyfriend”: 30 months required against the uncle who introduced his 11-year-old niece to sex toys - BruxellesToday</t>
+          <t>Vučić: Pristina enjoys "tacit support from the West" after the arrest of five Kosovo Serbs - KoSSev</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 14:01:00 GMT</t>
+          <t>Sun, 01 Mar 2026 22:50:36 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1UZzVxX2V1UGpTOHBkZy16amxENkFQMzRTQzRzOXRYTnpyYkl5S2lQMHFNM1pzNkdIOEhSbWE3azNaUGRLUERWbW9KMm5pSlN1RUo1ZHA0X2RtVTVINHhXdTNlWmV1cVdXc2hxZ05RTjhxaXNodG5OT1BHVEFKYTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPTGhWdTdOWlh3RUU1Y1pWMWs1VmZOT2lpaU9VQktRWkVwYVlPbzBFb3lKZ1VWb04yb1NHZlZoYjZ0bWU5OWp5dzdYNmY5RlNzSERoX2VlcmZuY1NLTVJnLTFwTURxekdReFMwMTNaVFVJMURZQzVEZG5oWnlXU19kT3o2ajFxM2dfTmVicnVCWDNEMHdNRHU2S0h4ZG5iSjdEWWlTSUhwNEJQdw?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -910,42 +910,42 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46082.58402777778</v>
+        <v>46082.95180555555</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Une collision “grave” avec un tram à Etterbeek: un homme coincé dans sa voiture - 7sur7.be</t>
+          <t>Explosie bij woning in Eindhoven veroorzaakt brand: ‘Mijn huis stinkt naar benzine’ - StadIndex</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A “serious” collision with a tram in Etterbeek: a man stuck in his car - 7sur7.be</t>
+          <t>Explosion at home in Eindhoven causes fire: 'My house stinks of petrol' - StadIndex</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 10:40:00 GMT</t>
+          <t>Mon, 02 Mar 2026 05:02:00 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTlg0a1R2dENOYnlpTzFUT0JqT1U2b0wteHBuZklBLUc4cFdqQjVmeGdQenBNVTh4eXpjMTBHNDdSOUczZlZuWjg0d2VqSGROQ1ZySGZUNTJKSWhxVXR3ZHdwV2xBekx4a3lwLXN6bUw5dk5wUzFSNHJ5RlduR05qZkhLQU93RVFudVhvRnE0MUlZb1o1em1EWVMwZkp5ZXRWZWhQVTdhNVZPYnhGUHo4ekdYMEdEN210R3hZbA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPamlPT081SHhSNnBIWnRLXzRITFZhYjNnTjVDMmhiVmhuUEZNbHFQa2xTRDNueF9FMm5UQ2sxTXh2alBsaXdPbS1JVk5tZ3BQSzlZeEwxaHZ0QmdBbWhOcmZRc2NkbW1pRURxbzlKZnkzNUNQS0p1eTR3NWE3ZzdJbzZCY21QSEQ1U3VJQXFFV3BJMWR6Q1hYS01Qb0h6MGMzOHNHLVBEVWRzM2ZrR1RTaWh3SjE4TTY2?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46082.44444444445</v>
+        <v>46083.20972222222</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Depuis Bruxelles, des Congolais de la diaspora montent contre la déstabilisation de la RDC - Radio Okapi |</t>
+          <t>World leaders urge return to talks after U.S. and Israeli strikes kill Iran leader Ali Khamenei - WRDW</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>From Brussels, Congolese from the diaspora are rising against the destabilization of the DRC - Radio Okapi |</t>
+          <t>World leaders urge return to talks after U.S. and Israeli strikes kill Iran leader Ali Khamenei - WRDW</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 08:22:30 GMT</t>
+          <t>Sun, 01 Mar 2026 11:38:00 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOM2JsbUlfVE5LZ1ktX2swbExvX1JmTDdmRWxkS0d1WXg2WGhKRnNzWXpkV3gzTkhwNHBzeWl3WU5SQTlhVXdxQkt6V240OU9hXzZXd05ZNWFIREJ1U2xhMHF4bFlFa2xkSnZYWk9ZSS1wUU1VR0RoYW1Pb29XbUR5bHdfRE1YMjZHbmFQTmdrVHgxVTkyS2l0Sm1CNnJkWVR1Yk1vR1N6Y3RvU05GNkU3UXJOclF2UDRkRVl3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQcmZXbmpXeWQ4cC1kTXNGVFk5eVZtREpLdUNzb0d3WjFqd001eVVra3lDRVVuREdMWGxFa1NaUDhXS1FyNGZMaDh5VG5vU2gwS0JYN00tQU9rSUhRVVZHbjBUWG1td3piOERTblNzRHFiVjNBampXd2l5M2NtU21PNENfTjVfNVRlb3F5c2Mzc0tFUG9VWUdWVmVhM3p5dUhFbWtYYjY2N3poRHNHVmoxanJ6dmktbXdOMkloOTFjZzRiXzlyX29YVVZXelRTWknSAc8BQVVfeXFMUHJmV25qV3lkOHAtZE1zRlRZOXlWbURKS3VDc29Hd1oxandNNXlVa2t5Q0VVbkRHTFhsRWtTWlA4V0tRcjRmTGg4eVRub1NoMEtCWDdNLUFPa0lIUVVWR24wVFhtbXd6YjhEU25Tc0RxYlYzQWpqV3dpeTNjbVNtTzRDX041XzVUZW9xeXNjM3NLRVBvVVlHVlZlYTN6eXVIRW1rWGI2Njd6aERzR1ZqMWpyenZpLW13TjJJaDkxY2c0Yl85cl9vWFVWV3pUU1pJ?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,42 +1020,42 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46082.34895833334</v>
+        <v>46082.48472222222</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Euerbach: Autofahrer flüchtet vor Polizeikontrolle - Radio Gong Würzburg</t>
+          <t>Latest developments after US, Israeli strikes kill Iran’s Khamenei - Brussels Signal</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Euerbach: Driver flees from police checkpoint - Radio Gong Würzburg</t>
+          <t>Latest developments after US, Israeli strikes kill Iran’s Khamenei - Brussels Signal</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 13:09:00 GMT</t>
+          <t>Sun, 01 Mar 2026 10:03:46 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQeVZJNy1mVGIzZ2V2emN6c3VYYWs3dFM5S1BPQ05yLV9UOGVnQk1NWUM3a3VZVlhNWnJYeGptS0tNSHN1cEtxX0o5VHFBc2t5X3ZWTGt4SkstOG9WZEowZzhVNkVTVGJDOEhZU242Z0d5VEJGZXVGS093bGVza0VYcXBvUFpjenRSWlI1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNM2cyc0hkVVN6OWl4b015NEg5OE9WRDFCTURIczFfenZ3ZzFWQzlpdk84dW1fYkhSTDhvcXliQW92cWJLODlEbUplV1JZS0VPWDdBMWNfTFdOTFU3dUpLZm9TdkdnQXRtdzhkYk5ReTJyLU1rb3VaMGFKSkhSR2F1eWt3cTV1NFRtMXFfbGllMmZlT084dkZlNjBTNzcxUjFY?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,52 +1065,52 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46082.54791666667</v>
+        <v>46082.41928240741</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Unfallfluchten, Autokratzer und Eierwerfer | Foto: Jens Buettner (dpa) - main-echo.de</t>
+          <t>EU warns against long war, urges ‘credible transition’ in Iran - The Straits Times</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Hit and run, car crashes and egg throwers | Photo: Jens Buettner (dpa) - main-echo.de</t>
+          <t>EU warns against long war, urges ‘credible transition’ in Iran - The Straits Times</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 11:36:26 GMT</t>
+          <t>Sun, 01 Mar 2026 20:08:12 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPS1hnZDFGQkVqeE9hRTlRY1pNbVBtbmRKbEkwSzZIQzRSVENyMFczOXllOGg3SUxYaG8ybngtOTVEeU0zWWZfZnFPRUdBYVA0NmVmSmVuZUs0OGJvdFFhX1VNWUZzaV9DdnRGcWRDX2kxZklMemw2SkdFaDFoZ0NtVHdXZEJnZnlRU2NhZDlLc05Kb2dLTnk3bmJ5YnN6QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPbjV1ZzJsb2RRVkF3QW9ERjVUdDNwRF9wOWhVV1FlSnhRcDFsVjRZOUViQ1FtVlR1RXVMSTBCalAydEJiMHpGUU50cGFzTlRnNDAwVEtjQmxZREJuVkRHcWdrMExCXzkyOXktQnEzdHVMMnBzS2Qtb0x3Qkt5LXVIMzVCQ1Y1YU5uaUpkY3Y2NWFad0pOTzBsNkUxM05yNkljSVB4WDNpZ3FxcGdoWFFEQlNjWFVkVWxFYm9GaTBXZDBVT3ls?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,52 +1120,52 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46082.48363425926</v>
+        <v>46082.83902777778</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>15-Jähriger liefert sich Verfolgungsjagd durch Aschaffenburger Innenstadt | Foto: Carsten Rehder (dpa) - main-echo.de</t>
+          <t>Guet-apens pour une Rolex à 13.500 euros : deux suspects recherchés après leur fuite vers Bruxelles - BruxellesToday</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15-year-old chases through Aschaffenburg city center | Photo: Carsten Rehder (dpa) - main-echo.de</t>
+          <t>Ambush for a Rolex at 13,500 euros: two suspects sought after their flight to Brussels - BruxellesToday</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 10:01:41 GMT</t>
+          <t>Mon, 02 Mar 2026 06:01:00 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOd2twSWJDYWhXVjhyclZ1RF81NGxFbTUxamlzWm0xU1VKRk5OT3pGS0xUbWkzMWlpOEZCT1Q3UHFnNUlNb2xTTmdnczZmcThvVVp1RkJWQXRJd3hBT2NLN1o3TnNlZ3NXX1p4UDZhSVV2aWhoTGY3Ujc4RkFwczVtSThFODBRaDdra1V5ZjhSV1BWcll1MWV5RktjTDRaYzRMMVgwNEJpdTRwQnVLNWt6S3YxaWU3ZzJtUDdnVHFadlJrbmFhdlJtZlFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPUHlidGVkQUZMTXVkNGUxa3c0dmlXLVhRSU04VmkyT2duWmUzdmdDa3l4Y29xU0FDeXJZaUdtNm5lWTJlTnVpVTFuZWllblNNSTZyTzdrbXQ4cHhKd2hTSTBpRlpDYjN5STZEUzc5b0RDQnliYW40WFRVMnRJSTgtbnZrdnhHZ3g3RDYwbmJ3TkJYWUQ2RkI3Ym1rNGFlUFZZcl80ZXMwWHNLcHB0Y1hORUhBS1U3V3pXQXR1VUViRjdlNUg1QzMwLVhDcmo5VGx2eElCZHNGSVltZzhTbXc?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,52 +1175,52 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46082.41783564815</v>
+        <v>46083.25069444445</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nach Messerangriff in Würzburg: Keine Hinweise auf Psychose | Foto: Michaela Johannsen (dpa) - main-echo.de</t>
+          <t>Un lundi au soleil: le point sur les prévisions - 7sur7.be</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>After knife attack in Würzburg: No evidence of psychosis | Photo: Michaela Johannsen (dpa) - main-echo.de</t>
+          <t>A Monday in the sun: update on the forecasts - 7sur7.be</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 10:37:20 GMT</t>
+          <t>Mon, 02 Mar 2026 06:15:00 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxONkM3U0l6TFZWaUF1dV9CX1hqcWV1TjM5c1kzTWxlcjNreWN0aVFhXzZsUDRIOHZVcjdKcnRaSElTZGgtejljajdXYWhBbTltVkQ0RnYxaklMUW5VMGgxN3hGbVJrVktrSHN0dFF0MzZXSTF5QlVKeVRZVFluV2JNSWxvZzdMeW9IYndWN2t2MUlQMmR4a0ZLNGkxMFUwNTJjTVdNb1F2VnFHMS1PR3JVZ0YyaS14UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNSDl1b2FBU2ZmQ3VNXzNCRHlEUUxvWE14YjZUOXpYRnR1bldsV2dpM0NLRUFGWHQ2Q2VfVDRabTVSX0dvbHkyS1A2SDNHVmJrYTlTamNlQ2pYajZ2S0RDU2w0WUxydndodkU1a2tJY25sd2FkdmlRYzB6c1JrdllSTGN3bFlKd2hvamNRVUZZMA?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,52 +1230,52 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46082.44259259259</v>
+        <v>46083.26041666666</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Darum ermittelt die Staatsanwaltschaft gegen Beamten der Polizei Marktheidenfeld | Foto: Marijan Murat/dpa - main-echo.de</t>
+          <t>Kuurne-Bruxelles-Kuurne 2026 : Matthew Brennan remporte au sprint sa première classique - TodayCycling</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>That's why the public prosecutor's office is investigating officers from the Marktheidenfeld police Photo: Marijan Murat/dpa - main-echo.de</t>
+          <t>Kuurne-Brussels-Kuurne 2026: Matthew Brennan wins his first classic in the sprint - TodayCycling</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 11:08:20 GMT</t>
+          <t>Sun, 01 Mar 2026 15:55:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxOQkU2ci1Ieng4YXBFbzM0eTFFZWl3ZzVkcFE3SkZRNFpSWERhdld2dWJRR1l0UWZxQTNMbmNVV09yOGUwbnpfakYxSnBTX25Ca1A0OGhrcngtV0c4ZzJSb0V6Y2FNczFVa3NXd1B6eV9KcHoyOUNkLU9wbVFsdGxzNzVxNXFyV3ZucGlTc2NWbVJpNUxpRnV3Sm9oYnNBRklDal9nblZWMTExNmRHNlpON0dMNUlha285WkVOczVyU0ZBaElXWS1RR0FQdjNlT0RfbEtRT1hzd01YSzQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQdjIyN1lVN09IXzFyVWJUWnhTaFBwN0ZNT2lMbm96OHJlejZuNmFLNnlTQTB0UVdleXZIWXpWcUNYZW80VTBtdXlfVmZsdTZfNmFid0VsdGw5YUpoZ0x1MDNPanNPbmhXeS1HaVdIdWR6Rnp3M2ZYazlnWWR6Y0ctMGVQbFA0ZjVPUWtfTzBvOXNNY1c1Ym1RUUVFc19sd3lWald6aUxWSkdDU3JvMzhRcA?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,52 +1285,52 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46082.46412037037</v>
+        <v>46082.66319444445</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Blitzer in Würzburg aktuell am Sonntag: Hier nimmt die Polizei am 01.03.2026 Raser ins Visier - News.de</t>
+          <t>Alerte à l’hôpital Erasme après une fuite d’oxygène - BruxellesToday</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Speed ​​cameras in Würzburg currently on Sunday: Here the police are targeting speeders on March 1st, 2026 - News.de</t>
+          <t>Alert at Erasme hospital after an oxygen leak - BruxellesToday</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 13:15:55 GMT</t>
+          <t>Sun, 01 Mar 2026 14:54:00 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxOWEs0WUU4QzFMVWt2eS1pSnctVGxnLXBLQWZBZllOSkltR0JzTDRKdk1NUVlhdXNWLURtTUUyZXY0ZnVZZFhrQmxTNy1SdW5OYWNLc1RSNmtKM1lkQ2V2dWNLQXNSUm1JQWFDcG52YmFMVktwVW1KdGZRWVBUNURRODUtT2txZ3RvOEtTRlQtNVRqbV80VDF0eWRIYlB1R0lqek55bjNFWE5WWVQ2ZVo5LXFjVUgtSFJkUGV5WklaRGhENk9ZcTBTb0FYNUdEa0ZxS29McXpnZWJieUVmSE5ka0k0ZFpocXfSAewBQVVfeXFMTk5mTXF1M1NvOEZVVFhlTXk1eWg1YVg5T053TEtMRWNfN3NlWm5ENmZiSEVpTFpJVTc5M1hJaW5TakpNa1dLZTJ5LThOTFJsQndBVnY5MEFTTXQwSmZZcjZOckVISmloS2ZyVjlYU1NUVGRhc3RVRldEck4yZlJDa3pObHFxWFRJdTNUMHlIeXJ1YmpWUXRnLXJoeHZGMTl4M0ZyNVVkZDdkN1VJLWtrMkh3UU12cmxtcUlpc0FqSDVybmdFcTBxR1l4X050cW03S3daSDBhbHZmTXBpUzd4TmhqSHhwNDdzcmZ5UWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPMl93WEtqRkh4Z2JPclhwUkRtR014UGREazVwV2JmcXhiQ3MwZmNaVXVRd25tNkR6S25uYWM2cTJ1TWNsTjc1cjFGdXdpY1NkNEFHMHB5M09NdEhqY0NrZElBVE1jREh2WTFsR3RpeUpkSUw5TV9sbVZLaXRrZWRlUDEtWW1mLTRQSWFBbGlNYWZpTTNpMUdBRkZNWU1LQWFM?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46082.55271990741</v>
+        <v>46082.62083333333</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Polizei-News Nürnberg, 01.03.26: Halskette entrissen - Zeugen gesucht - News.de</t>
+          <t>Deux personnes tuées par un tireur à Austin, le FBI penche pour un “acte de terrorisme” - 7sur7.be</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Police News Nuremberg, March 1, 2026: Necklace snatched - witnesses wanted - News.de</t>
+          <t>Two people killed by shooter in Austin, FBI leans towards “act of terrorism” - 7sur7.be</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 10:47:02 GMT</t>
+          <t>Sun, 01 Mar 2026 19:08:00 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQeG9XaEpTdFVBeGRuMjdSYXR1SlhLSS04X1hlaVFSY3Rnd0YtRzJNdFppVVRPTERnQkZrZWw2NUFndmhyRm1Wa09XT2hUak1lOEdWREI2TVdqTENZZldXZGVRQVJDZGhESHJnYy1na2Q1d2t4bndpbEI5dFdWUndpVXItb2oxYjA1S0p0N3o3REhIdUFlUUx0atIBngFBVV95cUxOWGtnVDZuUmZtbzQxRzFJUmhiUkh6ajNrb1pRS2lZXzV1S2JrYmQyUkJDdzFfUTF2bDVka2hmRlNTYU5zM1E5cDVfOWpJYVY2dDRYNEJuUkYzUUZYTVlBZmd1SnE4OXZRcXFjZlh4aGtEb09uQkdyMWhpVEE1WXM5eDZRWlpSX3lUSjFSakl4enctenUxblp3ZUJmNjdKQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPbm0xcHVOZE5NdmliVld3bUxrY1cwMlVUTkNxM1Vld3F3UkgwQ2VBQ0t5RVBkWlNmaUJGZ3BsOWhFUGFhQzdpLWdtOExZcFkyLXFwT25qLWl2V0tYUkZfd3ZnNGo2RTQzNGMtS0ZGYjdrc2pFNDlwWjJUTm1YQnRyd1hSNUJPdkNSb2xkU0NCT3ZfcWYyUU9wUXV2M2tSRm1ramxNTUhOLWVfeU14WTQ4cTZ3MEJQZGxURWgzdURnSjN6cTZxdWo4?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46082.4493287037</v>
+        <v>46082.79722222222</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Polizeifahndung Nürnberg, 01.03.26: Bei Verkehrskontrolle Betäubungsmittel und mehrere Fahndungsnotierungen festgestellt - News.de</t>
+          <t>Depuis Bruxelles, des Congolais de la diaspora montent contre la déstabilisation de la RDC - Radio Okapi |</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Police search Nuremberg, March 1, 2026: Narcotics and several wanted notices were found during a traffic stop - News.de</t>
+          <t>From Brussels, Congolese from the diaspora are rising against the destabilization of the DRC - Radio Okapi |</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 10:47:01 GMT</t>
+          <t>Sun, 01 Mar 2026 08:22:30 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNOEpNcTJyeUE4VGRHSm5aQk5fcGh3MTlmcmppeDFDaVpuN0lGMVFRQWRxM294ekUyNjFYUVozdHZqWVZsVVhpV0R1T0tZV0lnelJZSG9ucWY1elBlUG1NdHVGemE3UV85YlpSd2VOQlBoR24yd1QxVHgyWlNXdkkyOUt0STFJRWhKaXZjcldQMVg1MWt6MG1nWWZTTVRBNzg5d3VXOFFibzVLWDloUVFHZHlaV0R2bUlFZ3JmQWxJMNIBxAFBVV95cUxOVlN3Y1lGMXd3VU9xTVhFbmpwN2YzTHdTZ3Rla0ZldnRRc3l3bjFWT1Zpbk8ySlp2TDNvX1J6M1NfdHFSOXlMVGVMVUNRV2ZyenMyNzhiLWhIQlotNXpHVHAtODlxWlJuTzdJX2hNb1NfYjJudS1yeVZJbHA5eVhIdVZjWm10Q09IZHBmcnhzQ0N2WkExZm1WQkNmNW8zQWo5MUFGR1BqcFBRRlV4LWdkVUw4Y1lCTVFnNkFhQXdkWmZTQzNI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOM2JsbUlfVE5LZ1ktX2swbExvX1JmTDdmRWxkS0d1WXg2WGhKRnNzWXpkV3gzTkhwNHBzeWl3WU5SQTlhVXdxQkt6V240OU9hXzZXd05ZNWFIREJ1U2xhMHF4bFlFa2xkSnZYWk9ZSS1wUU1VR0RoYW1Pb29XbUR5bHdfRE1YMjZHbmFQTmdrVHgxVTkyS2l0Sm1CNnJkWVR1Yk1vR1N6Y3RvU05GNkU3UXJOclF2UDRkRVl3?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46082.44931712963</v>
+        <v>46082.34895833334</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Polizei-News Nürnberg, 01.03.26: Gestohlenes Lieferfahrzeug tauchte bei Ladendiebstahl wieder auf - News.de</t>
+          <t>"C'était pour l'aider à se préparer à un copain" : 30 mois requis contre l'oncle qui a initié sa nièce de 11 ans aux sextoys - BruxellesToday</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Police News Nuremberg, March 1, 2026: Stolen delivery vehicle reappeared in case of shoplifting - News.de</t>
+          <t>“It was to help her prepare for a boyfriend”: 30 months required against the uncle who introduced his 11-year-old niece to sex toys - BruxellesToday</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 10:47:02 GMT</t>
+          <t>Sun, 01 Mar 2026 14:01:00 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNb0lKZ3pJVmVhOEQ1LTViWTI2czQyM1RFaE5IY0hlMncyaVhLRDE2cGFuQk82YldJZHo4bWpVanh3OGN6MzQyOERyQ3Rqd29BNmd1X1FVdFFqU0ZwNEZYVndubFBaZ19NWVlJZGw5dnhnVVJiVGRJekgzX3lGUEtpZVFKbVUtS0VVNGdCc3V4R0t4dkk2enU4b1FR0gGaAUFVX3lxTE1vSUpneklWZWE4RDUtNWJZMjZzNDIzVEVoTkhjSGUydzJpWEtEMTZwYW5CTzZiV0lkejhtalVqeHc4Y3ozNDI4RHJDdGp3b0E2Z3VfUVV0UWpTRnA0RlhWd25sUFpnX01ZWUlkbDl2eGdVUmJUZEl6SDNfeUZQS2llUUptVS1LRVU0Z0JzdXhHS3h2STZ6dThvUVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1UZzVxX2V1UGpTOHBkZy16amxENkFQMzRTQzRzOXRYTnpyYkl5S2lQMHFNM1pzNkdIOEhSbWE3azNaUGRLUERWbW9KMm5pSlN1RUo1ZHA0X2RtVTVINHhXdTNlWmV1cVdXc2hxZ05RTjhxaXNodG5OT1BHVEFKYTQ?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46082.4493287037</v>
+        <v>46082.58402777778</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Amtsbekannter 29-Jähriger tickt in Ingolstadt aus: Drei Polizisten verletzt - Pfaffenhofen Today</t>
+          <t>Il venait "juste pour s'amuser et faire du sport": le Wavrien Nicolas Nolf repart avec le titre de champion de Belgique de biathlon virtuel - L'Avenir</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Well-known 29-year-old ticks off in Ingolstadt: Three police officers injured - Pfaffenhofen Today</t>
+          <t>He came "just to have fun and do sport": Wavrian Nicolas Nolf leaves with the title of Belgian virtual biathlon champion - L'Avenir</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 12:57:08 GMT</t>
+          <t>Mon, 02 Mar 2026 06:03:00 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBvamRMTVlQOWd3bWlUcUFZUGxnVUR1V2ZHLVBFTUJMMTVvVWs5b3RSWVVUdGxOWnAzZHpTRnVUY0dxMG5vRnNzSGRqWXlEM2RGTHRIXy1MZzNOdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywJBVV95cUxQR1ZmMW1Fc1ExcUtXWkRKejNfOHdPRTNIdU1OU2Rma0lqNDNZUldJMnpRWThSRi0zTUp4UkFJdXlSYVNOVUozZUFtUU1zcnpzZnhhMzRDb05CQ0NFOFZVQm9hVUo3WnRHTWZxSnFSSVRjQXNYbWtUaE9WX29Md0NCbVdpaWdac19rSkUwekxLVXNUaDl1YUpYVU4zai1Cb0JwOWZMZU94bFpBb0o1eG9fRTMtaElEeGxCV0o1RFpkSV9pTnd0UDVYVmdvM2JlaEFjRGg0a3k0WXR4MDlRV2UzWUxJdWx2YTJnWnZwQnpQWENwdHIwM1RWX2c3WUlTTjA3SVltSkdlWENkaFBVUG9TZE1sd3daUjhCUnZaVjhqNFVFQlZ6S2NNR2FCQ2FUYmwteEYwX21BS3NYMDRxb3c4OHJ0eVA4eWRvUDNn?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46082.53967592592</v>
+        <v>46083.25208333333</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Kontrolle auf der A9 bei Manching: Etliche Anzeigen für Fahrer und Firmen-Chef - Pfaffenhofen Today</t>
+          <t>Seraing crée la surprise en Challenger Pro League, fin de match folle entre le RWDM et Eupen ! - Walfoot.be</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Control on the A9 near Manching: Several advertisements for drivers and company bosses - Pfaffenhofen Today</t>
+          <t>Seraing creates a surprise in the Challenger Pro League, a crazy end to the match between RWDM and Eupen! - Walfoot.be</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 13:49:11 GMT</t>
+          <t>Sun, 01 Mar 2026 18:00:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTFBmZ08ybkRQM00xOGNTdThLX3BqWFBrM0FyZHFfcUY5RTJheWcyVFFYTmdmaGdxbEVWZ1AwYW9rTHlkZmw1ZUF3Ym4ybEFfWjE3enRjM0RuczFPaWNGNGxjNzhR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQSVdCZVhPM2hFS2NOMjV1RHZBQ1R2OUtOdUw3YTBJeDBEWXFMbWJ1Zng0amg0YXR2bDM5d280RTY2LUdleFJMd21Tc3JZVHdDampsZ0dzelkwRlFGOHU5dWNFYkJLMzAwWGRvaTlUR01qeVdTbUJHYVE4WVZBNVlGVWRCdUhPdkVCSEdDc3htM3NiWFVwcDFWaTg2SThha3VpWE50V0pkT1prSW80ZFdoVmNQdDNGeWdwLU43QkZTWkhET1gzTkxnNDl3eFJPWnfSAc8BQVVfeXFMUElXQmVYTzNoRUtjTjI1dUR2QUNUdjlLTnVMN2EwSXgwRFlxTG1idWZ4NGpoNGF0dmwzOXdvNEU2Ni1HZXhSTHdtU3NyWVR3Q2pqbGdHc3pZMEZRRjh1OXVjRWJCSzMwMFhkb2k5VEdNanlXU21CR2FROFlWQTVZRlVkQnVIT3ZFQkhHQ3N4bTNzYlhVcHAxVmk4Nkk4YWt1aVhOdFdKZE9aa0lvNGRXaFZjUHQzRnlncC1ON0JGU1pIRE9YM05MZzQ5d3hST1p3?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46082.57582175926</v>
+        <v>46082.75</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FC Ingolstadt 04 - MSV Duisburg ai prediction 04.03.2026 3. Liga - Livetipsportal.com</t>
+          <t>Le 62e Salon de l'agriculture s'achève, bien moins fréquenté et marqué par la crise agricole - Boursorama</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>FC Ingolstadt 04 - MSV Duisburg ai prediction 03/04/2026 3. Liga - Livetipsportal.com</t>
+          <t>The 62nd Agricultural Show ends, much less attended and marked by the agricultural crisis - Boursorama</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 08:01:06 GMT</t>
+          <t>Sun, 01 Mar 2026 17:50:16 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPbUtOZV96NU56ZDlBa3d6VGZWMVczSTY1aG9RdmxpWEZHTDhzMllMMDVrSmZWTWlWN1ZLcDhYc0xtTGg0TWkxaFdlSU1RWHFwMlV0UkpaS2piLTZkcEN4MzJxQmtxSG1NUk1JSXR3QUFlaUp4V1QyMkJyc1JJb0NIQVFjSHFFeGNWdDJUMUFCSVRMQ3Y5cDN1NlVoS2F0VEs3NXhVdA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgJBVV95cUxQNWtfcmVzRldfMHc1V1plUl9ZRUkxRG1WaklZUUtlMjFwNEd5YUlic3FhWjViS1JtbVlxLV9XZTZWa214RVUwbEZudUQ3RWZqQklrYkUzaFhfU09hR1RfLXVLeVhIMVh4WWpDZmpGRlktV1VqdnRYc0pIbXNjZ05oWXppbFFYZHRmZlNvTWg4S1JORnI5bzl6ejFTMlVpS19DTEtZQkZFam5BSmFqRXVBdDRDcVpYSFdEZkxSRE9BMDlVZUZ1WVpfVU03ZWcwazY0VFg5Rmt4OGpQUlA3TUZtMlZWTlpGeERidmw1NG1tbUtoQlo1MExjZUY5cTltM0pobDI0Z2dfeW5xSjJfRkJkVXI2SzJhZ9IBlgJBVV95cUxQNWtfcmVzRldfMHc1V1plUl9ZRUkxRG1WaklZUUtlMjFwNEd5YUlic3FhWjViS1JtbVlxLV9XZTZWa214RVUwbEZudUQ3RWZqQklrYkUzaFhfU09hR1RfLXVLeVhIMVh4WWpDZmpGRlktV1VqdnRYc0pIbXNjZ05oWXppbFFYZHRmZlNvTWg4S1JORnI5bzl6ejFTMlVpS19DTEtZQkZFam5BSmFqRXVBdDRDcVpYSFdEZkxSRE9BMDlVZUZ1WVpfVU03ZWcwazY0VFg5Rmt4OGpQUlA3TUZtMlZWTlpGeERidmw1NG1tbUtoQlo1MExjZUY5cTltM0pobDI0Z2dfeW5xSjJfRkJkVXI2SzJhZw?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46082.33409722222</v>
+        <v>46082.74324074074</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Six Roald Dahl films returning to Bicester cinema - Yahoo News UK</t>
+          <t>Fréquentation en baisse au Salon international de l'agriculture 2023 : enjeux et perspectives - actudrancy.fr</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Six Roald Dahl films returning to Bicester cinema - Yahoo News UK</t>
+          <t>Attendance down at the 2023 International Agricultural Show: challenges and prospects - actudrancy.fr</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 13:00:00 GMT</t>
+          <t>Sun, 01 Mar 2026 20:37:26 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5mTFh3b0RaTmlseVlPMXZzQnBfZXB0enJuSVJGdlNvWHU2TTZpSTUxMkZqWHo5Nk9oT2lFWEU0aW9pUFZOajR0ZHBjZFh6c210X0ZRRmpWaVNDRUJUaDhKNUJXekx1RG56NFFTVDhPTDlKQmdrN2RGYnQ2UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUEFVX3lxTFBrN05wd25MUDlRdlRSclMzTjE5OHpLMkVYMzVLeEZWZWhJMkRZS2RpZVk4ZWsxd0JwcnNheDk0QldJU2o1djRCWkRMZFNMb0VG?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46082.54166666666</v>
+        <v>46082.8593287037</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pupils debate internet access at Kildare semi-finals - kildare-nationalist.ie</t>
+          <t>Ochsenfurt: Motorradfahrer entzieht sich Polizeikontrolle – Polizei sucht Zeugen und Geschädigte - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Pupils debate internet access at Kildare semi-finals - kildare-nationalist.ie</t>
+          <t>Ochsenfurt: Motorcyclist evades police control - police are looking for witnesses and victims - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 14:00:40 GMT</t>
+          <t>Sun, 01 Mar 2026 12:35:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPTWJxUFhsRzQzVmxqRXpJZG03bVcyemlKcUNGU2RxSXBYeVp5Zk5tSE5sV1pEYnJubno5ZFpuQXFuSGZfVTRPUldROEZLUFotRGkxNVFNQXBBOFp4cnU1LV9vZWtTU2RoYmdDLVdzQ2J1bVRUTGJYRUJQNW5YZWZWYXhyeWhZWWdaRHVOSVVFZVlPWW8tOG5qWXdyVEw2T2hQak0tYnFpdWVLa0Ew?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQVXA2NDNpRXpEUDRhemFHQktDR0U4NklXcE1iT1ZNSGdQclJvZlhwbEdTWmVGT3VzQ3RZc1ZINGc3ckp4X1lzbTM4Mm5wbEY3Yk82WUtxNGIzRWNxVElBTlZtb1FyNDZMdGZtZ0w5VFNtQk41ZkdPNGxCaFYyamFCWkdfU1g4SHFlTkM0UjNFbzIxQ09HYkNMY1BMall3RlQwVFVkcE5td0NSYjJUcTVFLXUxNlhvWGd6dFQ2aVpPczVMc2pCOGRiSjlUaw?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46082.5837962963</v>
+        <v>46082.52430555555</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Kildare primary school 'not fit for purpose' according to report - Kildare Now</t>
+          <t>Euerbach: Autofahrer flüchtet vor Polizeikontrolle - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Kildare primary school 'not fit for purpose' according to report - Kildare Now</t>
+          <t>Euerbach: Driver flees from police checkpoint - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 12:00:00 GMT</t>
+          <t>Sun, 01 Mar 2026 13:09:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNbzRkZllMTmxqd01mM1QyV3FDM2tyWDIwTFF6R1luYWxDWVU2MXFOMU90amFRd0tEWXRxbURFU3hZODlTREYzTXB6ZUJNVG1fTFRCS2ZsMnZ6ZThUUEZCTlI4bDFyZnZaUXp6dGloZmFCNGF0T3NxNF9Vcmh6VVQyWDlXZFZ5ZnJzcXR6bGVqMy1uZWNPZzFsTlJhWUxaVVpPT2RVLXp0VFN1Mkp1WUFQd2lyby1Vb2VGaGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQeVZJNy1mVGIzZ2V2emN6c3VYYWs3dFM5S1BPQ05yLV9UOGVnQk1NWUM3a3VZVlhNWnJYeGptS0tNSHN1cEtxX0o5VHFBc2t5X3ZWTGt4SkstOG9WZEowZzhVNkVTVGJDOEhZU242Z0d5VEJGZXVGS093bGVza0VYcXBvUFpjenRSWlI1UQ?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46082.5</v>
+        <v>46082.54791666667</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The two things you should never do when washing your wool clothing - Bicester Advertiser</t>
+          <t>Unfallfluchten, Autokratzer und Eierwerfer | Foto: Jens Buettner (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>The two things you should never do when washing your wool clothing - Bicester Advertiser</t>
+          <t>Hit and run, car crashes and egg throwers | Photo: Jens Buettner (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 09:35:50 GMT</t>
+          <t>Sun, 01 Mar 2026 11:36:26 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxQc3RlblhnN3BZTFNvT0RpRnBDNFMzdG5hOXhGS2FMUXhxdGh6THN5eDg1eTQzbG9vZjFxN2xwLXZmVXpDdzZUOU9aQjZqaE8zS0M5TEVEbFZnd1BHRUpuRl95cjFERmpUcVQ4S1dnZFk1d1MteVVlbEZlNHdtMm9LTmw2eUFSMTN2OGE0NHRyRlBqSGZHNjhPZElYbnJFRnVyZDZQODQ3UjRtaWhxWmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPS1hnZDFGQkVqeE9hRTlRY1pNbVBtbmRKbEkwSzZIQzRSVENyMFczOXllOGg3SUxYaG8ybngtOTVEeU0zWWZfZnFPRUdBYVA0NmVmSmVuZUs0OGJvdFFhX1VNWUZzaV9DdnRGcWRDX2kxZklMemw2SkdFaDFoZ0NtVHdXZEJnZnlRU2NhZDlLc05Kb2dLTnk3bmJ5YnN6QQ?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46082.39988425926</v>
+        <v>46082.48363425926</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>The one brushing method you should always avoid to help save your teeth - Bicester Advertiser</t>
+          <t>15-Jähriger liefert sich Verfolgungsjagd durch Aschaffenburger Innenstadt | Foto: Carsten Rehder (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>The one brushing method you should always avoid to help save your teeth - Bicester Advertiser</t>
+          <t>15-year-old chases through Aschaffenburg city center | Photo: Carsten Rehder (dpa) - main-echo.de</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sun, 01 Mar 2026 14:06:21 GMT</t>
+          <t>Sun, 01 Mar 2026 10:01:41 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQQlhIM2o4LVBqUDFMam82c3lCMHJSUlllTnA0cXVHUzlRb05QNEZkLUlWTjd3b0ZLRlNRTTNSWlgxMzBFV3I5cF9pbDlLR2dnaGJ5SzM5WG0yQkE1TGtXTmx3ZU9vZDdjTUJUcGZsVlVjX2pvdm16YmJ6bF83V3FKQkVMMlpXdm1NOXl0S3VUTTRXM2N3cnZMTzJNZ0Y2MmZ4aXJPaUdHUnJfaTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOd2twSWJDYWhXVjhyclZ1RF81NGxFbTUxamlzWm0xU1VKRk5OT3pGS0xUbWkzMWlpOEZCT1Q3UHFnNUlNb2xTTmdnczZmcThvVVp1RkJWQXRJd3hBT2NLN1o3TnNlZ3NXX1p4UDZhSVV2aWhoTGY3Ujc4RkFwczVtSThFODBRaDdra1V5ZjhSV1BWcll1MWV5RktjTDRaYzRMMVgwNEJpdTRwQnVLNWt6S3YxaWU3ZzJtUDdnVHFadlJrbmFhdlJtZlFB?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,76 +1945,956 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46082.58774305556</v>
+        <v>46082.41783564815</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Schweinfurt: Vermisstenfall Jakub Michalik – auch nach vier Monaten keine Spur - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Schweinfurt: Jakub Michalik missing person case - no trace even after four months - Charivari Würzburg</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Mon, 02 Mar 2026 04:46:00 GMT</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQcmJxZ1Q4T3QzNzFMbWJ4Y21pcnpEYmRyNEd6VHc0SjBibVB5N29ULVFlZjNKb2JnNEJCU09MN3J1N1I0eUFWWDhPV3p0a0xHd0VEalFBdlRsVHctY1MtM3dCeWxEODJNbk9oeG44UUdnWThwaFBnZ3E0b2RhcW5BUk9peXA5anlhTjJYbVdyVmJKNm50S0d5RU96MmprWWhwaWJOUUNjdGxlVjFGeElubEln?oc=5</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>46083.19861111111</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Blitzer in Würzburg aktuell am Sonntag: Hier nimmt die Polizei am 01.03.2026 Raser ins Visier - News.de</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Speed ​​cameras in Würzburg currently on Sunday: Here the police are targeting speeders on March 1st, 2026 - News.de</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 13:15:00 GMT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxOWEs0WUU4QzFMVWt2eS1pSnctVGxnLXBLQWZBZllOSkltR0JzTDRKdk1NUVlhdXNWLURtTUUyZXY0ZnVZZFhrQmxTNy1SdW5OYWNLc1RSNmtKM1lkQ2V2dWNLQXNSUm1JQWFDcG52YmFMVktwVW1KdGZRWVBUNURRODUtT2txZ3RvOEtTRlQtNVRqbV80VDF0eWRIYlB1R0lqek55bjNFWE5WWVQ2ZVo5LXFjVUgtSFJkUGV5WklaRGhENk9ZcTBTb0FYNUdEa0ZxS29McXpnZWJieUVmSE5ka0k0ZFpocXfSAewBQVVfeXFMTk5mTXF1M1NvOEZVVFhlTXk1eWg1YVg5T053TEtMRWNfN3NlWm5ENmZiSEVpTFpJVTc5M1hJaW5TakpNa1dLZTJ5LThOTFJsQndBVnY5MEFTTXQwSmZZcjZOckVISmloS2ZyVjlYU1NUVGRhc3RVRldEck4yZlJDa3pObHFxWFRJdTNUMHlIeXJ1YmpWUXRnLXJoeHZGMTl4M0ZyNVVkZDdkN1VJLWtrMkh3UU12cmxtcUlpc0FqSDVybmdFcTBxR1l4X050cW03S3daSDBhbHZmTXBpUzd4TmhqSHhwNDdzcmZ5UWM?oc=5</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>46082.55208333334</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Polizei-News Nürnberg, 01.03.26: Halskette entrissen - Zeugen gesucht - News.de</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Police News Nuremberg, March 1, 2026: Necklace snatched - witnesses wanted - News.de</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 10:47:02 GMT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQeG9XaEpTdFVBeGRuMjdSYXR1SlhLSS04X1hlaVFSY3Rnd0YtRzJNdFppVVRPTERnQkZrZWw2NUFndmhyRm1Wa09XT2hUak1lOEdWREI2TVdqTENZZldXZGVRQVJDZGhESHJnYy1na2Q1d2t4bndpbEI5dFdWUndpVXItb2oxYjA1S0p0N3o3REhIdUFlUUx0atIBngFBVV95cUxOWGtnVDZuUmZtbzQxRzFJUmhiUkh6ajNrb1pRS2lZXzV1S2JrYmQyUkJDdzFfUTF2bDVka2hmRlNTYU5zM1E5cDVfOWpJYVY2dDRYNEJuUkYzUUZYTVlBZmd1SnE4OXZRcXFjZlh4aGtEb09uQkdyMWhpVEE1WXM5eDZRWlpSX3lUSjFSakl4enctenUxblp3ZUJmNjdKQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>46082.4493287037</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Amtsbekannter 29-Jähriger tickt in Ingolstadt aus: Drei Polizisten verletzt - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Well-known 29-year-old ticks off in Ingolstadt: Three police officers injured - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 12:57:08 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiX0FVX3lxTE1nb0NGcXYtSjFUQkVJTnNHZDZCcXpRdi1mcENMVktDV2pyWWdtUklpMTZmaWtxdExjMDNJWjBuNmp0VHhVR1A2TDFtTXBKM3ljYTJlVmx4TG5vN0d2cmI4?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46082.53967592592</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Kontrolle auf der A9 bei Manching: Etliche Anzeigen für Fahrer und Firmen-Chef - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Control on the A9 near Manching: Several advertisements for drivers and company bosses - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 13:49:11 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE1WY0pYZ29WQVlFX1hMOE04QXpUZjViY0lqcE9QWHZfa0pMbjYzdnlSUl9mUHRNQTZGVWJmOVZFR2R0b0RfQkU5c3p3RzFpaVBmX2FBYk1wQXVBbXVDbGFOdkc1RUNsYUU?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46082.57582175926</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Aufregung in Asyl-Unterkunft bei Manching: 52-Jährige kassiert mehrere Strafanzeigen - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Excitement in asylum accommodation near Manching: 52-year-old receives several criminal charges - Pfaffenhofen Today</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 17:32:11 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBXY1dMRkpKMHJsWFNTVlJteUtiVmUyMnFwdnZCMXQ3bWRRX2wxUkJNc2hBUXphenRvWXR5SjA0Um9NSUlZclZQbjV2NWdkclFtdnhNMjBsUUxXaFRLc0hyRE9mV2R0aVo2NDNsekVXbVluVnc?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46082.73068287037</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Olivia Dean crowned as UK queen of pop among BRIT Awards 2026 winners - Bicester Advertiser</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Olivia Dean crowned as UK queen of pop among BRIT Awards 2026 winners - Bicester Advertiser</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Sun, 01 Mar 2026 07:25:50 GMT</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPUXFMbjZnaFZBWFlqR0xoSU1pTWpQVGY4SnFXa3NlOGhTSHdHYkkxdEpWSDVHZDgtY3V5VXZlU3AtbnBWUHFsWkl6cnJfeVJYOW5hcEJpa01HMXNhVDZZY3N5VTBpdGpDYnVoRld1VGhiN1pIQlAyWWlwLVlkRW82c3MzVTRKOGl4bjZac3VRdDdNWFB6RjRrZkF2V0piVEJ5V1AxUC1OVEoydG5LMDNCR3RsS3RhdHI2TThrN21xNA?oc=5</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Emotional Geri Halliwell fights back tears after major news - Bicester Advertiser</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Emotional Geri Halliwell fights back tears after major news - Bicester Advertiser</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 12:42:25 GMT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxQSnh6eGk4bkhzX0JmSkpfdVBnbjVOamVyQmp6T1JGUG1Fc2dRckZjU0ZqR3BHWXVhWEpEdmFtWDM5Q0pnQnBwS01kems4ZzdiVTFiSEtYa2liMERsaTctNUxnTnJRd0s5S0xDaUlmTTdzU0ZDbnFoOW56eWRmNEt4ZWYxdkRfTFpHQXJOeHBQZVN5WlpRQ2trQUstVTdFWFVkWnB6WkpEZjhLS1NPMHZSMjFR?oc=5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>en-GB</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>GB:en</t>
         </is>
       </c>
-      <c r="K29" s="1" t="n">
-        <v>46082.30960648148</v>
+      <c r="K35" s="1" t="n">
+        <v>46082.52945601852</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Six Roald Dahl films returning to Bicester cinema - Yahoo News UK</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Six Roald Dahl films returning to Bicester cinema - Yahoo News UK</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 13:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5mTFh3b0RaTmlseVlPMXZzQnBfZXB0enJuSVJGdlNvWHU2TTZpSTUxMkZqWHo5Nk9oT2lFWEU0aW9pUFZOajR0ZHBjZFh6c210X0ZRRmpWaVNDRUJUaDhKNUJXekx1RG56NFFTVDhPTDlKQmdrN2RGYnQ2UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46082.54166666666</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>St Brigid camino route in Kildare to be explored - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>St Brigid camino route in Kildare to be explored - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Mon, 02 Mar 2026 07:04:22 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNVXIxQkR5R0J0d0JRQ3NVQUFyMGp0aUlWSFVHaVlmdWtpUGx2SkRKS0RkODl2TFF3V1E2X2lsV2ZJMElHX1VUdHE5TUhER0xDeW5yWHFiamowZDNTRGV0bk9FSjhhYndJRk1EbjlnMjkxYlhnOXRPdjFUb19UUUEyakd6QkRwMG5ZUm1RT2dKS2tCaUdlQ2gyOV9WWWd2Tk5TNEtfbkF0SQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46083.29469907407</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Kildare train service improvement delays 'will impact housing and pollution' - Kildare Live Leinster Leader</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Kildare train service improvement delays 'will impact housing and pollution' - Kildare Live Leinster Leader</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 21:00:43 GMT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPeW82cnJ5RFdlT3NxbXptLXVmbDBHb1hwc2lROXA2eXFMQjlDaklhMV82WjdtMm5jNnFfYzJNWTRiYTRnVGNuWnR2Y25WMDU3eFpCUElHaV9CLTdwVktJMVZVbjhGOE1HdWw1cTR2MWdQQ1hXQVJxaGoyMWJ6QmhPdXdRSUM0cW5xeE9NdVhFSXZqVDliak10aVZHb0hyTk9Zd3BRWlVDQnlJSEpZdzhyVkRXVGkwSEJUaWtDMWU5Snlra2JxU2VyTFVIa0c2dw?oc=5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>46082.87549768519</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Kildare primary school 'not fit for purpose' according to report - Kildare Now</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Kildare primary school 'not fit for purpose' according to report - Kildare Now</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 12:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNbzRkZllMTmxqd01mM1QyV3FDM2tyWDIwTFF6R1luYWxDWVU2MXFOMU90amFRd0tEWXRxbURFU3hZODlTREYzTXB6ZUJNVG1fTFRCS2ZsMnZ6ZThUUEZCTlI4bDFyZnZaUXp6dGloZmFCNGF0T3NxNF9Vcmh6VVQyWDlXZFZ5ZnJzcXR6bGVqMy1uZWNPZzFsTlJhWUxaVVpPT2RVLXp0VFN1Mkp1WUFQd2lyby1Vb2VGaGc?oc=5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>46082.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Pupils debate internet access at Kildare semi-finals - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Pupils debate internet access at Kildare semi-finals - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 14:03:56 GMT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPTWJxUFhsRzQzVmxqRXpJZG03bVcyemlKcUNGU2RxSXBYeVp5Zk5tSE5sV1pEYnJubno5ZFpuQXFuSGZfVTRPUldROEZLUFotRGkxNVFNQXBBOFp4cnU1LV9vZWtTU2RoYmdDLVdzQ2J1bVRUTGJYRUJQNW5YZWZWYXhyeWhZWWdaRHVOSVVFZVlPWW8tOG5qWXdyVEw2T2hQak0tYnFpdWVLa0Ew?oc=5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>46082.58606481482</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Cathal Dowling hattrick helps Kildare secure vital away league victory over Down - Kildare Now</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Cathal Dowling hattrick helps Kildare secure vital away league victory over Down - Kildare Now</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 15:54:00 GMT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxNMDl3OTF1NlZKQkp3dEt0YzV3VWcyZU5nYzhEWGc4VHo5NUNPZHYzN1h1UWtXSmxZZXZOTzFFNmhpRkhkS21BWllPZVdVY1RtbWJIZmF6RHdzTE5aNjF6YnJmSUg4dkpJOXZKVU5GdGE0cDVBeURBRG10WlFUZnpwMEZCb092cGM4cDZ5dEdYbFBzb1FlQnlfY2x1Ymszb1plSkNiWEROVXZuN05rZklEeGxmdHdhdzU0VjFmN2dIdklyZU43c01ZVw?oc=5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>46082.6625</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Jessie Buckley: Hamnet role changed who I am - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Jessie Buckley: Hamnet role changed who I am - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Mon, 02 Mar 2026 07:49:40 GMT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPSE5UbG05ZXhhYmJRYmFCUVk2YjlwdDRHUlpfVGI0TmhhbnFfV3FjWXRjaWU4UnRNTTA2ejRhSXQ3SDJjVWNSajh1ZGJqRzZPWDh4MjRUQk5GVGxraERHWDRKcVhYU1dKUW1ScDlraC1KMWRjRFdUWkdQYW9IajRweDdJMWxRQmV4WFA0MkJoM0ZZOU93T0swc3RGNHhhX2xk?oc=5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>46083.32615740741</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Man killed after being struck by lorry in early-morning incident as gardai shut part of busy motorway - Irish Mirror</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Man killed after being struck by lorry in early-morning incident as gardai shut part of busy motorway - Irish Mirror</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Mon, 02 Mar 2026 01:40:15 GMT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxNNDBMUndkeDhKTTBBOXBocFptRjhrOVRoREpMck8wbmZlXy1YSWxYX1ZvNDFXQkZLdmRqcExHWkxnY0ZJZ3BocXRKaVRxeFlrUVlSSkhKS2dTR3EzY2h4aXg1SDJLczRKcmZ6dm1RenV6OFhnS2NYODFCaS1WOFpYbHZkcENrd9IBiwFBVV95cUxQNFRzNjFRbnRyVkxndW5OZmdlVG1YbFZYWGh3TjlKOWhlcnFpUUZKRDhwN1hySTVaM08wQlBPTDJDdjBHdGRuSVF4UzFzazUxZV9QSmtWMERFUTVISlB5Q2Y5MDZTYm9XZlM2RGJtVFJpbmlaLUFCbExPZ19mSm5XRU1GalRxX0lMdTVR?oc=5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>46083.06961805555</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Government has ‘given up’ on emissions targets, says O’Gorman - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Government has ‘given up’ on emissions targets, says O’Gorman - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 16:23:58 GMT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxPY2xBcVRCUkt3TGgzcUNSRWNPVEhDb09zLXRxTkt4NW5XX24yYlNwNEFYUVRyOEhCMjZEYUVKVWprOXFOeDhFZXB5bk1IQ2xVdEVRT0s4MjducjlSQkFGWmFBd2NXN2ZuLWl5cWZSaW9OUmsxSm5XNHBZRnA5TlVxcGxhYkVOb0NkeGE4YmpPRjVWX3djYzUydDBleHAtTXBmR09tdG5UTHlWWmM2OUI2V0JJYw?oc=5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>46082.68331018519</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Village Bicester Kildare (fallback)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>What the papers say: Sunday's front pages - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>What the papers say: Sunday's front pages - kildare-nationalist.ie</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Sun, 01 Mar 2026 11:33:53 GMT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxORW1hSjdTN0cxWkI5LXpXdm1RMzJVQ3FhUFhZLU1RVFNvN2ZSZXFaNDJzSkRrR0E0NXdGOVhLcS16TzdzY1NrYWdyaDZCM0pJbHdQR0NmUGZSaFJ1UTZwbVhSMHlud0RMcHRCMU9rVDJaZTRCNDE0UVVTQzQ3TkN5N09DQzNCdVpaMVRXVGt3VUl4WTIyU3VJT0VDQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>46082.48186342593</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-04 07:45 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail SA Unsponsored ADR (OTCMKTS:BMRRY) Short Interest Update - Defense World</t>
+          <t>B&amp;M European Value Retail PLC Financial Statements – FWB:7Z5 - TradingView</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail SA Unsponsored ADR (OTCMKTS:BMRRY) Short Interest Update - Defense World</t>
+          <t>B&amp;M European Value Retail PLC Financial Statements – FWB:7Z5 - TradingView</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:50 GMT</t>
+          <t>Tue, 03 Mar 2026 19:46:15 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQUDdDeWo5RzlVN0w5d2tnVmdEdngxcjRPbWpJeTZsM3dWWG52dlJ5enpWNXV1MTl6amp3VnlSWEYxQVNrd1F1RmtwSWdKaFJLTVVCSlNGQnBBLWg0Z0lnRzVJbFMwNF9aR0JYNy1JdVJoVmpUblhmNURpMXpQSUdrMjZKVDI5b3AtYnN5NVptMjBOY2N0aHk2VGR4U2tZUDRmM3VzWTBiUmhiLXVsYlpMV0ZWcjdDRFJ3dmJpTzhLRy0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFB5WG8yUE0xU29rT2hoaUV3T0J6NW80OEhtbTBWaDlScTM1cDQtdWtXRnJLeW5hMERhMDhXaDdaY05TYWZCdV9pbExFU2tJMU43NUpVbGVVN2Y1T2M3VUJHdnpDaDNXRmdPNmItcU5WX3FEQQ?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46084.33391203704</v>
+        <v>46084.82378472222</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - BBC</t>
+          <t>B&amp;M European Value Retail SA Unsponsored ADR (OTCMKTS:BMRRY) Short Interest Update - Defense World</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - BBC</t>
+          <t>B&amp;M European Value Retail SA Unsponsored ADR (OTCMKTS:BMRRY) Short Interest Update - Defense World</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 13:48:56 GMT</t>
+          <t>Tue, 03 Mar 2026 08:00:50 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5OcGdYb3UtdHZwRFRyTUg4UTBFc2FhTEhHa1dSTVVjN1B4eG13dWx6OThKV0J6aGVxV21ybENrbjJQWU1CQ2tidE1nVkZtNjJUX3BKWFBpRDJNdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQUDdDeWo5RzlVN0w5d2tnVmdEdngxcjRPbWpJeTZsM3dWWG52dlJ5enpWNXV1MTl6amp3VnlSWEYxQVNrd1F1RmtwSWdKaFJLTVVCSlNGQnBBLWg0Z0lnRzVJbFMwNF9aR0JYNy1JdVJoVmpUblhmNURpMXpQSUdrMjZKVDI5b3AtYnN5NVptMjBOY2N0aHk2VGR4U2tZUDRmM3VzWTBiUmhiLXVsYlpMV0ZWcjdDRFJ3dmJpTzhLRy0?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46084.57564814815</v>
+        <v>46084.33391203704</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>From solitary cells to 60-square-metre luxury suites in Nara, Japan - Travel Tomorrow</t>
+          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - BBC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>From solitary cells to 60-square-metre luxury suites in Nara, Japan - Travel Tomorrow</t>
+          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - BBC</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 12:38:18 GMT</t>
+          <t>Tue, 03 Mar 2026 13:48:56 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPSjNBS1ZkQm9HT05sTUUyOWFMckVYUTFLS01GZVFvOFpYVlgyY2V6c1o2TGlURE1WRE5OMFNFNzdQbGc0SVFEMjZ5YzdJTVpaTU5PbG1lbWlibVAxeVdVYW9sVU54UlUxR1ZkWkhBNVdUaW91U3pJazhaYjg4bkN4WnpNeE55QURFbmZ6ZllvT0tMUTRKSmp5WE5B?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5OcGdYb3UtdHZwRFRyTUg4UTBFc2FhTEhHa1dSTVVjN1B4eG13dWx6OThKV0J6aGVxV21ybENrbjJQWU1CQ2tidE1nVkZtNjJUX3BKWFBpRDJNdw?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -630,47 +630,47 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46084.52659722222</v>
+        <v>46084.57564814815</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gulf airlines resume limited repatriation flights amid ongoing airspace closures - Travel Tomorrow</t>
+          <t>REVIEW: 'Dhamroo in Headington is superb, elevating Oxford's extensive, rich, Indian culinary heritage even further' - Ox In A Box</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Gulf airlines resume limited repatriation flights amid ongoing airspace closures - Travel Tomorrow</t>
+          <t>REVIEW: 'Dhamroo in Headington is superb, elevating Oxford's extensive, rich, Indian culinary heritage even further' - Ox In A Box</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 10:03:13 GMT</t>
+          <t>Tue, 03 Mar 2026 16:22:36 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOaDNsMGE4d1NqeUR0WC1NVGpRSUVoSFo4MEVXNGJvc3V0YUtkbmZ2NXhRc1RLUE1xVVJnMWthaVplaHRILWRBRmhhYWhBZHA2Y2xmakUwa3A0TnRHcDRDZUZjZHRMUWZBSDhRWkROVGthaXBFT0ZhYjN3VjJ0cEdKNUxtYkJWZm43YTloRnAwMU1aanI1N2F2UkRERnV2Z0dRbXVkblZWb2ZQUTZZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPZzhidTZVdW41ZkxVc18xTFF1d0Q4Smx2OGZHa2R2dkNTWW5Jdjhka0d2c2gxV1dLLVc5azFPY0NjU21jY21nQkRKbTRjcThRVlp0UkdIaVdqbGlJb3I4THRrN3dMbHJreXd4R3ZwN1I5NXF6MVlTNUkxaEJHRzNpQVk2ZWVqUi1DaXFBYzBMQ0JQNmplRFdONFdkTjI2dUxfWTBfYXJoZy1kMmlDaGxQX0JiendYSTNpT3I2eERIbmY4R3k1WUN1S3gtMnRaZw?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -685,47 +685,47 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46084.41890046297</v>
+        <v>46084.68236111111</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Scammers target stranded Middle East travellers as flights resume cautiously - Travel Tomorrow</t>
+          <t>“De Hollanders willen mij pakken”: hoe een ripdeal in Temse uitmondde in chaos en een schietpartij - GVA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Scammers target stranded Middle East travellers as flights resume cautiously - Travel Tomorrow</t>
+          <t>“The Dutch want to get me”: how a rip deal in Temse resulted in chaos and a shooting - GVA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 10:53:30 GMT</t>
+          <t>Wed, 04 Mar 2026 04:30:13 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNcEhKbmlNTTNmaDNNeTdza0I3dlo0RVJxNHNmY1RCNkpHUW1CeGZ4T3EzZzM5SlVDR1pfUFV6ZDd2VkxBRVE0Z2FOaldOUVFCM2dXY1BaMlJaM0V3OTZXYzZ0aGFCZTdnbFk4eDhCQklmMTIzNWRBMHRDRmhFc3VTM2FKSU5VYk9XRmw3VTNmYjhqNEsxOUNvblBEVnp3UWJCV1ZqaXNDUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxPQ0wxRHBWd2V3V3lpMlBGbTV5WG5wdm45eEpxaC1OdHVHTl9wT3hxWkxMY3ZjYzNaUkVMVmpVWTRmcGxjVTdBSmM4OXk5UFJDQnlfcE1yTnZsLTlHb0hvdzNqcTU2akZmVmgtS2JhYWdpN2lZUU5rOTNaMG0xNlRqMzF0dTdCMFVsM3R2ck5ab1lrQnJBMmxGR0FFMi1uTF9JX29rUXpPeW9wUUZVUVRhVjh3VmNUb2R1THFkWmZJRXp5WFE1MzgwaU1WR2EzOXdHbnd0Q0duSmdwNEhHcVBNZUJnb1o1ejRYWE5PUG1yTlNUWFplZHRsYnB3?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -745,42 +745,42 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46084.45381944445</v>
+        <v>46085.18765046296</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Qatar and UAE cover hotel and meal costs for stranded travellers amid Iran strikes - Travel Tomorrow</t>
+          <t>Nederlandse rechtbank veroordeelt spilfiguur achter aanslagen in Antwerpen en Kalmthout | Foto - HLN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Qatar and UAE cover hotel and meal costs for stranded travellers amid Iran strikes - Travel Tomorrow</t>
+          <t>Dutch court convicts key figure behind attacks in Antwerp and Kalmthout | Photo - HLN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 12:03:18 GMT</t>
+          <t>Wed, 04 Mar 2026 03:41:26 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOVHpBX0U3czhQU254VDJtc3pEOHJuTklCQW0xR2dHTjZYVlVPQms0NGU1R2tMUGNTQ01DTjdFRl8zWWNmZnZBbllJSnFOWkpRNmRxLUFzYTJzSWtGdU9VUFNlTC1OR2VwMEpNR3lHTjZGRGlyMmpqU1lFeW5FV0FXRlNwN1V2V3pVYUpWZnpnY3V1bU5HUWhibWJwbGFQckF1azZQbDJqeFl0dXAtYTZz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPa3llNGRiVzV0c3ZtYS1icXVTT0xRdGJLQnA1bXIyb0FnMFFINzNCaUF3YjNIREZTTkFmNlF2c05NS1Z5LWF0THNBbWJ2VWZCWHNhZXRPWE9JbF9IQ1E5d0xUU2o0eGszbGNPUGFmZTJiMHhiaXU5cElWcDJrVTAtMjBaWDZ2VWdIaHB6VWIwekE1YldtaFhkbUhNdW15MkpfWjhEUjdzRVBmUEUxNERoSWl4VHprY25xLUlUZUJPQkNTS3ZrazRNRHlnMU1iNXhwRGc?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -800,42 +800,42 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46084.50229166666</v>
+        <v>46085.15377314815</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Le trafic ferroviaire interrompu entre Mons et La Louvière après la découverte d’un obus - 7sur7.be</t>
+          <t>Mehul Choksi, brein achter grootste bankschandaal van India, zit vast in Antwerpen: ‘Ik denk niet dat hij veel in zijn cel zit’ - De Morgen</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Rail traffic interrupted between Mons and La Louvière after the discovery of a shell - 7sur7.be</t>
+          <t>Mehul Choksi, mastermind behind India's largest banking scandal, is in custody in Antwerp: 'I don't think he spends much time in his cell' - De Morgen</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 11:44:00 GMT</t>
+          <t>Wed, 04 Mar 2026 02:00:00 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxQZDZSNnVsUWZDa3JORUI0NGFIMVM1M2RTWWxFOGlpelRpc2ZzWklYOHVWQTdERVptNlV6bUR6SWdrXzAyY3pnaERMc0ZzU1JYUEczVjR1Tk0wVlZEWVBYQzk2ak9fZXQ5ZkhGMG5zQUN2MFBoNmlkSzRJak1XdWhhZUp0UWZUazNEVVllcHFQc0VnenBRdlM5UWxvTERhZXk3VzR2aVdQVk05M0Q4NU5Gbm5TLVBNTnRvMmJIYW84aExRZ1cxSlFhWHlLbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxPaGF2cEdlN29zTmRyUWlTUlk3eUIyLUlNVWU5R0FkQjhWUTR2UnhuM0ZjNml3ZVBDRUtUNXNwd1FBNDFrRFBBTlo5SGZBQXBhT0ZkclVQMTFqa1dzVHhqUElGWTEzUWFjVFZwM0dtcXNOWTVtY1c5MkpQelZoWEstVnlYVE5kXzZwRHVtRFllc0E0ejdFb3U4dHlRSVlfQjFReUpsUW1naWM4RUt6T2tnR29NRXY0QUtOX251c0RDZVdGX25ZWkxmc3d1bm5CSEtoUG1HWDJaMEpLSFU0YnFPS0x6TE4yT1RKTGo0Y0pmRUE0QTJEcGc?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -855,42 +855,42 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46084.48888888889</v>
+        <v>46085.08333333334</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Politiezone LRH groeit uit tot vierde grootste van Vlaanderen en zet sterk in op innovatie en welzijn - VRT</t>
+          <t>“België moet extra waakzaam zijn”: advocaten vragen om zakenman niet uit te leveren aan India - GVA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Police zone LRH is growing into the fourth largest in Flanders and is strongly committed to innovation and well-being - VRT</t>
+          <t>“Belgium must be extra vigilant”: lawyers ask not to extradite businessman to India - GVA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 11:14:04 GMT</t>
+          <t>Wed, 04 Mar 2026 00:36:00 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNQzBHbHAyU01oQm5BQndQc3c4QW1fUENOU0RSNzV6djdtT0txQWhqQ0M0dURidnhBQXNFQy00c2Vxb2N0VEZTQkZNdmhtbmpFUm1rV001WXNnX3pWMUt2Y2JJYlhoUFdGXzlVVHlwbVp0N1pfYkRjV29ZWWhUMG5FUUlnY3BIalhCMk5YZXFvcFhyWWRNSEh5YmpiT0tmQ2czSnI2b2hUWjU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxQclFTMjExVXM3c1hjNWdaaHVsc3RxeU45X3BvLWpwRkU4MEF4VldCRmNhQW96U1dBNjRNZmNkRFlXWVR4X3Q5S2pBQXhhOEdKMFpqV21ncEc5R0VTdlZQM1ZZYWJQbmJXc2VyMlpvMXBuRzF6cUFLdWp4YlZNcTVmWExvUGVDRzRnRkViYjRsbV9wWHd6ZXlGVWlYT0c5N1ZvdTBRY2dOZnN0RWlSRms1akpWaXJBd1cxQ29qNjVReGhPYnZfMGh4QnpyTk9aekpZNnZOaEdTYUpzUlprR0lQWlZQLWJHc1FJUEN4TWlsNVd6OVdRMTMtdzhn?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,38 +914,38 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46084.46810185185</v>
+        <v>46085.025</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>"Jouer au Real Madrid sans boire ni fumer ? Je n'aurais pas été aussi heureux", la décla folle de Radja Nainggolan - 90min.com</t>
+          <t>Na noodkreet van De Coninckplein: stad heeft zowel “zachte” als “harde” maatregelen tegen overlast | Foto - HLN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>"Playing for Real Madrid without drinking or smoking? I wouldn't have been so happy", Radja Nainggolan's crazy statement - 90min.com</t>
+          <t>After a cry for help from De Coninckplein: the city has both “soft” and “hard” measures against nuisance | Photo - HLN</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 13:24:58 GMT</t>
+          <t>Tue, 03 Mar 2026 15:45:44 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxOcTlPUUVuNTU5VXNYZEpFcUVSV2drN0x0QVhuNDJlR0UzekxMYzNQRjZEWTBRRnFBSVNXOHhKbjdSdGNZRktHYlZDZkF6R0ZDQ2dhbFlZMFhhdEtSdWJSVWxKUVRrWWoyY0FmV1RaUEk1cWxucG5uX2dyRWg3Sm5GakIzZmUteVl4NzFOR3ZpMEZ2QnRXSjZHZGpOVUtyVjJabXY5X1VFUkVjU3BRSWZwdW44ZGY5c0ZfejJBXzVBOEQzQmJpRnRzVnRYX1ZjTWs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNRDY2VGluVm5jTmtYSjN2Sk9ELXZWTHE5UVJIdUlfSGpfd1dVWjZXeWxrdEZzdWtpT0xXeFJkTDFoVzE2ZnV1NGFQaTBmU1lFNWk3OVBqNndlS1V6MjNiTHVoalhfOE9Ua05KSTFrZEh4SFk1MVFvaC05OC0wNG1IVUthaVJIMmpBMzhCd0FCRlhjRlpEVTFudERJMVRDVTdHbWt1bE1nZmtXOXJ2VFJtSjZPSXYzcXVLOXpmNHVXWHdBQnlRSkM2YXdZa2VMTnNQS1k5YXFwekJwZw?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -965,42 +965,42 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46084.55900462963</v>
+        <v>46084.65675925926</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Motorradfahrer entzieht sich Polizeikontrolle - aschaffenburg.news</t>
+          <t>Marc Coucke staat voor explosie bij Anderlecht - Voetbal24.be</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Motorcyclist evades police control - aschaffenburg.news</t>
+          <t>Marc Coucke faces explosion at Anderlecht - Voetbal24.be</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:01:52 GMT</t>
+          <t>Tue, 03 Mar 2026 21:02:23 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQNFJMUnI2aHBGNWFoMUxrZGFMU210UUFnY1BpQjEwRklTZzY5d0NvQTJWRmVoMDcxa3dFSXJtbmt3NnpWNXJYbnp2blgzeTdCdFJwUEJrT3lDYUNqRWVqOEE5ZnNsTlZ0WE5XTk5KcWVHT1BQdi1GNUhnM0k4VzQ0WWduRXFXMDlUZkFIRnRKYV82czlOTUZYaFVPTmF6ejlFWGkyb21kMy1NTGdBSmh4SjU3YXJLYU5mbFNr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOenBXLWIzUzlpVEs5VmxpN0c5OXoxdlBldWZmaHBJTGtfYnhxRkJXc21WYmRZdS1ScHZ6cG5fX2VXYUdLb3k0dnVya2RLd2VkakpfMWhnMEt1ajBtQ19VeUEzU01CcEpLTFhxcGhmc0R6WEg5U1RGQ04zeHFpay1pYVQtRzVQaVJyaWRPYg?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,52 +1010,52 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46084.33462962963</v>
+        <v>46084.87665509259</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Würzburg: 20-Jährige springt in Würzburg ihrer Tasche hinterher in den Main – dann wird die Strömung zu stark - Main-Post</t>
+          <t>Brussels convenes regional security council to assess Iran war fallout on transport - VisaHQ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Würzburg: 20-year-old jumps into the Main in Würzburg after her bag - then the current becomes too strong - Main-Post</t>
+          <t>Brussels convenes regional security council to assess Iran war fallout on transport - VisaHQ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 12:25:00 GMT</t>
+          <t>Wed, 04 Mar 2026 01:09:35 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_gFBVV95cUxNeHhnMEw5TFQ1RjlfUmtic1BINHB0TjhuTE9PeVVsU1M4T0IxMXd5TXVOdnlxLUtMU0JQSG5rMWN6d0oxaGYtR1FQQVhua194UUpFMDRSNGVhRF9IZ3k5Mko0MzZBOUdhYVVDcTJCUTR2bTdzRl80YWVKOVhUdG16dWlTSTliZE4xYTZPOFRGSmJnQ21FeWEwQ0hROW1HUVVUM29uQXkyRjhqdjJYU2xGRTh5TzRDTXdGd05SOVhDLUh0VjNTWmpST0tGM2dfUWJlb0NiVV93Q2J0bnVJX0xNZU81Yk80RFI4aFp0R1Z0LUhiSVd4Y0FfVldJQ2FyQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNOU9vNTNLNUFZX2tzT0ZPclU2QmppTU1BdDk4RnZsdmNVN0tZQ1JpdkN0MmpHel82Sks0cHJYZ3VJbmhsVlA3emI2RHdwSkhWdDlDS2thbTg3OGxoaXhGSHRFUVlLd1h1dzY3MGxBcjFxbW5MMTFVVUtCU3UyZUlsbWlKSndXQTlmNmp4SzJVNW41RlR5empmdjgxT2VRNlVGMkZYeHdTUWR2UElEUmExN1Vlb2ZZWXltU251QmRURHNLbWN6?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,52 +1065,52 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46084.51736111111</v>
+        <v>46085.04832175926</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Couragierte Zeugin: Frau in Würzburg aus dem Main gerettet - Fränkische Nachrichten</t>
+          <t>Japan’s former Nara prison to reopen as luxury hotel in 2026 - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Courageous witness: Woman rescued from the Main in Würzburg - Fränkische Nachrichten</t>
+          <t>Japan’s former Nara prison to reopen as luxury hotel in 2026 - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 13:08:00 GMT</t>
+          <t>Tue, 03 Mar 2026 14:53:22 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNc2E2VHJ1WHJER2dBTS1KckNNN2J5MXhxTWNMZXUtdk1QT2FJdFFxTThyazA3OHVqSU5WZUdkSl9FdVJjTXFadk5jNGpSczZBN0s0MFg5dU94bGJJVjhlRzB5cklLSkNCWlpfczJFdmFQRzFxa1h2ZW5nTk5EbGs0bFF1RmpNVUt6dW9pZ2ZZQVloczJFbW1KUHRpVnlrZldhQzVHYlAydzRzbl9uZFUxYnNTWUNiOGhuaTMzdFVXZUoyNEM0NXNmRS11aWNhV09p?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxORXZ2Q3RxOGlvM0VYOVFqNGFZQW5uR1RhYThfWktpNVFPamZtU1p0anVJaWhuZ0VwWkRuZjI0SXJuUUktQjZnaW83ZHg4MXZKZGtxMGxxa0RRUnZrdUJMTHpiWVZsQnNEOVVoUlY1RF9FUlFZLUltdGpUaEFFWHRhbFhBaE9JbHFBS2pZdlM2Zk0?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,52 +1120,52 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46084.54722222222</v>
+        <v>46084.62039351852</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Nach Körperverletzungsdelikt bei einem Angriff auf eine junge Frau: Polizei sucht Zeugen zu Vorfall - Mainfranken News</t>
+          <t>Orbán and Zelenskyy clash again over Druzhba, with Brussels caught in between - inkl</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>After bodily harm in an attack on a young woman: police are looking for witnesses to the incident - Mainfranken News</t>
+          <t>Orbán and Zelenskyy clash again over Druzhba, with Brussels caught in between - inkl</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 11:56:53 GMT</t>
+          <t>Tue, 03 Mar 2026 14:20:24 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxNSXh2YzdNVG5LWVVHdHpqY0t0TmNSNUVnb2hmdXZocWt6R3pJbW1WaFJpQWlzV3ZWX0p3T0NzVHdPTEdFcWNudnBJYjRMRTdDVm9UNzB4RW1iMmV2R01QMjVPVTNPdFNnVENkQW1LVkFSUENsT0ZCend6UWxtVUJXVk9HUUlGZmt0d0lJa2lZa25UQ1ZLT0hEREpuZWdkNi05ZkJmY1NaN0Q5WTFEZ3NzenJCSFQyamZ0U3VsQnRNejY0aDdmMzNyczNDci12Wk1zR3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOX3RodzgzbUlvRzlDbUlIaXlsMVY4cGFlVHBpcXdIZVhieC1TOWxUcnIxM21JWWFKa3UzcnM2M1NWTWNpbERYVU5jV1JqWk9sRi1JTFFlQkdLeVBHYnNOaTF3VEpKcm1TZERPTHRTMmJ5QlIwQkZDRnBTYUhyMWhiOWstcTBlVnpwNGQ4a25pY05hWVVmMlFSOEp2cjJ2WVJWeDlTdQ?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,52 +1175,52 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46084.49783564815</v>
+        <v>46084.5975</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Geld bei Recyclinghof gestohlen - aschaffenburg.news</t>
+          <t>Scammers target stranded Middle East travellers as flights resume cautiously - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Money stolen from recycling center - aschaffenburg.news</t>
+          <t>Scammers target stranded Middle East travellers as flights resume cautiously - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 12:10:48 GMT</t>
+          <t>Tue, 03 Mar 2026 16:38:28 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOWVdzTy02UFpDU0RUaEZDdUVhZzVpTlRQUV94bzMyVFNQVEhfekhjVF9RMXRpSkhRaDZZSlZwQUU3WWdTTk5SREJCZHFVNUQxV0N3V3MtWHM2cVJ0a21GQUZQM1VDUUhrQzRMVlZOQ0VDUkJKaExUakdtT0ducVM1a3VHOFhiQk40c01LYmZtSFduUGtYR2xsZDMyank5azAzNXljRWc0S0xsLThZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNcEhKbmlNTTNmaDNNeTdza0I3dlo0RVJxNHNmY1RCNkpHUW1CeGZ4T3EzZzM5SlVDR1pfUFV6ZDd2VkxBRVE0Z2FOaldOUVFCM2dXY1BaMlJaM0V3OTZXYzZ0aGFCZTdnbFk4eDhCQklmMTIzNWRBMHRDRmhFc3VTM2FKSU5VYk9XRmw3VTNmYjhqNEsxOUNvblBEVnp3UWJCV1ZqaXNDUQ?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,52 +1230,52 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46084.5075</v>
+        <v>46084.69337962963</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Polizei-News Essen, 03.03.26: Erst entblößt, dann Beamte angegriffen und verletzt - Bundespolizei nimmt Mann in Gewahrsam - News.de</t>
+          <t>Gulf airlines resume limited repatriation flights amid ongoing airspace closures - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Police News Essen, March 3, 2026: First exposed, then officers attacked and injured - Federal police take man into custody - News.de</t>
+          <t>Gulf airlines resume limited repatriation flights amid ongoing airspace closures - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:39:03 GMT</t>
+          <t>Tue, 03 Mar 2026 10:03:13 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQR282WG9oUEV3czI4VkQ2UWs0MlBUam44eFNJaG1HdVRZcXo4ajFocE1IamwyX0dmZDRRbFYyalZoSXlrRDVDV0JqMzJlRHZISUtlMVgxVVZrZWRmOVRBOS1qNzJiWUx0T004UndMUjZONExYZkZkdFNaNDhWSGk2R25n0gGHAUFVX3lxTE9lRml3azhxUFZYaEFKV0xCeHN4NlNEbjNiTGMtcWl6ZlRqSmd2UzV3Ny1EUHRBX0VTdEJ0ZjVRRXNsd0tuWkJjblBLNFhHUWlMQWtwSm5PNGhaQjIxR3ZLUTI2S2FnaWVKT280NnhZRjNwN3hDekw2QmJiUUpLalRnR2gwN3o1QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOaDNsMGE4d1NqeUR0WC1NVGpRSUVoSFo4MEVXNGJvc3V0YUtkbmZ2NXhRc1RLUE1xVVJnMWthaVplaHRILWRBRmhhYWhBZHA2Y2xmakUwa3A0TnRHcDRDZUZjZHRMUWZBSDhRWkROVGthaXBFT0ZhYjN3VjJ0cEdKNUxtYkJWZm43YTloRnAwMU1aanI1N2F2UkRERnV2Z0dRbXVkblZWb2ZQUTZZ?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,52 +1285,52 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46084.36045138889</v>
+        <v>46084.41890046297</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Polizeifahndung Essen, 03.03.26: Mülheim an der Ruhr - Unbekannter raubt Schuhe - Fotofahndung - News.de</t>
+          <t>Qatar and UAE cover hotel and meal costs for stranded travellers amid Iran strikes - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Police search Essen, 03.03.26: Mülheim an der Ruhr - Unknown person steals shoes - Photo search - News.de</t>
+          <t>Qatar and UAE cover hotel and meal costs for stranded travellers amid Iran strikes - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:58:02 GMT</t>
+          <t>Tue, 03 Mar 2026 12:03:18 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNeEhBVjNKQ3IyQWFuQUF4SFNqV2FlSEF2ang1Ym1jSGZTd1lZSmt4bzR2QzF5UUtVTXZNRk12dUluajMzYWROYV9RZ21teUtMWjl4SldZVHc0VmRhSHIxOC1lUkFhRFFDRkZ5NUY4dmQxZGkxa0NfMElCbktqUXgwMTZTSU14VS1Peld1TWp5b9IBlAFBVV95cUxPaUxNUmctTk5ESXJTOGJxY1IxTElrLTlxQVhQeTJhR1k1QkVIeXpXSjBiOU5GRkVGOW14bFlvNEc4MlBYUTlhUmtvRTFkNG5xTjhPQUhkc3lOZWt3d0dyVGxXRXhLOHJySWE5YWtnSWdpOXdHMjNmVUFhTEZyS0xMSUQ4SjlWZnUzU1JMSk9WTHVkTjdf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOVHpBX0U3czhQU254VDJtc3pEOHJuTklCQW0xR2dHTjZYVlVPQms0NGU1R2tMUGNTQ01DTjdFRl8zWWNmZnZBbllJSnFOWkpRNmRxLUFzYTJzSWtGdU9VUFNlTC1OR2VwMEpNR3lHTjZGRGlyMmpqU1lFeW5FV0FXRlNwN1V2V3pVYUpWZnpnY3V1bU5HUWhibWJwbGFQckF1azZQbDJqeFl0dXAtYTZz?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,52 +1340,52 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46084.37363425926</v>
+        <v>46084.50229166666</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mobile Blitzer in Würzburg aktuell am Dienstag: Hier nimmt die Polizei am 03.03.2026 Raser ins Visier - News.de</t>
+          <t>Un feu de trottinette électrique force l’évacuation de 15 personnes à Laeken - BruxellesToday</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mobile speed cameras in Würzburg currently on Tuesday: Here the police are targeting speeders on March 3rd, 2026 - News.de</t>
+          <t>Electric scooter fire forces evacuation of 15 people in Laeken - BruxellesToday</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 09:17:14 GMT</t>
+          <t>Wed, 04 Mar 2026 06:50:00 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxNaVhMSGJlU0h0ZE5yX0pYdmw2dklXLVkxOW9iZVJVOFU5cFgzLUV3T1JTTVE1TkRNSU1LdW5fNzdEQ1hTRGpqRkQ2QmtVdi1fSlZWTmRXTDROWFhtbjVhdkQzTFRmSVhuOHkxQm1nc2hLWThGaUpUWWNoQWNZQmp6cGZ5MWR6R0ZGb0RsVUVKZlVhLWFvRWhDNXBjaTk0NTJrendEdkJRTmdCNFNvUXh6c3hIeGRYbmx0NGNfbFIxS29KN05uYlRMemFsX20xaDVXa21aYjhiWjFMaExtU19rQm9WRFRkN1h4aEt3a2Mxc9IB9AFBVV95cUxQWm50SS1NaFQwYXdEV2FHd09vZkU2aU5ZNi1vTVY0SWNpcmlYaUZGSkhWZW5JMlppQS1wMWVPR3BOaER4dlFteUZtS2EzQ01tVjFESGg0VzJsMW1id2pUbzdFZ3N3MTFEYldBYW1qU2cteVdqNGJXSVZrd0pjMFpTOTRuOENMbVlDMlVqRkR2dUJIV1B0OWlzUGZpeHJLMDJyZjdoOVhXeng5eFNOeW1hMllDU0NyaUxpV2pQcVdtTE5BTTZYdEp1VUFzTHBLQ3plc1VkZS1sMWgzSWJpTjN3dHpsYXhaNHpjaTZ3QWw2a3JlajNB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPYll3M3RrSlRzRkNFVU56VE1BLVNXYlhKRGpZNUNzV2lWYXYteVhuVWFkWU8zOG1GS1NCREh5MjJmS2dOUGttcGx5OWpRVnlESTIxUk5zOWk4Tmp3ZGRZOUt4SjRKOXFvOXpSOHRTTWNSbWdIN0dXcXlDUGNsbmNWbXI5NkxwRWVEZ2c?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46084.3869675926</v>
+        <v>46085.28472222222</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MSV Duisburg will in Ingolstadt mit aller Macht auswärts punkten - NRZ</t>
+          <t>Accident entre un bus et une trottinette dans le centre de Bruxelles, un blessé grave - 7sur7.be</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MSV Duisburg wants to score away with all its might in Ingolstadt - NRZ</t>
+          <t>Accident between a bus and a scooter in the center of Brussels, one seriously injured - 7sur7.be</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 11:39:47 GMT</t>
+          <t>Tue, 03 Mar 2026 14:20:00 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOOG8zal9jWVRFRDhFUkpVdDM5a3ZiOVgwN0N1Z1FyTW83TGtDZ2RDODg3MWlvQ0RwMlpMMUh6bWprSlBoSnBiazE2bC1FYlNQTzM1cVR6VWpnRk1lVWgzdEhjZWtkWEpOcUNrMEhDVHZXMlFxODZwbmNNVDRqbWpmUWc1VlVuWEh0QmRydWl5Y0JQY0phQmprOTdyTjJUYmdSVkNUN1VlSk1Hby1HNjVJTlZXS2YwVW5wWUZwekh1M0g1TkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPQnU4MW8xU2xJWUhPMGJMZDdyY1dUakw1Q1VZVE1FbURPNDd3RjhIZEpFUXJvbDJhT0c2c3F2M0xMQ3BTeUNseVRYaGV3NWdhdENINnBiaGh1bjQ4b2V6Y3EyZ2JoUTBFb0gyWk5UeHlLTmNkLUc4dk1PcVV0Z2FTemxGdzktWmZtT2dLNzRacW1mZUx2ZGxuRE9EcDUzT3JRdzZad3lwZGRCa3hwZ2ptNnpZODd4bHNGZ1Etd0liTWVIYUlGNF9F?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46084.48596064815</v>
+        <v>46084.59722222222</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>„Die Brandmauer muss eingerissen werden“ - SZ.de</t>
+          <t>Pendant que Meeus savoure sa première victoire de la saison, Van Aert vit une fin de course cruelle sur le GP Samyn - lanouvellerepublique.fr</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>“The firewall must be torn down” - SZ.de</t>
+          <t>While Meeus enjoys his first victory of the season, Van Aert experiences a cruel end to the race at the GP Samyn - lanouvellerepublique.fr</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 14:00:39 GMT</t>
+          <t>Tue, 03 Mar 2026 17:47:47 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQRTB2RG5rbTlia0xPRnJNaDNKazNkUHRkM2tpU2NwS3FPdWQyM05yM1pDUV9sYUVJTjBKdTZROWktNm81alcxLUtMRmQ1VWRxRnU3Ukx3RTNRenlxMnBBckw2Rno2R0JhWWpOOGkya2hmVlN0eGtXLUloMDl0ZUw2WHYxRXJxREZ2dXRUWEtmQk5KSzQ5MlFISGRlYjdfcXoxdUFKaEo2X2JSY2s?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxQeGNhNjdob2ZlcGlsTmFwMzNveFFGUEdObjcwRk1xXzBvZUpaVzJRT1ctUFZLWjhqUGFzMWl5N0FNcFo4aXBfQW90UWVOWWllNzVaZ3g1ZkhQVk1peDItZzZVTXRVQi1CUEpZbm85QUljdkhBZW1XemM4ZWtIU0Z6ekIyLUdBb0YtUEF0SWp2b3c1VVpIRWxQUjNUQU1yX0ZfLWFwZGZlOHo5OW5yYkhwSDJMQzk2MEpyanFVOXAzZXdyYTViN0lMVDVPNmJNakx5ZTlJNnctRllidGtqSjJJTjJ1RWFtWlVZRnhFaWNnNUp1VS1VQ2JGOFZhOWc?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46084.58378472222</v>
+        <v>46084.74151620371</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ingolstadt 2026: Die wichtigsten Events und Konzerte im Überblick - Joyn</t>
+          <t>Dossier saharien : Bruxelles et Helsinki appuient le Maroc - Perspectives Med</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Ingolstadt 2026: The most important events and concerts at a glance - Joyn</t>
+          <t>Saharan file: Brussels and Helsinki support Morocco - Perspectives Med</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 13:16:32 GMT</t>
+          <t>Tue, 03 Mar 2026 10:07:00 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOQW5wT3NsbThvWjJzNU9YZXFDTTEzc0dPMG02MFlCVDdtYzZoRnBMSkNpblF4bFF3b2p0RWQtckduOV9sNkdEQ1hvZEI4bzNWNHZFN0RNaXAzbEs5TUVwNjdxQWU0V3lXZWpWbHRKeTRrX2Y5UjgtMTQwTEh2RXJSUTRkN295aHJGZXptVnZTUHBZS1AyV0pIZlRkNU1nLXAtYWU4QWk4MDJhZWJrZWREbEFkTkk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPcGtuZU9VcVhXVDhuZ0Jxc3dwMk9oVk9IOFRDOTR4bHozLXFBaFpESHlmaXQ5Q0lmU05wOVpOYzFRUnktY0M2U1dLVjZPYi1yenB6c05uRHFhLWdyLW1OWFl0VDMzSHlkbklXVVRhRzNLSEtnU1hkd1pqRVhLcUplNnJ4WndlNDgwWDJoQkhR?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46084.55314814814</v>
+        <v>46084.42152777778</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Noch bis in den April: Bauarbeiten und Vollsperrung auf der St2214 zwischen Ingolstadt und Neuburg - Augsburger Allgemeine</t>
+          <t>Politiezone LRH groeit uit tot vierde grootste van Vlaanderen en zet sterk in op innovatie en welzijn - VRT</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Until April: construction work and full closure on the St2214 between Ingolstadt and Neuburg - Augsburger Allgemeine</t>
+          <t>Police zone LRH is growing into the fourth largest in Flanders and is strongly committed to innovation and well-being - VRT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 11:57:07 GMT</t>
+          <t>Tue, 03 Mar 2026 11:14:04 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxOSU1LWDd5M0FZWl9KZUZmMWQyWUR3aWxFS0JQZVExUGNPOE96cEJIUXBxTUVydVJRT29tR0NVR1Z1c093UnplXzBlOTQxUmIzczJDODM3QWYxd3ZBZ0lmM2xWUFlmVWdibjJUem5tblAxbkE0bHhOWThLdDlaOEU2U2tNY1NfdzV1M3U2WFo5UmFOV3dkR3VEWHdOdTZKc1JJS2VFcmczal9sWk13ZWNtY1lZX20zeTdW?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNQzBHbHAyU01oQm5BQndQc3c4QW1fUENOU0RSNzV6djdtT0txQWhqQ0M0dURidnhBQXNFQy00c2Vxb2N0VEZTQkZNdmhtbmpFUm1rV001WXNnX3pWMUt2Y2JJYlhoUFdGXzlVVHlwbVp0N1pfYkRjV29ZWWhUMG5FUUlnY3BIalhCMk5YZXFvcFhyWWRNSEh5YmpiT0tmQ2czSnI2b2hUWjU?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46084.49799768518</v>
+        <v>46084.46810185185</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ingolstadt – Duisburg Tipp, KI-Prognose &amp; Quoten | 04.03.2026 - Wettfreunde</t>
+          <t>Leegstaande Euroscoop in Lanaken krijgt opnieuw vandalen over de vloer - VRT</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ingolstadt – Duisburg tip, AI forecast &amp; odds | 03/04/2026 - Betting friends</t>
+          <t>Vacant Euroscoop in Lanaken is visited by vandals again - VRT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:17:08 GMT</t>
+          <t>Wed, 04 Mar 2026 07:05:11 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNYndrMHNObHBnYW16UkJfMklTelp4Z0Y0SGNhTkFPY2UxTzBtLVNkVDVzbFd4S0szcmg4UnVrRGJTRjlJWkppNkxRVjBjWmNUTHNYd1JUeGFHZFl0UWdfbElqRndfLWhkVkt4ZEI1Y19OTlpTOVg4MC1RZzhJeTVERnFHOEtsVE9kSFl5RWJEcWFSaHc2TzVZS25hZ2tiNUk2X3JB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQMkp3Q0Y2TE5WdzZWbzNMOXM4cWxsV3BjS3ZJbFR1cmdiWGhsT2FFd3VmX2pJa1YtZDJHR29meURRaVIxMll2TWF3UWNZb0JKSnJwOFhxZUoycEY5aTkwMGw3ZTRkSDBIdHNZb0szcVB1ak1fa25nQjNOTlVXNFBFaVphY3RBOXlxby1RcHAwTUczMUkwX2V5MlZQQQ?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46084.34523148148</v>
+        <v>46085.29526620371</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FC Ingolstadt 04: Nächstes Spiel in der 3. Liga gegen MSV Duisburg - News.de</t>
+          <t>Man (38) uit Maaseik veroordeeld voor belaging en mishandeling vriendin - VRT</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FC Ingolstadt 04: Next game in the 3rd league against MSV Duisburg - News.de</t>
+          <t>Man (38) from Maaseik convicted of harassing and assaulting girlfriend - VRT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:30:28 GMT</t>
+          <t>Tue, 03 Mar 2026 16:15:56 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQeU4wYlprcDlibEJOQzlWN0xsclJEVmw2bHhMbnJpbTFCNGE0SHV5elpyUThqZ1ZxTWlfeDVNUkdROS1lSGpVS2h0LWk4cnpFSkFGb1hmNDM4aDFNOVlHQWpfSjNtUzJmY3RSS1RfZUNZOFBOejBYamJBV3pBYTdLbUpvX3ZtRzJjUFJFMjVxbnU4ZjA0MGNqc29wYW9jX2lBbW5TVlRCZnJGaWZjREM1QzgwNnBtZENUSFktSktBVmhqQVRvZ3c5cEs2Qktia1hPRjhTVlZTRjVGWjNvUjlUUjAxRWJnRTVzMExNcWpTdzlSWF9KM3g3SmFlZGRXMmJuR1kzM3cwZ9IBjAJBVV95cUxNY2I3R0ZleTRXREVwRjZpdGZJSDhyVjJhclFjd24zTWsxeWVOemd2QzlHRUtiWG5pZmpTX0VsT0oweWQyMGJlUGtCTTl4U1ZDMVJmTnpvdVk1VFRvcm9WNzdNZlJJMTUwVDdNSzlTTFhpYnd1bG1INHZGRXB0NkRIdldJVlZXakxoX1NsRU9zS1BLNXNwTHZzOG42RU1CZVRoRUMta3pBZXJySjF4Q2tTU0dnMXdzLUh5YVowS1RMdWdIV1JlLWh6b29jZ3VQQm5EZWhHSXlmbHhzcXMwclR3RnZiY0FEaEtpN0lkQkRKaTJmQmxnLWdTaGtsbWY4dkZYQXhPRmU4dHdnNmoy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOR0ZuWWktRWVtekNncUp5WVg2eDI4MTB3QXBoNlhrQW56aHZmNERBVzBJNEd3LV9CbWRCWnk4YXpsSEtTcmRXcmpvczZLNnF0d015c0J5RG9yWlBkNExvcVRtWFd0ZXZpNDhqQUllOXNCTkVjWkh4VlhnX2g5M1VxOTdBQ1FEVUJFUWJOSDM4NU5WSUVKUUVUTzZZRkszVU8ySG00c2taWlc?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46084.35449074074</v>
+        <v>46084.67773148148</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BRK Ingolstadt: Sophia Bartsch zur stellvertretenden Kreisgeschäftsführerin ernannt - Donaukurier</t>
+          <t>Présidentielle 2027 : « Je ne souhaite pas être Première ministre », déclare Marine Le Pen - Ouest-France</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>BRK Ingolstadt: Sophia Bartsch appointed deputy district manager - Donaukurier</t>
+          <t>Presidential election 2027: “I do not want to be Prime Minister”, declares Marine Le Pen - Ouest-France</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:58 GMT</t>
+          <t>Wed, 04 Mar 2026 07:00:35 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiS0FVX3lxTE9ndFN4ZUlaQjNDcFVHXzduNkR1S1BWUlFRcjRWaGJIY21wcl82dmV4QkpfWC1odVZjN2pCQ292S2FUVjFnX3gwamlhcw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNaXpoRXJLeWJJdF90aDdBaTlRblZrSGI3U2JFOFJ3UEgxSzlvN3FEZ1FyR0xrTHBrUUI2QjlsUXJZUnh5M1MwYzRySzI5eXhHbGNXNy1KZTZ5RDNmREZZTER6MzJ6Q3JoSUpQcGpzUGdReHRaNS1wc1l5U0hUWV9uMDhFZ0NGNkJBWEFmbm5Fa3RFX29yQUxyY1d2WGZqdHJvTTJTOWhWZHcxY0gtTVczRjdSQkhpcG5POHFEandoMlpSVGJGREY4Z0dkN1FMWWtfZk04dGROYmRZNWZHcUFacHVBcVJEd3ktZXN3T0d6dEZfWTE4XzY0MHZQckgzenZtRUE?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46084.33400462963</v>
+        <v>46085.29207175926</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MSV Duisburg zu Gast in Ingolstadt: TV, Anreise und Schiedsrichter - NRZ</t>
+          <t>"Jouer au Real Madrid sans boire ni fumer ? Je n'aurais pas été aussi heureux", la décla folle de Radja Nainggolan - 90min.com</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MSV Duisburg visits Ingolstadt: TV, arrival and referee - NRZ</t>
+          <t>"Playing for Real Madrid without drinking or smoking? I wouldn't have been so happy", Radja Nainggolan's crazy statement - 90min.com</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 14:34:00 GMT</t>
+          <t>Tue, 03 Mar 2026 13:24:58 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPUXA2V0tHY05YSnpLSlEyc29makk4ekVNeTF1RjZtV1IxMlEwazhCTnNsSkJiakVPeEZ4MnBsRnoxRkZwYVR4a2VqRlJPMDVhVGxnVVpzajdGWllheDNzSTFmeHFpNW13RE5sczhaTjdUMHViUmVGM09rajJWaGdIM0xCVXp4YXhiMDhiZEdBazJxd0ZMNWpqejRJVVB0eGxjcXNZWEU0R3pWVzhrRThuNnNycVBUa2dNZmF0T0FyaEtoUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxOcTlPUUVuNTU5VXNYZEpFcUVSV2drN0x0QVhuNDJlR0UzekxMYzNQRjZEWTBRRnFBSVNXOHhKbjdSdGNZRktHYlZDZkF6R0ZDQ2dhbFlZMFhhdEtSdWJSVWxKUVRrWWoyY0FmV1RaUEk1cWxucG5uX2dyRWg3Sm5GakIzZmUteVl4NzFOR3ZpMEZ2QnRXSjZHZGpOVUtyVjJabXY5X1VFUkVjU3BRSWZwdW44ZGY5c0ZfejJBXzVBOEQzQmJpRnRzVnRYX1ZjTWs?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46084.60694444444</v>
+        <v>46084.55900462963</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Unerlaubt in der Fußgängerzone unterwegs: Polizei Ingolstadt erwischt Rad- und E-Scooter-Fahrer - Augsburger Allgemeine</t>
+          <t>Cambriolage du musée du Louvre : l’ex-présidente Laurence des Cars annule sa venue devant la commission d’enquête - Ouest-France</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Traveling illegally in the pedestrian zone: Ingolstadt police catch cyclists and e-scooter drivers - Augsburger Allgemeine</t>
+          <t>Burglary of the Louvre museum: ex-president Laurence des Cars cancels her appearance before the commission of inquiry - Ouest-France</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 11:57:19 GMT</t>
+          <t>Tue, 03 Mar 2026 17:23:26 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNNmtqcWw2djRyX2xZN3dBOFBPLTVsS1JfN18xRGJTU2VVMko1cktrakp1N25VMjE2cXJHVnBiYkh1Z3BmR2VtVnJXTjdWYkFYVEgtQTRUeURoenBTZGYtbVYwN3FmZ0hpcnB1LWF5X3U4NllIRjBheW5YdjZLbFBIcnhsdTNYQ0lHa1JWYktKM1hiMkpqVzhLNTVYdmxJVF9naVFnRmtpS1N1VHdvR0hlTUNvam1Ec3NqcjBPQUxR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAJBVV95cUxNbUpRSFZ1S3dkb1FyUEVhUm9jamdENGZvSjU4dVJob2VWeGVNSldLaGl2QVJEalBPZVhyRXY5czhEODVRSmxGMHhLaTY2UVQ1SnBFYzJDR1F1TFhUMUxQa0h6cDFuZkpJMjZ4bEpKS2pOWWlVUE9wUWNVWkZRal9xem94dmxyN1FtOGxmQnhkLWtzc0s2ZTg1UjI2VkZ4blZxTHkzUTY1VXoxcUdtX280YzFpWFF5S1NhbHVuaERJd2xUQWo3cFlnY3JRdGFlOFIwYjhMbnlqVXhJTWUyVjN2NG1xLTh5TmZDZVhzVFlrYzJOX1dmbGl0Y0ZpZlBaaUVZUDgzRmVZNHZ5aE1GdUs0WUdQRUlzTGd5?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46084.49813657408</v>
+        <v>46084.72460648148</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>„Ich schlitterte immer mehr in die Abhängigkeit“: Wie drei Ingolstädter von ihrer Alkoholsucht loskamen - Augsburger Allgemeine</t>
+          <t>Super handball League - Bocholt déroule face à Bevo, Visé gagne contre Eupen - Starsporttv</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>“I slipped more and more into dependence”: How three Ingolstadt residents got rid of their alcohol addiction - Augsburger Allgemeine</t>
+          <t>Super handball League - Bocholt takes on Bevo, Visé wins against Eupen - Starsporttv</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 11:00:00 GMT</t>
+          <t>Tue, 03 Mar 2026 23:04:31 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPNUxMVDVsTDNRUWFDeGVDaVBGMVg0NEhTQ1IyZjl3NktQXzRheFp5WlBTVW1JY1h2dHQ1OFBNTHd6QTh4WHdJYlg1YzVKSXM2VFdBT1NvbU5MRnZmdVRyZWZNNEhmaXlNc1I4NzJxby1HTFNYekJnbVRiS2xkaTMzWmtoaXM3TU1TYkljckNPTHZMQ1VOUW15c0NNUEdJT2Q2NHpSNkpVWkxReWZIWklFV1UzeWEwTkpuR0daWFFRamd5aEZJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxON245ZG8tbl9WNGVUZUk5enZRaWI1R2FMLXUyc2xkbktOY296d0ZFUHZGcC13UW5NYi1HZzBNZ21oTmFnY0UwbFA0ZXdFUGduQl9PTXlVVkpoQ1YzaTFkbHNCSktDTUlMa1B3bUZQTlpOSk9UWFotLWxUejg1TDQySms5anFhU2tzT0lLcHhVaEk3VmFVb1FaVUpDNldfaDVOc2hkeU9rVm9QWkU?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46084.45833333334</v>
+        <v>46084.96146990741</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ex-Schanzer Sussek: „Jetzt habe ich den richtigen Verein für mich gefunden“ - Donaukurier</t>
+          <t>Glasgow to host UCI Cyclocross World Cup in December 2026 - Cyclist</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Ex-Schanzer Sussek: “Now I have found the right club for me” - Donaukurier</t>
+          <t>Glasgow to host UCI Cyclocross World Cup in December 2026 - Cyclist</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 10:45:54 GMT</t>
+          <t>Tue, 03 Mar 2026 17:56:46 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiS0FVX3lxTE5NT3ZtYXFxR2FuT2JUaElFem02UTRwdWJyRkZvWDVBNVJpVlREeml2cmROUktsMFFNdXE3ZFlRSzN5RDA2Wjd5LWp6bw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE95UG5Yek51VHZwQmtmMkhsVmctb0lOVmFzQm5HalIzUTNyVjVaS01pcXJkRzNpdXRaTW8zdmluSl9OQzFkdmEyMklOaWpNUmRhNlBCUS02dnNnQzdxTVE0ZkZYRFZqSGpNQjZEbjBsWG14ZXVKQVJF?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46084.44854166666</v>
+        <v>46084.74775462963</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Kunden vor verschlossenen Türen: Warum sind im Westpark Ingolstadt gerade so viele Läden zu? - Augsburger Allgemeine</t>
+          <t>Maxim Van Laere - nascar.eu</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Customers in front of closed doors: Why are so many shops closed in Westpark Ingolstadt? - Augsburger Allgemeine</t>
+          <t>Maxim Van Laere - nascar.eu</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 09:30:00 GMT</t>
+          <t>Wed, 04 Mar 2026 00:10:51 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5gFBVV95cUxQQmdZSzJNZmxDSHpQcDJKcG1wOTlZNlBlRDR0UUE0a3VFQ05ZbTUzR2lZVTFkNU1mT3VMV0FacHhlRjF5LXpZazdCalZDVFRVazZKUW42ODlybnRFbnNzODNYeElBeDZUWG15LVpqb1dUZmp0bDh2a2tyaVVBWDdpcktfZmh0d0lqM0pFZXNZMFdZQ3U1MkR5bFl6dmFtQ1ZoUUdiblZyeFJaLUxPWG1RbjU5MG81ZDJ3Y0JGZGhNNF83aFRqT1BIaWpOTk0tX1NIdTBhNDVVTElaWWticDFTX3phOVdjUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE5lTWhadGJfQ2M5Y0IzRXpncVlha1FyMlBDMUZlOUVZVXV6dG5tWWstaTFkNWhvcnNFQVJ3R1BTcGxTa18wX0pSZVRXU2dWZWdKaUVHbkNJNA?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46084.39583333334</v>
+        <v>46085.00753472222</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Ingolstadt")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ingolstädter Friedhöfe decken nur 60 Prozent ihrer Kosten – Gebühren wurden erhöht - Donaukurier</t>
+          <t>Polizei sucht Zeugen nach Körperverletzung in Würzburg - Newsallianz.de</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Ingolstadt cemeteries only cover 60 percent of their costs - fees have been increased - Donaukurier</t>
+          <t>Police are looking for witnesses after assault in Würzburg - Newsallianz.de</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 10:00:41 GMT</t>
+          <t>Tue, 03 Mar 2026 14:50:38 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxPMERxVWJ0Q2ZBNkxTWXRQVlZUNVJlZTZRREtfeGhDeElDS1ZmMGF2cndBWUJNYm9FQjBjUHIzQURTMzVtaUlVSW5rZ2REaHhzRWFsYmZ6MFFkVGJBc1pfU0NzbE9WM3ZwNUNYME1vZllQV2FzdzEzUE9LQVN0WDBRZ2N1Z01WdzNlYUdJTnY4R1JoZk9WM0hjcUtYZFFNbGxVdkFIV0diY3JEcnBzRGJtWFlEdlgtdkE3aXF1c1FMVHhNNG1EOW9aX1F2MWdLNVBlR0tCZnBB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQU0wwMXNXYWtOU2NVamtSb1hPWXV3V1B0cGdJNVg5bGZYRzMtVEhIdTFzdlFrMmE0Y2NiTXRoa0xNV1VnV1Y0Mjh2MFVCLVVHSHFiOUhCYUhaY1VzQmpxWEhxUXg2eDZpeVQybHYyal9SY0pTMU0xSl9lV2lBVExDNGJSUHc1ZzRmQUZpakI0R3VFb21paFE?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2124,7 +2124,832 @@
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46084.4171412037</v>
+        <v>46084.61849537037</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Polizei Würzburg ermittelt nach Angriff auf junge Frau - Fränkische Nachrichten</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Würzburg police investigate after attack on young woman - Fränkische Nachrichten</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 15:10:00 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPS1FqWE95NFlIajJKZ1VRYy02QWVaTFc2a2hFMFNvdk4xNkN5Tm5JSXFXX0txRXV2YlV0ZVpPLUUtODR0Y3NIUTd2NFo1MGZ4aGtqdmxBWmticm9uVEdHTTJENE9NWE5kV1VyUWljVmJvdWFYcXRFM2wwakdnSXp6UDhFR2JXREJBYVI5cW4wZnkwaXEyQnhzZHUzWmhyOVpvNC03YXpVNkVHVDQ0YTd5LUNMNFo1WlJjczhYcnlCNGY4ZWcxZmMzSm92alI?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46084.63194444445</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Motorradfahrer entzieht sich Polizeikontrolle - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Motorcyclist evades police control - aschaffenburg.news</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 08:01:52 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQNFJMUnI2aHBGNWFoMUxrZGFMU210UUFnY1BpQjEwRklTZzY5d0NvQTJWRmVoMDcxa3dFSXJtbmt3NnpWNXJYbnp2blgzeTdCdFJwUEJrT3lDYUNqRWVqOEE5ZnNsTlZ0WE5XTk5KcWVHT1BQdi1GNUhnM0k4VzQ0WWduRXFXMDlUZkFIRnRKYV82czlOTUZYaFVPTmF6ejlFWGkyb21kMy1NTGdBSmh4SjU3YXJLYU5mbFNr?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46084.33462962963</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Polizei-News Essen, 03.03.26: Erst entblößt, dann Beamte angegriffen und verletzt - Bundespolizei nimmt Mann in Gewahrsam - News.de</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Police News Essen, March 3, 2026: First exposed, then officers attacked and injured - Federal police take man into custody - News.de</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 08:39:03 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQR282WG9oUEV3czI4VkQ2UWs0MlBUam44eFNJaG1HdVRZcXo4ajFocE1IamwyX0dmZDRRbFYyalZoSXlrRDVDV0JqMzJlRHZISUtlMVgxVVZrZWRmOVRBOS1qNzJiWUx0T004UndMUjZONExYZkZkdFNaNDhWSGk2R25n0gGHAUFVX3lxTE9lRml3azhxUFZYaEFKV0xCeHN4NlNEbjNiTGMtcWl6ZlRqSmd2UzV3Ny1EUHRBX0VTdEJ0ZjVRRXNsd0tuWkJjblBLNFhHUWlMQWtwSm5PNGhaQjIxR3ZLUTI2S2FnaWVKT280NnhZRjNwN3hDekw2QmJiUUpLalRnR2gwN3o1QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46084.36045138889</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Polizeifahndung Essen, 03.03.26: Mülheim an der Ruhr - Unbekannter raubt Schuhe - Fotofahndung - News.de</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Police search Essen, 03.03.26: Mülheim an der Ruhr - Unknown person steals shoes - Photo search - News.de</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 08:58:02 GMT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNeEhBVjNKQ3IyQWFuQUF4SFNqV2FlSEF2ang1Ym1jSGZTd1lZSmt4bzR2QzF5UUtVTXZNRk12dUluajMzYWROYV9RZ21teUtMWjl4SldZVHc0VmRhSHIxOC1lUkFhRFFDRkZ5NUY4dmQxZGkxa0NfMElCbktqUXgwMTZTSU14VS1Peld1TWp5b9IBlAFBVV95cUxPaUxNUmctTk5ESXJTOGJxY1IxTElrLTlxQVhQeTJhR1k1QkVIeXpXSjBiOU5GRkVGOW14bFlvNEc4MlBYUTlhUmtvRTFkNG5xTjhPQUhkc3lOZWt3d0dyVGxXRXhLOHJySWE5YWtnSWdpOXdHMjNmVUFhTEZyS0xMSUQ4SjlWZnUzU1JMSk9WTHVkTjdf?oc=5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>46084.37363425926</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Village Ingolstadt (fallback)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>FC Ingolstadt 04 vs. Verl: Live game updates, stats, play-by-play - Yahoo Sports</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FC Ingolstadt 04 vs. Verl: Live game updates, stats, play-by-play - Yahoo Sports</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 19:08:32 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOeEdEZWE0UnZickRnVkFJMjJZYXhGbUNyMldocDNRV0FhV0hIcG0tVUlvenphVTIzTVl1X2NsdE0yT1lCM08xTmJDd2FZVzR3VE1XRVhaT01iNWtEdkMtZ3dtdDV1NnFCR3llSmp4OHJaSGdqTXE3RVY1YmlfTlFUOV9n?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46084.79759259259</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Sciopero trasporti marzo 2026: quando si fermano treni, aerei e mezzi pubblici locali - ItaliaOggi</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Transport strike March 2026: when trains, planes and local public transport stop - ItaliaOggi</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 04:47:37 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOQzJqcF85TU9pOVRPcWoyYzFJYzJYRGx2X3I0QnI0cVJNRG05UUZCNl93YlEtUEpKZFZ1WnhXSlUyTm1ZbTMxQ0xKdURUaVNvd1RiaVFVUWdSWXpGNm10MzB3Vmp5WlcwSTY1czhaQUZoQXg1OHVHUDFmallBNEhmdWdLc0hpbmNzR1QwbGNxSUhjU29VS2huUnVKcjQ3dnNmby1MMENEOFV5MjVBRkJYLUgyeUxoZlE4ai0tY2ZQdzZ4cUtPTWlhc3hJNFVBUmZQYUdNbk5xV1ktRG5QdjZJSnJ3?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46085.1997337963</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Manifestazione contro la guerra in Iran: insulti e urla tra attivisti di sinistra e iraniani - milanotoday.it</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Demonstration against the war in Iran: insults and shouting between left-wing and Iranian activists - milanotoday.it</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 17:51:11 GMT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1rV1RFMGRuaW1saXNVdzRUU2ZQT1hBQ016SjlwS193TmN4NlZNZTdGa29SOFBfOEM2RDNKc3R5Zk9UaFBwYzIwdHE4TXZXM3A0LUpZajJuNl9KTjZsalg5dzY4aXZLN2VROW1mYnRjdWJ1QUl3YlJZ?oc=5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>46084.74387731482</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Protesta a Bologna, operai al lavoro nel parco. Sotto il carcere presidio in solidarietà con gli arrestati - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Protest in Bologna, workers at work in the park. Under the prison garrison in solidarity with those arrested - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 13:06:50 GMT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNQk90eVFYLXRKNXpjX2dwNEh3YlV6VDJQUG9UQ2lrSzc4Mk5hU09lQnBRTktOSExQelVFdVJzRUpRSldlUXpESTVDTzZqNEVTN3JZeFl6alZLQlZRU0FmOVBhbGxGV05CbXlkZFZETUJHMzQtdVZVcy0yWDVpUFVmRy1QdWlQMjJCTDZua3FhWjlwQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>46084.54641203704</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>L’8 marzo (e il 9) di Non Una di Meno a Bologna - Radio Città Fujiko</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>March 8th (and 9th) of Non Una di Meno in Bologna - Radio Città Fujiko</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 08:16:33 GMT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOSkhqSmFpMGxENUp4dWplZ1JvRm9WVkhoT0l0OFNZdWUwTkhjckYtLVY2a2NBSHp4NmdkdVVjN2E2X2dTVGMxby1TRmQzWWJ3c0ctbXhLNDM1QUVOV0QzTEM2alJmbko3cE9oVl95bnpBUTY5VVZEUlVpdmZHX3BDbEw1NA?oc=5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>46084.34482638889</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Scioperi marzo 2026: il calendario completo delle agitazioni sindacali. Il 9 marzo si ferma la scuola - Orizzonte Scuola Notizie</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Strikes March 2026: the complete calendar of industrial unrest. School stops on March 9th - Orizzonte Scuola Notizie</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 09:40:43 GMT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPTlZLTDNGWk9rdFhBc01zWkdKSFBua0xMSWdXZGg3S0dIWE1lVGdmdDV0ZnM4T0tfTFRzOTB2cUdMOFpvU2k1TGZRY3RFaTZ3bG5fYWpENndUNDA3ZWEyTVVzU2NLYmhKdmJyYWRsc1VubllKTUlHVnFtUTgzOXpuVzVQdWdqZGhMY3ByaGZaVURDS3JrbWxpbDE3QkszQ04zR2lkc2VEV3NOaU1uN2Jqb3d1NlBrcWwyWGxSVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>46084.40327546297</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Libera Masseria, da dieci anni simbolo di presidio sociale - Chiesa di Milano</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Libera Masseria, a symbol of social protection for ten years - Church of Milan</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 06:08:27 GMT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNRXFDNlozZS1kVU9ZX2Mtejh0TDdkYnk4ekZ5eVBSTVJCZW1rOXhVa3VRdkRQaXRGeGhMYlpidDJNNmFsdVVhSURtYkg4a005MGtFclZyOUtINkpxQ2JoTTcySjNuWlN2Vmo3dnVBS2RnRXRNejNZSG14S0VkdmJNdEhTNXN5d1VRUHZaenN1N1pHWkUxcWJ5bVpIclFFWnNZaHc?oc=5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>46085.25586805555</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Decreto sicurezza, una pioggia di multe per bloccare proteste e dissenso - il manifesto</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Security decree, a shower of fines to block protests and dissent - the manifesto</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 23:27:19 GMT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNOFV3a2hDcnZCQXk3OEN1M29RWVllOXk5bVBHUDdDSFdqdjJRWGpkZmtWYWN2cnhYSUM4aUU5N3VMdTVLVjJ6NWVzNkp5VXVJbW9RcUVETXF2cVRQcW1rRVNfWk05TWdTMjVVNENHQ1I1ZjBWalU1SlBONFFlTTM0QlNYeWl2QWc0TkRtQl9sa19Ybmk3VVFQSk1n?oc=5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>46084.97730324074</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Bufera Marelli: bonus solo agli impiegati, scatta lo sciopero - BolognaToday</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Marelli storm: bonus only for employees, strike starts - BolognaToday</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Wed, 04 Mar 2026 06:58:55 GMT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE1EMHk3T3ZKUjFscGhxNUllb0dfY29FVHpPbXBrLVlRUk1iUmFqaVlRRVlCaFM3R3EwakNwQ3NHQ3MwRVJMLXUzcktmNzhEVHg5NnBzUXRLbWRSMXh6NXoycDBvVkdndXMxOUdOZXpNRkFjQ2pKZmdRSFRpSQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>46085.29091435186</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BOLOGNA: LACRIMOGENI AD ALTEZZA D’UOMO E CARICHE CONTRO I MU.BASTA. “IL PILASTRO NON SI ARRENDE. LA MOBILITAZIONE CONTINUA” - Radio Onda d`Urto</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>BOLOGNA: TEAR GAS AT HEAD LEVEL AND CHARGES AGAINST THE MU.BASTA. "THE PILLAR DOES NOT GIVE UP. THE MOBILITATION CONTINUES" - Radio Onda d`Urto</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 17:03:00 GMT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxPeXYzSTlPeHl3YURqRmZBMF85QnBDY052czQ5R2oxWUpDbDA4SHZoVm9RdHYyd1NsR3gzUzFnNFNrcXViMVVRWE1Rcm9qS09TSHp3aTE0WEVjV21tVHZUTzVyem1xSWhXeUZwdFo0cUZ3MlB1MHBEcjlxN1h5bzlQQmlXYWY2cmRObTY4SkRGSHJKdHVoODVZYk9mVmUxenI1b1BROXN6cC1tNzFfbTg1RDItX2pycWlTV1lpM1lub2pxdE1mSDU2MlpJRl9xQ1hyUWNlczJ1Ukk0Y283LXRhV0V5YVhMNGVvX3p1LUl5LUc?oc=5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>46084.71041666667</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>No, la CGIL non ha proclamato uno sciopero per “la caduta del regime iraniano” - facta.news</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>No, the CGIL did not call a strike for "the fall of the Iranian regime" - facta.news</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Tue, 03 Mar 2026 14:39:03 GMT</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE1uNE8xSWNWZFB4ZE9kS2paaVdWTENqc0loVDR2N3hYR0g0eEJZVkdiOUVtc1gyUy1BMjV4NXhTdC03YTF4ZjVhRGZlaGRaLW9zY0VnVmtqUm1tYjN0NVp0Rk41YWNLLU9hWEFOTWFNR2FFbzhlTkktUzdB?oc=5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>46084.61045138889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-04 14:40 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail PLC Financial Statements – FWB:7Z5 - TradingView</t>
+          <t>Scotch Corner Outlet Village targets £25.5m via stock market funding - Place Yorkshire</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail PLC Financial Statements – FWB:7Z5 - TradingView</t>
+          <t>Scotch Corner Outlet Village targets £25.5m via stock market funding - Place Yorkshire</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 19:46:15 GMT</t>
+          <t>Wed, 04 Mar 2026 11:05:00 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFB5WG8yUE0xU29rT2hoaUV3T0J6NW80OEhtbTBWaDlScTM1cDQtdWtXRnJLeW5hMERhMDhXaDdaY05TYWZCdV9pbExFU2tJMU43NUpVbGVVN2Y1T2M3VUJHdnpDaDNXRmdPNmItcU5WX3FEQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQR2N3S2wwWnplWVd0aXVKcVl1bXFJODNTODZacEFHc1EwVGdNck4yanVhSUw4b3B0eHNMSExFZ190R1c1QkZIdlFZU25ZUm93bjI3UjNIaGd1TEtkZnprRmtPbTFQcEdWVjFrTWZkaU5QNEUwdUJPWDU1d240UThpMjFpX3pTU0xMZ0FXN3ctNkRTU1VVS3A0WlpxQjFzbk5iaE5V?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46084.82378472222</v>
+        <v>46085.46180555555</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail SA Unsponsored ADR (OTCMKTS:BMRRY) Short Interest Update - Defense World</t>
+          <t>Major update on new Yorkshire designer village packed with big names earmarked for 2027 opening - Yorkshire Live</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail SA Unsponsored ADR (OTCMKTS:BMRRY) Short Interest Update - Defense World</t>
+          <t>Major update on new Yorkshire designer village packed with big names earmarked for 2027 opening - Yorkshire Live</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:00:50 GMT</t>
+          <t>Wed, 04 Mar 2026 11:22:47 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQUDdDeWo5RzlVN0w5d2tnVmdEdngxcjRPbWpJeTZsM3dWWG52dlJ5enpWNXV1MTl6amp3VnlSWEYxQVNrd1F1RmtwSWdKaFJLTVVCSlNGQnBBLWg0Z0lnRzVJbFMwNF9aR0JYNy1JdVJoVmpUblhmNURpMXpQSUdrMjZKVDI5b3AtYnN5NVptMjBOY2N0aHk2VGR4U2tZUDRmM3VzWTBiUmhiLXVsYlpMV0ZWcjdDRFJ3dmJpTzhLRy0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQcXM3clpMbVJwQlg3VUxyNlc2RnVjRV91cElXVHpRS1IxREhsX1FldnI2dExXdXhkZ3NwRVVmanAtRzBxYmF4X1lFM2w3a0k1bmR2MHBsMm9Bd0tWTWlSaGlhX21iR19FZXBXREhmWUxGNl9YNFExQl9rUWFWdmxhX2FFVlNmclVQVnNNY2hZSHdLQ3ZBTFRZeGY4Y2x0b3PSAaQBQVVfeXFMTUJKVjQxdVNCakYzclJYMUt4aWFIYWVON2NidElPX1U0dHJoTHl4NzJFVld6WXAyY3JsY19vTzhaSXBSZmNPVVI0dVNnanRxVlFaaElDS2hoSTF6QnNUdHRWcHdHOUE2eWRfZk9vVktXZmZUR1dPMkE2a05fRW55OFV1eW5uUS15UzZLRGwzeW9jTFZxNS01YnFzWHNfa1gyN09idHg?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46084.33391203704</v>
+        <v>46085.47415509259</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - BBC</t>
+          <t>“Our vision is to make perfectly imperfect hotels” Oberland co-founders - Boutique Hotelier</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - BBC</t>
+          <t>“Our vision is to make perfectly imperfect hotels” Oberland co-founders - Boutique Hotelier</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 13:48:56 GMT</t>
+          <t>Wed, 04 Mar 2026 09:40:46 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5OcGdYb3UtdHZwRFRyTUg4UTBFc2FhTEhHa1dSTVVjN1B4eG13dWx6OThKV0J6aGVxV21ybENrbjJQWU1CQ2tidE1nVkZtNjJUX3BKWFBpRDJNdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTFBjWFppNUg2TTJaQWVrRWwyWkU3MnBjN29EN1ZnaU5EUTF6bkpZZ3BHT3I3NV9aTEo1RVROWjFWT3AzaGgyZDA4X1lROVc0dHI3dnA1R05qdFRTUEEtOGRVV1V2eWktQUlMVWw1XzR6Z0p6RHY4dE0wSEFjUQ?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46084.57564814815</v>
+        <v>46085.40331018518</v>
       </c>
     </row>
     <row r="5">
@@ -655,22 +655,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>REVIEW: 'Dhamroo in Headington is superb, elevating Oxford's extensive, rich, Indian culinary heritage even further' - Ox In A Box</t>
+          <t>East West Rail scheme: A route to prosperity - Property Week</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>REVIEW: 'Dhamroo in Headington is superb, elevating Oxford's extensive, rich, Indian culinary heritage even further' - Ox In A Box</t>
+          <t>East West Rail scheme: A route to prosperity - Property Week</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 16:22:36 GMT</t>
+          <t>Wed, 04 Mar 2026 11:48:37 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPZzhidTZVdW41ZkxVc18xTFF1d0Q4Smx2OGZHa2R2dkNTWW5Jdjhka0d2c2gxV1dLLVc5azFPY0NjU21jY21nQkRKbTRjcThRVlp0UkdIaVdqbGlJb3I4THRrN3dMbHJreXd4R3ZwN1I5NXF6MVlTNUkxaEJHRzNpQVk2ZWVqUi1DaXFBYzBMQ0JQNmplRFdONFdkTjI2dUxfWTBfYXJoZy1kMmlDaGxQX0JiendYSTNpT3I2eERIbmY4R3k1WUN1S3gtMnRaZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxQbml3OVFpWmRDX2RqZGowaV9UYjlMLXpTbV9MMFZwMC0yempxd3JyUlZFODhOanNqZEpac3pZMGVtNTBGSDdoY1ljWTZWMHZmVXhVY1dxNTdhR1JQUjBSWm1OdzlXbXZUN3h0WG9sbDRXZExZMGVTU0ZRbUhlZHpkczIzR1phazg?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -694,38 +694,38 @@
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46084.68236111111</v>
+        <v>46085.49209490741</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>“De Hollanders willen mij pakken”: hoe een ripdeal in Temse uitmondde in chaos en een schietpartij - GVA</t>
+          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - AOL.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>“The Dutch want to get me”: how a rip deal in Temse resulted in chaos and a shooting - GVA</t>
+          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - AOL.com</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 04:30:13 GMT</t>
+          <t>Wed, 04 Mar 2026 10:55:19 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxPQ0wxRHBWd2V3V3lpMlBGbTV5WG5wdm45eEpxaC1OdHVHTl9wT3hxWkxMY3ZjYzNaUkVMVmpVWTRmcGxjVTdBSmM4OXk5UFJDQnlfcE1yTnZsLTlHb0hvdzNqcTU2akZmVmgtS2JhYWdpN2lZUU5rOTNaMG0xNlRqMzF0dTdCMFVsM3R2ck5ab1lrQnJBMmxGR0FFMi1uTF9JX29rUXpPeW9wUUZVUVRhVjh3VmNUb2R1THFkWmZJRXp5WFE1MzgwaU1WR2EzOXdHbnd0Q0duSmdwNEhHcVBNZUJnb1o1ejRYWE5PUG1yTlNUWFplZHRsYnB3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE84UkdzeExGN2xLSUh5VnBiUlNFTkI1ZWl1bVo2RFVEeVUwdnZaSjNuS2hrOVhlam9pamJzUTRGRWZsOER6Y0hXRFpxTGs4bXZzdTZ4YXNxVlVaNXpCUTVuT3pHeXVlOHA5V3FLZHVUa3ZtYVV4aXNVUDZEek4?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,21 +735,21 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46085.18765046296</v>
+        <v>46085.45508101852</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nederlandse rechtbank veroordeelt spilfiguur achter aanslagen in Antwerpen en Kalmthout | Foto - HLN</t>
+          <t>Schietpartij in restaurant in Zele - HLN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Dutch court convicts key figure behind attacks in Antwerp and Kalmthout | Photo - HLN</t>
+          <t>Shooting in restaurant in Zele - HLN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 03:41:26 GMT</t>
+          <t>Wed, 04 Mar 2026 10:50:34 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPa3llNGRiVzV0c3ZtYS1icXVTT0xRdGJLQnA1bXIyb0FnMFFINzNCaUF3YjNIREZTTkFmNlF2c05NS1Z5LWF0THNBbWJ2VWZCWHNhZXRPWE9JbF9IQ1E5d0xUU2o0eGszbGNPUGFmZTJiMHhiaXU5cElWcDJrVTAtMjBaWDZ2VWdIaHB6VWIwekE1YldtaFhkbUhNdW15MkpfWjhEUjdzRVBmUEUxNERoSWl4VHprY25xLUlUZUJPQkNTS3ZrazRNRHlnMU1iNXhwRGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQNFZaVVFnMVRvSjVGNXZZRVEtTE1OWmJObEI5dlZQdkdOa2tLUkJTVWVrdmd5ZHZFblRWdlBrRi1FbE0zTkFyWWNIbERSdmZ6MmREZUYzUmEyblVUa2gzQTBrS2M1cFRiMGpmSmxyV3Vqb3gtdFI0OVdqWno2UnE3Z01najNmdw?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46085.15377314815</v>
+        <v>46085.45178240741</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mehul Choksi, brein achter grootste bankschandaal van India, zit vast in Antwerpen: ‘Ik denk niet dat hij veel in zijn cel zit’ - De Morgen</t>
+          <t>Man probeert iPhone aan te kopen via valse bankapp en vlucht weg: “Bij zijn arrestatie 1 kg hasj gevonden” - Nieuwsblad</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mehul Choksi, mastermind behind India's largest banking scandal, is in custody in Antwerp: 'I don't think he spends much time in his cell' - De Morgen</t>
+          <t>Man tries to purchase iPhone via fake banking app and flees: “1 kg of hashish found during his arrest” - Nieuwsblad</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 02:00:00 GMT</t>
+          <t>Wed, 04 Mar 2026 14:14:07 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxPaGF2cEdlN29zTmRyUWlTUlk3eUIyLUlNVWU5R0FkQjhWUTR2UnhuM0ZjNml3ZVBDRUtUNXNwd1FBNDFrRFBBTlo5SGZBQXBhT0ZkclVQMTFqa1dzVHhqUElGWTEzUWFjVFZwM0dtcXNOWTVtY1c5MkpQelZoWEstVnlYVE5kXzZwRHVtRFllc0E0ejdFb3U4dHlRSVlfQjFReUpsUW1naWM4RUt6T2tnR29NRXY0QUtOX251c0RDZVdGX25ZWkxmc3d1bm5CSEtoUG1HWDJaMEpLSFU0YnFPS0x6TE4yT1RKTGo0Y0pmRUE0QTJEcGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNVkUycDI4NVZMR1BEbDRxbTRxSkFKSmtPTTFmNEwySjdWLUhfOUJDMXBXLVFqdVBrVm9KNFl3MDRrOVh0akdWLUZtZjFWV1paRVB5Y043QlpQOGJuaHJzLVhiMDY3YzNxZW9YRER3ZEhWcXZlYnBQUE9jSWM3djIzT3V3Y0ltSXVsTWsxVVdtRUxpbG9FWVhUM0JRVkhCeXUzWUh4a0hJT05rV1AwcjhvTGoyQURRSjF3ZVBWRFdsQnp2dGE4cy1PSFdyZFo4bmRoVENveWNhU0ZwazQySXpieW1SeXJWNUIyWVN6RGdqUUVnclU5WVJQS0Framt2WnkydXU3dWJBd3BwSGEya21QZVBVc0VUNkwtWGdz?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46085.08333333334</v>
+        <v>46085.59313657408</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>“België moet extra waakzaam zijn”: advocaten vragen om zakenman niet uit te leveren aan India - GVA</t>
+          <t>Ex-partner van slachtoffer Grote Markt opgepakt op verdenking van moord - GVA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>“Belgium must be extra vigilant”: lawyers ask not to extradite businessman to India - GVA</t>
+          <t>Ex-partner of Grote Markt victim arrested on suspicion of murder - GVA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 00:36:00 GMT</t>
+          <t>Wed, 04 Mar 2026 13:09:50 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxQclFTMjExVXM3c1hjNWdaaHVsc3RxeU45X3BvLWpwRkU4MEF4VldCRmNhQW96U1dBNjRNZmNkRFlXWVR4X3Q5S2pBQXhhOEdKMFpqV21ncEc5R0VTdlZQM1ZZYWJQbmJXc2VyMlpvMXBuRzF6cUFLdWp4YlZNcTVmWExvUGVDRzRnRkViYjRsbV9wWHd6ZXlGVWlYT0c5N1ZvdTBRY2dOZnN0RWlSRms1akpWaXJBd1cxQ29qNjVReGhPYnZfMGh4QnpyTk9aekpZNnZOaEdTYUpzUlprR0lQWlZQLWJHc1FJUEN4TWlsNVd6OVdRMTMtdzhn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPblgyQ3R2S3VTZkY3X05lVTBvQlRSNWttdkNtSHNHSUdjT0N6MXlsRXFQRXRwRjFjNEk1TlhNa3dvc2xnWTlnZVBYdXB3ZzlWYV9acG5tTTdlWUNDclRVdFQ0N0sybHRDN01QN3dHQnFWSG5FelZnT2hlcDQ5R1laUTJZQ1ItN01mV180Rlg0Yk1fQWEtLXFLQm5wUDVCUTRDbFV5MC0zVjZfMjNjSldobw?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46085.025</v>
+        <v>46085.54849537037</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Na noodkreet van De Coninckplein: stad heeft zowel “zachte” als “harde” maatregelen tegen overlast | Foto - HLN</t>
+          <t>“Dit nieuws schrikt ondernemers af”: bezorgde Unizo-voorzitter nadat criminelen schoten lossen op bedrijventerrein - Nieuwsblad</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>After a cry for help from De Coninckplein: the city has both “soft” and “hard” measures against nuisance | Photo - HLN</t>
+          <t>“This news scares entrepreneurs”: concerned Unizo chairman after criminals fire shots on business park - Nieuwsblad</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 15:45:44 GMT</t>
+          <t>Wed, 04 Mar 2026 10:37:23 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxNRDY2VGluVm5jTmtYSjN2Sk9ELXZWTHE5UVJIdUlfSGpfd1dVWjZXeWxrdEZzdWtpT0xXeFJkTDFoVzE2ZnV1NGFQaTBmU1lFNWk3OVBqNndlS1V6MjNiTHVoalhfOE9Ua05KSTFrZEh4SFk1MVFvaC05OC0wNG1IVUthaVJIMmpBMzhCd0FCRlhjRlpEVTFudERJMVRDVTdHbWt1bE1nZmtXOXJ2VFJtSjZPSXYzcXVLOXpmNHVXWHdBQnlRSkM2YXdZa2VMTnNQS1k5YXFwekJwZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxPZGNOQTRyWVRtbmF6T05zTmYtS3ZIU0FSaVI5Q1drcFBXVFhqVkJ5UjFGcnVldUlBQ1ZzZkJXVTZWUEpiWXFTZ3B5S3FESklhcW95Q1o3ekZBemhERFMwVi10a3NoZG9jWFNQUVFIRGw3Mms3TGZKdndvaU1ZZDJpUzdVTW00YlFSc01RLUFWTkVWVXMzc05mTUJfU1JQQTRiMm8xd0NzMWZTZWVZbnlMTWtObFpzR0ZqWktDOWNYMHFDY21NeV9OTGJuNG94VkhNNXVjelhRTmRUblY4UXoyWUZGM3hLMlJ6UHJpYklXVl9KODRnRmxCaFNJc3prWjZTTE4taA?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,38 +969,38 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46084.65675925926</v>
+        <v>46085.44262731481</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Marc Coucke staat voor explosie bij Anderlecht - Voetbal24.be</t>
+          <t>As Israelis and Palestinians, We Shall Go Together to Brussels – Le Taurillon - treffpunkteuropa.de</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Marc Coucke faces explosion at Anderlecht - Voetbal24.be</t>
+          <t>As Israelis and Palestinians, We Shall Go Together to Brussels – Le Taurillon - treffpunkteuropa.de</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 21:02:23 GMT</t>
+          <t>Wed, 04 Mar 2026 13:04:46 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxOenBXLWIzUzlpVEs5VmxpN0c5OXoxdlBldWZmaHBJTGtfYnhxRkJXc21WYmRZdS1ScHZ6cG5fX2VXYUdLb3k0dnVya2RLd2VkakpfMWhnMEt1ajBtQ19VeUEzU01CcEpLTFhxcGhmc0R6WEg5U1RGQ04zeHFpay1pYVQtRzVQaVJyaWRPYg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQamJub2NMM2dvT1JKYkl5bUNOa2stb0tBb0FCZ1AxN3BLV3NFcHdaQW1takY2cld6V2RVeUNyNVFvNDNFZ3VkVGRWblBDNktqdU5UY2E4YnVyYmpsN0x6dE1QZGxWOXpWc3NFc21nejlsRnNKWWFoQTI5RnhkMU1GRTRPbmt4RzdUU2w4QVM5YWNkNWh6Tlo4cA?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1020,11 +1020,11 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46084.87665509259</v>
+        <v>46085.54497685185</v>
       </c>
     </row>
     <row r="12">
@@ -1040,22 +1040,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Brussels convenes regional security council to assess Iran war fallout on transport - VisaHQ</t>
+          <t>The Iran war will be long, bloody, and ruinous - Brussels Signal</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Brussels convenes regional security council to assess Iran war fallout on transport - VisaHQ</t>
+          <t>The Iran war will be long, bloody, and ruinous - Brussels Signal</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 01:09:35 GMT</t>
+          <t>Wed, 04 Mar 2026 08:20:35 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxNOU9vNTNLNUFZX2tzT0ZPclU2QmppTU1BdDk4RnZsdmNVN0tZQ1JpdkN0MmpHel82Sks0cHJYZ3VJbmhsVlA3emI2RHdwSkhWdDlDS2thbTg3OGxoaXhGSHRFUVlLd1h1dzY3MGxBcjFxbW5MMTFVVUtCU3UyZUlsbWlKSndXQTlmNmp4SzJVNW41RlR5empmdjgxT2VRNlVGMkZYeHdTUWR2UElEUmExN1Vlb2ZZWXltU251QmRURHNLbWN6?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPYnI4Z0dJSXREZkUwZGdCT00yZFpjM1VOQ2xLVTNQR1lmUTZ5ajNUZldiUUZfUnF5STMySzVSOXp1bTdpLTl5djFfOHNiNk5NWVB1TUpiSHBrakR2UW9yeWZtc1JlWlhjejR4NDUtc1EySnlhVHBNVk1rdmZYZ1lIamZybkw5QQ?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46085.04832175926</v>
+        <v>46085.34762731481</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Japan’s former Nara prison to reopen as luxury hotel in 2026 - Travel Tomorrow</t>
+          <t>UK catamaran company to offer wind-powered crossings to France in 2026 - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Japan’s former Nara prison to reopen as luxury hotel in 2026 - Travel Tomorrow</t>
+          <t>UK catamaran company to offer wind-powered crossings to France in 2026 - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 14:53:22 GMT</t>
+          <t>Wed, 04 Mar 2026 10:08:42 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxORXZ2Q3RxOGlvM0VYOVFqNGFZQW5uR1RhYThfWktpNVFPamZtU1p0anVJaWhuZ0VwWkRuZjI0SXJuUUktQjZnaW83ZHg4MXZKZGtxMGxxa0RRUnZrdUJMTHpiWVZsQnNEOVVoUlY1RF9FUlFZLUltdGpUaEFFWHRhbFhBaE9JbHFBS2pZdlM2Zk0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPRndSQjBkbER5Y2Q3MXRDT3U4TXF5cFpocmk4bFYyQ2VESnl6bWhmMFJzOWtSUFk5T0pJb1NkNXhSUGtTS1hqM0lNQkFaNF90QlB3LWdCNzdyV2RtTDdjNGZTbVZHSmFSaVFlYjNCT21FWmV1NFJyeTVSdDJXMVc2V3Z6VC0wMVB0QlBGdThtVWZDRlNRNHdDTEM1R1plX00?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46084.62039351852</v>
+        <v>46085.42270833333</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Orbán and Zelenskyy clash again over Druzhba, with Brussels caught in between - inkl</t>
+          <t>Pakistan confirms airspace fully open amid fake news reports - Travel Tomorrow</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Orbán and Zelenskyy clash again over Druzhba, with Brussels caught in between - inkl</t>
+          <t>Pakistan confirms airspace fully open amid fake news reports - Travel Tomorrow</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 14:20:24 GMT</t>
+          <t>Wed, 04 Mar 2026 09:43:42 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOX3RodzgzbUlvRzlDbUlIaXlsMVY4cGFlVHBpcXdIZVhieC1TOWxUcnIxM21JWWFKa3UzcnM2M1NWTWNpbERYVU5jV1JqWk9sRi1JTFFlQkdLeVBHYnNOaTF3VEpKcm1TZERPTHRTMmJ5QlIwQkZDRnBTYUhyMWhiOWstcTBlVnpwNGQ4a25pY05hWVVmMlFSOEp2cjJ2WVJWeDlTdQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNcDV5Nng5NkR0d2dBLThJRi1pYXZvTDRRNG45SW9sSkwyUGtOYUJCd0tNRGlBZmE5WFVNcDhyT0ZSbzBBWGR2cHFORHJZbUx1R0daSUNUc0hKTFJ6bVFITmFIbkNVWHdvdXJzel9BV3ZaUVVkMExwaEl2dTJTdHA1c1ZyQWtCaThKVF9sdGRzS2FnZw?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,38 +1189,38 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46084.5975</v>
+        <v>46085.40534722222</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Scammers target stranded Middle East travellers as flights resume cautiously - Travel Tomorrow</t>
+          <t>2 twintigers krijgen werkstraffen voor tientallen graffititags in Hasselt - VRT</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Scammers target stranded Middle East travellers as flights resume cautiously - Travel Tomorrow</t>
+          <t>2 people in their twenties receive community service for dozens of graffiti tags in Hasselt - VRT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 16:38:28 GMT</t>
+          <t>Wed, 04 Mar 2026 13:31:44 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNcEhKbmlNTTNmaDNNeTdza0I3dlo0RVJxNHNmY1RCNkpHUW1CeGZ4T3EzZzM5SlVDR1pfUFV6ZDd2VkxBRVE0Z2FOaldOUVFCM2dXY1BaMlJaM0V3OTZXYzZ0aGFCZTdnbFk4eDhCQklmMTIzNWRBMHRDRmhFc3VTM2FKSU5VYk9XRmw3VTNmYjhqNEsxOUNvblBEVnp3UWJCV1ZqaXNDUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQNXc5M1hIZG1lamVwVzlxLXhzTl9LMFRfXzlCdzgzV293ZXVWRnRaTHk2VGdqQ25fT2YyazdjY3prUDRYcFAzYkZFQ0VxYmhEejlVTmg4eDJfQ0hrWmpUV29Wc3JqdmFCWEZNUk1PblBVaWJ4cEQ4N1hjbVF4SHBLdGJDR1ZQdmVpaHdRWEtGOXp6VmJxRlRTV29VaUpLSlZhT2ptakxIVjY?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46084.69337962963</v>
+        <v>46085.5637037037</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Gulf airlines resume limited repatriation flights amid ongoing airspace closures - Travel Tomorrow</t>
+          <t>Une grande première: la Coupe du monde de cyclocross va faire escale en Écosse - 7sur7.be</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Gulf airlines resume limited repatriation flights amid ongoing airspace closures - Travel Tomorrow</t>
+          <t>A great first: the Cyclocross World Cup will stop in Scotland - 7sur7.be</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 10:03:13 GMT</t>
+          <t>Wed, 04 Mar 2026 10:15:00 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOaDNsMGE4d1NqeUR0WC1NVGpRSUVoSFo4MEVXNGJvc3V0YUtkbmZ2NXhRc1RLUE1xVVJnMWthaVplaHRILWRBRmhhYWhBZHA2Y2xmakUwa3A0TnRHcDRDZUZjZHRMUWZBSDhRWkROVGthaXBFT0ZhYjN3VjJ0cEdKNUxtYkJWZm43YTloRnAwMU1aanI1N2F2UkRERnV2Z0dRbXVkblZWb2ZQUTZZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQV2I0NHFLMHZJTmdoR0ZjSkxId213ZlVqTzBLSWJTRDJTV2FtWl9pdm1IWjJSZ0ppODhESlVfRlhTdXEtY0IyWVU0NTlRUDU0WTRJSjZRb1VxY2tXa2RDNDJNempQa1NwTW02Q2kzNHBOb2tIcE5yd2ptMXRUUXNLUUlOWEtCTHlwLW0wT2p4OE1yTDdlWUFVbjNHdEZHaUlRM3BaSEVJZWUwMmZQdEkzYTJCQVpSRjlm?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46084.41890046297</v>
+        <v>46085.42708333334</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>Local Town Maasmechelen English (fallback)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Qatar and UAE cover hotel and meal costs for stranded travellers amid Iran strikes - Travel Tomorrow</t>
+          <t>The best of both worlds at KPMG Accountancy Hasselt - KPMG</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Qatar and UAE cover hotel and meal costs for stranded travellers amid Iran strikes - Travel Tomorrow</t>
+          <t>The best of both worlds at KPMG Accountancy Hasselt - KPMG</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 12:03:18 GMT</t>
+          <t>Wed, 04 Mar 2026 09:33:41 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOVHpBX0U3czhQU254VDJtc3pEOHJuTklCQW0xR2dHTjZYVlVPQms0NGU1R2tMUGNTQ01DTjdFRl8zWWNmZnZBbllJSnFOWkpRNmRxLUFzYTJzSWtGdU9VUFNlTC1OR2VwMEpNR3lHTjZGRGlyMmpqU1lFeW5FV0FXRlNwN1V2V3pVYUpWZnpnY3V1bU5HUWhibWJwbGFQckF1azZQbDJqeFl0dXAtYTZz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPSHFXOC1teDYxSmhWNzFrdE9tbVU4SzBqcFliY0NaRURpRjNoUE5Fb19HcDQ1WGt2YVVfS2k1bHM2VU9ta2d6VzVOemtuSmdiRGI3Z3l6OS1lTV9CemNrRTVqRXNULXUzS1NScm1paVp5N3RvbFVaUEJ0UG93XzJDY1ViWmxZdDNxVDlFNUxiTjRLcTF4a1ZmU2VPcHNxSEpPdHcyM3VGRlA?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1345,47 +1345,47 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46084.50229166666</v>
+        <v>46085.3983912037</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Un feu de trottinette électrique force l’évacuation de 15 personnes à Laeken - BruxellesToday</t>
+          <t>Brendlorenzen: 17-Jähriger liefert sich Verfolgungsjagd mit der Polizei - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Electric scooter fire forces evacuation of 15 people in Laeken - BruxellesToday</t>
+          <t>Brendlorenzen: 17-year-old chases police - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 06:50:00 GMT</t>
+          <t>Wed, 04 Mar 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPYll3M3RrSlRzRkNFVU56VE1BLVNXYlhKRGpZNUNzV2lWYXYteVhuVWFkWU8zOG1GS1NCREh5MjJmS2dOUGttcGx5OWpRVnlESTIxUk5zOWk4Tmp3ZGRZOUt4SjRKOXFvOXpSOHRTTWNSbWdIN0dXcXlDUGNsbmNWbXI5NkxwRWVEZ2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxOMlByX0xhT2xSOEZLTWpXczBQVnlCVWZ1T0ZacGJ6Wm15Z3AxS250RVZBVHczVDkxNTBtQmJDZ1V5MTVNc1N3MDlZWmpUSFRGQmZyckM1SEZ4TkRQbXBybHhqUG5fcDI1QVFnZ1dmckRPNWpiU3A3OXQyV1UtLWxBaFZLQ1dyWjRjMHdHbE5RSlFSU3dQcjF3RnJZeHF3RkUxc1FnOEQxbzV3RjJ4?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,52 +1395,52 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46085.28472222222</v>
+        <v>46085.58333333334</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Accident entre un bus et une trottinette dans le centre de Bruxelles, un blessé grave - 7sur7.be</t>
+          <t>Kitzingen: Herrenlose nasse Tüte und drei Unbekannte beschäftigen Polizei - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Accident between a bus and a scooter in the center of Brussels, one seriously injured - 7sur7.be</t>
+          <t>Kitzingen: Abandoned wet bag and three unknown people employ the police - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 14:20:00 GMT</t>
+          <t>Wed, 04 Mar 2026 13:15:00 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxPQnU4MW8xU2xJWUhPMGJMZDdyY1dUakw1Q1VZVE1FbURPNDd3RjhIZEpFUXJvbDJhT0c2c3F2M0xMQ3BTeUNseVRYaGV3NWdhdENINnBiaGh1bjQ4b2V6Y3EyZ2JoUTBFb0gyWk5UeHlLTmNkLUc4dk1PcVV0Z2FTemxGdzktWmZtT2dLNzRacW1mZUx2ZGxuRE9EcDUzT3JRdzZad3lwZGRCa3hwZ2ptNnpZODd4bHNGZ1Etd0liTWVIYUlGNF9F?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPay1CSjA4VWZzbnZsRjhMZXVram52bGlHeWY3ZUJ0NjhGc19HMWlYNFFWVnNTcEc5X0NvbWtNVGQ5dTBBQWN4WnVZb09lbHY1QzhrSTNmWWtrUzFIZDBNY01fM0ZCR1VtWVRlQVFLWGNBWExlQTJITkQxNzg0T3ZkQXFSZXNhaGt0TXVZYlg5Ymp1X2FpeWoxNnRjNlFJRXJQVWQwdDF2dDJPMDFk?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,52 +1450,52 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46084.59722222222</v>
+        <v>46085.55208333334</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pendant que Meeus savoure sa première victoire de la saison, Van Aert vit une fin de course cruelle sur le GP Samyn - lanouvellerepublique.fr</t>
+          <t>Würzburg: 20-Jährige springt in Würzburg ihrer Tasche hinterher in den Main – dann wird die Strömung zu stark - Main-Post</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>While Meeus enjoys his first victory of the season, Van Aert experiences a cruel end to the race at the GP Samyn - lanouvellerepublique.fr</t>
+          <t>Würzburg: 20-year-old jumps into the Main in Würzburg after her bag - then the current becomes too strong - Main-Post</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 17:47:47 GMT</t>
+          <t>Wed, 04 Mar 2026 08:40:27 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxQeGNhNjdob2ZlcGlsTmFwMzNveFFGUEdObjcwRk1xXzBvZUpaVzJRT1ctUFZLWjhqUGFzMWl5N0FNcFo4aXBfQW90UWVOWWllNzVaZ3g1ZkhQVk1peDItZzZVTXRVQi1CUEpZbm85QUljdkhBZW1XemM4ZWtIU0Z6ekIyLUdBb0YtUEF0SWp2b3c1VVpIRWxQUjNUQU1yX0ZfLWFwZGZlOHo5OW5yYkhwSDJMQzk2MEpyanFVOXAzZXdyYTViN0lMVDVPNmJNakx5ZTlJNnctRllidGtqSjJJTjJ1RWFtWlVZRnhFaWNnNUp1VS1VQ2JGOFZhOWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxPcm5yQ1ZsbXpfaGUxU1lKcnp1bjJLRG1QTk05eU5PbEZEV216dFBQaFU3Vk5nVlZjLUpLRjVmSGFZQVlkeVlTaUJic0N6elZ0dWJ6SDR3RE5CbjZiYngwcUZKVU1NTW8yQjcyaWtUMXRYT3ktSF9kbjNnQ3RtRzFhMnBQdWMyS002WjhWaXNXVTMtRktSUzdsODRBYVFKSDNXWUh4Zk9oOUdDdHJFekpfN19hZ3RJMUR3dGhubU93TW5PeUNWdFRFUTBLS2I4aHpiOHFrTkZuUkhQYXdDMmhSMkYzRFd4T25iN3cxWXFDNEpXR0RBVzBYbG9FY1JuWEhFREdOUEJXZw?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,52 +1505,52 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46084.74151620371</v>
+        <v>46085.36142361111</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dossier saharien : Bruxelles et Helsinki appuient le Maroc - Perspectives Med</t>
+          <t>Polizeibericht: Krommenthal | 13-Jährige vermisst - Wer kann Hinweise geben? - meine-news.de</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Saharan file: Brussels and Helsinki support Morocco - Perspectives Med</t>
+          <t>Police report: Krommenthal | 13-year-old missing - who can provide information? - my-news.de</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 10:07:00 GMT</t>
+          <t>Wed, 04 Mar 2026 13:44:53 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPcGtuZU9VcVhXVDhuZ0Jxc3dwMk9oVk9IOFRDOTR4bHozLXFBaFpESHlmaXQ5Q0lmU05wOVpOYzFRUnktY0M2U1dLVjZPYi1yenB6c05uRHFhLWdyLW1OWFl0VDMzSHlkbklXVVRhRzNLSEtnU1hkd1pqRVhLcUplNnJ4WndlNDgwWDJoQkhR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxPSGt1eXRTbXRLNE1SZnJnYUJHNHFpa2NSV25oWE4tQ1EyYmh4N0lCX1NicDFVSTcxdDBNVEZPQVRYUm9LQUZZcjdoODlqQjd1VkI0LWRNSkgzOVhRaDBHUXYwUTBMYnZtTm12dWw5SWVCSmlBNVdJbV9BRnAzVXY5d1Mwa3FDQW5SdjJUSXBUSGZLeUp5Mlpaa1FjQlJWdUZlN1pXVGZjekhGQzRNSFY2RVJoTjY?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46084.42152777778</v>
+        <v>46085.57283564815</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Politiezone LRH groeit uit tot vierde grootste van Vlaanderen en zet sterk in op innovatie en welzijn - VRT</t>
+          <t>Hundebiss und mehrere Sachbeschädigungen in Würzburg - SW1.News</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Police zone LRH is growing into the fourth largest in Flanders and is strongly committed to innovation and well-being - VRT</t>
+          <t>Dog bite and multiple property damage in Würzburg - SW1.News</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 11:14:04 GMT</t>
+          <t>Wed, 04 Mar 2026 12:35:01 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNQzBHbHAyU01oQm5BQndQc3c4QW1fUENOU0RSNzV6djdtT0txQWhqQ0M0dURidnhBQXNFQy00c2Vxb2N0VEZTQkZNdmhtbmpFUm1rV001WXNnX3pWMUt2Y2JJYlhoUFdGXzlVVHlwbVp0N1pfYkRjV29ZWWhUMG5FUUlnY3BIalhCMk5YZXFvcFhyWWRNSEh5YmpiT0tmQ2czSnI2b2hUWjU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxObndrOEIwTm5pWjU4b25EaHRKRThqRGU1WUFTdldNa0UzQ043ZGEySnFnX0JYVkppSDlSbEc2Zkp4RWhuQmg5SDk1Y2NQOW91YnM2NjJRTXpFNDd2LVM3RU9kVGhYVUEtSjA5Ml85UGYzTXZHblh5V0UwRmJNRFBPN2lsNWtmT0QzQmt3SzRNVFBFa0w3SXRB?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46084.46810185185</v>
+        <v>46085.52431712963</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Leegstaande Euroscoop in Lanaken krijgt opnieuw vandalen over de vloer - VRT</t>
+          <t>Wiesthal: 13-Jährige vermisst - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Vacant Euroscoop in Lanaken is visited by vandals again - VRT</t>
+          <t>Wiesthal: 13-year-old missing - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 07:05:11 GMT</t>
+          <t>Wed, 04 Mar 2026 14:10:00 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQMkp3Q0Y2TE5WdzZWbzNMOXM4cWxsV3BjS3ZJbFR1cmdiWGhsT2FFd3VmX2pJa1YtZDJHR29meURRaVIxMll2TWF3UWNZb0JKSnJwOFhxZUoycEY5aTkwMGw3ZTRkSDBIdHNZb0szcVB1ak1fa25nQjNOTlVXNFBFaVphY3RBOXlxby1RcHAwTUczMUkwX2V5MlZQQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9QWEtqdUh5RG9WRjQ1OFFtR0FtTC1lUlhSaXl1Uk5fdUVtWW1RN0VOY2c5ckxIZTdoNWYxNmVxRGZJTEQxd2lLdzRkZ1AtMmVSSHpia3NqSWNtNTktLVFQVFZ0U0NVWWZpcHJuQXRua3E?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46085.29526620371</v>
+        <v>46085.59027777778</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Man (38) uit Maaseik veroordeeld voor belaging en mishandeling vriendin - VRT</t>
+          <t>Polizeibericht: Heimbuchenthal | Navigationsgerät sowie eine Dashcam entwendet - meine-news.de</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Man (38) from Maaseik convicted of harassing and assaulting girlfriend - VRT</t>
+          <t>Police report: Heimbuchenthal | Navigation device and a dashcam stolen - meine-news.de</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 16:15:56 GMT</t>
+          <t>Wed, 04 Mar 2026 10:48:36 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOR0ZuWWktRWVtekNncUp5WVg2eDI4MTB3QXBoNlhrQW56aHZmNERBVzBJNEd3LV9CbWRCWnk4YXpsSEtTcmRXcmpvczZLNnF0d015c0J5RG9yWlBkNExvcVRtWFd0ZXZpNDhqQUllOXNCTkVjWkh4VlhnX2g5M1VxOTdBQ1FEVUJFUWJOSDM4NU5WSUVKUUVUTzZZRkszVU8ySG00c2taWlc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOeC12WEU5ZjFwOWhJT18xck40MWZvNnU3bElqYlhJbkJ4X21pMDV6bk9udkgwUFdiT3dmdE9qNnlkM0ZNQm1iQVF3NlcxRm0tRXJsM015SUJiRE1yTzFMdFRuVUpLSVZKM3RMZFlZOC1uMWNWUUU0Q2FNUjNNSGoyeG1SUTQyNkhvUldFU1ZxTjE2Vm5VdlY3U3k0dXBsX2VqLXZiaGxRaWpINm9DUjdOUDd5QUlMOVZ0NVBtakpKaw?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46084.67773148148</v>
+        <v>46085.45041666667</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Présidentielle 2027 : « Je ne souhaite pas être Première ministre », déclare Marine Le Pen - Ouest-France</t>
+          <t>Diebstahl vom Firmenhof einer Kitzinger Werkstatt: Wer hat von einem Mercedes alle vier Reifen abmontiert und entwendet? - Mainfranken News</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Presidential election 2027: “I do not want to be Prime Minister”, declares Marine Le Pen - Ouest-France</t>
+          <t>Theft from the yard of a Kitzingen workshop: Who removed and stole all four tires from a Mercedes? - Mainfranken News</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 07:00:35 GMT</t>
+          <t>Wed, 04 Mar 2026 11:01:00 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggJBVV95cUxNaXpoRXJLeWJJdF90aDdBaTlRblZrSGI3U2JFOFJ3UEgxSzlvN3FEZ1FyR0xrTHBrUUI2QjlsUXJZUnh5M1MwYzRySzI5eXhHbGNXNy1KZTZ5RDNmREZZTER6MzJ6Q3JoSUpQcGpzUGdReHRaNS1wc1l5U0hUWV9uMDhFZ0NGNkJBWEFmbm5Fa3RFX29yQUxyY1d2WGZqdHJvTTJTOWhWZHcxY0gtTVczRjdSQkhpcG5POHFEandoMlpSVGJGREY4Z0dkN1FMWWtfZk04dGROYmRZNWZHcUFacHVBcVJEd3ktZXN3T0d6dEZfWTE4XzY0MHZQckgzenZtRUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxNUUlvdXEzcmJoV3pwdXM5NXJGdWd4S1Vod05IUXdmcmlvVDBMUmpPaDQwRHQ1akpXWXNfdHNnRlB0UU9DT01mYUtXTjdROFdVWXBvQzJxUzQ1X2g1UnlxdjNtR3g3ME83Q01mZGdXT1lJUTJCcmtFVXVuSVZXOElVaU1ZRWNaZ3JFbjhwU0NDeHlPUjJDNHR0d1IwaXFLU1c0a0tNZHp0Uk9tOXJSUFpLQ3VlaE5nQWxkclIzYl90dzd4NkdUdGowMHBvV3lxaktlcklNU3dZem1yUXYteEFXaEtVam1hS1d6SEJj?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46085.29207175926</v>
+        <v>46085.45902777778</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>"Jouer au Real Madrid sans boire ni fumer ? Je n'aurais pas été aussi heureux", la décla folle de Radja Nainggolan - 90min.com</t>
+          <t>Mainfranken: Mehrere Fahrten unter Alkohol- und Drogeneinfluss - Charivari Würzburg</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>"Playing for Real Madrid without drinking or smoking? I wouldn't have been so happy", Radja Nainggolan's crazy statement - 90min.com</t>
+          <t>Mainfranken: Several trips under the influence of alcohol and drugs - Charivari Würzburg</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 13:24:58 GMT</t>
+          <t>Wed, 04 Mar 2026 13:30:00 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxOcTlPUUVuNTU5VXNYZEpFcUVSV2drN0x0QVhuNDJlR0UzekxMYzNQRjZEWTBRRnFBSVNXOHhKbjdSdGNZRktHYlZDZkF6R0ZDQ2dhbFlZMFhhdEtSdWJSVWxKUVRrWWoyY0FmV1RaUEk1cWxucG5uX2dyRWg3Sm5GakIzZmUteVl4NzFOR3ZpMEZ2QnRXSjZHZGpOVUtyVjJabXY5X1VFUkVjU3BRSWZwdW44ZGY5c0ZfejJBXzVBOEQzQmJpRnRzVnRYX1ZjTWs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNQ0JlWndGZThFV05fbmpFMFl0emdISk4tb2NxLU8teVFFN2RCQl8xRGxKbzJ3Wm9JUnhUSlNQMmFjbEt0RVZkWGNZWEJVcGVYaTdaLW9iZjZaaEphS1U1dl9YVnVkOVFtN1o1dnlwanRDWk1BUHpkOWpZMmxMOWlic094OS1lWXd2ellTNDhLN1FCaHhUdUR4OUVfM2NKQQ?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46084.55900462963</v>
+        <v>46085.5625</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cambriolage du musée du Louvre : l’ex-présidente Laurence des Cars annule sa venue devant la commission d’enquête - Ouest-France</t>
+          <t>Polizei stoppt Fahrer in Mainfranken: Verdacht auf Drogenkonsum - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Burglary of the Louvre museum: ex-president Laurence des Cars cancels her appearance before the commission of inquiry - Ouest-France</t>
+          <t>Police stop driver in Mainfranken: suspected drug use - Fränkische Nachrichten</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 17:23:26 GMT</t>
+          <t>Wed, 04 Mar 2026 10:14:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAJBVV95cUxNbUpRSFZ1S3dkb1FyUEVhUm9jamdENGZvSjU4dVJob2VWeGVNSldLaGl2QVJEalBPZVhyRXY5czhEODVRSmxGMHhLaTY2UVQ1SnBFYzJDR1F1TFhUMUxQa0h6cDFuZkpJMjZ4bEpKS2pOWWlVUE9wUWNVWkZRal9xem94dmxyN1FtOGxmQnhkLWtzc0s2ZTg1UjI2VkZ4blZxTHkzUTY1VXoxcUdtX280YzFpWFF5S1NhbHVuaERJd2xUQWo3cFlnY3JRdGFlOFIwYjhMbnlqVXhJTWUyVjN2NG1xLTh5TmZDZVhzVFlrYzJOX1dmbGl0Y0ZpZlBaaUVZUDgzRmVZNHZ5aE1GdUs0WUdQRUlzTGd5?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxQamMxVW9weWRHZUlYMXhucTBuT3JTR2NxN3otOGZ3di1CUHNpUkxIQmF1UmdSSG94TXhYUVl5dnFwX0xzX0R0Mmx6V3J3dUNyTjRhVXZTamI4WHpWeWRmY1NLbF9fM1pzRk1hbU9CQ0VPZk5hamRQb1NSeGEyQWRTdDk1dXZXMXVLUS00d3FFdFNiY3BXMThFbnRfNURubVlEMkdUeVBkTW5YSDFtRjB2UzB4S2praEpPUGE3Q2tsWTRSU2RuRzV4S0tFZEIxWEVRWWRUMTFB?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46084.72460648148</v>
+        <v>46085.42638888889</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Super handball League - Bocholt déroule face à Bevo, Visé gagne contre Eupen - Starsporttv</t>
+          <t>Mobile Blitzer in Reichenberg aktuell am Mittwoch: Mobile Blitzer am 04.03.2026 - News.de</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Super handball League - Bocholt takes on Bevo, Visé wins against Eupen - Starsporttv</t>
+          <t>Mobile speed cameras in Reichenberg currently on Wednesday: Mobile speed cameras on March 4th, 2026 - News.de</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 23:04:31 GMT</t>
+          <t>Wed, 04 Mar 2026 09:19:50 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxON245ZG8tbl9WNGVUZUk5enZRaWI1R2FMLXUyc2xkbktOY296d0ZFUHZGcC13UW5NYi1HZzBNZ21oTmFnY0UwbFA0ZXdFUGduQl9PTXlVVkpoQ1YzaTFkbHNCSktDTUlMa1B3bUZQTlpOSk9UWFotLWxUejg1TDQySms5anFhU2tzT0lLcHhVaEk3VmFVb1FaVUpDNldfaDVOc2hkeU9rVm9QWkU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxOOHZFZUVtMGU4WDBJZURfZUJNbl80eGNVODV3WVRfSUE4X3dDcUhTZnhtX255M20tTU4zdzB1V3NjQzU2UUc5SHNIcGx5Q0txNWVYVHJlWVJjYVZUY2x3dXdKc3dfc3UtN1B1VEtCWEFrYTd2VzFLT3FnNHF6V3JLTnJVWnVXeXBBSGNRVzR4NzBKMk94Uk5wanVITHRHMWJWdlR6YTZ4TGpxemJ2UEI5cG5GQ2tfUi1JOVRURzhCR2hJSUF1MUY0NDRySV9IS3hfYVRQU3BCWnl0cVZwSDY3aTBzTW1HRjDSAewBQVVfeXFMTTE0d2NMeXFlSEhHb0VCb0JIOXJRQ19rbXRQY1p4Z0QwX0V1ZlhVZ0lBQlludlAtZEZiWGVIX1hTNGhyc3EyM3RXNFByZjNKMFlPN3Bib05MV3pzZERpWFBxSndfdXl1ZUs1VGlqeGZoT0EzalBOWXRhY2hXSTNlUURITFFIOTNoRmpEbElzMW5rQ1dUSXFweFZJUUpRM3hIRlBRbEI4ak0yV3JfSml0UERzYmJIUDdQMkdzMFlhVWZHOXFnV05IdTRrZkpwWVMtd1RwT1R1LW5obXc5RFVybkpnMTczYU5xS2lnczk?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46084.96146990741</v>
+        <v>46085.38877314814</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Glasgow to host UCI Cyclocross World Cup in December 2026 - Cyclist</t>
+          <t>Schulstreik in Ingolstadt: Schulleiter der FOS/BOS droht Schüler:innen mit Anzeige wegen angeblichen Hausfriedensbruch - Klasse Gegen Klasse</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Glasgow to host UCI Cyclocross World Cup in December 2026 - Cyclist</t>
+          <t>School strike in Ingolstadt: FOS/BOS headmaster threatens to report students for alleged trespassing - class against class</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 17:56:46 GMT</t>
+          <t>Wed, 04 Mar 2026 13:30:45 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE95UG5Yek51VHZwQmtmMkhsVmctb0lOVmFzQm5HalIzUTNyVjVaS01pcXJkRzNpdXRaTW8zdmluSl9OQzFkdmEyMklOaWpNUmRhNlBCUS02dnNnQzdxTVE0ZkZYRFZqSGpNQjZEbjBsWG14ZXVKQVJF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNR09RdFFZMHhDSnlzdk5MQ3BwUGJxRWN1NVpKZVFEZklEX01yTGNUUVJmZzdhUTkwM3ltbEVSeG1RQk1EWFJfSWpHVXdRRHM3bnpVRUZtR0NPazVKelM4UzJIdk95Sy12Wkg5TG5veWRrMzZYbTV1Q3VuZElUUkRhUHVkdWR1ZEpMMGxGdlphYnk1UnE2U0pPa19fOUM2MXJpN2R5Rm5Qd1Y0SnY5UjdpZWpCT1o0T3JLMUhaaUo5WWNJMk41d1UzV0Rha2VfRGM3Vzl5Z2FhTnVXMWUwSXZ3Mk91Y2VFTlk?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,52 +2000,52 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46084.74775462963</v>
+        <v>46085.56302083333</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Maxim Van Laere - nascar.eu</t>
+          <t>Lebensgefährliche Verletzungen: Motorrad-Fahrer (21) verunglückt bei Ingolstadt - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Maxim Van Laere - nascar.eu</t>
+          <t>Life-threatening injuries: Motorcycle driver (21) has an accident near Ingolstadt - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 00:10:51 GMT</t>
+          <t>Wed, 04 Mar 2026 13:35:11 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE5lTWhadGJfQ2M5Y0IzRXpncVlha1FyMlBDMUZlOUVZVXV6dG5tWWstaTFkNWhvcnNFQVJ3R1BTcGxTa18wX0pSZVRXU2dWZWdKaUVHbkNJNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1mc3FhTmxyanVMeFB6YU1hNjFXWjdZOTJEaFBSS0ZOX1poR3NhanQ0Z3gwMHEwN0p0MHVsTnRYQWJDbTl6LUVQRW9xenlpZy1RMXpOSllRb3hUUGtWQVhLN0gzUEY?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,52 +2055,52 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46085.00753472222</v>
+        <v>46085.56609953703</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Polizei sucht Zeugen nach Körperverletzung in Würzburg - Newsallianz.de</t>
+          <t>Audi Suggests Gas-Fueled Supercar Could Return One Day - inkl</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Police are looking for witnesses after assault in Würzburg - Newsallianz.de</t>
+          <t>Audi Suggests Gas-Fueled Supercar Could Return One Day - inkl</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 14:50:38 GMT</t>
+          <t>Wed, 04 Mar 2026 10:54:24 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQU0wwMXNXYWtOU2NVamtSb1hPWXV3V1B0cGdJNVg5bGZYRzMtVEhIdTFzdlFrMmE0Y2NiTXRoa0xNV1VnV1Y0Mjh2MFVCLVVHSHFiOUhCYUhaY1VzQmpxWEhxUXg2eDZpeVQybHYyal9SY0pTMU0xSl9lV2lBVExDNGJSUHc1ZzRmQUZpakI0R3VFb21paFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNcDFiaGtUYkRPWFR3TExMelFqR01CZ1dEVzVmTGhIMk5fOV8zUHlyZU5iRVhQNXQxcEtObjNscG1sNm1POXlXOGtkZHdvXzJBMmhkWUY3ajJDZzlWa1pLR2t1VUczVjhCOUkwVDJLS1Z4LW9QTDJEa3l1R0pLalE1UVBmR1p0OUU?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,52 +2110,52 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46084.61849537037</v>
+        <v>46085.45444444445</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Polizei Würzburg ermittelt nach Angriff auf junge Frau - Fränkische Nachrichten</t>
+          <t>Audi Becomes The Latest To Want A Luxury 4x4 Off Roader - Auto Spies</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Würzburg police investigate after attack on young woman - Fränkische Nachrichten</t>
+          <t>Audi Becomes The Latest To Want A Luxury 4x4 Off Roader - Auto Spies</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 15:10:00 GMT</t>
+          <t>Wed, 04 Mar 2026 13:03:11 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPS1FqWE95NFlIajJKZ1VRYy02QWVaTFc2a2hFMFNvdk4xNkN5Tm5JSXFXX0txRXV2YlV0ZVpPLUUtODR0Y3NIUTd2NFo1MGZ4aGtqdmxBWmticm9uVEdHTTJENE9NWE5kV1VyUWljVmJvdWFYcXRFM2wwakdnSXp6UDhFR2JXREJBYVI5cW4wZnkwaXEyQnhzZHUzWmhyOVpvNC03YXpVNkVHVDQ0YTd5LUNMNFo1WlJjczhYcnlCNGY4ZWcxZmMzSm92alI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE9McURiYnVhNWEyYWg3MUlaV2pHMldzem4tT21ldUt0dTBINGQ1Und5UXhpWWhHU3pCWkFTOTFlWEJPMHR2WHBKYTFJN1ozTndUeUdsYlZqaTBfWFdCZjE5VU5LNEJsTDdpc0NZcWdB?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,52 +2165,52 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46084.63194444445</v>
+        <v>46085.54387731481</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Las Rozas La Roca (fallback)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Motorradfahrer entzieht sich Polizeikontrolle - aschaffenburg.news</t>
+          <t>Captain Fresh completes acquisition of Frime to expand tuna presence in Europe - WEAREAQUACULTURE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Motorcyclist evades police control - aschaffenburg.news</t>
+          <t>Captain Fresh completes acquisition of Frime to expand tuna presence in Europe - WEAREAQUACULTURE</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:01:52 GMT</t>
+          <t>Wed, 04 Mar 2026 10:06:37 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQNFJMUnI2aHBGNWFoMUxrZGFMU210UUFnY1BpQjEwRklTZzY5d0NvQTJWRmVoMDcxa3dFSXJtbmt3NnpWNXJYbnp2blgzeTdCdFJwUEJrT3lDYUNqRWVqOEE5ZnNsTlZ0WE5XTk5KcWVHT1BQdi1GNUhnM0k4VzQ0WWduRXFXMDlUZkFIRnRKYV82czlOTUZYaFVPTmF6ejlFWGkyb21kMy1NTGdBSmh4SjU3YXJLYU5mbFNr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOTndjdnR6NEdJQlVUV0xKNm1lUFVlbUxIOHdOaHhRYXIzSmdKUjM3eTNLTWU2VmNDVHg3NVNVRXFHTEdPM2RLVFYwSnAzRDlMT0NFei1mbkNJVHJfdVBNTEpxWGUyODhXNDZSczlzT3VvU2k3UTcyTFRfQWx3QXJUZHFCRW8zRHdmd3lYWWpjUzVrcjFqNDkxUlNoYzZ2OUJnbjIxNHFKOGNZRUZqQVFPbzJ3RWF1MFNyenlqWNIBygFBVV95cUxPTzdBRVQ0VWlkcUowZzBaVF9Fa05DWDM4U0hsN0N1eHFsWHo4clBwODNmcEJzdkhZczJjR001SGtzSFhTaXljYkNtbDM2ZHhaNVN1dDdQWGtfTi1VbFVhbWZwRXhiS2d3a1Y3NUZibFdReUZ0enhaZ3NoN0p1S0ZDMk1aMkVSNXBETjQ2VWcxUVlWYi10WlNzMjJqa19hdE51YUVBRlk5SWh6cWVsQjh2S0pyQ1lFOGNyRzNVUmZiNm5LVVBjUW1SVWVB?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,52 +2220,52 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46084.33462962963</v>
+        <v>46085.42126157408</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Polizei-News Essen, 03.03.26: Erst entblößt, dann Beamte angegriffen und verletzt - Bundespolizei nimmt Mann in Gewahrsam - News.de</t>
+          <t>LATEST: Work to start immediately on €17m Army building in Kildare - Kildare Now</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Police News Essen, March 3, 2026: First exposed, then officers attacked and injured - Federal police take man into custody - News.de</t>
+          <t>LATEST: Work to start immediately on €17m Army building in Kildare - Kildare Now</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:39:03 GMT</t>
+          <t>Wed, 04 Mar 2026 11:31:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQR282WG9oUEV3czI4VkQ2UWs0MlBUam44eFNJaG1HdVRZcXo4ajFocE1IamwyX0dmZDRRbFYyalZoSXlrRDVDV0JqMzJlRHZISUtlMVgxVVZrZWRmOVRBOS1qNzJiWUx0T004UndMUjZONExYZkZkdFNaNDhWSGk2R25n0gGHAUFVX3lxTE9lRml3azhxUFZYaEFKV0xCeHN4NlNEbjNiTGMtcWl6ZlRqSmd2UzV3Ny1EUHRBX0VTdEJ0ZjVRRXNsd0tuWkJjblBLNFhHUWlMQWtwSm5PNGhaQjIxR3ZLUTI2S2FnaWVKT280NnhZRjNwN3hDekw2QmJiUUpLalRnR2gwN3o1QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxONy1yNllPOVZRNjN0V1JZaHprY09YR2MxNE5Oa3ZScUQweEFySHMtZ0VxdXFveExvM083eVlLSnpjdzN1T1NtWHdsUTczYjEyVkdidmtvOUR4eElsaGQtaFc4bk1zcmpza0ctcFN4ZkxZTUZIRlR0bWRqaXdDYTNrY2NTVGhsdDc3WWMyLUZDZ0k0MGZRSjNRVVlWZmZMZi1kQl81c2dFRFQ2R3FWdE1TZzRtMm9xMDlkRkpJXw?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,52 +2275,52 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46084.36045138889</v>
+        <v>46085.47986111111</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Polizeifahndung Essen, 03.03.26: Mülheim an der Ruhr - Unbekannter raubt Schuhe - Fotofahndung - News.de</t>
+          <t>Kildare Ranks Third in Ireland for Maternity and Paternity Benefit Claims in Latest Figures - kfmradio.com</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Police search Essen, 03.03.26: Mülheim an der Ruhr - Unknown person steals shoes - Photo search - News.de</t>
+          <t>Kildare Ranks Third in Ireland for Maternity and Paternity Benefit Claims in Latest Figures - kfmradio.com</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:58:02 GMT</t>
+          <t>Wed, 04 Mar 2026 12:36:26 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNeEhBVjNKQ3IyQWFuQUF4SFNqV2FlSEF2ang1Ym1jSGZTd1lZSmt4bzR2QzF5UUtVTXZNRk12dUluajMzYWROYV9RZ21teUtMWjl4SldZVHc0VmRhSHIxOC1lUkFhRFFDRkZ5NUY4dmQxZGkxa0NfMElCbktqUXgwMTZTSU14VS1Peld1TWp5b9IBlAFBVV95cUxPaUxNUmctTk5ESXJTOGJxY1IxTElrLTlxQVhQeTJhR1k1QkVIeXpXSjBiOU5GRkVGOW14bFlvNEc4MlBYUTlhUmtvRTFkNG5xTjhPQUhkc3lOZWt3d0dyVGxXRXhLOHJySWE5YWtnSWdpOXdHMjNmVUFhTEZyS0xMSUQ4SjlWZnUzU1JMSk9WTHVkTjdf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxPdmRhanNRS2dUV3F4RUphRWpNR1FONmlicVlOa3FHckpGMm9YdWk4R1lHQ1cyR1VJdFRvUGczTklrSGpZUTJZdkFlSWZPa0JTYUJuRWxDWndDNzlyNVNVbEswTl9Hak5VMTZrRGw4RUxlSGhCNlpXWW9wWWtEQVA0blZhcThfdlpWYUpjMzNUNVl5em9rVVl6Q0h6dEp5VHEyakxnNVpOaFZUSFBTSC1vTkgzWWlVN1NhT1pmOGlCbWNVbThGV3hwajVaTmw?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,52 +2330,52 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46084.37363425926</v>
+        <v>46085.52530092592</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Village Ingolstadt (fallback)</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FC Ingolstadt 04 vs. Verl: Live game updates, stats, play-by-play - Yahoo Sports</t>
+          <t>Kildare still battling on all fronts after mixed weekend - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FC Ingolstadt 04 vs. Verl: Live game updates, stats, play-by-play - Yahoo Sports</t>
+          <t>Kildare still battling on all fronts after mixed weekend - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 19:08:32 GMT</t>
+          <t>Wed, 04 Mar 2026 11:00:39 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOeEdEZWE0UnZickRnVkFJMjJZYXhGbUNyMldocDNRV0FhV0hIcG0tVUlvenphVTIzTVl1X2NsdE0yT1lCM08xTmJDd2FZVzR3VE1XRVhaT01iNWtEdkMtZ3dtdDV1NnFCR3llSmp4OHJaSGdqTXE3RVY1YmlfTlFUOV9n?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPRWJQc1RFR2JLakctbmhlZTlXbjVRRDJhUFI3YkY1TVdFMXR6SWVqRmlsZzczNnllUnZlMVZrVTlPQjRJRDlvWmtpWTYzV24xYkVobndycGREZVdkT3UwaDM4b3ItUUlNME9KZUg1WldUZG9YNE9iUXM4UnJxc1JhSTY2STJVamJPeDg5R3lvdUNIU0xnSkQxWG9ObmRHYWN5S1hUNG1mOFdyNnlraWJiVHVB?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2399,38 +2399,38 @@
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46084.79759259259</v>
+        <v>46085.45878472222</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sciopero trasporti marzo 2026: quando si fermano treni, aerei e mezzi pubblici locali - ItaliaOggi</t>
+          <t>Kildare Death Notices for today: Wednesday, March 4 2026 - Kildare Live Leinster Leader</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Transport strike March 2026: when trains, planes and local public transport stop - ItaliaOggi</t>
+          <t>Kildare Death Notices for today: Wednesday, March 4 2026 - Kildare Live Leinster Leader</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 04:47:37 GMT</t>
+          <t>Wed, 04 Mar 2026 10:03:11 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOQzJqcF85TU9pOVRPcWoyYzFJYzJYRGx2X3I0QnI0cVJNRG05UUZCNl93YlEtUEpKZFZ1WnhXSlUyTm1ZbTMxQ0xKdURUaVNvd1RiaVFVUWdSWXpGNm10MzB3Vmp5WlcwSTY1czhaQUZoQXg1OHVHUDFmallBNEhmdWdLc0hpbmNzR1QwbGNxSUhjU29VS2huUnVKcjQ3dnNmby1MMENEOFV5MjVBRkJYLUgyeUxoZlE4ai0tY2ZQdzZ4cUtPTWlhc3hJNFVBUmZQYUdNbk5xV1ktRG5QdjZJSnJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxNQjBiT1JIREpwc18ydmlwbGd6a2NZdlpnMEhjTUhtak5MUUI0Uk1ORjBUVnJVWjRxNGVlcElyWl94OHZyV1hOTEgwcHcxUlBCX1pueTR4UHZqTmNzSktrNzFSSVZVSERDejBNRnVpVE9QSng4MmpuVDc2LUEtS0VfeldRSC1QSXdwYmtaQWZrTmplS2E1amhMTTZmT1BDRklDWlM0ZEl0TEpOU0dvMFE?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,52 +2440,52 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46085.1997337963</v>
+        <v>46085.41887731481</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Manifestazione contro la guerra in Iran: insulti e urla tra attivisti di sinistra e iraniani - milanotoday.it</t>
+          <t>Shotguns, bolt-action rifles and cash stolen from Kildare residence - Kildare Now</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Demonstration against the war in Iran: insults and shouting between left-wing and Iranian activists - milanotoday.it</t>
+          <t>Shotguns, bolt-action rifles and cash stolen from Kildare residence - Kildare Now</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 17:51:11 GMT</t>
+          <t>Wed, 04 Mar 2026 13:05:00 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1rV1RFMGRuaW1saXNVdzRUU2ZQT1hBQ016SjlwS193TmN4NlZNZTdGa29SOFBfOEM2RDNKc3R5Zk9UaFBwYzIwdHE4TXZXM3A0LUpZajJuNl9KTjZsalg5dzY4aXZLN2VROW1mYnRjdWJ1QUl3YlJZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQWGVUVkVXSktfakdoUmNrbHhvTHN1aEdHbmp3RE9JcnJCdGJyVTFRQ2ZDTFRIaDZFanYxaVJwdlFhenlnTHltejA4STROZ0pJZG9KOUY3SFA3bkxQVlVEdjZJWXlHMXJpODlFbHFhX3k3azZTeGM4WkFJd1V0b1V1Vy1XR3U5S3lIY2lhYmFRRjhGTWdTTFVxY21SSmJEZ1U4UnVMS2ZoSzk1RThmUVFaeHFMcVc0UXFoWU1rdEhsdw?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,52 +2495,52 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46084.74387731482</v>
+        <v>46085.54513888889</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Protesta a Bologna, operai al lavoro nel parco. Sotto il carcere presidio in solidarietà con gli arrestati - Il Resto del Carlino</t>
+          <t>COMMENT: Is Kildare's season Slip Sliding Away? - Kildare Now</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Protest in Bologna, workers at work in the park. Under the prison garrison in solidarity with those arrested - Il Resto del Carlino</t>
+          <t>COMMENT: Is Kildare's season Slip Sliding Away? - Kildare Now</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 13:06:50 GMT</t>
+          <t>Wed, 04 Mar 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNQk90eVFYLXRKNXpjX2dwNEh3YlV6VDJQUG9UQ2lrSzc4Mk5hU09lQnBRTktOSExQelVFdVJzRUpRSldlUXpESTVDTzZqNEVTN3JZeFl6alZLQlZRU0FmOVBhbGxGV05CbXlkZFZETUJHMzQtdVZVcy0yWDVpUFVmRy1QdWlQMjJCTDZua3FhWjlwQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxQbkhRUmJDUVhJVElCZ0s3UHMwbThhcXkxQWY3UGJhbG5LRlZQVXlNSkJlVEpzS29TcGZRcC1PUlJTQ19lTVM5Um5UdVhXNXplVUVKdUZWSFM0VWZXR1VydnlWT0VjbHFiVUhCVElHTXJsTGZhc3VybVEtVWRXYVNNblljWDVTZ1ZNUE9ndE1VZHoyV2hjSWk4Nm93?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,52 +2550,52 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46084.54641203704</v>
+        <v>46085.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>L’8 marzo (e il 9) di Non Una di Meno a Bologna - Radio Città Fujiko</t>
+          <t>Recent floods crisis in Kildare raised in Seanad - Kildare Now</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>March 8th (and 9th) of Non Una di Meno in Bologna - Radio Città Fujiko</t>
+          <t>Recent floods crisis in Kildare raised in Seanad - Kildare Now</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 08:16:33 GMT</t>
+          <t>Wed, 04 Mar 2026 12:30:00 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxOSkhqSmFpMGxENUp4dWplZ1JvRm9WVkhoT0l0OFNZdWUwTkhjckYtLVY2a2NBSHp4NmdkdVVjN2E2X2dTVGMxby1TRmQzWWJ3c0ctbXhLNDM1QUVOV0QzTEM2alJmbko3cE9oVl95bnpBUTY5VVZEUlVpdmZHX3BDbEw1NA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNMEV5cHl6dUl5SGlLclVRQkhDY1BVQmREcU1CbmJ6ME8zQ2dzakJlUlFNb1FQRDBPUWZtNUZGd1BBQlNtZ3VCcXBVREFDUWpuYjNNNGc5NTgyUlBXSmR6dlRpQTZydFBwblc0aFF5REpfdTNxSlBsczFib011X2dTM3dGdUdMLUJCV0JKbS1qcktZOTZPOXp6cGFBb09NUC0yaXdzQ0hlNA?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,52 +2605,52 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46084.34482638889</v>
+        <v>46085.52083333334</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Scioperi marzo 2026: il calendario completo delle agitazioni sindacali. Il 9 marzo si ferma la scuola - Orizzonte Scuola Notizie</t>
+          <t>Tesco shoppers complain ‘screaming’ self-checkouts leave them avoiding UK stores - Bicester Advertiser</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Strikes March 2026: the complete calendar of industrial unrest. School stops on March 9th - Orizzonte Scuola Notizie</t>
+          <t>Tesco shoppers complain ‘screaming’ self-checkouts leave them avoiding UK stores - Bicester Advertiser</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 09:40:43 GMT</t>
+          <t>Wed, 04 Mar 2026 10:41:33 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPTlZLTDNGWk9rdFhBc01zWkdKSFBua0xMSWdXZGg3S0dIWE1lVGdmdDV0ZnM4T0tfTFRzOTB2cUdMOFpvU2k1TGZRY3RFaTZ3bG5fYWpENndUNDA3ZWEyTVVzU2NLYmhKdmJyYWRsc1VubllKTUlHVnFtUTgzOXpuVzVQdWdqZGhMY3ByaGZaVURDS3JrbWxpbDE3QkszQ04zR2lkc2VEV3NOaU1uN2Jqb3d1NlBrcWwyWGxSVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQZk1reU9iRkFScFZXUmhPdEFqR0gyMXUwTUtGSEtPTVdUVVRwSlVZei00dWxZMTU5RG03bHd0V2JWei1BWnBHNVUyek01eWdTZllrQTM4V2dDa2JqUUIwTDQxdldoQ0tLaU1vOWlVMGFLVk9kYnN1OWJpLWNGTnhfaC0wam5SOFozcXNIQjBRMDRqbzMzeEo5aGpiMTBEWEhLVHc0?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,52 +2660,52 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46084.40327546297</v>
+        <v>46085.44552083333</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Libera Masseria, da dieci anni simbolo di presidio sociale - Chiesa di Milano</t>
+          <t>Owner of almost 30 Oxfordshire pubs considering significant job cuts - Bicester Advertiser</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Libera Masseria, a symbol of social protection for ten years - Church of Milan</t>
+          <t>Owner of almost 30 Oxfordshire pubs considering significant job cuts - Bicester Advertiser</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 06:08:27 GMT</t>
+          <t>Wed, 04 Mar 2026 09:22:10 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNRXFDNlozZS1kVU9ZX2Mtejh0TDdkYnk4ekZ5eVBSTVJCZW1rOXhVa3VRdkRQaXRGeGhMYlpidDJNNmFsdVVhSURtYkg4a005MGtFclZyOUtINkpxQ2JoTTcySjNuWlN2Vmo3dnVBS2RnRXRNejNZSG14S0VkdmJNdEhTNXN5d1VRUHZaenN1N1pHWkUxcWJ5bVpIclFFWnNZaHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPTWRaeDFMSGZFd3hsWGY3RE1BSWJGTVBMbmcxSGpfQkVoeXh3MnJvN0x2b1BwdmUzTDZFeTVIR3l5N2pEbzlXSzdXY2VvU0V3RWpRT29venR6a2Jja2c0Z1Rkb0lHSi1Rc3o2RW9qcUtCVU85b3VhOEhwb3BmX1h6T3dUeDBhcExhSmJ1U09US0VaR2xqaDN0aEtIVXF5WWhxRjhyNVVKVTZVRjg?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46085.25586805555</v>
+        <v>46085.39039351852</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Decreto sicurezza, una pioggia di multe per bloccare proteste e dissenso - il manifesto</t>
+          <t>Enoch Burke’s mother and sister jailed for contempt of court - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Security decree, a shower of fines to block protests and dissent - the manifesto</t>
+          <t>Enoch Burke’s mother and sister jailed for contempt of court - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Tue, 03 Mar 2026 23:27:19 GMT</t>
+          <t>Wed, 04 Mar 2026 12:00:49 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxNOFV3a2hDcnZCQXk3OEN1M29RWVllOXk5bVBHUDdDSFdqdjJRWGpkZmtWYWN2cnhYSUM4aUU5N3VMdTVLVjJ6NWVzNkp5VXVJbW9RcUVETXF2cVRQcW1rRVNfWk05TWdTMjVVNENHQ1I1ZjBWalU1SlBONFFlTTM0QlNYeWl2QWc0TkRtQl9sa19Ybmk3VVFQSk1n?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOLUNkaG5xcGVXRkk5c2NlWEV6Q0c3d05Sek9tTHI4RHVyYmFoRkV3YVdsZXU1M1lOR3Fkcm5YNlU5NnJyMzBXUUdpMFBKeEtsZTREMXdYMzc2WGNUTUNfMHVBWTYxOFFNZTh3aVVkNXl2Tm5IVWFWOXBsemplbjZVUGd5bzhzRWxtZEZJMVRrNUNwOEtqaEJHT0t6TVhKeWhGMHdyWXhHZVBfS1VCb3N5N2Q5Q0pNdw?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46084.97730324074</v>
+        <v>46085.50056712963</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>High Level City Italy Italian</t>
+          <t>Village Bicester Kildare (fallback)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester" OR "Kildare") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bufera Marelli: bonus solo agli impiegati, scatta lo sciopero - BolognaToday</t>
+          <t>What the papers say: Wednesday's front pages - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Marelli storm: bonus only for employees, strike starts - BolognaToday</t>
+          <t>What the papers say: Wednesday's front pages - kildare-nationalist.ie</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Wed, 04 Mar 2026 06:58:55 GMT</t>
+          <t>Wed, 04 Mar 2026 08:39:38 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE1EMHk3T3ZKUjFscGhxNUllb0dfY29FVHpPbXBrLVlRUk1iUmFqaVlRRVlCaFM3R3EwakNwQ3NHQ3MwRVJMLXUzcktmNzhEVHg5NnBzUXRLbWRSMXh6NXoycDBvVkdndXMxOUdOZXpNRkFjQ2pKZmdRSFRpSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxQRkM4dnFoUlNCZTdtdkx4VFN6WFRUN0ZmRVI5d0ZjVF9PWndxUFdRMEw5V2xHY1FiczBReGVzVTQ5aHRUT1JwWDhJT1Y5cWI1TGpuVGxNcWdHVjRFOUsycnFqRnRpaTBKQmJkSHpCYmFYc0hPMXg2emhzeW5OdENxSl9teXlyV2tlY0ZoMGJ2OFlvaHhnTkdoRVhoWTJtQkE?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,131 +2825,21 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>it</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>IT:it</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46085.29091435186</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>BOLOGNA: LACRIMOGENI AD ALTEZZA D’UOMO E CARICHE CONTRO I MU.BASTA. “IL PILASTRO NON SI ARRENDE. LA MOBILITAZIONE CONTINUA” - Radio Onda d`Urto</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>BOLOGNA: TEAR GAS AT HEAD LEVEL AND CHARGES AGAINST THE MU.BASTA. "THE PILLAR DOES NOT GIVE UP. THE MOBILITATION CONTINUES" - Radio Onda d`Urto</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Tue, 03 Mar 2026 17:03:00 GMT</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxPeXYzSTlPeHl3YURqRmZBMF85QnBDY052czQ5R2oxWUpDbDA4SHZoVm9RdHYyd1NsR3gzUzFnNFNrcXViMVVRWE1Rcm9qS09TSHp3aTE0WEVjV21tVHZUTzVyem1xSWhXeUZwdFo0cUZ3MlB1MHBEcjlxN1h5bzlQQmlXYWY2cmRObTY4SkRGSHJKdHVoODVZYk9mVmUxenI1b1BROXN6cC1tNzFfbTg1RDItX2pycWlTV1lpM1lub2pxdE1mSDU2MlpJRl9xQ1hyUWNlczJ1Ukk0Y283LXRhV0V5YVhMNGVvX3p1LUl5LUc?oc=5</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K45" s="1" t="n">
-        <v>46084.71041666667</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>High Level City Italy Italian</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>No, la CGIL non ha proclamato uno sciopero per “la caduta del regime iraniano” - facta.news</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>No, the CGIL did not call a strike for "the fall of the Iranian regime" - facta.news</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Tue, 03 Mar 2026 14:39:03 GMT</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE1uNE8xSWNWZFB4ZE9kS2paaVdWTENqc0loVDR2N3hYR0g0eEJZVkdiOUVtc1gyUy1BMjV4NXhTdC03YTF4ZjVhRGZlaGRaLW9zY0VnVmtqUm1tYjN0NVp0Rk41YWNLLU9hWEFOTWFNR2FFbzhlTkktUzdB?oc=5</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>it</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>IT:it</t>
-        </is>
-      </c>
-      <c r="K46" s="1" t="n">
-        <v>46084.61045138889</v>
+        <v>46085.36085648148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-06 07:46 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail (LON:BME) Share Price Passes Below 200 Day Moving Average - Here's What Happened - MarketBeat</t>
+          <t>B&amp;M European Value Retail (LON:BME) Share Price Passes Below 200 Day Moving Average – Here’s What Happened - Defense World</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M European Value Retail (LON:BME) Share Price Passes Below 200 Day Moving Average - Here's What Happened - MarketBeat</t>
+          <t>B&amp;M European Value Retail (LON:BME) Share Price Passes Below 200 Day Moving Average – Here’s What Happened - Defense World</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 08:20:14 GMT</t>
+          <t>Fri, 06 Mar 2026 02:49:13 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxON0pnSWY4cWJFRDgxLXRXUy14RnJYVnFGWUlpZnAyQXI2b2hFLXV5MDN5U2NuRHFpalE1RURiU2dsTWZPeFRFeXViT29QOTNfaHM2YTZzUG4ycldHQXdRLWNEWUpHZUp1R01fZy1KUzJ5dTVyVVFxZU03d0VUd2lESTZUc1FwTm52VXk1TllnaUVtZGZKMEVBWTRMOFZCZWpuWXZKWDVlUFVUdXp5b2lxMHJtS3UtbHZnc2Rscld3Y3UyNGUyZVJxXy1mOVQxRkUyelpHT0hmanJIQkI5cHFGUEE5UEtUVV8t?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxOUGVTblc3d1ZLQ0tXZnRxT2NmNjd4QWpYaUtDTVJ5R3lPRVFBaDhQV05Hb0syVHJYRHNaT0Q2ZEpCM19WbHptNXR5TTZoRVRtTzhLa2pUSkc3YjlGX2J6QmlmV3lpOWktdTZ3SHhsVlNpSlFkMnJFQ2pSN3lscTJPQzIwQklrNHVVcHVQSFVvWGcyNzFwYi1BUzdMVGlnQ3dvMWppVVQ2Ul9NNHF4NzREVUR0Sm5udlN2QTY4ZVFwa1p5VEdKTG16aEhBSjYxSTEzQU1vTGJvV2hab1R2?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46086.34738425926</v>
+        <v>46087.11751157408</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>London Marylebone Incident</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>All lines blocked at London Marylebone – here’s what you need to know - London Now</t>
+          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - AOL.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>All lines blocked at London Marylebone – here’s what you need to know - London Now</t>
+          <t>'I make between £800 and £2,000 a month on zero-hours contracts. There's no consistency' - AOL.com</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 08:40:35 GMT</t>
+          <t>Thu, 05 Mar 2026 15:33:05 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQXzZyNjEtU1lDd2ZvOFY2VDB5c2k2RktPMXpTNERSdXVwYUZUTVBDSkVkMzhSTVgyU2hISUFuNVc4QXlXTVE1LXk2UnJHQTZNWEl1b2Z0ZkEzMFBaR3NBZlNLSmN3cTdfOWU5anowVkFoS2QxSnRYZXVQT1lOLURJanNkZmVfazlhS1ZNR1JGdmdCZndzdWNsU1lvUWxNZ0hLUFJvSA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE84UkdzeExGN2xLSUh5VnBiUlNFTkI1ZWl1bVo2RFVEeVUwdnZaSjNuS2hrOVhlam9pamJzUTRGRWZsOER6Y0hXRFpxTGs4bXZzdTZ4YXNxVlVaNXpCUTVuT3pHeXVlOHA5V3FLZHVUa3ZtYVV4aXNVUDZEek4?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46086.3615162037</v>
+        <v>46086.64797453704</v>
       </c>
     </row>
     <row r="4">
@@ -600,22 +600,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>‘Casey 2’ inquiry launched into Met’s overhaul since Sarah Everard murder - London Evening Standard</t>
+          <t>All lines blocked at London Marylebone – here’s what you need to know - London Now</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>‘Casey 2’ inquiry launched into Met’s overhaul since Sarah Everard murder - London Evening Standard</t>
+          <t>All lines blocked at London Marylebone – here’s what you need to know - London Now</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:04:28 GMT</t>
+          <t>Thu, 05 Mar 2026 08:40:35 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQRGRYNEt2RkxuTUpFLWlULUNkTzU0LV9zTUgzRkZ6dEt6aUNZWk9uMGJYOTlYeHNHd2JjZm9mUk15aUxNWVh2VFNMWDUtMExNdFp4X0x6N2RCak5iNHp3V2hvVW13LXlqRmNNalFDcXM2S2NOM29xNzFHdjBPZ3d1MzlWaGdPVVNuVTdwYm5oOGc0SHozWU5NdURJRGk4SEJzbmtRME1SSXNFTmh6WlJKdlI5V1B2Y2xhbWNvQk5tWElGNm5Pek9Cb1hqTzY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNWTRrdVIxT2VyazRBVXhDWnlBYnNsbkk0TDNucEdrLXJYczMxeXlGN3d2OWZlS1F5NGRYVFIzMXhnQ3RwSERERldwVTlrcGtkeWdUVF9YQl81SHdpdnNDMmtSZTZyRVF1VHpjajFQeHhqVnV4SWJ3Y0c4NHlUX3NZTXNzdWpMVGFIMkw2MGJMVlZaem5hYW80aFpqdEg?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46086.50310185185</v>
+        <v>46086.3615162037</v>
       </c>
     </row>
     <row r="5">
@@ -710,22 +710,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Husband of Labour MP questioned after arrest on suspicion of spying for China - London Evening Standard</t>
+          <t>‘Casey 2’ inquiry launched into Met’s overhaul since Sarah Everard murder - London Evening Standard</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Husband of Labour MP questioned after arrest on suspicion of spying for China - London Evening Standard</t>
+          <t>‘Casey 2’ inquiry launched into Met’s overhaul since Sarah Everard murder - London Evening Standard</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:13:35 GMT</t>
+          <t>Thu, 05 Mar 2026 14:04:44 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxORUVZbnJyTFJnaHFvMEs3M1ZPdVhfMFE3RGIwMXlhQ1pZOGd2WXI2elB5Wl9tZThnZFlaLWN5Zms5ZENfa1JKcmM1a2Y0SXZUS0w1bng5UmxCSkE1d2NIRWdEc1Q2emlMSV9sQjRMRnRZdG5nMkVyMUhmRTVndG0zWnRqcWp3dmdQN2tIY0llc25aZnlZdnE4VjFOZFdkZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxQRGRYNEt2RkxuTUpFLWlULUNkTzU0LV9zTUgzRkZ6dEt6aUNZWk9uMGJYOTlYeHNHd2JjZm9mUk15aUxNWVh2VFNMWDUtMExNdFp4X0x6N2RCak5iNHp3V2hvVW13LXlqRmNNalFDcXM2S2NOM29xNzFHdjBPZ3d1MzlWaGdPVVNuVTdwYm5oOGc0SHozWU5NdURJRGk4SEJzbmtRME1SSXNFTmh6WlJKdlI5V1B2Y2xhbWNvQk5tWElGNm5Pek9Cb1hqTzY?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46086.42609953704</v>
+        <v>46086.58662037037</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Raver nicknamed Nasty guilty of killing deaf woman with single punch - London Evening Standard</t>
+          <t>Husband of Labour MP questioned after arrest on suspicion of spying for China - London Evening Standard</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Raver nicknamed Nasty guilty of killing deaf woman with single punch - London Evening Standard</t>
+          <t>Husband of Labour MP questioned after arrest on suspicion of spying for China - London Evening Standard</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:22:34 GMT</t>
+          <t>Thu, 05 Mar 2026 10:13:35 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNYkpSTEpxbHo2QjFzS0l5RUtCeXpaS0huMzhYQ01oS2NoYTdweHR5cnJtM3M4eXVZZmhWLVdFWlF2eWUwbXZvTHNVVF95TFN3ckh5SURGV1U3WmRVQVhSWDdUZFY5MXdpZnBNMHlCdFZyLTZVTlJVd3owNUtyNG1VcTlPNWdqbS1Ea1RaR3pRVFl2bk90dEZJaDNBM25UcUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxORUVZbnJyTFJnaHFvMEs3M1ZPdVhfMFE3RGIwMXlhQ1pZOGd2WXI2elB5Wl9tZThnZFlaLWN5Zms5ZENfa1JKcmM1a2Y0SXZUS0w1bng5UmxCSkE1d2NIRWdEc1Q2emlMSV9sQjRMRnRZdG5nMkVyMUhmRTVndG0zWnRqcWp3dmdQN2tIY0llc25aZnlZdnE4VjFOZFdkZw?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46086.55733796296</v>
+        <v>46086.42609953704</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Risks from Chinese spying ‘not receding’, Speaker warns parliamentary staff - London Evening Standard</t>
+          <t>Raver nicknamed Nasty guilty of killing deaf woman with single punch - London Evening Standard</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Risks from Chinese spying ‘not receding’, Speaker warns parliamentary staff - London Evening Standard</t>
+          <t>Raver nicknamed Nasty guilty of killing deaf woman with single punch - London Evening Standard</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:55:38 GMT</t>
+          <t>Thu, 05 Mar 2026 13:22:34 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNLTlsTzJZS3lUWUl5Z2lfRjEwZDFkaHVXTWdFUzhtRFZINmVYUnpYQ21XdklOM3MzMlhLYmsxRW5URWk1UFViUENZaElPUkNiUXZlc2pndFdtWjdtVGtrTzVYRnFmNmNuY2tLelhiRm5Uemh3NnRSdGxSN0REVFVMRmdpbmVSZnJSY1ZvRkZJTG5qbFJZUnpGTFZvZlBnOFg4cy1ici11eDVfNXJfWi1BVw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNYkpSTEpxbHo2QjFzS0l5RUtCeXpaS0huMzhYQ01oS2NoYTdweHR5cnJtM3M4eXVZZmhWLVdFWlF2eWUwbXZvTHNVVF95TFN3ckh5SURGV1U3WmRVQVhSWDdUZFY5MXdpZnBNMHlCdFZyLTZVTlJVd3owNUtyNG1VcTlPNWdqbS1Ea1RaR3pRVFl2bk90dEZJaDNBM25UcUU?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,38 +859,38 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46086.49696759259</v>
+        <v>46086.55733796296</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station") AND (incident OR disruption OR closure OR police OR bomb OR explosion OR stabbing OR shooting OR "suspicious package")</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Is gedwongen hulpverlening het redmiddel voor drugsoverlast De Coninckplein? “Een zéér drastische maatregel” - GVA</t>
+          <t>Risks from Chinese spying ‘not receding’, Speaker warns parliamentary staff - London Evening Standard</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Is forced assistance the remedy for drug nuisance at De Coninckplein? “A very drastic measure” - GVA</t>
+          <t>Risks from Chinese spying ‘not receding’, Speaker warns parliamentary staff - London Evening Standard</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:00:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:48:45 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxPbFFlNC13N1ZqSXpHRW8xRkw5VzMwNFQ3ZkVCenhDSHpwTk56eE9OVjA1eGRyNkpHVEs3RTcwVTR6eEpiRWx2bURwSHIzZ0N4MWpFRWFkaHZ6ZFltdFRkd2l5SWlXd2RYc2g1QnZxZWVISDd1UmJHckZIM2dwcy1IN2dBVDlxZDFGYS1oWjgtWHVoUHdtdlJCN1EtNnpMRENXWlB0WnpKakt4RUs4NWIwNW9YMlN2c1FpbXJjNktnbHBWcTJKM3JvTVpoUTVrTHYxeEh5QUs2RDZmdWw4YlRpN0xXWVpRc0IxU0daVmNYVEh0eG9DcXNEeDRQNEs0cDhISnB3eTVfaE5uaC16bUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNLTlsTzJZS3lUWUl5Z2lfRjEwZDFkaHVXTWdFUzhtRFZINmVYUnpYQ21XdklOM3MzMlhLYmsxRW5URWk1UFViUENZaElPUkNiUXZlc2pndFdtWjdtVGtrTzVYRnFmNmNuY2tLelhiRm5Uemh3NnRSdGxSN0REVFVMRmdpbmVSZnJSY1ZvRkZJTG5qbFJZUnpGTFZvZlBnOFg4cy1ici11eDVfNXJfWi1BVw?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,21 +900,21 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46086.41666666666</v>
+        <v>46086.4921875</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Appie vzw gaat ijsberen en Lowieke herdenken voor goede doel in De Mosten: “IJsbaden heeft therapeutisch effect” - GVA</t>
+          <t>Gewonde bij steekpartij in centrum Antwerpen: geen levensgevaar - VRT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Appie vzw will commemorate polar bears and Lowieke for a good cause in De Mosten: “Ice baths have a therapeutic effect” - GVA</t>
+          <t>Injured in stabbing in the center of Antwerp: no danger to life - VRT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:17:52 GMT</t>
+          <t>Thu, 05 Mar 2026 17:04:04 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAJBVV95cUxPVFdZdWhfOVkxMXBvdjRWYjdWakRGd2JWU2hBZFVMenBrVEV1LTJZZE13NzA5NTdaMXlMMGcyZWxQcGNHem44dHdhOExuZWRfSFhPS2laTXhqMkF5OXZqeDQ3TE5HN2hlRGc1amc1MXZXMldicHFjeW5xS05Ld0FVVWRob1B4TE03OHdhZGZESk5YWVB6MG1xUUlRT3FZTFVBRzRST1F3YzBrRHVOWWhzTXkyNVlKN1gwcGZDUUNIbWxOQzVFR21VR2hBdzFGTC1VYzA2TVdpbVY1aDc5VnR0SkhBVWRJbjRRdWVSS3RYSUdkSmNiLU9RNnlMay11VjlKaG5RSUl6aTJucklHdFlBcA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPVXFjb09feVVNLUtDRS1FYWNmQ19ZMmFST0VvOXZuNlhTVFBPSjVSUlgwZ2ZrTTZJMGkzSV85aXFWb2lQa1dUTlA4ckNBLUNsbWFVSnJ2NkZNc04yNS01MjVuU0tPTTV6SVFMR0dHMS1fYlNrS2VtdzlvVjF6aTNxY1hfazJOUDFMMjNmZE1aTm82QQ?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46086.47074074074</v>
+        <v>46086.71115740741</v>
       </c>
     </row>
     <row r="11">
@@ -985,22 +985,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Peiskos Quartet verzorgt springplankconcert in Protestantse Kerk - De Limburger</t>
+          <t>Jessy Mackenzie getuigt na MeToo-bom in muziekwereld: “Ik werd als 18-jarige zelf gemanipuleerd” - HLN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Peiskos Quartet provides springboard concert in Protestant Church - De Limburger</t>
+          <t>Jessy Mackenzie testifies after MeToo bomb in the music world: “I was manipulated as an 18-year-old” - HLN</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:48:20 GMT</t>
+          <t>Fri, 06 Mar 2026 05:49:43 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQTHpzcmN5ZGQtX2hmRzgzSEtEZGxMREdQbWVmQ0lKLTlLMHllV2FNbDI2b254V05UQXpmV2ZHaXJPME80amxBbkp6U2pHV1JORFd2TWlOXzg4NDJEWi1UY1BqNTFHLXJyRTMxTDdidjcxalhxOEg1UXd3RlNNaEhpVFltRmRrQ3VZNmJ5aUdPQzZNTGR0dXJMdXZ6dkhiMUJHMVM2UFlwdnlVcm1vTExJSkxJcG1SN1J4M2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNbmFXaGpuakhNRHo4c0pwWUNiV2laTWk2V3RSMWlWdXJlTnljZ2dSWnBHOGd1SmlaSnZEV1o0dzBaVUpoMjRWUzRmWnk3MFpyVEhuSzFMX0VYbDNiZkdxTVpnWXNhZVMzb2ZEZExnU1ZKMTkxaTFZcHR5dk94UHJRVXB1U0lEYUoyYTBxR2k5TEd6cmpBZGROcTdoX0owOWNieUtTX0k4WF9La3NWbHNtVU5kRmJVUVAxR0E5Vl9SZGFZc0QwY3Q4N05aQQ?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,38 +1024,38 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46086.49189814815</v>
+        <v>46087.24285879629</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Exclusive-NATO's Rutte Does Not See Need to Invoke Art. 5 After Missile Incident - U.S. News &amp; World Report</t>
+          <t>Hij fraudeerde voor miljarden, zit nu vast in Antwerpen en wil absoluut niet uitgeleverd worden: wie is Mehul Choski? ‘Sinds zijn arrestatie worden we gestalkt door een leger journalisten uit India’ - Humo: The Wild Site</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Exclusive-NATO's Rutte Does Not See Need to Invoke Art. 5 After Missile Incident - U.S. News &amp; World Report</t>
+          <t>He committed billions in fraud, is now stuck in Antwerp and absolutely does not want to be extradited: who is Mehul Choski? 'Since his arrest we have been stalked by an army of journalists from India' - Humo: The Wild Site</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:09:41 GMT</t>
+          <t>Thu, 05 Mar 2026 14:42:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPMWV6eThHVk0zYkVfRkE0ZmUtdUFHT3dqUUFzVGhDYnVkV09vclBBQ1NKc2kyUE40eGtFckFWTDVvXzhUc3Bxb3Bhdk91bjZfV0Uza1dGNHVLd2NwZkhuNHhRQlgzZmxxNVNPaTZTM2N1Wm5FR3FZYmJaVmczblVvandnNTc0eWxkSkdPc0F2MjdaUjlyekFCRUlXQmp0SHh2TDBub3NyVFpKYjAxa3BYRDVsc2NaMEdObVpydEg3NWVadjZsWHJlQVl3U3lkWHlOWGYzclFJZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizwJBVV95cUxQYk0wNDFJbHNnMUp3VF9MU1ZfZkttOGkyM1FCbWlUNUNKZUtoOGN5UG5jRnNibjFJczlXNWFIYlVWS2drUkFtUlg3Z290UWtaVDFob19TOUFHZUQ0bS1pZ09SSTBjVTRwN3gzSFBoR1A5SllEcGEtR2FRTERqTDBhZHE2eTh4eHJuZzJfUGZadGg5cFlWWFNMa19vOWRRS1FLQ043dWJ1ZkRxRVR3ZTZGUjlzNGFaMDJKSndSNTliR2ZncXUxM1U5dkwtVTA4NFZuUVpFR29NWF9DOFJxcDBaenNGUGNwOGloYXpPRGY4SFFlYnRLZy1iVkRnLW1LUjdDTjF1QmVIeTBCQU5XRFVWeVhGY3I5aHkwbEFJX1JSTDNaaWk4UHhyWUtkMWlKd1hSeW5CdHZoX3o0OTlzR05Lbk5kNnZsSjUxLXRJZWNSYw?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46086.50672453704</v>
+        <v>46086.6125</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Iranian regime “conservative”? Never, the mullahs are like 19th century Bolsheviks - Brussels Signal</t>
+          <t>Britney Spears slingerde over de weg voor arrestatie: zangeres “extreem emotioneel” en naar ziekenhuis gebracht - HLN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Iranian regime “conservative”? Never, the mullahs are like 19th century Bolsheviks - Brussels Signal</t>
+          <t>Britney Spears swung across the road for arrest: singer “extremely emotional” and taken to hospital - HLN</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:03:11 GMT</t>
+          <t>Fri, 06 Mar 2026 05:52:43 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWWFncXVOemxxYm1qOXpycnVRQmRza0Y1NlByR0ZRY0ZQVmVBTlJoTEpoV1dxMENHekJVeE4ySWJSZXBvdTVZeFN1SVZVbERnLVBuZFV1R0syNHNEMThfamlVcUlZNnIzYXZsV185NXdINjhMU1VaWVg2YklRU2U4dXhERHRlMm9hWldXbWpZRVotNTZwUmpaQVFGWi1wM1I3bjlpNTJLQUY2NEpoaDNZU0RQNA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxNcnpOSEFlSGJZeUZqQ0JuUl9TZVJ5cnU1eGJTeTJDUEVIc1F3RDhXQ2xydWdRcVdRVHM1WGx0djYwdmhBckRzWXBoWVdCbUtyRTlxR3pZeWtNZEJQMlZYbjY5alQxRmVPRTBydnpMNmVDNC13dUhkOXRtZHd1RkIxR0VURUcxYUpaNFVJdFREQ2hzMHRKZGVXejgteEtLZDlNTzUwcnRaWE5TdmF5WFBBeEQ2WEhic1RIZWVTMk9SbGZRUkllY3QxNzVGOUtSNFlrMWdEdGFrWTZCeGM3a2RMRnNFNA?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46086.46054398148</v>
+        <v>46087.24494212963</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>French appeals court lowers charges against police officer facing trial for killing of teenager - The Straits Times</t>
+          <t>Jente Bogaerts (Chocolatjeeke) is ‘Strafste Onderneemster’ van Antwerpen: “Ik wil vooral niet te groot worden zodat de kwaliteit blijft behouden” - GVA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>French appeals court lowers charges against police officer facing trial for killing of teenager - The Straits Times</t>
+          <t>Jente Bogaerts (Chocolatjeeke) is 'Toughest Entrepreneur' in Antwerp: "I especially don't want to grow too big so that the quality is maintained" - GVA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:39:02 GMT</t>
+          <t>Fri, 06 Mar 2026 04:59:09 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxQYlRrLUhUUWEyZkdaV3d1clQ3ZnhNY3BUdzFXd3I3bE01VWt4NlhFYVFkMnVIOHQzWkhaVEhXUDI1T2tkc3dpNUYtcXlYenVCbFV1NGx5NG9VRFFFMU8yMWxqeEJCVXpyMkdoQjBPYzc1blBGR3FKcjdQZW9NNklVTHZ0bWdBUnZqcnhJS0MzMGNTYzZWZ0JOSllDSzd6OWxITWg1VTNpSXBvSVV6ei1QU3BQamVnUHZXcGpzRldMOGVwQVcxR0FTWTBtSXU2UWdvUHo0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgJBVV95cUxQX0plWHRybDFBTHViUF8tM3h1eWpYaG4tTFVNYllTSkdVdG9nTEpHb0M0cVp3eDcwN2FTckU2UWZVZkFiSHk3cVJic2I2Vmdid19XZ2RNZFRwYTBBZWFGMkNKRVFOZFFORG5aTExfc1NzYnR2U2lPTmlnWlRfYWgxRnAwSFFDUGpZLWN5UFAwMkpzdEs2Y3E1VVQ3bFlKOFVwV0p1VVRhUDBFOGxHYTM1TVNlblVhX1lwdk9WV2FqRjdHSlpVYVMwQjFycHRoQWQ1QlMyLTNRUlZmanhlWGRQVzVVV280TFJkNHhvd3dvLXBPS2pKZEFEUGNkc3pneVJHLUh0WHRtaFFHMEpQbkF2dHBuWUZhT3dFZHZaN3FpeVFEc2s2ZmdXQ2lfQjVjODl1RzhVa0xn?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46086.52710648148</v>
+        <v>46087.20774305556</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Syrian man handed 13-year sentence for Berlin Holocaust memorial stabbing - The Straits Times</t>
+          <t>Wat te doen dit weekend in Antwerpen? Van drumspektakel tot boekenzoektocht - HLN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Syrian man handed 13-year sentence for Berlin Holocaust memorial stabbing - The Straits Times</t>
+          <t>What to do this weekend in Antwerp? From drum spectacle to book search - HLN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:43:54 GMT</t>
+          <t>Fri, 06 Mar 2026 05:01:12 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQekhHR1Y3eXo2SU41d1h0aTlmS0NkWG9UUWtHbDRVQVJrUlJjMW9VTjdZV0FIcks5QnV4d09XeHBZUzlwQzJqczBlakF1QklVV1B3OTBDbU13bFNqbUhHNmp2WkZyUmdjUTJIcEU1Y21XcEFiR1piRml2ZFZxZHNiX2Rpckg2NngzUUNSd19LRVoycXBuZEhqQmdaV21mNkctd3JrbFNlZFBXc3FRYzNTRC1OVXlEQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNcmZkUkVvOC1fc2s1QkowTDFlNTE4aXMwUkMzVzhHa3BhNkVPZ1did284S0tDYmNzaGY2Y0tTd2RITjdwalFVNUxwQV9oNEhWT21kaU1wU1NhQWxELWk4SjJBTjRkYmpMOWU3Slg3eGJEc1kta0dVaVdJaE0xMFFfUkNyblcyZkhfcGxYUy05WVQ2VnpNb0dvdTRKNm5MeU8tTlVFTmVDNjBOaDJkN0JFX2Frcw?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46086.44715277778</v>
+        <v>46087.20916666667</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>NATO's Rutte backs Macron's nuclear revamp but says US umbrella is ultimate guarantee - The Straits Times</t>
+          <t>Iraans-Antwerpse Wali Sediqi stapt uit N-VA door partijstandpunt over oorlog: “Uitspraken van Francken doen pijn” - GVA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NATO's Rutte backs Macron's nuclear revamp but says US umbrella is ultimate guarantee - The Straits Times</t>
+          <t>Iranian-Antwerp Wali Sediqi leaves N-VA due to party position on war: “Francken's statements hurt” - GVA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:59:02 GMT</t>
+          <t>Thu, 05 Mar 2026 19:39:31 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNRFdDN25TY1M3X3J2LUNyOXdPV2dHWU80VHhxUHBtRFJDWVd0Ql94d3dpOGNNRnZMTDBIbHNPcDQ2UHJucWNqVGlJbkNqV1Fxb1hHV29adnlWeVNHSHVUM0VPX2xpSEJEMDFqMFBGTlBUYmk0NWJIclRRa1JpS1VBRXJHYjBQTExJN3ptWERsWTZ2a1ZlRVNLNGJZU3pQb2VxWENoLXdsTl83VWpVazdMTVd5TkZXR2NSNkZGdzRPdHdkU1E3cHAyM0YzZERqM052MHVLSQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAJBVV95cUxOZEY2SjEzVTlJdlF4Z3dWQzlacGlnTUg0bnFEbENtMVNLWWpncmM4ZXBQMDV0c1ZqY1NEOU82Z09jSHZreHg1QXdCRVhOdDNJUmIxMW1hNDZnMnVEYWs1bHBFSnhtc0RFdkctYjI2bHAwMDZKa1hKWHYwWFpreVY1OHczS0prRmQ3R1pkcGRqdlFQVDlUMmhRU3lDNGdndkFIOGV5ei1LQ3l3Qm9iQmxJbHNiTjNRbDNzSHJmdDc4N3RfbkY1Zk9WbkZtWUtER0hkem5CWjIzd0dmQU52SU5jNm1kbkdSTXN6VlN2LXVjWWtHaWNyWE96eGNjQWJSZ3JsZVBQYQ?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46086.54099537037</v>
+        <v>46086.8191087963</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Highlights of NATO chief's interview with Reuters - The Straits Times</t>
+          <t>Drie kwartier file op E313 naar Antwerpen door ongeval bij Antwerpen-Oost - HLN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Highlights of NATO chief's interview with Reuters - The Straits Times</t>
+          <t>Three quarters of an hour traffic jam on E313 to Antwerp due to accident near Antwerp East - HLN</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:34:14 GMT</t>
+          <t>Thu, 05 Mar 2026 23:16:55 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQMHVuSWM5TXZWbG16VmZIT2EtVmY4OUZWZWltU2RyZGg0U3JCTkpNVnNscGhhUHZ3RFhxeEpVUmJXRUdFTnUyZ0IzSHo1d2g1NElSS1B0bFZvV0s3eGJiOS0xNTU2TDVTYkFFV2JvMEZMQWt2VVVXZmEwREVQVGQtQnJ1MFhFQUlTMHhZYUZyOEFfM1pf?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxOZlpocl92Q1c2ZVdZbnY5RWlpeVBaai1MeDl2d0FvLVd5ai00Y3h3c2RBQzQzN29lOGtDV1lPTmJPME5KZlRUTWpDbHlrVnF3RWl4M1JfYnlCVGl0X1pTWmlzNDVLVVFaYy1FMWZiZTgtZXZpTWVrT05SQ1A2V1hjU0lQS0tLYXY3MFVGb0JrcHk4clZNaFEweDRwVnQ4YXBVN1ZGWVlIQXRZeEtzLTNBMGZn?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,42 +1350,42 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46086.56543981482</v>
+        <v>46086.97008101852</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Le Conseil Régional de Sécurité "afin d’évaluer les impacts potentiels pour Bruxelles" aura lieu ce mercredi - BX1</t>
+          <t>Leerlingen van het Stella Matutinacollege ontdekken de Belgische politiek in Brussel - HLN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>The Regional Security Council "in order to assess the potential impacts for Brussels" will take place this Wednesday - BX1</t>
+          <t>Students from the Stella Matutina College discover Belgian politics in Brussels - HLN</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:27:13 GMT</t>
+          <t>Thu, 05 Mar 2026 10:18:10 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOWjdWYjBpeFFCU3pQU3lsNVhTM2tKUEFFS2stQXhsVWtMbkhRdjRUdU1ucDF1MkkzWGJfczVMcWFGaVZrc3VrQXBVWGpTVmREeDI3M2xlZ21Vd0NFX18waHVmNElJVEQxZzI5d2w1SVlYRzg4eXcwbHNDaGNxUDlkMHpKc1ZaZXY2WF83SmdUZkthd2hiaUdFcGo5czM5TWZoaTJELUxqc29ORHJCOWtZeUV3ZG43YXl3UE5kaHZpUzN2WWhCbHQ4ajBFeGU5cU1VYVBZTkExYktIR054c1R2OE9lNElJMXNNQ2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQaWNBS3NPQjk2TC1WNmJmd3A3bEV3N283bFQxbjFkQWU5WTRmbmljTHBEQ1ZmUEw4TjNCMnNuaUxKOGlGSzA2Nm9fNllzeTc2R0hWMDhJdVhfeDNHLUFxbFJhdEZXblRrQ2trVGxzcWdfS2tOTFpUWjNzT3BNSUtsLTRZV0Mzd0Myd0k0ZHdXNXFua1NwRlJkbjM1SDIwV3htM082TVFiMkFjOWxwQUlUc1c2MC15N2lqdFE?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1405,42 +1405,42 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46086.39390046296</v>
+        <v>46086.42928240741</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Les attentats de Bruxelles : un avocat raconte de l’intérieur "le procès du siècle" - RTBF</t>
+          <t>Mondriaan sommeerde skaeve huse-adviseur kritiek terug te nemen onder dreiging van kort geding - De Limburger</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>The Brussels attacks: a lawyer tells the story of “the trial of the century” from the inside - RTBF</t>
+          <t>Mondriaan ordered Skaeve Huse advisor to take back criticism under threat of summary proceedings - De Limburger</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:44:58 GMT</t>
+          <t>Thu, 05 Mar 2026 20:15:00 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQRm5qeU1rVEVIelU3UWlRTjRfd05tN0FkS0dMMWxWdUpmVTE2cHRyRUJYMlVMd2Z4VXQ1elE5d1dXZzE1b2VkTlFUMmVnMVF1ZW93UGNSWFVTeEZCdnZyUktXR2hWcXI1cWFNRk1qdEpYRG1VdTFmSEhRTkdueUNrdWlsUGduNXJLSTFEY05CWXRuNDdnNTJIZWdxYVhPVlBzMnZtb3JtS2tEOTVKQWpvcVdtQ0dmblE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxPa3N3Snc4WVhFOGlOcHdmbWdIQ3ViN1RJRjE2VzJpczNqYk9QYXdfbWpqVmNsMGlxNmVTOGRXOWhFRGhEeVVzUEZ1azM0c0libUZOSlFyZi1JZDE0Yk9lbHVDc2RjemlubTR1WTlucUJnYThSQ0lxdklSaWhFUHdjcHpVbndkV2hFNzh4cUFwTllXcHBFLXQ5d1ZYbmxKZjRPNkVoSVBLbHdoQ3FlYTdncGtBNUs5QUFTVFB2RE9IdXVuY1dzZ3VrcE0xQ2VkY0lWRzRlREdiTHJfUWc1d0xEdHdn?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46086.57289351852</v>
+        <v>46086.84375</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Violence policière : Un homme décède dans un commissariat à Anvers - Bruxelles Dévie</t>
+          <t>Simulator in Brusselse Beurs laat je straatintimidatie door de ogen van een vrouw voelen - VRT</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Police violence: A man dies in a police station in Antwerp - Brussels Dévie</t>
+          <t>Simulator in Brussels Stock Exchange lets you feel street harassment through the eyes of a woman - VRT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:35:29 GMT</t>
+          <t>Fri, 06 Mar 2026 06:46:18 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPdTBXMGxpUkx1QmpoRlNSMFdDMXRYSnBndUVKWjl4V2lmU19ydW5aTGhLQW9OMU9hOFNOc0llZUd0OFU1RGhjV2haQjV4dHlmRmpRUm1MSWtRTE9oeDMwNkIzZTBHbnZ6UlZFTVJGWDVadmI2SFZ2UWM5SXAtbldPN1FzZExDRnYzblk3Z3NmdkFRTXVNcjdxbG5jRGxsbVRWdEhiMDZB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQeVl0ZVFCeUFqOEM1MFU4ekVhWDI5Q29iYXdRSXpyZHVCeTdIVjVrektHc2dLOW1hcFA1Yk9aTEo3WEFYdU1KdjdudFFKOWlIQ3FvcTFWcFVYM1dUZEJmOXBJUFpYbFpkcWt1eVl2Z3h3N1JsNlhTSlpKYXlHbGlaSklmV2huZ19KWl9LNGRtd3Zsdlp3SFBlUVlXTzk0XzdD?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46086.48297453704</v>
+        <v>46087.28215277778</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Le Facilitateur Marchés publics durables reprend du service - Bruxelles Environnement</t>
+          <t>Overleven­de van aanslag in metrostati­on Maalbeek ontmoet ‘man met het hoedje’: “Als je oog in oog staat, kan je de mens niet negeren” - HLN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>The Sustainable Public Procurement Facilitator is back in action - Brussels Environment</t>
+          <t>Survivor of attack in Maalbeek metro station meets 'man with the hat': “When you are face to face, you cannot ignore the person” - HLN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:12:19 GMT</t>
+          <t>Fri, 06 Mar 2026 06:59:50 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNSGdLRmRMY0pueC1PRUZnS1NGVF82Si1CeW8wVnpZeEY4T3A5VzJ6V2xncWRSMTZRemh3QjZkWXhBSnNkNm5EeXNOOVdRaUNQSG9UbG14WVZJTUhsUTJqOFNVeGIyZjhYdllQRXUtOEhKeks1UC1IUVFyZUhKNGp3alhkOWZSMmk4VnQ0eHRXOXBUR2tpXzE0LS1CbmM4OVlMNkd0aEZyYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxNTWlGV2dfLTlIYjVXS1Byc091SVUxSWc3VWttSS1KTld1ZGRsN1FtQWFXSFV4QUtqMGNBcEtuVVZlUjh1UFNxUlkxSXFxZ0Izc2hwZVRjSGNBMEk0LThwNlV2S1UyX25PaFo3Z0JoWDNTenNfb0ZPTV9rTm9XYmpZWDRIUmdfdW1LSmp2MUVFY1Z6dUZJNmd2WGNxamEyc0hlUjYzVEtpMDJUUnROdWJmMWVLUmxUQ3pXUlVyTXdpREI1c1pNWVdVdU9QY1lBazlyVWQ3SEZHVFE2TF9NcTJieUcyYjFIb1pzNXZOeE8zdi1TRjNFMlp5eUhQOA?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1570,42 +1570,42 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46086.46688657408</v>
+        <v>46087.29155092593</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>“Bruxelles, vous êtes prêts?”: Helena en concert privé, la Stib vous offre des places - 7sur7.be</t>
+          <t>'BouwBoost' moet meer betaalbare woningen opleveren: zoveel leegstaande bedrijfspanden telt Antwerpen - HLN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>“Brussels, are you ready?”: Helena in a private concert, the Stib offers you tickets - 7sur7.be</t>
+          <t>'BouwBoost' must deliver more affordable housing: there are so many vacant business premises in Antwerp - HLN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:49:00 GMT</t>
+          <t>Fri, 06 Mar 2026 07:31:45 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPajcxNDVjOTV5bUtNUnN3OGJjaVBlQmZIdnIybVVXdE9aSkh5N3NmWmhpQ0lFMmlLQzh6OHRJM1NDbHh2WTNyeUF6Y1Q2Y0VyWUhGWjIxZl9Fd3J4ejJNVC1iQ3M3U1pxR0h1QkZqdFV4bXpWZlFlb1AxNlh1Vm51SGpCbmQtUlJiU2haM0c4cjBHSmpzSHJOWUNTa2lOX3JPcHdkZlpBbjlmQ1J2Yi1PLU1ZdjN3OFZvNlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxOdnJvT3piSUQ0Q3RhelFYQzg5U1NzNE9wdGxWMVhHbkpxOWJZY2FnWFFxeXRQcGFvV1hOS20zMTI2SmphMDk4anNxQW13dm5haWtTWHBjSWNZcTVnbUpGNEEtdnl2Z3dtRkRCUi04R2xDZDNXbUZYUEFzbE1DeGotajlhSmVnVHFRVExCYnJZRk1KWjRVNi1hem5yNWxpQVpNNWtVamk4dXVjUW9vdjYzbURyak1rUjZjcTdwNHlZYzMyVkdEVS1GeHkySGloZW5JS2Q0?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1625,42 +1625,42 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46086.57569444444</v>
+        <v>46087.31371527778</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>"A Bruxelles, la menace est stable, mais haute, et extrêmement élevée à certains endroits" - La Libre.be</t>
+          <t>Politieagent redt man uit kanaal in Molenbeek: slachtoffer moet gereanimeerd worden - HLN</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>“In Brussels, the threat is stable, but high, and extremely high in certain places” - La Libre.be</t>
+          <t>Police officer rescues man from canal in Molenbeek: victim must be resuscitated - HLN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:02:00 GMT</t>
+          <t>Thu, 05 Mar 2026 16:33:12 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxOOGUxcWdPU2ZiSC1TMmJ3NVh4YklCa3JwdTE3XzJCWWVibzNiNS1ETGtxYUMxQ2dSN1VmbWJuajBnOU9nYkw3Tll0WVlvLTNibW9XMWw5dEhxcjFwSGMtVy1sazJKaE91SG43am5PYVhkRkprbWFEUFB4N3A5T3pGalEtWWdkeU1hbVllS3dYSHZUQmNDYmtMNldObXRlZU9jZGEzR2toV2hkNkh0UEdIN2tZS3dDeC0yX0VjcFRYdjF0dHVMUkpVdFprVGFtdzZYV0lELS1ITloyMXYtc3hvUkRDTUZodmwtMklGTmM1cUgxTEVjNjhF?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxON19odDlPTDZMTFgtUnZlS2I1UXRSSFY0dkxoYlBvYnM4bktJOW5Vd2dXbEhueWlXZjlfaGlSc0Y3cDRvR1JoLW1MNkstZWdVazFYdHc2ODFvZVpzMC0ybFlGLVFDOWRkanZXM1k4U0xLcWhjdWtValZPY0Z4RElwS3QzM1RoT1Vhc2trRGRQQ2Y2Q1FObVo1ZUktYUp1MjlTYkJGazBBdUZvTWdkMUxNNU5ka0VkZ0hvSW1v?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1680,42 +1680,42 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46086.41805555556</v>
+        <v>46086.68972222223</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Manifestation nationale du 12 mars: les aéroports de Bruxelles et Charleroi fortement perturbés - L'Echo</t>
+          <t>Centrum Jean Gol vecht uitsluiting van Brusselse Boekenbeurs aan voor de rechtbank - HLN</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>National demonstration on March 12: Brussels and Charleroi airports severely disrupted - L'Echo</t>
+          <t>Centrum Jean Gol challenges exclusion from the Brussels Book Fair in court - HLN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:29:51 GMT</t>
+          <t>Thu, 05 Mar 2026 17:07:58 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxQTWViYjY5SC1VVWxBV01DMVFaazU5Q2lEVnZRQXZ5Y29ITTl4M0U1N29Hb2s0UXcyaHBCbUpIMjhMaFB0bnlDZV9jUVVTdU1NZl9lOTZjT3l5ZUEyc1Q4WTdnNEh2bmMxbFoxaGw4TUJDSjcyTXNDaWtGdi0zXzNMTmJuYjY3UVQwdFVsQmJ2djdPSnpLeThad09VWEN1Y2UyRVJibmd0ZVVsamhYR2tybEVrZkYzRVEzMWduVkpDN2wzcmhXb2pIOU42Z1NCTVlqRGV5dmw5dU5TUEpzZTFjYUd2YnFJLXdaSnVGS0I0ZDAtY2xkXzVmLQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQZ2FYLTBWSDlvdnVGbEY2QjhMNUdmR2xRMHU1OE4xRVVoS3pZU1BxOGlCRUdXNnVYRjd3WnJaR19MRkhOUTlUMVNYczQ3SVZFVkFkdHhCc3QydEVMcHRPMHRQclpENTIzcG1ReEtqME1jZThjNWw0MlRDSk9JTVY3TlJEMG1Pci1HUVYyMHRxSDkwX0doRkxXek16NU03NFBVSVl4SVRmYUpITG5pZGUyU2pFNUY0ZXlJanZZ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1735,42 +1735,42 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46086.4790625</v>
+        <v>46086.71386574074</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bruxelles : 100 nouveaux kots pour les étudiants aux revenus modestes - Le Soir</t>
+          <t>Bromfiets vlucht weg voor politie tijdens controleactie - HLN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Brussels: 100 new kots for students with modest incomes - Le Soir</t>
+          <t>Moped flees from police during inspection - HLN</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:33:56 GMT</t>
+          <t>Thu, 05 Mar 2026 15:41:23 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNWkduYlNTYllkYWtoNW5EQkdmM0hVdi1jTzlYV1VSQUpoNVM0VDZSTDdxdEpiajdfUUFTQzRYSXhrWW90Q0x4Y1AwQ1hORjgwT2REMF9scXpTLTQtc09menc0LVJRblVKd3VRVWFScy05OFJ0QzUwamRQSVhucUY5U3Q3UXJrcGxBZmFoY3hncXhaeGUzX0RsaXZ5SVpfZUlfMG5Pb1A0eVFHeElYQmdCd3hFMm9DZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOT29PMkZtem9ORktTUXF6b29naHlGVy03bXJvOGVkcm1uTlFWbjdpVUFfRDZmV0QyejZOS3c3b3laTldQYmhTd2Z3endZNGhNd0JMc2JtbU55LTlhUU02cEJTWGcybzlvUWtGZ2pJdlhUR2dsWklGS1hxcE5JQThqWkVYajd3OTFzVjZXeGw1MERHWFkxVmlJZTl3?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1790,42 +1790,42 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46086.39856481482</v>
+        <v>46086.65373842593</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Inédit à Bruxelles: Auderghem s'associe à dix commerces, la STIB et la police contre le harcèlement de rue, "l'idée n'est pas de remplacer le 112" - L'Avenir</t>
+          <t>7-jarige Enzo verliest been na busongeval in Sint-Gillis - HLN</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Unprecedented in Brussels: Auderghem joins forces with ten businesses, the STIB and the police against street harassment, "the idea is not to replace 112" - L'Avenir</t>
+          <t>7-year-old Enzo loses leg after bus accident in Sint-Gillis - HLN</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:52:00 GMT</t>
+          <t>Thu, 05 Mar 2026 09:53:07 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgJBVV95cUxOb19pczBBYncyZU1kOGZweTRjaEtjVUVFX0FTZFAzcjZVRnA0S2dEdWFnZHJFdU9Wci04UzdvZG01VENzRVlybllBb1VDeWt3UVF6VG5meVNMQ3c5bVVfZHJsQjZJZGFkdnFpT3dOeHB6ZDZMeTlTNm1PVXpYMURjVUtZNE1FQkctS3FIREFmYjVkalpXRi1YblZvcHJOX1BqTktIS3BHdzlQMFRNQUc5OTFmdVZkWXNzNE5CQU01dVZab0pOYldhTmVqd2FSWWpOa3hQZUszUldwUnNMWS1acTRwakZubDNCaUZCWnpDTEhlMUdweFFlbW82ZU5hcFlTWTUwNHMwVVYxYmx2bzlqaFpxbE1ZUWd2c0F2QnJ2ZG1SaWhDb2Mzb0l2SVBKQ1JuVnFjcTZnSFdvZTVnN1NWb1NLeHprVFZ4WW5fM3h3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQQUxRNVFaYkM2dVN1NG56YWw4OHZaQnQ1aWJZRlp1cmNrbVpEM0ZQVlVsTWs0LV9yemctZkwxWmY1Yk1kWDM3ZGo4RGlmT1oyb19iUS1uY1FmYWFBT2FRRkZ6X1BmdmJlUERaQUdNNmNQYXVrdG1kTUlucExSR0J3d2NLYjBmaUFOalpmcGluUnFnbjRuZnFSNA?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1845,42 +1845,42 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46086.53611111111</v>
+        <v>46086.41188657407</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Rénovation durable du siège ING Marnix à Bruxelles avec Rockfon Mono Acoustic - Architectura</t>
+          <t>Dutch suspect denies firing gun that killed Antwerp girl, 11; Will fight extradition - NL Times</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sustainable renovation of the ING Marnix headquarters in Brussels with Rockfon Mono Acoustic - Architectura</t>
+          <t>Dutch suspect denies firing gun that killed Antwerp girl, 11; Will fight extradition - NL Times</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:52:29 GMT</t>
+          <t>Thu, 05 Mar 2026 18:30:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNenFFZjRYbFJiV0tsM1FGbDUwVkZqR3dGMGFZcEcybzJkVkE5SmdLNVhPTDJHei10TThRVFBfRnJOYWdRY09ydDRWSzN6a0FKSXRSZ1hvSjF2RVRfbzhzaVU2aTlGLUZaSVptNlJtVkg0cjF3aHNnUDNTcnM0a1NWMHBYUndjVlZBbVhMeGJqQ0V3SXJ6bG5HQVBRQmwxWWdzYjh0cUhlMlRmS05IZWdGZlJTLXlqR0V1M2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQR0V5WXBFM2Rfckp3d0xhd1dKYWVlcVNqTF9IeWROV0hrUzdlekM1SmtSSTN1NVYwd25TSlNxYzRrSWJHS3JzVmJMelRqaW4xSDVRNk1wcVpFVWI4dEh2aDgtUUc3ZlBVMVVvQjRyU3lCRkFrN1A0UUlubnpndHBZeldFREwxY3B4RGNHTnhQUUtNWU1kbFR1NXdTX1JxVk1LU2VLOGg2czZLVUk?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1900,42 +1900,42 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46086.53644675926</v>
+        <v>46086.77083333334</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Entre clubbing et jeu culte, ce show immersif de 3 heures à Bruxelles est l’expérience la plus électrique du moment à partager entre amis - Bruxelles Secrète</t>
+          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WKZO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Between clubbing and cult game, this 3-hour immersive show in Brussels is the most electric experience of the moment to share with friends - Bruxelles Secrète</t>
+          <t>Exclusive-NATO’s Rutte does not see need to invoke Art. 5 after missile incident - WKZO</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:01:08 GMT</t>
+          <t>Thu, 05 Mar 2026 12:58:54 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE04Y2dfVmtRMmZkMUV4VThJMjJTbWwwMEd5Tm5mc1gtT25VUEd4QjBzUVBZUjhVeWFsai02Q0R5eGFtNzN6YXp5cE4tNEp1akI3MnZRaktyUHZ2c0kzZXY1dE9LYWktX3pvcWtWNEFXZEc5ZkotVDV4QUFxTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxNM0FqSFEtMzdndE01OU1VandUNm04Um1fM2l1MWlfQzh0WlllWEY2dzNBYnJOdF9FSllVUW90R2Rjd0xfYllXaGhmZlBnTmEtVlVjcUFPcmNMOEhTYi03UFhrZlo0SEZKOV9iWmE2OUV5ZGZlV1ZZVmZzQ2ZqLVR2T3JZNWR0VHo5S252emwtVE5nY2dXMTFFOWxPR3ZqckRJZkF4SVlCRlBTWXc?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1955,42 +1955,42 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46086.4174537037</v>
+        <v>46086.54090277778</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Avec le printemps reviennent les Recyparks à Bruxelles - RTBF</t>
+          <t>‘Chinese Starbucks’ where you can buy a €1 coffee is coming to Brussels - The Brussels Times</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>With spring, the Recyparks return to Brussels - RTBF</t>
+          <t>‘Chinese Starbucks’ where you can buy a €1 coffee is coming to Brussels - The Brussels Times</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:44:32 GMT</t>
+          <t>Fri, 06 Mar 2026 05:07:55 GMT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNb3AxdENtVjFmVjJ2MG4wa0JITHdCT0JBSUVOcnFWeVJGTU5pOFlndmJqWFhSekpyWXMydHdwZ1hOeTBselRYem0zZld1UVd4YmdpRDNpMzNVYVFHRnlUTVhwYzkxSUhUOGdwUUhBMGJReWRBSmlOUDVRUTZuWWdtRlBURUxkT2VZSFlVNGh2TGZqM083VGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQT0xCRlFwRl9uV0t3alMwcVBmenFzcHEzdEFjRHRzUXR0eWlNeVdsWXJrMGRCc1JQdVFRT0hUNUlzelV5RXllODBsZktoZlZRczluLWZsMXJoM3RLeFZYRTF3bjBpSnRIb0J4eGVfcnlGaU1CcE9JS1Q0NjZRUGluN09uTjVUUUJqdXhBM2JIN2NqZURnd0t6UWVZV2V6WVhtSDQ1QXEyeGR3c3N2WHFKczdXd0hlemM?oc=5</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2010,42 +2010,42 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K29" s="1" t="n">
-        <v>46086.57259259259</v>
+        <v>46087.21383101852</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>L'enfant de 7 ans renversé par un bus TEC à Bruxelles est toujours en danger de mort - La Libre.be</t>
+          <t>Iranian regime “conservative”? Never, the mullahs are like 19th century Bolsheviks - Brussels Signal</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>The 7-year-old child hit by a TEC bus in Brussels is still in danger of death - La Libre.be</t>
+          <t>Iranian regime “conservative”? Never, the mullahs are like 19th century Bolsheviks - Brussels Signal</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:19:00 GMT</t>
+          <t>Thu, 05 Mar 2026 11:03:11 GMT</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxPekRWV2p3WERVU3hpUzR2c1BiRjc1amFMX2pwVmVMOTZ0MktFUVI5enpiQVZIdnBzVGE5RFNzR01LNVhwRXVyV2VLZWlRVzVtdUZfZi1hWE9CSVJ5WGlNNTFzUzRLU0JtckNkaDR0bUxtcUFZZVg3bERZS21JSTRnMDdqUlpnc0l2TUJVM2JGX3duak42NVc4WWtWY1pIVTJXTFBkWFc3RUozdFRtX1VjNmlxY1Zra1ZvcmpfbUQxQXUwN1hqc2FIWlB1cnN2cmRUSV80NDlwaDV5dkFFVHBnYnp3SjVwcUNxV3hfeHV0VUFsWXU1Nmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxOWWFncXVOemxxYm1qOXpycnVRQmRza0Y1NlByR0ZRY0ZQVmVBTlJoTEpoV1dxMENHekJVeE4ySWJSZXBvdTVZeFN1SVZVbERnLVBuZFV1R0syNHNEMThfamlVcUlZNnIzYXZsV185NXdINjhMU1VaWVg2YklRU2U4dXhERHRlMm9hWldXbWpZRVotNTZwUmpaQVFGWi1wM1I3bjlpNTJLQUY2NEpoaDNZU0RQNA?oc=5</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2065,42 +2065,42 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K30" s="1" t="n">
-        <v>46086.47152777778</v>
+        <v>46086.46054398148</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Le Centre Jean Gol conteste son exclusion de la Foire du livre de Bruxelles devant les tribunaux - Le Soir</t>
+          <t>NATO’s Rutte backs Macron’s nuclear revamp but says US umbrella is ultimate guarantee - The Straits Times</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>The Jean Gol Center challenges its exclusion from the Brussels Book Fair in court - Le Soir</t>
+          <t>NATO’s Rutte backs Macron’s nuclear revamp but says US umbrella is ultimate guarantee - The Straits Times</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:24:30 GMT</t>
+          <t>Thu, 05 Mar 2026 13:24:02 GMT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQdjQ1cUE0b2RpNlFweEJVWmlQaFV0clhDSU01ZExLQWZnbTc5NnFVUTdaMERUYjVDRUJuN282NzFCbmpJeW5IdEQ0cjgwRTFQZHZDdXdwLWtDdXRjcUY5ZVBBZDJHOS1WbnYzYkFaOUd5TTc3MnBKcVZBUjFYSWswdWQ0cGlfRVhlTzJzUTZ4ZHZJS0lMX2VUMWhUS2otQzJmRzJKdjRSc2luWmJRdHJKU1ZEdXFnZ1RVeUUwbVNNTjY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPaFRaS05qcUN5akFOdXlYTDdtQW5LSE9uMTQ0TUUwc3IxT3hkYmtPdW5PLWtYMGRhaGNCNy1qcFl2NWhJZkw1REljbVdoNTZEMlVtN3R2czE4Vi1GYmt5eEFzN1FmaW9FY0ZtNlBJSWdDdkNvYVhobkpwX3FRVnBfbXEyV01IZGUtQzVRQTBRM1FCNjZlZW81M3hkSHVCUUpRR3lHUlNfaENSTmNTS29aa3dpUXh5RngzNkc3Zm0tWGQ4VGhJUk8wUXNnUzFSaU1ldlE?oc=5</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2120,42 +2120,42 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K31" s="1" t="n">
-        <v>46086.55868055556</v>
+        <v>46086.55835648148</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Attaque contre l'Iran : La Défense rapatriera des Belges coincés aux Émirats arabes unis jusqu'à Bruxelles - BX1</t>
+          <t>Antony Blinken warns US can't sustain shooting down '$20,000 Iranian drones' with costly interceptors as markets, munition pressure builds - MSN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Attack on Iran: Defense will repatriate Belgians stuck in the United Arab Emirates to Brussels - BX1</t>
+          <t>Antony Blinken warns US can't sustain shooting down '$20,000 Iranian drones' with costly interceptors as markets, munition pressure builds - MSN</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:55:00 GMT</t>
+          <t>Fri, 06 Mar 2026 02:58:21 GMT</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxNWFlvLVl2eE9uZm10WV9XV1E3UjV0c2xpYmVOLTgtSzZhVHJNcWpKaG5uWXZFT09OeWNIZnRfVFZtVWRaekN4VDRraTFhN0Y4dnBJSUxlUFlEYkhIUkZMNUFhckJ6NU1RT3lramk1SXBkR1ZfdHp0WWEtWEROWmYwdVE1bkpMTk9FbGlsMWZQQW54X0IxLUVNcC00VDZJNHVlV1R3aXNsNXJEMnlZM3VQSk8xSmFXRGpQSF9hb0NFR1ZqV1pfOFFtV1FfemtvQ0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwJBVV95cUxPa1d5QUF1VUpDajQwWDM1ZXhBNFBBWDhXbUtBSmR4WDFrVkw2dl9wY3pDWmUzdkNtSXVuaUdlM0ZiQjlTeVhqRFhuZ053Yjd5Nm45aVgzYTBaZlJheFA0eFVFaVJNVENOSXREMnVSQXVkaTIxeFhOUWViaVYyblpkRG1reG54b1lXZlpOV29Mb2ZoU0NiTENCdUlPc0V6UUFOSjFIUjJKZVhBT2lYaHFZNU1nRE9OZVpqQ09GZzAxcWlNV1dabmFrbkt3amtDNVk2azBONFlOZmMtX1NzaUF3RHFISnhpUEhtTnJUMlE0b1JHbVlpZjhtbzBtcjA1elpZeWlMZ2JZNEYxOXg1Q1J1MVgyVnFMcXJ6aWZMcjl0eG9LVDlqZktSdmZKSjctbk1NdER0bHNjYw?oc=5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2175,42 +2175,42 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K32" s="1" t="n">
-        <v>46086.49652777778</v>
+        <v>46087.12385416667</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Médiathèque Nouvelle fera des adieux festifs au public lors d’un festival à Bruxelles - RTBF</t>
+          <t>French appeals court lowers charges against police officer facing trial for killing of teenager - The Straits Times</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Médiathèque Nouvelle will bid a festive farewell to the public during a festival in Brussels - RTBF</t>
+          <t>French appeals court lowers charges against police officer facing trial for killing of teenager - The Straits Times</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:04:31 GMT</t>
+          <t>Thu, 05 Mar 2026 12:39:02 GMT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNRGJhTnJGS0FxTWdVM3M1YmFNc2ZWU0lMUmVGZ0UtOWxyMGFzX1JMV1prMHMwZUZUajRidUlyMWpZWjE5R1VJZEhyYVlFVVVSUGVDbHdwWTlWZjQzTU8zSTVpNURQWE1QczJxUm1YT2dCT0cyTGtTZU9YVU45dmltZ3loRUttVGIybG5IRFV6TXdMTVhya2UyR2dvd0s0VzcxeGE0Z0JoOHQ0Z2IyUXZCU0UxUlBVMVZyNUZaY2xnZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxNWFlaQXR6UWFyUDVwVkdLaE42OENlcnNpb3lmZXhYeTdTQmtQUmRaMnVLcy1ETXVoQm1BVFBQTEdrQktpWnB4YnZRQkxYZHNGXzhtV3JjOHFtelVlcVZpck5HMXBIUm1pQVdzUEFqeEJtaHpKeElISDhyMFVhY005ZWFoN3ZWRnI0S3d6OVpmSHZnaHloZTBFbWt6RkhQaXZUOXlHN09mRHN3bDU2alFyd0o3MU81UHZIN0J4ZkFrSHZoSjhXbC1JZUR0RkZWbzd1WWw5QTczVHd6VmpJNUVqeVF3?oc=5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2230,42 +2230,42 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K33" s="1" t="n">
-        <v>46086.41980324074</v>
+        <v>46086.52710648148</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Les Best Brands Awards 2026 seront remis le 12 mars à Bruxelles - pub.be</t>
+          <t>Hristanov on the ITN action in the Ministry of Agriculture: A dirty and muddy war, whose main target is me - fakti.bg</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>The Best Brands Awards 2026 will be presented on March 12 in Brussels - pub.be</t>
+          <t>Hristanov on the ITN action in the Ministry of Agriculture: A dirty and muddy war, whose main target is me - fakti.bg</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:56:29 GMT</t>
+          <t>Thu, 05 Mar 2026 16:10:00 GMT</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPakg2RDFaQjJYc1NhUWJYNEdVWlhxZUthUXlGUGpGbzQ1eTd3amFIWHJMS0t4eTJIUTFmVngtT1pPTVZiT0tmckFoZzN0ZHFLYTByNXVfanFwbjUtVjhoSktXSDZhd0hqTVZKaU1XcjRQNmZqTzZZVk1MVGx6NkR6MU1aVU5hbUR2b2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxOb3NNdllQNmZUbjRpeElOdUczdm1WQTh1U0VpSFNETnF5OTVNQ3BHRHBVX2hodmtDR0djR2dfNllJeGMwN19GMVE5cDdkS3N5NEZIQUxhbjhSVjhYYVVBbDhrV0VoT0tUSVZQWHVvQWs5ekpVWVZObGQ1ODZ3ZFpKZVlDQ0JaamFra3R1aHl6eHBrSUEyZDBHcWpVZlozaVlkQmNqSURrUURxQUhTUzlFZ3ljdkhLYnYxSkU4ODYxd3hDYkxTRmRtSTFkMEE4dEhfVl8ydA?oc=5</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2285,42 +2285,42 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K34" s="1" t="n">
-        <v>46086.49755787037</v>
+        <v>46086.67361111111</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Le Centre Jean Gol accepte la main tendue par la Foire du livre - 7sur7.be</t>
+          <t>Highlights of NATO chief's interview with Reuters - The Straits Times</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>The Jean Gol Center accepts the hand extended by the Book Fair - 7sur7.be</t>
+          <t>Highlights of NATO chief's interview with Reuters - The Straits Times</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:15:00 GMT</t>
+          <t>Thu, 05 Mar 2026 13:34:14 GMT</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOYmhrWDJuQzdKVDJ5LTRpYWdfUDNETmZyVF9ZcjlkdHpsdmotTU1sV0RqNDJmS2sxTmZpRlkzR3d3VG5HSl95blRoNV85dk5lb3Z5RUNEaHQwWHlRTC0yYmhBT1prekU0TEhodG1jcHhpZ0k4UkVGSzQyVVZjbkMtcnVjbXZUcFhiQXlMWmxtd2o5ZHhjTXQ3al8yWkk4R01WYnhEQ1ZB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPTS04RHVLWjdNWW10NTdRM0V2ZUtvYnllbUJYSW9laTRoNmdvbWpqSXBnaGpfOWR3RHBjWXo2TGdzZXpKalB5YmxOWGtJWjJ5TzJBM0NoWTJXSlBVc21hVGlGbjB2MERwRkJ6UGJ5SzRaUWZWT0ZmZ25aeGJTMEZNeENVTXMyN1l1cDVTWTFzMnlmRGRmdmZFQXQ2b00xcldxejN3?oc=5</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2340,42 +2340,42 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K35" s="1" t="n">
-        <v>46086.59375</v>
+        <v>46086.56543981482</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>High Level City Belgium French (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Le Parc Ouest de Molenbeek demeurera accessible au public de manière permanente - RTBF</t>
+          <t>“La démocratie ne s’impose pas par les bombes”: manifestation à Bruxelles pour dénoncer la “guerre d’agression” contre l’Iran - 7sur7.be</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Molenbeek West Park will remain permanently accessible to the public - RTBF</t>
+          <t>“Democracy cannot be imposed by bombs”: demonstration in Brussels to denounce the “war of aggression” against Iran - 7sur7.be</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:48:32 GMT</t>
+          <t>Thu, 05 Mar 2026 21:02:00 GMT</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNUUNVOG55OEtBNXFkSTdWTHluaWpQeTUwUUpIWGlKYW12N0NNSUpxQVJQYTcxSGFMSmhZTDgxSlVYaV95MVpjeWs0cjlpaENuMDhBU3k4M2k0X0tMOFNzYkU5S2ZwenJfNG01bmRXUzQtc0dDRzludGhmWFdXMVZwNmkwMHZmdGxudTV4amdHQTdRampMU0hlWW0tcGpPMGRMd0p6Z25pc1FnTGNuNW8zUEFyMEVzZ00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQMFZCRXc2MnpLUDlGenZIb000SVd6eC1nSnZ4YVZwNkNrelN1TU1mRU9NZ3FDTUJwQTRXZmlLeUlOUGlVU3JNbzdFRHhLVDF0VjhvNDZhb2JpVWpPQVg1aklaWnQ3NEJQMWRoWndsZnJGMlBEN2NuU05CR3BIb1RPRXUtV2NPQmZjMHFvc0Z1YmlVNzhtRXdFV2dha3NrTVBNc21VOE5GMnF5Tm1HeS0zZlR0LUJ6eHdLTlhsMW1YWVhVTHlqTlc0bk5PS2ROX2xOODVhZGVmX3FJLWRiTGZtTngwcmh5Y0tBRE5Kakln?oc=5</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2399,38 +2399,38 @@
         </is>
       </c>
       <c r="K36" s="1" t="n">
-        <v>46086.49203703704</v>
+        <v>46086.87638888889</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Maasmechelaren worden online bevraagd over parkeren - HBVL</t>
+          <t>Face au retard et à l'explosion du budget, le projet de stade national de hockey à Uccle ne sera pas poursuivi - BX1</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Maasmechelen residents are asked online about parking - HBVL</t>
+          <t>Faced with the delay and the explosion of the budget, the national hockey stadium project in Uccle will not be continued - BX1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:07:01 GMT</t>
+          <t>Thu, 05 Mar 2026 14:03:00 GMT</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQUjY4UVB0MnZjN0hnUmhCTGF1RHNyMzlrVGk4Q2JvV0NGb2h6djZFRHd3NktaaW9nYmNOY2Q2V3UzY3FJM3RISXItenBrMEZ4ZVZhQURoVkZtRGpiVEo2WTl1VjZoUU8wT3ppV2ZGcjNuVlRoZW5WbXl6Nzl1ZWZJNHVfREpldW5oSXp3am1tMVd6OUE4Z3A2eFRsNVVITlh3NUxaS0FFOEFISkptSVBnd1h2aw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxNLXkxaU1WSE5WbkJ1cVNYbGhFXy11VkpRUjdnaGJlZkhxdnk1YmpjT2JTOHVySkNnN243UkpZT19rSDRmQmdGd0ZkeUdaM2JWS050b3BUWlpjS3RkV0FLNEhjemM5SlZGdFZzNldMdmstVEVla0ZfZ3NQTVdUYUN4bGRHZFdPUTlIS3NCQ1ljUnZmeE85X2hHVGM0d2VJWTh1RWNpVTAxWnZuVGZSN0x3ZXVlZm9KZkZndUx0TW5Nd1B3RlhKS3RNaklPZy1GQS1wbDNmLWxGbw?oc=5</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2450,17 +2450,17 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K37" s="1" t="n">
-        <v>46086.54653935185</v>
+        <v>46086.58541666667</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2470,22 +2470,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Theater over onze angst voor de dood komt naar CC Hasselt: “Voorstelling gaat uiteindelijk over de tijd die we nog hebben” - HLN</t>
+          <t>Jeux paralympiques 2026. « Je n’y serais pas allé » : Maxime Montaggioni réagit à la cérémonie d’ouverture sans athlète - Ouest-France</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Theater about our fear of death comes to CC Hasselt: “The performance is ultimately about the time we still have” - HLN</t>
+          <t>2026 Paralympic Games. “I wouldn’t have gone”: Maxime Montaggioni reacts to the opening ceremony without an athlete - Ouest-France</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:42:44 GMT</t>
+          <t>Fri, 06 Mar 2026 05:34:02 GMT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxNR0VjTmo2b2hjTGVEZDJDamwxTlo0ckVBNGVuSEltVEFQUTlibzhrNTJkSUhnR2poVGhCRjZOQXJ3WDZFaVIzcGhsdHc2SHZrQWhlNFpNV29yZWI2RDZhb0VNOVF6dV9YMDBKWDFlQmZ3Q1BfMFRYbU40a2xfVXpKUVdCZ3lmaU0xZVlxeGh5eXdDUzJOckxEYk9GeHBhSW5aekRWdXFGQTNpbnltZFFIWVRWT0RyWkNxSERFRzBPR1o0WVNVblJFemFtbTNYYU9PbkZxQjJSbDZ2djE1SmhaSGx3SDJKV0t4aEZULQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwJBVV95cUxNcHFOLVZ3VElQa2s0UXRnTFRaeS1ERkl2dlpBcmwyVTE3SGo5M3h0Y2NzQWJyazFkaUdYR0FXSlFNVTR6RzlvR1B6ako4VzFHNUxFeFdRMzRpdEFtbkVEWHhwQkx3WVc0MGN1amtQTF9SV1JYb3FRNTRrVkwtVUw4THpTVFloWDVrZlVxYnNnVDNJZlVudVhVNGtTWWFTY29SSUt5OV9rWjhIRkVrYTlhSVRsS0RHN0lHNF9PQ1JNRW5SOHEtSkxsdzc0aDZCemM0NXdvdWo5Q2haYVp4a0dWZHMtUjVqQlZiTTMtdDFBVml1S3E4NFJic1pHcm9mMDZ6XzlRU19BQkhuX1MwS183R3dKUGZDQzd3SXhN?oc=5</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2505,17 +2505,17 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K38" s="1" t="n">
-        <v>46086.61300925926</v>
+        <v>46087.23196759259</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2525,22 +2525,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Filmopnames met Charlotte Timmers voor nieuwe “spannende fictiereeks” in Hasselt - Nieuwsblad</t>
+          <t>Futsal Benfica Auderghem - Anderlecht</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Filming with Charlotte Timmers for new “exciting fiction series” in Hasselt - Nieuwsblad</t>
+          <t>Futsal Benfica Auderghem - Anderlecht</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:52:50 GMT</t>
+          <t>Thu, 05 Mar 2026 14:09:11 GMT</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxOU0c4QlVSb1p4TzhubGwyWDZqYkZRZEtrMmZCSmliS3g5ZDZYS3pyay1LNFZpRENKZ2E2Z2pSR3IxRThONmg5RDlEUk1sNy1MeHdDRUdLRHY2ODRUZFdRSVdISzZfd2drMjBDai1wb2o1QlhuQ0JMUFpDS0I2djhBZUE4M0piam1aODc4SndLUzhFWlBGRHlnaktPZ1czWnJTZkNKOU1DR3oxcDhlOFdDc0ZRbjltNjMwRTZxaTVRWFNfTEU1T2hKV1RsMG94ajA2Sk94bDcwQkY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE5scURuclV0anR4NDRjYWFCWU9Ea0wtSG9JYTNEdTU5Z2NxdTlpQ2Zjcl9XOGRLZEFFcTVhVHZxTzdiUDVoeFpYaUZfWS1ZNFdKcFE?oc=5</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2560,17 +2560,17 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K39" s="1" t="n">
-        <v>46086.57835648148</v>
+        <v>46086.58971064815</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2580,22 +2580,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Grandbrothers verenigen klassiek en elektronisch in Brussel en Hasselt - whathappens.be</t>
+          <t>"Panique et peur" : les prisonniers politiques iraniens sous le feu des bombes israélo-américaines - France 24</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Grandbrothers unite classical and electronic in Brussels and Hasselt - whathappens.be</t>
+          <t>“Panic and fear”: Iranian political prisoners under fire from Israeli-American bombs - France 24</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:29:52 GMT</t>
+          <t>Thu, 05 Mar 2026 17:51:50 GMT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOdWJwR01POUpWUDlVMXFpM05EMlRTdlBEYXNDV2NPOHctc1pKR2I3M0tLemYyRHhBYmFmck42ODBsU09pbzRqaE9kNXZSOG9LM0pTRVlRREN1bW10WXk4V3R2NXZSNlRFUFNueUlZREdBMUl2OThNYU04X3NrbjZJczlubEJ2VDdKdTdjUkxSeTFCOTVGaFlMOEFIczA5UzJfeEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPQ0Jad1J6Z212Z1psd3ZsZmFRVG5VV3NpMjVDWjlVTy14U2NIRVgwa1NiTU9STTNzS0JiTW9YdG91d3JwLWtyNnRLMUJpVkdfYU5qZWNJMlQ2RXQ5M1pLQzNiNzZZNUdDNzEybW9vMEkxUmlZR29xblBHUm8zamE1WWdhM21UWTJ4VnZIdjZFRmhBcWJKNzhiNTY5bnRTVGUxOE1BQ0phYVN4MUVHZW16d2NuTEk2LXVhMlhkTFRvX1VRdzJQMWhfQTJXVXp4d1NRU0FuX3ByY2VBaUlJTll5S3VieHlYNXh4R2Vubg?oc=5</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2615,17 +2615,17 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K40" s="1" t="n">
-        <v>46086.39574074074</v>
+        <v>46086.7443287037</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Maasmechelen French (fallback)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2635,22 +2635,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>RESTOTIP. Gezellig tafelen tussen de bedrijven bij Het Cordaat op de Corda Campus in Hasselt - HLN</t>
+          <t>À León, vivre l’Europe autrement : une mobilité EURECA-PRO au cœur de l’Espagne - Université de Lorraine</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>RESTORATION TIP. Pleasant dining between the companies at Het Cordaat on the Corda Campus in Hasselt - HLN</t>
+          <t>In León, experience Europe differently: EURECA-PRO mobility in the heart of Spain - University of Lorraine</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:03:19 GMT</t>
+          <t>Fri, 06 Mar 2026 07:04:28 GMT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQNURtcTYxd0E1ZU93alAtNUNMYVozS1pqTl9JdzMzZU0zUkdkVEtBeWNPM2F0d2Fzclc2UktPUXVpSTVTWkxFRUhadHNhbDNpaUo2NUVkdnVIWmNsV2hucVNtMjI2RVl6Rk0zNXNDVmtsX3FMOVJDRmNkN2NzU2pzb1NRdFdSQXFYb1BDVFhGRHhDZWZRc05KdVFSYXgzYzJvNVZweHRsR1k5cXFERG1uNjNCcmh2R2JFTGNpNEpaME5zcVVXcW5z?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQdURSV1JodjJHTkx5VnRNNkhKZ3prQmUtbXVTcFgtUlVnSHM1VjFEUkVJanFWRjBhZ2dOTlE2bGdLTTRkY3QwYXlMY0dvNE83aDFHbWhuSWl5Qk5pUzFiZ3JkdlRsZ0RXVUJfVDFlWDdHVTB5NWZNN2pCVVFyUy1obDdKUTU5OWp5WGxVYUlFS3FQcEd2YnRha08wNGR2TUp6OHVhY1VVX1VhaEhFdERXM0JhN0VrU2RG?oc=5</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2670,42 +2670,42 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K41" s="1" t="n">
-        <v>46086.4189699074</v>
+        <v>46087.29476851852</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>OPROEP: Zit jij morgen op repatriëringsvlucht vanuit het Midden-Oosten? - HBVL</t>
+          <t>Pressemeldungen des Polizeipräsidiums Unterfranken vom 05.03.2026 - Polizei Bayern</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>CALL: Are you on a repatriation flight from the Middle East tomorrow? - HBVL</t>
+          <t>Press releases from the Lower Franconia Police Headquarters from March 5th, 2026 - Bavaria Police</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:53:20 GMT</t>
+          <t>Thu, 05 Mar 2026 19:39:06 GMT</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPSXh5ejNOS1Z3STRIM2lvcnk1QVFTZmNHSlJhQjJ4aTRTVmRZMnNXVXdaLWtWZWhXUFZnUWdZTm5qWE9KMWlMOWdYeHdaUHQ0eUUtcDNtQ1ZCWGtlTDJ6STY0S25WdHNmZm9mQ3lpQzV2QzVobTFTcktUaG9xWjNJSk9fVVFYaE13WDNwUFhBcHBxamk4ZjRCVms3YlRaN1VtbkhucWR1NHkyMzBad2lIdkJCU0ZqUUxSSUVaUXdMMEl6M1hT?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNQ1NITk0yV3NhWm53dEx4eDBjQXU5N2NKckJfeFZEcXlybjYwbk01dFcwSW80eFctUzFadlNxYUhZRUNNaW5FNm9ITFF2bHRBX3owNnVaa1MtLXR3a21lUnh3Z21QRXdHUEM0WEV3VS1Qc1I5Z3h6eFlGdFEyUzdpa0hB?oc=5</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2715,52 +2715,52 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K42" s="1" t="n">
-        <v>46086.5787037037</v>
+        <v>46086.81881944444</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Niemand draaide voor Genkenaar Aron in ‘The voice’, maar nu mag hij optreden op Het Schlagerfestival - Nieuwsblad</t>
+          <t>Einsatz von Polizei und Feuerwehr am Hauptbahnhof in Würzburg: Das steckt dahinter - Main-Post</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Nobody played for Genkenaar Aron in 'The voice', but now he can perform at the Schlagerfestival - Nieuwsblad</t>
+          <t>Deployment of the police and fire brigade at the main train station in Würzburg: That's what's behind it - Main-Post</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:00:00 GMT</t>
+          <t>Thu, 05 Mar 2026 14:30:00 GMT</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQN1NCWUFhWDE3VlY0V1g4OUNxcHRVaV9kOXk2bVdBU2JrYTBOcUJrNUlON21WM1h3eXZ2NEVQUVBXWkI0UGwxZ0JyM3FDNnFuckdQZ0RibVVGajlNSi1MUjVIUDZWWkx4RTRCTF9ZWGJBUGl2XzhLd0xHODdYMGs4N1NDMTBiLWZUZDdWbEhWUnQ0ekxyd3NBdXlSQXRQOE5LTEFLRW5pVmVldzdaM1hjX1Qtd0ZreDFORjR4YTNQRzNmVThpdEdNeFNrSWRrNEp5QUxXMFBmUzhaVmxFemVvaE5pcDFWQWQ5V0IzbUpn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxNYkdBVUxTOWF6bzYwenRRN01oVXNFNE5DR0hXeVZzalpxOC1tdnM1dG1RT0JZRnFvdDV2QlY2bm84MzZTUWFvR0MzNHBPQ29sN0hZVWlqRjBfTHB0UnBEOTJYaFBieFlyQ3NKYTA5OTVNNzdvV2wzcUhYY1pKTWZWTjFPbHBUY1BucXJzZXo2ZUFYS2pZbmVjWWNVWkZEdTl3S3dRX0VsVkhTVkxpbmVKVkJhN3NGdFF6T2c?oc=5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2770,52 +2770,52 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K43" s="1" t="n">
-        <v>46086.5</v>
+        <v>46086.60416666666</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Zestiger lichtgewond na botsing in Tongeren - HBVL</t>
+          <t>Nach schwerer Attacke auf Mann in Waldaschaff: Polizei sucht nach mutmaßlicher Tatwaffe | Foto: Stephanie Renger - main-echo.de</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Sixty-something slightly injured after collision in Tongeren - HBVL</t>
+          <t>After a serious attack on a man in Waldaschaff: Police search for suspected murder weapon | Photo: Stephanie Renger - main-echo.de</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:42:58 GMT</t>
+          <t>Thu, 05 Mar 2026 11:08:46 GMT</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNUjhnZ1pBc3VTQkFvbDJDWlU2aGgzWEJtS3dQQVZaQ0NsbE03ckcyU1JXcnJ5NVZhWG12ZTk3VnZtZEpoQU5vd1J0THBodXlub3o2a0R0MGJJTTUtblhoY21nbXZVX0NqUXNCVHBvR3o5dFV2WUhvSVVnQWlPaVpJd2I0dlkyekdHc2ZkOVptUzRJQUdpajNUQlBCLVBVem4xNEFJTVZ6WjJkVFBQbkl3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2wFBVV95cUxPaDJ2TlE2U0ZLVURRWjZfaEdCZTd0OE1pZGI4WUs2YXg3NVQyeDkxNjdIYTFRLUhacWxJZUhHdzF5alJDbGltNUdwSFpfLWNMb2NWSDBJMEFqUGZPd1lKcWNFVjFTSEFfSGZ5aUxIVWM1VWVMaHMyVGx5QjhPdVphRnUxTnQzSGJEM0djcVJFUlJhU2lwb3JVV0x3emxJZ0o1V2JRWWFpRmRGaVBGR3VDanRuYjc2a3FkZ09ISHJ2TVlSY0ZERGo0RVVnUURVQllrSlpwTl9QYVJfVEk?oc=5</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2825,52 +2825,52 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K44" s="1" t="n">
-        <v>46086.57150462963</v>
+        <v>46086.4644212963</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Na horrorcrash met 160 km/u doet topwaterskiër Tim Lisens voor het eerst verhaal: “Mijn hoofd zat alleen nog vast dankzij mijn wervelkolom” - HLN</t>
+          <t>Mellrichstadt: Polizei nimmt falsche Spendensammler fest - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>After a horror crash at 160 km/h, top water skier Tim Lisens tells his story for the first time: “My head was only stuck thanks to my spine” - HLN</t>
+          <t>Mellrichstadt: Police arrest fake fundraisers - Radio Gong Würzburg</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:28:14 GMT</t>
+          <t>Thu, 05 Mar 2026 17:00:00 GMT</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwJBVV95cUxQSVI3MzBISm1mWHdRNzJJam1FTVBITjBpX0VCRDNmQ2RRNVl0RVVwbG5ZeTJLWjBva1FmSXRPdXhSSHV4c2p1cmpoT3dfQTNqenVheXZSUkJndEdXTEhUQW9EQlZkbmpYUDRWYWRXVmNtbDlzZC1oVGtBaWN0ekhFVzljWHhZTm54Yk05U2VJcnAtMUFkM2U0Qy1aX0NpV0JZR1NiOVhDb1Q3c2VrT3AtWXRUekw4YVMyYmlEQnhYSXNDQkw2VE1fazN5YnBoT0FSdUxEYjBod3o1UmNtNzJiblFjcVZxTlp4WHFJY0N6bmNDY013OER4eHNCM25IbjQyMGZ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQNVpjWXJISUZrLS1kaVU1UzVKV3Y3RVJhZ2wyOVRmOEwzaVB2QkhqMnRRVWpYNldnam1iUlRoel84YWpZZGRXdHktc3B1dmNqcHZncWNlY0hpRDJuRzAtbWlPNENJU1FDSmZ0anJPcEtZajIwVl90TU9JUXlVZnFESHgxaE03a1JzaEcwYTNzenVmRjQ?oc=5</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2880,52 +2880,52 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K45" s="1" t="n">
-        <v>46086.56127314815</v>
+        <v>46086.70833333334</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Wertheim German</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Dertiger lokt meisje (11) op spelplatform Roblox en vraagt naaktbeelden in ruil voor virtueel geld - HBVL</t>
+          <t>Blitzer in Blankenbach aktuell am Donnerstag: Hier nimmt die Polizei am 05.03.2026 Raser ins Visier - News.de</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Thirty-something lures girl (11) to gaming platform Roblox and asks for nude images in exchange for virtual money - HBVL</t>
+          <t>Speed ​​cameras in Blankenbach currently on Thursday: Here the police are targeting speeders on March 5th, 2026 - News.de</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:47:18 GMT</t>
+          <t>Thu, 05 Mar 2026 13:15:39 GMT</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxQR1BXTWZLVUpBenZ2REFtOVowekVzOEEyOTc1bmk1NGl2ZXhUUmFFeG1hUFlETk1LM2pvOVRTXy14ZzA4c2RwUmNJTWRrRktkVGVmdm5UWTBaY1pCYlJyckt5bGtmSG9qcGZIT3BQdUFmbWtGOXBPZTFSYTBlN2pYUkRuVjMwV2JjTHBwMWE2RFZLZFU4UkZ2aG1ETG4zTkVaOG1Vd2NvdFdmQnZCREUxWTFkLTNnQVlpMEJxR09YdkdYVDZ0LW1JY0czVFEyeS1lT01TOFV1WVpxanBMQWRIMkN2bXJtdjhyd1AyRVJPUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwJBVV95cUxNT3dZVW1WQzJkMWU4NV9lNTdWT3ZKdjhQWlJVSi1FSXZianZmYVpHUWZKMWx3LVVUSnFXSWlEUmJHREJLdVV4UVRoSUtSS3JfSUpLdGRwUHhsZ1J1bF9uVlQ4UEVYVE0zSTB1bzJJWnZYcm43T2p4LTdQekg1Vk9jaUJfVFItNGZYZkVycFZhT3h5UjBudkJYSmxMZDFYLThvVGFZLWtOOXFtVnRqOVVpVzNWTmlqSWhtQjBhamZXSUw2TUpmLXQ0eGRGaDQzYmtyRzhhQVlhaUpJVEZiRk5rQ2NKc0s4Y1ljWUw4TFVvMHhzMkhNT2QxNDZfYUtLTm4xZzFpT0xDSkI3bGQ5cXhTb0ZnSHdiUW_SAZwCQVVfeXFMTWgybGRuOHJFRHpxcWVON0NYZW9NSjdFY1phYV9mZm84NDFpcGF6Nk1tY3hNS0ZXb1JtNzNGOTdhMUpxeDRMQUR5akdOZUVKMU5FOTE4MWRJYXlWRXgxM0dKTDJabVBpdGk3aF9DVkJDZmRtV2dELUZSbWtaOGRCNDVLZWxmS284T3RGcGoyR2c1U0ZpZnNoMEduUmZLOHRweFFFTWJ1ZE9wQjh1NVVZTXM4dGRNTjIxaFFMTkQ0N2UwTk5Pd0RkWUJkMVVZV2N1T0hQQmRqZ0VzOHBkajU5d0hvYnczSkFMRjRmcTlPUUVEVFhHb1Jwb2dpUVhnS1c0cjREX3ZQdktKMVNDdlJ2NlJ1LUgtMDJGNEVkOFQ?oc=5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2935,52 +2935,52 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K46" s="1" t="n">
-        <v>46086.49118055555</v>
+        <v>46086.55253472222</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ontvoerder van 13-jarige tiener uit Genk werd voor zijn assisenproces maar liefst vier keer uit het verkeer geplukt voor gevaarlijk rijgedrag: “Ik gebruik geen drugs, mevrouw” - HLN</t>
+          <t>Opinion | Of Course Trump Bombed Iran - The New York Times</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Kidnapper of a 13-year-old teenager from Genk was picked up from traffic no fewer than four times before his assize trial for dangerous driving: “I don't use drugs, madam” - HLN</t>
+          <t>Opinion | Of Course Trump Bombed Iran - The New York Times</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:53:20 GMT</t>
+          <t>Thu, 05 Mar 2026 10:03:00 GMT</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgJBVV95cUxNYnVMZFRaSXRiOXBFdGlyeDBUUHFkYUJ5Z0ZZanlUWDdaTkFLdXRpWE8xUVFGOWhkX3BYNGp6a2NpbVlGNnZDNkY3ckxzUlM5aHAyWFNoZ05NTktuUUNHQktQUjZiWXBQaGJBcG1jdFFTZHlQdkdkOFp5QkFKZ2RvbFNfOTFRVW92U3V0Uk9zczhqRnlsR2JxdkhKbEQ1ekp0RVpzRUZFbE1LX2FaamZ2a1hDbXdLdF9fY0s2YmtHVmlFN0dEMXpNTzhvQVQ1RnBTWllMaC1LRVpjYjFJVHNFdXVfWHMyZTRFQ24wSXVqSUhRZ3h3blJRcGtIM3hXU1pGRkMyaDNkYlZneGo4NUg3bkV0MjNXallTS0E3WS1pMm5ScklnQThrdVhhYXQydlVWdWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxNbmhEOW1POGNRa3YxZXAwb2Y1dzVzNW1NWW5VUWp6MGxPdEZMS1l5RGo5c1JISHNNYlFaY1kyS1p3VjFKam5hRWpMV1NuU1hVcm4wTTNLTlhhRG8tcy04cko2TnlHc1FIbzJ5WTl1ZHVCTkRvbTBKNVhHczhpX3pHWEcwQQ?oc=5</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2990,52 +2990,52 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K47" s="1" t="n">
-        <v>46086.49537037037</v>
+        <v>46086.41875</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Nieuw skatepark in Sint-Lambrechts-Herk officieel geopend: “Toegankelijk voor beginners, uitdagend voor ervaren skaters” - HLN</t>
+          <t>FIU Medicine Earns Full LCME Accreditation Through 2033 - FIU Herbert Wertheim College of Medicine</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>New skate park in Sint-Lambrechts-Herk officially opened: “Accessible for beginners, challenging for experienced skaters” - HLN</t>
+          <t>FIU Medicine Earns Full LCME Accreditation Through 2033 - FIU Herbert Wertheim College of Medicine</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:28:19 GMT</t>
+          <t>Thu, 05 Mar 2026 15:27:30 GMT</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxOUXU3Qlc4ajRYM2pYTngwMHV5aDIwQ21aU2xYSkIxWnpRWUluM2FCc3VaQ0E1UDJ2Ukhyc1ZBbmQ2dl9LZVE2UzN1ME03ZExFS01HOE0tVF9fRy1WQkVwNUFMdXNEbXFzbmF0UHVhR0R4Z2Rrc0p4Z3FQY1pxVFl1SGVWbnhkbzRjeEFjTnozdVQ0dGZ0R0o5ZVJaekxjdlFfWEtvME1NMS1xODBqQXBXRmRlaGZKVmIxaXpXeHZCWHQxXzRfY09FNkZkZnlCdWZjMy1FTUtEaERuUHNjZ1dZSXlrWHNsbVBv?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPaV9PT2tESnE4NVdQZTdxVkt4RTg5T2dmUHQ3cDBsUnRTSWZfSWxsUDZrYkFWcUt1RVpsak9hTVYyaldJMjljQm8tQ2JKM1RCS096ZDVKN0d6MkNjRm9penNFRDZ6Q3VoZEdBRlZxYzN0SUs1YWlMMUR5R2J4N1RYNFNXMUVoRVJyZGtIdzdSRGROMmpfalRvNUdtUm1UZnJNTVE?oc=5</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3045,52 +3045,52 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K48" s="1" t="n">
-        <v>46086.43633101852</v>
+        <v>46086.64409722222</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Village Wertheim (fallback)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Nieuw postgraduaat bij PXL: “Directe impact op miljarden aan publieke middelen” - HBVL</t>
+          <t>Government lists Hizb ut-Tahrir as banned hate group - The Australian Jewish News</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>New postgraduate degree at PXL: “Direct impact on billions in public resources” - HBVL</t>
+          <t>Government lists Hizb ut-Tahrir as banned hate group - The Australian Jewish News</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:42:36 GMT</t>
+          <t>Thu, 05 Mar 2026 22:36:59 GMT</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPRUdyV1F6VUExZi0zZGliejJLWXQwR0FjX2NSc1ZhcThtY0ViT21VMzA1bXY5RkFGZ19IZ2tPQkxydjZ4dFkteG1rTHprX2g4VmtiUXpTTEgzM3JyTHZER3kzTUd0TF9ZRmNiR3ZnODhzNGMzYXBOMHl3anNnS0I5ZDFDZ2FQaFRWTVdJdG83WFVoYkNMMjZwZVphZkN3TXFSUnkzaWlNNFg2YWtqZl9mcG9HbzhuazdmWEFLeHBJZXhkYV8xMjZQWklYbUlMZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPNWpUdWdpZEJfdEZFZW1xYXBYRjJHMEJId3lkU1E0cnZjVTFOOHlrbnRlcDNfdWFXLU9zZVZXVnpnaWJKUzM5eFFBMUtOdWdUVWM1TGdfZ3ZOdGtYdWZ5a3FtSU52cXgySEFNWXVESzVRcXJZYWFwYkxvejZXYVpLRlhWWWxuLV9mZVdyN1NabVQzMFJsVkRRWHBR0gGfAUFVX3lxTE9NMlVoTWxBbWRINW9WMlVnU0xLcHQzMy10eUlha3FoZWFxQXZ5dVFJR0o0c1VEU3I0Z2pwUGtoV05LVGxmOVYzVnd5MnJlV3VUWkVDRjc3elUtYkp1ZUVhLUhRbU1ka0FPUGsxTFVRTjh0eDVBQXR1ZEF0M0Z4U0hCbmhXeWsyNF9uV1pucGk4UVJSSXYzSXo2Z1NDT1lZNA?oc=5</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3100,52 +3100,52 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K49" s="1" t="n">
-        <v>46086.52958333334</v>
+        <v>46086.94234953704</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Obligatiehouders vangen bot in Triamant-zaak: rechter wijst eis van 16 miljoen euro af - HLN</t>
+          <t>1,6 Promille: Polizei stoppt Autofahrer auf Münchner Straße - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Bondholders are caught in the Triamant case: judge rejects demand for 16 million euros - HLN</t>
+          <t>1.6 per mille: Police stop drivers on Münchner Straße - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:31:07 GMT</t>
+          <t>Fri, 06 Mar 2026 07:09:38 GMT</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOenl6dm0tQjZodVlvUVJHRFNoUE1HSXJoSHZUMEM4ZkJpUHBvM2kxa0ozMnh4a19OMVJkUEdsSzhvUlN3bVVlTFV6ZEw4X2VMLXgyVGtPQ1VpTXR1OXFpTTN0Rm5rM3NWZ3JtZDQ1WHBDY1l4eFQycW5KY3RLY1F3emVBNFpuQktjTThXLTZyOVljamJMZFI4MG83bnZ0VVFHVlVvSUsxQmY5Rm03bnQ3YXc5QWlhLWpNOTVZZUZvMA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOS2VjakpKWkFXaW84T043bWJBSHFSNDlZX3BTTUYtU2Vfb3JUQnZlTVFFeDRHRFNJcEJhVGw3OFphaUg5eWNLTUtmUlZ2M0xBQWVwQ3ZtNXVTSDU5djVpWWo3QTFTVWpIenE5MGtmS0NndWFRejVLQTJLTEZKWlY3QVVjUFdiaFEybHFhZ3N5NWZ3S0JBQjJGejVqeVgxdHMwUFZiZWtSTjBtYi1iLVVSQzJEemdxUTh5MlVETDctTUZtV0RDTUo1RmJGaw?oc=5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3155,52 +3155,52 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K50" s="1" t="n">
-        <v>46086.3966087963</v>
+        <v>46087.29835648148</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Marie-Joël Kessen, 64 jaar - HBVL</t>
+          <t>Schüler gegen Wehrpflicht: Auch in Ingolstadt wollen Schüler heute demonstriereren - HITRADIO RT1</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Marie-Joël Kessen, 64 years old - HBVL</t>
+          <t>Students against conscription: Students also want to demonstrate in Ingolstadt today - HITRADIO RT1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:02:57 GMT</t>
+          <t>Thu, 05 Mar 2026 09:34:00 GMT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxORnpMTHYtWTN4YnFrU1B3dkh0TkV0cllraW1nY053czlPRzFObThaQS1JcTB3cktiN0R2a3hpX3RBeWltMGlFWVpnQURaWDMzbl92VUZNMkp4ODBPSG41NmFNZlhMOGp4dm0tdTAtTG0wNE9JLURzc1pJSzNkd0ZFa2xmUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOT0dXeC0yU2RmcTNoWDM2dWJzZ0doZHN3OTNFSXNPWlF6YW84VGVWX1Vob2ptVXdVcGVLQ29GaUJjOWdaQllpYU1IYU9Ia3hiNWVGYjA4RUR2SGx2NUh3Nll6Z01JVlI2MTg3U0dXS1hZSEZxbHJnYXdyZ2dRX0duamF0RTQyaWU1SDY5WGcxT2FseFQ4TzlaRkdvaUttN3pCR0ppeGRid21PSUxMcjY5ek5Qb3psUQ?oc=5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3210,52 +3210,52 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K51" s="1" t="n">
-        <v>46086.41871527778</v>
+        <v>46086.39861111111</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Zware klap tussen twee auto’s op N74 in Zonhoven - HBVL</t>
+          <t>Ingolstadt: Unbekannte brechen in Golf-Club ein und flüchten mit Golf-Mobil - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Heavy impact between two cars on N74 in Zonhoven - HBVL</t>
+          <t>Ingolstadt: Unknown people break into the golf club and escape in a golf cart - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:54:25 GMT</t>
+          <t>Thu, 05 Mar 2026 11:52:22 GMT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQUUdXNUV2OEJCREs1MkpwMTVsLUplVWxRVTh5X05xVmFUZXRfR1ZJeWU4MVVjU2hVel9UUjdPbjlpUW5RNFZ0amlmVzh0YmFrZXJiWGhISFpHLVhLeVpveVd6aS1SeC0yc1lKQXRnSjVIb2Y3VWVGV1ZzZEd2U0tuUzNZa2lTaGFRSTJiUXdPRWpkVGh6bXQ5NTVEcVFJWHhNMU8wNFBqWjY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTFBudV94ay1OLWFZclZ4QkUxX1IwczJvN1NQQ0wxWDd4N3lIS2o4akd0cHRWVm5uZ19zeEhsTWhyT0tpOFQzeHNxNlRzWE5tbjVicHhjTml1N1NnMm1wbG9kM3pLR19hTWlSb2VZaHJR?oc=5</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3265,52 +3265,52 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K52" s="1" t="n">
-        <v>46086.49612268519</v>
+        <v>46086.49469907407</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>107 obligatiehouders vroegen samen 16 miljoen euro na faillissement Triamant, maar krijgen ongelijk: geen schadevergoeding en zélf opdraaien voor kosten - HLN</t>
+          <t>30-Jähriger aus Manching verletzt sich bei Moped-Unglück in Ingolstadt - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>107 bondholders together asked for 16 million euros after Triamant bankruptcy, but were wrong: no compensation and had to pay costs themselves - HLN</t>
+          <t>30-year-old from Manching is injured in a moped accident in Ingolstadt - Pfaffenhofen Today</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:19:59 GMT</t>
+          <t>Thu, 05 Mar 2026 13:25:11 GMT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgJBVV95cUxOQXlsb3RhUHhjR0JoZDNnNnY1eE9LZk4zWjNoaFI3dm41dWt3MjFmdGUxT3Fzd0lUYnNrWlVsZ3FQcF9aMHVtM3FjSmUtM3hNRGVPV3kxbDhTU1ZKd3M1NnY3Q2k5REk1WmQxUnU3bk82OUxQVzFqUjZseDBvTHVhdERyWUdwUEU3dkNadDRxcHJLR3l0X0lTNlhJWjF0QnZqYnNPVVlhUUVET3ZUbUY4M0JHUnQ1TUVYUHY2cWNRbTFRQ2RlTHdpQU1TRmppc0hvZDY0c2UxUUxBcHBwWkl2OUpSLWlfWE1TVFdqOTRYWE94Y1NVSFU3cFBueUhfdmk3bEhKNjFqc3RaLUlWVEg1YXdIVlhjZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBSa1pzbUFsOWxJUk1UdXVwZjF2VkVlOGtMS0JMMjJGcUw4SVhSd2NzS25KYkU2NnNoRmFmeHJYcGN6UHFILVBmVm4tOFJoeHFDWkV1LXNiczJKZw?oc=5</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3320,52 +3320,52 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K53" s="1" t="n">
-        <v>46086.38887731481</v>
+        <v>46086.55915509259</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>Local Town Ingolstadt German</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Futsal Benfica Auderghem - Anderlecht</t>
+          <t>Fußgänger stößt mit einem Bus zusammen: Fahrtgast verletzt sich - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Futsal Benfica Auderghem - Anderlecht</t>
+          <t>Pedestrian collides with a bus: passenger is injured - Augsburger Allgemeine</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:09:11 GMT</t>
+          <t>Thu, 05 Mar 2026 13:57:30 GMT</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE5scURuclV0anR4NDRjYWFCWU9Ea0wtSG9JYTNEdTU5Z2NxdTlpQ2Zjcl9XOGRLZEFFcTVhVHZxTzdiUDVoeFpYaUZfWS1ZNFdKcFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxQX3VTMjFDSE5HLURMWEpVNGpfdkJvMTJZVkpib1dLdGQ3b2g3cnhCcmZyeGNZN0JlUXNNZXdpMDg4RUlwbWhtalVyb0JEM0g5My05QUJxRl9OUnZ4eXdLOXI4aUtJNGRvUUxfTktOOU1VNVROX1FWdzZaOWliVUtzejNMTDBBNHVVOXE3ZUt4bVFMdDRsdEVZY1ZMX3V4c3luSEM2bWl3STNFU29LcWNyOEpXYW1lZ3Y4dHNhUFc1bmlvYTB5bTFIb2k2RDdwdWdTaVpWcFd3SFRHcmtOZkN2RG0zci0?oc=5</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3375,52 +3375,52 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>de</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>DE:de</t>
         </is>
       </c>
       <c r="K54" s="1" t="n">
-        <v>46086.58971064815</v>
+        <v>46086.58159722222</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Ingolstadt (fallback)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Ingolstadt Village" OR "Ingolstadt") AND (shopping OR outlet OR luxury OR retail OR news)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Polizeibericht: Raum Aschaffenburg | Küchenbrand - Keine Verletzten, Pkws angefahren - Unfallflucht - meine-news.de</t>
+          <t>Here are the best-selling new luxury cars ᐉ News from Fakti.bg - Auto - fakti.bg</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Police report: Aschaffenburg area | Kitchen fire - no injuries, cars hit - hit and run - meine-news.de</t>
+          <t>Here are the best-selling new luxury cars ᐉ News from Fakti.bg - Auto - fakti.bg</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:32:07 GMT</t>
+          <t>Fri, 06 Mar 2026 07:27:00 GMT</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQNjdBaHdqMl9NT0d2UUhqUzRZVHBYaFVadWRnUzE3S0p5Vm9VT1FTZWZyaWdHZWx4VUtReTVUbThlSDdEd1RKTFlycFFjTEpDbzBhUGRjUmhDai14NnE4bEttc1RiT1FkNVhKZURQUWpMa053WldacVdvVEVFRmZKWWdwREpaU1l0UXJiOGtRZEVJNTRrcW8zNDZlbzhnd3ZVMV81Tl9WT2x6X2hYcXIxUUV4bjBqeUpCZ3BQejFnNndPa3BTVkZsY0tvd3dQT1V4Tk4tWlFkZFZodmdIWE9Ocw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9XeUtoeU1qYk9ZanR4MEJhUXhwUEpTUVliNVlJSFdtNml0WFdqdmJRRlBfajJyYXdoT3RkUUJfWWFtb3hXSXNadGpWcVVqTDZ1MGdtOWJXZHBPRm9HVXQ4eUhMRkpMSlk3cHJMZm1MX01IVm1aNlM1dTVSTDBEZXc?oc=5</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3430,52 +3430,52 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K55" s="1" t="n">
-        <v>46086.56396990741</v>
+        <v>46087.31041666667</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Village Bicester Kildare</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Sugar Plum Sweetery Win Westmeath Enterprise Award - Midlands 103</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Sugar Plum Sweetery Win Westmeath Enterprise Award - Midlands 103</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:23:17 GMT</t>
+          <t>Thu, 05 Mar 2026 10:19:43 GMT</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQS1dwX0x2SDQ2ejY1OFVvTGJzNGpfUTdjdThEZDhGQXBsWHJTeWwwMzgwUDlaLVFUZERvSVlrandHUC02WFlrZC1lZE1nYkFTV2k2eVJaR0xfSVdPZ1ZPeFlud1hfb3BtQ3lyUzZuX0p2NkdYeDFpS25wNEpaRnhaV3NYcmJxMVBiajJFSS1XQnpQNDE0d2VEUkhWbmpKcERjbnZWeVBxOUxSUVdKSXpWNXByOGZBak94T1IwMQ?oc=5</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3485,52 +3485,52 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K56" s="1" t="n">
-        <v>46086.39116898148</v>
+        <v>46086.43035879629</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Schweinfurt: Neue Polizeikameras in der Innenstadt offiziell vorgestellt - Radio Gong Würzburg</t>
+          <t>Milano, brutale accoltellamento per una battuta: arrestati quattro minorenni per tentato omicidio - Affaritaliani.it</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Schweinfurt: New police cameras officially presented in the city center - Radio Gong Würzburg</t>
+          <t>Milan, brutal stabbing over a joke: four minors arrested for attempted murder - Affaritaliani.it</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 14:30:00 GMT</t>
+          <t>Thu, 05 Mar 2026 12:05:39 GMT</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNZ3RZa1V5ZmJlTWZzTk83QzNjRmRpWGxaelpwSFBxTElkTC1pQUhiSTVWbGR3akxqQU5sTVBxaGI1eGVXV1c4NnZibE9Pd3I2VTJDNDVHVWp6RVRIVzhSV19CNkVCeENocXpLSHpHVFdsVV91VHZia2Z1d2hUTUF3N2ZtQkZtdF9XUVVGNGs5RFFfNElpbDkzaG5OY0Jqbm84WUdOZ1ZEQTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPc3Q5NXBQa0xPYXUxMnpyQzFYRVNrTEZUTm1MTVQ3NUNkaTFnVi1HVjQ0Qy1xQWdQaXNYMDZfRW52M0swVTJodnB3ZHhmOWVQUFBPT0JUTnJKX3Y5Vklkc0o0MjhfZUV5MVRnNTRHNFdQSC1DbnQxeENJd1ZtOExZcW55eHlHYTVsbXBJb0ltZnBFQ0FyZjZaNm5oYUJMMnBlT0hQbllQMHlUYVB3dnFDSTBlZEVoRnRnWFpZei1qX084cmEwbFFvVVpvZmRxUDdQelE?oc=5</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3540,52 +3540,52 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K57" s="1" t="n">
-        <v>46086.60416666666</v>
+        <v>46086.50392361111</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Tod von Messerangreifer aus Würzburg: Keine Hinweise auf Verbrechen - Joyn</t>
+          <t>Lagarde contestata a Bologna: lancio di uova contro i fantocci e tensioni con la polizia | VIDEO - BolognaToday</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Death of knife attacker from Würzburg: No evidence of crime - Joyn</t>
+          <t>Lagarde contested in Bologna: throwing eggs at the puppets and tensions with the police | VIDEO - BolognaToday</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:08:26 GMT</t>
+          <t>Thu, 05 Mar 2026 19:35:08 GMT</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQV2RSWFRMaUpHNWlYYm5ON3U3QUN6UEFhZWRiUWZWYzY4RGhNYWo5TWJlLVNNMThIVU9qZTV0NFpqM3BuUTlidVYtQW9ENXdCUlF4Ul9vaEk5Q3RWbmU3Y3FHOU1Zc05CTFh3LWVQdzk3RTlhR2xhc1ZBMFdjWFg4UEJFb2YtbWxVOVcyVDFlMGJ4eHQwZ3AybEJRU1hkQXhwcm1MNXpTVGhhRFNUbzhwWVVTVkR2aHdB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxQWEZZN0poc2JXa0ZpR2FmdWtlcjhLQjNIWG5maUZDbnMycEYteHJsU0RuVTZsZjl3MF9jRUxlR25lX3VXelVtdlFqNmJLLTRzQ29DMWprVGpGNTdTcWVrUFRzcjZyZlFsMC1lOWlKdzd6VjltWEpzQ0tMaHVzMDBnT1hFbWxSdw?oc=5</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3595,52 +3595,52 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K58" s="1" t="n">
-        <v>46086.46418981482</v>
+        <v>46086.81606481481</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>POL-LB: Großbottwar: auf offener Straße geschlagen und beleidigt – Zeugen gesucht - BlickLokal</t>
+          <t>Manifestazione contro Lagarde, un centinaio in corteo - RaiNews</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>POL-LB: Großbottwar: beaten and insulted on the street - witnesses wanted - BlickLokal</t>
+          <t>Demonstration against Lagarde, around a hundred in procession - RaiNews</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:59:19 GMT</t>
+          <t>Thu, 05 Mar 2026 16:26:00 GMT</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNaE0ybnFYUTY4b25kNkIyNjBhbmlaWk1wUmQxaTdGMERNRXVybEtXYldaS1NoYXltQ0dyeGpvcXBSUzBDRnZxMnFvVzJZdXFDeXlCX2Z1RlRjYkxmcmFpbmVZU0UzTGNmTm11bFVZNkFiQ0l6cTVvR2UzbmdPSGI3LWV3NDd4UTc2dFNEWEpnR2NOT3BZNWFlVE5nX0Q4NWVZS2w4cVVGS3psWEJKSGlOR01B0gGyAUFVX3lxTE1oTTJucVhRNjhvbmQ2QjI2MGFuaVpaTXBSZDFpN0YwRE1FdXJsS1diV1pLU2hheW1DR3J4am9xcFJTMENGdnEycW9XMll1cUN5eUJfZnVGVGNiTGZyYWluZVlTRTNMY2ZObXVsVVk2QWJDSXpxNW9HZTNuZ09IYjctZXc0N3hRNzZ0U0RYSmdHY05PcFk1YWVUTmdfRDg1ZVlLbDhxVUZLemxYQkpIaU5HTUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxQS3NiTEpkdkJTbUxBSkxjNVM3LVR1dDdrWlk0Mm45ZWFuMUkwUGMycDV2V2N0N3BlVVYwZzZVdnB0YmtnSHVpZzVWY0NaOW1nOVRJRk95ZGRZcGlpazJSOWEtR253dV9IdEdsdVExOVBKLW1JWjZnRXNGakozTVRsc3J4TkwxRzhUSE9ZQzZYQUEtQnBzZlhOeURmY2dqYjZzMk84OVJZRjVaREVUMnhNR21KaUZ6elh0dW0zM1pVWk1peHhNNGViYTROTFVGVTJ5ZDJIRjhQSTVpN3dERkxYdm44eUc5Vlc30gHuAUFVX3lxTFA3eHpsXzhzaTdlQTcwNi1NVjB5aXl6VFVTQXlTWXlTLU1JWTEyZDNndjdqeDI2WjRBaFhPcHFaMzRRSXN4UHBfRWpLYV91X3pqN1lfclBhSkU2S2JIekdVNEVqalNmNml3UUVWdkN0XzJFSktObXBaS3gyMmlUZUFTRTdwQW02ZlQ5Y3Q3NEt0al9ZdTV1Umkzc2xhd21QZHFNVkRWVVA3WDVFOFVoY1N2a09BTVZnSVJyc19LeXdEd21wREFEOGtQQWptdkZHQW8weVRxRExnZjhicm1aRUE1N2h2V01haC1oVjA1X3c?oc=5</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3650,52 +3650,52 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K59" s="1" t="n">
-        <v>46086.4578587963</v>
+        <v>46086.68472222222</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Blitzer in Blankenbach aktuell am Donnerstag: Hier nimmt die Polizei am 05.03.2026 Raser ins Visier - News.de</t>
+          <t>La protesta contro Christine Lagarde alla Johns Hopkins a Bologna, foto imbrattate di sangue e fantocci: contestate anche Meloni e Schlein - Il Resto del Carlino</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Speed ​​cameras in Blankenbach currently on Thursday: Here the police are targeting speeders on March 5th, 2026 - News.de</t>
+          <t>The protest against Christine Lagarde at Johns Hopkins in Bologna, photos smeared with blood and puppets: Meloni and Schlein also protested - Il Resto del Carlino</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:15:39 GMT</t>
+          <t>Thu, 05 Mar 2026 20:03:11 GMT</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwJBVV95cUxNT3dZVW1WQzJkMWU4NV9lNTdWT3ZKdjhQWlJVSi1FSXZianZmYVpHUWZKMWx3LVVUSnFXSWlEUmJHREJLdVV4UVRoSUtSS3JfSUpLdGRwUHhsZ1J1bF9uVlQ4UEVYVE0zSTB1bzJJWnZYcm43T2p4LTdQekg1Vk9jaUJfVFItNGZYZkVycFZhT3h5UjBudkJYSmxMZDFYLThvVGFZLWtOOXFtVnRqOVVpVzNWTmlqSWhtQjBhamZXSUw2TUpmLXQ0eGRGaDQzYmtyRzhhQVlhaUpJVEZiRk5rQ2NKc0s4Y1ljWUw4TFVvMHhzMkhNT2QxNDZfYUtLTm4xZzFpT0xDSkI3bGQ5cXhTb0ZnSHdiUW_SAZwCQVVfeXFMTWgybGRuOHJFRHpxcWVON0NYZW9NSjdFY1phYV9mZm84NDFpcGF6Nk1tY3hNS0ZXb1JtNzNGOTdhMUpxeDRMQUR5akdOZUVKMU5FOTE4MWRJYXlWRXgxM0dKTDJabVBpdGk3aF9DVkJDZmRtV2dELUZSbWtaOGRCNDVLZWxmS284T3RGcGoyR2c1U0ZpZnNoMEduUmZLOHRweFFFTWJ1ZE9wQjh1NVVZTXM4dGRNTjIxaFFMTkQ0N2UwTk5Pd0RkWUJkMVVZV2N1T0hQQmRqZ0VzOHBkajU5d0hvYnczSkFMRjRmcTlPUUVEVFhHb1Jwb2dpUVhnS1c0cjREX3ZQdktKMVNDdlJ2NlJ1LUgtMDJGNEVkOFQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOb0xhNC1rT0cwTEY2anRVZ29LVkRqYUROS1ItWFJZWnd6WktZNTRQY3RYYkcwTEo4dVUtRTJIUWtXbVVPT1lYRjhfdk43MGlZWGl3QzhubXlNUFFGNWpTQWhzc0RZbFJnQ2VETHZQUTZWQzA4VF9LWkNIQTdSeDZNZDEzdkRleW9nandhWERVUUlReHo3SnpHSGU3WW1vZw?oc=5</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3705,52 +3705,52 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K60" s="1" t="n">
-        <v>46086.55253472222</v>
+        <v>46086.83554398148</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Golfcart als Fluchtauto: Polizei sucht nach Einbrechern - Augsburger Allgemeine</t>
+          <t>Sciopero generale, aerei e ATM: marzo di passione a Milano - Milano Weekend</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Golf cart as a getaway car: Police looking for burglars - Augsburger Allgemeine</t>
+          <t>General strike, planes and ATM: march of passion in Milan - Milan Weekend</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 11:58:55 GMT</t>
+          <t>Thu, 05 Mar 2026 18:37:46 GMT</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQcF9qT1l3cEVrUDlCWUxhaEZRV3F3VFBCOUdXejUwNVdCZ1hLOFBpa2pUX2c4R3EzWV9PMGJPU2VYTHFmUHBfbkxyYWhPUzlIS05LNjdIamJvVDRTWFlwMmt0ZEVXM0FLU0Q5ZWpoN3kxVzRQUkRaUVl0aDc5WWRraGozWFFhLXhQTy11NFlBbGlFM0FyemRDN21CdUtTRTdMSWtuNDc4bjFMbW5Ia25iRVRPWDkxcjdWQWhsd3BOdUNOejFucGhr?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFB6cHBiM2lyVlRvcDBibW1wZzE4NnV4SXJad0NVbW82dDJCUkt3aml4LUx3OWtWc09DNl9PbmZUbDhjRGZpeWxQdEliOERkSU1fT0JnUFFXVGs4czI4T0Z3Vlh0ZnJnb2FXejU5eUpzUmR4QkhUQWc?oc=5</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3760,52 +3760,52 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K61" s="1" t="n">
-        <v>46086.49924768518</v>
+        <v>46086.77622685185</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Schüler gegen Wehrpflicht: Auch in Ingolstadt wollen Schüler heute demonstriereren - HITRADIO RT1</t>
+          <t>Bologna, manifestazione contro presidente BCE Lagarde a Bologna - Local Team</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Students against conscription: Students also want to demonstrate in Ingolstadt today - HITRADIO RT1</t>
+          <t>Bologna, demonstration against ECB president Lagarde in Bologna - Local Team</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 09:34:00 GMT</t>
+          <t>Thu, 05 Mar 2026 19:02:46 GMT</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOT0dXeC0yU2RmcTNoWDM2dWJzZ0doZHN3OTNFSXNPWlF6YW84VGVWX1Vob2ptVXdVcGVLQ29GaUJjOWdaQllpYU1IYU9Ia3hiNWVGYjA4RUR2SGx2NUh3Nll6Z01JVlI2MTg3U0dXS1hZSEZxbHJnYXdyZ2dRX0duamF0RTQyaWU1SDY5WGcxT2FseFQ4TzlaRkdvaUttN3pCR0ppeGRid21PSUxMcjY5ek5Qb3psUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOcS16d3UtZjJBd0xCU0oxUENYQXZEMXBBWHVqRDg1ZEZsaFBDWlZPdzdCZGcyT25pUmd6UmltNkhmOWhHZUVxQWQzcmJrYjB6SmU2N3JKRWxvRy1TbllVMXN5R0hlTVBiWjlOd19ld282R04zTkVpMkFCZ2t4b2RWd2RVckhhdzQwaDBZZU5uNnFDeHZGcVlRZmI0T2ZjRXl1WUFLcnNuVnZkM1E?oc=5</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3815,52 +3815,52 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K62" s="1" t="n">
-        <v>46086.39861111111</v>
+        <v>46086.79358796297</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>30-Jähriger aus Manching verletzt sich bei Moped-Unglück in Ingolstadt - Pfaffenhofen Today</t>
+          <t>Milano. Giù le mani dal Medio Oriente, corteo - Contropiano</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>30-year-old from Manching is injured in a moped accident in Ingolstadt - Pfaffenhofen Today</t>
+          <t>Milan. Hands off the Middle East, march - Counterpiano</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:25:11 GMT</t>
+          <t>Fri, 06 Mar 2026 05:35:45 GMT</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBSa1pzbUFsOWxJUk1UdXVwZjF2VkVlOGtMS0JMMjJGcUw4SVhSd2NzS25KYkU2NnNoRmFmeHJYcGN6UHFILVBmVm4tOFJoeHFDWkV1LXNiczJKZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE9iQWdVLUdzdUtOSi02Vkd1SXRLV1Z6RjYteFROY1NLeHVwcmsyY0ZlaUJrZl9jU2tMakhrMkhyV0dtam1CdmtYdlRMdE9DcDI2VDBrOGg2ejhac1Ywek9SRFhGdTBwN1hFd3BvY1dKTHp2UjZMMHNpMzU4R3ZjdTQ?oc=5</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3870,52 +3870,52 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K63" s="1" t="n">
-        <v>46086.55915509259</v>
+        <v>46087.23315972222</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Local Town Ingolstadt German</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Fußgänger stößt mit einem Bus zusammen: Fahrtgast verletzt sich - Augsburger Allgemeine</t>
+          <t>Il presidio degli studenti davanti alla Prefettura di Milano - Il Giorno</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Pedestrian collides with a bus: passenger is injured - Augsburger Allgemeine</t>
+          <t>The student demonstration in front of the Prefecture of Milan - Il Giorno</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 13:57:30 GMT</t>
+          <t>Thu, 05 Mar 2026 17:30:39 GMT</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxQX3VTMjFDSE5HLURMWEpVNGpfdkJvMTJZVkpib1dLdGQ3b2g3cnhCcmZyeGNZN0JlUXNNZXdpMDg4RUlwbWhtalVyb0JEM0g5My05QUJxRl9OUnZ4eXdLOXI4aUtJNGRvUUxfTktOOU1VNVROX1FWdzZaOWliVUtzejNMTDBBNHVVOXE3ZUt4bVFMdDRsdEVZY1ZMX3V4c3luSEM2bWl3STNFU29LcWNyOEpXYW1lZ3Y4dHNhUFc1bmlvYTB5bTFIb2k2RDdwdWdTaVpWcFd3SFRHcmtOZkN2RG0zci0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQZDNOUlJVSGtBeklfME5NUHM4bGVyamNmLXVYLTROalIwZ0ltSU15SkxoRGNGVTg5QmZGVnAteEFqaFFyNEVQUVEydUNlNkdmcGZGdmdSczJQV1h0TEZrZzh0eklQUEZVYVFYYXI5eEZkUm5Vb182RXVub3NUMnkySzVITml4dk1wdHFpMjgxLVpGWUZ5SWN6WW1WejNOcmxy?oc=5</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3925,52 +3925,52 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K64" s="1" t="n">
-        <v>46086.58159722222</v>
+        <v>46086.72961805556</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Village Bicester Kildare</t>
+          <t>High Level City Italy Italian</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>("Bicester Village" OR "Kildare Village" OR "Bicester outlet" OR "Kildare outlet")</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Sugar Plum Sweetery To Represent Westmeath At National Enterprise Awards - Midlands 103</t>
+          <t>Lagarde a Bologna, la contestazione contro la guerra e la presidente della Bce - Radio Città Fujiko</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Sugar Plum Sweetery To Represent Westmeath At National Enterprise Awards - Midlands 103</t>
+          <t>Lagarde in Bologna, the anti-war protest and the president of the ECB - Radio Città Fujiko</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 10:19:43 GMT</t>
+          <t>Thu, 05 Mar 2026 10:40:36 GMT</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQS1dwX0x2SDQ2ejY1OFVvTGJzNGpfUTdjdThEZDhGQXBsWHJTeWwwMzgwUDlaLVFUZERvSVlrandHUC02WFlrZC1lZE1nYkFTV2k2eVJaR0xfSVdPZ1ZPeFlud1hfb3BtQ3lyUzZuX0p2NkdYeDFpS25wNEpaRnhaV3NYcmJxMVBiajJFSS1XQnpQNDE0d2VEUkhWbmpKcERjbnZWeVBxOUxSUVdKSXpWNXByOGZBak94T1IwMQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOSGV6dU5VcXRBQXJleXZ4SWNGNHA3eFVhOXNVMDItMkw0WU5zc3NHa1FlTmhFcTFqbHc5SjBudU01cXhvS3NVNE9NZktCZUVUWElPZjFmZmlzZmV4S0F0LUMxWDUyLWEtMHRycFAwVXJhLXJSSFdycS1KeFRSeUczT0xtMFA3cTFjbUtHZWdFN2p2S0ZkQUtCWVRFRUJveFJOazM0UmdHNHplWHd0a1I0?oc=5</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3980,21 +3980,21 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>it</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>IT:it</t>
         </is>
       </c>
       <c r="K65" s="1" t="n">
-        <v>46086.43035879629</v>
+        <v>46086.44486111111</v>
       </c>
     </row>
     <row r="66">
@@ -4005,27 +4005,27 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>("Milano" OR "Bologna") AND ("minaccia bomba" OR "pacco sospetto" OR "pacco esplosivo" OR sparatoria OR accoltellamento OR "attentato" OR "operazione di polizia" OR esplosione OR evacuazione) AND -Olimpiadi AND -pattinaggio AND -sci AND -Cortina AND -calcio AND -Serie AND -mercato</t>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Milano, brutale accoltellamento per una battuta: arrestati quattro minorenni per tentato omicidio - Affaritaliani</t>
+          <t>8 marzo 2026 a Milano: manifestazioni ed iniziative in città - Secret Milano</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Milan, brutal stabbing over a joke: four minors arrested for attempted murder - Affaritaliani</t>
+          <t>8 March 2026 in Milan: events and initiatives in the city - Secret Milano</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Thu, 05 Mar 2026 12:05:39 GMT</t>
+          <t>Thu, 05 Mar 2026 11:35:18 GMT</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxPc3Q5NXBQa0xPYXUxMnpyQzFYRVNrTEZUTm1MTVQ3NUNkaTFnVi1HVjQ0Qy1xQWdQaXNYMDZfRW52M0swVTJodnB3ZHhmOWVQUFBPT0JUTnJKX3Y5Vklkc0o0MjhfZUV5MVRnNTRHNFdQSC1DbnQxeENJd1ZtOExZcW55eHlHYTVsbXBJb0ltZnBFQ0FyZjZaNm5oYUJMMnBlT0hQbllQMHlUYVB3dnFDSTBlZEVoRnRnWFpZei1qX084cmEwbFFvVVpvZmRxUDdQelE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE0zNG9wSnU3bzNFOFdoSXB3dU02ZGxVQVdkSm55d3lveGNYUnZBcHZhSTZfanBzbkRuN196ZnNHMHFNNU4zMEdvd3hrY2ItVklrZkNqSFBOWGZfN19vemx5WUN0UDgyeWdwaE5IcFlScGI?oc=5</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -4049,7 +4049,612 @@
         </is>
       </c>
       <c r="K66" s="1" t="n">
-        <v>46086.50392361111</v>
+        <v>46086.48284722222</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Sciopero generale e corteo: stop a scuole, sanità e uffici pubblici - BolognaToday</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>General strike and march: stop in schools, healthcare and public offices - BolognaToday</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 08:10:00 GMT</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE9LRk82di1uN2ZNLXJCbjJ5Zld4X2NvbzdVOS1mZEdwcEdFcGhUT0w3LVpWR29sdS1ZQ2RDSTNBSGpFWDY0S1NYQ1EzRW5ZUTNNcjNJelhLS2FKVl80eS1WLThWNlRpN1BJNThfMWV5TFluZ3lGSDlvQTRzbjlyZw?oc=5</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K67" s="1" t="n">
+        <v>46086.34027777778</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>A Milano come a Berlino e Torino la protesta degli studenti contro la guerra, nel mirino il ministro Crosetto: “No alla leva obbligatoria e a politiche guerrafondaie” - Il Giorno</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>In Milan, as in Berlin and Turin, the student protest against the war, with Minister Crosetto in the crosshairs: "No to compulsory military service and warmongering policies" - Il Giorno</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 17:40:08 GMT</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOckxLdjYzSkI3YXV6WFdReEd4eUZ0emc3V0NXYjJpaVJ3YVZUSUFEUWhMZlNlMDVXVHFzSUR2dUhWdWFtdkNXUGpjNHZ4amwyU3l1R1hwMWtzUGFneVk4SHFLV3ZSNlJtQmJBMnJtcGdtY2lPc3FrOHZPRFRUM0kyZ1pEQnZtS3p5OE50RXRCSlM2c19iTFFVUDBsZ1ZNSlVVY1paaEhkS2QtbGpUd1FCZS0xM2dxRG1VaTlHXw?oc=5</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K68" s="1" t="n">
+        <v>46086.7362037037</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Esprime solidarietà alla Palestina, salta la liberazione anticipata - il manifesto</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Expresses solidarity with Palestine, skips early release - the manifesto</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 23:15:15 GMT</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNQkt2Z1VuakNxejFXYlU0dWZGQmZWbnZremVlbFRuLVhqU3M0OUdBRDRPaFR3RnNURkxiSGUyc3U4ajg3X0tOSGRhdXhqSTFXQ0ZNbG9SWl9lLTZaR0JtNlZFRVZaSnRKREFJSzM4Zi1aNWNrcG5USFN4OUhoWVp2MWpJZERpY2ZKVFowTXpXNW55Ulk?oc=5</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K69" s="1" t="n">
+        <v>46086.96892361111</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Bologna, spintoni tra Digos e i manifestanti contro la Lagarde - RaiNews</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Bologna, shoving between Digos and protesters against Lagarde - RaiNews</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 18:59:03 GMT</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi3AFBVV95cUxQaE81ai1nMXNqTFE4N3pIcV9zMkpqMlRkazlHcWpEQ19TZnZRSWdxYlNNN1FGclVBRW9zQ1o1bU1YcHNkaFF6ZDZUUV9ubDNUUFVzYjhvc3lKOWVrbkROLW03bXJ1TkUxQkF0QjNMTDhpV0Jnd1NFQXBva1hyTDhEemFkQVQ2RzY3RHdVNjI0blYyeGVBUllDRW9JenlFem5INlVlM29jcGVsX0hPWHRzYUdVQVBQeTh5WnZack52UmFHV3diWEl0cEcyT1Fwd3VYYXRtc3VUNy1lOXF10gHcAUFVX3lxTFBoTzVqLWcxc2pMUTg3ekhxX3MySmoyVGRrOUdxakRDX1NmdlFJZ3FiU003UUZyVUFFb3NDWjVtTVhwc2RoUXpkNlRRX25sM1RQVXNiOG9zeUo5ZWtuRE4tbTdtcnVORTFCQXRCM0xMOGlXQmd3U0VBcG9rWHJMOER6YWRBVDZHNjdEd1U2MjRuVjJ4ZUFSWUNFb0l6eUV6bkg2VWUzb2NwZWxfSE9YdHNhR1VBUFB5OHladlpyTnZSYUdXd2JYSXRwRzJPUXB3dVhhdG1zdVQ3LWU5cXU?oc=5</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="n">
+        <v>46086.79100694445</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>La “Milano-Meda” a pagamento? Scattano tre flashmob: "No al ticket" - Il Giorno</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>The “Milano-Meda” for a fee? Three flashmobs break out: "No to tickets" - Il Giorno</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Fri, 06 Mar 2026 03:50:15 GMT</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOazU0bFcyZnBuLVZvbXpESl9SY2xwdV9JajZBcFFGVHhOQ2xQV2tFNUVRZFZESUNRVmN1UkFZWlNMb0tUQWpyRWg1VTRUY0d6SzRTNkR6TDdQeV9Jb1NNRGp4U1N6cWhTWXB3dmVZUTZSWFktRGI0dS1FU2N3TGhjTE5FUUtEV3pBNWxr?oc=5</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K71" s="1" t="n">
+        <v>46087.15989583333</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Sciopero generale del 9 marzo, si fermano anche i mezzi pubblici? Chi aderisce e chi no - Moveo by Telepass</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>General strike on March 9th, will public transport also stop? Who joins and who doesn't - Moveo by Telepass</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 09:02:48 GMT</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBOOFg4aFJ1RXNfSmpYTUJoRDBiazE1WXB3alBabWhpQTVFa2MwbG5qUmFSQVJaQzU5RVJyU1FZLUV1Y2h6RmN5RXB2dWNvZ2FrTUoyX1VCSW1xS3lNT0IwS0VVclhLUFZ4Z196dndCYnpadw?oc=5</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K72" s="1" t="n">
+        <v>46086.37694444445</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Pilastro, presidio smantellato. Maxi-multe della Digos a tre attivisti. Applicato il nuovo decreto sicurezza - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Pillar, garrison dismantled. Maxi fines from Digos to three activists. The new safety decree has been applied - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 12:00:34 GMT</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxNdk9YZlR2TXl2eFF2dC1ia245VjR4VkhvVnFHYk1SYmZ4a3I3LTZ3dUczNTRCdDVXMnlXMDRvWkVQOEdlZTZEeTNJckRobHBqUjY3aVdmV0VZWEFHaDdMeXhvNEhkamlFZnJHOEVpSEgtaUVQTzRkTlhiZWhpcW9DWWV0TTg4RVRuX3BQRXVlTE9oVkxrYkZFZ1lKMEI3dmJZNUg3XzIwVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K73" s="1" t="n">
+        <v>46086.50039351852</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Anci: "La scuola è il presidio di comunità, di inclusione e di relazione con il territorio" - NewTuscia</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Anci: "The school is the garrison of community, inclusion and relationship with the territory" - NewTuscia</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 15:04:05 GMT</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxPY3NzMGlUZmtfb2NzX216VUxCUzZCUVNja29NbGk0ZDhfUFhvdTd4NnZ6aHc4b1hzaV9tOFM1SUprZ2E0eVhUWWVVTF96TW1uZlhhU0oyaGhkNkQ0UXoxSXIzZEV4U05VZXBwTG1Va3ZjM3BFVnE2VkdEWG00azA0ZURJal8xWV9yQ0NhWTJONWpEOW4wMldEU2NDQ2JaQXZIU183RXhqYm5JVnZNN1lXa2ktLWMyOWg0YW5qUkVCbXVoQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K74" s="1" t="n">
+        <v>46086.62783564815</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Local Town Fidenza Italian</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Morto dopo essere stato accoltellato al torace a Parma, fidanzata di Cristopher Gaston Ogando indagata - Virgilio</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Christopher Gaston Ogando's girlfriend died after being stabbed in the chest in Parma - Virgilio</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 19:13:00 GMT</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxPSHFvaWdSMlRmMDdVZzFfY0x2MmFqTTFabHNWVTRmWlBVcFpHdlVBQ2JJM0l4dVhKNWQtTHY3WG1XT1JBeVdiemhKdThJY2xqU3FGYUlTNFA0dHNyLVNzQTR3Z0h2X3ZzQTYyRlZHUEhMSl82WXZkaHhPMnpGbXpIaVhjRjdCT0g2bm56R1BqQ3YyaWl5NmxVMmotR0o2U1JIazV3aUVvRXp1M1ZGc0Z1Ry15WHN6bUF3UlVSSUE5TFZabjFheG1LSzhKdG5wbGhiRDgzU3I5TmfSAd4BQVVfeXFMT3k2aVBGajNUYWdGZTBRUHlkZmxmcEs5NmFYYjhJWEZkNldGemRCbER5Y3ZhZGx1blN4OHNTeEtzN0VnODJ2eXMtenhYT2oxbFpFZXVHdDlualZJMG02SFVhRThwY3VOcjNVY2NrTDE0bl9nMlh4X0ZVdzg1SnQ4VFZmeW5rMnJBaG1xZFNQTGY5OUJsb3VrTGd3S3FWZjMwMzFMTURsQlpxeU1kY3A1ZzdVaDZrd0pFcVBKZkpxUzZoNzJYTWhWMUhCR09qWmR6SlBhMG41cmtqb0RSQlZR?oc=5</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K75" s="1" t="n">
+        <v>46086.80069444444</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Local Town Fidenza Italian</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Parma, giovane accoltellato e ucciso dopo una lite. Indagata la fidanzata - la Repubblica</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Parma, young man stabbed and killed after an argument. Girlfriend investigated - la Repubblica</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 09:52:47 GMT</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxQN1l6dGtNYjF6NU1iblhlUW9ZalhKb3ZnS3REMEZfakZ4MUJyd2piYlFKcjcxUmNqNk9WZ0ZCMEFRejlxY1VtRktQbm12cVB4aXFhTFBNMUtyT29ZX3VfTUdNUDgzbHNVazVxVElXTWg0VnhZSFN2X0dsUkhDVnNyS3BsSXAxZGwtZTg0eXFIbDItNjk3eTdTc1pnLU5CTGZyNkt5VXBpYlJiVU1STTR4Sm5ZZkR0cHAxNVA0?oc=5</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K76" s="1" t="n">
+        <v>46086.41165509259</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Local Town Fidenza Italian</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>("Fidenza" OR "Parma" OR "Piacenza" OR "Cremona") AND (protesta OR "minaccia bomba" OR esplosione OR sparatoria OR accoltellamento OR evacuazione OR "operazione di polizia" OR arresto) AND -calcio AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>"Visite private pagate in contanti": medico primario arrestato dai Nas di Parma - ParmaToday</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>"Private visits paid in cash": primary doctor arrested by the Parma NAS - ParmaToday</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Thu, 05 Mar 2026 08:04:08 GMT</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPWmtETkZER3RWclhUT0dfWHRFMjZSR0wwOGQ2LTRWOFVlVWMwTFR0Q2pHMm10TmZoVHN6LVlQZWxITTU2RVB1OFRvWjdxQlpVZmN5V0xjSkVqcGdXUUllX2RoaS1Ua0haRWs0M2dDX19XbU03LXRxZGxEakZmTUYzVUU3ZlJhZE9YdGlreDZpdl9wOFE3OEE?oc=5</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K77" s="1" t="n">
+        <v>46086.3362037037</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-12 07:54 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Value Retail Brand</t>
+          <t>Brand Protest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>B&amp;M 'luxury' £10 afternoon tea gift set hamper selling fast for Mother's Day - The Mirror</t>
+          <t>India’s luxury split: Hermès grows as Gucci, Dior lose momentum - Mint</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B&amp;M 'luxury' £10 afternoon tea gift set hamper selling fast for Mother's Day - The Mirror</t>
+          <t>India’s luxury split: Hermès grows as Gucci, Dior lose momentum - Mint</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 11:56:00 GMT</t>
+          <t>Thu, 12 Mar 2026 00:30:11 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOd2R5cndGLTI5OXhkS0ZmUm9mVTN0ZGw4ZTJ1bTNobmt0UlF3cVhsd2RxS25iSnJJazNGUi12RFpjN1pQX3NwYmtIUHpORUxUT2QyNm4yVldOaFpSaDRhZEE4Zm51NEVySExkbFF1RDZEZDFDdF9xamJmX0pRTzhqRnZtZWdCMTc0WG02TkxB0gGOAUFVX3lxTE53ZHlyd0YtMjk5eGRLRmZSb2ZVM3RkbDhlMnVtM2hua3RSUXdxWGx3ZHFLbmJKcklrM0ZSLXZEWmM3WlBfc3Bia0hQek5FTFRPZDI2bjJWV05oWlJoNGFkQThmbnU0RXJITGRsUXVENkRkMUN0X3FqYmZfSlFPOGpGdm1lZ0IxNzRYbTZOTEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOM2V3eW12YTAzS3hsWjluZnQwMWtaQWVUVG1KMnBMN3lFZUNJbEcxazZoeURqWFpZUG9iSFlQa2l4V0xIRWJVQ1NxS1NVcDlOb3BSTlMyZENscGdIdkFfNVZWSkFCdmNkLWtyVVR6WDlDT3lELTU1RnB3X01obEFLYUNUeU9pbzA3RnR4MktIbUdKOXVPMm1KLU51OU9IcmRkRi03Yl9XV1VyWmhtemZYUHNNdkxQTUhreDBjZmc4TGrSAcYBQVVfeXFMTXROUGotWjdVaHMwREh6RTJvM3l4dzNVMGdvbWo0R1J1cC1nSGR3U1MwMEtnaVZhZXloQzllNkpMc09qanpKTl83WWYtY1p5cXVfOVdyUjZIOEdicFBTTnMxOFgxejcyeVhQT2UwTkZIT3BnYjZjUHJUM2ljVy1TT28wckN2N0ZMdkItNXFoT0FkYnR2U0pDa3BQNW5qQy0yaUhUTEFCMmZGVjdxbzUwWGhjN3pveGw5NUc1R3VaaGw3YXlZYUl3?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,38 +529,38 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46092.49722222222</v>
+        <v>46093.02096064815</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Brand Protest</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>("Gucci" OR "Ralph Lauren" OR "Dior" OR "Armani" OR "Louis Vuitton" OR "Burberry" OR "Prada" OR "Nike" OR "Canada Goose" OR "Hugo Boss" OR "Moncler" OR "Saint Laurent" OR "Loro Piana" OR "Lacoste" OR "Versace" OR "Jimmy Choo" OR "Michael Kors" OR "Missoni" OR "Kiton" OR "Aquazzura" OR "Tumi") AND ("protest" OR "animal rights" OR "fur free" OR "PETA" OR "activist") AND -BAFTA AND -"red carpet" AND -"awards" AND -"wears" AND -"dressed in"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Oxford City Council sets out 2026/27 priorities with homes, rental reform and Local Plan at centre - Oxfordshire Guardian</t>
+          <t>Still think the 'devil' wears Prada? Fashion has moved on, she now wears Sasuphi - The Star | Malaysia</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Oxford City Council sets out 2026/27 priorities with homes, rental reform and Local Plan at centre - Oxfordshire Guardian</t>
+          <t>Still think the 'devil' wears Prada? Fashion has moved on, she now wears Sasuphi - The Star | Malaysia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 09:47:00 GMT</t>
+          <t>Thu, 12 Mar 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOTUM4UVFBWUdtMkczU0oyVnUxMmY4MEloYVZUV1AwOGNjVkljNmxNYkczVzA4SUlleWZjQ1RobDV5bXRLekVDb3NWSV9mYVhIQXlFZkVhcGZKRXdSdWRpLW9KcW5jekw0NjJtZGdoVXNBMGdSRHl4LXRmX0RNMnpiTlhlWldvaTJ0ZkNDOXlCYVVGSzEtcUpJNkNsb0FGZ3FHRGZZWkdfei1nVzVWVWJWRzlqTFNuNWtzQ2FCZDNIV1BOSzRJMV9vODZZQnQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPRVhla2xTbnVldEFlRTV0WmZvNFVaNzFiekw0bkZfLTNfTDVrMHlCcWljTTBrdUdwQjZmQkpDbnVVR2MtMGhZS1hnTnhxN2ZtblNVRERVbC1DQmxVNXRoOWhvdWhTaUdwTUJwal9NTGtibC1KcVZkQU04OGJwUURyNWUzRVRuQ3k4cEc1d0I1b05DMUFrYXROSFNTSWpUSEkxQjFoQmFySXlTRDMzZmhaVE9KbmFLaUIyWG9tNmc3dFZkZnN3LTFWbjJ3?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46092.40763888889</v>
+        <v>46093.29166666666</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Oxford City Council Considers Compulsory Purchase To Unlock Jericho Wharf Redevelopment - Oxfordshire Guardian</t>
+          <t>B&amp;M European Value Retail S.A. (LON:BME) Given Average Recommendation of "Moderate Buy" by Brokerages - MarketBeat</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Oxford City Council Considers Compulsory Purchase To Unlock Jericho Wharf Redevelopment - Oxfordshire Guardian</t>
+          <t>B&amp;M European Value Retail S.A. (LON:BME) Given Average Recommendation of "Moderate Buy" by Brokerages - MarketBeat</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 09:34:55 GMT</t>
+          <t>Thu, 12 Mar 2026 07:00:18 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPRmtEelk3OGVpSHhUcEs3aDZaVlNpSERjdWdGeWV6SGp5VDd0akpISHIxVk5SaHpJd2RHNmlKcUFROE9GUUkxb3E3SUdhT0xROWtJZ2xiVUtZNk9LQWxGWXdhajFxWGdPUzZ4QTl3ZGpOV0Q3WEs1Qjc5cjVEZWdaSU1saE9nb2RqT29RU3dLV3hxQmFYTUVEQjA0cFZDcFhsaGlDcXJhRi1tbDFEdUtsOTFVaFBIMm43VTFqWk1Dbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxQMW1ZazNjYjlzNjJ6VEQ0SE1mbEphMlRka0pzU19pMllxWXdQdXRUQ0F6cEtwRmdMNkxULTdSdXpQMDJLWm9aNjdNLXI1LV9rRVdsaXp2RUZLVWlJSlBmVURnN3pqbU9hc1V4eXlxUEg0SzlESkNQSEo0Q3E4QmlvdXo3N0pvRTRvdzcwc0dRUDlXV195Skk2WDFRZUJpeVVkMG14Q0dkZ1Jrc3VhazZlOTB5TlRtV2hUaXd5SF9LN3Vnbmc3QUVOZmt1MlRoOVZfdnIwWkp1TDkzS3gxZ0ZNOA?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46092.39924768519</v>
+        <v>46093.291875</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ook na explosie aan synagoge blijft CD&amp;V militairen op straat koppelen aan overbevolking in gevangenissen - De Standaard</t>
+          <t>G Sachs Upbeat About Condiment/ Prepared Food Sector, Favoring HAITIAN FLAV, ANJOY FOOD; CN Essential Goods Demand for Spring Festival Beats, Focus on Cost Fluctuations - AASTOCKS.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Even after explosion at synagogue, CD&amp;V continues to link soldiers on the street to overcrowding in prisons - De Standaard</t>
+          <t>G Sachs Upbeat About Condiment/ Prepared Food Sector, Favoring HAITIAN FLAV, ANJOY FOOD; CN Essential Goods Demand for Spring Festival Beats, Focus on Cost Fluctuations - AASTOCKS.com</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 11:30:00 GMT</t>
+          <t>Thu, 12 Mar 2026 04:00:00 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPWm5INmp3TE9Ea094R1RRb3RfSWVWczhtdXFfZWFxNGh1MjJrZVRyRU1KWXVGcFJldm5GWVVQbG5yZENqbmpzaGtzZktaNU5NQ0NzMnRtRVpTT1lTNVNTbk12bHB2NWtpVUlJOUlZNTFUeDdlZUJuVlRpY1NGSDJBZlNyeGcwVEpiRjNxN1AxM2xyYVVxVGp0bkJjd2QtNVhpSnd3RmJOVmZfTW1RZHBJcmZxN0NqWjFkbXJvZkNpRFNlbjRDNEM5dnJRSUVZQkM2OU5oUm5mZHFSM2NhRVRzcjE5RG1SWFh1?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE9EQlgyU2d4MjFiSVQ1VGtxd0lhX0c0cDJRbEZ2WHdvcXZCR2tPVkQ0SFF2eThMdEVTdzZuemNPTVBHSktqYUM4OHNndDVQWEpWUmVLWTVYaFlhY1A4b1NHc3FEMGVyeTN6WnEtcGVOUQ?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46092.47916666666</v>
+        <v>46093.16666666666</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Grote delen van Dresden geëvacueerd na vondst van bom uit Tweede Wereldoorlog: 18.000 mensen uit huis gehaald - HBVL</t>
+          <t>B&amp;M's cheap gaming chair similar to Amazon's £361 option - Bristol Live</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Large parts of Dresden evacuated after the discovery of a Second World War bomb: 18,000 people removed from their homes - HBVL</t>
+          <t>B&amp;M's cheap gaming chair similar to Amazon's £361 option - Bristol Live</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 11:08:26 GMT</t>
+          <t>Thu, 12 Mar 2026 03:30:00 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxOaUd3V2VENnFXcnJOM1VWejdqQTF1VVdEdG96TVByWnRwb2NyY2l4T1F4M0RyZC04VWVYa2RLY19HZWk3RFZTT09jY1hHcjFxZHFwSTNneDRFRTBqZEIxTzZ4VzZlNWFsM3ZwNldsN0Qtd1gtWWlyTlk1SDh5anl4aXBuV3NsRk5uZmZIYk82SFJMeHV6N1FtckpoV2I2YlBWanZob3dwczI5Q2VCOG5Nb0VpNzR0N0Vwdm80emFZdndENlZDZ3ZXdDAwVnAxM0ctdDZjUEdrZEg0QzNXMWR0Q3YtUndZYk1ldkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPazB4RGtNMUJ0dG5qU1ExNWZHbnFoZ0F6azZqY0lWUnd1VW9YNVpJMnZzOUxIZVRwcDZEbXVOSUdOLVQ4eWdHSm5rdW9fb193SkxzREtVbE5aV1Y0Y2FWLVVGcVEteUM5a19McTc2SjF5TnNWUi1jdGFvS1A3bVNoaG12eTVucnJkOElUS3VZWWV3UEVpVUMwdHpnNUllQlB4?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,52 +735,52 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46092.46418981482</v>
+        <v>46093.14583333334</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Politie zoekt verdachte van poging doodslag tijdens oudejaarsnacht - Nieuwsblad</t>
+          <t>B&amp;M 'luxury' £10 afternoon tea gift set hamper selling fast for Mother's Day - The Mirror</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Police are looking for a suspect in attempted manslaughter during New Year's Eve - Nieuwsblad</t>
+          <t>B&amp;M 'luxury' £10 afternoon tea gift set hamper selling fast for Mother's Day - The Mirror</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 10:36:29 GMT</t>
+          <t>Wed, 11 Mar 2026 11:56:00 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxNLTVFdlhWbWZMMjdqaWlvajI2SW9FcDRrclVZUkVkRG82M0tUZ2FGV0I3dDV4dFkzSzczUmxDZjVyX25mNUpjR1kxaFQ3TmhHUEJMbzVvYm4xWnF1dngzYVBVaUt0b282bUd6aGJ4WFBtNWNFTWRrckpsV0VxMTEyV0lvWHFZaVdEbGFXczk1dFZiYUlyZ0FVZ2V4V1MyUFAxZndmWmYzblR5M3AtYl90NXVmbkpLMVBzUWlMZDM0b0wxdjhxN2ZsQUg4STRNZld0UW1IM2kySUpEUHhneU0yd21sVmdoem80Zmd6NnE2VHJkRHJNVEFYaDc3aGE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOSXBVWXBiN2loWldCcy1OWDYtRkp6dnNZVTRDZk5OdEdWcmJsdnpELVBVbFlJTHpPS21jUWZmc09vNDlqLVRIU2IzdThvM1FpMmQxT2hTUWY2YjQxbW9CLUJpYzBManpGa0hKQWVjT1BfZll6ZXh6MURqVk0wdXNQeFlGNGR3WEF40gGOAUFVX3lxTE53ZHlyd0YtMjk5eGRLRmZSb2ZVM3RkbDhlMnVtM2hua3RSUXdxWGx3ZHFLbmJKcklrM0ZSLXZEWmM3WlBfc3Bia0hQek5FTFRPZDI2bjJWV05oWlJoNGFkQThmbnU0RXJITGRsUXVENkRkMUN0X3FqYmZfSlFPOGpGdm1lZ0IxNzRYbTZOTEE?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -790,52 +790,52 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46092.44200231481</v>
+        <v>46092.49722222222</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Woningbrand op Demertstraat in Maastricht - AD.nl</t>
+          <t>Interface Systems Strengthens Alarm Monitoring Against Cellular Jamming and Break-Ins - The Manila Times</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>House fire on Demertstraat in Maastricht - AD.nl</t>
+          <t>Interface Systems Strengthens Alarm Monitoring Against Cellular Jamming and Break-Ins - The Manila Times</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 12:56:00 GMT</t>
+          <t>Wed, 11 Mar 2026 12:18:05 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxONHVMdmRTVDlwYWMzM2hHeFVpQjBUaVI4alJjVUNqSW13ZnZKc2JDMDdyNW14bWRTUWMxa2x5MTBBSDVXR21oNDRfWFFiMnFqSU1xb0ZHbnpCT1RHTUxCS3BwNEZCN01uN3hLSkxJMV91dS01T0gySExGRk5WQkRkbWNhbE9ScjVxdGk3WGRZV3JfSWt6YWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxPN1pha0NtemlhWDViNVQ0ZnBoMlNLSjNBOHZ6bE5TVEFIbFdOTmp2UDZFc1M2eTlSMW5YTl80VDV3a0ZzVGJCM05hV0JwbGJoWEJ1SmkyR0NwbXNYV1JrUURmT2Y0SjBseExLRGNqZ2VlWWk2bHBUZlhzU0xjdEhSMTlsb01fRGZmWFVuRmJXSzNQSU5QRUlEcDF5SkJfeTJCYjJDRHpRSGxXTGtUak5iTUYybEdIaGdzV24zck1rMWFBRG9Dd2lscXV0VUJPaFNIeHMyYVVFS2RoX2tLSGxhd1dfTzFuNUd5S29WSzZyVm_SAfYBQVVfeXFMTjBPMlJpMFBzbWRCU1BJR1lrZmYtbjdMcGZvSk44MUtZZVo0X3B6Z2hYZ0Fjb0FmYkJhSEZoeGpHUWpHcHhaQXhMclpXR1VUSmFfOHJlS3BjaDlhS1JrTnByVTBoR0o0LWNFVlc4WVczdVBVazlvX2JfLXFaR1dsYkJmQ0RGZk9qUGJiOUMwOGw3alFkZzNYa0o3T2NqT3ROR3VfZ29BcGszdndTNXJrVDl0UWQ4UzBRSjhvQXdhVmZkSlhfc3lwcTBiWi1Fc1RDR01tSEdDbEtzWEs4bDQ1NmM1cl8wLXBFcndnal80cVdXQkxHc2Vn?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -845,52 +845,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46092.53888888889</v>
+        <v>46092.51255787037</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kinderopvang ’t Toetertje in Borsbeek gesloten na klacht over oud-begeleider: “Dit sloeg in als een bom” - HLN</t>
+          <t>Store gallery: Dyson opens first UK off-price store at Bicester Village - Retail Week</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Childcare 't Toetertje in Borsbeek closed after a complaint about former supervisor: "This hit like a bomb" - HLN</t>
+          <t>Store gallery: Dyson opens first UK off-price store at Bicester Village - Retail Week</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 08:07:27 GMT</t>
+          <t>Wed, 11 Mar 2026 15:58:45 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxNQll6Zm5NS01XY2xnTlRRWEtoQzN0Z09wLW5yZGYyN1pDblNDS3RwU0JER0k5RXZjYmZIRzFTVnhrd1hjY3JycGg5V1ZBaE4zaUt4RkRRNmRTVTlWOHRueXV3RVVyZ3B4c1pjNWtqa0pXNFRxQzlRYXZjUWk5aGVFdV9BWU9FX3dMcnY2QkRiTU8wMTdnMEIzTW1hbTJ4QkI1Tk9ELUFvWEFFQjN1UDlSZkdoZHpoeUt1UGFYNFZxWE45WWhmYVV5aG5Ud3ltSEpxckZFbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxOMVhpenJ0TVlBcTRBZDRDUDhsS1VPNFAxU1pIVkZUYkhFQ0pVX2NBd0lDc0hFMF8wM0Z1SXpVQ1BxckNiQ2FlZm5uRkJHWHNvdjFydnJSb1J1YkFuVldDeUc5LV9hazhrdXE2TzczeEJsZnRMX0NnUkl4M1NmbVdHTXREalJWMnE0cFlKS1VZV2NKX0N0RW9NRW5hVlpNRnZvZEEwQkFkdEhrU0E?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -900,52 +900,52 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46092.33850694444</v>
+        <v>46092.66579861111</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Kindercarnaval in Schriek houdt vast aan kleurrijke traditie: “Confetti mag als het niet regent” - Nieuwsblad</t>
+          <t>Swiss Cult Bear St. Bakery Makes Its Debut Cookie Phenomenon To The UK: All You Need To Know - Travel And Tour World</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Children's carnival in Schriek adheres to colorful tradition: “Confetti is allowed if it is not raining” - Nieuwsblad</t>
+          <t>Swiss Cult Bear St. Bakery Makes Its Debut Cookie Phenomenon To The UK: All You Need To Know - Travel And Tour World</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 10:12:17 GMT</t>
+          <t>Wed, 11 Mar 2026 21:24:18 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgJBVV95cUxOcFRYRTNNZ1ZBeDhqY1RaSnlST1NCQXZYTFF5U2xaMXd4UFdwVkcySVRkS1A2MWRmckFuWVo4a0h3WUg0RUh3OF9LOGZTRFNWaW40SnM5LXpTVHNQTC1jNUI2S2paZVNvTVAwblZLN2loQ3BKb1ctUlJPcUhuVHhCM2NfQWFkaTBPZHZ5ZVpWbTBHSDNHZmZ6ZWtuR0sxMWdjYTN1a1d5VTZoNG0zOTlBRnl6cXNacTNBeFEyQUpwQ2FtOXR0R21UTTRRM2tVc0xyX2tUY3lLc0NmcnFOMV9YeDF3enNFbTYwclJ4OHcxYnNmVTB6SGtrR1R5cnROUFM0dkx2M1FOaktVT2xIWEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOOU9ROEZfY3VnX2lUbUFSV3pvdUlLR2ltUVBVZTZ5TUZiNWthX3gzSVpRa2pNNGxqOVk1dHlBSTZGNEtIZFpsVlNVX2ZuaVV0Qk9ZaWxHNTlSS1RMdU9idGpuTHQtLU1HZ0F2allaN2h5NXVsaXl1UEVGblZLN2JjczFmVklXTjRUTVdPOGFWa2kzRTM3UWJ2OTh1ci1qS1hVVWJxNDVYcnlGY25Gak9PUUJSQ3VFdjc4SlpDZG5DVzI0cFpBc0dES2dtckdHemt2cXVVVVhR?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -955,52 +955,52 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46092.42519675926</v>
+        <v>46092.891875</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Station Tegelen gedegradeerd van villa naar abri: beter bereikbaar, maar minder comfortabel - De Limburger</t>
+          <t>Zalando says AI is improving output, announces Levi’s partnership - Retail Week</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Tegelen station downgraded from villa to bus shelter: more accessible, but less comfortable - De Limburger</t>
+          <t>Zalando says AI is improving output, announces Levi’s partnership - Retail Week</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 08:08:21 GMT</t>
+          <t>Thu, 12 Mar 2026 07:02:46 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxQNU0yYXp6WHZoQ0tib3RFclhaTU91Y2VDS1dLYmhuRHVhZnhvVWdaU0lEYzlUWElCaXZBN0V0MHBYSG9xV1ZUTWtVZnQydWNjY1Z0Mkp6cFBwU0pTand2bW9lQWNDSTZfUGpDczRHUmFreU9NOFg3UDR0ZlJHX1huVHB6eEhVQTI4ODhJOHBqempsRXc2MjhUdExlR1FZdUV5cUV5RExEN0JhUGFRMUw4a1BEODRYd0U0SEhuVGhISmJwWTNNS0NtX19zdVdfcG1XdDB2b3U0ejNrOElkaTJ4MVRYbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQSGFqbTVlbXhzQWlNa0UyTkZpYVRCbXRhZ3hQSE5xUElUTDEtMG1BT0FBTm1nZGtxQ2hqQm10R3pYU3l0TmVIbkdVWklKcmJFUFVaZ0J3bC1wd3IzeEVEYmw5Um5MSzBld0RpMXY5MkFEcmNaMjZ4QWY1c2pBN0VSSjY0OE4xLUZJLWVDS0ZkN2FYZE5EbVRIc1owWURmblk3S19jN1RvV1lZcTg?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1010,52 +1010,52 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46092.33913194444</v>
+        <v>46093.29358796297</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Brilliant Meteor Seen From Passenger Plane: Viral Video Captures Rare Sky Explosion Near Brussels Flight - Travel And Tour World</t>
+          <t>Ook na explosie aan synagoge blijft CD&amp;V militairen op straat koppelen aan overbevolking in gevangenissen - De Standaard</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Brilliant Meteor Seen From Passenger Plane: Viral Video Captures Rare Sky Explosion Near Brussels Flight - Travel And Tour World</t>
+          <t>Even after explosion at synagogue, CD&amp;V continues to link soldiers on the street to overcrowding in prisons - De Standaard</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 10:41:47 GMT</t>
+          <t>Wed, 11 Mar 2026 11:30:00 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNS3ptNHhkandKaDN4RV9OZTlTd2J2ZFRLcmNzZjZTZFhBeDVNdGxrbVFBX3NTWjUwdXkzWUR3aVE1M0VxdjQ1VVotOE0tQUpIRXlnUFRrS2F2UmxOWkM5OWhFYWRpUGxTcHdCbWIxLWR6b1I3Z29lYjlNZG5jWi1oMjJsdDA5dThxM2I1cV83QW93VF9VMDRPWWlkZnhkcDJFYmZjTWZVNEcxVjR3Ny0wclJ5c01zUlRDTVdIZ2ExcVVhNEFnV0YyNDdQdkxBQ0dLa3lvdGNvWUJrNVFLMm1qLW5fTXdaNUk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPWm5INmp3TE9Ea094R1RRb3RfSWVWczhtdXFfZWFxNGh1MjJrZVRyRU1KWXVGcFJldm5GWVVQbG5yZENqbmpzaGtzZktaNU5NQ0NzMnRtRVpTT1lTNVNTbk12bHB2NWtpVUlJOUlZNTFUeDdlZUJuVlRpY1NGSDJBZlNyeGcwVEpiRjNxN1AxM2xyYVVxVGp0bkJjd2QtNVhpSnd3RmJOVmZfTW1RZHBJcmZxN0NqWjFkbXJvZkNpRFNlbjRDNEM5dnJRSUVZQkM2OU5oUm5mZHFSM2NhRVRzcjE5RG1SWFh1?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1075,42 +1075,42 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46092.44568287037</v>
+        <v>46092.47916666666</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>High Level City Belgium English</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>"Still Shaken": Flyer Posts Video Of Explosion Outside Plane Window - NDTV</t>
+          <t>Oorlog verhoogt druk: regering buigt zich vrijdag opnieuw over militairen op straat - BRUZZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>"Still Shaken": Flyer Posts Video Of Explosion Outside Plane Window - NDTV</t>
+          <t>War increases pressure: government will again consider soldiers on the streets on Friday - BRUZZ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 09:22:45 GMT</t>
+          <t>Wed, 11 Mar 2026 16:11:23 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNWHpaeEp2VkVkM2hyUDExVXA3RTc0Z2xsVlowaFR1cERoUzluZ3hNSGtJY3VtT056YzQtQlFYaHFPT3FmMTVrT05mWnN2aGYycXlyQmljTldMa2pXMWYzYzZxdlI5cnQzWEM2RHMxTUtWRVFBc3RubGlHQU93a21zU29mWGR2TWVLeU52RmNvaTJlb1VWS1NVM2QxYWRGa0JRNmNv0gGrAUFVX3lxTE9lLUs3NHk5S19jQVNHN2VoMHRBd3NQTTRoT1RtaXJVZU9WeWRzZXhkN3p6eVVlYTBkeF9GOTd1LVhJUGlqR3JoWTlLUF85S1ZiZ0NnU25sbVlEcV9ReVBnUU9jYWcxQmZSQTZ2TWFaZzcwUE9SUmk3aFFEcjc2dEl3TFI2VDM4ekJ5cm5WQ21IQjR4dEZBMGdYckprcWtwTVR1ZFR2bk0yalg4TQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxPTENYQ041bmJHcmhMVGtUX0l0M3hqaUlNYVFDWGFDUUNjNS00Tzd6aFM4MW5LUC1IOFZ5eGpMM0VhU0czNEpOd3RNNnRGQ1pQcDU1LTkxVzQwc2pIVDM4c0JGNUk5QWtVN3BzaXBFRVVrTHZXWGxlRG51VzNHZGR4RGthMWxELThRVk12cWFiRDVYY0ZSMzFDNUpFQUh2WDFzVmgyNHpCVC01ajBBNUwtRnNrQkVYcGdYN3MzdWxtT1pRcFRldzZzRG5BYWhIOUlt?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1130,42 +1130,42 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>BE:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46092.39079861111</v>
+        <v>46092.67457175926</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Antisémitisme : Une synagogue ciblée par une explosion à Liège - Bruxelles Dévie</t>
+          <t>Vijftigduizend bloemen op Tefaf Maastricht: ‘Twee keer per dag checken we elk exemplaar om te kijken of het nog mooi bloeit’ - De Limburger</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Anti-Semitism: A synagogue targeted by an explosion in Liège - Bruxelles Dévie</t>
+          <t>Fifty thousand flowers at Tefaf Maastricht: 'We check each specimen twice a day to see if it is still blooming beautifully' - De Limburger</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 12:00:42 GMT</t>
+          <t>Thu, 12 Mar 2026 07:52:43 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQVTljYTdkYnQtMWwyQk92d0JxejlzTUU1Nm1LR1BHcHJrUVpjSUJOQUtWWUhNTmFOcS1WWm9KcVJwX1k0Zl83dHU0UHQzYXRPYXU5UEZwMjc4YUdhQXVobWVJd083Q2VJSGdTX0Mtbm94ZEJiNUM2UzltVG40UUlkTjVKQnRwaUUxUE84QUNoSXJSQWlFM09UZHNiTVJmY0th?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigJBVV95cUxON2FIS1Z2S3FqVm1uLUJmRUE5a2RLS1FPRUdwOXNrV3F1RmQwNFVneXYyWnlONGkzMXIxY2x3Q3NaZl9CV0plQllyTDRPYkVZLUg4OUVPcm1sMHNiZjdzZ0lpX0xDWGthUG5fQjBTOUJGVmh0aWwxbjRUYVVId0QwcnhTSFJHSjluVWhlZmJQQ1Vha2N3aXR4YXMtbVhVaXhha1VUeS14NmFMbzdBTE9ETDRBX2tjeGpNbzB0QWRQakhpbkFIN244bk1WaUNTSEpBTzlOR0lSQzIzQ0F1azNfNFVhYUxabzJTc09jRWM2VjY5ZWpHczdKU3h6cGdNRHlHTzFTTHF1XzE0dw?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1185,42 +1185,42 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46092.50048611111</v>
+        <v>46093.32827546296</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>"Ces jeunes vont tuer quelqu’un si on ne fait rien" : la mère de Camilia, brûlée à la sortie de l’école, lance un appel - BruxellesToday</t>
+          <t>Centrum voor gezinsplanning in Brussel gevandaliseerd met anti-abortusboodschappen - Nieuwsblad</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>“These young people are going to kill someone if we don’t do anything”: Camilia’s mother, burned after leaving school, launches an appeal - BruxellesToday</t>
+          <t>Family planning center in Brussels vandalized with anti-abortion messages - Nieuwsblad</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 12:45:30 GMT</t>
+          <t>Wed, 11 Mar 2026 15:16:36 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNbVk5RFR6ekdyQzRndzJucmdEY1g5dy1FT05mcnlKejJwaEtpU25oU01QOURwUmFkcTI4NkYzeTFRV1RKUW1Ycm45d0x1bFgzTHdDVWJJM1pDa1AyMFRwWmc1REJVSjNmQmRxZTRiWE5yMGNRUGdIaTROVUxCVGtRLS1mOUZFSktkRnNyWEMyUTdjRmVKWUZCX2J0QVhaSWxpSVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxPMVJDM3JCNzgzbFZuSTVOSWR4V3h6UWstbW5aeW84M3ZTVkhDT2tXQ0xhTEhkRnQwMFNKbTNoeS01M0wzVU11d3g2Z2R3RUIzV2VCeGJkaURTQmlDNU1Sb3BIbTBLTVNLOFZLNm9sbks2UlVqSjByVy1LQ2hjUUJ3NlItT2d4TnA2RS1MWkxWVEFaQURwZkQ5aUVsSkN4RVVDZHNTbmhPM21jTUFiT0ZGck4wVVVMdGFYOVV1ZVdUbTZHbHNWcDEzSV8zYkxCYTgyOXN2bGU2SE5LNG1qUlE?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1240,42 +1240,42 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46092.53159722222</v>
+        <v>46092.63652777778</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>La Belgique docile : l'angle mort de Liège. Sur la récidive structurelle de l'État belge face à l'antisémitisme (Carte blanche) - 21News</t>
+          <t>Politie zoekt verdachte van poging doodslag tijdens oudejaarsnacht - Nieuwsblad</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Docile Belgium: Liège’s blind spot. On the structural recidivism of the Belgian state in the face of anti-Semitism (Carte blanche) - 21News</t>
+          <t>Police are looking for a suspect in attempted manslaughter during New Year's Eve - Nieuwsblad</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 13:22:28 GMT</t>
+          <t>Wed, 11 Mar 2026 10:36:29 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQVjE4cUhJNkMwUlBmdWZfOXlwa0tUU0tMVlBBajZlWU9fVUpENm04NFhqV0ZKUG43WDhsdEhTUHl5S3NDQUc2dk9PNk1scUJXSk5TNFczZHZySWI2VkVnTGEyTzk4Q2ZVdlVvYTc3VnBBV1Y0anNkc1BUVWxsS1BFNVNWUS1JWlg2bk9SZTBURVVFZ21VXzhRSHRaM1Z3TGxqSUE5MHVzUURxU3NJWGsxLTJoVW5YMi1xS2FKekkxZThBNjk4T2h4ZmI0eUZNRWQtTm1sOVBveGQ2QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi_AFBVV95cUxNLTVFdlhWbWZMMjdqaWlvajI2SW9FcDRrclVZUkVkRG82M0tUZ2FGV0I3dDV4dFkzSzczUmxDZjVyX25mNUpjR1kxaFQ3TmhHUEJMbzVvYm4xWnF1dngzYVBVaUt0b282bUd6aGJ4WFBtNWNFTWRrckpsV0VxMTEyV0lvWHFZaVdEbGFXczk1dFZiYUlyZ0FVZ2V4V1MyUFAxZndmWmYzblR5M3AtYl90NXVmbkpLMVBzUWlMZDM0b0wxdjhxN2ZsQUg4STRNZld0UW1IM2kySUpEUHhneU0yd21sVmdoem80Zmd6NnE2VHJkRHJNVEFYaDc3aGE?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1295,42 +1295,42 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46092.55726851852</v>
+        <v>46092.44200231481</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Engie ontmantelt oude windturbines op Europark Lanaken, Ecopower bouwt 4 nieuwe - VRT</t>
+          <t>Woningbrand op Demertstraat in Maastricht - AD.nl</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Engie dismantles old wind turbines at Europark Lanaken, Ecopower builds 4 new ones - VRT</t>
+          <t>House fire on Demertstraat in Maastricht - AD.nl</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 13:41:47 GMT</t>
+          <t>Wed, 11 Mar 2026 12:56:00 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNQnV0LXR3UnpaU2s0MVhyQUU0ZGJCOWd3dl9LLWZMQXNhMUF3d1p1UENxeFFBTGtwMWt3NlVjamxIbW55UldIZW81RGh0dFpVS3ozSDFZcDYzSDhlZmttTTNnNHNJdmdQVkFhXzQ3NC0yNG9DRjlTZWFGdXloZE03YkhtTVNyZlFzLXRSV3FtXzNPa2lSeG5QMEd3ZVFfQ21hbVlHM1YwdlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxONHVMdmRTVDlwYWMzM2hHeFVpQjBUaVI4alJjVUNqSW13ZnZKc2JDMDdyNW14bWRTUWMxa2x5MTBBSDVXR21oNDRfWFFiMnFqSU1xb0ZHbnpCT1RHTUxCS3BwNEZCN01uN3hLSkxJMV91dS01T0gySExGRk5WQkRkbWNhbE9ScjVxdGk3WGRZV3JfSWt6YWc?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1354,38 +1354,38 @@
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46092.57068287037</v>
+        <v>46092.53888888889</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Thales Alenia Space visée par une action d'activistes pro-palestiniens à Hasselt - DHnet</t>
+          <t>Brand op Op de Hoogmaas in Maastricht - Alarmeringen</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Thales Alenia Space targeted by action by pro-Palestinian activists in Hasselt - DHnet</t>
+          <t>Fire on the Hoogmaas in Maastricht - Alarms</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 11:55:00 GMT</t>
+          <t>Wed, 11 Mar 2026 17:45:59 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxOejN1S1hock02U2lpQ3pSd0ZHRDdSX0JjQ3ljb1VUcFViZVhza0M5UkszZDhpdHJiX1dnd3dneHdmU2dzaWl0Xy15enluNTlZOTZNYjF1dHQ1U0oxdXVBTi1HSzRuNDNVbXczbXQ5OGNWeW5jTEdKcmtKVkE3SGljY1VxbS1iQlFjSVQ4ZGdtV2c4eGRPUldOcnpFOF8xclBiQlNfcHlNX1kyWFc1UE5pcm5Qdld0ZnR2Rm51bGdkUWZYZzQ2aG5vcHFDbjZ3UlNCcmVrdGdfYVZpZThTSG9Da0RzWGRWZFAxekFnYmpoUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxQZ2t4UWpQX1lVNkExamZiMHE5ZHQ2Zmo3VUFtMVhkeE96SkFiVUtMOWNWMmhsUGZ1MGZTaGxGWGs1SUZtemQweWc5UDZyaHJxSnVlNkJFT0szSHF5bGVORE9mTXFaekh5Rzd2QzRLQ0ZhamdWR2lDZGtseHJpMjR0XzY2Y2ZnVWl1ci1uRG85STd5NmlNTXBvX0RoUXkwbS1OQTl5M0I1SlpyekJFYnpLSE96SVlvaTdzRFNYN3JVX3hTZkht?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1405,42 +1405,42 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46092.49652777778</v>
+        <v>46092.74026620371</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Six endroits en Belgique où admirer les cerisiers du Japon en fleurs - SoSoir</t>
+          <t>Grote delen van Dresden geëvacueerd na vondst van bom uit Tweede Wereldoorlog: 18.000 mensen uit huis gehaald - GVA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Six places in Belgium to admire Japanese cherry trees in bloom - SoSoir</t>
+          <t>Large parts of Dresden evacuated after the discovery of a Second World War bomb: 18,000 people removed from their homes - GVA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 13:09:00 GMT</t>
+          <t>Wed, 11 Mar 2026 10:13:29 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOMW9jWkNSd0d1elpkNllRWi10VnhmOGZBaXN2bl9qYjJvSnU2SlJ6N3NVS2ZrbTZoazg3RVNrV2Z4TmNlNEo4VUlydFROTUhvOVdBX05vX3FudjBxWXpTcDV0WW56TWJ5VThRNjhvWTZxR2c3Y3pDS3ZOb0FCcTFURHFDLXY1b1gxdlp1a3hoQTBzRDBlbnFFRTVoYTg3V2dvcVVObG1pSTdZN1NvZUdOaXVhYXJKYlFxMTJj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxQblg5QURSWTJjZWZsTEJZRUpxUDFHcEhrem1KazJISTV5TUlyeUp4REF4SlBkeUZ4Vy1HRXVvMHB4aWoyOWNocDA2aFdtTUdXTmxVRVRfNTlWVzVPZzA2WXBEMlp1aHVsNmFObnN3V2dEMTRHMV9mU1RGMjJqR2tqOHpnR25YcEtGWndOcWM1UUZkVERfcHhGajExSDYzZ0VYMk9lcG5lWG5lbjl6M0VDS3RnVWxDQU1INl9Ic3BKeVdDQ1N0bUROUGpuMUlmMS1fRnhwb1NzR3oyM21pM19ZSUY0bVBpbllU?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46092.54791666667</v>
+        <v>46092.4260300926</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Hausse du pétrole: en Asie, des compagnies aériennes ajustent leurs prix - Boursorama</t>
+          <t>Zijn de Iraanse sleeper cells al actief in België? Urgent veligheidsprobleem dreigt - De Morgen</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Rise in oil: in Asia, airlines adjust their prices - Boursorama</t>
+          <t>Are the Iranian sleeper cells already active in Belgium? Urgent safety problem looms - De Morgen</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 07:51:40 GMT</t>
+          <t>Wed, 11 Mar 2026 19:18:00 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxOT09qeTI1UmQydzhVLWFndU1xamwtTEY2bnRPNmhzcEZxalhyWGY5dHlGYXZGa1FVWkxBWU94cEtrNk9Yb1hZNTlubDFGbnJVVlZjTFFLTDlTSDhqeUtEekt1Z25SSU1UeEItLXVFMzRkaGlfMlVUNXgteTBkNTZ1YzIzQVU3WFNGM29nWE5IdGEtOWRCaGVLcjZPYWpjTzdKV1F3X2QyVG5aTVBYLXBaNWIwbkJWSzlGSy10SkJiRlhIYnZidnFRYVQ2OFpDRWdIdUoycVNiWkRFQnlaNHpSaThIWW9EUmfSAecBQVVfeXFMTk9PankyNVJkMnc4VS1hZ3VNcWpsLUxGNm50TzZoc3BGcWpYclhmOXR5RmF2RmtRVVpMQVlPeHBLazZPWG9YWTU5bmwxRm5yVVZWY0xRS0w5U0g4anlLRHpLdWduUklNVHhCLS11RTM0ZGhpXzJVVDV4LXkwZDU2dWMyM0FVN1hTRjNvZ1hOSHRhLTlkQmhlS3I2T2FqY083SldRd19kMlRuWk1QWC1wWjViMG5CVks5RkstdEpCYkZYSGJ2YnZxUWFUNjhaQ0VnSHVKMnFTYlpERUJ5WjR6Umk4SFlvRFJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxQbmJHLWc2MXQwUG9iOEhwV1lDdUJQNzN3bXI3VmZhU1dDVmZZOUNrSFFCMXR3MENveDlvdTd0YVF4M1lGVDVUWEtUZThqdGN0cnhDdV85MFdPYWFoWWduWjNlZGk2NHZTLVJQRUZEWUxHd1gyWWNGclNJRHoyOXljMkd5VXdvMUZiN2FkTG9nVld4T0M1NV9xSlRJNW9JeXc0X0puSWhqOW9lRkNIb1JYdlVxRno4NDlnUDhKNmg2ZEU?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46092.3275462963</v>
+        <v>46092.80416666667</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen English (fallback)</t>
+          <t>High Level City Belgium Dutch</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Margot Robbie debuts dramatic bob haircut and more celeb hair transformations - MSN</t>
+          <t>Verenigingen en gebuurten werken voor de derde keer samen voor Sint-Jozef Feest - Nieuwsblad</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Margot Robbie debuts dramatic bob haircut and more celeb hair transformations - MSN</t>
+          <t>Associations and neighborhoods are working together for the third time for Sint-Jozef Feast - Nieuwsblad</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 12:15:37 GMT</t>
+          <t>Wed, 11 Mar 2026 10:23:23 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxORjhwLTZKeGlTaC1KNmVuRVZ1V1lJcXEyLUJZOFNkTnc2TjZFVmdTUm9BVUFhaDFWMWVxWmUtSHhXdGtNTEtMWFp2N2dGTW9JZ25aY0FRNWJ5eDZrMjVpbkZtNHlTQlJPbHIza3J6aUVQNDlBWWRzZkZyZFU4VjBDTVhiY3ZXd3ZnY25jN2xrcml5Y0tVNi1MQzlyU25laVljSms5aXhjOGFPaHdkMnA4cE5nWWJmcnBkUXRieGFUV3FuWk0wNWVSdU9UcHA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxOZ3RELUxSVHlLMGV4c3dOVTg5VFFkWDRVWFAyZlBERGVVQ05nLW1RZldzb3ZfUFZEZlNXT0gyODFIM2ZzZkpETW9FYTRlSkRHZnd1enNONkw0SnExaW92cFJadGFHMTVBNWlmSmQ3N1A3Wnp1Y0NLbzZHM2pVUzlYcFZ0QzZwSFIxUHJoMHlGbFgyZm1rQmRHdXhnLWtkNThzTU5GZFRzYnJfUTJOWk5HZlJZMUZOc3pVYjI5ZDB6dzUxMTVMVkw1cllBQWZOQzFKc19VaHFxLUpMbGRMWmJzVEhKcF9QOVZyQWpr?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1560,52 +1560,52 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46092.51084490741</v>
+        <v>46092.4329050926</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Einsatz in Würzburg: Mann versprüht reizende Flüssigkeit in Mehrfamilienhaus - inSüdthüringen</t>
+          <t>Stabbing in Belgium-Luxembourg border ends in arrest - The Brussels Times</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Operation in Würzburg: Man sprays irritating liquid into an apartment building - in southern Thuringia</t>
+          <t>Stabbing in Belgium-Luxembourg border ends in arrest - The Brussels Times</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 11:30:47 GMT</t>
+          <t>Wed, 11 Mar 2026 20:53:08 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNa01iMnpqeWdYN2dFNWxZMXRzQ1JrUlFIUVJJUU1EV1RNVU0zcldmQXFQVVZ0MFhSVWRUNlFTalNvWVcyc3piNGFVZy02WGIwaEN4Ui1EVHdDUFBEMUlTT0NIRnMxa202RVdPc3pMamU4NDlOQ0pSVjRTTGprdmFiN0VjRDNIOVRxNHpkSUw2OEx4cG5SUVhjd2tCdmYtRVpYMkIwVFFiOE5sWFNQa1FiVlc2OTVoeXh1WGlRbjNFaEoxMS1QTFQ5a00weW85YkpCZklGWElNU1hUV0t6SjZVNjExUTF3TkdFQUp0ZjVhRDI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxQNnd5U0VsaF9CWk5TSWpMa1U0dVpvTWdlX2toaUhZdlJYbm90S1dmQURpaWtaN1hWMXpSRHJGRGhvSDRLdkdteTdRczhsQnRFQVVWTlgxeUx1dGhDWlpvaU9Meng0b2FDWjM2MUw0Q085QlFNMXQ1SnRjMTZ5U21yWUZGYzRVeFpwUTI4Zktqb2FfM0ht?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46092.47971064815</v>
+        <v>46092.87023148148</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Brilliant Meteor Seen From Passenger Plane: Viral Video Captures Rare Sky Explosion Near Brussels – Belgium , Flight - Travel And Tour World</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+          <t>Brilliant Meteor Seen From Passenger Plane: Viral Video Captures Rare Sky Explosion Near Brussels – Belgium , Flight - Travel And Tour World</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 09:21:02 GMT</t>
+          <t>Wed, 11 Mar 2026 10:41:47 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxNS3ptNHhkandKaDN4RV9OZTlTd2J2ZFRLcmNzZjZTZFhBeDVNdGxrbVFBX3NTWjUwdXkzWUR3aVE1M0VxdjQ1VVotOE0tQUpIRXlnUFRrS2F2UmxOWkM5OWhFYWRpUGxTcHdCbWIxLWR6b1I3Z29lYjlNZG5jWi1oMjJsdDA5dThxM2I1cV83QW93VF9VMDRPWWlkZnhkcDJFYmZjTWZVNEcxVjR3Ny0wclJ5c01zUlRDTVdIZ2ExcVVhNEFnV0YyNDdQdkxBQ0dLa3lvdGNvWUJrNVFLMm1qLW5fTXdaNUk?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46092.38960648148</v>
+        <v>46092.44568287037</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Eisingen: Motorradfahrer flieht vor der Polizei - Radio Gong Würzburg</t>
+          <t>"Still Shaken": Flyer Posts Video Of Explosion Outside Plane Window - NDTV</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Eisingen: Motorcyclist flees from the police - Radio Gong Würzburg</t>
+          <t>"Still Shaken": Flyer Posts Video Of Explosion Outside Plane Window - NDTV</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 13:00:00 GMT</t>
+          <t>Wed, 11 Mar 2026 09:22:45 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOWFdFb3JVaVBTR0Nzb2ZpOXktTF9lbkU4SVdmX3B3S08tN1d1blhTSFdUbEJFT2tzTXNGcHFzNDd0aFV2cGRtenVDTTAxeEM2b3pOVnpLdXItVWoxQkRIMmtOaHNZYTBrY1RIRGdrRnRoU040QXMyZGoxSE9JSDh0MW5BVV9tXzQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNWHpaeEp2VkVkM2hyUDExVXA3RTc0Z2xsVlowaFR1cERoUzluZ3hNSGtJY3VtT056YzQtQlFYaHFPT3FmMTVrT05mWnN2aGYycXlyQmljTldMa2pXMWYzYzZxdlI5cnQzWEM2RHMxTUtWRVFBc3RubGlHQU93a21zU29mWGR2TWVLeU52RmNvaTJlb1VWS1NVM2QxYWRGa0JRNmNv0gGrAUFVX3lxTE9lLUs3NHk5S19jQVNHN2VoMHRBd3NQTTRoT1RtaXJVZU9WeWRzZXhkN3p6eVVlYTBkeF9GOTd1LVhJUGlqR3JoWTlLUF85S1ZiZ0NnU25sbVlEcV9ReVBnUU9jYWcxQmZSQTZ2TWFaZzcwUE9SUmk3aFFEcjc2dEl3TFI2VDM4ekJ5cm5WQ21IQjR4dEZBMGdYckprcWtwTVR1ZFR2bk0yalg4TQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46092.54166666666</v>
+        <v>46092.39079861111</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Flucht im Landkreis Würzburg: 16-Jähriger prallt bei Verfolgungsjagd gegen Streifenwagen - Neue Presse Coburg</t>
+          <t>Le CD&amp;V persiste à lier les militaires dans les rues à la surpopulation carcérale, malgré l’explosion devant une synagogue - De Standaard</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Escape in the Würzburg district: 16-year-old crashes into patrol car during chase - Neue Presse Coburg</t>
+          <t>The CD&amp;V persists in linking the soldiers in the streets to prison overcrowding, despite the explosion in front of a synagogue - De Standaard</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 12:35:47 GMT</t>
+          <t>Thu, 12 Mar 2026 03:31:41 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxQektlYjRseWd4eWFzb0Y4RkkyU1k5ODZsTmFsVHNBaVowbnBCU2tMWXU5X0ZDVUhQUzRZYzFKMG4zWjJrTWViLVJVOW5mWDdpcTNKcUYtdnBaOE55dXhGTzU2akVVZ1RtLUlLdjJJbHZtczRlaVFtNFhUbTRzTFF3SVRhZE9pMzVEWDNNN3F0OUttSjRja1htTkQyd05vaXplM2pEd3dmQlVKa0hzMWszSDZaM2Zjd2ZfcURfOElYYlhLbzE4QnFRb0JTQ1J6YmxVU2FLc0tkNFhqbFZXXzg5b1g3WmdHYW9aZWxIR2Q1WlJCQWJpbWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-AFBVV95cUxOUEhlTGkzRklsbzMyYllvQnV1SDdnZ3NYaU04QVdFcGM1bHg1OXhtbE5uUlFHQWZ1elZ1TVkyLVB3UDF0d25XcXhJQUR1VG9rZlJBNFlTMUtGRm03U2M3T2hvRFQ0ZzEwTHZVTUgxTll0bk1GLVAzd1RXT0VTbnZId3RWei1yUTgxaVZHaVpuNTgtOElJZkIwZFIwWUNMRGtzTjFCcVZXejU4LUVNbnNNQWV4RlU2eDdFMFpFZVNjOEJoZ0I0LVBVTnhoMVZ2czcxaXJmUGsxTHcwMktTcWhLeVg3bHBmWHB4U2dXeVdBNVFpMnJYcW5ybw?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46092.52484953704</v>
+        <v>46093.14700231481</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Polizeieinsatz Aschaffenburg / Bamberg / Schweinfurt / Würzburg, 11.03.26: Zoll-Einsatz auf Baustellen in Franken - Bilanz des Hauptzollamts Schweinfurt - News.de</t>
+          <t>Antisémitisme : Une synagogue ciblée par une explosion à Liège - Bruxelles Dévie</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Police operation Aschaffenburg / Bamberg / Schweinfurt / Würzburg, March 11, 2026: Customs operation on construction sites in Franconia - Balance sheet of the main customs office in Schweinfurt - News.de</t>
+          <t>Anti-Semitism: A synagogue targeted by an explosion in Liège - Bruxelles Dévie</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 11:33:02 GMT</t>
+          <t>Wed, 11 Mar 2026 12:00:42 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQS2JkYzM1WUh3a0hOZmNfQXdqb2VWWHBvOHdCcVRMZTg4dmxxangxWkFrREZoY0JldW9uOVlnUkk2NTBrQnl5QVhYNjR5a1p0Y0wtd2VjdV85bS13RFZOU2ZWRVB0cGJKODV1WlpEb1hmZjdjaFBYNXVyUy1JWkhrWHRjLThudjNMa3FhbjNqeDg4eEFjRzhSY2tEcmVyQXRnM3ptbTVnd2IwX0FSVEJ1dDdqOXB3R3pfUFM2WTBWc1kxZWPSAcgBQVVfeXFMTVFBLTBrb05abEdaVk53VEZ6STNPRjQ5WVhjY1dPZmU2ajBieC1ScmdTMjVQWGdNdHlhWUFncElkTFQzalpNNDk0MXVULTMxc1hyUVhLYWIzVlc0OWFrR2pZSFJObmxDX0tOY3lCYTA5T1FLQkZRTl9pYXlUV1BJUTRsZmlfVTNqcEJmLVBpdzJHejJsTE9XcWl2aXlzMHBWdE9Nd011ZXdpSzZNbGFJU1F3VGd4YTAtbXV6YkpJY0ZER19jM2RjcW4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQVTljYTdkYnQtMWwyQk92d0JxejlzTUU1Nm1LR1BHcHJrUVpjSUJOQUtWWUhNTmFOcS1WWm9KcVJwX1k0Zl83dHU0UHQzYXRPYXU5UEZwMjc4YUdhQXVobWVJd083Q2VJSGdTX0Mtbm94ZEJiNUM2UzltVG40UUlkTjVKQnRwaUUxUE84QUNoSXJSQWlFM09UZHNiTVJmY0th?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46092.48127314815</v>
+        <v>46092.50048611111</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Village Wertheim (fallback)</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Zoonotic Viruses May Not Be “Special” Before Spillover - Technology Networks</t>
+          <t>Journée européenne des victimes du terrorisme : la Belgique commémore les attentats de Bruxelles - BruxellesToday</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Zoonotic Viruses May Not Be “Special” Before Spillover - Technology Networks</t>
+          <t>European Victims of Terrorism Day: Belgium commemorates the Brussels attacks - BruxellesToday</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Wed, 11 Mar 2026 09:02:26 GMT</t>
+          <t>Wed, 11 Mar 2026 15:55:00 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPYXU5WTNhYVBVM2x6R2NJY2JWNGM4T3hOVHFYUU9FMmFvSVJGeFRFZWtGU3YzcU9TOGRhUXRsbkJ3OUpDSjZyMV9QUXREblpqc1JyVTFjaFM4TDBBS0ZIQWVpdVdTVE1abWROMXFldjBsOXJYMGpuN3lQWVlwWTRlUHItZ19QT0NmaEhYWjhtVDMtNzYydEduUkRBdG04dXVVdExBRg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxOU2NCY21Gek5zVm84SDZNVjRnQkQ4UTlhekJULWZIUzVqNThuMmV2RVVCQlJybmlCaldndXJDbTd2OGdlSXNpc1lFUWtrTG16ZjdtQVpDbnBWYzRUQ1VTX2J2Mm80cWZBb0pJTnFJLTJCTzQ1dktpNFZFTVhnMWJwcWJuVXhLeWVBQzA1NV9wTTdxWE5tZGZfVkZVdjZwamRMV2EtZUJpOXA2SF9lQml1Y2VGQXZlUS1lVXdoZlVUNENXbklpcGVKUnFRblhyd01rYkFXNll3?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,76 +1890,2441 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>en-GB</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>GB:en</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46092.37668981482</v>
+        <v>46092.66319444445</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>La Belgique docile : l'angle mort de Liège. Sur la récidive structurelle de l'État belge face à l'antisémitisme (Carte blanche) - 21News</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Docile Belgium: Liège’s blind spot. On the structural recidivism of the Belgian state in the face of anti-Semitism (Carte blanche) - 21News</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 13:22:28 GMT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQVjE4cUhJNkMwUlBmdWZfOXlwa0tUU0tMVlBBajZlWU9fVUpENm04NFhqV0ZKUG43WDhsdEhTUHl5S3NDQUc2dk9PNk1scUJXSk5TNFczZHZySWI2VkVnTGEyTzk4Q2ZVdlVvYTc3VnBBV1Y0anNkc1BUVWxsS1BFNVNWUS1JWlg2bk9SZTBURVVFZ21VXzhRSHRaM1Z3TGxqSUE5MHVzUURxU3NJWGsxLTJoVW5YMi1xS2FKekkxZThBNjk4T2h4ZmI0eUZNRWQtTm1sOVBveGQ2QQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>46092.55726851852</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Dix ans après les attentats du 22 mars, Bruxelles rend hommage aux victimes - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Ten years after the attacks of March 22, Brussels pays tribute to the victims - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 12:41:00 GMT</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxQMHNjeTd1X08tWU0yaVZoa0pxTDNjSkotX3l2bXJNR3JzbGNnNzRvODNMb0VGazUzajBlLW9JMDZmU2lTYkJLTThZMTJFcEtFbWtISWdNN1NGTGFrTGNLbFFOa3kzcmxRSWpEMFAtVHU2b1h4SVhwcXhHR1dpVkdkMlpRRmRBblE2X3B4Z3pZeEI4czREZ2xwbzZTMk92SU5hNU03U1YyS0c3enhsV3NxWjlVV3E?oc=5</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>46092.52847222222</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>"Ces jeunes vont tuer quelqu’un si on ne fait rien" : la mère de Camilia, brûlée à la sortie de l’école, lance un appel à témoins - BruxellesToday</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>“These young people are going to kill someone if we don’t do anything”: Camilia’s mother, burned after leaving school, calls for witnesses - BruxellesToday</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 12:45:30 GMT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNbVk5RFR6ekdyQzRndzJucmdEY1g5dy1FT05mcnlKejJwaEtpU25oU01QOURwUmFkcTI4NkYzeTFRV1RKUW1Ycm45d0x1bFgzTHdDVWJJM1pDa1AyMFRwWmc1REJVSjNmQmRxZTRiWE5yMGNRUGdIaTROVUxCVGtRLS1mOUZFSktkRnNyWEMyUTdjRmVKWUZCX2J0QVhaSWxpSVE?oc=5</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>46092.53159722222</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>l’Iran a commencé à mouiller des mines dans le détroit d’Ormuz - Le Club de Mediapart</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Iran has started laying mines in the Strait of Hormuz - Le Club de Mediapart</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Thu, 12 Mar 2026 00:23:53 GMT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNT3VNdWpVTkFESFRJYTZiODBXN1hkdm9RTUpwUV9OTE5ObURocjktZnRyd1NLY3hiY0NvNkQzcEx6SlVZTXNKZllGSnlsZXl4VmVWeVR3N0lkSUdUMjREZFFRY3dpRml2eVhHd0tzcWZ4clRiQzJfV3dOeDhRbzFSel9wNUZ1dFQ3T1VfbHFScFY1YXp4WVI5X3BHekpmU2VQV1ctWmQtZ1ZCeXJyOHRlRA?oc=5</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>46093.01658564815</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>High Level City Belgium French</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Agression israélienne meurtrière contre le Liban : la politique de la terreur - Le Club de Mediapart</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Deadly Israeli aggression against Lebanon: the politics of terror - Le Club de Mediapart</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 10:21:31 GMT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQTnZ3OFFET05SVUk4RUFjclB6VXJlUjZjMFVRTThyNGROb3JSU0ZxR3V0UEVNc2ItdHVlc19UTXY5UTBmSGxiVlVVYVd3VTd1TjNQS2hOY3M1a1MwRG5oQm55YWZwSktZUi14X2FaZ2RxRXNTSVBXbHlFX2RnalRkY2tVQ0RtRXFtNXNuejROcVFrWUJCX1QwT2Fma0c1Mmlnc1Y1b3A3WU9McHpQUDRoWF84MVNpNmlkbmN4V0dtdDRzRDhKcjdF?oc=5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>46092.43160879629</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Hangjongeren teisteren winkelcentrum: handelaars schakelen politie in - made-in.be</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Loitering youth plague shopping center: traders call in police - made-in.be</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 16:20:31 GMT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQSHAwMk9VcXhsMHJBSjRnX2h3QkQwVHBDR1B6MnVpaTJQeWh6b3RBazdFQ01HaXFBZGRPYTZrOUozOGp2MHFPWW1IR3gtdzYzNHVXRHRxRmp1UmxlQTdWNlNySmxvazlZeS1xQ3gwSGptc1FQUFBRMEpXQmhrYWNmcG5zZDczTHowQ0p2aTZOWUE5VVZTSXRxWi1OWUM4ZGFTWFE?oc=5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>46092.68091435185</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen Dutch</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Engie ontmantelt oude windturbines op Europark Lanaken, Ecopower bouwt 4 nieuwe - VRT</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Engie dismantles old wind turbines at Europark Lanaken, Ecopower builds 4 new ones - VRT</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 13:41:47 GMT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNQnV0LXR3UnpaU2s0MVhyQUU0ZGJCOWd3dl9LLWZMQXNhMUF3d1p1UENxeFFBTGtwMWt3NlVjamxIbW55UldIZW81RGh0dFpVS3ozSDFZcDYzSDhlZmttTTNnNHNJdmdQVkFhXzQ3NC0yNG9DRjlTZWFGdXloZE03YkhtTVNyZlFzLXRSV3FtXzNPa2lSeG5QMEd3ZVFfQ21hbVlHM1YwdlE?oc=5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>BE:nl</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>46092.57068287037</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French (fallback)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Cross Car : les favoris déjà au rendez-vous de Maasmechelen - SpeedactionTV.be</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Cross Car: the favorites already at the meeting in Maasmechelen - SpeedactionTV.be</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 20:01:23 GMT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxORlFCaWFyQ3RJOENaNnBuT3RPLVVBNjlvVldrZGxYTUlnUFdoQTVsN280UXdKamlEYTdCc0pyZXlKTDBwbDJQcW5JM0pxMDFjUW1mWm51ZGJyWm5iMTNzX2tSa1FKSXdWSHR5TkRqdUs2c0J5dDNjaXZxOVBrd1hxdUJiZWp4bWk2RUhwaEZqUzhjTHZJTC1JQjE1VGg1X3FlQUE?oc=5</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>46092.83429398148</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French (fallback)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Six endroits en Belgique où admirer les cerisiers du Japon en fleurs - SoSoir</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Six places in Belgium to admire Japanese cherry trees in bloom - SoSoir</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 13:09:00 GMT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxOMW9jWkNSd0d1elpkNllRWi10VnhmOGZBaXN2bl9qYjJvSnU2SlJ6N3NVS2ZrbTZoazg3RVNrV2Z4TmNlNEo4VUlydFROTUhvOVdBX05vX3FudjBxWXpTcDV0WW56TWJ5VThRNjhvWTZxR2c3Y3pDS3ZOb0FCcTFURHFDLXY1b1gxdlp1a3hoQTBzRDBlbnFFRTVoYTg3V2dvcVVObG1pSTdZN1NvZUdOaXVhYXJKYlFxMTJj?oc=5</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>46092.54791666667</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French (fallback)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Thales Alenia Space visée par une action d'activistes pro-palestiniens à Hasselt - DHnet</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Thales Alenia Space targeted by action by pro-Palestinian activists in Hasselt - DHnet</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 11:55:00 GMT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7wFBVV95cUxOejN1S1hock02U2lpQ3pSd0ZHRDdSX0JjQ3ljb1VUcFViZVhza0M5UkszZDhpdHJiX1dnd3dneHdmU2dzaWl0Xy15enluNTlZOTZNYjF1dHQ1U0oxdXVBTi1HSzRuNDNVbXczbXQ5OGNWeW5jTEdKcmtKVkE3SGljY1VxbS1iQlFjSVQ4ZGdtV2c4eGRPUldOcnpFOF8xclBiQlNfcHlNX1kyWFc1UE5pcm5Qdld0ZnR2Rm51bGdkUWZYZzQ2aG5vcHFDbjZ3UlNCcmVrdGdfYVZpZThTSG9Da0RzWGRWZFAxekFnYmpoUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>46092.49652777778</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French (fallback)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Beveren sacré champion de Challenger Pro League malgré un RWDM accrocheur - L'Avenir</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Beveren crowned Challenger Pro League champion despite eye-catching RWDM - L'Avenir</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 21:05:00 GMT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7AFBVV95cUxPU25yUmxsUFJ1SlFvY0JrdnZWUXY3LURHTkN0WUtlc0lvMHNTeFo5Yk16RC1CUWEwS04zWXhyMHVoTjJraGQ5RjlLNnpjZUZZYWV3WUJldEhpSFd4dk15eTUxalBvNkpLQm41akNJbUxVNFhyLWFoR19GamFhblFaZ2x6LTlvcU9ZWGgtby1wYncxRElWZEwwaG05ay1rajlHaGxaWExRN3lKdXd5QnRkVWtJdDkzMW5FNmQzYTlfS2ZqTTZvR1paWUdHUHNBd0NCUTAxU3M4b182enNKVkVHVmlXcF9RSnhlTmF4Vg?oc=5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="n">
+        <v>46092.87847222222</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen French (fallback)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Une mère et son fils arrêtés pour menace d’attentat à Saint-Trond - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>A mother and her son arrested for threatening an attack in Saint-Trond - 7sur7.be</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 18:03:00 GMT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQZ3lOalV3NXdXQ0FqVnU4M1ZxQ01KMnBaUS1yU090ZWVKOWZycXhoNm0zTHF2SE5CcGJaSGQ0RnNNZWxyRXhHUWl6ZWNNWVh1Q3diZE1lWGZnU09INThaTnlhR2hIWERyS1JLR2xHZWRoSUpmc3BQWkJfLXoyS1ZQN1hwdEJMbFlMZ0VUNHF6bmtPNUhsZmNfcTljNzhVWUdVQWVyM1JwNA?oc=5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>BE:fr</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="n">
+        <v>46092.75208333333</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Margot Robbie debuts dramatic bob haircut and more celeb hair transformations - MSN</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Margot Robbie debuts dramatic bob haircut and more celeb hair transformations - MSN</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 12:15:37 GMT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxORjhwLTZKeGlTaC1KNmVuRVZ1V1lJcXEyLUJZOFNkTnc2TjZFVmdTUm9BVUFhaDFWMWVxWmUtSHhXdGtNTEtMWFp2N2dGTW9JZ25aY0FRNWJ5eDZrMjVpbkZtNHlTQlJPbHIza3J6aUVQNDlBWWRzZkZyZFU4VjBDTVhiY3ZXd3ZnY25jN2xrcml5Y0tVNi1MQzlyU25laVljSms5aXhjOGFPaHdkMnA4cE5nWWJmcnBkUXRieGFUV3FuWk0wNWVSdU9UcHA?oc=5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n">
+        <v>46092.51084490741</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Eileen Gu’s Shirt Is Held Together With Just a Few Buttons Amid PFW - mandatory.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Eileen Gu’s Shirt Is Held Together With Just a Few Buttons Amid PFW - mandatory.com</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 20:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOQzh0VVZoSkIxU0R5Y0pCV2cyekJkS2hfUlFIVnRfeThVajRlTE8xR29rM2RVQ1FjclFjamt3T2RQT3BtVnV4Q2dteVBwRWo2QWt4eGlCR29BX2lIT0Q0UUVfamMzMlRlbnUtQ1RuUWVTZzJpcElYZmZpQ0hmdWFmX2VlTER5U2FkcWpRbHNGOXk1WnUwYURZQTZtYjZwOElzTHh3btIBqgFBVV95cUxNYTB3a3I2eldBbmE5bEpXR2taSWpKZllyRERuTnJTRTFXMkQ1VDV6TjBobGtndzZ4X01iX2lxcFdUY24zcXhXb2NNUEF1QmpkTjhQdHZLeHFyU3VWckFXUDZITml6aUpsb0NmN2t4OThwQ2FYUnowWWJyTzlwUEdNWWVob0dRaGdKamZlWWRBejZaZ1g2c0c0SGJUbl9DNkpBTzJ3LU16TGp3Zw?oc=5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>46092.83333333334</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Local Town Maasmechelen English (fallback)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken")</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>How Oprah Winfrey's weight-loss journey led to a dramatic new look at Paris Fashion Week - IOL</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>How Oprah Winfrey's weight-loss journey led to a dramatic new look at Paris Fashion Week - IOL</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Thu, 12 Mar 2026 07:04:05 GMT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPbWY4V3BRX2M0ZmtWNWdtLVVjN3FBVXREVE43RU9WWDdwZHV1b25BOUpRcVlIV3pvdDVDREhIWWEtVEMycnJiQ0VNNktWczM4NTMzZ09vNjVSdE5qNE1hcGE0cjcweWhYc29CcGhVXy12UnA5SXc3VFMzT0JUbDBFSlcwNmFhWnNxSHdZZlVPeV8wRnFhM19rY0JKOUlYcFc5UDFjcGtMSk9RS1YwWEJKTTBkWk5pcWN5T0liSGVJdWVCSGVxZE5fNERMS0RsZG84Q0FTdm5QYw?oc=5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>46093.29450231481</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Einsatz von Polizei und Feuerwehr - reizende Flüssigkeit in Mehrfamilienhaus in Würzburg verteilt - main-echo.de</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Deployment of the police and fire brigade - irritating liquid distributed in an apartment building in Würzburg - main-echo.de</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 10:11:43 GMT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6AFBVV95cUxPZ2dxYWRENFFBbDM5SDBVNVRORC1qa1VnWURTWm9RNktXX1hvcG9OVXpObG5VNW40SS1RYmo1WTNxN0g0TTBRVll5NEZqblIwUEcwODBDTTlMNkxnUzVlN0RsQ1NCWm1saEpudU9ZaDliZDM2ZGtNeUlocGs0TkNJMGJpX2tCN0g3eHk1T1Bab29TU3l5LWtDeHA5WnVPb01pQ3NUV2xSTVBWaDBnXzg3TmgwWUV3Qkc0cHBiUy1XSVduekQ3UTM0WDdQS3VHdHItRmktREc1Z2NDX05NS3hUNDVTMkRpRGFw?oc=5</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="n">
+        <v>46092.42480324074</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Flucht im Landkreis Würzburg: 16-Jähriger prallt bei Verfolgungsjagd gegen Streifenwagen - Nordbayerischer Kurier</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Escape in the Würzburg district: 16-year-old crashes into patrol car during chase - Nordbayerischer Kurier</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 12:35:47 GMT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxNcF9QNXhGRkh4NGxuc1pTbWhaMEpOVS1MX3FWZ1pEallEQW9Mc3RuM0lRYU1xZGdGLVFZSWF1ZzZRaDRDY1NGeFFBS2ZOUk14OHUyMjVwZHBnRFJScVJfMVlqUmlLcFg1QmRKbFREU1ZFeDlIQ2xtbVczMTlVSlN6R2JPc2tvVUlnTVFwSEg1TFRqZTgxeGFTLXkyeS1WOExYcEhxdlZzbXV1VXlPcFNjMV9CcWJjRFhzNmpoUzhZajFQaFhGeXluaS1LYzJKeHhzc25XcUItdHlFT3otTWl6SmliTm9aSmY5cFRXR0RvWkdXQQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="n">
+        <v>46092.52484953704</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Eisingen: Motorradfahrer flieht vor der Polizei - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Eisingen: Motorcyclist flees from the police - Radio Gong Würzburg</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 13:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOWFdFb3JVaVBTR0Nzb2ZpOXktTF9lbkU4SVdmX3B3S08tN1d1blhTSFdUbEJFT2tzTXNGcHFzNDd0aFV2cGRtenVDTTAxeEM2b3pOVnpLdXItVWoxQkRIMmtOaHNZYTBrY1RIRGdrRnRoU040QXMyZGoxSE9JSDh0MW5BVV9tXzQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="n">
+        <v>46092.54166666666</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>in-und-um-schweinfurt.de - Schweinfurt Main-Rhön - in-und-um-schweinfurt.de</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Thu, 12 Mar 2026 01:52:09 GMT</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTE03RUZJdVVWTG5jTlA1R0dmc2YyQ3Z2S1ExYmhkN0FENFJGamUwenJsSFFPWGpKc3B2aFBaeHRYVDR3aWM1SXg0YWZFVDk0N3d4a0Jz?oc=5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="n">
+        <v>46093.07788194445</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Einsatz in Würzburg: Mann versprüht reizende Flüssigkeit in Mehrfamilienhaus - inSüdthüringen</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Operation in Würzburg: Man sprays irritating liquid into an apartment building - in southern Thuringia</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 11:30:47 GMT</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxNa01iMnpqeWdYN2dFNWxZMXRzQ1JrUlFIUVJJUU1EV1RNVU0zcldmQXFQVVZ0MFhSVWRUNlFTalNvWVcyc3piNGFVZy02WGIwaEN4Ui1EVHdDUFBEMUlTT0NIRnMxa202RVdPc3pMamU4NDlOQ0pSVjRTTGprdmFiN0VjRDNIOVRxNHpkSUw2OEx4cG5SUVhjd2tCdmYtRVpYMkIwVFFiOE5sWFNQa1FiVlc2OTVoeXh1WGlRbjNFaEoxMS1QTFQ5a00weW85YkpCZklGWElNU1hUV0t6SjZVNjExUTF3TkdFQUp0ZjVhRDI?oc=5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="n">
+        <v>46092.47971064815</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Polizeieinsatz Aschaffenburg, 11.03.2026: +++ Aktuelle Öffentlichkeitsfahndung +++ - News.de</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Police operation Aschaffenburg, March 11, 2026: +++ Current public search +++ - News.de</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 19:37:01 GMT</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQeUZidWwyWnI2WDJaYjdXajZSTkZVT05ZcnVsT18tUmFxTHlCS1dMLWhfaWVFQ0VWWG5tcFhQNEpqYnRRVE05eU54ZDBvZkU1VUFwVEc5aWtwdWgteVAyYWFVOWw4M1VxdlltZU9wVzZ1NDJHbTdFeFJDeGlaOWN3YVBLX3l5V3RiN3hzQ1ZadG1hLWJtbjFVRE4zdEdaVV8xN3lGenhtMEIyLVloNXdRZUg0d9IBuAFBVV95cUxNM2VMRUFETFFVQ1ZlZnFCV0dZQ0hkeHNpd3dkWlg1UUdGNEZpbE9FVklHSVhkODdON3VjcXctZ0k2emhNNVRqRUNEQmlpaHlMNWh0YjBJZHo3VVpBU0NNajFXRC14S3R0N2ZMMlUwbEFaVWNiZkdVWnNiNGFjdHgzT1o3N2JIRlhzdnJXNjhqTEx1Zk9wZ0NOckpqNHFYSzVHbnRKLXhMSFR6WjBfc0x0WXdlSWxXOWR0?oc=5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="n">
+        <v>46092.81737268518</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Local Town Wertheim German</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Polizeieinsatz Aschaffenburg / Bamberg / Schweinfurt / Würzburg, 11.03.26: Zoll-Einsatz auf Baustellen in Franken - Bilanz des Hauptzollamts Schweinfurt - News.de</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Police operation Aschaffenburg / Bamberg / Schweinfurt / Würzburg, March 11, 2026: Customs operation on construction sites in Franconia - Balance sheet of the main customs office in Schweinfurt - News.de</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 11:33:02 GMT</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQS2JkYzM1WUh3a0hOZmNfQXdqb2VWWHBvOHdCcVRMZTg4dmxxangxWkFrREZoY0JldW9uOVlnUkk2NTBrQnl5QVhYNjR5a1p0Y0wtd2VjdV85bS13RFZOU2ZWRVB0cGJKODV1WlpEb1hmZjdjaFBYNXVyUy1JWkhrWHRjLThudjNMa3FhbjNqeDg4eEFjRzhSY2tEcmVyQXRnM3ptbTVnd2IwX0FSVEJ1dDdqOXB3R3pfUFM2WTBWc1kxZWPSAcgBQVVfeXFMTVFBLTBrb05abEdaVk53VEZ6STNPRjQ5WVhjY1dPZmU2ajBieC1ScmdTMjVQWGdNdHlhWUFncElkTFQzalpNNDk0MXVULTMxc1hyUVhLYWIzVlc0OWFrR2pZSFJObmxDX0tOY3lCYTA5T1FLQkZRTl9pYXlUV1BJUTRsZmlfVTNqcEJmLVBpdzJHejJsTE9XcWl2aXlzMHBWdE9Nd011ZXdpSzZNbGFJU1F3VGd4YTAtbXV6YkpJY0ZER19jM2RjcW4?oc=5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>46092.48127314815</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Zoonotic Viruses May Not Be “Special” Before Spillover - Technology Networks</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Zoonotic Viruses May Not Be “Special” Before Spillover - Technology Networks</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 09:02:26 GMT</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPYXU5WTNhYVBVM2x6R2NJY2JWNGM4T3hOVHFYUU9FMmFvSVJGeFRFZWtGU3YzcU9TOGRhUXRsbkJ3OUpDSjZyMV9QUXREblpqc1JyVTFjaFM4TDBBS0ZIQWVpdVdTVE1abWROMXFldjBsOXJYMGpuN3lQWVlwWTRlUHItZ19QT0NmaEhYWjhtVDMtNzYydEduUkRBdG04dXVVdExBRg?oc=5</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>46092.37668981482</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Debate continues over contentious terror law tweaks - Lismore City News</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Debate continues over contentious terror law tweaks - Lismore City News</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 13:51:53 GMT</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNZDFOQ1VfVU1FTEJOLTl6anhsckxiVHFNOFg4VGNpdEpQdUxqV21uYjQwR2lNdDhlVk9tQmdHZWtkSmF4d2VwVTJvNzBiUHJyNjcxT0Zwd2doLXR2U1FCX3ZIY1h6b3FYdWNkM1I2WldsbERkeWxXUmc3WWNVTXNfR3ppNVgySTBoZUpRMFZaakJrVEZfTUg5b3piT2lnYmwtdE13?oc=5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>46092.57769675926</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Village Wertheim (fallback)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>("Wertheim Village" OR "Wertheim") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>A Blood Test Could Predict Dementia 25 Years Before Symptoms - Technology Networks</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>A Blood Test Could Predict Dementia 25 Years Before Symptoms - Technology Networks</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 13:38:07 GMT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPMFQzWk1icGFIcE5BV25VSmxQWmprRnExVTNHX0ZUdl9KMlhVenRxdmJxcmpVeUE0cVU5TjJFOW5JRkpIUjBvUHNodHpaWXo3cFRwSUIwOFQydGc2VDg4REhVVlk5dDhmSEppaEZMMHBVQVp3T1hoOWtWTVR2ZzRPTmg1ZS1ON25OS3FYZGJKcHVpT0ZyRW9NVFBLUW5NTlpGLVhjR21hWXk1ckVFOHduN1ZSVTd5Z0JfRm5J?oc=5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="n">
+        <v>46092.56813657407</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>Local Town Ingolstadt German</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Unbekannte stehlen mehrere Kisten mit Pfand aus dem Hinterhof eines Lokals - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Unknown people steal several boxes with deposits from the back yard of a restaurant - Augsburger Allgemeine</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Thu, 12 Mar 2026 06:22:45 GMT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxNcEMxVGMwMENOTDFNSTUwZ2RCLUlzdW1TMEVQRzJBWVdwVmNvbF9QZ0cwcGdUYVo3Qzdxai1Xa0N4c0xEek55TDhDT2pVbzlBOUF2ekFDY3c4UDNXVmJHRmk0bFFKUGtldFRodlI1eF9Tb0dnNlAzeHR1b1J5RmM2Zk9IeXJucE9BWWFUdk90bXdHUWM2N3pUMUhSc0ZtRjhocmtrMmZ1Z3o1Z1BrN0dybENVdTV2ZS15NTRadFhLMTA5N3NUN0RsWUlqOUpWNERI?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="n">
+        <v>46093.26579861111</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
         <is>
           <t>A9-Crash bei Langenbruck fordert vier Verletzte und drei demolierte Autos - Pfaffenhofen Today</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>A9 crash near Langenbruck leaves four injured and three demolished cars - Pfaffenhofen Today</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>Wed, 11 Mar 2026 13:37:21 GMT</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE16WFUtbU00dXYzbVc1U1JmQkxUNjdFNTNSaElrdTVWX01ZajY5MTFmaWhvdFN0VGVGcURHTUhoVEoxSWtiaGxqSmhGcklJSzFLaVRqMW9HUjNPUGlDck5qUUhZNU5HM2VrcHc?oc=5</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>google_rss</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE15WlZpWFZxa0UxN0Q3VFlaWlYyRHRRTUs2c3l0a3pBQzEzVUsyVUZ0V2JxbkVoNmd6d3dTcVRnb0txdEd6SnVmMllUNHhEcjFpb0sxMWxGNHVtTENpYy1uLWVkVS1OdkplMXFnWkY1TQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>DE:de</t>
         </is>
       </c>
-      <c r="K28" s="1" t="n">
+      <c r="K54" s="1" t="n">
         <v>46092.56760416667</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Local Town Ingolstadt German</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>("Ingolstadt") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Audi AND -Auto AND -Wetter</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Augsburg/Lindau/Kempten/Ingolstadt/Schwaben/Oberbayern - Die Finanzkontrolle Schwarzarbeit (FKS) des - AD HOC NEWS</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Augsburg/Lindau/Kempten/Ingolstadt/Swabia/Upper Bavaria - The financial control of undeclared work (FKS) - AD HOC NEWS</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 12:10:19 GMT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOek15VnBiZ0oydm40X0xYem4zSzg0R1R6TzFLNGUzWURZWWx6Zk91cUZWNVI5UDByRk9JMzg0MllQWWltOEhuOG1RTURiS1JNYllPMlU2RFBBbDR0dVBMT092UWlUMk91bGZHS29RT2RUMlg3U2dfR05MQnZjWl83cDJFakdHejF0aXVoOVhlY2ViZXRVeUdrRDdOcXBTanNzbmd2Vi1BWXpFNjItRjBHXw?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>DE:de</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="n">
+        <v>46092.50716435185</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>High Level City Spain Spanish</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>("Madrid" OR "Barcelona") AND ("amenaza de bomba" OR "paquete sospechoso" OR "paquete explosivo" OR "ataque con cuchillo" OR "tiroteo" OR "atentado" OR "operación policial" OR "evacuación" OR "artefacto explosivo") AND -fútbol AND -fichaje AND -Liga AND -transferencia</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>11M en Madrid: el atentado que dejó 193 muertos y cambió España - NewsDigitales</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>11M in Madrid: the attack that left 193 dead and changed Spain - NewsDigitales</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 17:34:39 GMT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQNlNJLVFjSHlGS0tIc1NDTkVUVHVMU1FSVEVvUlVxU25LY0dTdWtRbEU0UlYwWmQyS0c4bGdVOW9xc1FlQ2lnS3A0VnlxZEdEd1lkdlpUOV9ibF91ZWJLWWhmT0FHMlFid2JwclhxVzIwTGx4NHJ3enN2MGQ2aUhlTkV2RGpBTUE3QXhEaVR6VTNIMzFfeUZsejlIN3VCTEstclVrcURKMUM?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>ES:es</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="n">
+        <v>46092.73239583334</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>High Level City Spain Spanish</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>("Madrid" OR "Barcelona") AND ("amenaza de bomba" OR "paquete sospechoso" OR "paquete explosivo" OR "ataque con cuchillo" OR "tiroteo" OR "atentado" OR "operación policial" OR "evacuación" OR "artefacto explosivo") AND -fútbol AND -fichaje AND -Liga AND -transferencia</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Cronología del 11M en Madrid: de los atentados en Atocha a las elecciones generales el 14M - Diario AS</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Chronology of 11M in Madrid: from the attacks in Atocha to the general elections on 14M - Diario AS</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 09:20:57 GMT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxQYVdsNnJobzV3b1R6d2t5ZDNmV0F3TUt3elhqQmRNekNFakZWV1JUN3dISmQwZEZEN1RRVjZLR2pSeDhKQWtqam10YkdURlVYaEN6VGIyQ05YeDJqSW5MQTZ6QWRudW5mbUg4N19UVkFwc25jQjJvRE5NUXZGRE9VcklUOEdua1Vmd2tPVFF2bC1kb2hPTGREU3pKQkZCTVVSZTNxdTBDSUVnVWtMbDBkYzdvOHUyNDJLQ1BfM3hTM2dfc3lFR1lGLXB6ZEw5amNz0gHkAUFVX3lxTE5UbDlQUXU1cTJxOWZnSGp5YV9EZHQ5STM5b2FGdVBSeVBKNm5IMzdpV1B3and3YV9QNTk4YWZKZWc1VG1SeG9GaVYtWmZlSXJwN0pZdnNiMnBZUHdDQkk0TjNRNGRrU1QyMlltUzVITW5JYm8zeHRzNmdQOWJoSnl4aUthcmJmNkVnRW96SXlycm5QclJCUWh1SFBLanlhMWw0ZVlqenpMZ05wblNXOHdNZ3YzVTZucHY5aEI2RUhiQlJYY0JuVUJjcmZyNUpLcTFreGNzQS14ZzhtcDhMNXlTS2RCTw?oc=5</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>ES:es</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="n">
+        <v>46092.38954861111</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Village Las Rozas La Roca (fallback)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>("Las Rozas Village" OR "La Roca Village" OR "Las Rozas" OR "La Roca") AND (shopping OR outlet OR luxury OR retail OR news)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Neinver closes 2025 with sales of 1.72 billion (+5%) - Il Sole 24 ORE</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Neinver closes 2025 with sales of 1.72 billion (+5%) - Il Sole 24 ORE</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 14:50:53 GMT</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOZkpTeGh6MkdLdmw3MmhrT1dqRFJaMEtlZ3lBYzhiV3RNbkdDSS1CbFpVSUMweGFGV2IwSEF2MUMwOXpGTG43X1JHYk8ySy04cWhSckJBRU93QVlqaUhIN2trRTU2LVFyazY4LVBpcHg3TUE1cFFvZl9xOG44MURSSlVmX1Z6UV9TdlhCNnF3THZCYVVkV1E?oc=5</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>GB:en</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="n">
+        <v>46092.61866898148</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>High Level City Italy English</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>March 11, 2026: Milan among the top 10 most polluted cities in the world - IQAir</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>March 11, 2026: Milan among the top 10 most polluted cities in the world - IQAir</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 16:59:44 GMT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQNm1OTXI4S0lpZWNna2VlSzBVc2swa3Q5S2VfUjA1dFBuN294V21sYnQ5VWZPSGpIY3dSTlA0V1hKNUpSNE90eUI2V2xTWi1nMHJZWFI2aXYwc1ZfMVIxRU1zRl9TbFljNEpxRGg1SFQ4bG5GMHloOV9EeHR6T3BxTzFYR0J1d09IUEY5RHdsb19yNnBmTFlBVVhENFp2cjJucV93ZlF0SHZoM2M?oc=5</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>IT:en</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="n">
+        <v>46092.70814814815</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>High Level City Italy English</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>("Milan" OR "Milano" OR "Bologna") AND ("Italy" OR "Italian") AND (protest OR demonstration OR rally OR "civil unrest" OR strike OR blockade OR march) AND -football AND -transfer AND -Serie AND -"fashion week" AND -catwalk AND -runway</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Rome &amp; Milan Airports Suffer 21 Cancellations, 81 Delays Amid Middle-East Airspace Reroutes - VisaHQ</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Rome &amp; Milan Airports Suffer 21 Cancellations, 81 Delays Amid Middle-East Airspace Reroutes - VisaHQ</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Thu, 12 Mar 2026 00:29:52 GMT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxPdHJWUVJSeDJPdmE2UWpoelhNTlV3TzAwS2JBaTV5TDdBcU9pSEIydXE3MlNNZEVSUEd4aTRsZkdBemdZTnQxWnR6WTNnTVRpVkk4MDRBT3B1dkp6bnQxdVRwcHdNY2g1QUk5U01rSmVIdnNMR1NYT01sRi04dWJuOEwxUFVyRmJoU2IxTkg5bEZuYXhIRksxZzNKQU53ZU02UEZkQWdjcXhybnVtYTZLRjRrUGtsUndxS0Zkd3hrOU5NeHh0aVYwSjluNA?oc=5</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>en-GB</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>IT:en</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="n">
+        <v>46093.02074074074</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Bologna, corteo pro Palestina al Pilastro - Local Team</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Bologna, pro-Palestine demonstration at the Pilastro - Local Team</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 19:52:33 GMT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOQVRUbVB4VGJsdjUzYkJqU25pV2hLM2I4NThiNzNOSHVUb2l6dmtBdUtLamV1cmtkY2lHNjZWNzV4MWlWM3BHay04M2JYcjdDSXdXbExBcE1ELXZGLW1SeUEwbmxndFF1clhWYklSLUdhZnJwaXpsSVpUWEVzb0tIUGRCdkdDZGxlYWJmODlB?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="n">
+        <v>46092.82815972222</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Brigata Ebraica e corteo del 25 Aprile. Arci: benvenuti senza bandiera d’Israele - Il Giorno</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Jewish Brigade and procession on April 25th. Arci: welcome without the flag of Israel - Il Giorno</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Thu, 12 Mar 2026 04:44:40 GMT</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxOZmozeHN3NGhRRTBKT3dEZlFseHQ1X2I5X1pfWXJGb2ktUTU0WFkyTDFEQk1Lb0dzWTNBakZnT1JRZjJyend6TGRmaklsOHJWcko5UnFabjRzUVRybTdpbS1heVhxTDNLRFBYajYxQ1VxUmRGSUJVem1iYS1EcU5RM1V3?oc=5</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="n">
+        <v>46093.19768518519</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Milano Cortina: tedeschi divisi su forme di protesta contro i russi - ANSA</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Milan Cortina: Germans divided on forms of protest against the Russians - ANSA</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 17:49:08 GMT</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8gFBVV95cUxOZGZpM09EOHJsZU50bmFJU3hxNlNwNi1pS19ua0JXSVJFaWVBS2p2WWQ2TG9jLVN5enRWSm0ySlYtaWJ3NERqOTFvazNfMkk5Qy1TX0lOODByTFQ2WW1KU1Fza1lrVko3bUJGcDZhSzQyaXZvOXF1SmZSUVgwbHNVTUFlUVZvQ0JSMHl0MWR6bXRvRFV3ZXlsU0ZzX2RWYzJVQVN1UGR4aG9jUUhLYnVlQlBzQkFNRkwyWnYxOXBFcFhrTy1PUnJWVHk3OVlBY20tN3ZFMjRUdlMtSml1U1dGZDUya2k3d2pUNnBYZlNSQkRxUdIB8gFBVV95cUxOZGZpM09EOHJsZU50bmFJU3hxNlNwNi1pS19ua0JXSVJFaWVBS2p2WWQ2TG9jLVN5enRWSm0ySlYtaWJ3NERqOTFvazNfMkk5Qy1TX0lOODByTFQ2WW1KU1Fza1lrVko3bUJGcDZhSzQyaXZvOXF1SmZSUVgwbHNVTUFlUVZvQ0JSMHl0MWR6bXRvRFV3ZXlsU0ZzX2RWYzJVQVN1UGR4aG9jUUhLYnVlQlBzQkFNRkwyWnYxOXBFcFhrTy1PUnJWVHk3OVlBY20tN3ZFMjRUdlMtSml1U1dGZDUya2k3d2pUNnBYZlNSQkRxUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K63" s="1" t="n">
+        <v>46092.7424537037</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Coldiretti protesta a Milano, le prime risposte di Regione Lombardia - La Quinta T di Cremona</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Coldiretti protests in Milan, the first responses from the Lombardy Region - La Quinta T of Cremona</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 12:51:59 GMT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQd0E0akR2MUVDOFlPNEtKdlRkNk4ta3FlRFJiVTE3eFJnZjVMSDJRTjJkZ0pZcWgybGNONDFfTzhlcTFmMzNRa2RQdnA4eW9Da0lTWkF4SVVBM011VUVkc2o4TExrcjI2d1RWZDB5Q3E4VWtpeGZDcXRCTjh2NzFMNWNWVk4yMHFqVzlnci1yYXNzekxtVjZESzdsU0RpTVVVWlRYcmEwUVQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="n">
+        <v>46092.53609953704</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>La lettera del sindaco Lepore ai cittadini di Bologna - BolognaToday</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Mayor Lepore's letter to the citizens of Bologna - BolognaToday</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 08:19:39 GMT</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOV0VVUUxLREdvc3hyYXJmNGtaYTZiM0t3NGU2dnJUeWRYOTlPVjNqUkpVOUhER0pHcXNWU0FEcVE2Q1o4c2ozcmxza0pFSjd0MW9KbHRjcHhEUTNJbzFKWnN1SVpvTXNIbVZRdzVJN2N0SzNaMmZLWEFZMmtxcnY3ZHVBd1R0N0ZlSkdRdlIyODNiUXFa?oc=5</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="n">
+        <v>46092.34697916666</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>BOLOGNA: CONTINUA LA RESISTENZA AL PARCO DEL PILASTRO. “BLOCCATO PER ORE IL CANTIERE” - Radio Onda d`Urto</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>BOLOGNA: THE RESISTANCE AT PILASTRO PARK CONTINUES. “CONSTRUCTION SITE BLOCKED FOR HOURS” - Radio Onda d`Urto</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 11:58:00 GMT</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNcDdpSURBSnZlTE9CNFhCSThFRFRuLU5LMGx3b2Ftd3RoenRGXzg1RU5zU1A1Nll4MXA4MTRLbDRRaDhzam9kUC1IUDdIQ0ZJbVA5Zl9XQXZXMzZXamxZSzI4NWhsYzlzSktweUhiSjY1RXdNYXdIYnZrRGtNQ0EzZW94ai12MTZjNEJ4akRSOE03cDZ1SGVCMTVvZjdYdHk0RXN0QXVobUo2dnFDVVNUMG1vS29DQnU0UEtibERPLTg?oc=5</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K66" s="1" t="n">
+        <v>46092.49861111111</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Nuovo corteo al Pilastro: in strada anche i Giovani palestinesi - BolognaToday</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>New procession at the Pillar: Young Palestinians also on the streets - BolognaToday</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 09:26:43 GMT</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNS2tYVFc0WWw1bmFHU2xkdjNVckNMdHU5VXlraG0tRzFad01IbWpBWlhXN0lwY1RiQnN2di0xWnVWVTRGWlU5NGhkU1I3OTlWSU9IVVVOQmFDQnhwSngtLWVBbkZnekxFVVBaX1J5Nk1Gc1JaV29nZkl1UXFQaDVMNHBxY3l1eTNVTGlEVmVlajM2aklNekI5UHBWd0c2dw?oc=5</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K67" s="1" t="n">
+        <v>46092.39355324074</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Pilastro, doppia protesta: blocchi al cantiere e corteo / Video - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Pilastro, double protest: blockades at the construction site and procession / Video - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Thu, 12 Mar 2026 07:37:04 GMT</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQbWNHaTlwWVVqTVJRdWR1ZE9INEZla3hjQ2lxSWV1RnZ3MWRPYUtSdmxZLUZobjZIRnZVcGZLNnR4WmhmQjIzeGJTLVNuNE9nbnI3S2duNUV0S3IwaVVRY2JZb3liQnBlS2VELTU0MkJvNmk1dFRrdnFpQURRLUFfNjAxZzByb0puX1RLOFF6VUliMmptRTQxdQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K68" s="1" t="n">
+        <v>46093.3174074074</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Lanci di sassi contro le auto nel lecchese, identificati tre 13enni - Local Team</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Throwing stones at cars in the Lecco area, three 13 year olds identified - Local Team</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 17:02:15 GMT</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOdVpNS0s5MS05WnZXaFpqdFVROGVxYXNWR1Vnc3BOTlptaE94UFRYM3d3bnFwaTBYRVFKOC05WDlVbUw4NWQ0RTI5eVZDTzBIWVRzd25YTE5LWkQ2V2RHZ3RTd3RaaS0ydElrdHlkSm1xYkstTHI3WjZLakdsR09lWi00b092eWk0UVk4OW5SQWxfQ1lTeExIM3duZVlkVzVUZnk5NE8tSXk2SFgzTEZZRw?oc=5</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K69" s="1" t="n">
+        <v>46092.70989583333</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Anche i Pro-Pal al presidio contro il cantiere MuBa al Pilastro - RaiNews</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Pro-Pal also protest against the MuBa al Pilastro construction site - RaiNews</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 22:08:00 GMT</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxPRWtKNHpUZ2tfU2Y3VjBoR0t5UDFfSm1HVEtkcThfUHVxZHVCTGtTamk2OXBIbnhqWjZwM050eXVtUVJLNHMxNVkzSC1YY1FnYTZYbFZfLWlqa25HRXk0a1BRd0M4QS1MUk5JT19RcXQ3aEdZVGpMUDU4SEtFWThwbWpiU1FyYXBxNjc3ZFRvZW1pQnFIT1VpcWV1bngzcEg1NzZseFZobU1ZaTJvWU5KZVN2cmwxMzZfRlozUmxOU3JTcWtteG5hS2ptWDJ4dmJGdE1vYS1Ocmk3TWlnR0t2d2xKNnJNVlo2ZkRDQWhWRnlNalhCX1HSAfsBQVVfeXFMTTJmMWU2SjlrWk9oRWJuV05YV0ZRLUpsSUtQdVRualpJeDVHS3lXVjBJdXc0Ujc5eXVBZU9EbzdKbTNsRFQxejJ4MUxoWHFRV3FBb0JVRkx1bUtFOU5ObU9LMkZzZHYzTDJYV3VhclJQNi1Td294M3M3X3hOSzBNX1g0RzlSaDUzdjAwTG5tMUdwQVB5SmtFaWU3QjNzRWZRVkNTclRBQ0F0eklYN1JjSFNFcFpwbGwxaTdyVFk5TG92SGhYSlFjQ1pqX3JYVkJqUnNma3RrRGJGbTFsNVJrc1lxa3dRZVFXcTEwZXZWNTZiZWlieUJXdFJSbVE?oc=5</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="n">
+        <v>46092.92222222222</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>High Level City Italy Italian</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>("Milano" OR "Bologna") AND (protesta OR manifestazione OR corteo OR sciopero OR blocco OR presidio OR "sit-in") AND -calcio AND -moda AND -"settimana della moda" AND -Serie AND -mercato</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Nuova protesta al Pilastro: attivisti in resistenza passiva al cantiere del Museo dei Bambini. Venti i denunciati - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>New protest at the Pillar: activists in passive resistance at the construction site of the Children's Museum. Twenty people reported - Il Resto del Carlino</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Wed, 11 Mar 2026 12:46:47 GMT</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQSzhhSGVXcDg0bEUzakNDc2hPSVpaLVd5Yms2VXpFWFNQUVBBZFl3emFrbVllRjZzakstdnFreUVTS0RUWUw3ODhjNklnUldYTi03SFo3Um1NaVVJZkhUcUxhaWRLaG52NE1haU5tclc0STdoNW1ueWdwOHloN0V2VzlESnRmcEVZ?oc=5</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>google_rss</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>IT:it</t>
+        </is>
+      </c>
+      <c r="K71" s="1" t="n">
+        <v>46092.53248842592</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update latest_deduped.xlsx [2026-03-14 08:02 UTC]
</commit_message>
<xml_diff>
--- a/data/latest_deduped.xlsx
+++ b/data/latest_deduped.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,32 +480,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BV Value Retail Crime (fallback)</t>
+          <t>Value Retail Brand</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>("Bicester Village")</t>
+          <t>"Value Retail" OR "Bicester Collection" OR "Chic Outlet Shopping"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Clarion Weekend, 13 March 2026 - Oxford Clarion</t>
+          <t>Net debt of B&amp;M European Value Retail PLC – LSX:A41PFG - TradingView</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Clarion Weekend, 13 March 2026 - Oxford Clarion</t>
+          <t>Net debt of B&amp;M European Value Retail PLC – LSX:A41PFG - TradingView</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 11:36:53 GMT</t>
+          <t>Sat, 14 Mar 2026 04:46:27 GMT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE84dWZjUElubW8teGVGUHpOdFVqTDZfaVlOQTJ1ZzQ5Tlo1ZkNTajJab2VjcmdXVEVfU055RDJ1VUxxRExDdE1iTm5GSFo4WkcteXVzTWRPSmc1OTRUaS03czNZX1Mwdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOTjdFY1A2LXZOTlJpaGp1dFhVa3pGcGFNb3F0NnNGUkcyTnRRSER4QzNRZGV0LVB1YktUS3NYZDVwQW4yOHVFS0tYM3lNX3JzeDVRNnZJVUdQcGRrVGR4aXpXQ0VIUWh6SU9YQkZ6bzVuQmh0OEEyMWJVYnRjRWdpMmR6R3pjclE4?oc=5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="K2" s="1" t="n">
-        <v>46094.48394675926</v>
+        <v>46095.19892361111</v>
       </c>
     </row>
     <row r="3">
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Openings of the week - MCA Insight</t>
+          <t>Clarion Weekend, 13 March 2026 - Oxford Clarion</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Openings of the week - MCA Insight</t>
+          <t>Clarion Weekend, 13 March 2026 - Oxford Clarion</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 09:05:43 GMT</t>
+          <t>Fri, 13 Mar 2026 11:36:53 GMT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE54bFJPZ0tJLWtqM0VNb05UZWloMG9kYkNucE5TRzNaMHRIV2lGd3VDR0tKQVhCVWwycVJsRW9pdGZWdWRnYUdtODdOSUVoZGNUZmZ1X1BTRnZYemFudFpadGwyV090TldCbXRoaXJZUFdHZm9ZZ05v?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE84dWZjUElubW8teGVGUHpOdFVqTDZfaVlOQTJ1ZzQ5Tlo1ZkNTajJab2VjcmdXVEVfU055RDJ1VUxxRExDdE1iTm5GSFo4WkcteXVzTWRPSmc1OTRUaS03czNZX1Mwdw?oc=5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -584,38 +584,38 @@
         </is>
       </c>
       <c r="K3" s="1" t="n">
-        <v>46094.3789699074</v>
+        <v>46094.48394675926</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BV Logistics Disruption</t>
+          <t>BV Value Retail Crime (fallback)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("DHL" OR "UPS" OR "DPD" OR "FedEx" OR "Royal Mail" OR "Parcelforce" OR "EVRI" OR "Dropit") AND (disruption OR strike OR failure OR delay) AND ("UK" OR "United Kingdom" OR "Britain") AND -dental AND -"pay dispute" AND -"postal vote"</t>
+          <t>("Bicester Village")</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Full list of North East postcodes affected by Royal Mail delivery disruption - Chronicle Live</t>
+          <t>Openings of the week - MCA Insight</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Full list of North East postcodes affected by Royal Mail delivery disruption - Chronicle Live</t>
+          <t>Openings of the week - MCA Insight</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 11:34:00 GMT</t>
+          <t>Fri, 13 Mar 2026 09:05:43 GMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxQelRHbS1keDhWdEVBWUdsWFlRMWlrSDhRTVVyZjVNTFp2V1AwNE43QXZaNEhFblZxR3VrMjNTSGRRaGVQWm9SaFlkUmlGM3ZkNHY3SWx5cFQyRUJsdXRqdTEwbTZ5SXVMb0owZ19zOW8zUjJuMlROQVU5VFBFdEgzRkVLdGtINjRJeENBVE95WE9JR0I4VUxr0gGcAUFVX3lxTE01OV92bldDLTdVY0FSQUV1OGFabG1KLTFCcnh0SmVkd25HcW56SC16M0JFQkNEV3FwSEpvcjM3Uk1wUFo4eEtPV19maUZnZ3JEaEk1SElVSUt3d1dPMjdPQnhPNFNsaXNRTWJENjRYUzhydEprLXBWMk0wZXZMWVExUGN4WVlBU3VjTnk5U2s0c2cxamdIY2wxOTVKeQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE54bFJPZ0tJLWtqM0VNb05UZWloMG9kYkNucE5TRzNaMHRIV2lGd3VDR0tKQVhCVWwycVJsRW9pdGZWdWRnYUdtODdOSUVoZGNUZmZ1X1BTRnZYemFudFpadGwyV090TldCbXRoaXJZUFdHZm9ZZ05v?oc=5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -639,38 +639,38 @@
         </is>
       </c>
       <c r="K4" s="1" t="n">
-        <v>46094.48194444444</v>
+        <v>46094.3789699074</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>BV Logistics Disruption</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("DHL" OR "UPS" OR "DPD" OR "FedEx" OR "Royal Mail" OR "Parcelforce" OR "EVRI" OR "Dropit") AND (disruption OR strike OR failure OR delay) AND ("UK" OR "United Kingdom" OR "Britain") AND -dental AND -"pay dispute" AND -"postal vote"</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>"Besparingen Demir leggen bom onder Brusselse kunstacademies” - Groen</t>
+          <t>Royal Mail delivery disruption hits 12 Hull postcodes — full list - Hull Live</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>“Demir's savings put a bomb under Brussels art academies” - Groen</t>
+          <t>Royal Mail delivery disruption hits 12 Hull postcodes — full list - Hull Live</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 12:31:02 GMT</t>
+          <t>Fri, 13 Mar 2026 10:20:00 GMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTFBCVndKS0xWbXdmUVRzU0hoemlVZFZ2QnFUOEIwbndhcnVLM1pJVXpsRm1BMHB4eTZUWlB1eGQwdFUzejNGQmtBZjdBR0RGR3BDMTZfR0lWVE9DNkNZY3VKVjlfT0xoTUNa?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPcExjVnZnNnhRS055RTFpWE1ES2R6NFhwMzU5Q2RobEJPcnlHbENBOGxDQlFEOWdvWWZZM1E2dlk1SktSZk5qTV94OFRLQXl3NG9pSktOeUtmby16cF9jSGtmNGd3N2hERWRRTlJEaW5ZUlpjLWZxSFBhMlROT0l3dGFCV0FFcWROZHlYaXViZ00yaV9UMWd4V1JJSUdjbFAtdlRrSXVWelhVUdIBrwFBVV95cUxQSGZsbURWanNsWFU3czZtQnZTcDkwd2h5OGctSVpCWVZ6OER6UHJ4WEdQMzctVGdiZG9POGlRZWxSUFVZZ2hVUzhfM3dTczJuekN4bXpNbE81LTMxZEhhREhOemRJbGtCNjNObEZBV3g2dHlMWTNWcVFWbl94dkhkVDRpNHRXU1pkVFdrb1QxVk1jWG56UHBZRk03RHBmV0ZDUU00SWZNTzVtN3Z4MjNR?oc=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -680,52 +680,52 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K5" s="1" t="n">
-        <v>46094.52155092593</v>
+        <v>46094.43055555555</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>London Marylebone Incident (fallback)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("London Marylebone" OR "Marylebone station")</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vier verdachten gevat voor drugshandel in Brusselse Noordwijk - HLN</t>
+          <t>Luxury six-bedroom home in Beaconsfield on sale for £3.5m - MSN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Four suspects arrested for drug trafficking in Brussels' Noordwijk - HLN</t>
+          <t>Luxury six-bedroom home in Beaconsfield on sale for £3.5m - MSN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 13:47:17 GMT</t>
+          <t>Sat, 14 Mar 2026 05:00:00 GMT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOdl8yVVNIYmcxbGR2U3p6TXBUQnRGTGxPbGlGS0h2MlRkcUdLNjRIN3NoXzBPU1FBdmtnMzUwcHBzeU1MVlNuV19DTzFFVzhGS0pHclpOMm5kUnN1NWVWbGRwRHRSaHp3Y2szYnQ2UEFYWDZKYU1Xd21lTlpKblBPZ0NRb25XZnVBUkZrRksyOE5wNjlzcEtsbmcta3E2RTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQakR2UDlXR1BXY3JqZ3BQMWF2aDRxZWcyZzVCbG1La2RaN0lNWnVXVmdBZE1iQXN0bWxvcHZheGJhZVFIbDRIUy1WOWhpZTdyUWg2UHNxZU1neHRmVXZseFdoMEZpWndVVEtPY3VOQnVhMm9UdmgxRTU0WG1RLTRzT3pMSndsYnYzQWxkUmRXVmpyQWdwYVRqc01ZQ1owdTJHajladDJHWHpzdXE1U3RmWFlFdkxReTQ?oc=5</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -735,21 +735,21 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>GB:en</t>
         </is>
       </c>
       <c r="K6" s="1" t="n">
-        <v>46094.57450231481</v>
+        <v>46095.20833333334</v>
       </c>
     </row>
     <row r="7">
@@ -765,22 +765,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Brussel peinst niet over verzachting EU-sancties tegen Rusland - Welingelichte Kringen</t>
+          <t>Politie onderzoekt explosie in Schaarbeek - VRT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Brussels is not considering easing EU sanctions against Russia - Well-Informed Circles</t>
+          <t>Police investigate explosion in Schaarbeek - VRT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 12:22:43 GMT</t>
+          <t>Sat, 14 Mar 2026 07:42:51 GMT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPQlJOcjF4VmJYRlExZVc2QzM1RVBvdU9FcmxueTRKSGJ0MjlIRlQwYmdWOW9HLW5NWjd6R29hQkJfRzhzTUVDRk0xUXJVX1hrRXlYaXl6eUNENWJXNEZJejIxd3g2dGc5V2xSa2dlZjc1WVZGT3hDdVFRYzZHaWx6ZTQxLVVqWEFsVU42dFF4Z2Z1dVFNckEyaGZaMjU2OGVjNHQtQUgzbXR1SVY4UkJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxObUJKWGVsdEJ1d19sNm05aGJvSmE3SEhNV1ZSTWRiU2xGbXhjSFVDcWRkcTJHbGRBOGpVXzdBb2tCMUJrTkxpampldnhwcDB4dUF2WVlqTkp5R0xXUWV2S195V2pMOG5NWTV5Uk5JX1l5VkFLYVNjdk80OXRHelZQWDd4bExQTmc?oc=5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="K7" s="1" t="n">
-        <v>46094.51577546296</v>
+        <v>46095.32142361111</v>
       </c>
     </row>
     <row r="8">
@@ -820,22 +820,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Situatie in het Midden-Oosten: updates Rijksoverheid | Ministeries - Rijksoverheid</t>
+          <t>"Besparingen Demir leggen bom onder Brusselse kunstacademies” - Groen</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Situation in the Middle East: updates from the National Government | Ministries - Central Government</t>
+          <t>“Demir's savings put a bomb under Brussels art academies” - Groen</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 14:00:48 GMT</t>
+          <t>Fri, 13 Mar 2026 12:31:02 GMT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOaXRZaWFKNXc1ZllOT09UOU40ZkRJczFFZnItQ3FvanVmbVcyRGNncHhvUmoyVVZ1TEdicjUyM0dLSW1mVGxxcU5YOHJqMDdRcERmbk1GeTZScl9iQUxXVjRjRk5kWDZRbHQxOXJpUEd1UGtob2JyVmNGNVpfdkJpQ1BkZ0Z3UERhdHRHYWxRa0VhclZMZmpuMkthWkNwem1JRUJYbjE3VEY3d2VUU0hYME14UVNyS0NvM0p3NlBKWVFESE9lSmw1SUdnX3QtTlpUUnFWamtTLVFpV2s4RldNa1d3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTFBCVndKS0xWbXdmUVRzU0hoemlVZFZ2QnFUOEIwbndhcnVLM1pJVXpsRm1BMHB4eTZUWlB1eGQwdFUzejNGQmtBZjdBR0RGR3BDMTZfR0lWVE9DNkNZY3VKVjlfT0xoTUNa?oc=5</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="K8" s="1" t="n">
-        <v>46094.58388888889</v>
+        <v>46094.52155092593</v>
       </c>
     </row>
     <row r="9">
@@ -875,22 +875,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Politie vangt dealer die handelde in 13 soorten drugs - HLN</t>
+          <t>Vier verdachten gevat voor drugshandel in Brusselse Noordwijk - HLN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Police catch dealer who dealt in 13 types of drugs - HLN</t>
+          <t>Four suspects arrested for drug trafficking in Brussels' Noordwijk - HLN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 15:26:07 GMT</t>
+          <t>Fri, 13 Mar 2026 13:47:17 GMT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOd1hZdk9vdWZKSVdTVDFKQldsbHNKc242OFhhcnRld0NTZTMyT0Zrc0I1ZEFoRVZ0cmt5Y3d1NC1KUUQ4VWxIRy15T05Od3FuNjJOUllzLTZSaTloUTY2Um5oQUVtdTZQRENHazJQdndSemxyX1B6Vy1WTnNpV0ZTWlMzNEdsOEFRc1FOYjFKZU8zWlhKMDRz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOdl8yVVNIYmcxbGR2U3p6TXBUQnRGTGxPbGlGS0h2MlRkcUdLNjRIN3NoXzBPU1FBdmtnMzUwcHBzeU1MVlNuV19DTzFFVzhGS0pHclpOMm5kUnN1NWVWbGRwRHRSaHp3Y2szYnQ2UEFYWDZKYU1Xd21lTlpKblBPZ0NRb25XZnVBUkZrRksyOE5wNjlzcEtsbmcta3E2RTA?oc=5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="K9" s="1" t="n">
-        <v>46094.64313657407</v>
+        <v>46094.57450231481</v>
       </c>
     </row>
     <row r="10">
@@ -930,22 +930,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ongeval met letsel op P. Debyelaan in Maastricht - AD.nl</t>
+          <t>Brussel peinst niet over verzachting EU-sancties tegen Rusland - Welingelichte Kringen</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Accident with injuries on P. Debyelaan in Maastricht - AD.nl</t>
+          <t>Brussels is not considering easing EU sanctions against Russia - Well-Informed Circles</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 12:23:00 GMT</t>
+          <t>Fri, 13 Mar 2026 12:22:43 GMT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNSzZNSXF4X0dCRnVOWHNaSFRlNzZ2VF84VEt1VzViUzFfT0szSm5TdXIyazBacm9GLVVFNzR6Y09SYmdEOE9jelBteGNsLXV6aldIdEVhbWcwQ09KMC1qdVJlcVg5WjFDVWNLczBUcnBWSXQxbmx6WEJZb0NCbEY3RGZ2cEJGSWlsY0MtbkV4RGoycThvLWFGcDZza2k5Zw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPQlJOcjF4VmJYRlExZVc2QzM1RVBvdU9FcmxueTRKSGJ0MjlIRlQwYmdWOW9HLW5NWjd6R29hQkJfRzhzTUVDRk0xUXJVX1hrRXlYaXl6eUNENWJXNEZJejIxd3g2dGc5V2xSa2dlZjc1WVZGT3hDdVFRYzZHaWx6ZTQxLVVqWEFsVU42dFF4Z2Z1dVFNckEyaGZaMjU2OGVjNHQtQUgzbXR1SVY4UkJ3?oc=5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="K10" s="1" t="n">
-        <v>46094.51597222222</v>
+        <v>46094.51577546296</v>
       </c>
     </row>
     <row r="11">
@@ -985,22 +985,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Milena is een van de vijf vrouwelijke straatveegsters in Brussel: “Nog nooit vreemde reacties gekregen” - Nieuwsblad</t>
+          <t>Twee verdachten opnieuw voor raadkamer in dossier van taximoord: enkelband blijft voor ene, andere blijft in cel - Nieuwsblad</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Milena is one of five female street sweepers in Brussels: “Never received any strange reactions” - Nieuwsblad</t>
+          <t>Two suspects again before the council chamber in the case of taxi murder: ankle bracelet remains for one, the other remains in cell - Nieuwsblad</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 09:44:05 GMT</t>
+          <t>Fri, 13 Mar 2026 23:06:15 GMT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxNVkxTMGJGcjJpT01BLUoxaUtlbFVmZzJBSEdEc3pTUTBIbnN3NEpkR1pRNXJGRm93dkNxdGdWSW1hNVhRbGxOTUctZjVaMERHbHNJSUxPVzRvdHVHMjdncWhfWUo4amJ1Rlp6ejNpTXlPaVVKUE5ZT2Uxc2daMlozVlBOejBvR0JGaGRXeFVQeXZXOG9ZbGs0b2pFd0VMelRiV0Jid3ZNZW9ISzc5eE5DSi16TjNFd2pObGNJcmFzcHNzY0VQemtRT1Vmb0l4UDllTmdsdzEzUWtyMlBicVVNRVl4WnVobHpUQkNtQzk3dmdnOXhmbWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwJBVV95cUxNZE94ZmtvTmZIMklveDB5bTUwaDN2dFBhTW5MUnFkeVcxaFo0c2RMRzE1cGdCYjJNcjh2X3ZOaXFFY3h0U1paamp5VWxwUHpPQ0x0Rm1qZHpRZzR6cUpHTGZodzdSN2FxUTkxREVrNF9PaHhLX3BEQmNPZ0ZFLXlxOGRpWXl4MnhPMGF5V2NLUjRWWmx5bHRpWEpSR09CT09hejZOZFloNEh5RFktakVQRW1NUnBPZ2xXZ0FwUVdKRXlmZTBvdDFCNHdnV1lOYVZISXBJNGlxc0NoRVlyZ2NnSFl3SVNFTzNON05TN3BwRGhET2lwektqRWRZNC1jbC1CMG9IbGZBYXBSbkU?oc=5</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="K11" s="1" t="n">
-        <v>46094.40561342592</v>
+        <v>46094.96267361111</v>
       </c>
     </row>
     <row r="12">
@@ -1040,22 +1040,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Vier verdachten aangehouden na explosie bij synagoge Rotterdam - Welingelichte Kringen</t>
+          <t>Politie vangt dealer die handelde in 13 soorten drugs - HLN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Four suspects arrested after explosion at synagogue Rotterdam - Welingelichte Kringen</t>
+          <t>Police catch dealer who dealt in 13 types of drugs - HLN</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 12:18:38 GMT</t>
+          <t>Fri, 13 Mar 2026 15:26:07 GMT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxORVM5TURHcFJ2dlg3Um8xUXRxS05QUzJKZzdzMlB5MGEtOWVjZTA2VXpYd1ZNLVBDQmRwVFkwUTVmRGRSaWY3eGxVUF8zT2J5QXFxTlgyTFhUYU1HZjFWeVBaQ1hiN3VHVWQ5V3loeVhVRzI0MVU0cllDWEZfRmhTdlVuWjQydW9UNjBRajMzdC1hVlFFYVJvanVlazV6dGdUUWcyRy1IS2lyNnVnTEtn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOd1hZdk9vdWZKSVdTVDFKQldsbHNKc242OFhhcnRld0NTZTMyT0Zrc0I1ZEFoRVZ0cmt5Y3d1NC1KUUQ4VWxIRy15T05Od3FuNjJOUllzLTZSaTloUTY2Um5oQUVtdTZQRENHazJQdndSemxyX1B6Vy1WTnNpV0ZTWlMzNEdsOEFRc1FOYjFKZU8zWlhKMDRz?oc=5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="K12" s="1" t="n">
-        <v>46094.51293981481</v>
+        <v>46094.64313657407</v>
       </c>
     </row>
     <row r="13">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Explosie bij chemiebedrijf in Wetteren: één arbeider met brandwonden naar ziekenhuis - HLN</t>
+          <t>Vier verdachten aangehouden na explosie bij synagoge Rotterdam - Welingelichte Kringen</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Explosion at chemical company in Wetteren: one worker taken to hospital with burns - HLN</t>
+          <t>Four suspects arrested after explosion at synagogue Rotterdam - Welingelichte Kringen</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 14:32:28 GMT</t>
+          <t>Fri, 13 Mar 2026 12:18:38 GMT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQQ2NTZTJTUzkxSGJ6eE1kc1dBcmxFcGl5ZmNfV2VPSll4WGx3MWIxaTFjaHU2dk9RMHFXdTEzdVI3N0ZacktZdk5RRkZHdi1YV0lsTXRzVGhFVWxaTms4Y204d2ZPczN0eWxlelFzdGxwX25lRW8yc3RZd2FfUDdWOV9YQUtaZF9CZFdBRnFrU090bzRhQm92cHJFR3RWVmtxOVU0TDR2cEpUMkhWMTFkcW9CNnplQmxyWmdoSllB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxORVM5TURHcFJ2dlg3Um8xUXRxS05QUzJKZzdzMlB5MGEtOWVjZTA2VXpYd1ZNLVBDQmRwVFkwUTVmRGRSaWY3eGxVUF8zT2J5QXFxTlgyTFhUYU1HZjFWeVBaQ1hiN3VHVWQ5V3loeVhVRzI0MVU0cllDWEZfRmhTdlVuWjQydW9UNjBRajMzdC1hVlFFYVJvanVlazV6dGdUUWcyRy1IS2lyNnVnTEtn?oc=5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="K13" s="1" t="n">
-        <v>46094.60587962963</v>
+        <v>46094.51293981481</v>
       </c>
     </row>
     <row r="14">
@@ -1150,22 +1150,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Man die neergeschoten werd na afzetten zoontje aan school nu zelf voor de rechter in zaak rond cocaïnesmokkel - GVA</t>
+          <t>Actievoerders protesteren aan wapenbeurs in Brussel waar minister Francken contracten laat ondertekenen - HLN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Man who was shot after dropping off son at school now in court in cocaine smuggling case - GVA</t>
+          <t>Campaigners protest at the arms fair in Brussels where Minister Francken has contracts signed - HLN</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 15:24:05 GMT</t>
+          <t>Fri, 13 Mar 2026 11:32:24 GMT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxQSWdETmNWcUc1d2F3MU5feXdka0pETkJJaXh2M2x1LU5KVlA0M0FfaUdSWkxSZFRGVktNb0g5UVByUGV6RTV6RFlNZnAxRndiTzF3TDJnaVpMX0xjUHVCeVM2c2d0RlJyQlo2VE1wd3Utb1RXdFd1NkxVTjlLZHJvZ1hXR3NaZU9UblJUbnZvOEttY0lBdGZ6R005NE41ZzY5UmpoaEE1d1JId3B6MF9EU3Y2TFZWeG1sYU81cXJMVWI1dG5IaXJlaUE0UDB4Wnh6QXpDX0N4aHAzOTY2UVVpSWV3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1wFBVV95cUxPMGFSUEg3NWFiYm1jN190Rm1zYVh2eGRZNWdXOFRDRGhBYTlFN2o1NUp6bkZGTUJVRGFvbGJNZnJ0dXFkQzdpYUxhQnNnRmUwRFlBdTZnZVp2aEk3VUZZaE9PVE0wcTdwOXVWd195TExCVVRYSFhYSklOSVB4alFKQ2lYTVVJZ2V6UkxyZkx5QXRxc05TSGpRcFBfTWZWRUdCdTdmaHFlaDJPbktSTkpCa0FZb0VSWDFoMlhZTDdkeUp5SV9ydWgxQUpPazFEazFsVl94YWNUMA?oc=5</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="K14" s="1" t="n">
-        <v>46094.64172453704</v>
+        <v>46094.48083333333</v>
       </c>
     </row>
     <row r="15">
@@ -1205,22 +1205,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Vijf verdachten in de cel na ontvoering voor losgeld in Opwijk - Nieuwsblad</t>
+          <t>Brussel loopt warm: deze ploegen staan aan de start van de 100km-run van Kom op tegen Kanker - HLN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Five suspects in jail after kidnapping for ransom in Opwijk - Nieuwsblad</t>
+          <t>Brussels is heating up: these teams are at the start of the 100km run of Kom op tegen Kanker - HLN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 14:36:55 GMT</t>
+          <t>Fri, 13 Mar 2026 15:02:17 GMT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxNR0pNY0h0MHRQa2VPeE56cWZMZmRxeDBOcHNVYmlNNHZHWFpJQXdpQmNZQzg1N3Z4bV9aMGlVcFNreGx3LTk2b2dKVHpReHYyLVpuT21DQ0RBclNnTEx4SkgtXy1yM0lUQVFmUFBqcloxQW5EaHBVZVB3aUJDaWluZUd0dVdHbTR5djZFUFhiakVrLU10M2QzWm0zUF8xS20xTzNqX0g1VWVBeXB3TDY1d24tQnk1R1E1MVZ4c2VrUWxsemxYM2xTMVVHSERIOWVkdzlPMjdveHhUUlFOSGtpdg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxOZEcwYmI2eVlXdnpkNXBZdkthaGVEODRLYUNBemVWZldIVC12RnR1Wmd6VGtBQWVOVVdJeFQ4SU9OYnI3amlxNnRiZWNlSi1Hd3lldlNlV1hncjdmenIwMzF0ck50YU5fdjZPV0lJdGtzcVJfX25ROXRaR1RjYjZfSmR4R3BTTk54My1KbDEtYXdNaDZzUDVMYmpYS2lUaENhWE00LTBnMjk0RXd3TzJmM3g3a2dnR0ZYemZrSHdLZm01ODA2Q044?oc=5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="K15" s="1" t="n">
-        <v>46094.60896990741</v>
+        <v>46094.62658564815</v>
       </c>
     </row>
     <row r="16">
@@ -1260,22 +1260,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Heeft het Iraanse regime met een radioboodschap ‘slapende terreurcellen’ wakker geschud? - HBVL</t>
+          <t>Schutter dodelijke schietpartij Virginia was IS-aanhanger - Nieuwsblad</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Did the Iranian regime wake up 'sleeping terror cells' with a radio message? - HBVL</t>
+          <t>Shooter in deadly Virginia shooting was an IS supporter - Nieuwsblad</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 10:00:00 GMT</t>
+          <t>Fri, 13 Mar 2026 11:08:32 GMT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQRmNlNHFRUmhTYzdnNWNmbHVsM0dnVlFJRFMxR21odk0tLThwNmNSR1lVaVVmcy1PMGVHanR5ZkVUQllqLUtfVlFpS04zV3RnLVByYW5pRmZJeXJkOHhZOG02emJZeVNENEdwNENhdmVobnRUU25BSWU0aTExRU8yQXFvcXpCTmNxdDJSeDMyNl9lQlRDOTZVU2lVYzdMVWtKRGxURk1lVGF4T0otUDBNUkVlV2VFVGlCYlRTMXp6dllIaEtUTDlJQ3o2MHNXeXFHS2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNNUVZVVpIbjlDWGpCay1fOXBQSXVTMkFEdWFXUjFVelZxeFNqcnlRVnR3TXhPMkZOUEtvUW9IWENJaTBaNGNnMmNWa2JjR3VQd0ZPQ3l6amJSbnFZcWZwTU1VRTBpRmJBeEZ6WHpJWGNBekVfRHRPNlA3dHI5bGlnYXpaXzdWWnBXdVJmVmxzZEhKdkhEOVF1VGQzTnh6bDFWY2gwY3lWMzY?oc=5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1299,38 +1299,38 @@
         </is>
       </c>
       <c r="K16" s="1" t="n">
-        <v>46094.41666666666</v>
+        <v>46094.46425925926</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>High Level City Belgium Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>("Brussel" OR "Antwerpen" OR "Maastricht") AND (bom OR bommelding OR "verdacht pakket" OR "onbeheerd pakket" OR explosie OR schietpartij OR steekpartij OR liquidatie OR arrestatie)</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Noodverordening uitgeroepen voor gepland protest XR - RTV Maastricht</t>
+          <t>War in the Middle East: latest developments - Brussels Signal</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Emergency decree declared for planned protest XR - RTV Maastricht</t>
+          <t>War in the Middle East: latest developments - Brussels Signal</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 11:17:37 GMT</t>
+          <t>Fri, 13 Mar 2026 13:37:33 GMT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNUG9IOW54bllBWUlkbDZsdHcycm9FeHFncUFPRXEtNXF0eGZoZHpJLTkzZlg3bE1HU05HMnN1bWhIOHNOWXRRa0JNYjlsNnVCRXNkSEtDaVlXRUx6UDFPblBlemVDenVmWkZKU1JuMGRZSGRlWEFTaE5VY28tZE5WWXJwbHhxYnpIUlVNZ2o5ZVp6ZUhybUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPVHZXaHdvQlhmSEk4V2pHZ1g5RHZLaHZRalBaZ3lTTzdvWDQwc3JEQW51U0RPOG04dlFxMzRHOHBfcUtvLWswLXZuOG1fWDhBLU8wQ2R5VTUwZ1R0RFZ4dU9sYXkzSUVCS1Qwa0RmamhQanVxdUJGbWs0cUZXRWlSM0hfSjhPQQ?oc=5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1350,11 +1350,11 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K17" s="1" t="n">
-        <v>46094.47056712963</v>
+        <v>46094.56774305556</v>
       </c>
     </row>
     <row r="18">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>War in the Middle East: latest developments - Brussels Signal</t>
+          <t>Synagogue attack in Liège sparks fears of Iran-linked terror networks in Europe - The Brussels Times</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>War in the Middle East: latest developments - Brussels Signal</t>
+          <t>Synagogue attack in Liège sparks fears of Iran-linked terror networks in Europe - The Brussels Times</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 13:37:33 GMT</t>
+          <t>Fri, 13 Mar 2026 10:08:43 GMT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPVHZXaHdvQlhmSEk4V2pHZ1g5RHZLaHZRalBaZ3lTTzdvWDQwc3JEQW51U0RPOG04dlFxMzRHOHBfcUtvLWswLXZuOG1fWDhBLU8wQ2R5VTUwZ1R0RFZ4dU9sYXkzSUVCS1Qwa0RmamhQanVxdUJGbWs0cUZXRWlSM0hfSjhPQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4AFBVV95cUxNclVCdGUyNHM2bXFUbEtCNzN6cTZaLTlaSWptT3ZuMWVBelJDQU4wcVk4XzQxelU4VjljR1liNW82YXNfNk5jZ2FjMzR4NXl4UVh2aHNjVExhR0phd3VKVExzYjRGSkxHRmM0QWZVVm5WZEc5bHg4ZnJzM3psbkFIdG1UWmtTQVdHcWVrU1Y5azRvRVp3NjRUR2JHdGNjeVoteEZKT2NoVnRFeEpZbnJxTW5KTTJybUFNeUdvQTJNYTBYOHFIVHFUSkg1SjZJWEZYT1lZNjdKQ0c0T3YtQTNJOA?oc=5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1409,38 +1409,38 @@
         </is>
       </c>
       <c r="K18" s="1" t="n">
-        <v>46094.56774305556</v>
+        <v>46094.42271990741</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>High Level City Belgium French</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>"Il y a un avant et un après": le témoignage d'un infirmier coordinateur 10 ans après les attentats de Bruxelles - Artsenkrant</t>
+          <t>Four arrested after synagogue blast in Rotterdam as possible Liège link investigated - The Brussels Times</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>“There is a before and an after”: the testimony of a nurse coordinator 10 years after the Brussels attacks - Artsenkrant</t>
+          <t>Four arrested after synagogue blast in Rotterdam as possible Liège link investigated - The Brussels Times</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 16:00:50 GMT</t>
+          <t>Fri, 13 Mar 2026 15:03:41 GMT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPejZiY2t4QVNVNjM4dDBhM2I1T1YwTWNTNnlWc3hzem82YU81bUljTDhCLXg4QVNBTXNRQzhYNVo4cldzSV9OdHVCRFhkZUNDT3p1V3Z6d2R6OVBXY1BKYkc5UWV3VjBvRC1rNkpqZlYtY0E5TTBhZmdzV3NFSmJrM19R?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxNQXN0a3dvd2FVbmVGWE05cFJkUEE5OTNGZF93UmUyTWpfajhuekxBRExmWVJkOXJHQ0dodUdDVWNmLWNra18yeUlTR3l1Ukk0VHFndndDcHBnU0JPTFdHRi1HOWFxQjd5SU9hcVc5Umd6aFBobUtSdXZhc1BFSEVsek1seGdwTms3TlYxR054bUg5QkpVQnFuRV9reXhhUzk0MV9tMnFBc2ctN3pQRnhKT3ZsQVpFUHItM19UN3Vtcw?oc=5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,42 +1460,42 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>BE:fr</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K19" s="1" t="n">
-        <v>46094.66724537037</v>
+        <v>46094.62755787037</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen Dutch</t>
+          <t>High Level City Belgium English</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
+          <t>("Brussels" OR "Antwerp" OR "Maastricht") AND (bomb OR explosion OR shooting OR stabbing OR "suspicious package" OR "bomb threat" OR "terror") AND -football AND -soccer AND -transfer</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Acht jaar cel voor Hasselaar (35) die zijn vriendin (40) probeerde te wurgen - VRT</t>
+          <t>Attack on Rotterdam synagogue by group claiming to target Jews - Brussels Signal</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Eight years in prison for Hasselaar (35) who tried to strangle his girlfriend (40) - VRT</t>
+          <t>Attack on Rotterdam synagogue by group claiming to target Jews - Brussels Signal</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 15:50:52 GMT</t>
+          <t>Fri, 13 Mar 2026 11:04:23 GMT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNYWFmUE5MQzJUNjhtN2hkUXlaZktuN2JqOUpnY096VkQ4YlJYb3dXZVA4WnEtVUlOcHoxQkg4SXZCNmdibDZnU2RmcVdvbW9HbFFqb2xDN3N5T2RxUVR3V3RPejh0bFhoZXF5T1J4QXp4TTNLWnRsNHlSM2h1TzF3Q3dvaFJ5Y2RCTW1KQmdLSmd1ajB4S1N2VlM3TQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNcVFFQjhkbDRsTUpNRXd2Y2RfOTB6VGhXd2JQZmpWM2w5X2JYcGhnTmU5d0JHUXpMUXFYMUl6TWJkX3NYYndZaTJkckp4N2NsakI1TXlidDc1T1IwalVkeFVMWG4tS1lYbW9ldlk3UUVSMTJHVE5sQ29aeFpvdWxjZzlyVU5McGVOTDZvQ1NZVGEwU2VwUjFWNWhHY3hzUQ?oc=5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>nl</t>
+          <t>en-GB</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1515,42 +1515,42 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>BE:nl</t>
+          <t>BE:en</t>
         </is>
       </c>
       <c r="K20" s="1" t="n">
-        <v>46094.66032407407</v>
+        <v>46094.46137731482</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Local Town Maasmechelen French</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (manifestation OR bombe OR explosion OR fusillade OR couteau OR évacuation OR police OR arrestation OR protestation)</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TC Hasselt - Deux suspects impliqués dans des vols de câbles de recharge arrêtés par la police - DHnet</t>
+          <t>"Il y a un avant et un après": le témoignage d'un infirmier coordinateur 10 ans après les attentats de Bruxelles - Artsenkrant</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TC Hasselt - Two suspects involved in charging cable thefts arrested by police - DHnet</t>
+          <t>“There is a before and an after”: the testimony of a nurse coordinator 10 years after the Brussels attacks - Artsenkrant</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 11:54:00 GMT</t>
+          <t>Fri, 13 Mar 2026 16:00:50 GMT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAJBVV95cUxQZWUwR1habWRyellFdDFzalUwRm5CT25pcHJBTVVISzMxMzMxTTcxV0ZyMHF5MWtiT3Jmenlfck9SODEzX0l0c29jV3pGTks3X0JaeEp1RkkzbFY3R3pyMU5yM2NFWXpqeV9pNER0UHhubVE5cGFGenVhVEF1bEM1NmNRekxTd2lMTkxtVkRnZ1JrTzFvSG04SHFoZjNZX1l1VzNYR3diSXdoQVNSU2dNNXNMUFM1Z3p4NEl6cHZQZ1JHY3JnenFkc0w0dUhRZU4zbVhGV2lreTVBaThiYkticmhRQWNrMGVEbjVsYlJFbVJMQ1VTeVJxNFhfd1lwU2xQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTFBNUFhkRkpkelVWLTJPQml6NFRtM19YNUs2T0w2a1pCR1JzczhhNkltd0FWNWt4LTJBTkFzRjlMdnVjZWlPdTdabHZiUXZTa19VVkU2MUgyT2w3VUhuaTVVYnZmUktJYXlCd0c5cg?oc=5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1574,38 +1574,38 @@
         </is>
       </c>
       <c r="K21" s="1" t="n">
-        <v>46094.49583333333</v>
+        <v>46094.66724537037</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Polizeieinsatz am Heuchelhof: Schlägerei mit mehreren Personen – mehrere Einsatzwagen vor Ort - Main-Post</t>
+          <t>"Avec 45 militaires à Bruxelles, on double le nombre de patrouilles": Bernard Quintin espère un déblocage ce vendredi - BX1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Police operation at Heuchelhof: Fight with several people - several emergency vehicles on site - Main-Post</t>
+          <t>“With 45 soldiers in Brussels, we double the number of patrols”: Bernard Quintin hopes for an unblocking this Friday - BX1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 14:43:00 GMT</t>
+          <t>Fri, 13 Mar 2026 08:21:00 GMT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxPN0pyLTJQdFFHbnMwaEphOFRndFJTYXZEY0RucENNeU5LM2RZMnhHNHk2Tm9sSVRLQloxNmxQYmR1VUVsdEhLLS1OYkVjWW9lWVBHMjNuY1REWWtWMkVYODRXSWNxRWlZRnRpaDBSUFMzckppLU9NaTJodWVEZk1mSTJNb0x0SnViUmtSUmRVVXgtUTVuV205d1hNNFJWZ19FaFNEYlFJVkF5S3ZVZk51TVpZdTF0cVphalRQTkJoOVZLdWhtZlpiYg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQNDhVa2xjT0U0XzNEOG9nZThTX1NKOGdocW82WFNwcEw2SFd3TUlXR3RrU2RIYlByNlhSSHRVQzI5eEZjYk43Rk81SG1fd25hMXloSWRmcjVVTGdWdTBfb0dxMzRSVlFuWnlxZmtkSGktNXc2YnVkOFV4MGllNDl2S1FPVHNkLXlXY0k2dkJXanhHVTZYVkpUc1YyMGtYYzd6a1dSVTVn?oc=5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1615,52 +1615,52 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K22" s="1" t="n">
-        <v>46094.61319444444</v>
+        <v>46094.34791666667</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Karlstadt: Festnahme nach zwei versuchten Einbrüchen in Bankgebäude - Radio Gong Würzburg</t>
+          <t>Stromae fait une apparition surprise sur scène au côté d’Orelsan lors d’un concert à Bruxelles - Ouest-France</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Karlstadt: Arrest after two attempted break-ins into bank buildings - Radio Gong Würzburg</t>
+          <t>Stromae makes a surprise appearance on stage alongside Orelsan during a concert in Brussels - Ouest-France</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 14:00:00 GMT</t>
+          <t>Fri, 13 Mar 2026 16:30:08 GMT</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPQUFJQVhNSXlmTHNxSG40alhRWkNRWGwtdUhHZzh2U280UXNCeVMxdEhQeGIwbi1RbjlicmlGTEgzbFYwZGR5TFBsM18tZS01YS0wTnYtdEZsVjNjMUwzenlHbVZ3ZmdmVjJ4elVNWUJHUDd2NmxScWQzNWNGZkFYajJQUkhCd21IWUJZUkVhcjJYdHNoRVhqdWhWLVI5cHJRRzJQOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwJBVV95cUxNdzV6ZTFSVWtDODdXVDBiVHE5czFMZWVaajhuc1p6dzVVS0NEN19ZdnAyX0ZOUGxXdVZXWXNOU0JSN3RDNGtSVHNHM3c3MVc0TE9lWU0tT1JHcFNwb2pYZVNRMkNGWVF5OHBadEpNbjhiZlV6ZFB0Z1VrN1IyVDNPNjJzS3VfNDltVExxWURWbVdPYjEzOWpKTTlsOHZrSldkM2NXVmFtMGI1V1FXZklLNmVIcC01ekNRYlNlMUx5ZTFFa3NNWDEwaTFiV2VRM19aOEVNNzdMZVBGS3lGbVVTWUY4QUpuVGh5SE9iN3FLelF3ZVVUdWRiazhrbHgtaUJ4Q2FlYmdSdlJjQ2FRT0s0?oc=5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,52 +1670,52 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K23" s="1" t="n">
-        <v>46094.58333333334</v>
+        <v>46094.68759259259</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fahrraddiebstahl an der Friedensbrücke Würzburg: Polizei sucht Geschädigte und Zeugen - Newsallianz.de</t>
+          <t>Le PS premier parti en Wallonie, le PTB creuse l’écart à Bruxelles, le MR recule: tout ce qu’il faut savoir - 7sur7.be</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Bicycle theft at the Peace Bridge in Würzburg: Police are looking for victims and witnesses - Newsallianz.de</t>
+          <t>The PS first party in Wallonia, the PTB widens the gap in Brussels, the MR retreats: everything you need to know - 7sur7.be</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 16:01:11 GMT</t>
+          <t>Fri, 13 Mar 2026 18:30:12 GMT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOMVo3QVJHcDVEN1p5NjVQUFpmbEZjaE1mTldEZ0xPU3RxZ0YzZEVCUE51bDlNOWN6NXF0Z3R2ZGlPd25MSHVlakJHY3pQa1U0b1hjZGIteGNYVUdMcWZXeUJpdFY2cmc1QnY4MlM0M2c0MjZIVU1Icm5nWS1QYlZ4cXEwN1ZzbjJvVExGU3lXOW1hLVlDU2hjdUZJcjZGVFFldHRva1NlTmMtcHFMUzhpQkhzeEE2dlVfcW0teTBORQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQaTNqdzVwMnJnUm1LM0RzcVRkSUJ0aDh1eGtJdXJ2cDExSExNMDBsbmNsYnNHdzV0VHBfTXkzZXJsM29PaWFWdUJwM2Z0VXhqREZKWWpIMDJTcDJ3aWZSaXJaeHVZTGs0UWNpU2tlNWtvYThCQ2ZGSFZKOGU4czVYZUJCam1fNnVreTA1TFBPekVCMHZRRTRZNy0yLXJZdzNzU1RacEJGTE80YUViM0N1QmE5N0ZxZGVGLWVtSmZfam80SldlMWc5eEppRVRNQVhVdG1xUWlqakRKUQ?oc=5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1725,52 +1725,52 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K24" s="1" t="n">
-        <v>46094.66748842593</v>
+        <v>46094.77097222222</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>High Level City Belgium French</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Bruxelles" OR "Anvers" OR "Maastricht") AND (bombe OR explosion OR fusillade OR agression OR couteau OR "colis suspect" OR "alerte à la bombe" OR attentat) AND -football AND -transfert</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Würzburg: Stadt positioniert sich gegen Rechtsextremismus - Charivari Würzburg</t>
+          <t>L'UE craint "des répercussions" sur sa "sécurité" après la levée des sanctions américaines sur le pétrole russ - Boursorama</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Würzburg: City positions itself against right-wing extremism - Charivari Würzburg</t>
+          <t>The EU fears "repercussions" on its "security" after the lifting of American sanctions on Russian oil - Boursorama</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 14:30:00 GMT</t>
+          <t>Fri, 13 Mar 2026 14:11:01 GMT</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPRk10TzF5U202bHdQV2lFM2xBS3Y2SlAxRUt6bTNWLUpDaHR0RW5jWHVSSVVNRWlvV2dSMm51QnZpLVRfY25FUU82WF92aVQycWFJS3Z3cHBveGV4SjloQzhOcHdrU19HUnpoRFpyLWFHeGkxZExUeXo4WTlXcVpZQ3JjSENJOHFCRTVnSm1ZTEdJbjNSdV94eG9tQ3l6SGpNTEs0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqwJBVV95cUxPM29taVFFX05odFh0aDBIaGJtakNzVk0xTzNBNHJ0MlpETUdkLW84eERKZkNkcnREdW1fbE1yMGxmMFZjYkdVWG5lcUF5U09YbzBMUnBQUVJ4VGpxWmZYZkNiNEQ5UDdmY3lDY3hYa2J5dEhJTTM4VEVhdmRSa050LWdHS3ZpOG9HVGlNU0d5YVgtLWl5MER2R3kwVExvdHNQRllBcFJlOVpKY1FlSTNyaG1GWE9VRndjUFh2VU5wcy1yLV9pT19zN2hlX0xNdVo1VEJObE1YVW50alREa25NZkZzUHFjSHlNV0RSRTdYZzFSZEc2SFVXeGZhZTNYelpmdmJUMHpUaTluMWxRWVNyZHBCTXVDSnFDZFJ5WktVMGJMY3pIZzUzTzBaa9IBqwJBVV95cUxPM29taVFFX05odFh0aDBIaGJtakNzVk0xTzNBNHJ0MlpETUdkLW84eERKZkNkcnREdW1fbE1yMGxmMFZjYkdVWG5lcUF5U09YbzBMUnBQUVJ4VGpxWmZYZkNiNEQ5UDdmY3lDY3hYa2J5dEhJTTM4VEVhdmRSa050LWdHS3ZpOG9HVGlNU0d5YVgtLWl5MER2R3kwVExvdHNQRllBcFJlOVpKY1FlSTNyaG1GWE9VRndjUFh2VU5wcy1yLV9pT19zN2hlX0xNdVo1VEJObE1YVW50alREa25NZkZzUHFjSHlNV0RSRTdYZzFSZEc2SFVXeGZhZTNYelpmdmJUMHpUaTluMWxRWVNyZHBCTXVDSnFDZFJ5WktVMGJMY3pIZzUzTzBaaw?oc=5</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1780,52 +1780,52 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:fr</t>
         </is>
       </c>
       <c r="K25" s="1" t="n">
-        <v>46094.60416666666</v>
+        <v>46094.5909837963</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Festnahme nach Überfall auf 90-Jährigen in Mainbernheim - Fränkische Nachrichten</t>
+          <t>Twee mannen aangehouden voor 20-tal diefstallen van laadkabels in Limburg en Luik - VRT</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Arrest after attack on 90-year-old in Mainbernheim - Fränkische Nachrichten</t>
+          <t>Two men arrested for 20 thefts of charging cables in Limburg and Liège - VRT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 13:58:00 GMT</t>
+          <t>Fri, 13 Mar 2026 10:30:14 GMT</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxPOTRIX0RoOWZKU1U5TzZUM0xRMkI3STBPZU5rMVA4bVBIbUJHWS1zZXJMQ3JkcjBFY3ZJY1l4eEZDN29iczM4dklFUE9aWm5ETUVOVTF1Yml3WE5Cc0prUnU0YmZFNjlOMkE2OElZakJMZHBNQ1JSRnFoeVBNWlJ3RE9WZHowNFd5eDg1MkxjdmdwNnB3dlBHeDZma1hoQ0xHcWZPMF9WNG9KRm1XSnpOSnhOdlJmSlJKZldHZDN0TGJoYWxHOXA1ZklmNGlveFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQV1ItcUhTWFh0S3p5alFDY0x0VktfOWZPR0FLSlJQRWpOcm9ORDRwZHJrdDRVYTVOTUZaM1dYTHhpMjNvWE1CRHFXU2UtX2UzMHJIdGotSDlLQzh1TWdOdzFKNDdqRFM0LTlkYjMxR2RTU3NpQnluamxhMmxISWFUSmE3YVFnMGJpYmU5bmJkcS10aW1vZXlNOEhPSzItc0Jhc3d2WXBPNzk?oc=5</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1835,52 +1835,52 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K26" s="1" t="n">
-        <v>46094.58194444444</v>
+        <v>46094.43766203704</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Auto auf Hösbacher Baumarkt-Parkplatz angefahren | Foto: Karl-Josef Hildenbrand (dpa) - main-echo.de</t>
+          <t>Moet er in het uitgaansleven in Hasselt strenger gecontroleerd worden op drugs? © Photo News - HLN</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Car hit in Hösbach hardware store parking lot | Photo: Karl-Josef Hildenbrand (dpa) - main-echo.de</t>
+          <t>Should there be stricter drug controls in the nightlife in Hasselt? © Photo News - HLN</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 12:02:52 GMT</t>
+          <t>Fri, 13 Mar 2026 08:52:33 GMT</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPV2pPSWd1MGZYTjlUcklycy1EeFVvOFpzTUVtclFNbXB3dHZFSGZ5ODQySThYcnBqaW9pZ2FBLUxCdGZlNzVxYWI1bkJoUGU5V09VMElvTG9PM3BZb0w2MDFpYk9OX1ZBLXF0WmR3ZEhTenY5TXJ1M0c3Sy1maldXN1o0Q2hTSHJiN1Q1NFI4dmlVVm5DY0hINm1ibjlpeGRnejlHb1FIb2w?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-wFBVV95cUxOa0xqS3BzTTJXUHoxajZVcjB6V2dsN29OUUZDWFc2TF9uZ2VQUXFmYkozYzd4R0g0SlBremRFeUs4LWpxLWhsWmk5MjYycGdXSDRLM09fU1NxRGxIUE5IOTVnNXBXNlNNM0dya2Z0c1BrYzBPTzdxYmhrR3hKNkdGUVA2bjJncWxyang0RHdKZk8zUDQ1UF9uLThVY05jM2ZUUXA2eHhRRXdFY3NsOG5rSy1mMG14aFU2Ty1rN2pvU3hkTHlKX1I2OFpBQ3pXRkh6TEhtNkJ2b3UwM1l4Z0Z5eWFMdDlNMWRHY1VKNUZZUHVUQlN4dDRUMTlSVQ?oc=5</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1890,52 +1890,52 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K27" s="1" t="n">
-        <v>46094.50199074074</v>
+        <v>46094.36982638889</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Auto in Wertheim angefahren und geflüchtet - Fränkische Nachrichten</t>
+          <t>Acht jaar cel voor Hasselaar (35) die zijn vriendin (40) probeerde te wurgen - VRT</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Car hit in Wertheim and fled - Fränkische Nachrichten</t>
+          <t>Eight years in prison for Hasselaar (35) who tried to strangle his girlfriend (40) - VRT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fri, 13 Mar 2026 11:32:00 GMT</t>
+          <t>Fri, 13 Mar 2026 15:50:52 GMT</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQYWlRcGkwT3dXd3dyWVZRZUZYSC1NYVpaY0V5UVNUbVR4Ulk1NmFTLXRhcWo1OXJrZWpvZEJCZ1d4YkcxLVRPakFzeUo4XzBrdTdiQV9ySk41RUNRRjBsdDBjR0RHUWlKckxPekhmR3ZWbmVsYjZwMmt6SlZ3RTJBcEdURnNUcVhESGt1S0FhUjNPY0w5NEdxMmxsY2x1N1I0NzY3TXl3TmM2Zy1IRjVrZUM5dmszUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNYWFmUE5MQzJUNjhtN2hkUXlaZktuN2JqOUpnY096VkQ4YlJYb3dXZVA4WnEtVUlOcHoxQkg4SXZCNmdibDZnU2RmcVdvbW9HbFFqb2xDN3N5T2RxUVR3V3RPejh0bFhoZXF5T1J4QXp4TTNLWnRsNHlSM2h1TzF3Q3dvaFJ5Y2RCTW1KQmdLSmd1ajB4S1N2VlM3TQ?oc=5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1945,52 +1945,52 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>de</t>
+          <t>nl</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>DE:de</t>
+          <t>BE:nl</t>
         </is>
       </c>
       <c r="K28" s="1" t="n">
-        <v>46094.48055555556</v>
+        <v>46094.66032407407</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Local Town Wertheim German</t>
+          <t>Local Town Maasmechelen Dutch</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>("Wertheim" OR "Würzburg" OR "Aschaffenburg") AND (Protest OR Bombe OR Bombendrohung OR Explosion OR Schießerei OR Polizei OR Evakuierung OR Terrorverdacht) AND -Wetter AND -Schnee</t>
+          <t>("Maasmechelen" OR "Hasselt" OR "Lanaken") AND (protest OR bom OR bommelding OR explosie OR schietpartij OR steekpartij OR evacuatie OR politie OR arrestatie) AND -sport AND -voetbal</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Militär-Konvoi auf Autobahn bei Erlangen: Unfall in Baustelle - A3 derzeit gesperrt - NN.de</t>
+